<commit_message>
Log 2026-07-02: noon TEST 17.2, evening recheck 15.4, dose 1.0 gal; add 4 photos + skimmer ruler
Noon FC 17.2 (CC 0.0) ran +2.1 over prediction; evening recheck 15.4
(CC 0.4) confirmed the noon reading was real, not a test error. Dosed
1.0 gal at 8:30 PM, projecting ~15.7 next noon. New: graduated ruler
mounted on skimmer to start tracking water level.
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1005">
+  <cellXfs count="1121">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -3327,6 +3327,354 @@
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="8" fillId="8" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -3803,7 +4151,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U42"/>
+  <dimension ref="A1:U45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -3973,34 +4321,34 @@
       <c r="U2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="969" t="inlineStr">
+      <c r="A3" s="1085" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="970" t="n"/>
-      <c r="C3" s="970" t="inlineStr">
+      <c r="B3" s="1086" t="n"/>
+      <c r="C3" s="1086" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="971" t="n"/>
-      <c r="E3" s="971" t="n"/>
-      <c r="F3" s="971" t="n"/>
-      <c r="G3" s="971" t="n"/>
-      <c r="H3" s="971" t="n"/>
-      <c r="I3" s="972" t="n"/>
-      <c r="J3" s="973" t="n"/>
-      <c r="K3" s="973" t="n"/>
-      <c r="L3" s="973" t="n"/>
-      <c r="M3" s="971" t="n"/>
-      <c r="N3" s="971" t="n"/>
-      <c r="O3" s="971" t="n"/>
-      <c r="P3" s="974" t="n"/>
-      <c r="Q3" s="971" t="n"/>
-      <c r="R3" s="971" t="n"/>
+      <c r="D3" s="1087" t="n"/>
+      <c r="E3" s="1087" t="n"/>
+      <c r="F3" s="1087" t="n"/>
+      <c r="G3" s="1087" t="n"/>
+      <c r="H3" s="1087" t="n"/>
+      <c r="I3" s="1088" t="n"/>
+      <c r="J3" s="1089" t="n"/>
+      <c r="K3" s="1089" t="n"/>
+      <c r="L3" s="1089" t="n"/>
+      <c r="M3" s="1087" t="n"/>
+      <c r="N3" s="1087" t="n"/>
+      <c r="O3" s="1087" t="n"/>
+      <c r="P3" s="1090" t="n"/>
+      <c r="Q3" s="1087" t="n"/>
+      <c r="R3" s="1087" t="n"/>
       <c r="S3" s="624" t="n"/>
-      <c r="T3" s="970" t="n"/>
+      <c r="T3" s="1086" t="n"/>
       <c r="U3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -4008,42 +4356,42 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="975" t="inlineStr">
+      <c r="A4" s="1091" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="976" t="inlineStr">
+      <c r="B4" s="1092" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="976" t="inlineStr">
+      <c r="C4" s="1092" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="977" t="n"/>
-      <c r="E4" s="977" t="n"/>
-      <c r="F4" s="977" t="n"/>
-      <c r="G4" s="977" t="n"/>
-      <c r="H4" s="977" t="n"/>
-      <c r="I4" s="978" t="n"/>
-      <c r="J4" s="979" t="n"/>
-      <c r="K4" s="979" t="n"/>
-      <c r="L4" s="979" t="n"/>
-      <c r="M4" s="977" t="n">
+      <c r="D4" s="1093" t="n"/>
+      <c r="E4" s="1093" t="n"/>
+      <c r="F4" s="1093" t="n"/>
+      <c r="G4" s="1093" t="n"/>
+      <c r="H4" s="1093" t="n"/>
+      <c r="I4" s="1094" t="n"/>
+      <c r="J4" s="1095" t="n"/>
+      <c r="K4" s="1095" t="n"/>
+      <c r="L4" s="1095" t="n"/>
+      <c r="M4" s="1093" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="977" t="n">
+      <c r="N4" s="1093" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="977" t="n"/>
-      <c r="P4" s="980" t="n"/>
-      <c r="Q4" s="977" t="n"/>
-      <c r="R4" s="977" t="n"/>
+      <c r="O4" s="1093" t="n"/>
+      <c r="P4" s="1096" t="n"/>
+      <c r="Q4" s="1093" t="n"/>
+      <c r="R4" s="1093" t="n"/>
       <c r="S4" s="631" t="n"/>
-      <c r="T4" s="976" t="n"/>
+      <c r="T4" s="1092" t="n"/>
       <c r="U4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -4051,56 +4399,56 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="981" t="inlineStr">
+      <c r="A5" s="1097" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="982" t="inlineStr">
+      <c r="B5" s="1098" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="982" t="inlineStr">
+      <c r="C5" s="1098" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="983" t="n">
+      <c r="D5" s="1099" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="983" t="n">
+      <c r="E5" s="1099" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="983" t="n">
+      <c r="F5" s="1099" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="983" t="n"/>
-      <c r="H5" s="983" t="n"/>
-      <c r="I5" s="984" t="n"/>
-      <c r="J5" s="985" t="n">
+      <c r="G5" s="1099" t="n"/>
+      <c r="H5" s="1099" t="n"/>
+      <c r="I5" s="1100" t="n"/>
+      <c r="J5" s="1101" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="985" t="n">
+      <c r="K5" s="1101" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="985" t="inlineStr">
+      <c r="L5" s="1101" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="983" t="n"/>
-      <c r="N5" s="983" t="n"/>
-      <c r="O5" s="983" t="n">
+      <c r="M5" s="1099" t="n"/>
+      <c r="N5" s="1099" t="n"/>
+      <c r="O5" s="1099" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="986" t="n">
+      <c r="P5" s="1102" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="983" t="n"/>
-      <c r="R5" s="983" t="n"/>
+      <c r="Q5" s="1099" t="n"/>
+      <c r="R5" s="1099" t="n"/>
       <c r="S5" s="813" t="n"/>
-      <c r="T5" s="982" t="n"/>
+      <c r="T5" s="1098" t="n"/>
       <c r="U5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -4108,42 +4456,42 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="987" t="inlineStr">
+      <c r="A6" s="1103" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="988" t="inlineStr">
+      <c r="B6" s="1104" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="988" t="inlineStr">
+      <c r="C6" s="1104" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="989" t="n"/>
-      <c r="E6" s="989" t="n"/>
-      <c r="F6" s="989" t="n"/>
-      <c r="G6" s="989" t="n"/>
-      <c r="H6" s="989" t="n"/>
-      <c r="I6" s="990" t="n"/>
-      <c r="J6" s="991" t="n"/>
-      <c r="K6" s="991" t="n"/>
-      <c r="L6" s="991" t="n"/>
-      <c r="M6" s="989" t="n">
+      <c r="D6" s="1105" t="n"/>
+      <c r="E6" s="1105" t="n"/>
+      <c r="F6" s="1105" t="n"/>
+      <c r="G6" s="1105" t="n"/>
+      <c r="H6" s="1105" t="n"/>
+      <c r="I6" s="1106" t="n"/>
+      <c r="J6" s="1107" t="n"/>
+      <c r="K6" s="1107" t="n"/>
+      <c r="L6" s="1107" t="n"/>
+      <c r="M6" s="1105" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="989" t="n">
+      <c r="N6" s="1105" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="989" t="n"/>
-      <c r="P6" s="992" t="n"/>
-      <c r="Q6" s="989" t="n"/>
-      <c r="R6" s="989" t="n"/>
+      <c r="O6" s="1105" t="n"/>
+      <c r="P6" s="1108" t="n"/>
+      <c r="Q6" s="1105" t="n"/>
+      <c r="R6" s="1105" t="n"/>
       <c r="S6" s="820" t="n"/>
-      <c r="T6" s="988" t="n"/>
+      <c r="T6" s="1104" t="n"/>
       <c r="U6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -4151,38 +4499,38 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="993" t="inlineStr">
+      <c r="A7" s="1109" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="994" t="inlineStr">
+      <c r="B7" s="1110" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="994" t="inlineStr">
+      <c r="C7" s="1110" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="995" t="n"/>
-      <c r="E7" s="995" t="n"/>
-      <c r="F7" s="995" t="n"/>
-      <c r="G7" s="995" t="n"/>
-      <c r="H7" s="995" t="n"/>
-      <c r="I7" s="996" t="n"/>
-      <c r="J7" s="997" t="n"/>
-      <c r="K7" s="997" t="n"/>
-      <c r="L7" s="997" t="n"/>
-      <c r="M7" s="995" t="n"/>
-      <c r="N7" s="995" t="n"/>
-      <c r="O7" s="995" t="n"/>
-      <c r="P7" s="998" t="n"/>
-      <c r="Q7" s="995" t="n"/>
-      <c r="R7" s="995" t="n"/>
+      <c r="D7" s="1111" t="n"/>
+      <c r="E7" s="1111" t="n"/>
+      <c r="F7" s="1111" t="n"/>
+      <c r="G7" s="1111" t="n"/>
+      <c r="H7" s="1111" t="n"/>
+      <c r="I7" s="1112" t="n"/>
+      <c r="J7" s="1113" t="n"/>
+      <c r="K7" s="1113" t="n"/>
+      <c r="L7" s="1113" t="n"/>
+      <c r="M7" s="1111" t="n"/>
+      <c r="N7" s="1111" t="n"/>
+      <c r="O7" s="1111" t="n"/>
+      <c r="P7" s="1114" t="n"/>
+      <c r="Q7" s="1111" t="n"/>
+      <c r="R7" s="1111" t="n"/>
       <c r="S7" s="827" t="n"/>
-      <c r="T7" s="994" t="n"/>
+      <c r="T7" s="1110" t="n"/>
       <c r="U7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -4190,38 +4538,38 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="969" t="inlineStr">
+      <c r="A8" s="1085" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="970" t="inlineStr">
+      <c r="B8" s="1086" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="970" t="inlineStr">
+      <c r="C8" s="1086" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="971" t="n"/>
-      <c r="E8" s="971" t="n"/>
-      <c r="F8" s="971" t="n"/>
-      <c r="G8" s="971" t="n"/>
-      <c r="H8" s="971" t="n"/>
-      <c r="I8" s="972" t="n"/>
-      <c r="J8" s="973" t="n"/>
-      <c r="K8" s="973" t="n"/>
-      <c r="L8" s="973" t="n"/>
-      <c r="M8" s="971" t="n"/>
-      <c r="N8" s="971" t="n"/>
-      <c r="O8" s="971" t="n"/>
-      <c r="P8" s="974" t="n"/>
-      <c r="Q8" s="971" t="n"/>
-      <c r="R8" s="971" t="n"/>
+      <c r="D8" s="1087" t="n"/>
+      <c r="E8" s="1087" t="n"/>
+      <c r="F8" s="1087" t="n"/>
+      <c r="G8" s="1087" t="n"/>
+      <c r="H8" s="1087" t="n"/>
+      <c r="I8" s="1088" t="n"/>
+      <c r="J8" s="1089" t="n"/>
+      <c r="K8" s="1089" t="n"/>
+      <c r="L8" s="1089" t="n"/>
+      <c r="M8" s="1087" t="n"/>
+      <c r="N8" s="1087" t="n"/>
+      <c r="O8" s="1087" t="n"/>
+      <c r="P8" s="1090" t="n"/>
+      <c r="Q8" s="1087" t="n"/>
+      <c r="R8" s="1087" t="n"/>
       <c r="S8" s="624" t="n"/>
-      <c r="T8" s="970" t="n"/>
+      <c r="T8" s="1086" t="n"/>
       <c r="U8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -4229,62 +4577,62 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="999" t="inlineStr">
+      <c r="A9" s="1115" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1000" t="inlineStr">
+      <c r="B9" s="1116" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1000" t="inlineStr">
+      <c r="C9" s="1116" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1001" t="n">
+      <c r="D9" s="1117" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1001" t="n">
+      <c r="E9" s="1117" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1001" t="n">
+      <c r="F9" s="1117" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1001" t="n">
+      <c r="G9" s="1117" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1001" t="n"/>
-      <c r="I9" s="1002" t="n"/>
-      <c r="J9" s="1003" t="n">
+      <c r="H9" s="1117" t="n"/>
+      <c r="I9" s="1118" t="n"/>
+      <c r="J9" s="1119" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1003" t="n">
+      <c r="K9" s="1119" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1003" t="inlineStr">
+      <c r="L9" s="1119" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1001" t="n"/>
-      <c r="N9" s="1001" t="n"/>
-      <c r="O9" s="1001" t="n">
+      <c r="M9" s="1117" t="n"/>
+      <c r="N9" s="1117" t="n"/>
+      <c r="O9" s="1117" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1004" t="n">
+      <c r="P9" s="1120" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1001" t="n"/>
-      <c r="R9" s="1001" t="n"/>
+      <c r="Q9" s="1117" t="n"/>
+      <c r="R9" s="1117" t="n"/>
       <c r="S9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="T9" s="1000" t="n"/>
+      <c r="T9" s="1116" t="n"/>
       <c r="U9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -4292,42 +4640,42 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="999" t="inlineStr">
+      <c r="A10" s="1115" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1000" t="inlineStr">
+      <c r="B10" s="1116" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1000" t="inlineStr">
+      <c r="C10" s="1116" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1001" t="n"/>
-      <c r="E10" s="1001" t="n"/>
-      <c r="F10" s="1001" t="n"/>
-      <c r="G10" s="1001" t="n"/>
-      <c r="H10" s="1001" t="n"/>
-      <c r="I10" s="1002" t="n"/>
-      <c r="J10" s="1003" t="n"/>
-      <c r="K10" s="1003" t="n"/>
-      <c r="L10" s="1003" t="inlineStr">
+      <c r="D10" s="1117" t="n"/>
+      <c r="E10" s="1117" t="n"/>
+      <c r="F10" s="1117" t="n"/>
+      <c r="G10" s="1117" t="n"/>
+      <c r="H10" s="1117" t="n"/>
+      <c r="I10" s="1118" t="n"/>
+      <c r="J10" s="1119" t="n"/>
+      <c r="K10" s="1119" t="n"/>
+      <c r="L10" s="1119" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1001" t="n"/>
-      <c r="N10" s="1001" t="n"/>
-      <c r="O10" s="1001" t="n"/>
-      <c r="P10" s="1004" t="n"/>
-      <c r="Q10" s="1001" t="n"/>
-      <c r="R10" s="1001" t="n"/>
+      <c r="M10" s="1117" t="n"/>
+      <c r="N10" s="1117" t="n"/>
+      <c r="O10" s="1117" t="n"/>
+      <c r="P10" s="1120" t="n"/>
+      <c r="Q10" s="1117" t="n"/>
+      <c r="R10" s="1117" t="n"/>
       <c r="S10" s="659" t="n"/>
-      <c r="T10" s="1000" t="n"/>
+      <c r="T10" s="1116" t="n"/>
       <c r="U10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -4335,42 +4683,42 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="999" t="inlineStr">
+      <c r="A11" s="1115" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1000" t="inlineStr">
+      <c r="B11" s="1116" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1000" t="inlineStr">
+      <c r="C11" s="1116" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1001" t="n"/>
-      <c r="E11" s="1001" t="n"/>
-      <c r="F11" s="1001" t="n"/>
-      <c r="G11" s="1001" t="n"/>
-      <c r="H11" s="1001" t="n"/>
-      <c r="I11" s="1002" t="n"/>
-      <c r="J11" s="1003" t="n"/>
-      <c r="K11" s="1003" t="n"/>
-      <c r="L11" s="1003" t="n"/>
-      <c r="M11" s="1001" t="n">
+      <c r="D11" s="1117" t="n"/>
+      <c r="E11" s="1117" t="n"/>
+      <c r="F11" s="1117" t="n"/>
+      <c r="G11" s="1117" t="n"/>
+      <c r="H11" s="1117" t="n"/>
+      <c r="I11" s="1118" t="n"/>
+      <c r="J11" s="1119" t="n"/>
+      <c r="K11" s="1119" t="n"/>
+      <c r="L11" s="1119" t="n"/>
+      <c r="M11" s="1117" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1001" t="n">
+      <c r="N11" s="1117" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1001" t="n"/>
-      <c r="P11" s="1004" t="n"/>
-      <c r="Q11" s="1001" t="n"/>
-      <c r="R11" s="1001" t="n"/>
+      <c r="O11" s="1117" t="n"/>
+      <c r="P11" s="1120" t="n"/>
+      <c r="Q11" s="1117" t="n"/>
+      <c r="R11" s="1117" t="n"/>
       <c r="S11" s="659" t="n"/>
-      <c r="T11" s="1000" t="n"/>
+      <c r="T11" s="1116" t="n"/>
       <c r="U11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -4378,38 +4726,38 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="975" t="inlineStr">
+      <c r="A12" s="1091" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="976" t="inlineStr">
+      <c r="B12" s="1092" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="976" t="inlineStr">
+      <c r="C12" s="1092" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="977" t="n"/>
-      <c r="E12" s="977" t="n"/>
-      <c r="F12" s="977" t="n"/>
-      <c r="G12" s="977" t="n"/>
-      <c r="H12" s="977" t="n"/>
-      <c r="I12" s="978" t="n"/>
-      <c r="J12" s="979" t="n"/>
-      <c r="K12" s="979" t="n"/>
-      <c r="L12" s="979" t="n"/>
-      <c r="M12" s="977" t="n"/>
-      <c r="N12" s="977" t="n"/>
-      <c r="O12" s="977" t="n"/>
-      <c r="P12" s="980" t="n"/>
-      <c r="Q12" s="977" t="n"/>
-      <c r="R12" s="977" t="n"/>
+      <c r="D12" s="1093" t="n"/>
+      <c r="E12" s="1093" t="n"/>
+      <c r="F12" s="1093" t="n"/>
+      <c r="G12" s="1093" t="n"/>
+      <c r="H12" s="1093" t="n"/>
+      <c r="I12" s="1094" t="n"/>
+      <c r="J12" s="1095" t="n"/>
+      <c r="K12" s="1095" t="n"/>
+      <c r="L12" s="1095" t="n"/>
+      <c r="M12" s="1093" t="n"/>
+      <c r="N12" s="1093" t="n"/>
+      <c r="O12" s="1093" t="n"/>
+      <c r="P12" s="1096" t="n"/>
+      <c r="Q12" s="1093" t="n"/>
+      <c r="R12" s="1093" t="n"/>
       <c r="S12" s="631" t="n"/>
-      <c r="T12" s="976" t="n"/>
+      <c r="T12" s="1092" t="n"/>
       <c r="U12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -4417,34 +4765,34 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="981" t="inlineStr">
+      <c r="A13" s="1097" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="982" t="n"/>
-      <c r="C13" s="982" t="inlineStr">
+      <c r="B13" s="1098" t="n"/>
+      <c r="C13" s="1098" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="983" t="n"/>
-      <c r="E13" s="983" t="n"/>
-      <c r="F13" s="983" t="n"/>
-      <c r="G13" s="983" t="n"/>
-      <c r="H13" s="983" t="n"/>
-      <c r="I13" s="984" t="n"/>
-      <c r="J13" s="985" t="n"/>
-      <c r="K13" s="985" t="n"/>
-      <c r="L13" s="985" t="n"/>
-      <c r="M13" s="983" t="n"/>
-      <c r="N13" s="983" t="n"/>
-      <c r="O13" s="983" t="n"/>
-      <c r="P13" s="986" t="n"/>
-      <c r="Q13" s="983" t="n"/>
-      <c r="R13" s="983" t="n"/>
+      <c r="D13" s="1099" t="n"/>
+      <c r="E13" s="1099" t="n"/>
+      <c r="F13" s="1099" t="n"/>
+      <c r="G13" s="1099" t="n"/>
+      <c r="H13" s="1099" t="n"/>
+      <c r="I13" s="1100" t="n"/>
+      <c r="J13" s="1101" t="n"/>
+      <c r="K13" s="1101" t="n"/>
+      <c r="L13" s="1101" t="n"/>
+      <c r="M13" s="1099" t="n"/>
+      <c r="N13" s="1099" t="n"/>
+      <c r="O13" s="1099" t="n"/>
+      <c r="P13" s="1102" t="n"/>
+      <c r="Q13" s="1099" t="n"/>
+      <c r="R13" s="1099" t="n"/>
       <c r="S13" s="813" t="n"/>
-      <c r="T13" s="982" t="n"/>
+      <c r="T13" s="1098" t="n"/>
       <c r="U13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -4452,52 +4800,52 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="987" t="inlineStr">
+      <c r="A14" s="1103" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="988" t="inlineStr">
+      <c r="B14" s="1104" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="988" t="inlineStr">
+      <c r="C14" s="1104" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="989" t="n"/>
-      <c r="E14" s="989" t="n">
+      <c r="D14" s="1105" t="n"/>
+      <c r="E14" s="1105" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="989" t="n">
+      <c r="F14" s="1105" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="989" t="n">
+      <c r="G14" s="1105" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="989" t="n"/>
-      <c r="I14" s="990" t="n"/>
-      <c r="J14" s="991" t="n"/>
-      <c r="K14" s="991" t="n"/>
-      <c r="L14" s="991" t="n"/>
-      <c r="M14" s="989" t="n"/>
-      <c r="N14" s="989" t="n"/>
-      <c r="O14" s="989" t="n">
+      <c r="H14" s="1105" t="n"/>
+      <c r="I14" s="1106" t="n"/>
+      <c r="J14" s="1107" t="n"/>
+      <c r="K14" s="1107" t="n"/>
+      <c r="L14" s="1107" t="n"/>
+      <c r="M14" s="1105" t="n"/>
+      <c r="N14" s="1105" t="n"/>
+      <c r="O14" s="1105" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="992" t="n">
+      <c r="P14" s="1108" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="989" t="n"/>
-      <c r="R14" s="989" t="n"/>
+      <c r="Q14" s="1105" t="n"/>
+      <c r="R14" s="1105" t="n"/>
       <c r="S14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="T14" s="988" t="n"/>
+      <c r="T14" s="1104" t="n"/>
       <c r="U14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -4505,42 +4853,42 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="987" t="inlineStr">
+      <c r="A15" s="1103" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="988" t="inlineStr">
+      <c r="B15" s="1104" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="988" t="inlineStr">
+      <c r="C15" s="1104" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="989" t="n"/>
-      <c r="E15" s="989" t="n"/>
-      <c r="F15" s="989" t="n"/>
-      <c r="G15" s="989" t="n"/>
-      <c r="H15" s="989" t="n"/>
-      <c r="I15" s="990" t="n"/>
-      <c r="J15" s="991" t="n"/>
-      <c r="K15" s="991" t="n"/>
-      <c r="L15" s="991" t="n"/>
-      <c r="M15" s="989" t="n">
+      <c r="D15" s="1105" t="n"/>
+      <c r="E15" s="1105" t="n"/>
+      <c r="F15" s="1105" t="n"/>
+      <c r="G15" s="1105" t="n"/>
+      <c r="H15" s="1105" t="n"/>
+      <c r="I15" s="1106" t="n"/>
+      <c r="J15" s="1107" t="n"/>
+      <c r="K15" s="1107" t="n"/>
+      <c r="L15" s="1107" t="n"/>
+      <c r="M15" s="1105" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="989" t="n">
+      <c r="N15" s="1105" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="989" t="n"/>
-      <c r="P15" s="992" t="n"/>
-      <c r="Q15" s="989" t="n"/>
-      <c r="R15" s="989" t="n"/>
+      <c r="O15" s="1105" t="n"/>
+      <c r="P15" s="1108" t="n"/>
+      <c r="Q15" s="1105" t="n"/>
+      <c r="R15" s="1105" t="n"/>
       <c r="S15" s="820" t="n"/>
-      <c r="T15" s="988" t="n"/>
+      <c r="T15" s="1104" t="n"/>
       <c r="U15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -4548,38 +4896,38 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="993" t="inlineStr">
+      <c r="A16" s="1109" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="994" t="inlineStr">
+      <c r="B16" s="1110" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="994" t="inlineStr">
+      <c r="C16" s="1110" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="995" t="n"/>
-      <c r="E16" s="995" t="n"/>
-      <c r="F16" s="995" t="n"/>
-      <c r="G16" s="995" t="n"/>
-      <c r="H16" s="995" t="n"/>
-      <c r="I16" s="996" t="n"/>
-      <c r="J16" s="997" t="n"/>
-      <c r="K16" s="997" t="n"/>
-      <c r="L16" s="997" t="n"/>
-      <c r="M16" s="995" t="n"/>
-      <c r="N16" s="995" t="n"/>
-      <c r="O16" s="995" t="n"/>
-      <c r="P16" s="998" t="n"/>
-      <c r="Q16" s="995" t="n"/>
-      <c r="R16" s="995" t="n"/>
+      <c r="D16" s="1111" t="n"/>
+      <c r="E16" s="1111" t="n"/>
+      <c r="F16" s="1111" t="n"/>
+      <c r="G16" s="1111" t="n"/>
+      <c r="H16" s="1111" t="n"/>
+      <c r="I16" s="1112" t="n"/>
+      <c r="J16" s="1113" t="n"/>
+      <c r="K16" s="1113" t="n"/>
+      <c r="L16" s="1113" t="n"/>
+      <c r="M16" s="1111" t="n"/>
+      <c r="N16" s="1111" t="n"/>
+      <c r="O16" s="1111" t="n"/>
+      <c r="P16" s="1114" t="n"/>
+      <c r="Q16" s="1111" t="n"/>
+      <c r="R16" s="1111" t="n"/>
       <c r="S16" s="827" t="n"/>
-      <c r="T16" s="994" t="n"/>
+      <c r="T16" s="1110" t="n"/>
       <c r="U16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -4587,38 +4935,38 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="969" t="inlineStr">
+      <c r="A17" s="1085" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="970" t="inlineStr">
+      <c r="B17" s="1086" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="970" t="inlineStr">
+      <c r="C17" s="1086" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="971" t="n"/>
-      <c r="E17" s="971" t="n"/>
-      <c r="F17" s="971" t="n"/>
-      <c r="G17" s="971" t="n"/>
-      <c r="H17" s="971" t="n"/>
-      <c r="I17" s="972" t="n"/>
-      <c r="J17" s="973" t="n"/>
-      <c r="K17" s="973" t="n"/>
-      <c r="L17" s="973" t="n"/>
-      <c r="M17" s="971" t="n"/>
-      <c r="N17" s="971" t="n"/>
-      <c r="O17" s="971" t="n"/>
-      <c r="P17" s="974" t="n"/>
-      <c r="Q17" s="971" t="n"/>
-      <c r="R17" s="971" t="n"/>
+      <c r="D17" s="1087" t="n"/>
+      <c r="E17" s="1087" t="n"/>
+      <c r="F17" s="1087" t="n"/>
+      <c r="G17" s="1087" t="n"/>
+      <c r="H17" s="1087" t="n"/>
+      <c r="I17" s="1088" t="n"/>
+      <c r="J17" s="1089" t="n"/>
+      <c r="K17" s="1089" t="n"/>
+      <c r="L17" s="1089" t="n"/>
+      <c r="M17" s="1087" t="n"/>
+      <c r="N17" s="1087" t="n"/>
+      <c r="O17" s="1087" t="n"/>
+      <c r="P17" s="1090" t="n"/>
+      <c r="Q17" s="1087" t="n"/>
+      <c r="R17" s="1087" t="n"/>
       <c r="S17" s="624" t="n"/>
-      <c r="T17" s="970" t="n"/>
+      <c r="T17" s="1086" t="n"/>
       <c r="U17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -4626,52 +4974,52 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="999" t="inlineStr">
+      <c r="A18" s="1115" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1000" t="inlineStr">
+      <c r="B18" s="1116" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1000" t="inlineStr">
+      <c r="C18" s="1116" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1001" t="n"/>
-      <c r="E18" s="1001" t="n">
+      <c r="D18" s="1117" t="n"/>
+      <c r="E18" s="1117" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1001" t="n">
+      <c r="F18" s="1117" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1001" t="n">
+      <c r="G18" s="1117" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1001" t="n"/>
-      <c r="I18" s="1002" t="n"/>
-      <c r="J18" s="1003" t="n"/>
-      <c r="K18" s="1003" t="n"/>
-      <c r="L18" s="1003" t="n"/>
-      <c r="M18" s="1001" t="n"/>
-      <c r="N18" s="1001" t="n"/>
-      <c r="O18" s="1001" t="n">
+      <c r="H18" s="1117" t="n"/>
+      <c r="I18" s="1118" t="n"/>
+      <c r="J18" s="1119" t="n"/>
+      <c r="K18" s="1119" t="n"/>
+      <c r="L18" s="1119" t="n"/>
+      <c r="M18" s="1117" t="n"/>
+      <c r="N18" s="1117" t="n"/>
+      <c r="O18" s="1117" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1004" t="n">
+      <c r="P18" s="1120" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1001" t="n"/>
-      <c r="R18" s="1001" t="n"/>
+      <c r="Q18" s="1117" t="n"/>
+      <c r="R18" s="1117" t="n"/>
       <c r="S18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="T18" s="1000" t="n"/>
+      <c r="T18" s="1116" t="n"/>
       <c r="U18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -4679,46 +5027,46 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="999" t="inlineStr">
+      <c r="A19" s="1115" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1000" t="inlineStr">
+      <c r="B19" s="1116" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1000" t="inlineStr">
+      <c r="C19" s="1116" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1001" t="n"/>
-      <c r="E19" s="1001" t="n"/>
-      <c r="F19" s="1001" t="n"/>
-      <c r="G19" s="1001" t="n"/>
-      <c r="H19" s="1001" t="n"/>
-      <c r="I19" s="1002" t="n"/>
-      <c r="J19" s="1003" t="n"/>
-      <c r="K19" s="1003" t="n"/>
-      <c r="L19" s="1003" t="n"/>
-      <c r="M19" s="1001" t="n">
+      <c r="D19" s="1117" t="n"/>
+      <c r="E19" s="1117" t="n"/>
+      <c r="F19" s="1117" t="n"/>
+      <c r="G19" s="1117" t="n"/>
+      <c r="H19" s="1117" t="n"/>
+      <c r="I19" s="1118" t="n"/>
+      <c r="J19" s="1119" t="n"/>
+      <c r="K19" s="1119" t="n"/>
+      <c r="L19" s="1119" t="n"/>
+      <c r="M19" s="1117" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1001" t="n">
+      <c r="N19" s="1117" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1001" t="n"/>
-      <c r="P19" s="1004" t="n"/>
-      <c r="Q19" s="1001" t="n"/>
-      <c r="R19" s="1001" t="n"/>
+      <c r="O19" s="1117" t="n"/>
+      <c r="P19" s="1120" t="n"/>
+      <c r="Q19" s="1117" t="n"/>
+      <c r="R19" s="1117" t="n"/>
       <c r="S19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="T19" s="1000" t="n"/>
+      <c r="T19" s="1116" t="n"/>
       <c r="U19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -4726,42 +5074,42 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="999" t="inlineStr">
+      <c r="A20" s="1115" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1000" t="inlineStr">
+      <c r="B20" s="1116" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1000" t="inlineStr">
+      <c r="C20" s="1116" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1001" t="n"/>
-      <c r="E20" s="1001" t="n"/>
-      <c r="F20" s="1001" t="n"/>
-      <c r="G20" s="1001" t="n"/>
-      <c r="H20" s="1001" t="n"/>
-      <c r="I20" s="1002" t="n"/>
-      <c r="J20" s="1003" t="n"/>
-      <c r="K20" s="1003" t="n"/>
-      <c r="L20" s="1003" t="n"/>
-      <c r="M20" s="1001" t="n"/>
-      <c r="N20" s="1001" t="n"/>
-      <c r="O20" s="1001" t="n"/>
-      <c r="P20" s="1004" t="n"/>
-      <c r="Q20" s="1001" t="n"/>
-      <c r="R20" s="1001" t="n"/>
+      <c r="D20" s="1117" t="n"/>
+      <c r="E20" s="1117" t="n"/>
+      <c r="F20" s="1117" t="n"/>
+      <c r="G20" s="1117" t="n"/>
+      <c r="H20" s="1117" t="n"/>
+      <c r="I20" s="1118" t="n"/>
+      <c r="J20" s="1119" t="n"/>
+      <c r="K20" s="1119" t="n"/>
+      <c r="L20" s="1119" t="n"/>
+      <c r="M20" s="1117" t="n"/>
+      <c r="N20" s="1117" t="n"/>
+      <c r="O20" s="1117" t="n"/>
+      <c r="P20" s="1120" t="n"/>
+      <c r="Q20" s="1117" t="n"/>
+      <c r="R20" s="1117" t="n"/>
       <c r="S20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="T20" s="1000" t="n"/>
+      <c r="T20" s="1116" t="n"/>
       <c r="U20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -4769,38 +5117,38 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="975" t="inlineStr">
+      <c r="A21" s="1091" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="976" t="inlineStr">
+      <c r="B21" s="1092" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="976" t="inlineStr">
+      <c r="C21" s="1092" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="977" t="n"/>
-      <c r="E21" s="977" t="n"/>
-      <c r="F21" s="977" t="n"/>
-      <c r="G21" s="977" t="n"/>
-      <c r="H21" s="977" t="n"/>
-      <c r="I21" s="978" t="n"/>
-      <c r="J21" s="979" t="n"/>
-      <c r="K21" s="979" t="n"/>
-      <c r="L21" s="979" t="n"/>
-      <c r="M21" s="977" t="n"/>
-      <c r="N21" s="977" t="n"/>
-      <c r="O21" s="977" t="n"/>
-      <c r="P21" s="980" t="n"/>
-      <c r="Q21" s="977" t="n"/>
-      <c r="R21" s="977" t="n"/>
+      <c r="D21" s="1093" t="n"/>
+      <c r="E21" s="1093" t="n"/>
+      <c r="F21" s="1093" t="n"/>
+      <c r="G21" s="1093" t="n"/>
+      <c r="H21" s="1093" t="n"/>
+      <c r="I21" s="1094" t="n"/>
+      <c r="J21" s="1095" t="n"/>
+      <c r="K21" s="1095" t="n"/>
+      <c r="L21" s="1095" t="n"/>
+      <c r="M21" s="1093" t="n"/>
+      <c r="N21" s="1093" t="n"/>
+      <c r="O21" s="1093" t="n"/>
+      <c r="P21" s="1096" t="n"/>
+      <c r="Q21" s="1093" t="n"/>
+      <c r="R21" s="1093" t="n"/>
       <c r="S21" s="631" t="n"/>
-      <c r="T21" s="976" t="n"/>
+      <c r="T21" s="1092" t="n"/>
       <c r="U21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -4808,38 +5156,38 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="981" t="inlineStr">
+      <c r="A22" s="1097" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="982" t="inlineStr">
+      <c r="B22" s="1098" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="982" t="inlineStr">
+      <c r="C22" s="1098" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="983" t="n"/>
-      <c r="E22" s="983" t="n"/>
-      <c r="F22" s="983" t="n"/>
-      <c r="G22" s="983" t="n"/>
-      <c r="H22" s="983" t="n"/>
-      <c r="I22" s="984" t="n"/>
-      <c r="J22" s="985" t="n"/>
-      <c r="K22" s="985" t="n"/>
-      <c r="L22" s="985" t="n"/>
-      <c r="M22" s="983" t="n"/>
-      <c r="N22" s="983" t="n"/>
-      <c r="O22" s="983" t="n"/>
-      <c r="P22" s="986" t="n"/>
-      <c r="Q22" s="983" t="n"/>
-      <c r="R22" s="983" t="n"/>
+      <c r="D22" s="1099" t="n"/>
+      <c r="E22" s="1099" t="n"/>
+      <c r="F22" s="1099" t="n"/>
+      <c r="G22" s="1099" t="n"/>
+      <c r="H22" s="1099" t="n"/>
+      <c r="I22" s="1100" t="n"/>
+      <c r="J22" s="1101" t="n"/>
+      <c r="K22" s="1101" t="n"/>
+      <c r="L22" s="1101" t="n"/>
+      <c r="M22" s="1099" t="n"/>
+      <c r="N22" s="1099" t="n"/>
+      <c r="O22" s="1099" t="n"/>
+      <c r="P22" s="1102" t="n"/>
+      <c r="Q22" s="1099" t="n"/>
+      <c r="R22" s="1099" t="n"/>
       <c r="S22" s="813" t="n"/>
-      <c r="T22" s="982" t="n"/>
+      <c r="T22" s="1098" t="n"/>
       <c r="U22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -4847,52 +5195,52 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="987" t="inlineStr">
+      <c r="A23" s="1103" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="988" t="inlineStr">
+      <c r="B23" s="1104" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="988" t="inlineStr">
+      <c r="C23" s="1104" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="989" t="n"/>
-      <c r="E23" s="989" t="n">
+      <c r="D23" s="1105" t="n"/>
+      <c r="E23" s="1105" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="989" t="n">
+      <c r="F23" s="1105" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="989" t="n">
+      <c r="G23" s="1105" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="989" t="n"/>
-      <c r="I23" s="990" t="n"/>
-      <c r="J23" s="991" t="n"/>
-      <c r="K23" s="991" t="n"/>
-      <c r="L23" s="991" t="n"/>
-      <c r="M23" s="989" t="n"/>
-      <c r="N23" s="989" t="n"/>
-      <c r="O23" s="989" t="n">
+      <c r="H23" s="1105" t="n"/>
+      <c r="I23" s="1106" t="n"/>
+      <c r="J23" s="1107" t="n"/>
+      <c r="K23" s="1107" t="n"/>
+      <c r="L23" s="1107" t="n"/>
+      <c r="M23" s="1105" t="n"/>
+      <c r="N23" s="1105" t="n"/>
+      <c r="O23" s="1105" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="992" t="n">
+      <c r="P23" s="1108" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="989" t="n"/>
-      <c r="R23" s="989" t="n"/>
+      <c r="Q23" s="1105" t="n"/>
+      <c r="R23" s="1105" t="n"/>
       <c r="S23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="T23" s="988" t="n"/>
+      <c r="T23" s="1104" t="n"/>
       <c r="U23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -4900,46 +5248,46 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="993" t="inlineStr">
+      <c r="A24" s="1109" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="994" t="inlineStr">
+      <c r="B24" s="1110" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="994" t="inlineStr">
+      <c r="C24" s="1110" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="995" t="n"/>
-      <c r="E24" s="995" t="n"/>
-      <c r="F24" s="995" t="n"/>
-      <c r="G24" s="995" t="n"/>
-      <c r="H24" s="995" t="n"/>
-      <c r="I24" s="996" t="n"/>
-      <c r="J24" s="997" t="n"/>
-      <c r="K24" s="997" t="n"/>
-      <c r="L24" s="997" t="n"/>
-      <c r="M24" s="995" t="n">
+      <c r="D24" s="1111" t="n"/>
+      <c r="E24" s="1111" t="n"/>
+      <c r="F24" s="1111" t="n"/>
+      <c r="G24" s="1111" t="n"/>
+      <c r="H24" s="1111" t="n"/>
+      <c r="I24" s="1112" t="n"/>
+      <c r="J24" s="1113" t="n"/>
+      <c r="K24" s="1113" t="n"/>
+      <c r="L24" s="1113" t="n"/>
+      <c r="M24" s="1111" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="995" t="n">
+      <c r="N24" s="1111" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="995" t="n"/>
-      <c r="P24" s="998" t="n"/>
-      <c r="Q24" s="995" t="n"/>
-      <c r="R24" s="995" t="n"/>
+      <c r="O24" s="1111" t="n"/>
+      <c r="P24" s="1114" t="n"/>
+      <c r="Q24" s="1111" t="n"/>
+      <c r="R24" s="1111" t="n"/>
       <c r="S24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="T24" s="994" t="n"/>
+      <c r="T24" s="1110" t="n"/>
       <c r="U24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -4947,60 +5295,60 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="969" t="inlineStr">
+      <c r="A25" s="1085" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="970" t="inlineStr">
+      <c r="B25" s="1086" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="970" t="inlineStr">
+      <c r="C25" s="1086" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="971" t="n">
+      <c r="D25" s="1087" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="971" t="n">
+      <c r="E25" s="1087" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="971" t="n">
+      <c r="F25" s="1087" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="971" t="n">
+      <c r="G25" s="1087" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="971" t="n"/>
-      <c r="I25" s="972" t="n"/>
-      <c r="J25" s="973" t="n">
+      <c r="H25" s="1087" t="n"/>
+      <c r="I25" s="1088" t="n"/>
+      <c r="J25" s="1089" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="973" t="n">
+      <c r="K25" s="1089" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="973" t="n">
+      <c r="L25" s="1089" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="971" t="n"/>
-      <c r="N25" s="971" t="n"/>
-      <c r="O25" s="971" t="n">
+      <c r="M25" s="1087" t="n"/>
+      <c r="N25" s="1087" t="n"/>
+      <c r="O25" s="1087" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="974" t="n">
+      <c r="P25" s="1090" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="971" t="n"/>
-      <c r="R25" s="971" t="n"/>
+      <c r="Q25" s="1087" t="n"/>
+      <c r="R25" s="1087" t="n"/>
       <c r="S25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="T25" s="970" t="n"/>
+      <c r="T25" s="1086" t="n"/>
       <c r="U25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -5008,46 +5356,46 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="975" t="inlineStr">
+      <c r="A26" s="1091" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="976" t="inlineStr">
+      <c r="B26" s="1092" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="976" t="inlineStr">
+      <c r="C26" s="1092" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="977" t="n"/>
-      <c r="E26" s="977" t="n"/>
-      <c r="F26" s="977" t="n"/>
-      <c r="G26" s="977" t="n"/>
-      <c r="H26" s="977" t="n"/>
-      <c r="I26" s="978" t="n"/>
-      <c r="J26" s="979" t="n"/>
-      <c r="K26" s="979" t="n"/>
-      <c r="L26" s="979" t="n"/>
-      <c r="M26" s="977" t="n">
+      <c r="D26" s="1093" t="n"/>
+      <c r="E26" s="1093" t="n"/>
+      <c r="F26" s="1093" t="n"/>
+      <c r="G26" s="1093" t="n"/>
+      <c r="H26" s="1093" t="n"/>
+      <c r="I26" s="1094" t="n"/>
+      <c r="J26" s="1095" t="n"/>
+      <c r="K26" s="1095" t="n"/>
+      <c r="L26" s="1095" t="n"/>
+      <c r="M26" s="1093" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="977" t="n">
+      <c r="N26" s="1093" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="977" t="n"/>
-      <c r="P26" s="980" t="n"/>
-      <c r="Q26" s="977" t="n"/>
-      <c r="R26" s="977" t="n"/>
+      <c r="O26" s="1093" t="n"/>
+      <c r="P26" s="1096" t="n"/>
+      <c r="Q26" s="1093" t="n"/>
+      <c r="R26" s="1093" t="n"/>
       <c r="S26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="T26" s="976" t="n"/>
+      <c r="T26" s="1092" t="n"/>
       <c r="U26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -5055,52 +5403,52 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="981" t="inlineStr">
+      <c r="A27" s="1097" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="982" t="inlineStr">
+      <c r="B27" s="1098" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="982" t="inlineStr">
+      <c r="C27" s="1098" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="983" t="n"/>
-      <c r="E27" s="983" t="n">
+      <c r="D27" s="1099" t="n"/>
+      <c r="E27" s="1099" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="983" t="n">
+      <c r="F27" s="1099" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="983" t="n">
+      <c r="G27" s="1099" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="983" t="n"/>
-      <c r="I27" s="984" t="n"/>
-      <c r="J27" s="985" t="n"/>
-      <c r="K27" s="985" t="n"/>
-      <c r="L27" s="985" t="n"/>
-      <c r="M27" s="983" t="n"/>
-      <c r="N27" s="983" t="n"/>
-      <c r="O27" s="983" t="n">
+      <c r="H27" s="1099" t="n"/>
+      <c r="I27" s="1100" t="n"/>
+      <c r="J27" s="1101" t="n"/>
+      <c r="K27" s="1101" t="n"/>
+      <c r="L27" s="1101" t="n"/>
+      <c r="M27" s="1099" t="n"/>
+      <c r="N27" s="1099" t="n"/>
+      <c r="O27" s="1099" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="986" t="n">
+      <c r="P27" s="1102" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="983" t="n"/>
-      <c r="R27" s="983" t="n"/>
+      <c r="Q27" s="1099" t="n"/>
+      <c r="R27" s="1099" t="n"/>
       <c r="S27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="T27" s="982" t="n"/>
+      <c r="T27" s="1098" t="n"/>
       <c r="U27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -5108,46 +5456,46 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="993" t="inlineStr">
+      <c r="A28" s="1109" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="994" t="inlineStr">
+      <c r="B28" s="1110" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="994" t="inlineStr">
+      <c r="C28" s="1110" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="995" t="n"/>
-      <c r="E28" s="995" t="n"/>
-      <c r="F28" s="995" t="n"/>
-      <c r="G28" s="995" t="n"/>
-      <c r="H28" s="995" t="n"/>
-      <c r="I28" s="996" t="n"/>
-      <c r="J28" s="997" t="n"/>
-      <c r="K28" s="997" t="n"/>
-      <c r="L28" s="997" t="n"/>
-      <c r="M28" s="995" t="n">
+      <c r="D28" s="1111" t="n"/>
+      <c r="E28" s="1111" t="n"/>
+      <c r="F28" s="1111" t="n"/>
+      <c r="G28" s="1111" t="n"/>
+      <c r="H28" s="1111" t="n"/>
+      <c r="I28" s="1112" t="n"/>
+      <c r="J28" s="1113" t="n"/>
+      <c r="K28" s="1113" t="n"/>
+      <c r="L28" s="1113" t="n"/>
+      <c r="M28" s="1111" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="995" t="n">
+      <c r="N28" s="1111" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="995" t="n"/>
-      <c r="P28" s="998" t="n"/>
-      <c r="Q28" s="995" t="n"/>
-      <c r="R28" s="995" t="n"/>
+      <c r="O28" s="1111" t="n"/>
+      <c r="P28" s="1114" t="n"/>
+      <c r="Q28" s="1111" t="n"/>
+      <c r="R28" s="1111" t="n"/>
       <c r="S28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="T28" s="994" t="n"/>
+      <c r="T28" s="1110" t="n"/>
       <c r="U28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -5155,52 +5503,52 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="969" t="inlineStr">
+      <c r="A29" s="1085" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="970" t="inlineStr">
+      <c r="B29" s="1086" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="970" t="inlineStr">
+      <c r="C29" s="1086" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="971" t="n"/>
-      <c r="E29" s="971" t="n">
+      <c r="D29" s="1087" t="n"/>
+      <c r="E29" s="1087" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="971" t="n">
+      <c r="F29" s="1087" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="971" t="n">
+      <c r="G29" s="1087" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="971" t="n"/>
-      <c r="I29" s="972" t="n"/>
-      <c r="J29" s="973" t="n"/>
-      <c r="K29" s="973" t="n"/>
-      <c r="L29" s="973" t="n"/>
-      <c r="M29" s="971" t="n"/>
-      <c r="N29" s="971" t="n"/>
-      <c r="O29" s="971" t="n">
+      <c r="H29" s="1087" t="n"/>
+      <c r="I29" s="1088" t="n"/>
+      <c r="J29" s="1089" t="n"/>
+      <c r="K29" s="1089" t="n"/>
+      <c r="L29" s="1089" t="n"/>
+      <c r="M29" s="1087" t="n"/>
+      <c r="N29" s="1087" t="n"/>
+      <c r="O29" s="1087" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="974" t="n">
+      <c r="P29" s="1090" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="971" t="n"/>
-      <c r="R29" s="971" t="n"/>
+      <c r="Q29" s="1087" t="n"/>
+      <c r="R29" s="1087" t="n"/>
       <c r="S29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="T29" s="970" t="n"/>
+      <c r="T29" s="1086" t="n"/>
       <c r="U29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -5208,42 +5556,42 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="975" t="inlineStr">
+      <c r="A30" s="1091" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="976" t="inlineStr">
+      <c r="B30" s="1092" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="976" t="inlineStr">
+      <c r="C30" s="1092" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="977" t="n"/>
-      <c r="E30" s="977" t="n"/>
-      <c r="F30" s="977" t="n"/>
-      <c r="G30" s="977" t="n"/>
-      <c r="H30" s="977" t="n"/>
-      <c r="I30" s="978" t="n"/>
-      <c r="J30" s="979" t="n"/>
-      <c r="K30" s="979" t="n"/>
-      <c r="L30" s="979" t="n"/>
-      <c r="M30" s="977" t="n"/>
-      <c r="N30" s="977" t="n"/>
-      <c r="O30" s="977" t="n"/>
-      <c r="P30" s="980" t="n"/>
-      <c r="Q30" s="977" t="n"/>
-      <c r="R30" s="977" t="n"/>
+      <c r="D30" s="1093" t="n"/>
+      <c r="E30" s="1093" t="n"/>
+      <c r="F30" s="1093" t="n"/>
+      <c r="G30" s="1093" t="n"/>
+      <c r="H30" s="1093" t="n"/>
+      <c r="I30" s="1094" t="n"/>
+      <c r="J30" s="1095" t="n"/>
+      <c r="K30" s="1095" t="n"/>
+      <c r="L30" s="1095" t="n"/>
+      <c r="M30" s="1093" t="n"/>
+      <c r="N30" s="1093" t="n"/>
+      <c r="O30" s="1093" t="n"/>
+      <c r="P30" s="1096" t="n"/>
+      <c r="Q30" s="1093" t="n"/>
+      <c r="R30" s="1093" t="n"/>
       <c r="S30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="T30" s="976" t="n"/>
+      <c r="T30" s="1092" t="n"/>
       <c r="U30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -5251,52 +5599,52 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="981" t="inlineStr">
+      <c r="A31" s="1097" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="982" t="inlineStr">
+      <c r="B31" s="1098" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="982" t="inlineStr">
+      <c r="C31" s="1098" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="983" t="n"/>
-      <c r="E31" s="983" t="n">
+      <c r="D31" s="1099" t="n"/>
+      <c r="E31" s="1099" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="983" t="n">
+      <c r="F31" s="1099" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="983" t="n">
+      <c r="G31" s="1099" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="983" t="n"/>
-      <c r="I31" s="984" t="n"/>
-      <c r="J31" s="985" t="n"/>
-      <c r="K31" s="985" t="n"/>
-      <c r="L31" s="985" t="n"/>
-      <c r="M31" s="983" t="n"/>
-      <c r="N31" s="983" t="n"/>
-      <c r="O31" s="983" t="n">
+      <c r="H31" s="1099" t="n"/>
+      <c r="I31" s="1100" t="n"/>
+      <c r="J31" s="1101" t="n"/>
+      <c r="K31" s="1101" t="n"/>
+      <c r="L31" s="1101" t="n"/>
+      <c r="M31" s="1099" t="n"/>
+      <c r="N31" s="1099" t="n"/>
+      <c r="O31" s="1099" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="986" t="n">
+      <c r="P31" s="1102" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="983" t="n"/>
-      <c r="R31" s="983" t="n"/>
+      <c r="Q31" s="1099" t="n"/>
+      <c r="R31" s="1099" t="n"/>
       <c r="S31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="T31" s="982" t="inlineStr">
+      <c r="T31" s="1098" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -5308,48 +5656,48 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="993" t="inlineStr">
+      <c r="A32" s="1109" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="994" t="inlineStr">
+      <c r="B32" s="1110" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="994" t="inlineStr">
+      <c r="C32" s="1110" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="995" t="n"/>
-      <c r="E32" s="995" t="n"/>
-      <c r="F32" s="995" t="n"/>
-      <c r="G32" s="995" t="n"/>
-      <c r="H32" s="995" t="n">
+      <c r="D32" s="1111" t="n"/>
+      <c r="E32" s="1111" t="n"/>
+      <c r="F32" s="1111" t="n"/>
+      <c r="G32" s="1111" t="n"/>
+      <c r="H32" s="1111" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="996" t="n"/>
-      <c r="J32" s="997" t="n"/>
-      <c r="K32" s="997" t="n"/>
-      <c r="L32" s="997" t="n"/>
-      <c r="M32" s="995" t="n">
+      <c r="I32" s="1112" t="n"/>
+      <c r="J32" s="1113" t="n"/>
+      <c r="K32" s="1113" t="n"/>
+      <c r="L32" s="1113" t="n"/>
+      <c r="M32" s="1111" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="995" t="n">
+      <c r="N32" s="1111" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="995" t="n"/>
-      <c r="P32" s="998" t="n"/>
-      <c r="Q32" s="995" t="n"/>
-      <c r="R32" s="995" t="n"/>
+      <c r="O32" s="1111" t="n"/>
+      <c r="P32" s="1114" t="n"/>
+      <c r="Q32" s="1111" t="n"/>
+      <c r="R32" s="1111" t="n"/>
       <c r="S32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="T32" s="994" t="n"/>
+      <c r="T32" s="1110" t="n"/>
       <c r="U32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -5357,48 +5705,48 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="969" t="inlineStr">
+      <c r="A33" s="1085" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="970" t="inlineStr">
+      <c r="B33" s="1086" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="970" t="inlineStr">
+      <c r="C33" s="1086" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="971" t="n"/>
-      <c r="E33" s="971" t="n">
+      <c r="D33" s="1087" t="n"/>
+      <c r="E33" s="1087" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="971" t="n">
+      <c r="F33" s="1087" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="971" t="n">
+      <c r="G33" s="1087" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="971" t="n"/>
-      <c r="I33" s="972" t="n">
+      <c r="H33" s="1087" t="n"/>
+      <c r="I33" s="1088" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="973" t="n"/>
-      <c r="K33" s="973" t="n"/>
-      <c r="L33" s="973" t="n"/>
-      <c r="M33" s="971" t="n"/>
-      <c r="N33" s="971" t="n"/>
-      <c r="O33" s="971" t="n">
+      <c r="J33" s="1089" t="n"/>
+      <c r="K33" s="1089" t="n"/>
+      <c r="L33" s="1089" t="n"/>
+      <c r="M33" s="1087" t="n"/>
+      <c r="N33" s="1087" t="n"/>
+      <c r="O33" s="1087" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="974" t="n">
+      <c r="P33" s="1090" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="971" t="n"/>
-      <c r="R33" s="971" t="n">
+      <c r="Q33" s="1087" t="n"/>
+      <c r="R33" s="1087" t="n">
         <v>79</v>
       </c>
       <c r="S33" s="624" t="inlineStr">
@@ -5406,7 +5754,7 @@
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="T33" s="970" t="inlineStr">
+      <c r="T33" s="1086" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -5418,48 +5766,48 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="975" t="inlineStr">
+      <c r="A34" s="1091" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="976" t="inlineStr">
+      <c r="B34" s="1092" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="976" t="inlineStr">
+      <c r="C34" s="1092" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="977" t="n"/>
-      <c r="E34" s="977" t="n"/>
-      <c r="F34" s="977" t="n"/>
-      <c r="G34" s="977" t="n"/>
-      <c r="H34" s="977" t="n">
+      <c r="D34" s="1093" t="n"/>
+      <c r="E34" s="1093" t="n"/>
+      <c r="F34" s="1093" t="n"/>
+      <c r="G34" s="1093" t="n"/>
+      <c r="H34" s="1093" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="978" t="n"/>
-      <c r="J34" s="979" t="n"/>
-      <c r="K34" s="979" t="n"/>
-      <c r="L34" s="979" t="n"/>
-      <c r="M34" s="977" t="n">
+      <c r="I34" s="1094" t="n"/>
+      <c r="J34" s="1095" t="n"/>
+      <c r="K34" s="1095" t="n"/>
+      <c r="L34" s="1095" t="n"/>
+      <c r="M34" s="1093" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="977" t="n">
+      <c r="N34" s="1093" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="977" t="n"/>
-      <c r="P34" s="980" t="n"/>
-      <c r="Q34" s="977" t="n"/>
-      <c r="R34" s="977" t="n"/>
+      <c r="O34" s="1093" t="n"/>
+      <c r="P34" s="1096" t="n"/>
+      <c r="Q34" s="1093" t="n"/>
+      <c r="R34" s="1093" t="n"/>
       <c r="S34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="T34" s="976" t="n"/>
+      <c r="T34" s="1092" t="n"/>
       <c r="U34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -5467,48 +5815,48 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="981" t="inlineStr">
+      <c r="A35" s="1097" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="982" t="inlineStr">
+      <c r="B35" s="1098" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="982" t="inlineStr">
+      <c r="C35" s="1098" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="983" t="n"/>
-      <c r="E35" s="983" t="n">
+      <c r="D35" s="1099" t="n"/>
+      <c r="E35" s="1099" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="983" t="n">
+      <c r="F35" s="1099" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="983" t="n">
+      <c r="G35" s="1099" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="983" t="n"/>
-      <c r="I35" s="984" t="n">
+      <c r="H35" s="1099" t="n"/>
+      <c r="I35" s="1100" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="985" t="n"/>
-      <c r="K35" s="985" t="n"/>
-      <c r="L35" s="985" t="n"/>
-      <c r="M35" s="983" t="n"/>
-      <c r="N35" s="983" t="n"/>
-      <c r="O35" s="983" t="n">
+      <c r="J35" s="1101" t="n"/>
+      <c r="K35" s="1101" t="n"/>
+      <c r="L35" s="1101" t="n"/>
+      <c r="M35" s="1099" t="n"/>
+      <c r="N35" s="1099" t="n"/>
+      <c r="O35" s="1099" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="986" t="n">
+      <c r="P35" s="1102" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="983" t="n"/>
-      <c r="R35" s="983" t="n">
+      <c r="Q35" s="1099" t="n"/>
+      <c r="R35" s="1099" t="n">
         <v>80</v>
       </c>
       <c r="S35" s="813" t="inlineStr">
@@ -5516,7 +5864,7 @@
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="T35" s="982" t="inlineStr">
+      <c r="T35" s="1098" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -5528,48 +5876,48 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="987" t="inlineStr">
+      <c r="A36" s="1103" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="988" t="inlineStr">
+      <c r="B36" s="1104" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="988" t="inlineStr">
+      <c r="C36" s="1104" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="989" t="n"/>
-      <c r="E36" s="989" t="n"/>
-      <c r="F36" s="989" t="n"/>
-      <c r="G36" s="989" t="n"/>
-      <c r="H36" s="989" t="n">
+      <c r="D36" s="1105" t="n"/>
+      <c r="E36" s="1105" t="n"/>
+      <c r="F36" s="1105" t="n"/>
+      <c r="G36" s="1105" t="n"/>
+      <c r="H36" s="1105" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="990" t="n"/>
-      <c r="J36" s="991" t="n"/>
-      <c r="K36" s="991" t="n"/>
-      <c r="L36" s="991" t="n"/>
-      <c r="M36" s="989" t="n">
+      <c r="I36" s="1106" t="n"/>
+      <c r="J36" s="1107" t="n"/>
+      <c r="K36" s="1107" t="n"/>
+      <c r="L36" s="1107" t="n"/>
+      <c r="M36" s="1105" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="989" t="n">
+      <c r="N36" s="1105" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="989" t="n"/>
-      <c r="P36" s="992" t="n"/>
-      <c r="Q36" s="989" t="n"/>
-      <c r="R36" s="989" t="n"/>
+      <c r="O36" s="1105" t="n"/>
+      <c r="P36" s="1108" t="n"/>
+      <c r="Q36" s="1105" t="n"/>
+      <c r="R36" s="1105" t="n"/>
       <c r="S36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="T36" s="988" t="n"/>
+      <c r="T36" s="1104" t="n"/>
       <c r="U36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -5577,40 +5925,40 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="993" t="inlineStr">
+      <c r="A37" s="1109" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="994" t="inlineStr">
+      <c r="B37" s="1110" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="994" t="inlineStr">
+      <c r="C37" s="1110" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="995" t="n"/>
-      <c r="E37" s="995" t="n"/>
-      <c r="F37" s="995" t="n"/>
-      <c r="G37" s="995" t="n"/>
-      <c r="H37" s="995" t="n"/>
-      <c r="I37" s="996" t="n"/>
-      <c r="J37" s="997" t="n"/>
-      <c r="K37" s="997" t="n"/>
-      <c r="L37" s="997" t="n"/>
-      <c r="M37" s="995" t="n"/>
-      <c r="N37" s="995" t="n"/>
-      <c r="O37" s="995" t="n"/>
-      <c r="P37" s="998" t="n"/>
-      <c r="Q37" s="995" t="n">
+      <c r="D37" s="1111" t="n"/>
+      <c r="E37" s="1111" t="n"/>
+      <c r="F37" s="1111" t="n"/>
+      <c r="G37" s="1111" t="n"/>
+      <c r="H37" s="1111" t="n"/>
+      <c r="I37" s="1112" t="n"/>
+      <c r="J37" s="1113" t="n"/>
+      <c r="K37" s="1113" t="n"/>
+      <c r="L37" s="1113" t="n"/>
+      <c r="M37" s="1111" t="n"/>
+      <c r="N37" s="1111" t="n"/>
+      <c r="O37" s="1111" t="n"/>
+      <c r="P37" s="1114" t="n"/>
+      <c r="Q37" s="1111" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="995" t="n"/>
+      <c r="R37" s="1111" t="n"/>
       <c r="S37" s="827" t="n"/>
-      <c r="T37" s="994" t="n"/>
+      <c r="T37" s="1110" t="n"/>
       <c r="U37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -5618,48 +5966,48 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="969" t="inlineStr">
+      <c r="A38" s="1085" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="970" t="inlineStr">
+      <c r="B38" s="1086" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="970" t="inlineStr">
+      <c r="C38" s="1086" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="971" t="n"/>
-      <c r="E38" s="971" t="n">
+      <c r="D38" s="1087" t="n"/>
+      <c r="E38" s="1087" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="971" t="n">
+      <c r="F38" s="1087" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="971" t="n">
+      <c r="G38" s="1087" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="971" t="n"/>
-      <c r="I38" s="972" t="n">
+      <c r="H38" s="1087" t="n"/>
+      <c r="I38" s="1088" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="973" t="n"/>
-      <c r="K38" s="973" t="n"/>
-      <c r="L38" s="973" t="n"/>
-      <c r="M38" s="971" t="n"/>
-      <c r="N38" s="971" t="n"/>
-      <c r="O38" s="971" t="n">
+      <c r="J38" s="1089" t="n"/>
+      <c r="K38" s="1089" t="n"/>
+      <c r="L38" s="1089" t="n"/>
+      <c r="M38" s="1087" t="n"/>
+      <c r="N38" s="1087" t="n"/>
+      <c r="O38" s="1087" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="974" t="n">
+      <c r="P38" s="1090" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="971" t="n"/>
-      <c r="R38" s="971" t="n">
+      <c r="Q38" s="1087" t="n"/>
+      <c r="R38" s="1087" t="n">
         <v>80.5</v>
       </c>
       <c r="S38" s="624" t="inlineStr">
@@ -5667,7 +6015,7 @@
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="T38" s="970" t="inlineStr">
+      <c r="T38" s="1086" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -5679,48 +6027,48 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="999" t="inlineStr">
+      <c r="A39" s="1115" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1000" t="inlineStr">
+      <c r="B39" s="1116" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1000" t="inlineStr">
+      <c r="C39" s="1116" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1001" t="n"/>
-      <c r="E39" s="1001" t="n"/>
-      <c r="F39" s="1001" t="n"/>
-      <c r="G39" s="1001" t="n"/>
-      <c r="H39" s="1001" t="n">
+      <c r="D39" s="1117" t="n"/>
+      <c r="E39" s="1117" t="n"/>
+      <c r="F39" s="1117" t="n"/>
+      <c r="G39" s="1117" t="n"/>
+      <c r="H39" s="1117" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1002" t="n"/>
-      <c r="J39" s="1003" t="n"/>
-      <c r="K39" s="1003" t="n"/>
-      <c r="L39" s="1003" t="n"/>
-      <c r="M39" s="1001" t="n">
+      <c r="I39" s="1118" t="n"/>
+      <c r="J39" s="1119" t="n"/>
+      <c r="K39" s="1119" t="n"/>
+      <c r="L39" s="1119" t="n"/>
+      <c r="M39" s="1117" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1001" t="n">
+      <c r="N39" s="1117" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1001" t="n"/>
-      <c r="P39" s="1004" t="n"/>
-      <c r="Q39" s="1001" t="n"/>
-      <c r="R39" s="1001" t="n"/>
+      <c r="O39" s="1117" t="n"/>
+      <c r="P39" s="1120" t="n"/>
+      <c r="Q39" s="1117" t="n"/>
+      <c r="R39" s="1117" t="n"/>
       <c r="S39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="T39" s="1000" t="n"/>
+      <c r="T39" s="1116" t="n"/>
       <c r="U39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -5728,40 +6076,40 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="975" t="inlineStr">
+      <c r="A40" s="1091" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="976" t="inlineStr">
+      <c r="B40" s="1092" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="976" t="inlineStr">
+      <c r="C40" s="1092" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="977" t="n"/>
-      <c r="E40" s="977" t="n"/>
-      <c r="F40" s="977" t="n"/>
-      <c r="G40" s="977" t="n"/>
-      <c r="H40" s="977" t="n"/>
-      <c r="I40" s="978" t="n"/>
-      <c r="J40" s="979" t="n"/>
-      <c r="K40" s="979" t="n"/>
-      <c r="L40" s="979" t="n"/>
-      <c r="M40" s="977" t="n"/>
-      <c r="N40" s="977" t="n"/>
-      <c r="O40" s="977" t="n"/>
-      <c r="P40" s="980" t="n"/>
-      <c r="Q40" s="977" t="n">
+      <c r="D40" s="1093" t="n"/>
+      <c r="E40" s="1093" t="n"/>
+      <c r="F40" s="1093" t="n"/>
+      <c r="G40" s="1093" t="n"/>
+      <c r="H40" s="1093" t="n"/>
+      <c r="I40" s="1094" t="n"/>
+      <c r="J40" s="1095" t="n"/>
+      <c r="K40" s="1095" t="n"/>
+      <c r="L40" s="1095" t="n"/>
+      <c r="M40" s="1093" t="n"/>
+      <c r="N40" s="1093" t="n"/>
+      <c r="O40" s="1093" t="n"/>
+      <c r="P40" s="1096" t="n"/>
+      <c r="Q40" s="1093" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="977" t="n"/>
+      <c r="R40" s="1093" t="n"/>
       <c r="S40" s="631" t="n"/>
-      <c r="T40" s="976" t="n"/>
+      <c r="T40" s="1092" t="n"/>
       <c r="U40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -5769,48 +6117,48 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="981" t="inlineStr">
+      <c r="A41" s="1097" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="982" t="inlineStr">
+      <c r="B41" s="1098" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="982" t="inlineStr">
+      <c r="C41" s="1098" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="983" t="n"/>
-      <c r="E41" s="983" t="n">
+      <c r="D41" s="1099" t="n"/>
+      <c r="E41" s="1099" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="983" t="n">
+      <c r="F41" s="1099" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="983" t="n">
+      <c r="G41" s="1099" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="983" t="n"/>
-      <c r="I41" s="984" t="n">
+      <c r="H41" s="1099" t="n"/>
+      <c r="I41" s="1100" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="985" t="n"/>
-      <c r="K41" s="985" t="n"/>
-      <c r="L41" s="985" t="n"/>
-      <c r="M41" s="983" t="n"/>
-      <c r="N41" s="983" t="n"/>
-      <c r="O41" s="983" t="n">
+      <c r="J41" s="1101" t="n"/>
+      <c r="K41" s="1101" t="n"/>
+      <c r="L41" s="1101" t="n"/>
+      <c r="M41" s="1099" t="n"/>
+      <c r="N41" s="1099" t="n"/>
+      <c r="O41" s="1099" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="986" t="n">
+      <c r="P41" s="1102" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="983" t="n"/>
-      <c r="R41" s="983" t="n">
+      <c r="Q41" s="1099" t="n"/>
+      <c r="R41" s="1099" t="n">
         <v>81</v>
       </c>
       <c r="S41" s="813" t="inlineStr">
@@ -5818,7 +6166,7 @@
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="T41" s="982" t="inlineStr">
+      <c r="T41" s="1098" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -5830,51 +6178,204 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="993" t="inlineStr">
+      <c r="A42" s="1109" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="994" t="inlineStr">
+      <c r="B42" s="1110" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="994" t="inlineStr">
+      <c r="C42" s="1110" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="995" t="n"/>
-      <c r="E42" s="995" t="n"/>
-      <c r="F42" s="995" t="n"/>
-      <c r="G42" s="995" t="n"/>
-      <c r="H42" s="995" t="n">
+      <c r="D42" s="1111" t="n"/>
+      <c r="E42" s="1111" t="n"/>
+      <c r="F42" s="1111" t="n"/>
+      <c r="G42" s="1111" t="n"/>
+      <c r="H42" s="1111" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="996" t="n"/>
-      <c r="J42" s="997" t="n"/>
-      <c r="K42" s="997" t="n"/>
-      <c r="L42" s="997" t="n"/>
-      <c r="M42" s="995" t="n">
+      <c r="I42" s="1112" t="n"/>
+      <c r="J42" s="1113" t="n"/>
+      <c r="K42" s="1113" t="n"/>
+      <c r="L42" s="1113" t="n"/>
+      <c r="M42" s="1111" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="995" t="n">
+      <c r="N42" s="1111" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="995" t="n"/>
-      <c r="P42" s="998" t="n"/>
-      <c r="Q42" s="995" t="n"/>
-      <c r="R42" s="995" t="n"/>
+      <c r="O42" s="1111" t="n"/>
+      <c r="P42" s="1114" t="n"/>
+      <c r="Q42" s="1111" t="n"/>
+      <c r="R42" s="1111" t="n"/>
       <c r="S42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="T42" s="994" t="n"/>
+      <c r="T42" s="1110" t="n"/>
       <c r="U42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="1085" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B43" s="1086" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="C43" s="1086" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="D43" s="1087" t="n"/>
+      <c r="E43" s="1087" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="F43" s="1087" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="1087" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="H43" s="1087" t="n"/>
+      <c r="I43" s="1088" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="J43" s="1089" t="n"/>
+      <c r="K43" s="1089" t="n"/>
+      <c r="L43" s="1089" t="n"/>
+      <c r="M43" s="1087" t="n"/>
+      <c r="N43" s="1087" t="n"/>
+      <c r="O43" s="1087" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="P43" s="1090" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="1087" t="n"/>
+      <c r="R43" s="1087" t="n">
+        <v>83</v>
+      </c>
+      <c r="S43" s="624" t="inlineStr">
+        <is>
+          <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
+        </is>
+      </c>
+      <c r="T43" s="1086" t="n"/>
+      <c r="U43" s="625" t="inlineStr">
+        <is>
+          <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="1115" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B44" s="1116" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="C44" s="1116" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="D44" s="1117" t="n"/>
+      <c r="E44" s="1117" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="F44" s="1117" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G44" s="1117" t="n"/>
+      <c r="H44" s="1117" t="n"/>
+      <c r="I44" s="1118" t="n"/>
+      <c r="J44" s="1119" t="n"/>
+      <c r="K44" s="1119" t="n"/>
+      <c r="L44" s="1119" t="n"/>
+      <c r="M44" s="1117" t="n"/>
+      <c r="N44" s="1117" t="n"/>
+      <c r="O44" s="1117" t="n"/>
+      <c r="P44" s="1120" t="n"/>
+      <c r="Q44" s="1117" t="n"/>
+      <c r="R44" s="1117" t="n"/>
+      <c r="S44" s="659" t="n"/>
+      <c r="T44" s="1116" t="inlineStr">
+        <is>
+          <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
+        </is>
+      </c>
+      <c r="U44" s="660" t="inlineStr">
+        <is>
+          <t>Evening recheck before dosing, requested for peace-of-mind after noon's unexpectedly high FC (17.2) and the R-0870 dosing question. Decline from noon (17.2 -&gt; 15.4 over ~7.25h, pool shaded after ~6:30PM) tracks a plausible hot/sunny-day afternoon loss -- consistent with noon reading being real, not a fluke. CC ticked up slightly (0.0 -&gt; 0.4), normal for end of a hot/high-use day, still low. FC loss/Pred error left blank on this row -- not a comparable 24h noon-to-noon measurement, would corrupt the loss-rate tracking if filled in via the standard formula. PHOTOS(4): wide pool shots both look clear/healthy, clean blue, no algae; zoomed liner-corner close-up shows normal blue speckled texture, no clear rust/stain progression. New this entry: John mounted a graduated ruler to the skimmer faceplate to start tracking water level -- photo documents the ruler installation, no specific level reading called out yet (nothing invented here; will log a real number once John reports one).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="1091" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B45" s="1092" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="C45" s="1092" t="inlineStr">
+        <is>
+          <t>DOSE</t>
+        </is>
+      </c>
+      <c r="D45" s="1093" t="n"/>
+      <c r="E45" s="1093" t="n"/>
+      <c r="F45" s="1093" t="n"/>
+      <c r="G45" s="1093" t="n"/>
+      <c r="H45" s="1093" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="I45" s="1094" t="n"/>
+      <c r="J45" s="1095" t="n"/>
+      <c r="K45" s="1095" t="n"/>
+      <c r="L45" s="1095" t="n"/>
+      <c r="M45" s="1093" t="n">
+        <v>1</v>
+      </c>
+      <c r="N45" s="1093" t="n">
+        <v>19</v>
+      </c>
+      <c r="O45" s="1093" t="n"/>
+      <c r="P45" s="1096" t="n"/>
+      <c r="Q45" s="1093" t="n"/>
+      <c r="R45" s="1093" t="n"/>
+      <c r="S45" s="631" t="inlineStr">
+        <is>
+          <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
+        </is>
+      </c>
+      <c r="T45" s="1092" t="n"/>
+      <c r="U45" s="632" t="inlineStr">
+        <is>
+          <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Water level (cm) column (col 19); log first reading 11.9 cm
John mounted a graduated ruler on the skimmer to track water level.
Inserts a new column after Water temp -- placed at 19 so the SEASON
TOTALS SUM formulas (cols 13/16/17 = M/P/Q) and merged A2:D2 are
untouched. Threads through append_log COLS, format_log widths/formats,
and build_site (log table + data.json). No dashboard chart yet -- will
add one once there are a few readings, like pH/TA/CYA. Baseline 11.9 cm
logged on the 7/2 evening TEST row.
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1121">
+  <cellXfs count="1157">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -3675,6 +3675,114 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -4151,7 +4259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U45"/>
+  <dimension ref="A1:V45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -4172,9 +4280,10 @@
     <col width="8" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="11" customWidth="1" min="18" max="18"/>
-    <col width="38" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="83.86" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="38" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="83.86" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -4270,15 +4379,20 @@
       </c>
       <c r="S1" s="790" t="inlineStr">
         <is>
+          <t>Water level (cm)</t>
+        </is>
+      </c>
+      <c r="T1" s="790" t="inlineStr">
+        <is>
           <t>Weather</t>
         </is>
       </c>
-      <c r="T1" s="790" t="inlineStr">
+      <c r="U1" s="790" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
       </c>
-      <c r="U1" s="791" t="inlineStr">
+      <c r="V1" s="791" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -4316,2064 +4430,2110 @@
         <v/>
       </c>
       <c r="R2" s="836" t="n"/>
-      <c r="S2" s="835" t="n"/>
+      <c r="S2" s="836" t="n"/>
       <c r="T2" s="835" t="n"/>
-      <c r="U2" s="839" t="n"/>
+      <c r="U2" s="835" t="n"/>
+      <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1085" t="inlineStr">
+      <c r="A3" s="1121" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1086" t="n"/>
-      <c r="C3" s="1086" t="inlineStr">
+      <c r="B3" s="1122" t="n"/>
+      <c r="C3" s="1122" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1087" t="n"/>
-      <c r="E3" s="1087" t="n"/>
-      <c r="F3" s="1087" t="n"/>
-      <c r="G3" s="1087" t="n"/>
-      <c r="H3" s="1087" t="n"/>
-      <c r="I3" s="1088" t="n"/>
-      <c r="J3" s="1089" t="n"/>
-      <c r="K3" s="1089" t="n"/>
-      <c r="L3" s="1089" t="n"/>
-      <c r="M3" s="1087" t="n"/>
-      <c r="N3" s="1087" t="n"/>
-      <c r="O3" s="1087" t="n"/>
-      <c r="P3" s="1090" t="n"/>
-      <c r="Q3" s="1087" t="n"/>
-      <c r="R3" s="1087" t="n"/>
-      <c r="S3" s="624" t="n"/>
-      <c r="T3" s="1086" t="n"/>
-      <c r="U3" s="625" t="inlineStr">
+      <c r="D3" s="1123" t="n"/>
+      <c r="E3" s="1123" t="n"/>
+      <c r="F3" s="1123" t="n"/>
+      <c r="G3" s="1123" t="n"/>
+      <c r="H3" s="1123" t="n"/>
+      <c r="I3" s="1124" t="n"/>
+      <c r="J3" s="1125" t="n"/>
+      <c r="K3" s="1125" t="n"/>
+      <c r="L3" s="1125" t="n"/>
+      <c r="M3" s="1123" t="n"/>
+      <c r="N3" s="1123" t="n"/>
+      <c r="O3" s="1123" t="n"/>
+      <c r="P3" s="1126" t="n"/>
+      <c r="Q3" s="1123" t="n"/>
+      <c r="R3" s="1123" t="n"/>
+      <c r="S3" s="1123" t="n"/>
+      <c r="T3" s="624" t="n"/>
+      <c r="U3" s="1122" t="n"/>
+      <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1091" t="inlineStr">
+      <c r="A4" s="1127" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1092" t="inlineStr">
+      <c r="B4" s="1128" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1092" t="inlineStr">
+      <c r="C4" s="1128" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1093" t="n"/>
-      <c r="E4" s="1093" t="n"/>
-      <c r="F4" s="1093" t="n"/>
-      <c r="G4" s="1093" t="n"/>
-      <c r="H4" s="1093" t="n"/>
-      <c r="I4" s="1094" t="n"/>
-      <c r="J4" s="1095" t="n"/>
-      <c r="K4" s="1095" t="n"/>
-      <c r="L4" s="1095" t="n"/>
-      <c r="M4" s="1093" t="n">
+      <c r="D4" s="1129" t="n"/>
+      <c r="E4" s="1129" t="n"/>
+      <c r="F4" s="1129" t="n"/>
+      <c r="G4" s="1129" t="n"/>
+      <c r="H4" s="1129" t="n"/>
+      <c r="I4" s="1130" t="n"/>
+      <c r="J4" s="1131" t="n"/>
+      <c r="K4" s="1131" t="n"/>
+      <c r="L4" s="1131" t="n"/>
+      <c r="M4" s="1129" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1093" t="n">
+      <c r="N4" s="1129" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1093" t="n"/>
-      <c r="P4" s="1096" t="n"/>
-      <c r="Q4" s="1093" t="n"/>
-      <c r="R4" s="1093" t="n"/>
-      <c r="S4" s="631" t="n"/>
-      <c r="T4" s="1092" t="n"/>
-      <c r="U4" s="632" t="inlineStr">
+      <c r="O4" s="1129" t="n"/>
+      <c r="P4" s="1132" t="n"/>
+      <c r="Q4" s="1129" t="n"/>
+      <c r="R4" s="1129" t="n"/>
+      <c r="S4" s="1129" t="n"/>
+      <c r="T4" s="631" t="n"/>
+      <c r="U4" s="1128" t="n"/>
+      <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1097" t="inlineStr">
+      <c r="A5" s="1133" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1098" t="inlineStr">
+      <c r="B5" s="1134" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1098" t="inlineStr">
+      <c r="C5" s="1134" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1099" t="n">
+      <c r="D5" s="1135" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1099" t="n">
+      <c r="E5" s="1135" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1099" t="n">
+      <c r="F5" s="1135" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1099" t="n"/>
-      <c r="H5" s="1099" t="n"/>
-      <c r="I5" s="1100" t="n"/>
-      <c r="J5" s="1101" t="n">
+      <c r="G5" s="1135" t="n"/>
+      <c r="H5" s="1135" t="n"/>
+      <c r="I5" s="1136" t="n"/>
+      <c r="J5" s="1137" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1101" t="n">
+      <c r="K5" s="1137" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1101" t="inlineStr">
+      <c r="L5" s="1137" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1099" t="n"/>
-      <c r="N5" s="1099" t="n"/>
-      <c r="O5" s="1099" t="n">
+      <c r="M5" s="1135" t="n"/>
+      <c r="N5" s="1135" t="n"/>
+      <c r="O5" s="1135" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1102" t="n">
+      <c r="P5" s="1138" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1099" t="n"/>
-      <c r="R5" s="1099" t="n"/>
-      <c r="S5" s="813" t="n"/>
-      <c r="T5" s="1098" t="n"/>
-      <c r="U5" s="814" t="inlineStr">
+      <c r="Q5" s="1135" t="n"/>
+      <c r="R5" s="1135" t="n"/>
+      <c r="S5" s="1135" t="n"/>
+      <c r="T5" s="813" t="n"/>
+      <c r="U5" s="1134" t="n"/>
+      <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1103" t="inlineStr">
+      <c r="A6" s="1139" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1104" t="inlineStr">
+      <c r="B6" s="1140" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1104" t="inlineStr">
+      <c r="C6" s="1140" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1105" t="n"/>
-      <c r="E6" s="1105" t="n"/>
-      <c r="F6" s="1105" t="n"/>
-      <c r="G6" s="1105" t="n"/>
-      <c r="H6" s="1105" t="n"/>
-      <c r="I6" s="1106" t="n"/>
-      <c r="J6" s="1107" t="n"/>
-      <c r="K6" s="1107" t="n"/>
-      <c r="L6" s="1107" t="n"/>
-      <c r="M6" s="1105" t="n">
+      <c r="D6" s="1141" t="n"/>
+      <c r="E6" s="1141" t="n"/>
+      <c r="F6" s="1141" t="n"/>
+      <c r="G6" s="1141" t="n"/>
+      <c r="H6" s="1141" t="n"/>
+      <c r="I6" s="1142" t="n"/>
+      <c r="J6" s="1143" t="n"/>
+      <c r="K6" s="1143" t="n"/>
+      <c r="L6" s="1143" t="n"/>
+      <c r="M6" s="1141" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1105" t="n">
+      <c r="N6" s="1141" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1105" t="n"/>
-      <c r="P6" s="1108" t="n"/>
-      <c r="Q6" s="1105" t="n"/>
-      <c r="R6" s="1105" t="n"/>
-      <c r="S6" s="820" t="n"/>
-      <c r="T6" s="1104" t="n"/>
-      <c r="U6" s="821" t="inlineStr">
+      <c r="O6" s="1141" t="n"/>
+      <c r="P6" s="1144" t="n"/>
+      <c r="Q6" s="1141" t="n"/>
+      <c r="R6" s="1141" t="n"/>
+      <c r="S6" s="1141" t="n"/>
+      <c r="T6" s="820" t="n"/>
+      <c r="U6" s="1140" t="n"/>
+      <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1109" t="inlineStr">
+      <c r="A7" s="1145" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1110" t="inlineStr">
+      <c r="B7" s="1146" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1110" t="inlineStr">
+      <c r="C7" s="1146" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1111" t="n"/>
-      <c r="E7" s="1111" t="n"/>
-      <c r="F7" s="1111" t="n"/>
-      <c r="G7" s="1111" t="n"/>
-      <c r="H7" s="1111" t="n"/>
-      <c r="I7" s="1112" t="n"/>
-      <c r="J7" s="1113" t="n"/>
-      <c r="K7" s="1113" t="n"/>
-      <c r="L7" s="1113" t="n"/>
-      <c r="M7" s="1111" t="n"/>
-      <c r="N7" s="1111" t="n"/>
-      <c r="O7" s="1111" t="n"/>
-      <c r="P7" s="1114" t="n"/>
-      <c r="Q7" s="1111" t="n"/>
-      <c r="R7" s="1111" t="n"/>
-      <c r="S7" s="827" t="n"/>
-      <c r="T7" s="1110" t="n"/>
-      <c r="U7" s="828" t="inlineStr">
+      <c r="D7" s="1147" t="n"/>
+      <c r="E7" s="1147" t="n"/>
+      <c r="F7" s="1147" t="n"/>
+      <c r="G7" s="1147" t="n"/>
+      <c r="H7" s="1147" t="n"/>
+      <c r="I7" s="1148" t="n"/>
+      <c r="J7" s="1149" t="n"/>
+      <c r="K7" s="1149" t="n"/>
+      <c r="L7" s="1149" t="n"/>
+      <c r="M7" s="1147" t="n"/>
+      <c r="N7" s="1147" t="n"/>
+      <c r="O7" s="1147" t="n"/>
+      <c r="P7" s="1150" t="n"/>
+      <c r="Q7" s="1147" t="n"/>
+      <c r="R7" s="1147" t="n"/>
+      <c r="S7" s="1147" t="n"/>
+      <c r="T7" s="827" t="n"/>
+      <c r="U7" s="1146" t="n"/>
+      <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
         </is>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1085" t="inlineStr">
+      <c r="A8" s="1121" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1086" t="inlineStr">
+      <c r="B8" s="1122" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1086" t="inlineStr">
+      <c r="C8" s="1122" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1087" t="n"/>
-      <c r="E8" s="1087" t="n"/>
-      <c r="F8" s="1087" t="n"/>
-      <c r="G8" s="1087" t="n"/>
-      <c r="H8" s="1087" t="n"/>
-      <c r="I8" s="1088" t="n"/>
-      <c r="J8" s="1089" t="n"/>
-      <c r="K8" s="1089" t="n"/>
-      <c r="L8" s="1089" t="n"/>
-      <c r="M8" s="1087" t="n"/>
-      <c r="N8" s="1087" t="n"/>
-      <c r="O8" s="1087" t="n"/>
-      <c r="P8" s="1090" t="n"/>
-      <c r="Q8" s="1087" t="n"/>
-      <c r="R8" s="1087" t="n"/>
-      <c r="S8" s="624" t="n"/>
-      <c r="T8" s="1086" t="n"/>
-      <c r="U8" s="625" t="inlineStr">
+      <c r="D8" s="1123" t="n"/>
+      <c r="E8" s="1123" t="n"/>
+      <c r="F8" s="1123" t="n"/>
+      <c r="G8" s="1123" t="n"/>
+      <c r="H8" s="1123" t="n"/>
+      <c r="I8" s="1124" t="n"/>
+      <c r="J8" s="1125" t="n"/>
+      <c r="K8" s="1125" t="n"/>
+      <c r="L8" s="1125" t="n"/>
+      <c r="M8" s="1123" t="n"/>
+      <c r="N8" s="1123" t="n"/>
+      <c r="O8" s="1123" t="n"/>
+      <c r="P8" s="1126" t="n"/>
+      <c r="Q8" s="1123" t="n"/>
+      <c r="R8" s="1123" t="n"/>
+      <c r="S8" s="1123" t="n"/>
+      <c r="T8" s="624" t="n"/>
+      <c r="U8" s="1122" t="n"/>
+      <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1115" t="inlineStr">
+      <c r="A9" s="1151" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1116" t="inlineStr">
+      <c r="B9" s="1152" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1116" t="inlineStr">
+      <c r="C9" s="1152" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1117" t="n">
+      <c r="D9" s="1153" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1117" t="n">
+      <c r="E9" s="1153" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1117" t="n">
+      <c r="F9" s="1153" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1117" t="n">
+      <c r="G9" s="1153" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1117" t="n"/>
-      <c r="I9" s="1118" t="n"/>
-      <c r="J9" s="1119" t="n">
+      <c r="H9" s="1153" t="n"/>
+      <c r="I9" s="1154" t="n"/>
+      <c r="J9" s="1155" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1119" t="n">
+      <c r="K9" s="1155" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1119" t="inlineStr">
+      <c r="L9" s="1155" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1117" t="n"/>
-      <c r="N9" s="1117" t="n"/>
-      <c r="O9" s="1117" t="n">
+      <c r="M9" s="1153" t="n"/>
+      <c r="N9" s="1153" t="n"/>
+      <c r="O9" s="1153" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1120" t="n">
+      <c r="P9" s="1156" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1117" t="n"/>
-      <c r="R9" s="1117" t="n"/>
-      <c r="S9" s="659" t="inlineStr">
+      <c r="Q9" s="1153" t="n"/>
+      <c r="R9" s="1153" t="n"/>
+      <c r="S9" s="1153" t="n"/>
+      <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="T9" s="1116" t="n"/>
-      <c r="U9" s="660" t="inlineStr">
+      <c r="U9" s="1152" t="n"/>
+      <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1115" t="inlineStr">
+      <c r="A10" s="1151" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1116" t="inlineStr">
+      <c r="B10" s="1152" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1116" t="inlineStr">
+      <c r="C10" s="1152" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1117" t="n"/>
-      <c r="E10" s="1117" t="n"/>
-      <c r="F10" s="1117" t="n"/>
-      <c r="G10" s="1117" t="n"/>
-      <c r="H10" s="1117" t="n"/>
-      <c r="I10" s="1118" t="n"/>
-      <c r="J10" s="1119" t="n"/>
-      <c r="K10" s="1119" t="n"/>
-      <c r="L10" s="1119" t="inlineStr">
+      <c r="D10" s="1153" t="n"/>
+      <c r="E10" s="1153" t="n"/>
+      <c r="F10" s="1153" t="n"/>
+      <c r="G10" s="1153" t="n"/>
+      <c r="H10" s="1153" t="n"/>
+      <c r="I10" s="1154" t="n"/>
+      <c r="J10" s="1155" t="n"/>
+      <c r="K10" s="1155" t="n"/>
+      <c r="L10" s="1155" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1117" t="n"/>
-      <c r="N10" s="1117" t="n"/>
-      <c r="O10" s="1117" t="n"/>
-      <c r="P10" s="1120" t="n"/>
-      <c r="Q10" s="1117" t="n"/>
-      <c r="R10" s="1117" t="n"/>
-      <c r="S10" s="659" t="n"/>
-      <c r="T10" s="1116" t="n"/>
-      <c r="U10" s="660" t="inlineStr">
+      <c r="M10" s="1153" t="n"/>
+      <c r="N10" s="1153" t="n"/>
+      <c r="O10" s="1153" t="n"/>
+      <c r="P10" s="1156" t="n"/>
+      <c r="Q10" s="1153" t="n"/>
+      <c r="R10" s="1153" t="n"/>
+      <c r="S10" s="1153" t="n"/>
+      <c r="T10" s="659" t="n"/>
+      <c r="U10" s="1152" t="n"/>
+      <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1115" t="inlineStr">
+      <c r="A11" s="1151" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1116" t="inlineStr">
+      <c r="B11" s="1152" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1116" t="inlineStr">
+      <c r="C11" s="1152" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1117" t="n"/>
-      <c r="E11" s="1117" t="n"/>
-      <c r="F11" s="1117" t="n"/>
-      <c r="G11" s="1117" t="n"/>
-      <c r="H11" s="1117" t="n"/>
-      <c r="I11" s="1118" t="n"/>
-      <c r="J11" s="1119" t="n"/>
-      <c r="K11" s="1119" t="n"/>
-      <c r="L11" s="1119" t="n"/>
-      <c r="M11" s="1117" t="n">
+      <c r="D11" s="1153" t="n"/>
+      <c r="E11" s="1153" t="n"/>
+      <c r="F11" s="1153" t="n"/>
+      <c r="G11" s="1153" t="n"/>
+      <c r="H11" s="1153" t="n"/>
+      <c r="I11" s="1154" t="n"/>
+      <c r="J11" s="1155" t="n"/>
+      <c r="K11" s="1155" t="n"/>
+      <c r="L11" s="1155" t="n"/>
+      <c r="M11" s="1153" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1117" t="n">
+      <c r="N11" s="1153" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1117" t="n"/>
-      <c r="P11" s="1120" t="n"/>
-      <c r="Q11" s="1117" t="n"/>
-      <c r="R11" s="1117" t="n"/>
-      <c r="S11" s="659" t="n"/>
-      <c r="T11" s="1116" t="n"/>
-      <c r="U11" s="660" t="inlineStr">
+      <c r="O11" s="1153" t="n"/>
+      <c r="P11" s="1156" t="n"/>
+      <c r="Q11" s="1153" t="n"/>
+      <c r="R11" s="1153" t="n"/>
+      <c r="S11" s="1153" t="n"/>
+      <c r="T11" s="659" t="n"/>
+      <c r="U11" s="1152" t="n"/>
+      <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
         </is>
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1091" t="inlineStr">
+      <c r="A12" s="1127" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1092" t="inlineStr">
+      <c r="B12" s="1128" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1092" t="inlineStr">
+      <c r="C12" s="1128" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1093" t="n"/>
-      <c r="E12" s="1093" t="n"/>
-      <c r="F12" s="1093" t="n"/>
-      <c r="G12" s="1093" t="n"/>
-      <c r="H12" s="1093" t="n"/>
-      <c r="I12" s="1094" t="n"/>
-      <c r="J12" s="1095" t="n"/>
-      <c r="K12" s="1095" t="n"/>
-      <c r="L12" s="1095" t="n"/>
-      <c r="M12" s="1093" t="n"/>
-      <c r="N12" s="1093" t="n"/>
-      <c r="O12" s="1093" t="n"/>
-      <c r="P12" s="1096" t="n"/>
-      <c r="Q12" s="1093" t="n"/>
-      <c r="R12" s="1093" t="n"/>
-      <c r="S12" s="631" t="n"/>
-      <c r="T12" s="1092" t="n"/>
-      <c r="U12" s="632" t="inlineStr">
+      <c r="D12" s="1129" t="n"/>
+      <c r="E12" s="1129" t="n"/>
+      <c r="F12" s="1129" t="n"/>
+      <c r="G12" s="1129" t="n"/>
+      <c r="H12" s="1129" t="n"/>
+      <c r="I12" s="1130" t="n"/>
+      <c r="J12" s="1131" t="n"/>
+      <c r="K12" s="1131" t="n"/>
+      <c r="L12" s="1131" t="n"/>
+      <c r="M12" s="1129" t="n"/>
+      <c r="N12" s="1129" t="n"/>
+      <c r="O12" s="1129" t="n"/>
+      <c r="P12" s="1132" t="n"/>
+      <c r="Q12" s="1129" t="n"/>
+      <c r="R12" s="1129" t="n"/>
+      <c r="S12" s="1129" t="n"/>
+      <c r="T12" s="631" t="n"/>
+      <c r="U12" s="1128" t="n"/>
+      <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1097" t="inlineStr">
+      <c r="A13" s="1133" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1098" t="n"/>
-      <c r="C13" s="1098" t="inlineStr">
+      <c r="B13" s="1134" t="n"/>
+      <c r="C13" s="1134" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1099" t="n"/>
-      <c r="E13" s="1099" t="n"/>
-      <c r="F13" s="1099" t="n"/>
-      <c r="G13" s="1099" t="n"/>
-      <c r="H13" s="1099" t="n"/>
-      <c r="I13" s="1100" t="n"/>
-      <c r="J13" s="1101" t="n"/>
-      <c r="K13" s="1101" t="n"/>
-      <c r="L13" s="1101" t="n"/>
-      <c r="M13" s="1099" t="n"/>
-      <c r="N13" s="1099" t="n"/>
-      <c r="O13" s="1099" t="n"/>
-      <c r="P13" s="1102" t="n"/>
-      <c r="Q13" s="1099" t="n"/>
-      <c r="R13" s="1099" t="n"/>
-      <c r="S13" s="813" t="n"/>
-      <c r="T13" s="1098" t="n"/>
-      <c r="U13" s="814" t="inlineStr">
+      <c r="D13" s="1135" t="n"/>
+      <c r="E13" s="1135" t="n"/>
+      <c r="F13" s="1135" t="n"/>
+      <c r="G13" s="1135" t="n"/>
+      <c r="H13" s="1135" t="n"/>
+      <c r="I13" s="1136" t="n"/>
+      <c r="J13" s="1137" t="n"/>
+      <c r="K13" s="1137" t="n"/>
+      <c r="L13" s="1137" t="n"/>
+      <c r="M13" s="1135" t="n"/>
+      <c r="N13" s="1135" t="n"/>
+      <c r="O13" s="1135" t="n"/>
+      <c r="P13" s="1138" t="n"/>
+      <c r="Q13" s="1135" t="n"/>
+      <c r="R13" s="1135" t="n"/>
+      <c r="S13" s="1135" t="n"/>
+      <c r="T13" s="813" t="n"/>
+      <c r="U13" s="1134" t="n"/>
+      <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1103" t="inlineStr">
+      <c r="A14" s="1139" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1104" t="inlineStr">
+      <c r="B14" s="1140" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1104" t="inlineStr">
+      <c r="C14" s="1140" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1105" t="n"/>
-      <c r="E14" s="1105" t="n">
+      <c r="D14" s="1141" t="n"/>
+      <c r="E14" s="1141" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1105" t="n">
+      <c r="F14" s="1141" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1105" t="n">
+      <c r="G14" s="1141" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1105" t="n"/>
-      <c r="I14" s="1106" t="n"/>
-      <c r="J14" s="1107" t="n"/>
-      <c r="K14" s="1107" t="n"/>
-      <c r="L14" s="1107" t="n"/>
-      <c r="M14" s="1105" t="n"/>
-      <c r="N14" s="1105" t="n"/>
-      <c r="O14" s="1105" t="n">
+      <c r="H14" s="1141" t="n"/>
+      <c r="I14" s="1142" t="n"/>
+      <c r="J14" s="1143" t="n"/>
+      <c r="K14" s="1143" t="n"/>
+      <c r="L14" s="1143" t="n"/>
+      <c r="M14" s="1141" t="n"/>
+      <c r="N14" s="1141" t="n"/>
+      <c r="O14" s="1141" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1108" t="n">
+      <c r="P14" s="1144" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1105" t="n"/>
-      <c r="R14" s="1105" t="n"/>
-      <c r="S14" s="820" t="inlineStr">
+      <c r="Q14" s="1141" t="n"/>
+      <c r="R14" s="1141" t="n"/>
+      <c r="S14" s="1141" t="n"/>
+      <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="T14" s="1104" t="n"/>
-      <c r="U14" s="821" t="inlineStr">
+      <c r="U14" s="1140" t="n"/>
+      <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1103" t="inlineStr">
+      <c r="A15" s="1139" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1104" t="inlineStr">
+      <c r="B15" s="1140" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1104" t="inlineStr">
+      <c r="C15" s="1140" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1105" t="n"/>
-      <c r="E15" s="1105" t="n"/>
-      <c r="F15" s="1105" t="n"/>
-      <c r="G15" s="1105" t="n"/>
-      <c r="H15" s="1105" t="n"/>
-      <c r="I15" s="1106" t="n"/>
-      <c r="J15" s="1107" t="n"/>
-      <c r="K15" s="1107" t="n"/>
-      <c r="L15" s="1107" t="n"/>
-      <c r="M15" s="1105" t="n">
+      <c r="D15" s="1141" t="n"/>
+      <c r="E15" s="1141" t="n"/>
+      <c r="F15" s="1141" t="n"/>
+      <c r="G15" s="1141" t="n"/>
+      <c r="H15" s="1141" t="n"/>
+      <c r="I15" s="1142" t="n"/>
+      <c r="J15" s="1143" t="n"/>
+      <c r="K15" s="1143" t="n"/>
+      <c r="L15" s="1143" t="n"/>
+      <c r="M15" s="1141" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1105" t="n">
+      <c r="N15" s="1141" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1105" t="n"/>
-      <c r="P15" s="1108" t="n"/>
-      <c r="Q15" s="1105" t="n"/>
-      <c r="R15" s="1105" t="n"/>
-      <c r="S15" s="820" t="n"/>
-      <c r="T15" s="1104" t="n"/>
-      <c r="U15" s="821" t="inlineStr">
+      <c r="O15" s="1141" t="n"/>
+      <c r="P15" s="1144" t="n"/>
+      <c r="Q15" s="1141" t="n"/>
+      <c r="R15" s="1141" t="n"/>
+      <c r="S15" s="1141" t="n"/>
+      <c r="T15" s="820" t="n"/>
+      <c r="U15" s="1140" t="n"/>
+      <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1109" t="inlineStr">
+      <c r="A16" s="1145" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1110" t="inlineStr">
+      <c r="B16" s="1146" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1110" t="inlineStr">
+      <c r="C16" s="1146" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1111" t="n"/>
-      <c r="E16" s="1111" t="n"/>
-      <c r="F16" s="1111" t="n"/>
-      <c r="G16" s="1111" t="n"/>
-      <c r="H16" s="1111" t="n"/>
-      <c r="I16" s="1112" t="n"/>
-      <c r="J16" s="1113" t="n"/>
-      <c r="K16" s="1113" t="n"/>
-      <c r="L16" s="1113" t="n"/>
-      <c r="M16" s="1111" t="n"/>
-      <c r="N16" s="1111" t="n"/>
-      <c r="O16" s="1111" t="n"/>
-      <c r="P16" s="1114" t="n"/>
-      <c r="Q16" s="1111" t="n"/>
-      <c r="R16" s="1111" t="n"/>
-      <c r="S16" s="827" t="n"/>
-      <c r="T16" s="1110" t="n"/>
-      <c r="U16" s="828" t="inlineStr">
+      <c r="D16" s="1147" t="n"/>
+      <c r="E16" s="1147" t="n"/>
+      <c r="F16" s="1147" t="n"/>
+      <c r="G16" s="1147" t="n"/>
+      <c r="H16" s="1147" t="n"/>
+      <c r="I16" s="1148" t="n"/>
+      <c r="J16" s="1149" t="n"/>
+      <c r="K16" s="1149" t="n"/>
+      <c r="L16" s="1149" t="n"/>
+      <c r="M16" s="1147" t="n"/>
+      <c r="N16" s="1147" t="n"/>
+      <c r="O16" s="1147" t="n"/>
+      <c r="P16" s="1150" t="n"/>
+      <c r="Q16" s="1147" t="n"/>
+      <c r="R16" s="1147" t="n"/>
+      <c r="S16" s="1147" t="n"/>
+      <c r="T16" s="827" t="n"/>
+      <c r="U16" s="1146" t="n"/>
+      <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1085" t="inlineStr">
+      <c r="A17" s="1121" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1086" t="inlineStr">
+      <c r="B17" s="1122" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1086" t="inlineStr">
+      <c r="C17" s="1122" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1087" t="n"/>
-      <c r="E17" s="1087" t="n"/>
-      <c r="F17" s="1087" t="n"/>
-      <c r="G17" s="1087" t="n"/>
-      <c r="H17" s="1087" t="n"/>
-      <c r="I17" s="1088" t="n"/>
-      <c r="J17" s="1089" t="n"/>
-      <c r="K17" s="1089" t="n"/>
-      <c r="L17" s="1089" t="n"/>
-      <c r="M17" s="1087" t="n"/>
-      <c r="N17" s="1087" t="n"/>
-      <c r="O17" s="1087" t="n"/>
-      <c r="P17" s="1090" t="n"/>
-      <c r="Q17" s="1087" t="n"/>
-      <c r="R17" s="1087" t="n"/>
-      <c r="S17" s="624" t="n"/>
-      <c r="T17" s="1086" t="n"/>
-      <c r="U17" s="625" t="inlineStr">
+      <c r="D17" s="1123" t="n"/>
+      <c r="E17" s="1123" t="n"/>
+      <c r="F17" s="1123" t="n"/>
+      <c r="G17" s="1123" t="n"/>
+      <c r="H17" s="1123" t="n"/>
+      <c r="I17" s="1124" t="n"/>
+      <c r="J17" s="1125" t="n"/>
+      <c r="K17" s="1125" t="n"/>
+      <c r="L17" s="1125" t="n"/>
+      <c r="M17" s="1123" t="n"/>
+      <c r="N17" s="1123" t="n"/>
+      <c r="O17" s="1123" t="n"/>
+      <c r="P17" s="1126" t="n"/>
+      <c r="Q17" s="1123" t="n"/>
+      <c r="R17" s="1123" t="n"/>
+      <c r="S17" s="1123" t="n"/>
+      <c r="T17" s="624" t="n"/>
+      <c r="U17" s="1122" t="n"/>
+      <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1115" t="inlineStr">
+      <c r="A18" s="1151" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1116" t="inlineStr">
+      <c r="B18" s="1152" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1116" t="inlineStr">
+      <c r="C18" s="1152" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1117" t="n"/>
-      <c r="E18" s="1117" t="n">
+      <c r="D18" s="1153" t="n"/>
+      <c r="E18" s="1153" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1117" t="n">
+      <c r="F18" s="1153" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1117" t="n">
+      <c r="G18" s="1153" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1117" t="n"/>
-      <c r="I18" s="1118" t="n"/>
-      <c r="J18" s="1119" t="n"/>
-      <c r="K18" s="1119" t="n"/>
-      <c r="L18" s="1119" t="n"/>
-      <c r="M18" s="1117" t="n"/>
-      <c r="N18" s="1117" t="n"/>
-      <c r="O18" s="1117" t="n">
+      <c r="H18" s="1153" t="n"/>
+      <c r="I18" s="1154" t="n"/>
+      <c r="J18" s="1155" t="n"/>
+      <c r="K18" s="1155" t="n"/>
+      <c r="L18" s="1155" t="n"/>
+      <c r="M18" s="1153" t="n"/>
+      <c r="N18" s="1153" t="n"/>
+      <c r="O18" s="1153" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1120" t="n">
+      <c r="P18" s="1156" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1117" t="n"/>
-      <c r="R18" s="1117" t="n"/>
-      <c r="S18" s="659" t="inlineStr">
+      <c r="Q18" s="1153" t="n"/>
+      <c r="R18" s="1153" t="n"/>
+      <c r="S18" s="1153" t="n"/>
+      <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="T18" s="1116" t="n"/>
-      <c r="U18" s="660" t="inlineStr">
+      <c r="U18" s="1152" t="n"/>
+      <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1115" t="inlineStr">
+      <c r="A19" s="1151" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1116" t="inlineStr">
+      <c r="B19" s="1152" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1116" t="inlineStr">
+      <c r="C19" s="1152" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1117" t="n"/>
-      <c r="E19" s="1117" t="n"/>
-      <c r="F19" s="1117" t="n"/>
-      <c r="G19" s="1117" t="n"/>
-      <c r="H19" s="1117" t="n"/>
-      <c r="I19" s="1118" t="n"/>
-      <c r="J19" s="1119" t="n"/>
-      <c r="K19" s="1119" t="n"/>
-      <c r="L19" s="1119" t="n"/>
-      <c r="M19" s="1117" t="n">
+      <c r="D19" s="1153" t="n"/>
+      <c r="E19" s="1153" t="n"/>
+      <c r="F19" s="1153" t="n"/>
+      <c r="G19" s="1153" t="n"/>
+      <c r="H19" s="1153" t="n"/>
+      <c r="I19" s="1154" t="n"/>
+      <c r="J19" s="1155" t="n"/>
+      <c r="K19" s="1155" t="n"/>
+      <c r="L19" s="1155" t="n"/>
+      <c r="M19" s="1153" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1117" t="n">
+      <c r="N19" s="1153" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1117" t="n"/>
-      <c r="P19" s="1120" t="n"/>
-      <c r="Q19" s="1117" t="n"/>
-      <c r="R19" s="1117" t="n"/>
-      <c r="S19" s="659" t="inlineStr">
+      <c r="O19" s="1153" t="n"/>
+      <c r="P19" s="1156" t="n"/>
+      <c r="Q19" s="1153" t="n"/>
+      <c r="R19" s="1153" t="n"/>
+      <c r="S19" s="1153" t="n"/>
+      <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="T19" s="1116" t="n"/>
-      <c r="U19" s="660" t="inlineStr">
+      <c r="U19" s="1152" t="n"/>
+      <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1115" t="inlineStr">
+      <c r="A20" s="1151" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1116" t="inlineStr">
+      <c r="B20" s="1152" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1116" t="inlineStr">
+      <c r="C20" s="1152" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1117" t="n"/>
-      <c r="E20" s="1117" t="n"/>
-      <c r="F20" s="1117" t="n"/>
-      <c r="G20" s="1117" t="n"/>
-      <c r="H20" s="1117" t="n"/>
-      <c r="I20" s="1118" t="n"/>
-      <c r="J20" s="1119" t="n"/>
-      <c r="K20" s="1119" t="n"/>
-      <c r="L20" s="1119" t="n"/>
-      <c r="M20" s="1117" t="n"/>
-      <c r="N20" s="1117" t="n"/>
-      <c r="O20" s="1117" t="n"/>
-      <c r="P20" s="1120" t="n"/>
-      <c r="Q20" s="1117" t="n"/>
-      <c r="R20" s="1117" t="n"/>
-      <c r="S20" s="659" t="inlineStr">
+      <c r="D20" s="1153" t="n"/>
+      <c r="E20" s="1153" t="n"/>
+      <c r="F20" s="1153" t="n"/>
+      <c r="G20" s="1153" t="n"/>
+      <c r="H20" s="1153" t="n"/>
+      <c r="I20" s="1154" t="n"/>
+      <c r="J20" s="1155" t="n"/>
+      <c r="K20" s="1155" t="n"/>
+      <c r="L20" s="1155" t="n"/>
+      <c r="M20" s="1153" t="n"/>
+      <c r="N20" s="1153" t="n"/>
+      <c r="O20" s="1153" t="n"/>
+      <c r="P20" s="1156" t="n"/>
+      <c r="Q20" s="1153" t="n"/>
+      <c r="R20" s="1153" t="n"/>
+      <c r="S20" s="1153" t="n"/>
+      <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="T20" s="1116" t="n"/>
-      <c r="U20" s="660" t="inlineStr">
+      <c r="U20" s="1152" t="n"/>
+      <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1091" t="inlineStr">
+      <c r="A21" s="1127" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1092" t="inlineStr">
+      <c r="B21" s="1128" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1092" t="inlineStr">
+      <c r="C21" s="1128" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1093" t="n"/>
-      <c r="E21" s="1093" t="n"/>
-      <c r="F21" s="1093" t="n"/>
-      <c r="G21" s="1093" t="n"/>
-      <c r="H21" s="1093" t="n"/>
-      <c r="I21" s="1094" t="n"/>
-      <c r="J21" s="1095" t="n"/>
-      <c r="K21" s="1095" t="n"/>
-      <c r="L21" s="1095" t="n"/>
-      <c r="M21" s="1093" t="n"/>
-      <c r="N21" s="1093" t="n"/>
-      <c r="O21" s="1093" t="n"/>
-      <c r="P21" s="1096" t="n"/>
-      <c r="Q21" s="1093" t="n"/>
-      <c r="R21" s="1093" t="n"/>
-      <c r="S21" s="631" t="n"/>
-      <c r="T21" s="1092" t="n"/>
-      <c r="U21" s="632" t="inlineStr">
+      <c r="D21" s="1129" t="n"/>
+      <c r="E21" s="1129" t="n"/>
+      <c r="F21" s="1129" t="n"/>
+      <c r="G21" s="1129" t="n"/>
+      <c r="H21" s="1129" t="n"/>
+      <c r="I21" s="1130" t="n"/>
+      <c r="J21" s="1131" t="n"/>
+      <c r="K21" s="1131" t="n"/>
+      <c r="L21" s="1131" t="n"/>
+      <c r="M21" s="1129" t="n"/>
+      <c r="N21" s="1129" t="n"/>
+      <c r="O21" s="1129" t="n"/>
+      <c r="P21" s="1132" t="n"/>
+      <c r="Q21" s="1129" t="n"/>
+      <c r="R21" s="1129" t="n"/>
+      <c r="S21" s="1129" t="n"/>
+      <c r="T21" s="631" t="n"/>
+      <c r="U21" s="1128" t="n"/>
+      <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
         </is>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1097" t="inlineStr">
+      <c r="A22" s="1133" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1098" t="inlineStr">
+      <c r="B22" s="1134" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1098" t="inlineStr">
+      <c r="C22" s="1134" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1099" t="n"/>
-      <c r="E22" s="1099" t="n"/>
-      <c r="F22" s="1099" t="n"/>
-      <c r="G22" s="1099" t="n"/>
-      <c r="H22" s="1099" t="n"/>
-      <c r="I22" s="1100" t="n"/>
-      <c r="J22" s="1101" t="n"/>
-      <c r="K22" s="1101" t="n"/>
-      <c r="L22" s="1101" t="n"/>
-      <c r="M22" s="1099" t="n"/>
-      <c r="N22" s="1099" t="n"/>
-      <c r="O22" s="1099" t="n"/>
-      <c r="P22" s="1102" t="n"/>
-      <c r="Q22" s="1099" t="n"/>
-      <c r="R22" s="1099" t="n"/>
-      <c r="S22" s="813" t="n"/>
-      <c r="T22" s="1098" t="n"/>
-      <c r="U22" s="814" t="inlineStr">
+      <c r="D22" s="1135" t="n"/>
+      <c r="E22" s="1135" t="n"/>
+      <c r="F22" s="1135" t="n"/>
+      <c r="G22" s="1135" t="n"/>
+      <c r="H22" s="1135" t="n"/>
+      <c r="I22" s="1136" t="n"/>
+      <c r="J22" s="1137" t="n"/>
+      <c r="K22" s="1137" t="n"/>
+      <c r="L22" s="1137" t="n"/>
+      <c r="M22" s="1135" t="n"/>
+      <c r="N22" s="1135" t="n"/>
+      <c r="O22" s="1135" t="n"/>
+      <c r="P22" s="1138" t="n"/>
+      <c r="Q22" s="1135" t="n"/>
+      <c r="R22" s="1135" t="n"/>
+      <c r="S22" s="1135" t="n"/>
+      <c r="T22" s="813" t="n"/>
+      <c r="U22" s="1134" t="n"/>
+      <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1103" t="inlineStr">
+      <c r="A23" s="1139" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1104" t="inlineStr">
+      <c r="B23" s="1140" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1104" t="inlineStr">
+      <c r="C23" s="1140" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1105" t="n"/>
-      <c r="E23" s="1105" t="n">
+      <c r="D23" s="1141" t="n"/>
+      <c r="E23" s="1141" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1105" t="n">
+      <c r="F23" s="1141" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1105" t="n">
+      <c r="G23" s="1141" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1105" t="n"/>
-      <c r="I23" s="1106" t="n"/>
-      <c r="J23" s="1107" t="n"/>
-      <c r="K23" s="1107" t="n"/>
-      <c r="L23" s="1107" t="n"/>
-      <c r="M23" s="1105" t="n"/>
-      <c r="N23" s="1105" t="n"/>
-      <c r="O23" s="1105" t="n">
+      <c r="H23" s="1141" t="n"/>
+      <c r="I23" s="1142" t="n"/>
+      <c r="J23" s="1143" t="n"/>
+      <c r="K23" s="1143" t="n"/>
+      <c r="L23" s="1143" t="n"/>
+      <c r="M23" s="1141" t="n"/>
+      <c r="N23" s="1141" t="n"/>
+      <c r="O23" s="1141" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1108" t="n">
+      <c r="P23" s="1144" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1105" t="n"/>
-      <c r="R23" s="1105" t="n"/>
-      <c r="S23" s="820" t="inlineStr">
+      <c r="Q23" s="1141" t="n"/>
+      <c r="R23" s="1141" t="n"/>
+      <c r="S23" s="1141" t="n"/>
+      <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="T23" s="1104" t="n"/>
-      <c r="U23" s="821" t="inlineStr">
+      <c r="U23" s="1140" t="n"/>
+      <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1109" t="inlineStr">
+      <c r="A24" s="1145" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1110" t="inlineStr">
+      <c r="B24" s="1146" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1110" t="inlineStr">
+      <c r="C24" s="1146" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1111" t="n"/>
-      <c r="E24" s="1111" t="n"/>
-      <c r="F24" s="1111" t="n"/>
-      <c r="G24" s="1111" t="n"/>
-      <c r="H24" s="1111" t="n"/>
-      <c r="I24" s="1112" t="n"/>
-      <c r="J24" s="1113" t="n"/>
-      <c r="K24" s="1113" t="n"/>
-      <c r="L24" s="1113" t="n"/>
-      <c r="M24" s="1111" t="n">
+      <c r="D24" s="1147" t="n"/>
+      <c r="E24" s="1147" t="n"/>
+      <c r="F24" s="1147" t="n"/>
+      <c r="G24" s="1147" t="n"/>
+      <c r="H24" s="1147" t="n"/>
+      <c r="I24" s="1148" t="n"/>
+      <c r="J24" s="1149" t="n"/>
+      <c r="K24" s="1149" t="n"/>
+      <c r="L24" s="1149" t="n"/>
+      <c r="M24" s="1147" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1111" t="n">
+      <c r="N24" s="1147" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1111" t="n"/>
-      <c r="P24" s="1114" t="n"/>
-      <c r="Q24" s="1111" t="n"/>
-      <c r="R24" s="1111" t="n"/>
-      <c r="S24" s="827" t="inlineStr">
+      <c r="O24" s="1147" t="n"/>
+      <c r="P24" s="1150" t="n"/>
+      <c r="Q24" s="1147" t="n"/>
+      <c r="R24" s="1147" t="n"/>
+      <c r="S24" s="1147" t="n"/>
+      <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="T24" s="1110" t="n"/>
-      <c r="U24" s="828" t="inlineStr">
+      <c r="U24" s="1146" t="n"/>
+      <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1085" t="inlineStr">
+      <c r="A25" s="1121" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1086" t="inlineStr">
+      <c r="B25" s="1122" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1086" t="inlineStr">
+      <c r="C25" s="1122" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1087" t="n">
+      <c r="D25" s="1123" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1087" t="n">
+      <c r="E25" s="1123" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1087" t="n">
+      <c r="F25" s="1123" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1087" t="n">
+      <c r="G25" s="1123" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1087" t="n"/>
-      <c r="I25" s="1088" t="n"/>
-      <c r="J25" s="1089" t="n">
+      <c r="H25" s="1123" t="n"/>
+      <c r="I25" s="1124" t="n"/>
+      <c r="J25" s="1125" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1089" t="n">
+      <c r="K25" s="1125" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1089" t="n">
+      <c r="L25" s="1125" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1087" t="n"/>
-      <c r="N25" s="1087" t="n"/>
-      <c r="O25" s="1087" t="n">
+      <c r="M25" s="1123" t="n"/>
+      <c r="N25" s="1123" t="n"/>
+      <c r="O25" s="1123" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1090" t="n">
+      <c r="P25" s="1126" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1087" t="n"/>
-      <c r="R25" s="1087" t="n"/>
-      <c r="S25" s="624" t="inlineStr">
+      <c r="Q25" s="1123" t="n"/>
+      <c r="R25" s="1123" t="n"/>
+      <c r="S25" s="1123" t="n"/>
+      <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="T25" s="1086" t="n"/>
-      <c r="U25" s="625" t="inlineStr">
+      <c r="U25" s="1122" t="n"/>
+      <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1091" t="inlineStr">
+      <c r="A26" s="1127" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1092" t="inlineStr">
+      <c r="B26" s="1128" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1092" t="inlineStr">
+      <c r="C26" s="1128" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1093" t="n"/>
-      <c r="E26" s="1093" t="n"/>
-      <c r="F26" s="1093" t="n"/>
-      <c r="G26" s="1093" t="n"/>
-      <c r="H26" s="1093" t="n"/>
-      <c r="I26" s="1094" t="n"/>
-      <c r="J26" s="1095" t="n"/>
-      <c r="K26" s="1095" t="n"/>
-      <c r="L26" s="1095" t="n"/>
-      <c r="M26" s="1093" t="n">
+      <c r="D26" s="1129" t="n"/>
+      <c r="E26" s="1129" t="n"/>
+      <c r="F26" s="1129" t="n"/>
+      <c r="G26" s="1129" t="n"/>
+      <c r="H26" s="1129" t="n"/>
+      <c r="I26" s="1130" t="n"/>
+      <c r="J26" s="1131" t="n"/>
+      <c r="K26" s="1131" t="n"/>
+      <c r="L26" s="1131" t="n"/>
+      <c r="M26" s="1129" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1093" t="n">
+      <c r="N26" s="1129" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1093" t="n"/>
-      <c r="P26" s="1096" t="n"/>
-      <c r="Q26" s="1093" t="n"/>
-      <c r="R26" s="1093" t="n"/>
-      <c r="S26" s="631" t="inlineStr">
+      <c r="O26" s="1129" t="n"/>
+      <c r="P26" s="1132" t="n"/>
+      <c r="Q26" s="1129" t="n"/>
+      <c r="R26" s="1129" t="n"/>
+      <c r="S26" s="1129" t="n"/>
+      <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="T26" s="1092" t="n"/>
-      <c r="U26" s="632" t="inlineStr">
+      <c r="U26" s="1128" t="n"/>
+      <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1097" t="inlineStr">
+      <c r="A27" s="1133" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1098" t="inlineStr">
+      <c r="B27" s="1134" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1098" t="inlineStr">
+      <c r="C27" s="1134" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1099" t="n"/>
-      <c r="E27" s="1099" t="n">
+      <c r="D27" s="1135" t="n"/>
+      <c r="E27" s="1135" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1099" t="n">
+      <c r="F27" s="1135" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1099" t="n">
+      <c r="G27" s="1135" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1099" t="n"/>
-      <c r="I27" s="1100" t="n"/>
-      <c r="J27" s="1101" t="n"/>
-      <c r="K27" s="1101" t="n"/>
-      <c r="L27" s="1101" t="n"/>
-      <c r="M27" s="1099" t="n"/>
-      <c r="N27" s="1099" t="n"/>
-      <c r="O27" s="1099" t="n">
+      <c r="H27" s="1135" t="n"/>
+      <c r="I27" s="1136" t="n"/>
+      <c r="J27" s="1137" t="n"/>
+      <c r="K27" s="1137" t="n"/>
+      <c r="L27" s="1137" t="n"/>
+      <c r="M27" s="1135" t="n"/>
+      <c r="N27" s="1135" t="n"/>
+      <c r="O27" s="1135" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1102" t="n">
+      <c r="P27" s="1138" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1099" t="n"/>
-      <c r="R27" s="1099" t="n"/>
-      <c r="S27" s="813" t="inlineStr">
+      <c r="Q27" s="1135" t="n"/>
+      <c r="R27" s="1135" t="n"/>
+      <c r="S27" s="1135" t="n"/>
+      <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="T27" s="1098" t="n"/>
-      <c r="U27" s="814" t="inlineStr">
+      <c r="U27" s="1134" t="n"/>
+      <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1109" t="inlineStr">
+      <c r="A28" s="1145" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1110" t="inlineStr">
+      <c r="B28" s="1146" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1110" t="inlineStr">
+      <c r="C28" s="1146" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1111" t="n"/>
-      <c r="E28" s="1111" t="n"/>
-      <c r="F28" s="1111" t="n"/>
-      <c r="G28" s="1111" t="n"/>
-      <c r="H28" s="1111" t="n"/>
-      <c r="I28" s="1112" t="n"/>
-      <c r="J28" s="1113" t="n"/>
-      <c r="K28" s="1113" t="n"/>
-      <c r="L28" s="1113" t="n"/>
-      <c r="M28" s="1111" t="n">
+      <c r="D28" s="1147" t="n"/>
+      <c r="E28" s="1147" t="n"/>
+      <c r="F28" s="1147" t="n"/>
+      <c r="G28" s="1147" t="n"/>
+      <c r="H28" s="1147" t="n"/>
+      <c r="I28" s="1148" t="n"/>
+      <c r="J28" s="1149" t="n"/>
+      <c r="K28" s="1149" t="n"/>
+      <c r="L28" s="1149" t="n"/>
+      <c r="M28" s="1147" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1111" t="n">
+      <c r="N28" s="1147" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1111" t="n"/>
-      <c r="P28" s="1114" t="n"/>
-      <c r="Q28" s="1111" t="n"/>
-      <c r="R28" s="1111" t="n"/>
-      <c r="S28" s="827" t="inlineStr">
+      <c r="O28" s="1147" t="n"/>
+      <c r="P28" s="1150" t="n"/>
+      <c r="Q28" s="1147" t="n"/>
+      <c r="R28" s="1147" t="n"/>
+      <c r="S28" s="1147" t="n"/>
+      <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="T28" s="1110" t="n"/>
-      <c r="U28" s="828" t="inlineStr">
+      <c r="U28" s="1146" t="n"/>
+      <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1085" t="inlineStr">
+      <c r="A29" s="1121" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1086" t="inlineStr">
+      <c r="B29" s="1122" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1086" t="inlineStr">
+      <c r="C29" s="1122" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1087" t="n"/>
-      <c r="E29" s="1087" t="n">
+      <c r="D29" s="1123" t="n"/>
+      <c r="E29" s="1123" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1087" t="n">
+      <c r="F29" s="1123" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1087" t="n">
+      <c r="G29" s="1123" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1087" t="n"/>
-      <c r="I29" s="1088" t="n"/>
-      <c r="J29" s="1089" t="n"/>
-      <c r="K29" s="1089" t="n"/>
-      <c r="L29" s="1089" t="n"/>
-      <c r="M29" s="1087" t="n"/>
-      <c r="N29" s="1087" t="n"/>
-      <c r="O29" s="1087" t="n">
+      <c r="H29" s="1123" t="n"/>
+      <c r="I29" s="1124" t="n"/>
+      <c r="J29" s="1125" t="n"/>
+      <c r="K29" s="1125" t="n"/>
+      <c r="L29" s="1125" t="n"/>
+      <c r="M29" s="1123" t="n"/>
+      <c r="N29" s="1123" t="n"/>
+      <c r="O29" s="1123" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1090" t="n">
+      <c r="P29" s="1126" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1087" t="n"/>
-      <c r="R29" s="1087" t="n"/>
-      <c r="S29" s="624" t="inlineStr">
+      <c r="Q29" s="1123" t="n"/>
+      <c r="R29" s="1123" t="n"/>
+      <c r="S29" s="1123" t="n"/>
+      <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="T29" s="1086" t="n"/>
-      <c r="U29" s="625" t="inlineStr">
+      <c r="U29" s="1122" t="n"/>
+      <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1091" t="inlineStr">
+      <c r="A30" s="1127" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1092" t="inlineStr">
+      <c r="B30" s="1128" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1092" t="inlineStr">
+      <c r="C30" s="1128" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1093" t="n"/>
-      <c r="E30" s="1093" t="n"/>
-      <c r="F30" s="1093" t="n"/>
-      <c r="G30" s="1093" t="n"/>
-      <c r="H30" s="1093" t="n"/>
-      <c r="I30" s="1094" t="n"/>
-      <c r="J30" s="1095" t="n"/>
-      <c r="K30" s="1095" t="n"/>
-      <c r="L30" s="1095" t="n"/>
-      <c r="M30" s="1093" t="n"/>
-      <c r="N30" s="1093" t="n"/>
-      <c r="O30" s="1093" t="n"/>
-      <c r="P30" s="1096" t="n"/>
-      <c r="Q30" s="1093" t="n"/>
-      <c r="R30" s="1093" t="n"/>
-      <c r="S30" s="631" t="inlineStr">
+      <c r="D30" s="1129" t="n"/>
+      <c r="E30" s="1129" t="n"/>
+      <c r="F30" s="1129" t="n"/>
+      <c r="G30" s="1129" t="n"/>
+      <c r="H30" s="1129" t="n"/>
+      <c r="I30" s="1130" t="n"/>
+      <c r="J30" s="1131" t="n"/>
+      <c r="K30" s="1131" t="n"/>
+      <c r="L30" s="1131" t="n"/>
+      <c r="M30" s="1129" t="n"/>
+      <c r="N30" s="1129" t="n"/>
+      <c r="O30" s="1129" t="n"/>
+      <c r="P30" s="1132" t="n"/>
+      <c r="Q30" s="1129" t="n"/>
+      <c r="R30" s="1129" t="n"/>
+      <c r="S30" s="1129" t="n"/>
+      <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="T30" s="1092" t="n"/>
-      <c r="U30" s="632" t="inlineStr">
+      <c r="U30" s="1128" t="n"/>
+      <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1097" t="inlineStr">
+      <c r="A31" s="1133" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1098" t="inlineStr">
+      <c r="B31" s="1134" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1098" t="inlineStr">
+      <c r="C31" s="1134" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1099" t="n"/>
-      <c r="E31" s="1099" t="n">
+      <c r="D31" s="1135" t="n"/>
+      <c r="E31" s="1135" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1099" t="n">
+      <c r="F31" s="1135" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1099" t="n">
+      <c r="G31" s="1135" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1099" t="n"/>
-      <c r="I31" s="1100" t="n"/>
-      <c r="J31" s="1101" t="n"/>
-      <c r="K31" s="1101" t="n"/>
-      <c r="L31" s="1101" t="n"/>
-      <c r="M31" s="1099" t="n"/>
-      <c r="N31" s="1099" t="n"/>
-      <c r="O31" s="1099" t="n">
+      <c r="H31" s="1135" t="n"/>
+      <c r="I31" s="1136" t="n"/>
+      <c r="J31" s="1137" t="n"/>
+      <c r="K31" s="1137" t="n"/>
+      <c r="L31" s="1137" t="n"/>
+      <c r="M31" s="1135" t="n"/>
+      <c r="N31" s="1135" t="n"/>
+      <c r="O31" s="1135" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1102" t="n">
+      <c r="P31" s="1138" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1099" t="n"/>
-      <c r="R31" s="1099" t="n"/>
-      <c r="S31" s="813" t="inlineStr">
+      <c r="Q31" s="1135" t="n"/>
+      <c r="R31" s="1135" t="n"/>
+      <c r="S31" s="1135" t="n"/>
+      <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="T31" s="1098" t="inlineStr">
+      <c r="U31" s="1134" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
       </c>
-      <c r="U31" s="814" t="inlineStr">
+      <c r="V31" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 10.6 (just below floor 11), CC 0.0. Loss 14.2-&gt;10.6 = ~3.6 ppm/24h = NORMAL sunny-day loss: morning was super sunny (weather.py noon snapshot wrongly read overcast). No demand issue - water clear, no algae, ladder not yet installed. PHOTOS (3): water CLEAR - bottom/steps crisp across deep+shallow, clean blue, no green/algae, waterline clean. Surface streaks = tree-shadow reflections (overcast). Shallow floor near steps shows mild mottling/light patches - reads as liner speckle pattern + lighting, NOT algae; no obvious iron/rust stain visible. For stain tracking, want a straight-down close-up of the suspected spot near returns in even shade (less glare).</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1109" t="inlineStr">
+      <c r="A32" s="1145" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1110" t="inlineStr">
+      <c r="B32" s="1146" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1110" t="inlineStr">
+      <c r="C32" s="1146" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1111" t="n"/>
-      <c r="E32" s="1111" t="n"/>
-      <c r="F32" s="1111" t="n"/>
-      <c r="G32" s="1111" t="n"/>
-      <c r="H32" s="1111" t="n">
+      <c r="D32" s="1147" t="n"/>
+      <c r="E32" s="1147" t="n"/>
+      <c r="F32" s="1147" t="n"/>
+      <c r="G32" s="1147" t="n"/>
+      <c r="H32" s="1147" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1112" t="n"/>
-      <c r="J32" s="1113" t="n"/>
-      <c r="K32" s="1113" t="n"/>
-      <c r="L32" s="1113" t="n"/>
-      <c r="M32" s="1111" t="n">
+      <c r="I32" s="1148" t="n"/>
+      <c r="J32" s="1149" t="n"/>
+      <c r="K32" s="1149" t="n"/>
+      <c r="L32" s="1149" t="n"/>
+      <c r="M32" s="1147" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1111" t="n">
+      <c r="N32" s="1147" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1111" t="n"/>
-      <c r="P32" s="1114" t="n"/>
-      <c r="Q32" s="1111" t="n"/>
-      <c r="R32" s="1111" t="n"/>
-      <c r="S32" s="827" t="inlineStr">
+      <c r="O32" s="1147" t="n"/>
+      <c r="P32" s="1150" t="n"/>
+      <c r="Q32" s="1147" t="n"/>
+      <c r="R32" s="1147" t="n"/>
+      <c r="S32" s="1147" t="n"/>
+      <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="T32" s="1110" t="n"/>
-      <c r="U32" s="828" t="inlineStr">
+      <c r="U32" s="1146" t="n"/>
+      <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1085" t="inlineStr">
+      <c r="A33" s="1121" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1086" t="inlineStr">
+      <c r="B33" s="1122" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1086" t="inlineStr">
+      <c r="C33" s="1122" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1087" t="n"/>
-      <c r="E33" s="1087" t="n">
+      <c r="D33" s="1123" t="n"/>
+      <c r="E33" s="1123" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1087" t="n">
+      <c r="F33" s="1123" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1087" t="n">
+      <c r="G33" s="1123" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1087" t="n"/>
-      <c r="I33" s="1088" t="n">
+      <c r="H33" s="1123" t="n"/>
+      <c r="I33" s="1124" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1089" t="n"/>
-      <c r="K33" s="1089" t="n"/>
-      <c r="L33" s="1089" t="n"/>
-      <c r="M33" s="1087" t="n"/>
-      <c r="N33" s="1087" t="n"/>
-      <c r="O33" s="1087" t="n">
+      <c r="J33" s="1125" t="n"/>
+      <c r="K33" s="1125" t="n"/>
+      <c r="L33" s="1125" t="n"/>
+      <c r="M33" s="1123" t="n"/>
+      <c r="N33" s="1123" t="n"/>
+      <c r="O33" s="1123" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1090" t="n">
+      <c r="P33" s="1126" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1087" t="n"/>
-      <c r="R33" s="1087" t="n">
+      <c r="Q33" s="1123" t="n"/>
+      <c r="R33" s="1123" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="624" t="inlineStr">
+      <c r="S33" s="1123" t="n"/>
+      <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="T33" s="1086" t="inlineStr">
+      <c r="U33" s="1122" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
       </c>
-      <c r="U33" s="625" t="inlineStr">
+      <c r="V33" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 12.8 (in band 13-15), CC 0.2 (trace = 1 drop; was 0.0 - watch). Loss ~3.0 ppm/19h from 6/27 eve dose (~15.8) - normal for a 67%-sun morning. Evening-dose routine holding well. WATER TEMP 79F. PHOTOS(4): water still clear (bottom visible), clean blue, no algae. Scattered debris specks (dirt/organic from landscaping today) on surface+floor + faint plume (stir-up/fresh dose) - cosmetic, filter/skim will clear; brush/vac if it settles. Straight-down near return: normal speckled liner, NO clear iron/rust stain (loose debris on top, not staining). Debris vacuumed + skimmed out same day -&gt; negligible Cl demand expected; treat tomorrow loss as normal.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1091" t="inlineStr">
+      <c r="A34" s="1127" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1092" t="inlineStr">
+      <c r="B34" s="1128" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1092" t="inlineStr">
+      <c r="C34" s="1128" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1093" t="n"/>
-      <c r="E34" s="1093" t="n"/>
-      <c r="F34" s="1093" t="n"/>
-      <c r="G34" s="1093" t="n"/>
-      <c r="H34" s="1093" t="n">
+      <c r="D34" s="1129" t="n"/>
+      <c r="E34" s="1129" t="n"/>
+      <c r="F34" s="1129" t="n"/>
+      <c r="G34" s="1129" t="n"/>
+      <c r="H34" s="1129" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1094" t="n"/>
-      <c r="J34" s="1095" t="n"/>
-      <c r="K34" s="1095" t="n"/>
-      <c r="L34" s="1095" t="n"/>
-      <c r="M34" s="1093" t="n">
+      <c r="I34" s="1130" t="n"/>
+      <c r="J34" s="1131" t="n"/>
+      <c r="K34" s="1131" t="n"/>
+      <c r="L34" s="1131" t="n"/>
+      <c r="M34" s="1129" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1093" t="n">
+      <c r="N34" s="1129" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1093" t="n"/>
-      <c r="P34" s="1096" t="n"/>
-      <c r="Q34" s="1093" t="n"/>
-      <c r="R34" s="1093" t="n"/>
-      <c r="S34" s="631" t="inlineStr">
+      <c r="O34" s="1129" t="n"/>
+      <c r="P34" s="1132" t="n"/>
+      <c r="Q34" s="1129" t="n"/>
+      <c r="R34" s="1129" t="n"/>
+      <c r="S34" s="1129" t="n"/>
+      <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="T34" s="1092" t="n"/>
-      <c r="U34" s="632" t="inlineStr">
+      <c r="U34" s="1128" t="n"/>
+      <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1097" t="inlineStr">
+      <c r="A35" s="1133" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1098" t="inlineStr">
+      <c r="B35" s="1134" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1098" t="inlineStr">
+      <c r="C35" s="1134" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1099" t="n"/>
-      <c r="E35" s="1099" t="n">
+      <c r="D35" s="1135" t="n"/>
+      <c r="E35" s="1135" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1099" t="n">
+      <c r="F35" s="1135" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1099" t="n">
+      <c r="G35" s="1135" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1099" t="n"/>
-      <c r="I35" s="1100" t="n">
+      <c r="H35" s="1135" t="n"/>
+      <c r="I35" s="1136" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1101" t="n"/>
-      <c r="K35" s="1101" t="n"/>
-      <c r="L35" s="1101" t="n"/>
-      <c r="M35" s="1099" t="n"/>
-      <c r="N35" s="1099" t="n"/>
-      <c r="O35" s="1099" t="n">
+      <c r="J35" s="1137" t="n"/>
+      <c r="K35" s="1137" t="n"/>
+      <c r="L35" s="1137" t="n"/>
+      <c r="M35" s="1135" t="n"/>
+      <c r="N35" s="1135" t="n"/>
+      <c r="O35" s="1135" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1102" t="n">
+      <c r="P35" s="1138" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1099" t="n"/>
-      <c r="R35" s="1099" t="n">
+      <c r="Q35" s="1135" t="n"/>
+      <c r="R35" s="1135" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="813" t="inlineStr">
+      <c r="S35" s="1135" t="n"/>
+      <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="T35" s="1098" t="inlineStr">
+      <c r="U35" s="1134" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
       </c>
-      <c r="U35" s="814" t="inlineStr">
+      <c r="V35" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.0 (in band 13-15, near aim), CC 0.2 (trace, holding ~0.2 - not climbing). Loss 2.3 ppm/24h (evening dose dodged afternoon UV). VERY sunny + hot week ahead -&gt; expect high daily UV demand; dose to top of band each evening for buffer, do NOT skip. PHOTOS(4): water clear+healthy (evening), clean blue, no algae, good clarity after dose+fill. Better stairs/return close-up: liner shows normal speckled pattern, NO clear iron/rust stain visible - if present it is subtle/masked. Ascorbic-acid SPOT TEST is the definitive check.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1103" t="inlineStr">
+      <c r="A36" s="1139" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1104" t="inlineStr">
+      <c r="B36" s="1140" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1104" t="inlineStr">
+      <c r="C36" s="1140" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1105" t="n"/>
-      <c r="E36" s="1105" t="n"/>
-      <c r="F36" s="1105" t="n"/>
-      <c r="G36" s="1105" t="n"/>
-      <c r="H36" s="1105" t="n">
+      <c r="D36" s="1141" t="n"/>
+      <c r="E36" s="1141" t="n"/>
+      <c r="F36" s="1141" t="n"/>
+      <c r="G36" s="1141" t="n"/>
+      <c r="H36" s="1141" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1106" t="n"/>
-      <c r="J36" s="1107" t="n"/>
-      <c r="K36" s="1107" t="n"/>
-      <c r="L36" s="1107" t="n"/>
-      <c r="M36" s="1105" t="n">
+      <c r="I36" s="1142" t="n"/>
+      <c r="J36" s="1143" t="n"/>
+      <c r="K36" s="1143" t="n"/>
+      <c r="L36" s="1143" t="n"/>
+      <c r="M36" s="1141" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1105" t="n">
+      <c r="N36" s="1141" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1105" t="n"/>
-      <c r="P36" s="1108" t="n"/>
-      <c r="Q36" s="1105" t="n"/>
-      <c r="R36" s="1105" t="n"/>
-      <c r="S36" s="820" t="inlineStr">
+      <c r="O36" s="1141" t="n"/>
+      <c r="P36" s="1144" t="n"/>
+      <c r="Q36" s="1141" t="n"/>
+      <c r="R36" s="1141" t="n"/>
+      <c r="S36" s="1141" t="n"/>
+      <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="T36" s="1104" t="n"/>
-      <c r="U36" s="821" t="inlineStr">
+      <c r="U36" s="1140" t="n"/>
+      <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1109" t="inlineStr">
+      <c r="A37" s="1145" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1110" t="inlineStr">
+      <c r="B37" s="1146" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1110" t="inlineStr">
+      <c r="C37" s="1146" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1111" t="n"/>
-      <c r="E37" s="1111" t="n"/>
-      <c r="F37" s="1111" t="n"/>
-      <c r="G37" s="1111" t="n"/>
-      <c r="H37" s="1111" t="n"/>
-      <c r="I37" s="1112" t="n"/>
-      <c r="J37" s="1113" t="n"/>
-      <c r="K37" s="1113" t="n"/>
-      <c r="L37" s="1113" t="n"/>
-      <c r="M37" s="1111" t="n"/>
-      <c r="N37" s="1111" t="n"/>
-      <c r="O37" s="1111" t="n"/>
-      <c r="P37" s="1114" t="n"/>
-      <c r="Q37" s="1111" t="n">
+      <c r="D37" s="1147" t="n"/>
+      <c r="E37" s="1147" t="n"/>
+      <c r="F37" s="1147" t="n"/>
+      <c r="G37" s="1147" t="n"/>
+      <c r="H37" s="1147" t="n"/>
+      <c r="I37" s="1148" t="n"/>
+      <c r="J37" s="1149" t="n"/>
+      <c r="K37" s="1149" t="n"/>
+      <c r="L37" s="1149" t="n"/>
+      <c r="M37" s="1147" t="n"/>
+      <c r="N37" s="1147" t="n"/>
+      <c r="O37" s="1147" t="n"/>
+      <c r="P37" s="1150" t="n"/>
+      <c r="Q37" s="1147" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1111" t="n"/>
-      <c r="S37" s="827" t="n"/>
-      <c r="T37" s="1110" t="n"/>
-      <c r="U37" s="828" t="inlineStr">
+      <c r="R37" s="1147" t="n"/>
+      <c r="S37" s="1147" t="n"/>
+      <c r="T37" s="827" t="n"/>
+      <c r="U37" s="1146" t="n"/>
+      <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1085" t="inlineStr">
+      <c r="A38" s="1121" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1086" t="inlineStr">
+      <c r="B38" s="1122" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1086" t="inlineStr">
+      <c r="C38" s="1122" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1087" t="n"/>
-      <c r="E38" s="1087" t="n">
+      <c r="D38" s="1123" t="n"/>
+      <c r="E38" s="1123" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1087" t="n">
+      <c r="F38" s="1123" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1087" t="n">
+      <c r="G38" s="1123" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1087" t="n"/>
-      <c r="I38" s="1088" t="n">
+      <c r="H38" s="1123" t="n"/>
+      <c r="I38" s="1124" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1089" t="n"/>
-      <c r="K38" s="1089" t="n"/>
-      <c r="L38" s="1089" t="n"/>
-      <c r="M38" s="1087" t="n"/>
-      <c r="N38" s="1087" t="n"/>
-      <c r="O38" s="1087" t="n">
+      <c r="J38" s="1125" t="n"/>
+      <c r="K38" s="1125" t="n"/>
+      <c r="L38" s="1125" t="n"/>
+      <c r="M38" s="1123" t="n"/>
+      <c r="N38" s="1123" t="n"/>
+      <c r="O38" s="1123" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1090" t="n">
+      <c r="P38" s="1126" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1087" t="n"/>
-      <c r="R38" s="1087" t="n">
+      <c r="Q38" s="1123" t="n"/>
+      <c r="R38" s="1123" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="624" t="inlineStr">
+      <c r="S38" s="1123" t="n"/>
+      <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="T38" s="1086" t="inlineStr">
+      <c r="U38" s="1122" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
       </c>
-      <c r="U38" s="625" t="inlineStr">
+      <c r="V38" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.6 (in band 13-15, near aim), CC 0.0 (the 0.2 trace cleared - higher FC worked). Loss 4.7 ppm/24h - hot very-sunny day; last night's 1.5 gal buffer absorbed it, still in band. Water 80.5F (warming). Hotter today (84F). PHOTOS(4): water clear+healthy (evening), clean blue, no algae, bottom visible; minor surface ripple from fill. No new stain concerns.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1115" t="inlineStr">
+      <c r="A39" s="1151" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1116" t="inlineStr">
+      <c r="B39" s="1152" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1116" t="inlineStr">
+      <c r="C39" s="1152" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1117" t="n"/>
-      <c r="E39" s="1117" t="n"/>
-      <c r="F39" s="1117" t="n"/>
-      <c r="G39" s="1117" t="n"/>
-      <c r="H39" s="1117" t="n">
+      <c r="D39" s="1153" t="n"/>
+      <c r="E39" s="1153" t="n"/>
+      <c r="F39" s="1153" t="n"/>
+      <c r="G39" s="1153" t="n"/>
+      <c r="H39" s="1153" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1118" t="n"/>
-      <c r="J39" s="1119" t="n"/>
-      <c r="K39" s="1119" t="n"/>
-      <c r="L39" s="1119" t="n"/>
-      <c r="M39" s="1117" t="n">
+      <c r="I39" s="1154" t="n"/>
+      <c r="J39" s="1155" t="n"/>
+      <c r="K39" s="1155" t="n"/>
+      <c r="L39" s="1155" t="n"/>
+      <c r="M39" s="1153" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1117" t="n">
+      <c r="N39" s="1153" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1117" t="n"/>
-      <c r="P39" s="1120" t="n"/>
-      <c r="Q39" s="1117" t="n"/>
-      <c r="R39" s="1117" t="n"/>
-      <c r="S39" s="659" t="inlineStr">
+      <c r="O39" s="1153" t="n"/>
+      <c r="P39" s="1156" t="n"/>
+      <c r="Q39" s="1153" t="n"/>
+      <c r="R39" s="1153" t="n"/>
+      <c r="S39" s="1153" t="n"/>
+      <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="T39" s="1116" t="n"/>
-      <c r="U39" s="660" t="inlineStr">
+      <c r="U39" s="1152" t="n"/>
+      <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1091" t="inlineStr">
+      <c r="A40" s="1127" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1092" t="inlineStr">
+      <c r="B40" s="1128" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1092" t="inlineStr">
+      <c r="C40" s="1128" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1093" t="n"/>
-      <c r="E40" s="1093" t="n"/>
-      <c r="F40" s="1093" t="n"/>
-      <c r="G40" s="1093" t="n"/>
-      <c r="H40" s="1093" t="n"/>
-      <c r="I40" s="1094" t="n"/>
-      <c r="J40" s="1095" t="n"/>
-      <c r="K40" s="1095" t="n"/>
-      <c r="L40" s="1095" t="n"/>
-      <c r="M40" s="1093" t="n"/>
-      <c r="N40" s="1093" t="n"/>
-      <c r="O40" s="1093" t="n"/>
-      <c r="P40" s="1096" t="n"/>
-      <c r="Q40" s="1093" t="n">
+      <c r="D40" s="1129" t="n"/>
+      <c r="E40" s="1129" t="n"/>
+      <c r="F40" s="1129" t="n"/>
+      <c r="G40" s="1129" t="n"/>
+      <c r="H40" s="1129" t="n"/>
+      <c r="I40" s="1130" t="n"/>
+      <c r="J40" s="1131" t="n"/>
+      <c r="K40" s="1131" t="n"/>
+      <c r="L40" s="1131" t="n"/>
+      <c r="M40" s="1129" t="n"/>
+      <c r="N40" s="1129" t="n"/>
+      <c r="O40" s="1129" t="n"/>
+      <c r="P40" s="1132" t="n"/>
+      <c r="Q40" s="1129" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1093" t="n"/>
-      <c r="S40" s="631" t="n"/>
-      <c r="T40" s="1092" t="n"/>
-      <c r="U40" s="632" t="inlineStr">
+      <c r="R40" s="1129" t="n"/>
+      <c r="S40" s="1129" t="n"/>
+      <c r="T40" s="631" t="n"/>
+      <c r="U40" s="1128" t="n"/>
+      <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1097" t="inlineStr">
+      <c r="A41" s="1133" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1098" t="inlineStr">
+      <c r="B41" s="1134" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1098" t="inlineStr">
+      <c r="C41" s="1134" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1099" t="n"/>
-      <c r="E41" s="1099" t="n">
+      <c r="D41" s="1135" t="n"/>
+      <c r="E41" s="1135" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1099" t="n">
+      <c r="F41" s="1135" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1099" t="n">
+      <c r="G41" s="1135" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1099" t="n"/>
-      <c r="I41" s="1100" t="n">
+      <c r="H41" s="1135" t="n"/>
+      <c r="I41" s="1136" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1101" t="n"/>
-      <c r="K41" s="1101" t="n"/>
-      <c r="L41" s="1101" t="n"/>
-      <c r="M41" s="1099" t="n"/>
-      <c r="N41" s="1099" t="n"/>
-      <c r="O41" s="1099" t="n">
+      <c r="J41" s="1137" t="n"/>
+      <c r="K41" s="1137" t="n"/>
+      <c r="L41" s="1137" t="n"/>
+      <c r="M41" s="1135" t="n"/>
+      <c r="N41" s="1135" t="n"/>
+      <c r="O41" s="1135" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1102" t="n">
+      <c r="P41" s="1138" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1099" t="n"/>
-      <c r="R41" s="1099" t="n">
+      <c r="Q41" s="1135" t="n"/>
+      <c r="R41" s="1135" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="813" t="inlineStr">
+      <c r="S41" s="1135" t="n"/>
+      <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="T41" s="1098" t="inlineStr">
+      <c r="U41" s="1134" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
       </c>
-      <c r="U41" s="814" t="inlineStr">
+      <c r="V41" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.8 (in band 13-15, at aim), CC 0.2 (trace). FC loss 5.1 ppm/24h (14.6 + 1.5gal dose - 14.8) - hottest/sunniest day yet (high 86F, ~12 sun hrs). Auto weather bucket said 'rain' from accumulated daily precip, but midday conditions are Clear/sunny (83% sun so far) - overrode to sunny bucket for dosing. PHOTOS(3): water clear+healthy (evening ~7:36PM), clean blue, bottom visible, no algae; a couple leaves floating (cosmetic - skimmer/filter clears). ZOOMED stair close-up (best look yet): normal blue speckled liner on the curved steps + decorative border; only minor debris/shadow in step corners; NO clear iron/rust or manganese stain visible - no progression vs prior days. Ascorbic-acid spot test remains the definitive check.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1109" t="inlineStr">
+      <c r="A42" s="1145" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1110" t="inlineStr">
+      <c r="B42" s="1146" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1110" t="inlineStr">
+      <c r="C42" s="1146" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1111" t="n"/>
-      <c r="E42" s="1111" t="n"/>
-      <c r="F42" s="1111" t="n"/>
-      <c r="G42" s="1111" t="n"/>
-      <c r="H42" s="1111" t="n">
+      <c r="D42" s="1147" t="n"/>
+      <c r="E42" s="1147" t="n"/>
+      <c r="F42" s="1147" t="n"/>
+      <c r="G42" s="1147" t="n"/>
+      <c r="H42" s="1147" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1112" t="n"/>
-      <c r="J42" s="1113" t="n"/>
-      <c r="K42" s="1113" t="n"/>
-      <c r="L42" s="1113" t="n"/>
-      <c r="M42" s="1111" t="n">
+      <c r="I42" s="1148" t="n"/>
+      <c r="J42" s="1149" t="n"/>
+      <c r="K42" s="1149" t="n"/>
+      <c r="L42" s="1149" t="n"/>
+      <c r="M42" s="1147" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1111" t="n">
+      <c r="N42" s="1147" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1111" t="n"/>
-      <c r="P42" s="1114" t="n"/>
-      <c r="Q42" s="1111" t="n"/>
-      <c r="R42" s="1111" t="n"/>
-      <c r="S42" s="827" t="inlineStr">
+      <c r="O42" s="1147" t="n"/>
+      <c r="P42" s="1150" t="n"/>
+      <c r="Q42" s="1147" t="n"/>
+      <c r="R42" s="1147" t="n"/>
+      <c r="S42" s="1147" t="n"/>
+      <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="T42" s="1110" t="n"/>
-      <c r="U42" s="828" t="inlineStr">
+      <c r="U42" s="1146" t="n"/>
+      <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1085" t="inlineStr">
+      <c r="A43" s="1121" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1086" t="inlineStr">
+      <c r="B43" s="1122" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1086" t="inlineStr">
+      <c r="C43" s="1122" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1087" t="n"/>
-      <c r="E43" s="1087" t="n">
+      <c r="D43" s="1123" t="n"/>
+      <c r="E43" s="1123" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1087" t="n">
+      <c r="F43" s="1123" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1087" t="n">
+      <c r="G43" s="1123" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1087" t="n"/>
-      <c r="I43" s="1088" t="n">
+      <c r="H43" s="1123" t="n"/>
+      <c r="I43" s="1124" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1089" t="n"/>
-      <c r="K43" s="1089" t="n"/>
-      <c r="L43" s="1089" t="n"/>
-      <c r="M43" s="1087" t="n"/>
-      <c r="N43" s="1087" t="n"/>
-      <c r="O43" s="1087" t="n">
+      <c r="J43" s="1125" t="n"/>
+      <c r="K43" s="1125" t="n"/>
+      <c r="L43" s="1125" t="n"/>
+      <c r="M43" s="1123" t="n"/>
+      <c r="N43" s="1123" t="n"/>
+      <c r="O43" s="1123" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1090" t="n">
+      <c r="P43" s="1126" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1087" t="n"/>
-      <c r="R43" s="1087" t="n">
+      <c r="Q43" s="1123" t="n"/>
+      <c r="R43" s="1123" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="624" t="inlineStr">
+      <c r="S43" s="1123" t="n"/>
+      <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="T43" s="1086" t="n"/>
-      <c r="U43" s="625" t="inlineStr">
+      <c r="U43" s="1122" t="n"/>
+      <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1115" t="inlineStr">
+      <c r="A44" s="1151" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1116" t="inlineStr">
+      <c r="B44" s="1152" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1116" t="inlineStr">
+      <c r="C44" s="1152" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1117" t="n"/>
-      <c r="E44" s="1117" t="n">
+      <c r="D44" s="1153" t="n"/>
+      <c r="E44" s="1153" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1117" t="n">
+      <c r="F44" s="1153" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1117" t="n"/>
-      <c r="H44" s="1117" t="n"/>
-      <c r="I44" s="1118" t="n"/>
-      <c r="J44" s="1119" t="n"/>
-      <c r="K44" s="1119" t="n"/>
-      <c r="L44" s="1119" t="n"/>
-      <c r="M44" s="1117" t="n"/>
-      <c r="N44" s="1117" t="n"/>
-      <c r="O44" s="1117" t="n"/>
-      <c r="P44" s="1120" t="n"/>
-      <c r="Q44" s="1117" t="n"/>
-      <c r="R44" s="1117" t="n"/>
-      <c r="S44" s="659" t="n"/>
-      <c r="T44" s="1116" t="inlineStr">
+      <c r="G44" s="1153" t="n"/>
+      <c r="H44" s="1153" t="n"/>
+      <c r="I44" s="1154" t="n"/>
+      <c r="J44" s="1155" t="n"/>
+      <c r="K44" s="1155" t="n"/>
+      <c r="L44" s="1155" t="n"/>
+      <c r="M44" s="1153" t="n"/>
+      <c r="N44" s="1153" t="n"/>
+      <c r="O44" s="1153" t="n"/>
+      <c r="P44" s="1156" t="n"/>
+      <c r="Q44" s="1153" t="n"/>
+      <c r="R44" s="1153" t="n"/>
+      <c r="S44" s="1153" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="T44" s="659" t="n"/>
+      <c r="U44" s="1152" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
       </c>
-      <c r="U44" s="660" t="inlineStr">
+      <c r="V44" s="660" t="inlineStr">
         <is>
           <t>Evening recheck before dosing, requested for peace-of-mind after noon's unexpectedly high FC (17.2) and the R-0870 dosing question. Decline from noon (17.2 -&gt; 15.4 over ~7.25h, pool shaded after ~6:30PM) tracks a plausible hot/sunny-day afternoon loss -- consistent with noon reading being real, not a fluke. CC ticked up slightly (0.0 -&gt; 0.4), normal for end of a hot/high-use day, still low. FC loss/Pred error left blank on this row -- not a comparable 24h noon-to-noon measurement, would corrupt the loss-rate tracking if filled in via the standard formula. PHOTOS(4): wide pool shots both look clear/healthy, clean blue, no algae; zoomed liner-corner close-up shows normal blue speckled texture, no clear rust/stain progression. New this entry: John mounted a graduated ruler to the skimmer faceplate to start tracking water level -- photo documents the ruler installation, no specific level reading called out yet (nothing invented here; will log a real number once John reports one).</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1091" t="inlineStr">
+      <c r="A45" s="1127" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1092" t="inlineStr">
+      <c r="B45" s="1128" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1092" t="inlineStr">
+      <c r="C45" s="1128" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1093" t="n"/>
-      <c r="E45" s="1093" t="n"/>
-      <c r="F45" s="1093" t="n"/>
-      <c r="G45" s="1093" t="n"/>
-      <c r="H45" s="1093" t="n">
+      <c r="D45" s="1129" t="n"/>
+      <c r="E45" s="1129" t="n"/>
+      <c r="F45" s="1129" t="n"/>
+      <c r="G45" s="1129" t="n"/>
+      <c r="H45" s="1129" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1094" t="n"/>
-      <c r="J45" s="1095" t="n"/>
-      <c r="K45" s="1095" t="n"/>
-      <c r="L45" s="1095" t="n"/>
-      <c r="M45" s="1093" t="n">
+      <c r="I45" s="1130" t="n"/>
+      <c r="J45" s="1131" t="n"/>
+      <c r="K45" s="1131" t="n"/>
+      <c r="L45" s="1131" t="n"/>
+      <c r="M45" s="1129" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1093" t="n">
+      <c r="N45" s="1129" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1093" t="n"/>
-      <c r="P45" s="1096" t="n"/>
-      <c r="Q45" s="1093" t="n"/>
-      <c r="R45" s="1093" t="n"/>
-      <c r="S45" s="631" t="inlineStr">
+      <c r="O45" s="1129" t="n"/>
+      <c r="P45" s="1132" t="n"/>
+      <c r="Q45" s="1129" t="n"/>
+      <c r="R45" s="1129" t="n"/>
+      <c r="S45" s="1129" t="n"/>
+      <c r="T45" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="T45" s="1092" t="n"/>
-      <c r="U45" s="632" t="inlineStr">
+      <c r="U45" s="1128" t="n"/>
+      <c r="V45" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
         </is>

</xml_diff>

<commit_message>
Log 2026-07-03 noon TEST: FC 16.6, CC 0.6, water 84.5F, level 11.8cm
Pred error +0.9 (model over-predicted loss again, less than 7/2's +2.1).
CC creeping 0.0->0.4->0.6, watch. fc_loss 4.1 noon-to-noon (corrected
from daily_calc's evening-recheck baseline). Also: switch push cadence
to twice daily -- push on each report-in (noon test, evening dose),
not bundled once, per John's request.
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1157">
+  <cellXfs count="1201">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -3999,6 +3999,138 @@
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4259,7 +4391,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V45"/>
+  <dimension ref="A1:V46"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -4436,35 +4568,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1121" t="inlineStr">
+      <c r="A3" s="1157" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1122" t="n"/>
-      <c r="C3" s="1122" t="inlineStr">
+      <c r="B3" s="1158" t="n"/>
+      <c r="C3" s="1158" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1123" t="n"/>
-      <c r="E3" s="1123" t="n"/>
-      <c r="F3" s="1123" t="n"/>
-      <c r="G3" s="1123" t="n"/>
-      <c r="H3" s="1123" t="n"/>
-      <c r="I3" s="1124" t="n"/>
-      <c r="J3" s="1125" t="n"/>
-      <c r="K3" s="1125" t="n"/>
-      <c r="L3" s="1125" t="n"/>
-      <c r="M3" s="1123" t="n"/>
-      <c r="N3" s="1123" t="n"/>
-      <c r="O3" s="1123" t="n"/>
-      <c r="P3" s="1126" t="n"/>
-      <c r="Q3" s="1123" t="n"/>
-      <c r="R3" s="1123" t="n"/>
-      <c r="S3" s="1123" t="n"/>
+      <c r="D3" s="1159" t="n"/>
+      <c r="E3" s="1159" t="n"/>
+      <c r="F3" s="1159" t="n"/>
+      <c r="G3" s="1159" t="n"/>
+      <c r="H3" s="1159" t="n"/>
+      <c r="I3" s="1160" t="n"/>
+      <c r="J3" s="1161" t="n"/>
+      <c r="K3" s="1161" t="n"/>
+      <c r="L3" s="1161" t="n"/>
+      <c r="M3" s="1159" t="n"/>
+      <c r="N3" s="1159" t="n"/>
+      <c r="O3" s="1159" t="n"/>
+      <c r="P3" s="1162" t="n"/>
+      <c r="Q3" s="1159" t="n"/>
+      <c r="R3" s="1159" t="n"/>
+      <c r="S3" s="1159" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1122" t="n"/>
+      <c r="U3" s="1158" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -4472,43 +4604,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1127" t="inlineStr">
+      <c r="A4" s="1163" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1128" t="inlineStr">
+      <c r="B4" s="1164" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1128" t="inlineStr">
+      <c r="C4" s="1164" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1129" t="n"/>
-      <c r="E4" s="1129" t="n"/>
-      <c r="F4" s="1129" t="n"/>
-      <c r="G4" s="1129" t="n"/>
-      <c r="H4" s="1129" t="n"/>
-      <c r="I4" s="1130" t="n"/>
-      <c r="J4" s="1131" t="n"/>
-      <c r="K4" s="1131" t="n"/>
-      <c r="L4" s="1131" t="n"/>
-      <c r="M4" s="1129" t="n">
+      <c r="D4" s="1165" t="n"/>
+      <c r="E4" s="1165" t="n"/>
+      <c r="F4" s="1165" t="n"/>
+      <c r="G4" s="1165" t="n"/>
+      <c r="H4" s="1165" t="n"/>
+      <c r="I4" s="1166" t="n"/>
+      <c r="J4" s="1167" t="n"/>
+      <c r="K4" s="1167" t="n"/>
+      <c r="L4" s="1167" t="n"/>
+      <c r="M4" s="1165" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1129" t="n">
+      <c r="N4" s="1165" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1129" t="n"/>
-      <c r="P4" s="1132" t="n"/>
-      <c r="Q4" s="1129" t="n"/>
-      <c r="R4" s="1129" t="n"/>
-      <c r="S4" s="1129" t="n"/>
+      <c r="O4" s="1165" t="n"/>
+      <c r="P4" s="1168" t="n"/>
+      <c r="Q4" s="1165" t="n"/>
+      <c r="R4" s="1165" t="n"/>
+      <c r="S4" s="1165" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1128" t="n"/>
+      <c r="U4" s="1164" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -4516,57 +4648,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1133" t="inlineStr">
+      <c r="A5" s="1169" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1134" t="inlineStr">
+      <c r="B5" s="1170" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1134" t="inlineStr">
+      <c r="C5" s="1170" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1135" t="n">
+      <c r="D5" s="1171" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1135" t="n">
+      <c r="E5" s="1171" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1135" t="n">
+      <c r="F5" s="1171" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1135" t="n"/>
-      <c r="H5" s="1135" t="n"/>
-      <c r="I5" s="1136" t="n"/>
-      <c r="J5" s="1137" t="n">
+      <c r="G5" s="1171" t="n"/>
+      <c r="H5" s="1171" t="n"/>
+      <c r="I5" s="1172" t="n"/>
+      <c r="J5" s="1173" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1137" t="n">
+      <c r="K5" s="1173" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1137" t="inlineStr">
+      <c r="L5" s="1173" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1135" t="n"/>
-      <c r="N5" s="1135" t="n"/>
-      <c r="O5" s="1135" t="n">
+      <c r="M5" s="1171" t="n"/>
+      <c r="N5" s="1171" t="n"/>
+      <c r="O5" s="1171" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1138" t="n">
+      <c r="P5" s="1174" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1135" t="n"/>
-      <c r="R5" s="1135" t="n"/>
-      <c r="S5" s="1135" t="n"/>
+      <c r="Q5" s="1171" t="n"/>
+      <c r="R5" s="1171" t="n"/>
+      <c r="S5" s="1171" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1134" t="n"/>
+      <c r="U5" s="1170" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -4574,43 +4706,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1139" t="inlineStr">
+      <c r="A6" s="1175" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1140" t="inlineStr">
+      <c r="B6" s="1176" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1140" t="inlineStr">
+      <c r="C6" s="1176" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1141" t="n"/>
-      <c r="E6" s="1141" t="n"/>
-      <c r="F6" s="1141" t="n"/>
-      <c r="G6" s="1141" t="n"/>
-      <c r="H6" s="1141" t="n"/>
-      <c r="I6" s="1142" t="n"/>
-      <c r="J6" s="1143" t="n"/>
-      <c r="K6" s="1143" t="n"/>
-      <c r="L6" s="1143" t="n"/>
-      <c r="M6" s="1141" t="n">
+      <c r="D6" s="1177" t="n"/>
+      <c r="E6" s="1177" t="n"/>
+      <c r="F6" s="1177" t="n"/>
+      <c r="G6" s="1177" t="n"/>
+      <c r="H6" s="1177" t="n"/>
+      <c r="I6" s="1178" t="n"/>
+      <c r="J6" s="1179" t="n"/>
+      <c r="K6" s="1179" t="n"/>
+      <c r="L6" s="1179" t="n"/>
+      <c r="M6" s="1177" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1141" t="n">
+      <c r="N6" s="1177" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1141" t="n"/>
-      <c r="P6" s="1144" t="n"/>
-      <c r="Q6" s="1141" t="n"/>
-      <c r="R6" s="1141" t="n"/>
-      <c r="S6" s="1141" t="n"/>
+      <c r="O6" s="1177" t="n"/>
+      <c r="P6" s="1180" t="n"/>
+      <c r="Q6" s="1177" t="n"/>
+      <c r="R6" s="1177" t="n"/>
+      <c r="S6" s="1177" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1140" t="n"/>
+      <c r="U6" s="1176" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -4618,39 +4750,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1145" t="inlineStr">
+      <c r="A7" s="1181" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1146" t="inlineStr">
+      <c r="B7" s="1182" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1146" t="inlineStr">
+      <c r="C7" s="1182" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1147" t="n"/>
-      <c r="E7" s="1147" t="n"/>
-      <c r="F7" s="1147" t="n"/>
-      <c r="G7" s="1147" t="n"/>
-      <c r="H7" s="1147" t="n"/>
-      <c r="I7" s="1148" t="n"/>
-      <c r="J7" s="1149" t="n"/>
-      <c r="K7" s="1149" t="n"/>
-      <c r="L7" s="1149" t="n"/>
-      <c r="M7" s="1147" t="n"/>
-      <c r="N7" s="1147" t="n"/>
-      <c r="O7" s="1147" t="n"/>
-      <c r="P7" s="1150" t="n"/>
-      <c r="Q7" s="1147" t="n"/>
-      <c r="R7" s="1147" t="n"/>
-      <c r="S7" s="1147" t="n"/>
+      <c r="D7" s="1183" t="n"/>
+      <c r="E7" s="1183" t="n"/>
+      <c r="F7" s="1183" t="n"/>
+      <c r="G7" s="1183" t="n"/>
+      <c r="H7" s="1183" t="n"/>
+      <c r="I7" s="1184" t="n"/>
+      <c r="J7" s="1185" t="n"/>
+      <c r="K7" s="1185" t="n"/>
+      <c r="L7" s="1185" t="n"/>
+      <c r="M7" s="1183" t="n"/>
+      <c r="N7" s="1183" t="n"/>
+      <c r="O7" s="1183" t="n"/>
+      <c r="P7" s="1186" t="n"/>
+      <c r="Q7" s="1183" t="n"/>
+      <c r="R7" s="1183" t="n"/>
+      <c r="S7" s="1183" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1146" t="n"/>
+      <c r="U7" s="1182" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -4658,39 +4790,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1121" t="inlineStr">
+      <c r="A8" s="1157" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1122" t="inlineStr">
+      <c r="B8" s="1158" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1122" t="inlineStr">
+      <c r="C8" s="1158" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1123" t="n"/>
-      <c r="E8" s="1123" t="n"/>
-      <c r="F8" s="1123" t="n"/>
-      <c r="G8" s="1123" t="n"/>
-      <c r="H8" s="1123" t="n"/>
-      <c r="I8" s="1124" t="n"/>
-      <c r="J8" s="1125" t="n"/>
-      <c r="K8" s="1125" t="n"/>
-      <c r="L8" s="1125" t="n"/>
-      <c r="M8" s="1123" t="n"/>
-      <c r="N8" s="1123" t="n"/>
-      <c r="O8" s="1123" t="n"/>
-      <c r="P8" s="1126" t="n"/>
-      <c r="Q8" s="1123" t="n"/>
-      <c r="R8" s="1123" t="n"/>
-      <c r="S8" s="1123" t="n"/>
+      <c r="D8" s="1159" t="n"/>
+      <c r="E8" s="1159" t="n"/>
+      <c r="F8" s="1159" t="n"/>
+      <c r="G8" s="1159" t="n"/>
+      <c r="H8" s="1159" t="n"/>
+      <c r="I8" s="1160" t="n"/>
+      <c r="J8" s="1161" t="n"/>
+      <c r="K8" s="1161" t="n"/>
+      <c r="L8" s="1161" t="n"/>
+      <c r="M8" s="1159" t="n"/>
+      <c r="N8" s="1159" t="n"/>
+      <c r="O8" s="1159" t="n"/>
+      <c r="P8" s="1162" t="n"/>
+      <c r="Q8" s="1159" t="n"/>
+      <c r="R8" s="1159" t="n"/>
+      <c r="S8" s="1159" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1122" t="n"/>
+      <c r="U8" s="1158" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -4698,63 +4830,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1151" t="inlineStr">
+      <c r="A9" s="1187" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1152" t="inlineStr">
+      <c r="B9" s="1188" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1152" t="inlineStr">
+      <c r="C9" s="1188" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1153" t="n">
+      <c r="D9" s="1189" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1153" t="n">
+      <c r="E9" s="1189" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1153" t="n">
+      <c r="F9" s="1189" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1153" t="n">
+      <c r="G9" s="1189" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1153" t="n"/>
-      <c r="I9" s="1154" t="n"/>
-      <c r="J9" s="1155" t="n">
+      <c r="H9" s="1189" t="n"/>
+      <c r="I9" s="1190" t="n"/>
+      <c r="J9" s="1191" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1155" t="n">
+      <c r="K9" s="1191" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1155" t="inlineStr">
+      <c r="L9" s="1191" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1153" t="n"/>
-      <c r="N9" s="1153" t="n"/>
-      <c r="O9" s="1153" t="n">
+      <c r="M9" s="1189" t="n"/>
+      <c r="N9" s="1189" t="n"/>
+      <c r="O9" s="1189" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1156" t="n">
+      <c r="P9" s="1192" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1153" t="n"/>
-      <c r="R9" s="1153" t="n"/>
-      <c r="S9" s="1153" t="n"/>
+      <c r="Q9" s="1189" t="n"/>
+      <c r="R9" s="1189" t="n"/>
+      <c r="S9" s="1189" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1152" t="n"/>
+      <c r="U9" s="1188" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -4762,43 +4894,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1151" t="inlineStr">
+      <c r="A10" s="1187" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1152" t="inlineStr">
+      <c r="B10" s="1188" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1152" t="inlineStr">
+      <c r="C10" s="1188" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1153" t="n"/>
-      <c r="E10" s="1153" t="n"/>
-      <c r="F10" s="1153" t="n"/>
-      <c r="G10" s="1153" t="n"/>
-      <c r="H10" s="1153" t="n"/>
-      <c r="I10" s="1154" t="n"/>
-      <c r="J10" s="1155" t="n"/>
-      <c r="K10" s="1155" t="n"/>
-      <c r="L10" s="1155" t="inlineStr">
+      <c r="D10" s="1189" t="n"/>
+      <c r="E10" s="1189" t="n"/>
+      <c r="F10" s="1189" t="n"/>
+      <c r="G10" s="1189" t="n"/>
+      <c r="H10" s="1189" t="n"/>
+      <c r="I10" s="1190" t="n"/>
+      <c r="J10" s="1191" t="n"/>
+      <c r="K10" s="1191" t="n"/>
+      <c r="L10" s="1191" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1153" t="n"/>
-      <c r="N10" s="1153" t="n"/>
-      <c r="O10" s="1153" t="n"/>
-      <c r="P10" s="1156" t="n"/>
-      <c r="Q10" s="1153" t="n"/>
-      <c r="R10" s="1153" t="n"/>
-      <c r="S10" s="1153" t="n"/>
+      <c r="M10" s="1189" t="n"/>
+      <c r="N10" s="1189" t="n"/>
+      <c r="O10" s="1189" t="n"/>
+      <c r="P10" s="1192" t="n"/>
+      <c r="Q10" s="1189" t="n"/>
+      <c r="R10" s="1189" t="n"/>
+      <c r="S10" s="1189" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1152" t="n"/>
+      <c r="U10" s="1188" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -4806,43 +4938,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1151" t="inlineStr">
+      <c r="A11" s="1187" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1152" t="inlineStr">
+      <c r="B11" s="1188" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1152" t="inlineStr">
+      <c r="C11" s="1188" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1153" t="n"/>
-      <c r="E11" s="1153" t="n"/>
-      <c r="F11" s="1153" t="n"/>
-      <c r="G11" s="1153" t="n"/>
-      <c r="H11" s="1153" t="n"/>
-      <c r="I11" s="1154" t="n"/>
-      <c r="J11" s="1155" t="n"/>
-      <c r="K11" s="1155" t="n"/>
-      <c r="L11" s="1155" t="n"/>
-      <c r="M11" s="1153" t="n">
+      <c r="D11" s="1189" t="n"/>
+      <c r="E11" s="1189" t="n"/>
+      <c r="F11" s="1189" t="n"/>
+      <c r="G11" s="1189" t="n"/>
+      <c r="H11" s="1189" t="n"/>
+      <c r="I11" s="1190" t="n"/>
+      <c r="J11" s="1191" t="n"/>
+      <c r="K11" s="1191" t="n"/>
+      <c r="L11" s="1191" t="n"/>
+      <c r="M11" s="1189" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1153" t="n">
+      <c r="N11" s="1189" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1153" t="n"/>
-      <c r="P11" s="1156" t="n"/>
-      <c r="Q11" s="1153" t="n"/>
-      <c r="R11" s="1153" t="n"/>
-      <c r="S11" s="1153" t="n"/>
+      <c r="O11" s="1189" t="n"/>
+      <c r="P11" s="1192" t="n"/>
+      <c r="Q11" s="1189" t="n"/>
+      <c r="R11" s="1189" t="n"/>
+      <c r="S11" s="1189" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1152" t="n"/>
+      <c r="U11" s="1188" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -4850,39 +4982,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1127" t="inlineStr">
+      <c r="A12" s="1163" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1128" t="inlineStr">
+      <c r="B12" s="1164" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1128" t="inlineStr">
+      <c r="C12" s="1164" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1129" t="n"/>
-      <c r="E12" s="1129" t="n"/>
-      <c r="F12" s="1129" t="n"/>
-      <c r="G12" s="1129" t="n"/>
-      <c r="H12" s="1129" t="n"/>
-      <c r="I12" s="1130" t="n"/>
-      <c r="J12" s="1131" t="n"/>
-      <c r="K12" s="1131" t="n"/>
-      <c r="L12" s="1131" t="n"/>
-      <c r="M12" s="1129" t="n"/>
-      <c r="N12" s="1129" t="n"/>
-      <c r="O12" s="1129" t="n"/>
-      <c r="P12" s="1132" t="n"/>
-      <c r="Q12" s="1129" t="n"/>
-      <c r="R12" s="1129" t="n"/>
-      <c r="S12" s="1129" t="n"/>
+      <c r="D12" s="1165" t="n"/>
+      <c r="E12" s="1165" t="n"/>
+      <c r="F12" s="1165" t="n"/>
+      <c r="G12" s="1165" t="n"/>
+      <c r="H12" s="1165" t="n"/>
+      <c r="I12" s="1166" t="n"/>
+      <c r="J12" s="1167" t="n"/>
+      <c r="K12" s="1167" t="n"/>
+      <c r="L12" s="1167" t="n"/>
+      <c r="M12" s="1165" t="n"/>
+      <c r="N12" s="1165" t="n"/>
+      <c r="O12" s="1165" t="n"/>
+      <c r="P12" s="1168" t="n"/>
+      <c r="Q12" s="1165" t="n"/>
+      <c r="R12" s="1165" t="n"/>
+      <c r="S12" s="1165" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1128" t="n"/>
+      <c r="U12" s="1164" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -4890,35 +5022,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1133" t="inlineStr">
+      <c r="A13" s="1169" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1134" t="n"/>
-      <c r="C13" s="1134" t="inlineStr">
+      <c r="B13" s="1170" t="n"/>
+      <c r="C13" s="1170" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1135" t="n"/>
-      <c r="E13" s="1135" t="n"/>
-      <c r="F13" s="1135" t="n"/>
-      <c r="G13" s="1135" t="n"/>
-      <c r="H13" s="1135" t="n"/>
-      <c r="I13" s="1136" t="n"/>
-      <c r="J13" s="1137" t="n"/>
-      <c r="K13" s="1137" t="n"/>
-      <c r="L13" s="1137" t="n"/>
-      <c r="M13" s="1135" t="n"/>
-      <c r="N13" s="1135" t="n"/>
-      <c r="O13" s="1135" t="n"/>
-      <c r="P13" s="1138" t="n"/>
-      <c r="Q13" s="1135" t="n"/>
-      <c r="R13" s="1135" t="n"/>
-      <c r="S13" s="1135" t="n"/>
+      <c r="D13" s="1171" t="n"/>
+      <c r="E13" s="1171" t="n"/>
+      <c r="F13" s="1171" t="n"/>
+      <c r="G13" s="1171" t="n"/>
+      <c r="H13" s="1171" t="n"/>
+      <c r="I13" s="1172" t="n"/>
+      <c r="J13" s="1173" t="n"/>
+      <c r="K13" s="1173" t="n"/>
+      <c r="L13" s="1173" t="n"/>
+      <c r="M13" s="1171" t="n"/>
+      <c r="N13" s="1171" t="n"/>
+      <c r="O13" s="1171" t="n"/>
+      <c r="P13" s="1174" t="n"/>
+      <c r="Q13" s="1171" t="n"/>
+      <c r="R13" s="1171" t="n"/>
+      <c r="S13" s="1171" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1134" t="n"/>
+      <c r="U13" s="1170" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -4926,53 +5058,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1139" t="inlineStr">
+      <c r="A14" s="1175" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1140" t="inlineStr">
+      <c r="B14" s="1176" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1140" t="inlineStr">
+      <c r="C14" s="1176" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1141" t="n"/>
-      <c r="E14" s="1141" t="n">
+      <c r="D14" s="1177" t="n"/>
+      <c r="E14" s="1177" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1141" t="n">
+      <c r="F14" s="1177" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1141" t="n">
+      <c r="G14" s="1177" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1141" t="n"/>
-      <c r="I14" s="1142" t="n"/>
-      <c r="J14" s="1143" t="n"/>
-      <c r="K14" s="1143" t="n"/>
-      <c r="L14" s="1143" t="n"/>
-      <c r="M14" s="1141" t="n"/>
-      <c r="N14" s="1141" t="n"/>
-      <c r="O14" s="1141" t="n">
+      <c r="H14" s="1177" t="n"/>
+      <c r="I14" s="1178" t="n"/>
+      <c r="J14" s="1179" t="n"/>
+      <c r="K14" s="1179" t="n"/>
+      <c r="L14" s="1179" t="n"/>
+      <c r="M14" s="1177" t="n"/>
+      <c r="N14" s="1177" t="n"/>
+      <c r="O14" s="1177" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1144" t="n">
+      <c r="P14" s="1180" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1141" t="n"/>
-      <c r="R14" s="1141" t="n"/>
-      <c r="S14" s="1141" t="n"/>
+      <c r="Q14" s="1177" t="n"/>
+      <c r="R14" s="1177" t="n"/>
+      <c r="S14" s="1177" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1140" t="n"/>
+      <c r="U14" s="1176" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -4980,43 +5112,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1139" t="inlineStr">
+      <c r="A15" s="1175" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1140" t="inlineStr">
+      <c r="B15" s="1176" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1140" t="inlineStr">
+      <c r="C15" s="1176" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1141" t="n"/>
-      <c r="E15" s="1141" t="n"/>
-      <c r="F15" s="1141" t="n"/>
-      <c r="G15" s="1141" t="n"/>
-      <c r="H15" s="1141" t="n"/>
-      <c r="I15" s="1142" t="n"/>
-      <c r="J15" s="1143" t="n"/>
-      <c r="K15" s="1143" t="n"/>
-      <c r="L15" s="1143" t="n"/>
-      <c r="M15" s="1141" t="n">
+      <c r="D15" s="1177" t="n"/>
+      <c r="E15" s="1177" t="n"/>
+      <c r="F15" s="1177" t="n"/>
+      <c r="G15" s="1177" t="n"/>
+      <c r="H15" s="1177" t="n"/>
+      <c r="I15" s="1178" t="n"/>
+      <c r="J15" s="1179" t="n"/>
+      <c r="K15" s="1179" t="n"/>
+      <c r="L15" s="1179" t="n"/>
+      <c r="M15" s="1177" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1141" t="n">
+      <c r="N15" s="1177" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1141" t="n"/>
-      <c r="P15" s="1144" t="n"/>
-      <c r="Q15" s="1141" t="n"/>
-      <c r="R15" s="1141" t="n"/>
-      <c r="S15" s="1141" t="n"/>
+      <c r="O15" s="1177" t="n"/>
+      <c r="P15" s="1180" t="n"/>
+      <c r="Q15" s="1177" t="n"/>
+      <c r="R15" s="1177" t="n"/>
+      <c r="S15" s="1177" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1140" t="n"/>
+      <c r="U15" s="1176" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -5024,39 +5156,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1145" t="inlineStr">
+      <c r="A16" s="1181" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1146" t="inlineStr">
+      <c r="B16" s="1182" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1146" t="inlineStr">
+      <c r="C16" s="1182" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1147" t="n"/>
-      <c r="E16" s="1147" t="n"/>
-      <c r="F16" s="1147" t="n"/>
-      <c r="G16" s="1147" t="n"/>
-      <c r="H16" s="1147" t="n"/>
-      <c r="I16" s="1148" t="n"/>
-      <c r="J16" s="1149" t="n"/>
-      <c r="K16" s="1149" t="n"/>
-      <c r="L16" s="1149" t="n"/>
-      <c r="M16" s="1147" t="n"/>
-      <c r="N16" s="1147" t="n"/>
-      <c r="O16" s="1147" t="n"/>
-      <c r="P16" s="1150" t="n"/>
-      <c r="Q16" s="1147" t="n"/>
-      <c r="R16" s="1147" t="n"/>
-      <c r="S16" s="1147" t="n"/>
+      <c r="D16" s="1183" t="n"/>
+      <c r="E16" s="1183" t="n"/>
+      <c r="F16" s="1183" t="n"/>
+      <c r="G16" s="1183" t="n"/>
+      <c r="H16" s="1183" t="n"/>
+      <c r="I16" s="1184" t="n"/>
+      <c r="J16" s="1185" t="n"/>
+      <c r="K16" s="1185" t="n"/>
+      <c r="L16" s="1185" t="n"/>
+      <c r="M16" s="1183" t="n"/>
+      <c r="N16" s="1183" t="n"/>
+      <c r="O16" s="1183" t="n"/>
+      <c r="P16" s="1186" t="n"/>
+      <c r="Q16" s="1183" t="n"/>
+      <c r="R16" s="1183" t="n"/>
+      <c r="S16" s="1183" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1146" t="n"/>
+      <c r="U16" s="1182" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -5064,39 +5196,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1121" t="inlineStr">
+      <c r="A17" s="1157" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1122" t="inlineStr">
+      <c r="B17" s="1158" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1122" t="inlineStr">
+      <c r="C17" s="1158" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1123" t="n"/>
-      <c r="E17" s="1123" t="n"/>
-      <c r="F17" s="1123" t="n"/>
-      <c r="G17" s="1123" t="n"/>
-      <c r="H17" s="1123" t="n"/>
-      <c r="I17" s="1124" t="n"/>
-      <c r="J17" s="1125" t="n"/>
-      <c r="K17" s="1125" t="n"/>
-      <c r="L17" s="1125" t="n"/>
-      <c r="M17" s="1123" t="n"/>
-      <c r="N17" s="1123" t="n"/>
-      <c r="O17" s="1123" t="n"/>
-      <c r="P17" s="1126" t="n"/>
-      <c r="Q17" s="1123" t="n"/>
-      <c r="R17" s="1123" t="n"/>
-      <c r="S17" s="1123" t="n"/>
+      <c r="D17" s="1159" t="n"/>
+      <c r="E17" s="1159" t="n"/>
+      <c r="F17" s="1159" t="n"/>
+      <c r="G17" s="1159" t="n"/>
+      <c r="H17" s="1159" t="n"/>
+      <c r="I17" s="1160" t="n"/>
+      <c r="J17" s="1161" t="n"/>
+      <c r="K17" s="1161" t="n"/>
+      <c r="L17" s="1161" t="n"/>
+      <c r="M17" s="1159" t="n"/>
+      <c r="N17" s="1159" t="n"/>
+      <c r="O17" s="1159" t="n"/>
+      <c r="P17" s="1162" t="n"/>
+      <c r="Q17" s="1159" t="n"/>
+      <c r="R17" s="1159" t="n"/>
+      <c r="S17" s="1159" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1122" t="n"/>
+      <c r="U17" s="1158" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -5104,53 +5236,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1151" t="inlineStr">
+      <c r="A18" s="1187" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1152" t="inlineStr">
+      <c r="B18" s="1188" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1152" t="inlineStr">
+      <c r="C18" s="1188" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1153" t="n"/>
-      <c r="E18" s="1153" t="n">
+      <c r="D18" s="1189" t="n"/>
+      <c r="E18" s="1189" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1153" t="n">
+      <c r="F18" s="1189" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1153" t="n">
+      <c r="G18" s="1189" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1153" t="n"/>
-      <c r="I18" s="1154" t="n"/>
-      <c r="J18" s="1155" t="n"/>
-      <c r="K18" s="1155" t="n"/>
-      <c r="L18" s="1155" t="n"/>
-      <c r="M18" s="1153" t="n"/>
-      <c r="N18" s="1153" t="n"/>
-      <c r="O18" s="1153" t="n">
+      <c r="H18" s="1189" t="n"/>
+      <c r="I18" s="1190" t="n"/>
+      <c r="J18" s="1191" t="n"/>
+      <c r="K18" s="1191" t="n"/>
+      <c r="L18" s="1191" t="n"/>
+      <c r="M18" s="1189" t="n"/>
+      <c r="N18" s="1189" t="n"/>
+      <c r="O18" s="1189" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1156" t="n">
+      <c r="P18" s="1192" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1153" t="n"/>
-      <c r="R18" s="1153" t="n"/>
-      <c r="S18" s="1153" t="n"/>
+      <c r="Q18" s="1189" t="n"/>
+      <c r="R18" s="1189" t="n"/>
+      <c r="S18" s="1189" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1152" t="n"/>
+      <c r="U18" s="1188" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -5158,47 +5290,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1151" t="inlineStr">
+      <c r="A19" s="1187" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1152" t="inlineStr">
+      <c r="B19" s="1188" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1152" t="inlineStr">
+      <c r="C19" s="1188" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1153" t="n"/>
-      <c r="E19" s="1153" t="n"/>
-      <c r="F19" s="1153" t="n"/>
-      <c r="G19" s="1153" t="n"/>
-      <c r="H19" s="1153" t="n"/>
-      <c r="I19" s="1154" t="n"/>
-      <c r="J19" s="1155" t="n"/>
-      <c r="K19" s="1155" t="n"/>
-      <c r="L19" s="1155" t="n"/>
-      <c r="M19" s="1153" t="n">
+      <c r="D19" s="1189" t="n"/>
+      <c r="E19" s="1189" t="n"/>
+      <c r="F19" s="1189" t="n"/>
+      <c r="G19" s="1189" t="n"/>
+      <c r="H19" s="1189" t="n"/>
+      <c r="I19" s="1190" t="n"/>
+      <c r="J19" s="1191" t="n"/>
+      <c r="K19" s="1191" t="n"/>
+      <c r="L19" s="1191" t="n"/>
+      <c r="M19" s="1189" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1153" t="n">
+      <c r="N19" s="1189" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1153" t="n"/>
-      <c r="P19" s="1156" t="n"/>
-      <c r="Q19" s="1153" t="n"/>
-      <c r="R19" s="1153" t="n"/>
-      <c r="S19" s="1153" t="n"/>
+      <c r="O19" s="1189" t="n"/>
+      <c r="P19" s="1192" t="n"/>
+      <c r="Q19" s="1189" t="n"/>
+      <c r="R19" s="1189" t="n"/>
+      <c r="S19" s="1189" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1152" t="n"/>
+      <c r="U19" s="1188" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -5206,43 +5338,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1151" t="inlineStr">
+      <c r="A20" s="1187" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1152" t="inlineStr">
+      <c r="B20" s="1188" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1152" t="inlineStr">
+      <c r="C20" s="1188" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1153" t="n"/>
-      <c r="E20" s="1153" t="n"/>
-      <c r="F20" s="1153" t="n"/>
-      <c r="G20" s="1153" t="n"/>
-      <c r="H20" s="1153" t="n"/>
-      <c r="I20" s="1154" t="n"/>
-      <c r="J20" s="1155" t="n"/>
-      <c r="K20" s="1155" t="n"/>
-      <c r="L20" s="1155" t="n"/>
-      <c r="M20" s="1153" t="n"/>
-      <c r="N20" s="1153" t="n"/>
-      <c r="O20" s="1153" t="n"/>
-      <c r="P20" s="1156" t="n"/>
-      <c r="Q20" s="1153" t="n"/>
-      <c r="R20" s="1153" t="n"/>
-      <c r="S20" s="1153" t="n"/>
+      <c r="D20" s="1189" t="n"/>
+      <c r="E20" s="1189" t="n"/>
+      <c r="F20" s="1189" t="n"/>
+      <c r="G20" s="1189" t="n"/>
+      <c r="H20" s="1189" t="n"/>
+      <c r="I20" s="1190" t="n"/>
+      <c r="J20" s="1191" t="n"/>
+      <c r="K20" s="1191" t="n"/>
+      <c r="L20" s="1191" t="n"/>
+      <c r="M20" s="1189" t="n"/>
+      <c r="N20" s="1189" t="n"/>
+      <c r="O20" s="1189" t="n"/>
+      <c r="P20" s="1192" t="n"/>
+      <c r="Q20" s="1189" t="n"/>
+      <c r="R20" s="1189" t="n"/>
+      <c r="S20" s="1189" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1152" t="n"/>
+      <c r="U20" s="1188" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -5250,39 +5382,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1127" t="inlineStr">
+      <c r="A21" s="1163" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1128" t="inlineStr">
+      <c r="B21" s="1164" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1128" t="inlineStr">
+      <c r="C21" s="1164" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1129" t="n"/>
-      <c r="E21" s="1129" t="n"/>
-      <c r="F21" s="1129" t="n"/>
-      <c r="G21" s="1129" t="n"/>
-      <c r="H21" s="1129" t="n"/>
-      <c r="I21" s="1130" t="n"/>
-      <c r="J21" s="1131" t="n"/>
-      <c r="K21" s="1131" t="n"/>
-      <c r="L21" s="1131" t="n"/>
-      <c r="M21" s="1129" t="n"/>
-      <c r="N21" s="1129" t="n"/>
-      <c r="O21" s="1129" t="n"/>
-      <c r="P21" s="1132" t="n"/>
-      <c r="Q21" s="1129" t="n"/>
-      <c r="R21" s="1129" t="n"/>
-      <c r="S21" s="1129" t="n"/>
+      <c r="D21" s="1165" t="n"/>
+      <c r="E21" s="1165" t="n"/>
+      <c r="F21" s="1165" t="n"/>
+      <c r="G21" s="1165" t="n"/>
+      <c r="H21" s="1165" t="n"/>
+      <c r="I21" s="1166" t="n"/>
+      <c r="J21" s="1167" t="n"/>
+      <c r="K21" s="1167" t="n"/>
+      <c r="L21" s="1167" t="n"/>
+      <c r="M21" s="1165" t="n"/>
+      <c r="N21" s="1165" t="n"/>
+      <c r="O21" s="1165" t="n"/>
+      <c r="P21" s="1168" t="n"/>
+      <c r="Q21" s="1165" t="n"/>
+      <c r="R21" s="1165" t="n"/>
+      <c r="S21" s="1165" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1128" t="n"/>
+      <c r="U21" s="1164" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -5290,39 +5422,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1133" t="inlineStr">
+      <c r="A22" s="1169" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1134" t="inlineStr">
+      <c r="B22" s="1170" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1134" t="inlineStr">
+      <c r="C22" s="1170" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1135" t="n"/>
-      <c r="E22" s="1135" t="n"/>
-      <c r="F22" s="1135" t="n"/>
-      <c r="G22" s="1135" t="n"/>
-      <c r="H22" s="1135" t="n"/>
-      <c r="I22" s="1136" t="n"/>
-      <c r="J22" s="1137" t="n"/>
-      <c r="K22" s="1137" t="n"/>
-      <c r="L22" s="1137" t="n"/>
-      <c r="M22" s="1135" t="n"/>
-      <c r="N22" s="1135" t="n"/>
-      <c r="O22" s="1135" t="n"/>
-      <c r="P22" s="1138" t="n"/>
-      <c r="Q22" s="1135" t="n"/>
-      <c r="R22" s="1135" t="n"/>
-      <c r="S22" s="1135" t="n"/>
+      <c r="D22" s="1171" t="n"/>
+      <c r="E22" s="1171" t="n"/>
+      <c r="F22" s="1171" t="n"/>
+      <c r="G22" s="1171" t="n"/>
+      <c r="H22" s="1171" t="n"/>
+      <c r="I22" s="1172" t="n"/>
+      <c r="J22" s="1173" t="n"/>
+      <c r="K22" s="1173" t="n"/>
+      <c r="L22" s="1173" t="n"/>
+      <c r="M22" s="1171" t="n"/>
+      <c r="N22" s="1171" t="n"/>
+      <c r="O22" s="1171" t="n"/>
+      <c r="P22" s="1174" t="n"/>
+      <c r="Q22" s="1171" t="n"/>
+      <c r="R22" s="1171" t="n"/>
+      <c r="S22" s="1171" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1134" t="n"/>
+      <c r="U22" s="1170" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -5330,53 +5462,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1139" t="inlineStr">
+      <c r="A23" s="1175" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1140" t="inlineStr">
+      <c r="B23" s="1176" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1140" t="inlineStr">
+      <c r="C23" s="1176" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1141" t="n"/>
-      <c r="E23" s="1141" t="n">
+      <c r="D23" s="1177" t="n"/>
+      <c r="E23" s="1177" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1141" t="n">
+      <c r="F23" s="1177" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1141" t="n">
+      <c r="G23" s="1177" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1141" t="n"/>
-      <c r="I23" s="1142" t="n"/>
-      <c r="J23" s="1143" t="n"/>
-      <c r="K23" s="1143" t="n"/>
-      <c r="L23" s="1143" t="n"/>
-      <c r="M23" s="1141" t="n"/>
-      <c r="N23" s="1141" t="n"/>
-      <c r="O23" s="1141" t="n">
+      <c r="H23" s="1177" t="n"/>
+      <c r="I23" s="1178" t="n"/>
+      <c r="J23" s="1179" t="n"/>
+      <c r="K23" s="1179" t="n"/>
+      <c r="L23" s="1179" t="n"/>
+      <c r="M23" s="1177" t="n"/>
+      <c r="N23" s="1177" t="n"/>
+      <c r="O23" s="1177" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1144" t="n">
+      <c r="P23" s="1180" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1141" t="n"/>
-      <c r="R23" s="1141" t="n"/>
-      <c r="S23" s="1141" t="n"/>
+      <c r="Q23" s="1177" t="n"/>
+      <c r="R23" s="1177" t="n"/>
+      <c r="S23" s="1177" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1140" t="n"/>
+      <c r="U23" s="1176" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -5384,47 +5516,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1145" t="inlineStr">
+      <c r="A24" s="1181" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1146" t="inlineStr">
+      <c r="B24" s="1182" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1146" t="inlineStr">
+      <c r="C24" s="1182" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1147" t="n"/>
-      <c r="E24" s="1147" t="n"/>
-      <c r="F24" s="1147" t="n"/>
-      <c r="G24" s="1147" t="n"/>
-      <c r="H24" s="1147" t="n"/>
-      <c r="I24" s="1148" t="n"/>
-      <c r="J24" s="1149" t="n"/>
-      <c r="K24" s="1149" t="n"/>
-      <c r="L24" s="1149" t="n"/>
-      <c r="M24" s="1147" t="n">
+      <c r="D24" s="1183" t="n"/>
+      <c r="E24" s="1183" t="n"/>
+      <c r="F24" s="1183" t="n"/>
+      <c r="G24" s="1183" t="n"/>
+      <c r="H24" s="1183" t="n"/>
+      <c r="I24" s="1184" t="n"/>
+      <c r="J24" s="1185" t="n"/>
+      <c r="K24" s="1185" t="n"/>
+      <c r="L24" s="1185" t="n"/>
+      <c r="M24" s="1183" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1147" t="n">
+      <c r="N24" s="1183" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1147" t="n"/>
-      <c r="P24" s="1150" t="n"/>
-      <c r="Q24" s="1147" t="n"/>
-      <c r="R24" s="1147" t="n"/>
-      <c r="S24" s="1147" t="n"/>
+      <c r="O24" s="1183" t="n"/>
+      <c r="P24" s="1186" t="n"/>
+      <c r="Q24" s="1183" t="n"/>
+      <c r="R24" s="1183" t="n"/>
+      <c r="S24" s="1183" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1146" t="n"/>
+      <c r="U24" s="1182" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -5432,61 +5564,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1121" t="inlineStr">
+      <c r="A25" s="1157" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1122" t="inlineStr">
+      <c r="B25" s="1158" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1122" t="inlineStr">
+      <c r="C25" s="1158" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1123" t="n">
+      <c r="D25" s="1159" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1123" t="n">
+      <c r="E25" s="1159" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1123" t="n">
+      <c r="F25" s="1159" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1123" t="n">
+      <c r="G25" s="1159" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1123" t="n"/>
-      <c r="I25" s="1124" t="n"/>
-      <c r="J25" s="1125" t="n">
+      <c r="H25" s="1159" t="n"/>
+      <c r="I25" s="1160" t="n"/>
+      <c r="J25" s="1161" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1125" t="n">
+      <c r="K25" s="1161" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1125" t="n">
+      <c r="L25" s="1161" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1123" t="n"/>
-      <c r="N25" s="1123" t="n"/>
-      <c r="O25" s="1123" t="n">
+      <c r="M25" s="1159" t="n"/>
+      <c r="N25" s="1159" t="n"/>
+      <c r="O25" s="1159" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1126" t="n">
+      <c r="P25" s="1162" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1123" t="n"/>
-      <c r="R25" s="1123" t="n"/>
-      <c r="S25" s="1123" t="n"/>
+      <c r="Q25" s="1159" t="n"/>
+      <c r="R25" s="1159" t="n"/>
+      <c r="S25" s="1159" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1122" t="n"/>
+      <c r="U25" s="1158" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -5494,47 +5626,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1127" t="inlineStr">
+      <c r="A26" s="1163" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1128" t="inlineStr">
+      <c r="B26" s="1164" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1128" t="inlineStr">
+      <c r="C26" s="1164" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1129" t="n"/>
-      <c r="E26" s="1129" t="n"/>
-      <c r="F26" s="1129" t="n"/>
-      <c r="G26" s="1129" t="n"/>
-      <c r="H26" s="1129" t="n"/>
-      <c r="I26" s="1130" t="n"/>
-      <c r="J26" s="1131" t="n"/>
-      <c r="K26" s="1131" t="n"/>
-      <c r="L26" s="1131" t="n"/>
-      <c r="M26" s="1129" t="n">
+      <c r="D26" s="1165" t="n"/>
+      <c r="E26" s="1165" t="n"/>
+      <c r="F26" s="1165" t="n"/>
+      <c r="G26" s="1165" t="n"/>
+      <c r="H26" s="1165" t="n"/>
+      <c r="I26" s="1166" t="n"/>
+      <c r="J26" s="1167" t="n"/>
+      <c r="K26" s="1167" t="n"/>
+      <c r="L26" s="1167" t="n"/>
+      <c r="M26" s="1165" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1129" t="n">
+      <c r="N26" s="1165" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1129" t="n"/>
-      <c r="P26" s="1132" t="n"/>
-      <c r="Q26" s="1129" t="n"/>
-      <c r="R26" s="1129" t="n"/>
-      <c r="S26" s="1129" t="n"/>
+      <c r="O26" s="1165" t="n"/>
+      <c r="P26" s="1168" t="n"/>
+      <c r="Q26" s="1165" t="n"/>
+      <c r="R26" s="1165" t="n"/>
+      <c r="S26" s="1165" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1128" t="n"/>
+      <c r="U26" s="1164" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -5542,53 +5674,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1133" t="inlineStr">
+      <c r="A27" s="1169" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1134" t="inlineStr">
+      <c r="B27" s="1170" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1134" t="inlineStr">
+      <c r="C27" s="1170" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1135" t="n"/>
-      <c r="E27" s="1135" t="n">
+      <c r="D27" s="1171" t="n"/>
+      <c r="E27" s="1171" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1135" t="n">
+      <c r="F27" s="1171" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1135" t="n">
+      <c r="G27" s="1171" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1135" t="n"/>
-      <c r="I27" s="1136" t="n"/>
-      <c r="J27" s="1137" t="n"/>
-      <c r="K27" s="1137" t="n"/>
-      <c r="L27" s="1137" t="n"/>
-      <c r="M27" s="1135" t="n"/>
-      <c r="N27" s="1135" t="n"/>
-      <c r="O27" s="1135" t="n">
+      <c r="H27" s="1171" t="n"/>
+      <c r="I27" s="1172" t="n"/>
+      <c r="J27" s="1173" t="n"/>
+      <c r="K27" s="1173" t="n"/>
+      <c r="L27" s="1173" t="n"/>
+      <c r="M27" s="1171" t="n"/>
+      <c r="N27" s="1171" t="n"/>
+      <c r="O27" s="1171" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1138" t="n">
+      <c r="P27" s="1174" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1135" t="n"/>
-      <c r="R27" s="1135" t="n"/>
-      <c r="S27" s="1135" t="n"/>
+      <c r="Q27" s="1171" t="n"/>
+      <c r="R27" s="1171" t="n"/>
+      <c r="S27" s="1171" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1134" t="n"/>
+      <c r="U27" s="1170" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -5596,47 +5728,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1145" t="inlineStr">
+      <c r="A28" s="1181" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1146" t="inlineStr">
+      <c r="B28" s="1182" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1146" t="inlineStr">
+      <c r="C28" s="1182" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1147" t="n"/>
-      <c r="E28" s="1147" t="n"/>
-      <c r="F28" s="1147" t="n"/>
-      <c r="G28" s="1147" t="n"/>
-      <c r="H28" s="1147" t="n"/>
-      <c r="I28" s="1148" t="n"/>
-      <c r="J28" s="1149" t="n"/>
-      <c r="K28" s="1149" t="n"/>
-      <c r="L28" s="1149" t="n"/>
-      <c r="M28" s="1147" t="n">
+      <c r="D28" s="1183" t="n"/>
+      <c r="E28" s="1183" t="n"/>
+      <c r="F28" s="1183" t="n"/>
+      <c r="G28" s="1183" t="n"/>
+      <c r="H28" s="1183" t="n"/>
+      <c r="I28" s="1184" t="n"/>
+      <c r="J28" s="1185" t="n"/>
+      <c r="K28" s="1185" t="n"/>
+      <c r="L28" s="1185" t="n"/>
+      <c r="M28" s="1183" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1147" t="n">
+      <c r="N28" s="1183" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1147" t="n"/>
-      <c r="P28" s="1150" t="n"/>
-      <c r="Q28" s="1147" t="n"/>
-      <c r="R28" s="1147" t="n"/>
-      <c r="S28" s="1147" t="n"/>
+      <c r="O28" s="1183" t="n"/>
+      <c r="P28" s="1186" t="n"/>
+      <c r="Q28" s="1183" t="n"/>
+      <c r="R28" s="1183" t="n"/>
+      <c r="S28" s="1183" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1146" t="n"/>
+      <c r="U28" s="1182" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -5644,53 +5776,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1121" t="inlineStr">
+      <c r="A29" s="1157" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1122" t="inlineStr">
+      <c r="B29" s="1158" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1122" t="inlineStr">
+      <c r="C29" s="1158" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1123" t="n"/>
-      <c r="E29" s="1123" t="n">
+      <c r="D29" s="1159" t="n"/>
+      <c r="E29" s="1159" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1123" t="n">
+      <c r="F29" s="1159" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1123" t="n">
+      <c r="G29" s="1159" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1123" t="n"/>
-      <c r="I29" s="1124" t="n"/>
-      <c r="J29" s="1125" t="n"/>
-      <c r="K29" s="1125" t="n"/>
-      <c r="L29" s="1125" t="n"/>
-      <c r="M29" s="1123" t="n"/>
-      <c r="N29" s="1123" t="n"/>
-      <c r="O29" s="1123" t="n">
+      <c r="H29" s="1159" t="n"/>
+      <c r="I29" s="1160" t="n"/>
+      <c r="J29" s="1161" t="n"/>
+      <c r="K29" s="1161" t="n"/>
+      <c r="L29" s="1161" t="n"/>
+      <c r="M29" s="1159" t="n"/>
+      <c r="N29" s="1159" t="n"/>
+      <c r="O29" s="1159" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1126" t="n">
+      <c r="P29" s="1162" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1123" t="n"/>
-      <c r="R29" s="1123" t="n"/>
-      <c r="S29" s="1123" t="n"/>
+      <c r="Q29" s="1159" t="n"/>
+      <c r="R29" s="1159" t="n"/>
+      <c r="S29" s="1159" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1122" t="n"/>
+      <c r="U29" s="1158" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -5698,43 +5830,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1127" t="inlineStr">
+      <c r="A30" s="1163" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1128" t="inlineStr">
+      <c r="B30" s="1164" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1128" t="inlineStr">
+      <c r="C30" s="1164" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1129" t="n"/>
-      <c r="E30" s="1129" t="n"/>
-      <c r="F30" s="1129" t="n"/>
-      <c r="G30" s="1129" t="n"/>
-      <c r="H30" s="1129" t="n"/>
-      <c r="I30" s="1130" t="n"/>
-      <c r="J30" s="1131" t="n"/>
-      <c r="K30" s="1131" t="n"/>
-      <c r="L30" s="1131" t="n"/>
-      <c r="M30" s="1129" t="n"/>
-      <c r="N30" s="1129" t="n"/>
-      <c r="O30" s="1129" t="n"/>
-      <c r="P30" s="1132" t="n"/>
-      <c r="Q30" s="1129" t="n"/>
-      <c r="R30" s="1129" t="n"/>
-      <c r="S30" s="1129" t="n"/>
+      <c r="D30" s="1165" t="n"/>
+      <c r="E30" s="1165" t="n"/>
+      <c r="F30" s="1165" t="n"/>
+      <c r="G30" s="1165" t="n"/>
+      <c r="H30" s="1165" t="n"/>
+      <c r="I30" s="1166" t="n"/>
+      <c r="J30" s="1167" t="n"/>
+      <c r="K30" s="1167" t="n"/>
+      <c r="L30" s="1167" t="n"/>
+      <c r="M30" s="1165" t="n"/>
+      <c r="N30" s="1165" t="n"/>
+      <c r="O30" s="1165" t="n"/>
+      <c r="P30" s="1168" t="n"/>
+      <c r="Q30" s="1165" t="n"/>
+      <c r="R30" s="1165" t="n"/>
+      <c r="S30" s="1165" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1128" t="n"/>
+      <c r="U30" s="1164" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -5742,53 +5874,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1133" t="inlineStr">
+      <c r="A31" s="1169" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1134" t="inlineStr">
+      <c r="B31" s="1170" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1134" t="inlineStr">
+      <c r="C31" s="1170" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1135" t="n"/>
-      <c r="E31" s="1135" t="n">
+      <c r="D31" s="1171" t="n"/>
+      <c r="E31" s="1171" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1135" t="n">
+      <c r="F31" s="1171" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1135" t="n">
+      <c r="G31" s="1171" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1135" t="n"/>
-      <c r="I31" s="1136" t="n"/>
-      <c r="J31" s="1137" t="n"/>
-      <c r="K31" s="1137" t="n"/>
-      <c r="L31" s="1137" t="n"/>
-      <c r="M31" s="1135" t="n"/>
-      <c r="N31" s="1135" t="n"/>
-      <c r="O31" s="1135" t="n">
+      <c r="H31" s="1171" t="n"/>
+      <c r="I31" s="1172" t="n"/>
+      <c r="J31" s="1173" t="n"/>
+      <c r="K31" s="1173" t="n"/>
+      <c r="L31" s="1173" t="n"/>
+      <c r="M31" s="1171" t="n"/>
+      <c r="N31" s="1171" t="n"/>
+      <c r="O31" s="1171" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1138" t="n">
+      <c r="P31" s="1174" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1135" t="n"/>
-      <c r="R31" s="1135" t="n"/>
-      <c r="S31" s="1135" t="n"/>
+      <c r="Q31" s="1171" t="n"/>
+      <c r="R31" s="1171" t="n"/>
+      <c r="S31" s="1171" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1134" t="inlineStr">
+      <c r="U31" s="1170" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -5800,49 +5932,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1145" t="inlineStr">
+      <c r="A32" s="1181" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1146" t="inlineStr">
+      <c r="B32" s="1182" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1146" t="inlineStr">
+      <c r="C32" s="1182" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1147" t="n"/>
-      <c r="E32" s="1147" t="n"/>
-      <c r="F32" s="1147" t="n"/>
-      <c r="G32" s="1147" t="n"/>
-      <c r="H32" s="1147" t="n">
+      <c r="D32" s="1183" t="n"/>
+      <c r="E32" s="1183" t="n"/>
+      <c r="F32" s="1183" t="n"/>
+      <c r="G32" s="1183" t="n"/>
+      <c r="H32" s="1183" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1148" t="n"/>
-      <c r="J32" s="1149" t="n"/>
-      <c r="K32" s="1149" t="n"/>
-      <c r="L32" s="1149" t="n"/>
-      <c r="M32" s="1147" t="n">
+      <c r="I32" s="1184" t="n"/>
+      <c r="J32" s="1185" t="n"/>
+      <c r="K32" s="1185" t="n"/>
+      <c r="L32" s="1185" t="n"/>
+      <c r="M32" s="1183" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1147" t="n">
+      <c r="N32" s="1183" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1147" t="n"/>
-      <c r="P32" s="1150" t="n"/>
-      <c r="Q32" s="1147" t="n"/>
-      <c r="R32" s="1147" t="n"/>
-      <c r="S32" s="1147" t="n"/>
+      <c r="O32" s="1183" t="n"/>
+      <c r="P32" s="1186" t="n"/>
+      <c r="Q32" s="1183" t="n"/>
+      <c r="R32" s="1183" t="n"/>
+      <c r="S32" s="1183" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1146" t="n"/>
+      <c r="U32" s="1182" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -5850,57 +5982,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1121" t="inlineStr">
+      <c r="A33" s="1157" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1122" t="inlineStr">
+      <c r="B33" s="1158" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1122" t="inlineStr">
+      <c r="C33" s="1158" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1123" t="n"/>
-      <c r="E33" s="1123" t="n">
+      <c r="D33" s="1159" t="n"/>
+      <c r="E33" s="1159" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1123" t="n">
+      <c r="F33" s="1159" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1123" t="n">
+      <c r="G33" s="1159" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1123" t="n"/>
-      <c r="I33" s="1124" t="n">
+      <c r="H33" s="1159" t="n"/>
+      <c r="I33" s="1160" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1125" t="n"/>
-      <c r="K33" s="1125" t="n"/>
-      <c r="L33" s="1125" t="n"/>
-      <c r="M33" s="1123" t="n"/>
-      <c r="N33" s="1123" t="n"/>
-      <c r="O33" s="1123" t="n">
+      <c r="J33" s="1161" t="n"/>
+      <c r="K33" s="1161" t="n"/>
+      <c r="L33" s="1161" t="n"/>
+      <c r="M33" s="1159" t="n"/>
+      <c r="N33" s="1159" t="n"/>
+      <c r="O33" s="1159" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1126" t="n">
+      <c r="P33" s="1162" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1123" t="n"/>
-      <c r="R33" s="1123" t="n">
+      <c r="Q33" s="1159" t="n"/>
+      <c r="R33" s="1159" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1123" t="n"/>
+      <c r="S33" s="1159" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1122" t="inlineStr">
+      <c r="U33" s="1158" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -5912,49 +6044,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1127" t="inlineStr">
+      <c r="A34" s="1163" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1128" t="inlineStr">
+      <c r="B34" s="1164" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1128" t="inlineStr">
+      <c r="C34" s="1164" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1129" t="n"/>
-      <c r="E34" s="1129" t="n"/>
-      <c r="F34" s="1129" t="n"/>
-      <c r="G34" s="1129" t="n"/>
-      <c r="H34" s="1129" t="n">
+      <c r="D34" s="1165" t="n"/>
+      <c r="E34" s="1165" t="n"/>
+      <c r="F34" s="1165" t="n"/>
+      <c r="G34" s="1165" t="n"/>
+      <c r="H34" s="1165" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1130" t="n"/>
-      <c r="J34" s="1131" t="n"/>
-      <c r="K34" s="1131" t="n"/>
-      <c r="L34" s="1131" t="n"/>
-      <c r="M34" s="1129" t="n">
+      <c r="I34" s="1166" t="n"/>
+      <c r="J34" s="1167" t="n"/>
+      <c r="K34" s="1167" t="n"/>
+      <c r="L34" s="1167" t="n"/>
+      <c r="M34" s="1165" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1129" t="n">
+      <c r="N34" s="1165" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1129" t="n"/>
-      <c r="P34" s="1132" t="n"/>
-      <c r="Q34" s="1129" t="n"/>
-      <c r="R34" s="1129" t="n"/>
-      <c r="S34" s="1129" t="n"/>
+      <c r="O34" s="1165" t="n"/>
+      <c r="P34" s="1168" t="n"/>
+      <c r="Q34" s="1165" t="n"/>
+      <c r="R34" s="1165" t="n"/>
+      <c r="S34" s="1165" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1128" t="n"/>
+      <c r="U34" s="1164" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -5962,57 +6094,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1133" t="inlineStr">
+      <c r="A35" s="1169" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1134" t="inlineStr">
+      <c r="B35" s="1170" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1134" t="inlineStr">
+      <c r="C35" s="1170" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1135" t="n"/>
-      <c r="E35" s="1135" t="n">
+      <c r="D35" s="1171" t="n"/>
+      <c r="E35" s="1171" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1135" t="n">
+      <c r="F35" s="1171" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1135" t="n">
+      <c r="G35" s="1171" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1135" t="n"/>
-      <c r="I35" s="1136" t="n">
+      <c r="H35" s="1171" t="n"/>
+      <c r="I35" s="1172" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1137" t="n"/>
-      <c r="K35" s="1137" t="n"/>
-      <c r="L35" s="1137" t="n"/>
-      <c r="M35" s="1135" t="n"/>
-      <c r="N35" s="1135" t="n"/>
-      <c r="O35" s="1135" t="n">
+      <c r="J35" s="1173" t="n"/>
+      <c r="K35" s="1173" t="n"/>
+      <c r="L35" s="1173" t="n"/>
+      <c r="M35" s="1171" t="n"/>
+      <c r="N35" s="1171" t="n"/>
+      <c r="O35" s="1171" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1138" t="n">
+      <c r="P35" s="1174" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1135" t="n"/>
-      <c r="R35" s="1135" t="n">
+      <c r="Q35" s="1171" t="n"/>
+      <c r="R35" s="1171" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1135" t="n"/>
+      <c r="S35" s="1171" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1134" t="inlineStr">
+      <c r="U35" s="1170" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -6024,49 +6156,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1139" t="inlineStr">
+      <c r="A36" s="1175" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1140" t="inlineStr">
+      <c r="B36" s="1176" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1140" t="inlineStr">
+      <c r="C36" s="1176" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1141" t="n"/>
-      <c r="E36" s="1141" t="n"/>
-      <c r="F36" s="1141" t="n"/>
-      <c r="G36" s="1141" t="n"/>
-      <c r="H36" s="1141" t="n">
+      <c r="D36" s="1177" t="n"/>
+      <c r="E36" s="1177" t="n"/>
+      <c r="F36" s="1177" t="n"/>
+      <c r="G36" s="1177" t="n"/>
+      <c r="H36" s="1177" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1142" t="n"/>
-      <c r="J36" s="1143" t="n"/>
-      <c r="K36" s="1143" t="n"/>
-      <c r="L36" s="1143" t="n"/>
-      <c r="M36" s="1141" t="n">
+      <c r="I36" s="1178" t="n"/>
+      <c r="J36" s="1179" t="n"/>
+      <c r="K36" s="1179" t="n"/>
+      <c r="L36" s="1179" t="n"/>
+      <c r="M36" s="1177" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1141" t="n">
+      <c r="N36" s="1177" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1141" t="n"/>
-      <c r="P36" s="1144" t="n"/>
-      <c r="Q36" s="1141" t="n"/>
-      <c r="R36" s="1141" t="n"/>
-      <c r="S36" s="1141" t="n"/>
+      <c r="O36" s="1177" t="n"/>
+      <c r="P36" s="1180" t="n"/>
+      <c r="Q36" s="1177" t="n"/>
+      <c r="R36" s="1177" t="n"/>
+      <c r="S36" s="1177" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1140" t="n"/>
+      <c r="U36" s="1176" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -6074,41 +6206,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1145" t="inlineStr">
+      <c r="A37" s="1181" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1146" t="inlineStr">
+      <c r="B37" s="1182" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1146" t="inlineStr">
+      <c r="C37" s="1182" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1147" t="n"/>
-      <c r="E37" s="1147" t="n"/>
-      <c r="F37" s="1147" t="n"/>
-      <c r="G37" s="1147" t="n"/>
-      <c r="H37" s="1147" t="n"/>
-      <c r="I37" s="1148" t="n"/>
-      <c r="J37" s="1149" t="n"/>
-      <c r="K37" s="1149" t="n"/>
-      <c r="L37" s="1149" t="n"/>
-      <c r="M37" s="1147" t="n"/>
-      <c r="N37" s="1147" t="n"/>
-      <c r="O37" s="1147" t="n"/>
-      <c r="P37" s="1150" t="n"/>
-      <c r="Q37" s="1147" t="n">
+      <c r="D37" s="1183" t="n"/>
+      <c r="E37" s="1183" t="n"/>
+      <c r="F37" s="1183" t="n"/>
+      <c r="G37" s="1183" t="n"/>
+      <c r="H37" s="1183" t="n"/>
+      <c r="I37" s="1184" t="n"/>
+      <c r="J37" s="1185" t="n"/>
+      <c r="K37" s="1185" t="n"/>
+      <c r="L37" s="1185" t="n"/>
+      <c r="M37" s="1183" t="n"/>
+      <c r="N37" s="1183" t="n"/>
+      <c r="O37" s="1183" t="n"/>
+      <c r="P37" s="1186" t="n"/>
+      <c r="Q37" s="1183" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1147" t="n"/>
-      <c r="S37" s="1147" t="n"/>
+      <c r="R37" s="1183" t="n"/>
+      <c r="S37" s="1183" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1146" t="n"/>
+      <c r="U37" s="1182" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -6116,57 +6248,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1121" t="inlineStr">
+      <c r="A38" s="1157" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1122" t="inlineStr">
+      <c r="B38" s="1158" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1122" t="inlineStr">
+      <c r="C38" s="1158" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1123" t="n"/>
-      <c r="E38" s="1123" t="n">
+      <c r="D38" s="1159" t="n"/>
+      <c r="E38" s="1159" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1123" t="n">
+      <c r="F38" s="1159" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1123" t="n">
+      <c r="G38" s="1159" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1123" t="n"/>
-      <c r="I38" s="1124" t="n">
+      <c r="H38" s="1159" t="n"/>
+      <c r="I38" s="1160" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1125" t="n"/>
-      <c r="K38" s="1125" t="n"/>
-      <c r="L38" s="1125" t="n"/>
-      <c r="M38" s="1123" t="n"/>
-      <c r="N38" s="1123" t="n"/>
-      <c r="O38" s="1123" t="n">
+      <c r="J38" s="1161" t="n"/>
+      <c r="K38" s="1161" t="n"/>
+      <c r="L38" s="1161" t="n"/>
+      <c r="M38" s="1159" t="n"/>
+      <c r="N38" s="1159" t="n"/>
+      <c r="O38" s="1159" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1126" t="n">
+      <c r="P38" s="1162" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1123" t="n"/>
-      <c r="R38" s="1123" t="n">
+      <c r="Q38" s="1159" t="n"/>
+      <c r="R38" s="1159" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1123" t="n"/>
+      <c r="S38" s="1159" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1122" t="inlineStr">
+      <c r="U38" s="1158" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -6178,49 +6310,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1151" t="inlineStr">
+      <c r="A39" s="1187" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1152" t="inlineStr">
+      <c r="B39" s="1188" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1152" t="inlineStr">
+      <c r="C39" s="1188" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1153" t="n"/>
-      <c r="E39" s="1153" t="n"/>
-      <c r="F39" s="1153" t="n"/>
-      <c r="G39" s="1153" t="n"/>
-      <c r="H39" s="1153" t="n">
+      <c r="D39" s="1189" t="n"/>
+      <c r="E39" s="1189" t="n"/>
+      <c r="F39" s="1189" t="n"/>
+      <c r="G39" s="1189" t="n"/>
+      <c r="H39" s="1189" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1154" t="n"/>
-      <c r="J39" s="1155" t="n"/>
-      <c r="K39" s="1155" t="n"/>
-      <c r="L39" s="1155" t="n"/>
-      <c r="M39" s="1153" t="n">
+      <c r="I39" s="1190" t="n"/>
+      <c r="J39" s="1191" t="n"/>
+      <c r="K39" s="1191" t="n"/>
+      <c r="L39" s="1191" t="n"/>
+      <c r="M39" s="1189" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1153" t="n">
+      <c r="N39" s="1189" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1153" t="n"/>
-      <c r="P39" s="1156" t="n"/>
-      <c r="Q39" s="1153" t="n"/>
-      <c r="R39" s="1153" t="n"/>
-      <c r="S39" s="1153" t="n"/>
+      <c r="O39" s="1189" t="n"/>
+      <c r="P39" s="1192" t="n"/>
+      <c r="Q39" s="1189" t="n"/>
+      <c r="R39" s="1189" t="n"/>
+      <c r="S39" s="1189" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1152" t="n"/>
+      <c r="U39" s="1188" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -6228,41 +6360,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1127" t="inlineStr">
+      <c r="A40" s="1163" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1128" t="inlineStr">
+      <c r="B40" s="1164" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1128" t="inlineStr">
+      <c r="C40" s="1164" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1129" t="n"/>
-      <c r="E40" s="1129" t="n"/>
-      <c r="F40" s="1129" t="n"/>
-      <c r="G40" s="1129" t="n"/>
-      <c r="H40" s="1129" t="n"/>
-      <c r="I40" s="1130" t="n"/>
-      <c r="J40" s="1131" t="n"/>
-      <c r="K40" s="1131" t="n"/>
-      <c r="L40" s="1131" t="n"/>
-      <c r="M40" s="1129" t="n"/>
-      <c r="N40" s="1129" t="n"/>
-      <c r="O40" s="1129" t="n"/>
-      <c r="P40" s="1132" t="n"/>
-      <c r="Q40" s="1129" t="n">
+      <c r="D40" s="1165" t="n"/>
+      <c r="E40" s="1165" t="n"/>
+      <c r="F40" s="1165" t="n"/>
+      <c r="G40" s="1165" t="n"/>
+      <c r="H40" s="1165" t="n"/>
+      <c r="I40" s="1166" t="n"/>
+      <c r="J40" s="1167" t="n"/>
+      <c r="K40" s="1167" t="n"/>
+      <c r="L40" s="1167" t="n"/>
+      <c r="M40" s="1165" t="n"/>
+      <c r="N40" s="1165" t="n"/>
+      <c r="O40" s="1165" t="n"/>
+      <c r="P40" s="1168" t="n"/>
+      <c r="Q40" s="1165" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1129" t="n"/>
-      <c r="S40" s="1129" t="n"/>
+      <c r="R40" s="1165" t="n"/>
+      <c r="S40" s="1165" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1128" t="n"/>
+      <c r="U40" s="1164" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -6270,57 +6402,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1133" t="inlineStr">
+      <c r="A41" s="1169" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1134" t="inlineStr">
+      <c r="B41" s="1170" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1134" t="inlineStr">
+      <c r="C41" s="1170" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1135" t="n"/>
-      <c r="E41" s="1135" t="n">
+      <c r="D41" s="1171" t="n"/>
+      <c r="E41" s="1171" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1135" t="n">
+      <c r="F41" s="1171" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1135" t="n">
+      <c r="G41" s="1171" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1135" t="n"/>
-      <c r="I41" s="1136" t="n">
+      <c r="H41" s="1171" t="n"/>
+      <c r="I41" s="1172" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1137" t="n"/>
-      <c r="K41" s="1137" t="n"/>
-      <c r="L41" s="1137" t="n"/>
-      <c r="M41" s="1135" t="n"/>
-      <c r="N41" s="1135" t="n"/>
-      <c r="O41" s="1135" t="n">
+      <c r="J41" s="1173" t="n"/>
+      <c r="K41" s="1173" t="n"/>
+      <c r="L41" s="1173" t="n"/>
+      <c r="M41" s="1171" t="n"/>
+      <c r="N41" s="1171" t="n"/>
+      <c r="O41" s="1171" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1138" t="n">
+      <c r="P41" s="1174" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1135" t="n"/>
-      <c r="R41" s="1135" t="n">
+      <c r="Q41" s="1171" t="n"/>
+      <c r="R41" s="1171" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1135" t="n"/>
+      <c r="S41" s="1171" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1134" t="inlineStr">
+      <c r="U41" s="1170" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -6332,49 +6464,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1145" t="inlineStr">
+      <c r="A42" s="1181" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1146" t="inlineStr">
+      <c r="B42" s="1182" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1146" t="inlineStr">
+      <c r="C42" s="1182" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1147" t="n"/>
-      <c r="E42" s="1147" t="n"/>
-      <c r="F42" s="1147" t="n"/>
-      <c r="G42" s="1147" t="n"/>
-      <c r="H42" s="1147" t="n">
+      <c r="D42" s="1183" t="n"/>
+      <c r="E42" s="1183" t="n"/>
+      <c r="F42" s="1183" t="n"/>
+      <c r="G42" s="1183" t="n"/>
+      <c r="H42" s="1183" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1148" t="n"/>
-      <c r="J42" s="1149" t="n"/>
-      <c r="K42" s="1149" t="n"/>
-      <c r="L42" s="1149" t="n"/>
-      <c r="M42" s="1147" t="n">
+      <c r="I42" s="1184" t="n"/>
+      <c r="J42" s="1185" t="n"/>
+      <c r="K42" s="1185" t="n"/>
+      <c r="L42" s="1185" t="n"/>
+      <c r="M42" s="1183" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1147" t="n">
+      <c r="N42" s="1183" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1147" t="n"/>
-      <c r="P42" s="1150" t="n"/>
-      <c r="Q42" s="1147" t="n"/>
-      <c r="R42" s="1147" t="n"/>
-      <c r="S42" s="1147" t="n"/>
+      <c r="O42" s="1183" t="n"/>
+      <c r="P42" s="1186" t="n"/>
+      <c r="Q42" s="1183" t="n"/>
+      <c r="R42" s="1183" t="n"/>
+      <c r="S42" s="1183" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1146" t="n"/>
+      <c r="U42" s="1182" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -6382,57 +6514,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1121" t="inlineStr">
+      <c r="A43" s="1157" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1122" t="inlineStr">
+      <c r="B43" s="1158" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1122" t="inlineStr">
+      <c r="C43" s="1158" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1123" t="n"/>
-      <c r="E43" s="1123" t="n">
+      <c r="D43" s="1159" t="n"/>
+      <c r="E43" s="1159" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1123" t="n">
+      <c r="F43" s="1159" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1123" t="n">
+      <c r="G43" s="1159" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1123" t="n"/>
-      <c r="I43" s="1124" t="n">
+      <c r="H43" s="1159" t="n"/>
+      <c r="I43" s="1160" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1125" t="n"/>
-      <c r="K43" s="1125" t="n"/>
-      <c r="L43" s="1125" t="n"/>
-      <c r="M43" s="1123" t="n"/>
-      <c r="N43" s="1123" t="n"/>
-      <c r="O43" s="1123" t="n">
+      <c r="J43" s="1161" t="n"/>
+      <c r="K43" s="1161" t="n"/>
+      <c r="L43" s="1161" t="n"/>
+      <c r="M43" s="1159" t="n"/>
+      <c r="N43" s="1159" t="n"/>
+      <c r="O43" s="1159" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1126" t="n">
+      <c r="P43" s="1162" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1123" t="n"/>
-      <c r="R43" s="1123" t="n">
+      <c r="Q43" s="1159" t="n"/>
+      <c r="R43" s="1159" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1123" t="n"/>
+      <c r="S43" s="1159" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1122" t="n"/>
+      <c r="U43" s="1158" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -6440,45 +6572,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1151" t="inlineStr">
+      <c r="A44" s="1187" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1152" t="inlineStr">
+      <c r="B44" s="1188" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1152" t="inlineStr">
+      <c r="C44" s="1188" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1153" t="n"/>
-      <c r="E44" s="1153" t="n">
+      <c r="D44" s="1189" t="n"/>
+      <c r="E44" s="1189" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1153" t="n">
+      <c r="F44" s="1189" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1153" t="n"/>
-      <c r="H44" s="1153" t="n"/>
-      <c r="I44" s="1154" t="n"/>
-      <c r="J44" s="1155" t="n"/>
-      <c r="K44" s="1155" t="n"/>
-      <c r="L44" s="1155" t="n"/>
-      <c r="M44" s="1153" t="n"/>
-      <c r="N44" s="1153" t="n"/>
-      <c r="O44" s="1153" t="n"/>
-      <c r="P44" s="1156" t="n"/>
-      <c r="Q44" s="1153" t="n"/>
-      <c r="R44" s="1153" t="n"/>
-      <c r="S44" s="1153" t="n">
+      <c r="G44" s="1189" t="n"/>
+      <c r="H44" s="1189" t="n"/>
+      <c r="I44" s="1190" t="n"/>
+      <c r="J44" s="1191" t="n"/>
+      <c r="K44" s="1191" t="n"/>
+      <c r="L44" s="1191" t="n"/>
+      <c r="M44" s="1189" t="n"/>
+      <c r="N44" s="1189" t="n"/>
+      <c r="O44" s="1189" t="n"/>
+      <c r="P44" s="1192" t="n"/>
+      <c r="Q44" s="1189" t="n"/>
+      <c r="R44" s="1189" t="n"/>
+      <c r="S44" s="1189" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1152" t="inlineStr">
+      <c r="U44" s="1188" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -6490,52 +6622,112 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1127" t="inlineStr">
+      <c r="A45" s="1163" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1128" t="inlineStr">
+      <c r="B45" s="1164" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1128" t="inlineStr">
+      <c r="C45" s="1164" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1129" t="n"/>
-      <c r="E45" s="1129" t="n"/>
-      <c r="F45" s="1129" t="n"/>
-      <c r="G45" s="1129" t="n"/>
-      <c r="H45" s="1129" t="n">
+      <c r="D45" s="1165" t="n"/>
+      <c r="E45" s="1165" t="n"/>
+      <c r="F45" s="1165" t="n"/>
+      <c r="G45" s="1165" t="n"/>
+      <c r="H45" s="1165" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1130" t="n"/>
-      <c r="J45" s="1131" t="n"/>
-      <c r="K45" s="1131" t="n"/>
-      <c r="L45" s="1131" t="n"/>
-      <c r="M45" s="1129" t="n">
+      <c r="I45" s="1166" t="n"/>
+      <c r="J45" s="1167" t="n"/>
+      <c r="K45" s="1167" t="n"/>
+      <c r="L45" s="1167" t="n"/>
+      <c r="M45" s="1165" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1129" t="n">
+      <c r="N45" s="1165" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1129" t="n"/>
-      <c r="P45" s="1132" t="n"/>
-      <c r="Q45" s="1129" t="n"/>
-      <c r="R45" s="1129" t="n"/>
-      <c r="S45" s="1129" t="n"/>
+      <c r="O45" s="1165" t="n"/>
+      <c r="P45" s="1168" t="n"/>
+      <c r="Q45" s="1165" t="n"/>
+      <c r="R45" s="1165" t="n"/>
+      <c r="S45" s="1165" t="n"/>
       <c r="T45" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1128" t="n"/>
+      <c r="U45" s="1164" t="n"/>
       <c r="V45" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="1193" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B46" s="1194" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="C46" s="1194" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="D46" s="1195" t="n"/>
+      <c r="E46" s="1195" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="F46" s="1195" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G46" s="1195" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H46" s="1195" t="n"/>
+      <c r="I46" s="1196" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="J46" s="1197" t="n"/>
+      <c r="K46" s="1197" t="n"/>
+      <c r="L46" s="1197" t="n"/>
+      <c r="M46" s="1195" t="n"/>
+      <c r="N46" s="1195" t="n"/>
+      <c r="O46" s="1195" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="P46" s="1198" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="1195" t="n"/>
+      <c r="R46" s="1195" t="n">
+        <v>84.5</v>
+      </c>
+      <c r="S46" s="1195" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="T46" s="1199" t="inlineStr">
+        <is>
+          <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
+        </is>
+      </c>
+      <c r="U46" s="1194" t="n"/>
+      <c r="V46" s="1200" t="inlineStr">
+        <is>
+          <t>25mL x0.2. FC 16.6, CC 0.6. (John wrote 'CC=16.6' but that's FC; a 16.6 combined chlorine is implausible -- logged as FC.) FC loss 4.1 ppm/24h = 17.2 (7/2 NOON) + 1.0gal x3.5 - 16.6, computed noon-to-noon; NOT the 2.3 daily_calc.py reported (it used the 7/2 evening recheck 15.4 as baseline -&gt; ~16.5h window, non-comparable). WATCH: CC creeping 0.0 -&gt; 0.4 -&gt; 0.6 over ~24h; still a trace, and higher FC should oxidize it away, but note the direction -- flag if it climbs past ~1.0. Pred error +0.9 (actual 16.6 vs 7/2 dose's 15.7 projection): model over-predicted loss again but by less than 7/2's +2.1 -- two straight hot/sunny days where real loss ran under the L24=5.0 estimate; watch a 3rd before nudging dose.py's l24_hot_sunny down. Water level 11.8 cm (was 11.9 on 7/2; -0.1 within ruler/reading noise, ruler adhesion still iffy). Hot day: high 94F, water 84.5F, ~13 sun hrs.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log 2026-07-03 evening: dose 1.0 gal @ 7:45pm (season 20.0), add 5 photos
Held FC up (full gallon despite FC 16.6) to clear the CC creep. Water
clear/healthy, no stain progression. One photo shows floating surface
debris -- likely the CC-creep source; recommend skimming. Projects ~15.1
next noon (7/4 forward-validation target).
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1201">
+  <cellXfs count="1237">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -4131,6 +4131,114 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4391,7 +4499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V46"/>
+  <dimension ref="A1:V47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -4568,35 +4676,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1157" t="inlineStr">
+      <c r="A3" s="1201" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1158" t="n"/>
-      <c r="C3" s="1158" t="inlineStr">
+      <c r="B3" s="1202" t="n"/>
+      <c r="C3" s="1202" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1159" t="n"/>
-      <c r="E3" s="1159" t="n"/>
-      <c r="F3" s="1159" t="n"/>
-      <c r="G3" s="1159" t="n"/>
-      <c r="H3" s="1159" t="n"/>
-      <c r="I3" s="1160" t="n"/>
-      <c r="J3" s="1161" t="n"/>
-      <c r="K3" s="1161" t="n"/>
-      <c r="L3" s="1161" t="n"/>
-      <c r="M3" s="1159" t="n"/>
-      <c r="N3" s="1159" t="n"/>
-      <c r="O3" s="1159" t="n"/>
-      <c r="P3" s="1162" t="n"/>
-      <c r="Q3" s="1159" t="n"/>
-      <c r="R3" s="1159" t="n"/>
-      <c r="S3" s="1159" t="n"/>
+      <c r="D3" s="1203" t="n"/>
+      <c r="E3" s="1203" t="n"/>
+      <c r="F3" s="1203" t="n"/>
+      <c r="G3" s="1203" t="n"/>
+      <c r="H3" s="1203" t="n"/>
+      <c r="I3" s="1204" t="n"/>
+      <c r="J3" s="1205" t="n"/>
+      <c r="K3" s="1205" t="n"/>
+      <c r="L3" s="1205" t="n"/>
+      <c r="M3" s="1203" t="n"/>
+      <c r="N3" s="1203" t="n"/>
+      <c r="O3" s="1203" t="n"/>
+      <c r="P3" s="1206" t="n"/>
+      <c r="Q3" s="1203" t="n"/>
+      <c r="R3" s="1203" t="n"/>
+      <c r="S3" s="1203" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1158" t="n"/>
+      <c r="U3" s="1202" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -4604,43 +4712,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1163" t="inlineStr">
+      <c r="A4" s="1207" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1164" t="inlineStr">
+      <c r="B4" s="1208" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1164" t="inlineStr">
+      <c r="C4" s="1208" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1165" t="n"/>
-      <c r="E4" s="1165" t="n"/>
-      <c r="F4" s="1165" t="n"/>
-      <c r="G4" s="1165" t="n"/>
-      <c r="H4" s="1165" t="n"/>
-      <c r="I4" s="1166" t="n"/>
-      <c r="J4" s="1167" t="n"/>
-      <c r="K4" s="1167" t="n"/>
-      <c r="L4" s="1167" t="n"/>
-      <c r="M4" s="1165" t="n">
+      <c r="D4" s="1209" t="n"/>
+      <c r="E4" s="1209" t="n"/>
+      <c r="F4" s="1209" t="n"/>
+      <c r="G4" s="1209" t="n"/>
+      <c r="H4" s="1209" t="n"/>
+      <c r="I4" s="1210" t="n"/>
+      <c r="J4" s="1211" t="n"/>
+      <c r="K4" s="1211" t="n"/>
+      <c r="L4" s="1211" t="n"/>
+      <c r="M4" s="1209" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1165" t="n">
+      <c r="N4" s="1209" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1165" t="n"/>
-      <c r="P4" s="1168" t="n"/>
-      <c r="Q4" s="1165" t="n"/>
-      <c r="R4" s="1165" t="n"/>
-      <c r="S4" s="1165" t="n"/>
+      <c r="O4" s="1209" t="n"/>
+      <c r="P4" s="1212" t="n"/>
+      <c r="Q4" s="1209" t="n"/>
+      <c r="R4" s="1209" t="n"/>
+      <c r="S4" s="1209" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1164" t="n"/>
+      <c r="U4" s="1208" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -4648,57 +4756,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1169" t="inlineStr">
+      <c r="A5" s="1213" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1170" t="inlineStr">
+      <c r="B5" s="1214" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1170" t="inlineStr">
+      <c r="C5" s="1214" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1171" t="n">
+      <c r="D5" s="1215" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1171" t="n">
+      <c r="E5" s="1215" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1171" t="n">
+      <c r="F5" s="1215" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1171" t="n"/>
-      <c r="H5" s="1171" t="n"/>
-      <c r="I5" s="1172" t="n"/>
-      <c r="J5" s="1173" t="n">
+      <c r="G5" s="1215" t="n"/>
+      <c r="H5" s="1215" t="n"/>
+      <c r="I5" s="1216" t="n"/>
+      <c r="J5" s="1217" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1173" t="n">
+      <c r="K5" s="1217" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1173" t="inlineStr">
+      <c r="L5" s="1217" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1171" t="n"/>
-      <c r="N5" s="1171" t="n"/>
-      <c r="O5" s="1171" t="n">
+      <c r="M5" s="1215" t="n"/>
+      <c r="N5" s="1215" t="n"/>
+      <c r="O5" s="1215" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1174" t="n">
+      <c r="P5" s="1218" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1171" t="n"/>
-      <c r="R5" s="1171" t="n"/>
-      <c r="S5" s="1171" t="n"/>
+      <c r="Q5" s="1215" t="n"/>
+      <c r="R5" s="1215" t="n"/>
+      <c r="S5" s="1215" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1170" t="n"/>
+      <c r="U5" s="1214" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -4706,43 +4814,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1175" t="inlineStr">
+      <c r="A6" s="1219" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1176" t="inlineStr">
+      <c r="B6" s="1220" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1176" t="inlineStr">
+      <c r="C6" s="1220" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1177" t="n"/>
-      <c r="E6" s="1177" t="n"/>
-      <c r="F6" s="1177" t="n"/>
-      <c r="G6" s="1177" t="n"/>
-      <c r="H6" s="1177" t="n"/>
-      <c r="I6" s="1178" t="n"/>
-      <c r="J6" s="1179" t="n"/>
-      <c r="K6" s="1179" t="n"/>
-      <c r="L6" s="1179" t="n"/>
-      <c r="M6" s="1177" t="n">
+      <c r="D6" s="1221" t="n"/>
+      <c r="E6" s="1221" t="n"/>
+      <c r="F6" s="1221" t="n"/>
+      <c r="G6" s="1221" t="n"/>
+      <c r="H6" s="1221" t="n"/>
+      <c r="I6" s="1222" t="n"/>
+      <c r="J6" s="1223" t="n"/>
+      <c r="K6" s="1223" t="n"/>
+      <c r="L6" s="1223" t="n"/>
+      <c r="M6" s="1221" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1177" t="n">
+      <c r="N6" s="1221" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1177" t="n"/>
-      <c r="P6" s="1180" t="n"/>
-      <c r="Q6" s="1177" t="n"/>
-      <c r="R6" s="1177" t="n"/>
-      <c r="S6" s="1177" t="n"/>
+      <c r="O6" s="1221" t="n"/>
+      <c r="P6" s="1224" t="n"/>
+      <c r="Q6" s="1221" t="n"/>
+      <c r="R6" s="1221" t="n"/>
+      <c r="S6" s="1221" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1176" t="n"/>
+      <c r="U6" s="1220" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -4750,39 +4858,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1181" t="inlineStr">
+      <c r="A7" s="1225" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1182" t="inlineStr">
+      <c r="B7" s="1226" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1182" t="inlineStr">
+      <c r="C7" s="1226" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1183" t="n"/>
-      <c r="E7" s="1183" t="n"/>
-      <c r="F7" s="1183" t="n"/>
-      <c r="G7" s="1183" t="n"/>
-      <c r="H7" s="1183" t="n"/>
-      <c r="I7" s="1184" t="n"/>
-      <c r="J7" s="1185" t="n"/>
-      <c r="K7" s="1185" t="n"/>
-      <c r="L7" s="1185" t="n"/>
-      <c r="M7" s="1183" t="n"/>
-      <c r="N7" s="1183" t="n"/>
-      <c r="O7" s="1183" t="n"/>
-      <c r="P7" s="1186" t="n"/>
-      <c r="Q7" s="1183" t="n"/>
-      <c r="R7" s="1183" t="n"/>
-      <c r="S7" s="1183" t="n"/>
+      <c r="D7" s="1227" t="n"/>
+      <c r="E7" s="1227" t="n"/>
+      <c r="F7" s="1227" t="n"/>
+      <c r="G7" s="1227" t="n"/>
+      <c r="H7" s="1227" t="n"/>
+      <c r="I7" s="1228" t="n"/>
+      <c r="J7" s="1229" t="n"/>
+      <c r="K7" s="1229" t="n"/>
+      <c r="L7" s="1229" t="n"/>
+      <c r="M7" s="1227" t="n"/>
+      <c r="N7" s="1227" t="n"/>
+      <c r="O7" s="1227" t="n"/>
+      <c r="P7" s="1230" t="n"/>
+      <c r="Q7" s="1227" t="n"/>
+      <c r="R7" s="1227" t="n"/>
+      <c r="S7" s="1227" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1182" t="n"/>
+      <c r="U7" s="1226" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -4790,39 +4898,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1157" t="inlineStr">
+      <c r="A8" s="1201" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1158" t="inlineStr">
+      <c r="B8" s="1202" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1158" t="inlineStr">
+      <c r="C8" s="1202" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1159" t="n"/>
-      <c r="E8" s="1159" t="n"/>
-      <c r="F8" s="1159" t="n"/>
-      <c r="G8" s="1159" t="n"/>
-      <c r="H8" s="1159" t="n"/>
-      <c r="I8" s="1160" t="n"/>
-      <c r="J8" s="1161" t="n"/>
-      <c r="K8" s="1161" t="n"/>
-      <c r="L8" s="1161" t="n"/>
-      <c r="M8" s="1159" t="n"/>
-      <c r="N8" s="1159" t="n"/>
-      <c r="O8" s="1159" t="n"/>
-      <c r="P8" s="1162" t="n"/>
-      <c r="Q8" s="1159" t="n"/>
-      <c r="R8" s="1159" t="n"/>
-      <c r="S8" s="1159" t="n"/>
+      <c r="D8" s="1203" t="n"/>
+      <c r="E8" s="1203" t="n"/>
+      <c r="F8" s="1203" t="n"/>
+      <c r="G8" s="1203" t="n"/>
+      <c r="H8" s="1203" t="n"/>
+      <c r="I8" s="1204" t="n"/>
+      <c r="J8" s="1205" t="n"/>
+      <c r="K8" s="1205" t="n"/>
+      <c r="L8" s="1205" t="n"/>
+      <c r="M8" s="1203" t="n"/>
+      <c r="N8" s="1203" t="n"/>
+      <c r="O8" s="1203" t="n"/>
+      <c r="P8" s="1206" t="n"/>
+      <c r="Q8" s="1203" t="n"/>
+      <c r="R8" s="1203" t="n"/>
+      <c r="S8" s="1203" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1158" t="n"/>
+      <c r="U8" s="1202" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -4830,63 +4938,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1187" t="inlineStr">
+      <c r="A9" s="1231" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1188" t="inlineStr">
+      <c r="B9" s="1232" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1188" t="inlineStr">
+      <c r="C9" s="1232" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1189" t="n">
+      <c r="D9" s="1233" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1189" t="n">
+      <c r="E9" s="1233" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1189" t="n">
+      <c r="F9" s="1233" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1189" t="n">
+      <c r="G9" s="1233" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1189" t="n"/>
-      <c r="I9" s="1190" t="n"/>
-      <c r="J9" s="1191" t="n">
+      <c r="H9" s="1233" t="n"/>
+      <c r="I9" s="1234" t="n"/>
+      <c r="J9" s="1235" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1191" t="n">
+      <c r="K9" s="1235" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1191" t="inlineStr">
+      <c r="L9" s="1235" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1189" t="n"/>
-      <c r="N9" s="1189" t="n"/>
-      <c r="O9" s="1189" t="n">
+      <c r="M9" s="1233" t="n"/>
+      <c r="N9" s="1233" t="n"/>
+      <c r="O9" s="1233" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1192" t="n">
+      <c r="P9" s="1236" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1189" t="n"/>
-      <c r="R9" s="1189" t="n"/>
-      <c r="S9" s="1189" t="n"/>
+      <c r="Q9" s="1233" t="n"/>
+      <c r="R9" s="1233" t="n"/>
+      <c r="S9" s="1233" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1188" t="n"/>
+      <c r="U9" s="1232" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -4894,43 +5002,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1187" t="inlineStr">
+      <c r="A10" s="1231" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1188" t="inlineStr">
+      <c r="B10" s="1232" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1188" t="inlineStr">
+      <c r="C10" s="1232" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1189" t="n"/>
-      <c r="E10" s="1189" t="n"/>
-      <c r="F10" s="1189" t="n"/>
-      <c r="G10" s="1189" t="n"/>
-      <c r="H10" s="1189" t="n"/>
-      <c r="I10" s="1190" t="n"/>
-      <c r="J10" s="1191" t="n"/>
-      <c r="K10" s="1191" t="n"/>
-      <c r="L10" s="1191" t="inlineStr">
+      <c r="D10" s="1233" t="n"/>
+      <c r="E10" s="1233" t="n"/>
+      <c r="F10" s="1233" t="n"/>
+      <c r="G10" s="1233" t="n"/>
+      <c r="H10" s="1233" t="n"/>
+      <c r="I10" s="1234" t="n"/>
+      <c r="J10" s="1235" t="n"/>
+      <c r="K10" s="1235" t="n"/>
+      <c r="L10" s="1235" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1189" t="n"/>
-      <c r="N10" s="1189" t="n"/>
-      <c r="O10" s="1189" t="n"/>
-      <c r="P10" s="1192" t="n"/>
-      <c r="Q10" s="1189" t="n"/>
-      <c r="R10" s="1189" t="n"/>
-      <c r="S10" s="1189" t="n"/>
+      <c r="M10" s="1233" t="n"/>
+      <c r="N10" s="1233" t="n"/>
+      <c r="O10" s="1233" t="n"/>
+      <c r="P10" s="1236" t="n"/>
+      <c r="Q10" s="1233" t="n"/>
+      <c r="R10" s="1233" t="n"/>
+      <c r="S10" s="1233" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1188" t="n"/>
+      <c r="U10" s="1232" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -4938,43 +5046,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1187" t="inlineStr">
+      <c r="A11" s="1231" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1188" t="inlineStr">
+      <c r="B11" s="1232" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1188" t="inlineStr">
+      <c r="C11" s="1232" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1189" t="n"/>
-      <c r="E11" s="1189" t="n"/>
-      <c r="F11" s="1189" t="n"/>
-      <c r="G11" s="1189" t="n"/>
-      <c r="H11" s="1189" t="n"/>
-      <c r="I11" s="1190" t="n"/>
-      <c r="J11" s="1191" t="n"/>
-      <c r="K11" s="1191" t="n"/>
-      <c r="L11" s="1191" t="n"/>
-      <c r="M11" s="1189" t="n">
+      <c r="D11" s="1233" t="n"/>
+      <c r="E11" s="1233" t="n"/>
+      <c r="F11" s="1233" t="n"/>
+      <c r="G11" s="1233" t="n"/>
+      <c r="H11" s="1233" t="n"/>
+      <c r="I11" s="1234" t="n"/>
+      <c r="J11" s="1235" t="n"/>
+      <c r="K11" s="1235" t="n"/>
+      <c r="L11" s="1235" t="n"/>
+      <c r="M11" s="1233" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1189" t="n">
+      <c r="N11" s="1233" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1189" t="n"/>
-      <c r="P11" s="1192" t="n"/>
-      <c r="Q11" s="1189" t="n"/>
-      <c r="R11" s="1189" t="n"/>
-      <c r="S11" s="1189" t="n"/>
+      <c r="O11" s="1233" t="n"/>
+      <c r="P11" s="1236" t="n"/>
+      <c r="Q11" s="1233" t="n"/>
+      <c r="R11" s="1233" t="n"/>
+      <c r="S11" s="1233" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1188" t="n"/>
+      <c r="U11" s="1232" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -4982,39 +5090,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1163" t="inlineStr">
+      <c r="A12" s="1207" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1164" t="inlineStr">
+      <c r="B12" s="1208" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1164" t="inlineStr">
+      <c r="C12" s="1208" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1165" t="n"/>
-      <c r="E12" s="1165" t="n"/>
-      <c r="F12" s="1165" t="n"/>
-      <c r="G12" s="1165" t="n"/>
-      <c r="H12" s="1165" t="n"/>
-      <c r="I12" s="1166" t="n"/>
-      <c r="J12" s="1167" t="n"/>
-      <c r="K12" s="1167" t="n"/>
-      <c r="L12" s="1167" t="n"/>
-      <c r="M12" s="1165" t="n"/>
-      <c r="N12" s="1165" t="n"/>
-      <c r="O12" s="1165" t="n"/>
-      <c r="P12" s="1168" t="n"/>
-      <c r="Q12" s="1165" t="n"/>
-      <c r="R12" s="1165" t="n"/>
-      <c r="S12" s="1165" t="n"/>
+      <c r="D12" s="1209" t="n"/>
+      <c r="E12" s="1209" t="n"/>
+      <c r="F12" s="1209" t="n"/>
+      <c r="G12" s="1209" t="n"/>
+      <c r="H12" s="1209" t="n"/>
+      <c r="I12" s="1210" t="n"/>
+      <c r="J12" s="1211" t="n"/>
+      <c r="K12" s="1211" t="n"/>
+      <c r="L12" s="1211" t="n"/>
+      <c r="M12" s="1209" t="n"/>
+      <c r="N12" s="1209" t="n"/>
+      <c r="O12" s="1209" t="n"/>
+      <c r="P12" s="1212" t="n"/>
+      <c r="Q12" s="1209" t="n"/>
+      <c r="R12" s="1209" t="n"/>
+      <c r="S12" s="1209" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1164" t="n"/>
+      <c r="U12" s="1208" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5022,35 +5130,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1169" t="inlineStr">
+      <c r="A13" s="1213" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1170" t="n"/>
-      <c r="C13" s="1170" t="inlineStr">
+      <c r="B13" s="1214" t="n"/>
+      <c r="C13" s="1214" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1171" t="n"/>
-      <c r="E13" s="1171" t="n"/>
-      <c r="F13" s="1171" t="n"/>
-      <c r="G13" s="1171" t="n"/>
-      <c r="H13" s="1171" t="n"/>
-      <c r="I13" s="1172" t="n"/>
-      <c r="J13" s="1173" t="n"/>
-      <c r="K13" s="1173" t="n"/>
-      <c r="L13" s="1173" t="n"/>
-      <c r="M13" s="1171" t="n"/>
-      <c r="N13" s="1171" t="n"/>
-      <c r="O13" s="1171" t="n"/>
-      <c r="P13" s="1174" t="n"/>
-      <c r="Q13" s="1171" t="n"/>
-      <c r="R13" s="1171" t="n"/>
-      <c r="S13" s="1171" t="n"/>
+      <c r="D13" s="1215" t="n"/>
+      <c r="E13" s="1215" t="n"/>
+      <c r="F13" s="1215" t="n"/>
+      <c r="G13" s="1215" t="n"/>
+      <c r="H13" s="1215" t="n"/>
+      <c r="I13" s="1216" t="n"/>
+      <c r="J13" s="1217" t="n"/>
+      <c r="K13" s="1217" t="n"/>
+      <c r="L13" s="1217" t="n"/>
+      <c r="M13" s="1215" t="n"/>
+      <c r="N13" s="1215" t="n"/>
+      <c r="O13" s="1215" t="n"/>
+      <c r="P13" s="1218" t="n"/>
+      <c r="Q13" s="1215" t="n"/>
+      <c r="R13" s="1215" t="n"/>
+      <c r="S13" s="1215" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1170" t="n"/>
+      <c r="U13" s="1214" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -5058,53 +5166,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1175" t="inlineStr">
+      <c r="A14" s="1219" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1176" t="inlineStr">
+      <c r="B14" s="1220" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1176" t="inlineStr">
+      <c r="C14" s="1220" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1177" t="n"/>
-      <c r="E14" s="1177" t="n">
+      <c r="D14" s="1221" t="n"/>
+      <c r="E14" s="1221" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1177" t="n">
+      <c r="F14" s="1221" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1177" t="n">
+      <c r="G14" s="1221" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1177" t="n"/>
-      <c r="I14" s="1178" t="n"/>
-      <c r="J14" s="1179" t="n"/>
-      <c r="K14" s="1179" t="n"/>
-      <c r="L14" s="1179" t="n"/>
-      <c r="M14" s="1177" t="n"/>
-      <c r="N14" s="1177" t="n"/>
-      <c r="O14" s="1177" t="n">
+      <c r="H14" s="1221" t="n"/>
+      <c r="I14" s="1222" t="n"/>
+      <c r="J14" s="1223" t="n"/>
+      <c r="K14" s="1223" t="n"/>
+      <c r="L14" s="1223" t="n"/>
+      <c r="M14" s="1221" t="n"/>
+      <c r="N14" s="1221" t="n"/>
+      <c r="O14" s="1221" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1180" t="n">
+      <c r="P14" s="1224" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1177" t="n"/>
-      <c r="R14" s="1177" t="n"/>
-      <c r="S14" s="1177" t="n"/>
+      <c r="Q14" s="1221" t="n"/>
+      <c r="R14" s="1221" t="n"/>
+      <c r="S14" s="1221" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1176" t="n"/>
+      <c r="U14" s="1220" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -5112,43 +5220,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1175" t="inlineStr">
+      <c r="A15" s="1219" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1176" t="inlineStr">
+      <c r="B15" s="1220" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1176" t="inlineStr">
+      <c r="C15" s="1220" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1177" t="n"/>
-      <c r="E15" s="1177" t="n"/>
-      <c r="F15" s="1177" t="n"/>
-      <c r="G15" s="1177" t="n"/>
-      <c r="H15" s="1177" t="n"/>
-      <c r="I15" s="1178" t="n"/>
-      <c r="J15" s="1179" t="n"/>
-      <c r="K15" s="1179" t="n"/>
-      <c r="L15" s="1179" t="n"/>
-      <c r="M15" s="1177" t="n">
+      <c r="D15" s="1221" t="n"/>
+      <c r="E15" s="1221" t="n"/>
+      <c r="F15" s="1221" t="n"/>
+      <c r="G15" s="1221" t="n"/>
+      <c r="H15" s="1221" t="n"/>
+      <c r="I15" s="1222" t="n"/>
+      <c r="J15" s="1223" t="n"/>
+      <c r="K15" s="1223" t="n"/>
+      <c r="L15" s="1223" t="n"/>
+      <c r="M15" s="1221" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1177" t="n">
+      <c r="N15" s="1221" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1177" t="n"/>
-      <c r="P15" s="1180" t="n"/>
-      <c r="Q15" s="1177" t="n"/>
-      <c r="R15" s="1177" t="n"/>
-      <c r="S15" s="1177" t="n"/>
+      <c r="O15" s="1221" t="n"/>
+      <c r="P15" s="1224" t="n"/>
+      <c r="Q15" s="1221" t="n"/>
+      <c r="R15" s="1221" t="n"/>
+      <c r="S15" s="1221" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1176" t="n"/>
+      <c r="U15" s="1220" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -5156,39 +5264,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1181" t="inlineStr">
+      <c r="A16" s="1225" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1182" t="inlineStr">
+      <c r="B16" s="1226" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1182" t="inlineStr">
+      <c r="C16" s="1226" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1183" t="n"/>
-      <c r="E16" s="1183" t="n"/>
-      <c r="F16" s="1183" t="n"/>
-      <c r="G16" s="1183" t="n"/>
-      <c r="H16" s="1183" t="n"/>
-      <c r="I16" s="1184" t="n"/>
-      <c r="J16" s="1185" t="n"/>
-      <c r="K16" s="1185" t="n"/>
-      <c r="L16" s="1185" t="n"/>
-      <c r="M16" s="1183" t="n"/>
-      <c r="N16" s="1183" t="n"/>
-      <c r="O16" s="1183" t="n"/>
-      <c r="P16" s="1186" t="n"/>
-      <c r="Q16" s="1183" t="n"/>
-      <c r="R16" s="1183" t="n"/>
-      <c r="S16" s="1183" t="n"/>
+      <c r="D16" s="1227" t="n"/>
+      <c r="E16" s="1227" t="n"/>
+      <c r="F16" s="1227" t="n"/>
+      <c r="G16" s="1227" t="n"/>
+      <c r="H16" s="1227" t="n"/>
+      <c r="I16" s="1228" t="n"/>
+      <c r="J16" s="1229" t="n"/>
+      <c r="K16" s="1229" t="n"/>
+      <c r="L16" s="1229" t="n"/>
+      <c r="M16" s="1227" t="n"/>
+      <c r="N16" s="1227" t="n"/>
+      <c r="O16" s="1227" t="n"/>
+      <c r="P16" s="1230" t="n"/>
+      <c r="Q16" s="1227" t="n"/>
+      <c r="R16" s="1227" t="n"/>
+      <c r="S16" s="1227" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1182" t="n"/>
+      <c r="U16" s="1226" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -5196,39 +5304,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1157" t="inlineStr">
+      <c r="A17" s="1201" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1158" t="inlineStr">
+      <c r="B17" s="1202" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1158" t="inlineStr">
+      <c r="C17" s="1202" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1159" t="n"/>
-      <c r="E17" s="1159" t="n"/>
-      <c r="F17" s="1159" t="n"/>
-      <c r="G17" s="1159" t="n"/>
-      <c r="H17" s="1159" t="n"/>
-      <c r="I17" s="1160" t="n"/>
-      <c r="J17" s="1161" t="n"/>
-      <c r="K17" s="1161" t="n"/>
-      <c r="L17" s="1161" t="n"/>
-      <c r="M17" s="1159" t="n"/>
-      <c r="N17" s="1159" t="n"/>
-      <c r="O17" s="1159" t="n"/>
-      <c r="P17" s="1162" t="n"/>
-      <c r="Q17" s="1159" t="n"/>
-      <c r="R17" s="1159" t="n"/>
-      <c r="S17" s="1159" t="n"/>
+      <c r="D17" s="1203" t="n"/>
+      <c r="E17" s="1203" t="n"/>
+      <c r="F17" s="1203" t="n"/>
+      <c r="G17" s="1203" t="n"/>
+      <c r="H17" s="1203" t="n"/>
+      <c r="I17" s="1204" t="n"/>
+      <c r="J17" s="1205" t="n"/>
+      <c r="K17" s="1205" t="n"/>
+      <c r="L17" s="1205" t="n"/>
+      <c r="M17" s="1203" t="n"/>
+      <c r="N17" s="1203" t="n"/>
+      <c r="O17" s="1203" t="n"/>
+      <c r="P17" s="1206" t="n"/>
+      <c r="Q17" s="1203" t="n"/>
+      <c r="R17" s="1203" t="n"/>
+      <c r="S17" s="1203" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1158" t="n"/>
+      <c r="U17" s="1202" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -5236,53 +5344,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1187" t="inlineStr">
+      <c r="A18" s="1231" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1188" t="inlineStr">
+      <c r="B18" s="1232" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1188" t="inlineStr">
+      <c r="C18" s="1232" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1189" t="n"/>
-      <c r="E18" s="1189" t="n">
+      <c r="D18" s="1233" t="n"/>
+      <c r="E18" s="1233" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1189" t="n">
+      <c r="F18" s="1233" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1189" t="n">
+      <c r="G18" s="1233" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1189" t="n"/>
-      <c r="I18" s="1190" t="n"/>
-      <c r="J18" s="1191" t="n"/>
-      <c r="K18" s="1191" t="n"/>
-      <c r="L18" s="1191" t="n"/>
-      <c r="M18" s="1189" t="n"/>
-      <c r="N18" s="1189" t="n"/>
-      <c r="O18" s="1189" t="n">
+      <c r="H18" s="1233" t="n"/>
+      <c r="I18" s="1234" t="n"/>
+      <c r="J18" s="1235" t="n"/>
+      <c r="K18" s="1235" t="n"/>
+      <c r="L18" s="1235" t="n"/>
+      <c r="M18" s="1233" t="n"/>
+      <c r="N18" s="1233" t="n"/>
+      <c r="O18" s="1233" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1192" t="n">
+      <c r="P18" s="1236" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1189" t="n"/>
-      <c r="R18" s="1189" t="n"/>
-      <c r="S18" s="1189" t="n"/>
+      <c r="Q18" s="1233" t="n"/>
+      <c r="R18" s="1233" t="n"/>
+      <c r="S18" s="1233" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1188" t="n"/>
+      <c r="U18" s="1232" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -5290,47 +5398,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1187" t="inlineStr">
+      <c r="A19" s="1231" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1188" t="inlineStr">
+      <c r="B19" s="1232" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1188" t="inlineStr">
+      <c r="C19" s="1232" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1189" t="n"/>
-      <c r="E19" s="1189" t="n"/>
-      <c r="F19" s="1189" t="n"/>
-      <c r="G19" s="1189" t="n"/>
-      <c r="H19" s="1189" t="n"/>
-      <c r="I19" s="1190" t="n"/>
-      <c r="J19" s="1191" t="n"/>
-      <c r="K19" s="1191" t="n"/>
-      <c r="L19" s="1191" t="n"/>
-      <c r="M19" s="1189" t="n">
+      <c r="D19" s="1233" t="n"/>
+      <c r="E19" s="1233" t="n"/>
+      <c r="F19" s="1233" t="n"/>
+      <c r="G19" s="1233" t="n"/>
+      <c r="H19" s="1233" t="n"/>
+      <c r="I19" s="1234" t="n"/>
+      <c r="J19" s="1235" t="n"/>
+      <c r="K19" s="1235" t="n"/>
+      <c r="L19" s="1235" t="n"/>
+      <c r="M19" s="1233" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1189" t="n">
+      <c r="N19" s="1233" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1189" t="n"/>
-      <c r="P19" s="1192" t="n"/>
-      <c r="Q19" s="1189" t="n"/>
-      <c r="R19" s="1189" t="n"/>
-      <c r="S19" s="1189" t="n"/>
+      <c r="O19" s="1233" t="n"/>
+      <c r="P19" s="1236" t="n"/>
+      <c r="Q19" s="1233" t="n"/>
+      <c r="R19" s="1233" t="n"/>
+      <c r="S19" s="1233" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1188" t="n"/>
+      <c r="U19" s="1232" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -5338,43 +5446,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1187" t="inlineStr">
+      <c r="A20" s="1231" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1188" t="inlineStr">
+      <c r="B20" s="1232" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1188" t="inlineStr">
+      <c r="C20" s="1232" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1189" t="n"/>
-      <c r="E20" s="1189" t="n"/>
-      <c r="F20" s="1189" t="n"/>
-      <c r="G20" s="1189" t="n"/>
-      <c r="H20" s="1189" t="n"/>
-      <c r="I20" s="1190" t="n"/>
-      <c r="J20" s="1191" t="n"/>
-      <c r="K20" s="1191" t="n"/>
-      <c r="L20" s="1191" t="n"/>
-      <c r="M20" s="1189" t="n"/>
-      <c r="N20" s="1189" t="n"/>
-      <c r="O20" s="1189" t="n"/>
-      <c r="P20" s="1192" t="n"/>
-      <c r="Q20" s="1189" t="n"/>
-      <c r="R20" s="1189" t="n"/>
-      <c r="S20" s="1189" t="n"/>
+      <c r="D20" s="1233" t="n"/>
+      <c r="E20" s="1233" t="n"/>
+      <c r="F20" s="1233" t="n"/>
+      <c r="G20" s="1233" t="n"/>
+      <c r="H20" s="1233" t="n"/>
+      <c r="I20" s="1234" t="n"/>
+      <c r="J20" s="1235" t="n"/>
+      <c r="K20" s="1235" t="n"/>
+      <c r="L20" s="1235" t="n"/>
+      <c r="M20" s="1233" t="n"/>
+      <c r="N20" s="1233" t="n"/>
+      <c r="O20" s="1233" t="n"/>
+      <c r="P20" s="1236" t="n"/>
+      <c r="Q20" s="1233" t="n"/>
+      <c r="R20" s="1233" t="n"/>
+      <c r="S20" s="1233" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1188" t="n"/>
+      <c r="U20" s="1232" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -5382,39 +5490,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1163" t="inlineStr">
+      <c r="A21" s="1207" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1164" t="inlineStr">
+      <c r="B21" s="1208" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1164" t="inlineStr">
+      <c r="C21" s="1208" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1165" t="n"/>
-      <c r="E21" s="1165" t="n"/>
-      <c r="F21" s="1165" t="n"/>
-      <c r="G21" s="1165" t="n"/>
-      <c r="H21" s="1165" t="n"/>
-      <c r="I21" s="1166" t="n"/>
-      <c r="J21" s="1167" t="n"/>
-      <c r="K21" s="1167" t="n"/>
-      <c r="L21" s="1167" t="n"/>
-      <c r="M21" s="1165" t="n"/>
-      <c r="N21" s="1165" t="n"/>
-      <c r="O21" s="1165" t="n"/>
-      <c r="P21" s="1168" t="n"/>
-      <c r="Q21" s="1165" t="n"/>
-      <c r="R21" s="1165" t="n"/>
-      <c r="S21" s="1165" t="n"/>
+      <c r="D21" s="1209" t="n"/>
+      <c r="E21" s="1209" t="n"/>
+      <c r="F21" s="1209" t="n"/>
+      <c r="G21" s="1209" t="n"/>
+      <c r="H21" s="1209" t="n"/>
+      <c r="I21" s="1210" t="n"/>
+      <c r="J21" s="1211" t="n"/>
+      <c r="K21" s="1211" t="n"/>
+      <c r="L21" s="1211" t="n"/>
+      <c r="M21" s="1209" t="n"/>
+      <c r="N21" s="1209" t="n"/>
+      <c r="O21" s="1209" t="n"/>
+      <c r="P21" s="1212" t="n"/>
+      <c r="Q21" s="1209" t="n"/>
+      <c r="R21" s="1209" t="n"/>
+      <c r="S21" s="1209" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1164" t="n"/>
+      <c r="U21" s="1208" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -5422,39 +5530,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1169" t="inlineStr">
+      <c r="A22" s="1213" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1170" t="inlineStr">
+      <c r="B22" s="1214" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1170" t="inlineStr">
+      <c r="C22" s="1214" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1171" t="n"/>
-      <c r="E22" s="1171" t="n"/>
-      <c r="F22" s="1171" t="n"/>
-      <c r="G22" s="1171" t="n"/>
-      <c r="H22" s="1171" t="n"/>
-      <c r="I22" s="1172" t="n"/>
-      <c r="J22" s="1173" t="n"/>
-      <c r="K22" s="1173" t="n"/>
-      <c r="L22" s="1173" t="n"/>
-      <c r="M22" s="1171" t="n"/>
-      <c r="N22" s="1171" t="n"/>
-      <c r="O22" s="1171" t="n"/>
-      <c r="P22" s="1174" t="n"/>
-      <c r="Q22" s="1171" t="n"/>
-      <c r="R22" s="1171" t="n"/>
-      <c r="S22" s="1171" t="n"/>
+      <c r="D22" s="1215" t="n"/>
+      <c r="E22" s="1215" t="n"/>
+      <c r="F22" s="1215" t="n"/>
+      <c r="G22" s="1215" t="n"/>
+      <c r="H22" s="1215" t="n"/>
+      <c r="I22" s="1216" t="n"/>
+      <c r="J22" s="1217" t="n"/>
+      <c r="K22" s="1217" t="n"/>
+      <c r="L22" s="1217" t="n"/>
+      <c r="M22" s="1215" t="n"/>
+      <c r="N22" s="1215" t="n"/>
+      <c r="O22" s="1215" t="n"/>
+      <c r="P22" s="1218" t="n"/>
+      <c r="Q22" s="1215" t="n"/>
+      <c r="R22" s="1215" t="n"/>
+      <c r="S22" s="1215" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1170" t="n"/>
+      <c r="U22" s="1214" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -5462,53 +5570,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1175" t="inlineStr">
+      <c r="A23" s="1219" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1176" t="inlineStr">
+      <c r="B23" s="1220" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1176" t="inlineStr">
+      <c r="C23" s="1220" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1177" t="n"/>
-      <c r="E23" s="1177" t="n">
+      <c r="D23" s="1221" t="n"/>
+      <c r="E23" s="1221" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1177" t="n">
+      <c r="F23" s="1221" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1177" t="n">
+      <c r="G23" s="1221" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1177" t="n"/>
-      <c r="I23" s="1178" t="n"/>
-      <c r="J23" s="1179" t="n"/>
-      <c r="K23" s="1179" t="n"/>
-      <c r="L23" s="1179" t="n"/>
-      <c r="M23" s="1177" t="n"/>
-      <c r="N23" s="1177" t="n"/>
-      <c r="O23" s="1177" t="n">
+      <c r="H23" s="1221" t="n"/>
+      <c r="I23" s="1222" t="n"/>
+      <c r="J23" s="1223" t="n"/>
+      <c r="K23" s="1223" t="n"/>
+      <c r="L23" s="1223" t="n"/>
+      <c r="M23" s="1221" t="n"/>
+      <c r="N23" s="1221" t="n"/>
+      <c r="O23" s="1221" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1180" t="n">
+      <c r="P23" s="1224" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1177" t="n"/>
-      <c r="R23" s="1177" t="n"/>
-      <c r="S23" s="1177" t="n"/>
+      <c r="Q23" s="1221" t="n"/>
+      <c r="R23" s="1221" t="n"/>
+      <c r="S23" s="1221" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1176" t="n"/>
+      <c r="U23" s="1220" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -5516,47 +5624,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1181" t="inlineStr">
+      <c r="A24" s="1225" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1182" t="inlineStr">
+      <c r="B24" s="1226" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1182" t="inlineStr">
+      <c r="C24" s="1226" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1183" t="n"/>
-      <c r="E24" s="1183" t="n"/>
-      <c r="F24" s="1183" t="n"/>
-      <c r="G24" s="1183" t="n"/>
-      <c r="H24" s="1183" t="n"/>
-      <c r="I24" s="1184" t="n"/>
-      <c r="J24" s="1185" t="n"/>
-      <c r="K24" s="1185" t="n"/>
-      <c r="L24" s="1185" t="n"/>
-      <c r="M24" s="1183" t="n">
+      <c r="D24" s="1227" t="n"/>
+      <c r="E24" s="1227" t="n"/>
+      <c r="F24" s="1227" t="n"/>
+      <c r="G24" s="1227" t="n"/>
+      <c r="H24" s="1227" t="n"/>
+      <c r="I24" s="1228" t="n"/>
+      <c r="J24" s="1229" t="n"/>
+      <c r="K24" s="1229" t="n"/>
+      <c r="L24" s="1229" t="n"/>
+      <c r="M24" s="1227" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1183" t="n">
+      <c r="N24" s="1227" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1183" t="n"/>
-      <c r="P24" s="1186" t="n"/>
-      <c r="Q24" s="1183" t="n"/>
-      <c r="R24" s="1183" t="n"/>
-      <c r="S24" s="1183" t="n"/>
+      <c r="O24" s="1227" t="n"/>
+      <c r="P24" s="1230" t="n"/>
+      <c r="Q24" s="1227" t="n"/>
+      <c r="R24" s="1227" t="n"/>
+      <c r="S24" s="1227" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1182" t="n"/>
+      <c r="U24" s="1226" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -5564,61 +5672,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1157" t="inlineStr">
+      <c r="A25" s="1201" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1158" t="inlineStr">
+      <c r="B25" s="1202" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1158" t="inlineStr">
+      <c r="C25" s="1202" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1159" t="n">
+      <c r="D25" s="1203" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1159" t="n">
+      <c r="E25" s="1203" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1159" t="n">
+      <c r="F25" s="1203" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1159" t="n">
+      <c r="G25" s="1203" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1159" t="n"/>
-      <c r="I25" s="1160" t="n"/>
-      <c r="J25" s="1161" t="n">
+      <c r="H25" s="1203" t="n"/>
+      <c r="I25" s="1204" t="n"/>
+      <c r="J25" s="1205" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1161" t="n">
+      <c r="K25" s="1205" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1161" t="n">
+      <c r="L25" s="1205" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1159" t="n"/>
-      <c r="N25" s="1159" t="n"/>
-      <c r="O25" s="1159" t="n">
+      <c r="M25" s="1203" t="n"/>
+      <c r="N25" s="1203" t="n"/>
+      <c r="O25" s="1203" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1162" t="n">
+      <c r="P25" s="1206" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1159" t="n"/>
-      <c r="R25" s="1159" t="n"/>
-      <c r="S25" s="1159" t="n"/>
+      <c r="Q25" s="1203" t="n"/>
+      <c r="R25" s="1203" t="n"/>
+      <c r="S25" s="1203" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1158" t="n"/>
+      <c r="U25" s="1202" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -5626,47 +5734,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1163" t="inlineStr">
+      <c r="A26" s="1207" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1164" t="inlineStr">
+      <c r="B26" s="1208" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1164" t="inlineStr">
+      <c r="C26" s="1208" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1165" t="n"/>
-      <c r="E26" s="1165" t="n"/>
-      <c r="F26" s="1165" t="n"/>
-      <c r="G26" s="1165" t="n"/>
-      <c r="H26" s="1165" t="n"/>
-      <c r="I26" s="1166" t="n"/>
-      <c r="J26" s="1167" t="n"/>
-      <c r="K26" s="1167" t="n"/>
-      <c r="L26" s="1167" t="n"/>
-      <c r="M26" s="1165" t="n">
+      <c r="D26" s="1209" t="n"/>
+      <c r="E26" s="1209" t="n"/>
+      <c r="F26" s="1209" t="n"/>
+      <c r="G26" s="1209" t="n"/>
+      <c r="H26" s="1209" t="n"/>
+      <c r="I26" s="1210" t="n"/>
+      <c r="J26" s="1211" t="n"/>
+      <c r="K26" s="1211" t="n"/>
+      <c r="L26" s="1211" t="n"/>
+      <c r="M26" s="1209" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1165" t="n">
+      <c r="N26" s="1209" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1165" t="n"/>
-      <c r="P26" s="1168" t="n"/>
-      <c r="Q26" s="1165" t="n"/>
-      <c r="R26" s="1165" t="n"/>
-      <c r="S26" s="1165" t="n"/>
+      <c r="O26" s="1209" t="n"/>
+      <c r="P26" s="1212" t="n"/>
+      <c r="Q26" s="1209" t="n"/>
+      <c r="R26" s="1209" t="n"/>
+      <c r="S26" s="1209" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1164" t="n"/>
+      <c r="U26" s="1208" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -5674,53 +5782,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1169" t="inlineStr">
+      <c r="A27" s="1213" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1170" t="inlineStr">
+      <c r="B27" s="1214" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1170" t="inlineStr">
+      <c r="C27" s="1214" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1171" t="n"/>
-      <c r="E27" s="1171" t="n">
+      <c r="D27" s="1215" t="n"/>
+      <c r="E27" s="1215" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1171" t="n">
+      <c r="F27" s="1215" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1171" t="n">
+      <c r="G27" s="1215" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1171" t="n"/>
-      <c r="I27" s="1172" t="n"/>
-      <c r="J27" s="1173" t="n"/>
-      <c r="K27" s="1173" t="n"/>
-      <c r="L27" s="1173" t="n"/>
-      <c r="M27" s="1171" t="n"/>
-      <c r="N27" s="1171" t="n"/>
-      <c r="O27" s="1171" t="n">
+      <c r="H27" s="1215" t="n"/>
+      <c r="I27" s="1216" t="n"/>
+      <c r="J27" s="1217" t="n"/>
+      <c r="K27" s="1217" t="n"/>
+      <c r="L27" s="1217" t="n"/>
+      <c r="M27" s="1215" t="n"/>
+      <c r="N27" s="1215" t="n"/>
+      <c r="O27" s="1215" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1174" t="n">
+      <c r="P27" s="1218" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1171" t="n"/>
-      <c r="R27" s="1171" t="n"/>
-      <c r="S27" s="1171" t="n"/>
+      <c r="Q27" s="1215" t="n"/>
+      <c r="R27" s="1215" t="n"/>
+      <c r="S27" s="1215" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1170" t="n"/>
+      <c r="U27" s="1214" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -5728,47 +5836,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1181" t="inlineStr">
+      <c r="A28" s="1225" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1182" t="inlineStr">
+      <c r="B28" s="1226" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1182" t="inlineStr">
+      <c r="C28" s="1226" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1183" t="n"/>
-      <c r="E28" s="1183" t="n"/>
-      <c r="F28" s="1183" t="n"/>
-      <c r="G28" s="1183" t="n"/>
-      <c r="H28" s="1183" t="n"/>
-      <c r="I28" s="1184" t="n"/>
-      <c r="J28" s="1185" t="n"/>
-      <c r="K28" s="1185" t="n"/>
-      <c r="L28" s="1185" t="n"/>
-      <c r="M28" s="1183" t="n">
+      <c r="D28" s="1227" t="n"/>
+      <c r="E28" s="1227" t="n"/>
+      <c r="F28" s="1227" t="n"/>
+      <c r="G28" s="1227" t="n"/>
+      <c r="H28" s="1227" t="n"/>
+      <c r="I28" s="1228" t="n"/>
+      <c r="J28" s="1229" t="n"/>
+      <c r="K28" s="1229" t="n"/>
+      <c r="L28" s="1229" t="n"/>
+      <c r="M28" s="1227" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1183" t="n">
+      <c r="N28" s="1227" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1183" t="n"/>
-      <c r="P28" s="1186" t="n"/>
-      <c r="Q28" s="1183" t="n"/>
-      <c r="R28" s="1183" t="n"/>
-      <c r="S28" s="1183" t="n"/>
+      <c r="O28" s="1227" t="n"/>
+      <c r="P28" s="1230" t="n"/>
+      <c r="Q28" s="1227" t="n"/>
+      <c r="R28" s="1227" t="n"/>
+      <c r="S28" s="1227" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1182" t="n"/>
+      <c r="U28" s="1226" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -5776,53 +5884,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1157" t="inlineStr">
+      <c r="A29" s="1201" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1158" t="inlineStr">
+      <c r="B29" s="1202" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1158" t="inlineStr">
+      <c r="C29" s="1202" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1159" t="n"/>
-      <c r="E29" s="1159" t="n">
+      <c r="D29" s="1203" t="n"/>
+      <c r="E29" s="1203" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1159" t="n">
+      <c r="F29" s="1203" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1159" t="n">
+      <c r="G29" s="1203" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1159" t="n"/>
-      <c r="I29" s="1160" t="n"/>
-      <c r="J29" s="1161" t="n"/>
-      <c r="K29" s="1161" t="n"/>
-      <c r="L29" s="1161" t="n"/>
-      <c r="M29" s="1159" t="n"/>
-      <c r="N29" s="1159" t="n"/>
-      <c r="O29" s="1159" t="n">
+      <c r="H29" s="1203" t="n"/>
+      <c r="I29" s="1204" t="n"/>
+      <c r="J29" s="1205" t="n"/>
+      <c r="K29" s="1205" t="n"/>
+      <c r="L29" s="1205" t="n"/>
+      <c r="M29" s="1203" t="n"/>
+      <c r="N29" s="1203" t="n"/>
+      <c r="O29" s="1203" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1162" t="n">
+      <c r="P29" s="1206" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1159" t="n"/>
-      <c r="R29" s="1159" t="n"/>
-      <c r="S29" s="1159" t="n"/>
+      <c r="Q29" s="1203" t="n"/>
+      <c r="R29" s="1203" t="n"/>
+      <c r="S29" s="1203" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1158" t="n"/>
+      <c r="U29" s="1202" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -5830,43 +5938,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1163" t="inlineStr">
+      <c r="A30" s="1207" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1164" t="inlineStr">
+      <c r="B30" s="1208" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1164" t="inlineStr">
+      <c r="C30" s="1208" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1165" t="n"/>
-      <c r="E30" s="1165" t="n"/>
-      <c r="F30" s="1165" t="n"/>
-      <c r="G30" s="1165" t="n"/>
-      <c r="H30" s="1165" t="n"/>
-      <c r="I30" s="1166" t="n"/>
-      <c r="J30" s="1167" t="n"/>
-      <c r="K30" s="1167" t="n"/>
-      <c r="L30" s="1167" t="n"/>
-      <c r="M30" s="1165" t="n"/>
-      <c r="N30" s="1165" t="n"/>
-      <c r="O30" s="1165" t="n"/>
-      <c r="P30" s="1168" t="n"/>
-      <c r="Q30" s="1165" t="n"/>
-      <c r="R30" s="1165" t="n"/>
-      <c r="S30" s="1165" t="n"/>
+      <c r="D30" s="1209" t="n"/>
+      <c r="E30" s="1209" t="n"/>
+      <c r="F30" s="1209" t="n"/>
+      <c r="G30" s="1209" t="n"/>
+      <c r="H30" s="1209" t="n"/>
+      <c r="I30" s="1210" t="n"/>
+      <c r="J30" s="1211" t="n"/>
+      <c r="K30" s="1211" t="n"/>
+      <c r="L30" s="1211" t="n"/>
+      <c r="M30" s="1209" t="n"/>
+      <c r="N30" s="1209" t="n"/>
+      <c r="O30" s="1209" t="n"/>
+      <c r="P30" s="1212" t="n"/>
+      <c r="Q30" s="1209" t="n"/>
+      <c r="R30" s="1209" t="n"/>
+      <c r="S30" s="1209" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1164" t="n"/>
+      <c r="U30" s="1208" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -5874,53 +5982,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1169" t="inlineStr">
+      <c r="A31" s="1213" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1170" t="inlineStr">
+      <c r="B31" s="1214" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1170" t="inlineStr">
+      <c r="C31" s="1214" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1171" t="n"/>
-      <c r="E31" s="1171" t="n">
+      <c r="D31" s="1215" t="n"/>
+      <c r="E31" s="1215" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1171" t="n">
+      <c r="F31" s="1215" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1171" t="n">
+      <c r="G31" s="1215" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1171" t="n"/>
-      <c r="I31" s="1172" t="n"/>
-      <c r="J31" s="1173" t="n"/>
-      <c r="K31" s="1173" t="n"/>
-      <c r="L31" s="1173" t="n"/>
-      <c r="M31" s="1171" t="n"/>
-      <c r="N31" s="1171" t="n"/>
-      <c r="O31" s="1171" t="n">
+      <c r="H31" s="1215" t="n"/>
+      <c r="I31" s="1216" t="n"/>
+      <c r="J31" s="1217" t="n"/>
+      <c r="K31" s="1217" t="n"/>
+      <c r="L31" s="1217" t="n"/>
+      <c r="M31" s="1215" t="n"/>
+      <c r="N31" s="1215" t="n"/>
+      <c r="O31" s="1215" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1174" t="n">
+      <c r="P31" s="1218" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1171" t="n"/>
-      <c r="R31" s="1171" t="n"/>
-      <c r="S31" s="1171" t="n"/>
+      <c r="Q31" s="1215" t="n"/>
+      <c r="R31" s="1215" t="n"/>
+      <c r="S31" s="1215" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1170" t="inlineStr">
+      <c r="U31" s="1214" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -5932,49 +6040,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1181" t="inlineStr">
+      <c r="A32" s="1225" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1182" t="inlineStr">
+      <c r="B32" s="1226" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1182" t="inlineStr">
+      <c r="C32" s="1226" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1183" t="n"/>
-      <c r="E32" s="1183" t="n"/>
-      <c r="F32" s="1183" t="n"/>
-      <c r="G32" s="1183" t="n"/>
-      <c r="H32" s="1183" t="n">
+      <c r="D32" s="1227" t="n"/>
+      <c r="E32" s="1227" t="n"/>
+      <c r="F32" s="1227" t="n"/>
+      <c r="G32" s="1227" t="n"/>
+      <c r="H32" s="1227" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1184" t="n"/>
-      <c r="J32" s="1185" t="n"/>
-      <c r="K32" s="1185" t="n"/>
-      <c r="L32" s="1185" t="n"/>
-      <c r="M32" s="1183" t="n">
+      <c r="I32" s="1228" t="n"/>
+      <c r="J32" s="1229" t="n"/>
+      <c r="K32" s="1229" t="n"/>
+      <c r="L32" s="1229" t="n"/>
+      <c r="M32" s="1227" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1183" t="n">
+      <c r="N32" s="1227" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1183" t="n"/>
-      <c r="P32" s="1186" t="n"/>
-      <c r="Q32" s="1183" t="n"/>
-      <c r="R32" s="1183" t="n"/>
-      <c r="S32" s="1183" t="n"/>
+      <c r="O32" s="1227" t="n"/>
+      <c r="P32" s="1230" t="n"/>
+      <c r="Q32" s="1227" t="n"/>
+      <c r="R32" s="1227" t="n"/>
+      <c r="S32" s="1227" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1182" t="n"/>
+      <c r="U32" s="1226" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -5982,57 +6090,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1157" t="inlineStr">
+      <c r="A33" s="1201" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1158" t="inlineStr">
+      <c r="B33" s="1202" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1158" t="inlineStr">
+      <c r="C33" s="1202" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1159" t="n"/>
-      <c r="E33" s="1159" t="n">
+      <c r="D33" s="1203" t="n"/>
+      <c r="E33" s="1203" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1159" t="n">
+      <c r="F33" s="1203" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1159" t="n">
+      <c r="G33" s="1203" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1159" t="n"/>
-      <c r="I33" s="1160" t="n">
+      <c r="H33" s="1203" t="n"/>
+      <c r="I33" s="1204" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1161" t="n"/>
-      <c r="K33" s="1161" t="n"/>
-      <c r="L33" s="1161" t="n"/>
-      <c r="M33" s="1159" t="n"/>
-      <c r="N33" s="1159" t="n"/>
-      <c r="O33" s="1159" t="n">
+      <c r="J33" s="1205" t="n"/>
+      <c r="K33" s="1205" t="n"/>
+      <c r="L33" s="1205" t="n"/>
+      <c r="M33" s="1203" t="n"/>
+      <c r="N33" s="1203" t="n"/>
+      <c r="O33" s="1203" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1162" t="n">
+      <c r="P33" s="1206" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1159" t="n"/>
-      <c r="R33" s="1159" t="n">
+      <c r="Q33" s="1203" t="n"/>
+      <c r="R33" s="1203" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1159" t="n"/>
+      <c r="S33" s="1203" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1158" t="inlineStr">
+      <c r="U33" s="1202" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -6044,49 +6152,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1163" t="inlineStr">
+      <c r="A34" s="1207" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1164" t="inlineStr">
+      <c r="B34" s="1208" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1164" t="inlineStr">
+      <c r="C34" s="1208" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1165" t="n"/>
-      <c r="E34" s="1165" t="n"/>
-      <c r="F34" s="1165" t="n"/>
-      <c r="G34" s="1165" t="n"/>
-      <c r="H34" s="1165" t="n">
+      <c r="D34" s="1209" t="n"/>
+      <c r="E34" s="1209" t="n"/>
+      <c r="F34" s="1209" t="n"/>
+      <c r="G34" s="1209" t="n"/>
+      <c r="H34" s="1209" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1166" t="n"/>
-      <c r="J34" s="1167" t="n"/>
-      <c r="K34" s="1167" t="n"/>
-      <c r="L34" s="1167" t="n"/>
-      <c r="M34" s="1165" t="n">
+      <c r="I34" s="1210" t="n"/>
+      <c r="J34" s="1211" t="n"/>
+      <c r="K34" s="1211" t="n"/>
+      <c r="L34" s="1211" t="n"/>
+      <c r="M34" s="1209" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1165" t="n">
+      <c r="N34" s="1209" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1165" t="n"/>
-      <c r="P34" s="1168" t="n"/>
-      <c r="Q34" s="1165" t="n"/>
-      <c r="R34" s="1165" t="n"/>
-      <c r="S34" s="1165" t="n"/>
+      <c r="O34" s="1209" t="n"/>
+      <c r="P34" s="1212" t="n"/>
+      <c r="Q34" s="1209" t="n"/>
+      <c r="R34" s="1209" t="n"/>
+      <c r="S34" s="1209" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1164" t="n"/>
+      <c r="U34" s="1208" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -6094,57 +6202,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1169" t="inlineStr">
+      <c r="A35" s="1213" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1170" t="inlineStr">
+      <c r="B35" s="1214" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1170" t="inlineStr">
+      <c r="C35" s="1214" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1171" t="n"/>
-      <c r="E35" s="1171" t="n">
+      <c r="D35" s="1215" t="n"/>
+      <c r="E35" s="1215" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1171" t="n">
+      <c r="F35" s="1215" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1171" t="n">
+      <c r="G35" s="1215" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1171" t="n"/>
-      <c r="I35" s="1172" t="n">
+      <c r="H35" s="1215" t="n"/>
+      <c r="I35" s="1216" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1173" t="n"/>
-      <c r="K35" s="1173" t="n"/>
-      <c r="L35" s="1173" t="n"/>
-      <c r="M35" s="1171" t="n"/>
-      <c r="N35" s="1171" t="n"/>
-      <c r="O35" s="1171" t="n">
+      <c r="J35" s="1217" t="n"/>
+      <c r="K35" s="1217" t="n"/>
+      <c r="L35" s="1217" t="n"/>
+      <c r="M35" s="1215" t="n"/>
+      <c r="N35" s="1215" t="n"/>
+      <c r="O35" s="1215" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1174" t="n">
+      <c r="P35" s="1218" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1171" t="n"/>
-      <c r="R35" s="1171" t="n">
+      <c r="Q35" s="1215" t="n"/>
+      <c r="R35" s="1215" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1171" t="n"/>
+      <c r="S35" s="1215" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1170" t="inlineStr">
+      <c r="U35" s="1214" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -6156,49 +6264,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1175" t="inlineStr">
+      <c r="A36" s="1219" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1176" t="inlineStr">
+      <c r="B36" s="1220" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1176" t="inlineStr">
+      <c r="C36" s="1220" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1177" t="n"/>
-      <c r="E36" s="1177" t="n"/>
-      <c r="F36" s="1177" t="n"/>
-      <c r="G36" s="1177" t="n"/>
-      <c r="H36" s="1177" t="n">
+      <c r="D36" s="1221" t="n"/>
+      <c r="E36" s="1221" t="n"/>
+      <c r="F36" s="1221" t="n"/>
+      <c r="G36" s="1221" t="n"/>
+      <c r="H36" s="1221" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1178" t="n"/>
-      <c r="J36" s="1179" t="n"/>
-      <c r="K36" s="1179" t="n"/>
-      <c r="L36" s="1179" t="n"/>
-      <c r="M36" s="1177" t="n">
+      <c r="I36" s="1222" t="n"/>
+      <c r="J36" s="1223" t="n"/>
+      <c r="K36" s="1223" t="n"/>
+      <c r="L36" s="1223" t="n"/>
+      <c r="M36" s="1221" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1177" t="n">
+      <c r="N36" s="1221" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1177" t="n"/>
-      <c r="P36" s="1180" t="n"/>
-      <c r="Q36" s="1177" t="n"/>
-      <c r="R36" s="1177" t="n"/>
-      <c r="S36" s="1177" t="n"/>
+      <c r="O36" s="1221" t="n"/>
+      <c r="P36" s="1224" t="n"/>
+      <c r="Q36" s="1221" t="n"/>
+      <c r="R36" s="1221" t="n"/>
+      <c r="S36" s="1221" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1176" t="n"/>
+      <c r="U36" s="1220" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -6206,41 +6314,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1181" t="inlineStr">
+      <c r="A37" s="1225" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1182" t="inlineStr">
+      <c r="B37" s="1226" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1182" t="inlineStr">
+      <c r="C37" s="1226" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1183" t="n"/>
-      <c r="E37" s="1183" t="n"/>
-      <c r="F37" s="1183" t="n"/>
-      <c r="G37" s="1183" t="n"/>
-      <c r="H37" s="1183" t="n"/>
-      <c r="I37" s="1184" t="n"/>
-      <c r="J37" s="1185" t="n"/>
-      <c r="K37" s="1185" t="n"/>
-      <c r="L37" s="1185" t="n"/>
-      <c r="M37" s="1183" t="n"/>
-      <c r="N37" s="1183" t="n"/>
-      <c r="O37" s="1183" t="n"/>
-      <c r="P37" s="1186" t="n"/>
-      <c r="Q37" s="1183" t="n">
+      <c r="D37" s="1227" t="n"/>
+      <c r="E37" s="1227" t="n"/>
+      <c r="F37" s="1227" t="n"/>
+      <c r="G37" s="1227" t="n"/>
+      <c r="H37" s="1227" t="n"/>
+      <c r="I37" s="1228" t="n"/>
+      <c r="J37" s="1229" t="n"/>
+      <c r="K37" s="1229" t="n"/>
+      <c r="L37" s="1229" t="n"/>
+      <c r="M37" s="1227" t="n"/>
+      <c r="N37" s="1227" t="n"/>
+      <c r="O37" s="1227" t="n"/>
+      <c r="P37" s="1230" t="n"/>
+      <c r="Q37" s="1227" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1183" t="n"/>
-      <c r="S37" s="1183" t="n"/>
+      <c r="R37" s="1227" t="n"/>
+      <c r="S37" s="1227" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1182" t="n"/>
+      <c r="U37" s="1226" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -6248,57 +6356,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1157" t="inlineStr">
+      <c r="A38" s="1201" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1158" t="inlineStr">
+      <c r="B38" s="1202" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1158" t="inlineStr">
+      <c r="C38" s="1202" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1159" t="n"/>
-      <c r="E38" s="1159" t="n">
+      <c r="D38" s="1203" t="n"/>
+      <c r="E38" s="1203" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1159" t="n">
+      <c r="F38" s="1203" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1159" t="n">
+      <c r="G38" s="1203" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1159" t="n"/>
-      <c r="I38" s="1160" t="n">
+      <c r="H38" s="1203" t="n"/>
+      <c r="I38" s="1204" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1161" t="n"/>
-      <c r="K38" s="1161" t="n"/>
-      <c r="L38" s="1161" t="n"/>
-      <c r="M38" s="1159" t="n"/>
-      <c r="N38" s="1159" t="n"/>
-      <c r="O38" s="1159" t="n">
+      <c r="J38" s="1205" t="n"/>
+      <c r="K38" s="1205" t="n"/>
+      <c r="L38" s="1205" t="n"/>
+      <c r="M38" s="1203" t="n"/>
+      <c r="N38" s="1203" t="n"/>
+      <c r="O38" s="1203" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1162" t="n">
+      <c r="P38" s="1206" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1159" t="n"/>
-      <c r="R38" s="1159" t="n">
+      <c r="Q38" s="1203" t="n"/>
+      <c r="R38" s="1203" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1159" t="n"/>
+      <c r="S38" s="1203" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1158" t="inlineStr">
+      <c r="U38" s="1202" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -6310,49 +6418,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1187" t="inlineStr">
+      <c r="A39" s="1231" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1188" t="inlineStr">
+      <c r="B39" s="1232" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1188" t="inlineStr">
+      <c r="C39" s="1232" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1189" t="n"/>
-      <c r="E39" s="1189" t="n"/>
-      <c r="F39" s="1189" t="n"/>
-      <c r="G39" s="1189" t="n"/>
-      <c r="H39" s="1189" t="n">
+      <c r="D39" s="1233" t="n"/>
+      <c r="E39" s="1233" t="n"/>
+      <c r="F39" s="1233" t="n"/>
+      <c r="G39" s="1233" t="n"/>
+      <c r="H39" s="1233" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1190" t="n"/>
-      <c r="J39" s="1191" t="n"/>
-      <c r="K39" s="1191" t="n"/>
-      <c r="L39" s="1191" t="n"/>
-      <c r="M39" s="1189" t="n">
+      <c r="I39" s="1234" t="n"/>
+      <c r="J39" s="1235" t="n"/>
+      <c r="K39" s="1235" t="n"/>
+      <c r="L39" s="1235" t="n"/>
+      <c r="M39" s="1233" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1189" t="n">
+      <c r="N39" s="1233" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1189" t="n"/>
-      <c r="P39" s="1192" t="n"/>
-      <c r="Q39" s="1189" t="n"/>
-      <c r="R39" s="1189" t="n"/>
-      <c r="S39" s="1189" t="n"/>
+      <c r="O39" s="1233" t="n"/>
+      <c r="P39" s="1236" t="n"/>
+      <c r="Q39" s="1233" t="n"/>
+      <c r="R39" s="1233" t="n"/>
+      <c r="S39" s="1233" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1188" t="n"/>
+      <c r="U39" s="1232" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -6360,41 +6468,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1163" t="inlineStr">
+      <c r="A40" s="1207" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1164" t="inlineStr">
+      <c r="B40" s="1208" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1164" t="inlineStr">
+      <c r="C40" s="1208" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1165" t="n"/>
-      <c r="E40" s="1165" t="n"/>
-      <c r="F40" s="1165" t="n"/>
-      <c r="G40" s="1165" t="n"/>
-      <c r="H40" s="1165" t="n"/>
-      <c r="I40" s="1166" t="n"/>
-      <c r="J40" s="1167" t="n"/>
-      <c r="K40" s="1167" t="n"/>
-      <c r="L40" s="1167" t="n"/>
-      <c r="M40" s="1165" t="n"/>
-      <c r="N40" s="1165" t="n"/>
-      <c r="O40" s="1165" t="n"/>
-      <c r="P40" s="1168" t="n"/>
-      <c r="Q40" s="1165" t="n">
+      <c r="D40" s="1209" t="n"/>
+      <c r="E40" s="1209" t="n"/>
+      <c r="F40" s="1209" t="n"/>
+      <c r="G40" s="1209" t="n"/>
+      <c r="H40" s="1209" t="n"/>
+      <c r="I40" s="1210" t="n"/>
+      <c r="J40" s="1211" t="n"/>
+      <c r="K40" s="1211" t="n"/>
+      <c r="L40" s="1211" t="n"/>
+      <c r="M40" s="1209" t="n"/>
+      <c r="N40" s="1209" t="n"/>
+      <c r="O40" s="1209" t="n"/>
+      <c r="P40" s="1212" t="n"/>
+      <c r="Q40" s="1209" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1165" t="n"/>
-      <c r="S40" s="1165" t="n"/>
+      <c r="R40" s="1209" t="n"/>
+      <c r="S40" s="1209" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1164" t="n"/>
+      <c r="U40" s="1208" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -6402,57 +6510,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1169" t="inlineStr">
+      <c r="A41" s="1213" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1170" t="inlineStr">
+      <c r="B41" s="1214" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1170" t="inlineStr">
+      <c r="C41" s="1214" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1171" t="n"/>
-      <c r="E41" s="1171" t="n">
+      <c r="D41" s="1215" t="n"/>
+      <c r="E41" s="1215" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1171" t="n">
+      <c r="F41" s="1215" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1171" t="n">
+      <c r="G41" s="1215" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1171" t="n"/>
-      <c r="I41" s="1172" t="n">
+      <c r="H41" s="1215" t="n"/>
+      <c r="I41" s="1216" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1173" t="n"/>
-      <c r="K41" s="1173" t="n"/>
-      <c r="L41" s="1173" t="n"/>
-      <c r="M41" s="1171" t="n"/>
-      <c r="N41" s="1171" t="n"/>
-      <c r="O41" s="1171" t="n">
+      <c r="J41" s="1217" t="n"/>
+      <c r="K41" s="1217" t="n"/>
+      <c r="L41" s="1217" t="n"/>
+      <c r="M41" s="1215" t="n"/>
+      <c r="N41" s="1215" t="n"/>
+      <c r="O41" s="1215" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1174" t="n">
+      <c r="P41" s="1218" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1171" t="n"/>
-      <c r="R41" s="1171" t="n">
+      <c r="Q41" s="1215" t="n"/>
+      <c r="R41" s="1215" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1171" t="n"/>
+      <c r="S41" s="1215" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1170" t="inlineStr">
+      <c r="U41" s="1214" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -6464,49 +6572,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1181" t="inlineStr">
+      <c r="A42" s="1225" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1182" t="inlineStr">
+      <c r="B42" s="1226" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1182" t="inlineStr">
+      <c r="C42" s="1226" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1183" t="n"/>
-      <c r="E42" s="1183" t="n"/>
-      <c r="F42" s="1183" t="n"/>
-      <c r="G42" s="1183" t="n"/>
-      <c r="H42" s="1183" t="n">
+      <c r="D42" s="1227" t="n"/>
+      <c r="E42" s="1227" t="n"/>
+      <c r="F42" s="1227" t="n"/>
+      <c r="G42" s="1227" t="n"/>
+      <c r="H42" s="1227" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1184" t="n"/>
-      <c r="J42" s="1185" t="n"/>
-      <c r="K42" s="1185" t="n"/>
-      <c r="L42" s="1185" t="n"/>
-      <c r="M42" s="1183" t="n">
+      <c r="I42" s="1228" t="n"/>
+      <c r="J42" s="1229" t="n"/>
+      <c r="K42" s="1229" t="n"/>
+      <c r="L42" s="1229" t="n"/>
+      <c r="M42" s="1227" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1183" t="n">
+      <c r="N42" s="1227" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1183" t="n"/>
-      <c r="P42" s="1186" t="n"/>
-      <c r="Q42" s="1183" t="n"/>
-      <c r="R42" s="1183" t="n"/>
-      <c r="S42" s="1183" t="n"/>
+      <c r="O42" s="1227" t="n"/>
+      <c r="P42" s="1230" t="n"/>
+      <c r="Q42" s="1227" t="n"/>
+      <c r="R42" s="1227" t="n"/>
+      <c r="S42" s="1227" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1182" t="n"/>
+      <c r="U42" s="1226" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -6514,57 +6622,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1157" t="inlineStr">
+      <c r="A43" s="1201" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1158" t="inlineStr">
+      <c r="B43" s="1202" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1158" t="inlineStr">
+      <c r="C43" s="1202" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1159" t="n"/>
-      <c r="E43" s="1159" t="n">
+      <c r="D43" s="1203" t="n"/>
+      <c r="E43" s="1203" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1159" t="n">
+      <c r="F43" s="1203" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1159" t="n">
+      <c r="G43" s="1203" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1159" t="n"/>
-      <c r="I43" s="1160" t="n">
+      <c r="H43" s="1203" t="n"/>
+      <c r="I43" s="1204" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1161" t="n"/>
-      <c r="K43" s="1161" t="n"/>
-      <c r="L43" s="1161" t="n"/>
-      <c r="M43" s="1159" t="n"/>
-      <c r="N43" s="1159" t="n"/>
-      <c r="O43" s="1159" t="n">
+      <c r="J43" s="1205" t="n"/>
+      <c r="K43" s="1205" t="n"/>
+      <c r="L43" s="1205" t="n"/>
+      <c r="M43" s="1203" t="n"/>
+      <c r="N43" s="1203" t="n"/>
+      <c r="O43" s="1203" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1162" t="n">
+      <c r="P43" s="1206" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1159" t="n"/>
-      <c r="R43" s="1159" t="n">
+      <c r="Q43" s="1203" t="n"/>
+      <c r="R43" s="1203" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1159" t="n"/>
+      <c r="S43" s="1203" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1158" t="n"/>
+      <c r="U43" s="1202" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -6572,45 +6680,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1187" t="inlineStr">
+      <c r="A44" s="1231" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1188" t="inlineStr">
+      <c r="B44" s="1232" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1188" t="inlineStr">
+      <c r="C44" s="1232" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1189" t="n"/>
-      <c r="E44" s="1189" t="n">
+      <c r="D44" s="1233" t="n"/>
+      <c r="E44" s="1233" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1189" t="n">
+      <c r="F44" s="1233" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1189" t="n"/>
-      <c r="H44" s="1189" t="n"/>
-      <c r="I44" s="1190" t="n"/>
-      <c r="J44" s="1191" t="n"/>
-      <c r="K44" s="1191" t="n"/>
-      <c r="L44" s="1191" t="n"/>
-      <c r="M44" s="1189" t="n"/>
-      <c r="N44" s="1189" t="n"/>
-      <c r="O44" s="1189" t="n"/>
-      <c r="P44" s="1192" t="n"/>
-      <c r="Q44" s="1189" t="n"/>
-      <c r="R44" s="1189" t="n"/>
-      <c r="S44" s="1189" t="n">
+      <c r="G44" s="1233" t="n"/>
+      <c r="H44" s="1233" t="n"/>
+      <c r="I44" s="1234" t="n"/>
+      <c r="J44" s="1235" t="n"/>
+      <c r="K44" s="1235" t="n"/>
+      <c r="L44" s="1235" t="n"/>
+      <c r="M44" s="1233" t="n"/>
+      <c r="N44" s="1233" t="n"/>
+      <c r="O44" s="1233" t="n"/>
+      <c r="P44" s="1236" t="n"/>
+      <c r="Q44" s="1233" t="n"/>
+      <c r="R44" s="1233" t="n"/>
+      <c r="S44" s="1233" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1188" t="inlineStr">
+      <c r="U44" s="1232" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -6622,49 +6730,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1163" t="inlineStr">
+      <c r="A45" s="1207" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1164" t="inlineStr">
+      <c r="B45" s="1208" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1164" t="inlineStr">
+      <c r="C45" s="1208" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1165" t="n"/>
-      <c r="E45" s="1165" t="n"/>
-      <c r="F45" s="1165" t="n"/>
-      <c r="G45" s="1165" t="n"/>
-      <c r="H45" s="1165" t="n">
+      <c r="D45" s="1209" t="n"/>
+      <c r="E45" s="1209" t="n"/>
+      <c r="F45" s="1209" t="n"/>
+      <c r="G45" s="1209" t="n"/>
+      <c r="H45" s="1209" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1166" t="n"/>
-      <c r="J45" s="1167" t="n"/>
-      <c r="K45" s="1167" t="n"/>
-      <c r="L45" s="1167" t="n"/>
-      <c r="M45" s="1165" t="n">
+      <c r="I45" s="1210" t="n"/>
+      <c r="J45" s="1211" t="n"/>
+      <c r="K45" s="1211" t="n"/>
+      <c r="L45" s="1211" t="n"/>
+      <c r="M45" s="1209" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1165" t="n">
+      <c r="N45" s="1209" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1165" t="n"/>
-      <c r="P45" s="1168" t="n"/>
-      <c r="Q45" s="1165" t="n"/>
-      <c r="R45" s="1165" t="n"/>
-      <c r="S45" s="1165" t="n"/>
+      <c r="O45" s="1209" t="n"/>
+      <c r="P45" s="1212" t="n"/>
+      <c r="Q45" s="1209" t="n"/>
+      <c r="R45" s="1209" t="n"/>
+      <c r="S45" s="1209" t="n"/>
       <c r="T45" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1164" t="n"/>
+      <c r="U45" s="1208" t="n"/>
       <c r="V45" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -6672,62 +6780,116 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1193" t="inlineStr">
+      <c r="A46" s="1213" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B46" s="1194" t="inlineStr">
+      <c r="B46" s="1214" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C46" s="1194" t="inlineStr">
+      <c r="C46" s="1214" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D46" s="1195" t="n"/>
-      <c r="E46" s="1195" t="n">
+      <c r="D46" s="1215" t="n"/>
+      <c r="E46" s="1215" t="n">
         <v>16.6</v>
       </c>
-      <c r="F46" s="1195" t="n">
+      <c r="F46" s="1215" t="n">
         <v>0.6</v>
       </c>
-      <c r="G46" s="1195" t="n">
+      <c r="G46" s="1215" t="n">
         <v>4.1</v>
       </c>
-      <c r="H46" s="1195" t="n"/>
-      <c r="I46" s="1196" t="n">
+      <c r="H46" s="1215" t="n"/>
+      <c r="I46" s="1216" t="n">
         <v>0.9</v>
       </c>
-      <c r="J46" s="1197" t="n"/>
-      <c r="K46" s="1197" t="n"/>
-      <c r="L46" s="1197" t="n"/>
-      <c r="M46" s="1195" t="n"/>
-      <c r="N46" s="1195" t="n"/>
-      <c r="O46" s="1195" t="n">
+      <c r="J46" s="1217" t="n"/>
+      <c r="K46" s="1217" t="n"/>
+      <c r="L46" s="1217" t="n"/>
+      <c r="M46" s="1215" t="n"/>
+      <c r="N46" s="1215" t="n"/>
+      <c r="O46" s="1215" t="n">
         <v>13.2</v>
       </c>
-      <c r="P46" s="1198" t="n">
+      <c r="P46" s="1218" t="n">
         <v>0</v>
       </c>
-      <c r="Q46" s="1195" t="n"/>
-      <c r="R46" s="1195" t="n">
+      <c r="Q46" s="1215" t="n"/>
+      <c r="R46" s="1215" t="n">
         <v>84.5</v>
       </c>
-      <c r="S46" s="1195" t="n">
+      <c r="S46" s="1215" t="n">
         <v>11.8</v>
       </c>
-      <c r="T46" s="1199" t="inlineStr">
+      <c r="T46" s="813" t="inlineStr">
         <is>
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U46" s="1194" t="n"/>
-      <c r="V46" s="1200" t="inlineStr">
+      <c r="U46" s="1214" t="inlineStr">
+        <is>
+          <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
+        </is>
+      </c>
+      <c r="V46" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 16.6, CC 0.6. (John wrote 'CC=16.6' but that's FC; a 16.6 combined chlorine is implausible -- logged as FC.) FC loss 4.1 ppm/24h = 17.2 (7/2 NOON) + 1.0gal x3.5 - 16.6, computed noon-to-noon; NOT the 2.3 daily_calc.py reported (it used the 7/2 evening recheck 15.4 as baseline -&gt; ~16.5h window, non-comparable). WATCH: CC creeping 0.0 -&gt; 0.4 -&gt; 0.6 over ~24h; still a trace, and higher FC should oxidize it away, but note the direction -- flag if it climbs past ~1.0. Pred error +0.9 (actual 16.6 vs 7/2 dose's 15.7 projection): model over-predicted loss again but by less than 7/2's +2.1 -- two straight hot/sunny days where real loss ran under the L24=5.0 estimate; watch a 3rd before nudging dose.py's l24_hot_sunny down. Water level 11.8 cm (was 11.9 on 7/2; -0.1 within ruler/reading noise, ruler adhesion still iffy). Hot day: high 94F, water 84.5F, ~13 sun hrs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1225" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B47" s="1226" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="C47" s="1226" t="inlineStr">
+        <is>
+          <t>DOSE</t>
+        </is>
+      </c>
+      <c r="D47" s="1227" t="n"/>
+      <c r="E47" s="1227" t="n"/>
+      <c r="F47" s="1227" t="n"/>
+      <c r="G47" s="1227" t="n"/>
+      <c r="H47" s="1227" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="I47" s="1228" t="n"/>
+      <c r="J47" s="1229" t="n"/>
+      <c r="K47" s="1229" t="n"/>
+      <c r="L47" s="1229" t="n"/>
+      <c r="M47" s="1227" t="n">
+        <v>1</v>
+      </c>
+      <c r="N47" s="1227" t="n">
+        <v>20</v>
+      </c>
+      <c r="O47" s="1227" t="n"/>
+      <c r="P47" s="1230" t="n"/>
+      <c r="Q47" s="1227" t="n"/>
+      <c r="R47" s="1227" t="n"/>
+      <c r="S47" s="1227" t="n"/>
+      <c r="T47" s="827" t="inlineStr">
+        <is>
+          <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
+        </is>
+      </c>
+      <c r="U47" s="1226" t="n"/>
+      <c r="V47" s="828" t="inlineStr">
+        <is>
+          <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log 2026-07-02 night EVENT - Clean: Magic Eraser waterline cleaning
John reported the overnight liner cleaning (melamine foam) as a likely
CC-creep contributor -- melamine is nitrogen-rich, so shed particles +
scrubbed waterline scum become chloramines. Inserted chronologically
(after 7/2 dose, before 7/3 test) to explain the CC bump in the record.
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1237">
+  <cellXfs count="1273">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -4131,6 +4131,114 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -4499,7 +4607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V47"/>
+  <dimension ref="A1:V48"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -4676,35 +4784,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1201" t="inlineStr">
+      <c r="A3" s="1237" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1202" t="n"/>
-      <c r="C3" s="1202" t="inlineStr">
+      <c r="B3" s="1238" t="n"/>
+      <c r="C3" s="1238" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1203" t="n"/>
-      <c r="E3" s="1203" t="n"/>
-      <c r="F3" s="1203" t="n"/>
-      <c r="G3" s="1203" t="n"/>
-      <c r="H3" s="1203" t="n"/>
-      <c r="I3" s="1204" t="n"/>
-      <c r="J3" s="1205" t="n"/>
-      <c r="K3" s="1205" t="n"/>
-      <c r="L3" s="1205" t="n"/>
-      <c r="M3" s="1203" t="n"/>
-      <c r="N3" s="1203" t="n"/>
-      <c r="O3" s="1203" t="n"/>
-      <c r="P3" s="1206" t="n"/>
-      <c r="Q3" s="1203" t="n"/>
-      <c r="R3" s="1203" t="n"/>
-      <c r="S3" s="1203" t="n"/>
+      <c r="D3" s="1239" t="n"/>
+      <c r="E3" s="1239" t="n"/>
+      <c r="F3" s="1239" t="n"/>
+      <c r="G3" s="1239" t="n"/>
+      <c r="H3" s="1239" t="n"/>
+      <c r="I3" s="1240" t="n"/>
+      <c r="J3" s="1241" t="n"/>
+      <c r="K3" s="1241" t="n"/>
+      <c r="L3" s="1241" t="n"/>
+      <c r="M3" s="1239" t="n"/>
+      <c r="N3" s="1239" t="n"/>
+      <c r="O3" s="1239" t="n"/>
+      <c r="P3" s="1242" t="n"/>
+      <c r="Q3" s="1239" t="n"/>
+      <c r="R3" s="1239" t="n"/>
+      <c r="S3" s="1239" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1202" t="n"/>
+      <c r="U3" s="1238" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -4712,43 +4820,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1207" t="inlineStr">
+      <c r="A4" s="1243" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1208" t="inlineStr">
+      <c r="B4" s="1244" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1208" t="inlineStr">
+      <c r="C4" s="1244" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1209" t="n"/>
-      <c r="E4" s="1209" t="n"/>
-      <c r="F4" s="1209" t="n"/>
-      <c r="G4" s="1209" t="n"/>
-      <c r="H4" s="1209" t="n"/>
-      <c r="I4" s="1210" t="n"/>
-      <c r="J4" s="1211" t="n"/>
-      <c r="K4" s="1211" t="n"/>
-      <c r="L4" s="1211" t="n"/>
-      <c r="M4" s="1209" t="n">
+      <c r="D4" s="1245" t="n"/>
+      <c r="E4" s="1245" t="n"/>
+      <c r="F4" s="1245" t="n"/>
+      <c r="G4" s="1245" t="n"/>
+      <c r="H4" s="1245" t="n"/>
+      <c r="I4" s="1246" t="n"/>
+      <c r="J4" s="1247" t="n"/>
+      <c r="K4" s="1247" t="n"/>
+      <c r="L4" s="1247" t="n"/>
+      <c r="M4" s="1245" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1209" t="n">
+      <c r="N4" s="1245" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1209" t="n"/>
-      <c r="P4" s="1212" t="n"/>
-      <c r="Q4" s="1209" t="n"/>
-      <c r="R4" s="1209" t="n"/>
-      <c r="S4" s="1209" t="n"/>
+      <c r="O4" s="1245" t="n"/>
+      <c r="P4" s="1248" t="n"/>
+      <c r="Q4" s="1245" t="n"/>
+      <c r="R4" s="1245" t="n"/>
+      <c r="S4" s="1245" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1208" t="n"/>
+      <c r="U4" s="1244" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -4756,57 +4864,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1213" t="inlineStr">
+      <c r="A5" s="1249" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1214" t="inlineStr">
+      <c r="B5" s="1250" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1214" t="inlineStr">
+      <c r="C5" s="1250" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1215" t="n">
+      <c r="D5" s="1251" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1215" t="n">
+      <c r="E5" s="1251" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1215" t="n">
+      <c r="F5" s="1251" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1215" t="n"/>
-      <c r="H5" s="1215" t="n"/>
-      <c r="I5" s="1216" t="n"/>
-      <c r="J5" s="1217" t="n">
+      <c r="G5" s="1251" t="n"/>
+      <c r="H5" s="1251" t="n"/>
+      <c r="I5" s="1252" t="n"/>
+      <c r="J5" s="1253" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1217" t="n">
+      <c r="K5" s="1253" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1217" t="inlineStr">
+      <c r="L5" s="1253" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1215" t="n"/>
-      <c r="N5" s="1215" t="n"/>
-      <c r="O5" s="1215" t="n">
+      <c r="M5" s="1251" t="n"/>
+      <c r="N5" s="1251" t="n"/>
+      <c r="O5" s="1251" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1218" t="n">
+      <c r="P5" s="1254" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1215" t="n"/>
-      <c r="R5" s="1215" t="n"/>
-      <c r="S5" s="1215" t="n"/>
+      <c r="Q5" s="1251" t="n"/>
+      <c r="R5" s="1251" t="n"/>
+      <c r="S5" s="1251" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1214" t="n"/>
+      <c r="U5" s="1250" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -4814,43 +4922,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1219" t="inlineStr">
+      <c r="A6" s="1255" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1220" t="inlineStr">
+      <c r="B6" s="1256" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1220" t="inlineStr">
+      <c r="C6" s="1256" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1221" t="n"/>
-      <c r="E6" s="1221" t="n"/>
-      <c r="F6" s="1221" t="n"/>
-      <c r="G6" s="1221" t="n"/>
-      <c r="H6" s="1221" t="n"/>
-      <c r="I6" s="1222" t="n"/>
-      <c r="J6" s="1223" t="n"/>
-      <c r="K6" s="1223" t="n"/>
-      <c r="L6" s="1223" t="n"/>
-      <c r="M6" s="1221" t="n">
+      <c r="D6" s="1257" t="n"/>
+      <c r="E6" s="1257" t="n"/>
+      <c r="F6" s="1257" t="n"/>
+      <c r="G6" s="1257" t="n"/>
+      <c r="H6" s="1257" t="n"/>
+      <c r="I6" s="1258" t="n"/>
+      <c r="J6" s="1259" t="n"/>
+      <c r="K6" s="1259" t="n"/>
+      <c r="L6" s="1259" t="n"/>
+      <c r="M6" s="1257" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1221" t="n">
+      <c r="N6" s="1257" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1221" t="n"/>
-      <c r="P6" s="1224" t="n"/>
-      <c r="Q6" s="1221" t="n"/>
-      <c r="R6" s="1221" t="n"/>
-      <c r="S6" s="1221" t="n"/>
+      <c r="O6" s="1257" t="n"/>
+      <c r="P6" s="1260" t="n"/>
+      <c r="Q6" s="1257" t="n"/>
+      <c r="R6" s="1257" t="n"/>
+      <c r="S6" s="1257" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1220" t="n"/>
+      <c r="U6" s="1256" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -4858,39 +4966,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1225" t="inlineStr">
+      <c r="A7" s="1261" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1226" t="inlineStr">
+      <c r="B7" s="1262" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1226" t="inlineStr">
+      <c r="C7" s="1262" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1227" t="n"/>
-      <c r="E7" s="1227" t="n"/>
-      <c r="F7" s="1227" t="n"/>
-      <c r="G7" s="1227" t="n"/>
-      <c r="H7" s="1227" t="n"/>
-      <c r="I7" s="1228" t="n"/>
-      <c r="J7" s="1229" t="n"/>
-      <c r="K7" s="1229" t="n"/>
-      <c r="L7" s="1229" t="n"/>
-      <c r="M7" s="1227" t="n"/>
-      <c r="N7" s="1227" t="n"/>
-      <c r="O7" s="1227" t="n"/>
-      <c r="P7" s="1230" t="n"/>
-      <c r="Q7" s="1227" t="n"/>
-      <c r="R7" s="1227" t="n"/>
-      <c r="S7" s="1227" t="n"/>
+      <c r="D7" s="1263" t="n"/>
+      <c r="E7" s="1263" t="n"/>
+      <c r="F7" s="1263" t="n"/>
+      <c r="G7" s="1263" t="n"/>
+      <c r="H7" s="1263" t="n"/>
+      <c r="I7" s="1264" t="n"/>
+      <c r="J7" s="1265" t="n"/>
+      <c r="K7" s="1265" t="n"/>
+      <c r="L7" s="1265" t="n"/>
+      <c r="M7" s="1263" t="n"/>
+      <c r="N7" s="1263" t="n"/>
+      <c r="O7" s="1263" t="n"/>
+      <c r="P7" s="1266" t="n"/>
+      <c r="Q7" s="1263" t="n"/>
+      <c r="R7" s="1263" t="n"/>
+      <c r="S7" s="1263" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1226" t="n"/>
+      <c r="U7" s="1262" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -4898,39 +5006,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1201" t="inlineStr">
+      <c r="A8" s="1237" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1202" t="inlineStr">
+      <c r="B8" s="1238" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1202" t="inlineStr">
+      <c r="C8" s="1238" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1203" t="n"/>
-      <c r="E8" s="1203" t="n"/>
-      <c r="F8" s="1203" t="n"/>
-      <c r="G8" s="1203" t="n"/>
-      <c r="H8" s="1203" t="n"/>
-      <c r="I8" s="1204" t="n"/>
-      <c r="J8" s="1205" t="n"/>
-      <c r="K8" s="1205" t="n"/>
-      <c r="L8" s="1205" t="n"/>
-      <c r="M8" s="1203" t="n"/>
-      <c r="N8" s="1203" t="n"/>
-      <c r="O8" s="1203" t="n"/>
-      <c r="P8" s="1206" t="n"/>
-      <c r="Q8" s="1203" t="n"/>
-      <c r="R8" s="1203" t="n"/>
-      <c r="S8" s="1203" t="n"/>
+      <c r="D8" s="1239" t="n"/>
+      <c r="E8" s="1239" t="n"/>
+      <c r="F8" s="1239" t="n"/>
+      <c r="G8" s="1239" t="n"/>
+      <c r="H8" s="1239" t="n"/>
+      <c r="I8" s="1240" t="n"/>
+      <c r="J8" s="1241" t="n"/>
+      <c r="K8" s="1241" t="n"/>
+      <c r="L8" s="1241" t="n"/>
+      <c r="M8" s="1239" t="n"/>
+      <c r="N8" s="1239" t="n"/>
+      <c r="O8" s="1239" t="n"/>
+      <c r="P8" s="1242" t="n"/>
+      <c r="Q8" s="1239" t="n"/>
+      <c r="R8" s="1239" t="n"/>
+      <c r="S8" s="1239" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1202" t="n"/>
+      <c r="U8" s="1238" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -4938,63 +5046,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1231" t="inlineStr">
+      <c r="A9" s="1267" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1232" t="inlineStr">
+      <c r="B9" s="1268" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1232" t="inlineStr">
+      <c r="C9" s="1268" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1233" t="n">
+      <c r="D9" s="1269" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1233" t="n">
+      <c r="E9" s="1269" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1233" t="n">
+      <c r="F9" s="1269" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1233" t="n">
+      <c r="G9" s="1269" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1233" t="n"/>
-      <c r="I9" s="1234" t="n"/>
-      <c r="J9" s="1235" t="n">
+      <c r="H9" s="1269" t="n"/>
+      <c r="I9" s="1270" t="n"/>
+      <c r="J9" s="1271" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1235" t="n">
+      <c r="K9" s="1271" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1235" t="inlineStr">
+      <c r="L9" s="1271" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1233" t="n"/>
-      <c r="N9" s="1233" t="n"/>
-      <c r="O9" s="1233" t="n">
+      <c r="M9" s="1269" t="n"/>
+      <c r="N9" s="1269" t="n"/>
+      <c r="O9" s="1269" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1236" t="n">
+      <c r="P9" s="1272" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1233" t="n"/>
-      <c r="R9" s="1233" t="n"/>
-      <c r="S9" s="1233" t="n"/>
+      <c r="Q9" s="1269" t="n"/>
+      <c r="R9" s="1269" t="n"/>
+      <c r="S9" s="1269" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1232" t="n"/>
+      <c r="U9" s="1268" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -5002,43 +5110,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1231" t="inlineStr">
+      <c r="A10" s="1267" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1232" t="inlineStr">
+      <c r="B10" s="1268" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1232" t="inlineStr">
+      <c r="C10" s="1268" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1233" t="n"/>
-      <c r="E10" s="1233" t="n"/>
-      <c r="F10" s="1233" t="n"/>
-      <c r="G10" s="1233" t="n"/>
-      <c r="H10" s="1233" t="n"/>
-      <c r="I10" s="1234" t="n"/>
-      <c r="J10" s="1235" t="n"/>
-      <c r="K10" s="1235" t="n"/>
-      <c r="L10" s="1235" t="inlineStr">
+      <c r="D10" s="1269" t="n"/>
+      <c r="E10" s="1269" t="n"/>
+      <c r="F10" s="1269" t="n"/>
+      <c r="G10" s="1269" t="n"/>
+      <c r="H10" s="1269" t="n"/>
+      <c r="I10" s="1270" t="n"/>
+      <c r="J10" s="1271" t="n"/>
+      <c r="K10" s="1271" t="n"/>
+      <c r="L10" s="1271" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1233" t="n"/>
-      <c r="N10" s="1233" t="n"/>
-      <c r="O10" s="1233" t="n"/>
-      <c r="P10" s="1236" t="n"/>
-      <c r="Q10" s="1233" t="n"/>
-      <c r="R10" s="1233" t="n"/>
-      <c r="S10" s="1233" t="n"/>
+      <c r="M10" s="1269" t="n"/>
+      <c r="N10" s="1269" t="n"/>
+      <c r="O10" s="1269" t="n"/>
+      <c r="P10" s="1272" t="n"/>
+      <c r="Q10" s="1269" t="n"/>
+      <c r="R10" s="1269" t="n"/>
+      <c r="S10" s="1269" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1232" t="n"/>
+      <c r="U10" s="1268" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -5046,43 +5154,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1231" t="inlineStr">
+      <c r="A11" s="1267" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1232" t="inlineStr">
+      <c r="B11" s="1268" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1232" t="inlineStr">
+      <c r="C11" s="1268" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1233" t="n"/>
-      <c r="E11" s="1233" t="n"/>
-      <c r="F11" s="1233" t="n"/>
-      <c r="G11" s="1233" t="n"/>
-      <c r="H11" s="1233" t="n"/>
-      <c r="I11" s="1234" t="n"/>
-      <c r="J11" s="1235" t="n"/>
-      <c r="K11" s="1235" t="n"/>
-      <c r="L11" s="1235" t="n"/>
-      <c r="M11" s="1233" t="n">
+      <c r="D11" s="1269" t="n"/>
+      <c r="E11" s="1269" t="n"/>
+      <c r="F11" s="1269" t="n"/>
+      <c r="G11" s="1269" t="n"/>
+      <c r="H11" s="1269" t="n"/>
+      <c r="I11" s="1270" t="n"/>
+      <c r="J11" s="1271" t="n"/>
+      <c r="K11" s="1271" t="n"/>
+      <c r="L11" s="1271" t="n"/>
+      <c r="M11" s="1269" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1233" t="n">
+      <c r="N11" s="1269" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1233" t="n"/>
-      <c r="P11" s="1236" t="n"/>
-      <c r="Q11" s="1233" t="n"/>
-      <c r="R11" s="1233" t="n"/>
-      <c r="S11" s="1233" t="n"/>
+      <c r="O11" s="1269" t="n"/>
+      <c r="P11" s="1272" t="n"/>
+      <c r="Q11" s="1269" t="n"/>
+      <c r="R11" s="1269" t="n"/>
+      <c r="S11" s="1269" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1232" t="n"/>
+      <c r="U11" s="1268" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -5090,39 +5198,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1207" t="inlineStr">
+      <c r="A12" s="1243" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1208" t="inlineStr">
+      <c r="B12" s="1244" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1208" t="inlineStr">
+      <c r="C12" s="1244" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1209" t="n"/>
-      <c r="E12" s="1209" t="n"/>
-      <c r="F12" s="1209" t="n"/>
-      <c r="G12" s="1209" t="n"/>
-      <c r="H12" s="1209" t="n"/>
-      <c r="I12" s="1210" t="n"/>
-      <c r="J12" s="1211" t="n"/>
-      <c r="K12" s="1211" t="n"/>
-      <c r="L12" s="1211" t="n"/>
-      <c r="M12" s="1209" t="n"/>
-      <c r="N12" s="1209" t="n"/>
-      <c r="O12" s="1209" t="n"/>
-      <c r="P12" s="1212" t="n"/>
-      <c r="Q12" s="1209" t="n"/>
-      <c r="R12" s="1209" t="n"/>
-      <c r="S12" s="1209" t="n"/>
+      <c r="D12" s="1245" t="n"/>
+      <c r="E12" s="1245" t="n"/>
+      <c r="F12" s="1245" t="n"/>
+      <c r="G12" s="1245" t="n"/>
+      <c r="H12" s="1245" t="n"/>
+      <c r="I12" s="1246" t="n"/>
+      <c r="J12" s="1247" t="n"/>
+      <c r="K12" s="1247" t="n"/>
+      <c r="L12" s="1247" t="n"/>
+      <c r="M12" s="1245" t="n"/>
+      <c r="N12" s="1245" t="n"/>
+      <c r="O12" s="1245" t="n"/>
+      <c r="P12" s="1248" t="n"/>
+      <c r="Q12" s="1245" t="n"/>
+      <c r="R12" s="1245" t="n"/>
+      <c r="S12" s="1245" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1208" t="n"/>
+      <c r="U12" s="1244" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5130,35 +5238,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1213" t="inlineStr">
+      <c r="A13" s="1249" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1214" t="n"/>
-      <c r="C13" s="1214" t="inlineStr">
+      <c r="B13" s="1250" t="n"/>
+      <c r="C13" s="1250" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1215" t="n"/>
-      <c r="E13" s="1215" t="n"/>
-      <c r="F13" s="1215" t="n"/>
-      <c r="G13" s="1215" t="n"/>
-      <c r="H13" s="1215" t="n"/>
-      <c r="I13" s="1216" t="n"/>
-      <c r="J13" s="1217" t="n"/>
-      <c r="K13" s="1217" t="n"/>
-      <c r="L13" s="1217" t="n"/>
-      <c r="M13" s="1215" t="n"/>
-      <c r="N13" s="1215" t="n"/>
-      <c r="O13" s="1215" t="n"/>
-      <c r="P13" s="1218" t="n"/>
-      <c r="Q13" s="1215" t="n"/>
-      <c r="R13" s="1215" t="n"/>
-      <c r="S13" s="1215" t="n"/>
+      <c r="D13" s="1251" t="n"/>
+      <c r="E13" s="1251" t="n"/>
+      <c r="F13" s="1251" t="n"/>
+      <c r="G13" s="1251" t="n"/>
+      <c r="H13" s="1251" t="n"/>
+      <c r="I13" s="1252" t="n"/>
+      <c r="J13" s="1253" t="n"/>
+      <c r="K13" s="1253" t="n"/>
+      <c r="L13" s="1253" t="n"/>
+      <c r="M13" s="1251" t="n"/>
+      <c r="N13" s="1251" t="n"/>
+      <c r="O13" s="1251" t="n"/>
+      <c r="P13" s="1254" t="n"/>
+      <c r="Q13" s="1251" t="n"/>
+      <c r="R13" s="1251" t="n"/>
+      <c r="S13" s="1251" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1214" t="n"/>
+      <c r="U13" s="1250" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -5166,53 +5274,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1219" t="inlineStr">
+      <c r="A14" s="1255" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1220" t="inlineStr">
+      <c r="B14" s="1256" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1220" t="inlineStr">
+      <c r="C14" s="1256" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1221" t="n"/>
-      <c r="E14" s="1221" t="n">
+      <c r="D14" s="1257" t="n"/>
+      <c r="E14" s="1257" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1221" t="n">
+      <c r="F14" s="1257" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1221" t="n">
+      <c r="G14" s="1257" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1221" t="n"/>
-      <c r="I14" s="1222" t="n"/>
-      <c r="J14" s="1223" t="n"/>
-      <c r="K14" s="1223" t="n"/>
-      <c r="L14" s="1223" t="n"/>
-      <c r="M14" s="1221" t="n"/>
-      <c r="N14" s="1221" t="n"/>
-      <c r="O14" s="1221" t="n">
+      <c r="H14" s="1257" t="n"/>
+      <c r="I14" s="1258" t="n"/>
+      <c r="J14" s="1259" t="n"/>
+      <c r="K14" s="1259" t="n"/>
+      <c r="L14" s="1259" t="n"/>
+      <c r="M14" s="1257" t="n"/>
+      <c r="N14" s="1257" t="n"/>
+      <c r="O14" s="1257" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1224" t="n">
+      <c r="P14" s="1260" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1221" t="n"/>
-      <c r="R14" s="1221" t="n"/>
-      <c r="S14" s="1221" t="n"/>
+      <c r="Q14" s="1257" t="n"/>
+      <c r="R14" s="1257" t="n"/>
+      <c r="S14" s="1257" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1220" t="n"/>
+      <c r="U14" s="1256" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -5220,43 +5328,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1219" t="inlineStr">
+      <c r="A15" s="1255" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1220" t="inlineStr">
+      <c r="B15" s="1256" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1220" t="inlineStr">
+      <c r="C15" s="1256" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1221" t="n"/>
-      <c r="E15" s="1221" t="n"/>
-      <c r="F15" s="1221" t="n"/>
-      <c r="G15" s="1221" t="n"/>
-      <c r="H15" s="1221" t="n"/>
-      <c r="I15" s="1222" t="n"/>
-      <c r="J15" s="1223" t="n"/>
-      <c r="K15" s="1223" t="n"/>
-      <c r="L15" s="1223" t="n"/>
-      <c r="M15" s="1221" t="n">
+      <c r="D15" s="1257" t="n"/>
+      <c r="E15" s="1257" t="n"/>
+      <c r="F15" s="1257" t="n"/>
+      <c r="G15" s="1257" t="n"/>
+      <c r="H15" s="1257" t="n"/>
+      <c r="I15" s="1258" t="n"/>
+      <c r="J15" s="1259" t="n"/>
+      <c r="K15" s="1259" t="n"/>
+      <c r="L15" s="1259" t="n"/>
+      <c r="M15" s="1257" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1221" t="n">
+      <c r="N15" s="1257" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1221" t="n"/>
-      <c r="P15" s="1224" t="n"/>
-      <c r="Q15" s="1221" t="n"/>
-      <c r="R15" s="1221" t="n"/>
-      <c r="S15" s="1221" t="n"/>
+      <c r="O15" s="1257" t="n"/>
+      <c r="P15" s="1260" t="n"/>
+      <c r="Q15" s="1257" t="n"/>
+      <c r="R15" s="1257" t="n"/>
+      <c r="S15" s="1257" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1220" t="n"/>
+      <c r="U15" s="1256" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -5264,39 +5372,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1225" t="inlineStr">
+      <c r="A16" s="1261" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1226" t="inlineStr">
+      <c r="B16" s="1262" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1226" t="inlineStr">
+      <c r="C16" s="1262" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1227" t="n"/>
-      <c r="E16" s="1227" t="n"/>
-      <c r="F16" s="1227" t="n"/>
-      <c r="G16" s="1227" t="n"/>
-      <c r="H16" s="1227" t="n"/>
-      <c r="I16" s="1228" t="n"/>
-      <c r="J16" s="1229" t="n"/>
-      <c r="K16" s="1229" t="n"/>
-      <c r="L16" s="1229" t="n"/>
-      <c r="M16" s="1227" t="n"/>
-      <c r="N16" s="1227" t="n"/>
-      <c r="O16" s="1227" t="n"/>
-      <c r="P16" s="1230" t="n"/>
-      <c r="Q16" s="1227" t="n"/>
-      <c r="R16" s="1227" t="n"/>
-      <c r="S16" s="1227" t="n"/>
+      <c r="D16" s="1263" t="n"/>
+      <c r="E16" s="1263" t="n"/>
+      <c r="F16" s="1263" t="n"/>
+      <c r="G16" s="1263" t="n"/>
+      <c r="H16" s="1263" t="n"/>
+      <c r="I16" s="1264" t="n"/>
+      <c r="J16" s="1265" t="n"/>
+      <c r="K16" s="1265" t="n"/>
+      <c r="L16" s="1265" t="n"/>
+      <c r="M16" s="1263" t="n"/>
+      <c r="N16" s="1263" t="n"/>
+      <c r="O16" s="1263" t="n"/>
+      <c r="P16" s="1266" t="n"/>
+      <c r="Q16" s="1263" t="n"/>
+      <c r="R16" s="1263" t="n"/>
+      <c r="S16" s="1263" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1226" t="n"/>
+      <c r="U16" s="1262" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -5304,39 +5412,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1201" t="inlineStr">
+      <c r="A17" s="1237" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1202" t="inlineStr">
+      <c r="B17" s="1238" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1202" t="inlineStr">
+      <c r="C17" s="1238" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1203" t="n"/>
-      <c r="E17" s="1203" t="n"/>
-      <c r="F17" s="1203" t="n"/>
-      <c r="G17" s="1203" t="n"/>
-      <c r="H17" s="1203" t="n"/>
-      <c r="I17" s="1204" t="n"/>
-      <c r="J17" s="1205" t="n"/>
-      <c r="K17" s="1205" t="n"/>
-      <c r="L17" s="1205" t="n"/>
-      <c r="M17" s="1203" t="n"/>
-      <c r="N17" s="1203" t="n"/>
-      <c r="O17" s="1203" t="n"/>
-      <c r="P17" s="1206" t="n"/>
-      <c r="Q17" s="1203" t="n"/>
-      <c r="R17" s="1203" t="n"/>
-      <c r="S17" s="1203" t="n"/>
+      <c r="D17" s="1239" t="n"/>
+      <c r="E17" s="1239" t="n"/>
+      <c r="F17" s="1239" t="n"/>
+      <c r="G17" s="1239" t="n"/>
+      <c r="H17" s="1239" t="n"/>
+      <c r="I17" s="1240" t="n"/>
+      <c r="J17" s="1241" t="n"/>
+      <c r="K17" s="1241" t="n"/>
+      <c r="L17" s="1241" t="n"/>
+      <c r="M17" s="1239" t="n"/>
+      <c r="N17" s="1239" t="n"/>
+      <c r="O17" s="1239" t="n"/>
+      <c r="P17" s="1242" t="n"/>
+      <c r="Q17" s="1239" t="n"/>
+      <c r="R17" s="1239" t="n"/>
+      <c r="S17" s="1239" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1202" t="n"/>
+      <c r="U17" s="1238" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -5344,53 +5452,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1231" t="inlineStr">
+      <c r="A18" s="1267" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1232" t="inlineStr">
+      <c r="B18" s="1268" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1232" t="inlineStr">
+      <c r="C18" s="1268" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1233" t="n"/>
-      <c r="E18" s="1233" t="n">
+      <c r="D18" s="1269" t="n"/>
+      <c r="E18" s="1269" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1233" t="n">
+      <c r="F18" s="1269" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1233" t="n">
+      <c r="G18" s="1269" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1233" t="n"/>
-      <c r="I18" s="1234" t="n"/>
-      <c r="J18" s="1235" t="n"/>
-      <c r="K18" s="1235" t="n"/>
-      <c r="L18" s="1235" t="n"/>
-      <c r="M18" s="1233" t="n"/>
-      <c r="N18" s="1233" t="n"/>
-      <c r="O18" s="1233" t="n">
+      <c r="H18" s="1269" t="n"/>
+      <c r="I18" s="1270" t="n"/>
+      <c r="J18" s="1271" t="n"/>
+      <c r="K18" s="1271" t="n"/>
+      <c r="L18" s="1271" t="n"/>
+      <c r="M18" s="1269" t="n"/>
+      <c r="N18" s="1269" t="n"/>
+      <c r="O18" s="1269" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1236" t="n">
+      <c r="P18" s="1272" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1233" t="n"/>
-      <c r="R18" s="1233" t="n"/>
-      <c r="S18" s="1233" t="n"/>
+      <c r="Q18" s="1269" t="n"/>
+      <c r="R18" s="1269" t="n"/>
+      <c r="S18" s="1269" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1232" t="n"/>
+      <c r="U18" s="1268" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -5398,47 +5506,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1231" t="inlineStr">
+      <c r="A19" s="1267" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1232" t="inlineStr">
+      <c r="B19" s="1268" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1232" t="inlineStr">
+      <c r="C19" s="1268" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1233" t="n"/>
-      <c r="E19" s="1233" t="n"/>
-      <c r="F19" s="1233" t="n"/>
-      <c r="G19" s="1233" t="n"/>
-      <c r="H19" s="1233" t="n"/>
-      <c r="I19" s="1234" t="n"/>
-      <c r="J19" s="1235" t="n"/>
-      <c r="K19" s="1235" t="n"/>
-      <c r="L19" s="1235" t="n"/>
-      <c r="M19" s="1233" t="n">
+      <c r="D19" s="1269" t="n"/>
+      <c r="E19" s="1269" t="n"/>
+      <c r="F19" s="1269" t="n"/>
+      <c r="G19" s="1269" t="n"/>
+      <c r="H19" s="1269" t="n"/>
+      <c r="I19" s="1270" t="n"/>
+      <c r="J19" s="1271" t="n"/>
+      <c r="K19" s="1271" t="n"/>
+      <c r="L19" s="1271" t="n"/>
+      <c r="M19" s="1269" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1233" t="n">
+      <c r="N19" s="1269" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1233" t="n"/>
-      <c r="P19" s="1236" t="n"/>
-      <c r="Q19" s="1233" t="n"/>
-      <c r="R19" s="1233" t="n"/>
-      <c r="S19" s="1233" t="n"/>
+      <c r="O19" s="1269" t="n"/>
+      <c r="P19" s="1272" t="n"/>
+      <c r="Q19" s="1269" t="n"/>
+      <c r="R19" s="1269" t="n"/>
+      <c r="S19" s="1269" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1232" t="n"/>
+      <c r="U19" s="1268" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -5446,43 +5554,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1231" t="inlineStr">
+      <c r="A20" s="1267" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1232" t="inlineStr">
+      <c r="B20" s="1268" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1232" t="inlineStr">
+      <c r="C20" s="1268" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1233" t="n"/>
-      <c r="E20" s="1233" t="n"/>
-      <c r="F20" s="1233" t="n"/>
-      <c r="G20" s="1233" t="n"/>
-      <c r="H20" s="1233" t="n"/>
-      <c r="I20" s="1234" t="n"/>
-      <c r="J20" s="1235" t="n"/>
-      <c r="K20" s="1235" t="n"/>
-      <c r="L20" s="1235" t="n"/>
-      <c r="M20" s="1233" t="n"/>
-      <c r="N20" s="1233" t="n"/>
-      <c r="O20" s="1233" t="n"/>
-      <c r="P20" s="1236" t="n"/>
-      <c r="Q20" s="1233" t="n"/>
-      <c r="R20" s="1233" t="n"/>
-      <c r="S20" s="1233" t="n"/>
+      <c r="D20" s="1269" t="n"/>
+      <c r="E20" s="1269" t="n"/>
+      <c r="F20" s="1269" t="n"/>
+      <c r="G20" s="1269" t="n"/>
+      <c r="H20" s="1269" t="n"/>
+      <c r="I20" s="1270" t="n"/>
+      <c r="J20" s="1271" t="n"/>
+      <c r="K20" s="1271" t="n"/>
+      <c r="L20" s="1271" t="n"/>
+      <c r="M20" s="1269" t="n"/>
+      <c r="N20" s="1269" t="n"/>
+      <c r="O20" s="1269" t="n"/>
+      <c r="P20" s="1272" t="n"/>
+      <c r="Q20" s="1269" t="n"/>
+      <c r="R20" s="1269" t="n"/>
+      <c r="S20" s="1269" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1232" t="n"/>
+      <c r="U20" s="1268" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -5490,39 +5598,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1207" t="inlineStr">
+      <c r="A21" s="1243" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1208" t="inlineStr">
+      <c r="B21" s="1244" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1208" t="inlineStr">
+      <c r="C21" s="1244" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1209" t="n"/>
-      <c r="E21" s="1209" t="n"/>
-      <c r="F21" s="1209" t="n"/>
-      <c r="G21" s="1209" t="n"/>
-      <c r="H21" s="1209" t="n"/>
-      <c r="I21" s="1210" t="n"/>
-      <c r="J21" s="1211" t="n"/>
-      <c r="K21" s="1211" t="n"/>
-      <c r="L21" s="1211" t="n"/>
-      <c r="M21" s="1209" t="n"/>
-      <c r="N21" s="1209" t="n"/>
-      <c r="O21" s="1209" t="n"/>
-      <c r="P21" s="1212" t="n"/>
-      <c r="Q21" s="1209" t="n"/>
-      <c r="R21" s="1209" t="n"/>
-      <c r="S21" s="1209" t="n"/>
+      <c r="D21" s="1245" t="n"/>
+      <c r="E21" s="1245" t="n"/>
+      <c r="F21" s="1245" t="n"/>
+      <c r="G21" s="1245" t="n"/>
+      <c r="H21" s="1245" t="n"/>
+      <c r="I21" s="1246" t="n"/>
+      <c r="J21" s="1247" t="n"/>
+      <c r="K21" s="1247" t="n"/>
+      <c r="L21" s="1247" t="n"/>
+      <c r="M21" s="1245" t="n"/>
+      <c r="N21" s="1245" t="n"/>
+      <c r="O21" s="1245" t="n"/>
+      <c r="P21" s="1248" t="n"/>
+      <c r="Q21" s="1245" t="n"/>
+      <c r="R21" s="1245" t="n"/>
+      <c r="S21" s="1245" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1208" t="n"/>
+      <c r="U21" s="1244" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -5530,39 +5638,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1213" t="inlineStr">
+      <c r="A22" s="1249" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1214" t="inlineStr">
+      <c r="B22" s="1250" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1214" t="inlineStr">
+      <c r="C22" s="1250" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1215" t="n"/>
-      <c r="E22" s="1215" t="n"/>
-      <c r="F22" s="1215" t="n"/>
-      <c r="G22" s="1215" t="n"/>
-      <c r="H22" s="1215" t="n"/>
-      <c r="I22" s="1216" t="n"/>
-      <c r="J22" s="1217" t="n"/>
-      <c r="K22" s="1217" t="n"/>
-      <c r="L22" s="1217" t="n"/>
-      <c r="M22" s="1215" t="n"/>
-      <c r="N22" s="1215" t="n"/>
-      <c r="O22" s="1215" t="n"/>
-      <c r="P22" s="1218" t="n"/>
-      <c r="Q22" s="1215" t="n"/>
-      <c r="R22" s="1215" t="n"/>
-      <c r="S22" s="1215" t="n"/>
+      <c r="D22" s="1251" t="n"/>
+      <c r="E22" s="1251" t="n"/>
+      <c r="F22" s="1251" t="n"/>
+      <c r="G22" s="1251" t="n"/>
+      <c r="H22" s="1251" t="n"/>
+      <c r="I22" s="1252" t="n"/>
+      <c r="J22" s="1253" t="n"/>
+      <c r="K22" s="1253" t="n"/>
+      <c r="L22" s="1253" t="n"/>
+      <c r="M22" s="1251" t="n"/>
+      <c r="N22" s="1251" t="n"/>
+      <c r="O22" s="1251" t="n"/>
+      <c r="P22" s="1254" t="n"/>
+      <c r="Q22" s="1251" t="n"/>
+      <c r="R22" s="1251" t="n"/>
+      <c r="S22" s="1251" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1214" t="n"/>
+      <c r="U22" s="1250" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -5570,53 +5678,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1219" t="inlineStr">
+      <c r="A23" s="1255" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1220" t="inlineStr">
+      <c r="B23" s="1256" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1220" t="inlineStr">
+      <c r="C23" s="1256" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1221" t="n"/>
-      <c r="E23" s="1221" t="n">
+      <c r="D23" s="1257" t="n"/>
+      <c r="E23" s="1257" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1221" t="n">
+      <c r="F23" s="1257" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1221" t="n">
+      <c r="G23" s="1257" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1221" t="n"/>
-      <c r="I23" s="1222" t="n"/>
-      <c r="J23" s="1223" t="n"/>
-      <c r="K23" s="1223" t="n"/>
-      <c r="L23" s="1223" t="n"/>
-      <c r="M23" s="1221" t="n"/>
-      <c r="N23" s="1221" t="n"/>
-      <c r="O23" s="1221" t="n">
+      <c r="H23" s="1257" t="n"/>
+      <c r="I23" s="1258" t="n"/>
+      <c r="J23" s="1259" t="n"/>
+      <c r="K23" s="1259" t="n"/>
+      <c r="L23" s="1259" t="n"/>
+      <c r="M23" s="1257" t="n"/>
+      <c r="N23" s="1257" t="n"/>
+      <c r="O23" s="1257" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1224" t="n">
+      <c r="P23" s="1260" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1221" t="n"/>
-      <c r="R23" s="1221" t="n"/>
-      <c r="S23" s="1221" t="n"/>
+      <c r="Q23" s="1257" t="n"/>
+      <c r="R23" s="1257" t="n"/>
+      <c r="S23" s="1257" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1220" t="n"/>
+      <c r="U23" s="1256" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -5624,47 +5732,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1225" t="inlineStr">
+      <c r="A24" s="1261" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1226" t="inlineStr">
+      <c r="B24" s="1262" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1226" t="inlineStr">
+      <c r="C24" s="1262" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1227" t="n"/>
-      <c r="E24" s="1227" t="n"/>
-      <c r="F24" s="1227" t="n"/>
-      <c r="G24" s="1227" t="n"/>
-      <c r="H24" s="1227" t="n"/>
-      <c r="I24" s="1228" t="n"/>
-      <c r="J24" s="1229" t="n"/>
-      <c r="K24" s="1229" t="n"/>
-      <c r="L24" s="1229" t="n"/>
-      <c r="M24" s="1227" t="n">
+      <c r="D24" s="1263" t="n"/>
+      <c r="E24" s="1263" t="n"/>
+      <c r="F24" s="1263" t="n"/>
+      <c r="G24" s="1263" t="n"/>
+      <c r="H24" s="1263" t="n"/>
+      <c r="I24" s="1264" t="n"/>
+      <c r="J24" s="1265" t="n"/>
+      <c r="K24" s="1265" t="n"/>
+      <c r="L24" s="1265" t="n"/>
+      <c r="M24" s="1263" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1227" t="n">
+      <c r="N24" s="1263" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1227" t="n"/>
-      <c r="P24" s="1230" t="n"/>
-      <c r="Q24" s="1227" t="n"/>
-      <c r="R24" s="1227" t="n"/>
-      <c r="S24" s="1227" t="n"/>
+      <c r="O24" s="1263" t="n"/>
+      <c r="P24" s="1266" t="n"/>
+      <c r="Q24" s="1263" t="n"/>
+      <c r="R24" s="1263" t="n"/>
+      <c r="S24" s="1263" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1226" t="n"/>
+      <c r="U24" s="1262" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -5672,61 +5780,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1201" t="inlineStr">
+      <c r="A25" s="1237" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1202" t="inlineStr">
+      <c r="B25" s="1238" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1202" t="inlineStr">
+      <c r="C25" s="1238" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1203" t="n">
+      <c r="D25" s="1239" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1203" t="n">
+      <c r="E25" s="1239" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1203" t="n">
+      <c r="F25" s="1239" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1203" t="n">
+      <c r="G25" s="1239" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1203" t="n"/>
-      <c r="I25" s="1204" t="n"/>
-      <c r="J25" s="1205" t="n">
+      <c r="H25" s="1239" t="n"/>
+      <c r="I25" s="1240" t="n"/>
+      <c r="J25" s="1241" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1205" t="n">
+      <c r="K25" s="1241" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1205" t="n">
+      <c r="L25" s="1241" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1203" t="n"/>
-      <c r="N25" s="1203" t="n"/>
-      <c r="O25" s="1203" t="n">
+      <c r="M25" s="1239" t="n"/>
+      <c r="N25" s="1239" t="n"/>
+      <c r="O25" s="1239" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1206" t="n">
+      <c r="P25" s="1242" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1203" t="n"/>
-      <c r="R25" s="1203" t="n"/>
-      <c r="S25" s="1203" t="n"/>
+      <c r="Q25" s="1239" t="n"/>
+      <c r="R25" s="1239" t="n"/>
+      <c r="S25" s="1239" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1202" t="n"/>
+      <c r="U25" s="1238" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -5734,47 +5842,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1207" t="inlineStr">
+      <c r="A26" s="1243" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1208" t="inlineStr">
+      <c r="B26" s="1244" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1208" t="inlineStr">
+      <c r="C26" s="1244" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1209" t="n"/>
-      <c r="E26" s="1209" t="n"/>
-      <c r="F26" s="1209" t="n"/>
-      <c r="G26" s="1209" t="n"/>
-      <c r="H26" s="1209" t="n"/>
-      <c r="I26" s="1210" t="n"/>
-      <c r="J26" s="1211" t="n"/>
-      <c r="K26" s="1211" t="n"/>
-      <c r="L26" s="1211" t="n"/>
-      <c r="M26" s="1209" t="n">
+      <c r="D26" s="1245" t="n"/>
+      <c r="E26" s="1245" t="n"/>
+      <c r="F26" s="1245" t="n"/>
+      <c r="G26" s="1245" t="n"/>
+      <c r="H26" s="1245" t="n"/>
+      <c r="I26" s="1246" t="n"/>
+      <c r="J26" s="1247" t="n"/>
+      <c r="K26" s="1247" t="n"/>
+      <c r="L26" s="1247" t="n"/>
+      <c r="M26" s="1245" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1209" t="n">
+      <c r="N26" s="1245" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1209" t="n"/>
-      <c r="P26" s="1212" t="n"/>
-      <c r="Q26" s="1209" t="n"/>
-      <c r="R26" s="1209" t="n"/>
-      <c r="S26" s="1209" t="n"/>
+      <c r="O26" s="1245" t="n"/>
+      <c r="P26" s="1248" t="n"/>
+      <c r="Q26" s="1245" t="n"/>
+      <c r="R26" s="1245" t="n"/>
+      <c r="S26" s="1245" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1208" t="n"/>
+      <c r="U26" s="1244" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -5782,53 +5890,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1213" t="inlineStr">
+      <c r="A27" s="1249" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1214" t="inlineStr">
+      <c r="B27" s="1250" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1214" t="inlineStr">
+      <c r="C27" s="1250" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1215" t="n"/>
-      <c r="E27" s="1215" t="n">
+      <c r="D27" s="1251" t="n"/>
+      <c r="E27" s="1251" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1215" t="n">
+      <c r="F27" s="1251" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1215" t="n">
+      <c r="G27" s="1251" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1215" t="n"/>
-      <c r="I27" s="1216" t="n"/>
-      <c r="J27" s="1217" t="n"/>
-      <c r="K27" s="1217" t="n"/>
-      <c r="L27" s="1217" t="n"/>
-      <c r="M27" s="1215" t="n"/>
-      <c r="N27" s="1215" t="n"/>
-      <c r="O27" s="1215" t="n">
+      <c r="H27" s="1251" t="n"/>
+      <c r="I27" s="1252" t="n"/>
+      <c r="J27" s="1253" t="n"/>
+      <c r="K27" s="1253" t="n"/>
+      <c r="L27" s="1253" t="n"/>
+      <c r="M27" s="1251" t="n"/>
+      <c r="N27" s="1251" t="n"/>
+      <c r="O27" s="1251" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1218" t="n">
+      <c r="P27" s="1254" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1215" t="n"/>
-      <c r="R27" s="1215" t="n"/>
-      <c r="S27" s="1215" t="n"/>
+      <c r="Q27" s="1251" t="n"/>
+      <c r="R27" s="1251" t="n"/>
+      <c r="S27" s="1251" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1214" t="n"/>
+      <c r="U27" s="1250" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -5836,47 +5944,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1225" t="inlineStr">
+      <c r="A28" s="1261" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1226" t="inlineStr">
+      <c r="B28" s="1262" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1226" t="inlineStr">
+      <c r="C28" s="1262" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1227" t="n"/>
-      <c r="E28" s="1227" t="n"/>
-      <c r="F28" s="1227" t="n"/>
-      <c r="G28" s="1227" t="n"/>
-      <c r="H28" s="1227" t="n"/>
-      <c r="I28" s="1228" t="n"/>
-      <c r="J28" s="1229" t="n"/>
-      <c r="K28" s="1229" t="n"/>
-      <c r="L28" s="1229" t="n"/>
-      <c r="M28" s="1227" t="n">
+      <c r="D28" s="1263" t="n"/>
+      <c r="E28" s="1263" t="n"/>
+      <c r="F28" s="1263" t="n"/>
+      <c r="G28" s="1263" t="n"/>
+      <c r="H28" s="1263" t="n"/>
+      <c r="I28" s="1264" t="n"/>
+      <c r="J28" s="1265" t="n"/>
+      <c r="K28" s="1265" t="n"/>
+      <c r="L28" s="1265" t="n"/>
+      <c r="M28" s="1263" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1227" t="n">
+      <c r="N28" s="1263" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1227" t="n"/>
-      <c r="P28" s="1230" t="n"/>
-      <c r="Q28" s="1227" t="n"/>
-      <c r="R28" s="1227" t="n"/>
-      <c r="S28" s="1227" t="n"/>
+      <c r="O28" s="1263" t="n"/>
+      <c r="P28" s="1266" t="n"/>
+      <c r="Q28" s="1263" t="n"/>
+      <c r="R28" s="1263" t="n"/>
+      <c r="S28" s="1263" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1226" t="n"/>
+      <c r="U28" s="1262" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -5884,53 +5992,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1201" t="inlineStr">
+      <c r="A29" s="1237" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1202" t="inlineStr">
+      <c r="B29" s="1238" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1202" t="inlineStr">
+      <c r="C29" s="1238" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1203" t="n"/>
-      <c r="E29" s="1203" t="n">
+      <c r="D29" s="1239" t="n"/>
+      <c r="E29" s="1239" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1203" t="n">
+      <c r="F29" s="1239" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1203" t="n">
+      <c r="G29" s="1239" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1203" t="n"/>
-      <c r="I29" s="1204" t="n"/>
-      <c r="J29" s="1205" t="n"/>
-      <c r="K29" s="1205" t="n"/>
-      <c r="L29" s="1205" t="n"/>
-      <c r="M29" s="1203" t="n"/>
-      <c r="N29" s="1203" t="n"/>
-      <c r="O29" s="1203" t="n">
+      <c r="H29" s="1239" t="n"/>
+      <c r="I29" s="1240" t="n"/>
+      <c r="J29" s="1241" t="n"/>
+      <c r="K29" s="1241" t="n"/>
+      <c r="L29" s="1241" t="n"/>
+      <c r="M29" s="1239" t="n"/>
+      <c r="N29" s="1239" t="n"/>
+      <c r="O29" s="1239" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1206" t="n">
+      <c r="P29" s="1242" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1203" t="n"/>
-      <c r="R29" s="1203" t="n"/>
-      <c r="S29" s="1203" t="n"/>
+      <c r="Q29" s="1239" t="n"/>
+      <c r="R29" s="1239" t="n"/>
+      <c r="S29" s="1239" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1202" t="n"/>
+      <c r="U29" s="1238" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -5938,43 +6046,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1207" t="inlineStr">
+      <c r="A30" s="1243" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1208" t="inlineStr">
+      <c r="B30" s="1244" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1208" t="inlineStr">
+      <c r="C30" s="1244" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1209" t="n"/>
-      <c r="E30" s="1209" t="n"/>
-      <c r="F30" s="1209" t="n"/>
-      <c r="G30" s="1209" t="n"/>
-      <c r="H30" s="1209" t="n"/>
-      <c r="I30" s="1210" t="n"/>
-      <c r="J30" s="1211" t="n"/>
-      <c r="K30" s="1211" t="n"/>
-      <c r="L30" s="1211" t="n"/>
-      <c r="M30" s="1209" t="n"/>
-      <c r="N30" s="1209" t="n"/>
-      <c r="O30" s="1209" t="n"/>
-      <c r="P30" s="1212" t="n"/>
-      <c r="Q30" s="1209" t="n"/>
-      <c r="R30" s="1209" t="n"/>
-      <c r="S30" s="1209" t="n"/>
+      <c r="D30" s="1245" t="n"/>
+      <c r="E30" s="1245" t="n"/>
+      <c r="F30" s="1245" t="n"/>
+      <c r="G30" s="1245" t="n"/>
+      <c r="H30" s="1245" t="n"/>
+      <c r="I30" s="1246" t="n"/>
+      <c r="J30" s="1247" t="n"/>
+      <c r="K30" s="1247" t="n"/>
+      <c r="L30" s="1247" t="n"/>
+      <c r="M30" s="1245" t="n"/>
+      <c r="N30" s="1245" t="n"/>
+      <c r="O30" s="1245" t="n"/>
+      <c r="P30" s="1248" t="n"/>
+      <c r="Q30" s="1245" t="n"/>
+      <c r="R30" s="1245" t="n"/>
+      <c r="S30" s="1245" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1208" t="n"/>
+      <c r="U30" s="1244" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -5982,53 +6090,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1213" t="inlineStr">
+      <c r="A31" s="1249" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1214" t="inlineStr">
+      <c r="B31" s="1250" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1214" t="inlineStr">
+      <c r="C31" s="1250" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1215" t="n"/>
-      <c r="E31" s="1215" t="n">
+      <c r="D31" s="1251" t="n"/>
+      <c r="E31" s="1251" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1215" t="n">
+      <c r="F31" s="1251" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1215" t="n">
+      <c r="G31" s="1251" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1215" t="n"/>
-      <c r="I31" s="1216" t="n"/>
-      <c r="J31" s="1217" t="n"/>
-      <c r="K31" s="1217" t="n"/>
-      <c r="L31" s="1217" t="n"/>
-      <c r="M31" s="1215" t="n"/>
-      <c r="N31" s="1215" t="n"/>
-      <c r="O31" s="1215" t="n">
+      <c r="H31" s="1251" t="n"/>
+      <c r="I31" s="1252" t="n"/>
+      <c r="J31" s="1253" t="n"/>
+      <c r="K31" s="1253" t="n"/>
+      <c r="L31" s="1253" t="n"/>
+      <c r="M31" s="1251" t="n"/>
+      <c r="N31" s="1251" t="n"/>
+      <c r="O31" s="1251" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1218" t="n">
+      <c r="P31" s="1254" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1215" t="n"/>
-      <c r="R31" s="1215" t="n"/>
-      <c r="S31" s="1215" t="n"/>
+      <c r="Q31" s="1251" t="n"/>
+      <c r="R31" s="1251" t="n"/>
+      <c r="S31" s="1251" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1214" t="inlineStr">
+      <c r="U31" s="1250" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -6040,49 +6148,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1225" t="inlineStr">
+      <c r="A32" s="1261" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1226" t="inlineStr">
+      <c r="B32" s="1262" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1226" t="inlineStr">
+      <c r="C32" s="1262" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1227" t="n"/>
-      <c r="E32" s="1227" t="n"/>
-      <c r="F32" s="1227" t="n"/>
-      <c r="G32" s="1227" t="n"/>
-      <c r="H32" s="1227" t="n">
+      <c r="D32" s="1263" t="n"/>
+      <c r="E32" s="1263" t="n"/>
+      <c r="F32" s="1263" t="n"/>
+      <c r="G32" s="1263" t="n"/>
+      <c r="H32" s="1263" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1228" t="n"/>
-      <c r="J32" s="1229" t="n"/>
-      <c r="K32" s="1229" t="n"/>
-      <c r="L32" s="1229" t="n"/>
-      <c r="M32" s="1227" t="n">
+      <c r="I32" s="1264" t="n"/>
+      <c r="J32" s="1265" t="n"/>
+      <c r="K32" s="1265" t="n"/>
+      <c r="L32" s="1265" t="n"/>
+      <c r="M32" s="1263" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1227" t="n">
+      <c r="N32" s="1263" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1227" t="n"/>
-      <c r="P32" s="1230" t="n"/>
-      <c r="Q32" s="1227" t="n"/>
-      <c r="R32" s="1227" t="n"/>
-      <c r="S32" s="1227" t="n"/>
+      <c r="O32" s="1263" t="n"/>
+      <c r="P32" s="1266" t="n"/>
+      <c r="Q32" s="1263" t="n"/>
+      <c r="R32" s="1263" t="n"/>
+      <c r="S32" s="1263" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1226" t="n"/>
+      <c r="U32" s="1262" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -6090,57 +6198,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1201" t="inlineStr">
+      <c r="A33" s="1237" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1202" t="inlineStr">
+      <c r="B33" s="1238" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1202" t="inlineStr">
+      <c r="C33" s="1238" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1203" t="n"/>
-      <c r="E33" s="1203" t="n">
+      <c r="D33" s="1239" t="n"/>
+      <c r="E33" s="1239" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1203" t="n">
+      <c r="F33" s="1239" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1203" t="n">
+      <c r="G33" s="1239" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1203" t="n"/>
-      <c r="I33" s="1204" t="n">
+      <c r="H33" s="1239" t="n"/>
+      <c r="I33" s="1240" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1205" t="n"/>
-      <c r="K33" s="1205" t="n"/>
-      <c r="L33" s="1205" t="n"/>
-      <c r="M33" s="1203" t="n"/>
-      <c r="N33" s="1203" t="n"/>
-      <c r="O33" s="1203" t="n">
+      <c r="J33" s="1241" t="n"/>
+      <c r="K33" s="1241" t="n"/>
+      <c r="L33" s="1241" t="n"/>
+      <c r="M33" s="1239" t="n"/>
+      <c r="N33" s="1239" t="n"/>
+      <c r="O33" s="1239" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1206" t="n">
+      <c r="P33" s="1242" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1203" t="n"/>
-      <c r="R33" s="1203" t="n">
+      <c r="Q33" s="1239" t="n"/>
+      <c r="R33" s="1239" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1203" t="n"/>
+      <c r="S33" s="1239" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1202" t="inlineStr">
+      <c r="U33" s="1238" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -6152,49 +6260,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1207" t="inlineStr">
+      <c r="A34" s="1243" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1208" t="inlineStr">
+      <c r="B34" s="1244" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1208" t="inlineStr">
+      <c r="C34" s="1244" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1209" t="n"/>
-      <c r="E34" s="1209" t="n"/>
-      <c r="F34" s="1209" t="n"/>
-      <c r="G34" s="1209" t="n"/>
-      <c r="H34" s="1209" t="n">
+      <c r="D34" s="1245" t="n"/>
+      <c r="E34" s="1245" t="n"/>
+      <c r="F34" s="1245" t="n"/>
+      <c r="G34" s="1245" t="n"/>
+      <c r="H34" s="1245" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1210" t="n"/>
-      <c r="J34" s="1211" t="n"/>
-      <c r="K34" s="1211" t="n"/>
-      <c r="L34" s="1211" t="n"/>
-      <c r="M34" s="1209" t="n">
+      <c r="I34" s="1246" t="n"/>
+      <c r="J34" s="1247" t="n"/>
+      <c r="K34" s="1247" t="n"/>
+      <c r="L34" s="1247" t="n"/>
+      <c r="M34" s="1245" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1209" t="n">
+      <c r="N34" s="1245" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1209" t="n"/>
-      <c r="P34" s="1212" t="n"/>
-      <c r="Q34" s="1209" t="n"/>
-      <c r="R34" s="1209" t="n"/>
-      <c r="S34" s="1209" t="n"/>
+      <c r="O34" s="1245" t="n"/>
+      <c r="P34" s="1248" t="n"/>
+      <c r="Q34" s="1245" t="n"/>
+      <c r="R34" s="1245" t="n"/>
+      <c r="S34" s="1245" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1208" t="n"/>
+      <c r="U34" s="1244" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -6202,57 +6310,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1213" t="inlineStr">
+      <c r="A35" s="1249" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1214" t="inlineStr">
+      <c r="B35" s="1250" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1214" t="inlineStr">
+      <c r="C35" s="1250" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1215" t="n"/>
-      <c r="E35" s="1215" t="n">
+      <c r="D35" s="1251" t="n"/>
+      <c r="E35" s="1251" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1215" t="n">
+      <c r="F35" s="1251" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1215" t="n">
+      <c r="G35" s="1251" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1215" t="n"/>
-      <c r="I35" s="1216" t="n">
+      <c r="H35" s="1251" t="n"/>
+      <c r="I35" s="1252" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1217" t="n"/>
-      <c r="K35" s="1217" t="n"/>
-      <c r="L35" s="1217" t="n"/>
-      <c r="M35" s="1215" t="n"/>
-      <c r="N35" s="1215" t="n"/>
-      <c r="O35" s="1215" t="n">
+      <c r="J35" s="1253" t="n"/>
+      <c r="K35" s="1253" t="n"/>
+      <c r="L35" s="1253" t="n"/>
+      <c r="M35" s="1251" t="n"/>
+      <c r="N35" s="1251" t="n"/>
+      <c r="O35" s="1251" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1218" t="n">
+      <c r="P35" s="1254" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1215" t="n"/>
-      <c r="R35" s="1215" t="n">
+      <c r="Q35" s="1251" t="n"/>
+      <c r="R35" s="1251" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1215" t="n"/>
+      <c r="S35" s="1251" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1214" t="inlineStr">
+      <c r="U35" s="1250" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -6264,49 +6372,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1219" t="inlineStr">
+      <c r="A36" s="1255" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1220" t="inlineStr">
+      <c r="B36" s="1256" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1220" t="inlineStr">
+      <c r="C36" s="1256" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1221" t="n"/>
-      <c r="E36" s="1221" t="n"/>
-      <c r="F36" s="1221" t="n"/>
-      <c r="G36" s="1221" t="n"/>
-      <c r="H36" s="1221" t="n">
+      <c r="D36" s="1257" t="n"/>
+      <c r="E36" s="1257" t="n"/>
+      <c r="F36" s="1257" t="n"/>
+      <c r="G36" s="1257" t="n"/>
+      <c r="H36" s="1257" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1222" t="n"/>
-      <c r="J36" s="1223" t="n"/>
-      <c r="K36" s="1223" t="n"/>
-      <c r="L36" s="1223" t="n"/>
-      <c r="M36" s="1221" t="n">
+      <c r="I36" s="1258" t="n"/>
+      <c r="J36" s="1259" t="n"/>
+      <c r="K36" s="1259" t="n"/>
+      <c r="L36" s="1259" t="n"/>
+      <c r="M36" s="1257" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1221" t="n">
+      <c r="N36" s="1257" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1221" t="n"/>
-      <c r="P36" s="1224" t="n"/>
-      <c r="Q36" s="1221" t="n"/>
-      <c r="R36" s="1221" t="n"/>
-      <c r="S36" s="1221" t="n"/>
+      <c r="O36" s="1257" t="n"/>
+      <c r="P36" s="1260" t="n"/>
+      <c r="Q36" s="1257" t="n"/>
+      <c r="R36" s="1257" t="n"/>
+      <c r="S36" s="1257" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1220" t="n"/>
+      <c r="U36" s="1256" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -6314,41 +6422,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1225" t="inlineStr">
+      <c r="A37" s="1261" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1226" t="inlineStr">
+      <c r="B37" s="1262" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1226" t="inlineStr">
+      <c r="C37" s="1262" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1227" t="n"/>
-      <c r="E37" s="1227" t="n"/>
-      <c r="F37" s="1227" t="n"/>
-      <c r="G37" s="1227" t="n"/>
-      <c r="H37" s="1227" t="n"/>
-      <c r="I37" s="1228" t="n"/>
-      <c r="J37" s="1229" t="n"/>
-      <c r="K37" s="1229" t="n"/>
-      <c r="L37" s="1229" t="n"/>
-      <c r="M37" s="1227" t="n"/>
-      <c r="N37" s="1227" t="n"/>
-      <c r="O37" s="1227" t="n"/>
-      <c r="P37" s="1230" t="n"/>
-      <c r="Q37" s="1227" t="n">
+      <c r="D37" s="1263" t="n"/>
+      <c r="E37" s="1263" t="n"/>
+      <c r="F37" s="1263" t="n"/>
+      <c r="G37" s="1263" t="n"/>
+      <c r="H37" s="1263" t="n"/>
+      <c r="I37" s="1264" t="n"/>
+      <c r="J37" s="1265" t="n"/>
+      <c r="K37" s="1265" t="n"/>
+      <c r="L37" s="1265" t="n"/>
+      <c r="M37" s="1263" t="n"/>
+      <c r="N37" s="1263" t="n"/>
+      <c r="O37" s="1263" t="n"/>
+      <c r="P37" s="1266" t="n"/>
+      <c r="Q37" s="1263" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1227" t="n"/>
-      <c r="S37" s="1227" t="n"/>
+      <c r="R37" s="1263" t="n"/>
+      <c r="S37" s="1263" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1226" t="n"/>
+      <c r="U37" s="1262" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -6356,57 +6464,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1201" t="inlineStr">
+      <c r="A38" s="1237" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1202" t="inlineStr">
+      <c r="B38" s="1238" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1202" t="inlineStr">
+      <c r="C38" s="1238" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1203" t="n"/>
-      <c r="E38" s="1203" t="n">
+      <c r="D38" s="1239" t="n"/>
+      <c r="E38" s="1239" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1203" t="n">
+      <c r="F38" s="1239" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1203" t="n">
+      <c r="G38" s="1239" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1203" t="n"/>
-      <c r="I38" s="1204" t="n">
+      <c r="H38" s="1239" t="n"/>
+      <c r="I38" s="1240" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1205" t="n"/>
-      <c r="K38" s="1205" t="n"/>
-      <c r="L38" s="1205" t="n"/>
-      <c r="M38" s="1203" t="n"/>
-      <c r="N38" s="1203" t="n"/>
-      <c r="O38" s="1203" t="n">
+      <c r="J38" s="1241" t="n"/>
+      <c r="K38" s="1241" t="n"/>
+      <c r="L38" s="1241" t="n"/>
+      <c r="M38" s="1239" t="n"/>
+      <c r="N38" s="1239" t="n"/>
+      <c r="O38" s="1239" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1206" t="n">
+      <c r="P38" s="1242" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1203" t="n"/>
-      <c r="R38" s="1203" t="n">
+      <c r="Q38" s="1239" t="n"/>
+      <c r="R38" s="1239" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1203" t="n"/>
+      <c r="S38" s="1239" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1202" t="inlineStr">
+      <c r="U38" s="1238" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -6418,49 +6526,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1231" t="inlineStr">
+      <c r="A39" s="1267" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1232" t="inlineStr">
+      <c r="B39" s="1268" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1232" t="inlineStr">
+      <c r="C39" s="1268" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1233" t="n"/>
-      <c r="E39" s="1233" t="n"/>
-      <c r="F39" s="1233" t="n"/>
-      <c r="G39" s="1233" t="n"/>
-      <c r="H39" s="1233" t="n">
+      <c r="D39" s="1269" t="n"/>
+      <c r="E39" s="1269" t="n"/>
+      <c r="F39" s="1269" t="n"/>
+      <c r="G39" s="1269" t="n"/>
+      <c r="H39" s="1269" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1234" t="n"/>
-      <c r="J39" s="1235" t="n"/>
-      <c r="K39" s="1235" t="n"/>
-      <c r="L39" s="1235" t="n"/>
-      <c r="M39" s="1233" t="n">
+      <c r="I39" s="1270" t="n"/>
+      <c r="J39" s="1271" t="n"/>
+      <c r="K39" s="1271" t="n"/>
+      <c r="L39" s="1271" t="n"/>
+      <c r="M39" s="1269" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1233" t="n">
+      <c r="N39" s="1269" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1233" t="n"/>
-      <c r="P39" s="1236" t="n"/>
-      <c r="Q39" s="1233" t="n"/>
-      <c r="R39" s="1233" t="n"/>
-      <c r="S39" s="1233" t="n"/>
+      <c r="O39" s="1269" t="n"/>
+      <c r="P39" s="1272" t="n"/>
+      <c r="Q39" s="1269" t="n"/>
+      <c r="R39" s="1269" t="n"/>
+      <c r="S39" s="1269" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1232" t="n"/>
+      <c r="U39" s="1268" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -6468,41 +6576,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1207" t="inlineStr">
+      <c r="A40" s="1243" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1208" t="inlineStr">
+      <c r="B40" s="1244" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1208" t="inlineStr">
+      <c r="C40" s="1244" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1209" t="n"/>
-      <c r="E40" s="1209" t="n"/>
-      <c r="F40" s="1209" t="n"/>
-      <c r="G40" s="1209" t="n"/>
-      <c r="H40" s="1209" t="n"/>
-      <c r="I40" s="1210" t="n"/>
-      <c r="J40" s="1211" t="n"/>
-      <c r="K40" s="1211" t="n"/>
-      <c r="L40" s="1211" t="n"/>
-      <c r="M40" s="1209" t="n"/>
-      <c r="N40" s="1209" t="n"/>
-      <c r="O40" s="1209" t="n"/>
-      <c r="P40" s="1212" t="n"/>
-      <c r="Q40" s="1209" t="n">
+      <c r="D40" s="1245" t="n"/>
+      <c r="E40" s="1245" t="n"/>
+      <c r="F40" s="1245" t="n"/>
+      <c r="G40" s="1245" t="n"/>
+      <c r="H40" s="1245" t="n"/>
+      <c r="I40" s="1246" t="n"/>
+      <c r="J40" s="1247" t="n"/>
+      <c r="K40" s="1247" t="n"/>
+      <c r="L40" s="1247" t="n"/>
+      <c r="M40" s="1245" t="n"/>
+      <c r="N40" s="1245" t="n"/>
+      <c r="O40" s="1245" t="n"/>
+      <c r="P40" s="1248" t="n"/>
+      <c r="Q40" s="1245" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1209" t="n"/>
-      <c r="S40" s="1209" t="n"/>
+      <c r="R40" s="1245" t="n"/>
+      <c r="S40" s="1245" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1208" t="n"/>
+      <c r="U40" s="1244" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -6510,57 +6618,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1213" t="inlineStr">
+      <c r="A41" s="1249" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1214" t="inlineStr">
+      <c r="B41" s="1250" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1214" t="inlineStr">
+      <c r="C41" s="1250" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1215" t="n"/>
-      <c r="E41" s="1215" t="n">
+      <c r="D41" s="1251" t="n"/>
+      <c r="E41" s="1251" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1215" t="n">
+      <c r="F41" s="1251" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1215" t="n">
+      <c r="G41" s="1251" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1215" t="n"/>
-      <c r="I41" s="1216" t="n">
+      <c r="H41" s="1251" t="n"/>
+      <c r="I41" s="1252" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1217" t="n"/>
-      <c r="K41" s="1217" t="n"/>
-      <c r="L41" s="1217" t="n"/>
-      <c r="M41" s="1215" t="n"/>
-      <c r="N41" s="1215" t="n"/>
-      <c r="O41" s="1215" t="n">
+      <c r="J41" s="1253" t="n"/>
+      <c r="K41" s="1253" t="n"/>
+      <c r="L41" s="1253" t="n"/>
+      <c r="M41" s="1251" t="n"/>
+      <c r="N41" s="1251" t="n"/>
+      <c r="O41" s="1251" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1218" t="n">
+      <c r="P41" s="1254" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1215" t="n"/>
-      <c r="R41" s="1215" t="n">
+      <c r="Q41" s="1251" t="n"/>
+      <c r="R41" s="1251" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1215" t="n"/>
+      <c r="S41" s="1251" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1214" t="inlineStr">
+      <c r="U41" s="1250" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -6572,49 +6680,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1225" t="inlineStr">
+      <c r="A42" s="1261" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1226" t="inlineStr">
+      <c r="B42" s="1262" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1226" t="inlineStr">
+      <c r="C42" s="1262" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1227" t="n"/>
-      <c r="E42" s="1227" t="n"/>
-      <c r="F42" s="1227" t="n"/>
-      <c r="G42" s="1227" t="n"/>
-      <c r="H42" s="1227" t="n">
+      <c r="D42" s="1263" t="n"/>
+      <c r="E42" s="1263" t="n"/>
+      <c r="F42" s="1263" t="n"/>
+      <c r="G42" s="1263" t="n"/>
+      <c r="H42" s="1263" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1228" t="n"/>
-      <c r="J42" s="1229" t="n"/>
-      <c r="K42" s="1229" t="n"/>
-      <c r="L42" s="1229" t="n"/>
-      <c r="M42" s="1227" t="n">
+      <c r="I42" s="1264" t="n"/>
+      <c r="J42" s="1265" t="n"/>
+      <c r="K42" s="1265" t="n"/>
+      <c r="L42" s="1265" t="n"/>
+      <c r="M42" s="1263" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1227" t="n">
+      <c r="N42" s="1263" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1227" t="n"/>
-      <c r="P42" s="1230" t="n"/>
-      <c r="Q42" s="1227" t="n"/>
-      <c r="R42" s="1227" t="n"/>
-      <c r="S42" s="1227" t="n"/>
+      <c r="O42" s="1263" t="n"/>
+      <c r="P42" s="1266" t="n"/>
+      <c r="Q42" s="1263" t="n"/>
+      <c r="R42" s="1263" t="n"/>
+      <c r="S42" s="1263" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1226" t="n"/>
+      <c r="U42" s="1262" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -6622,57 +6730,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1201" t="inlineStr">
+      <c r="A43" s="1237" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1202" t="inlineStr">
+      <c r="B43" s="1238" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1202" t="inlineStr">
+      <c r="C43" s="1238" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1203" t="n"/>
-      <c r="E43" s="1203" t="n">
+      <c r="D43" s="1239" t="n"/>
+      <c r="E43" s="1239" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1203" t="n">
+      <c r="F43" s="1239" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1203" t="n">
+      <c r="G43" s="1239" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1203" t="n"/>
-      <c r="I43" s="1204" t="n">
+      <c r="H43" s="1239" t="n"/>
+      <c r="I43" s="1240" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1205" t="n"/>
-      <c r="K43" s="1205" t="n"/>
-      <c r="L43" s="1205" t="n"/>
-      <c r="M43" s="1203" t="n"/>
-      <c r="N43" s="1203" t="n"/>
-      <c r="O43" s="1203" t="n">
+      <c r="J43" s="1241" t="n"/>
+      <c r="K43" s="1241" t="n"/>
+      <c r="L43" s="1241" t="n"/>
+      <c r="M43" s="1239" t="n"/>
+      <c r="N43" s="1239" t="n"/>
+      <c r="O43" s="1239" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1206" t="n">
+      <c r="P43" s="1242" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1203" t="n"/>
-      <c r="R43" s="1203" t="n">
+      <c r="Q43" s="1239" t="n"/>
+      <c r="R43" s="1239" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1203" t="n"/>
+      <c r="S43" s="1239" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1202" t="n"/>
+      <c r="U43" s="1238" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -6680,45 +6788,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1231" t="inlineStr">
+      <c r="A44" s="1267" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1232" t="inlineStr">
+      <c r="B44" s="1268" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1232" t="inlineStr">
+      <c r="C44" s="1268" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1233" t="n"/>
-      <c r="E44" s="1233" t="n">
+      <c r="D44" s="1269" t="n"/>
+      <c r="E44" s="1269" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1233" t="n">
+      <c r="F44" s="1269" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1233" t="n"/>
-      <c r="H44" s="1233" t="n"/>
-      <c r="I44" s="1234" t="n"/>
-      <c r="J44" s="1235" t="n"/>
-      <c r="K44" s="1235" t="n"/>
-      <c r="L44" s="1235" t="n"/>
-      <c r="M44" s="1233" t="n"/>
-      <c r="N44" s="1233" t="n"/>
-      <c r="O44" s="1233" t="n"/>
-      <c r="P44" s="1236" t="n"/>
-      <c r="Q44" s="1233" t="n"/>
-      <c r="R44" s="1233" t="n"/>
-      <c r="S44" s="1233" t="n">
+      <c r="G44" s="1269" t="n"/>
+      <c r="H44" s="1269" t="n"/>
+      <c r="I44" s="1270" t="n"/>
+      <c r="J44" s="1271" t="n"/>
+      <c r="K44" s="1271" t="n"/>
+      <c r="L44" s="1271" t="n"/>
+      <c r="M44" s="1269" t="n"/>
+      <c r="N44" s="1269" t="n"/>
+      <c r="O44" s="1269" t="n"/>
+      <c r="P44" s="1272" t="n"/>
+      <c r="Q44" s="1269" t="n"/>
+      <c r="R44" s="1269" t="n"/>
+      <c r="S44" s="1269" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1232" t="inlineStr">
+      <c r="U44" s="1268" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -6730,164 +6838,204 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1207" t="inlineStr">
+      <c r="A45" s="1267" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1208" t="inlineStr">
+      <c r="B45" s="1268" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1208" t="inlineStr">
+      <c r="C45" s="1268" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1209" t="n"/>
-      <c r="E45" s="1209" t="n"/>
-      <c r="F45" s="1209" t="n"/>
-      <c r="G45" s="1209" t="n"/>
-      <c r="H45" s="1209" t="n">
+      <c r="D45" s="1269" t="n"/>
+      <c r="E45" s="1269" t="n"/>
+      <c r="F45" s="1269" t="n"/>
+      <c r="G45" s="1269" t="n"/>
+      <c r="H45" s="1269" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1210" t="n"/>
-      <c r="J45" s="1211" t="n"/>
-      <c r="K45" s="1211" t="n"/>
-      <c r="L45" s="1211" t="n"/>
-      <c r="M45" s="1209" t="n">
+      <c r="I45" s="1270" t="n"/>
+      <c r="J45" s="1271" t="n"/>
+      <c r="K45" s="1271" t="n"/>
+      <c r="L45" s="1271" t="n"/>
+      <c r="M45" s="1269" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1209" t="n">
+      <c r="N45" s="1269" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1209" t="n"/>
-      <c r="P45" s="1212" t="n"/>
-      <c r="Q45" s="1209" t="n"/>
-      <c r="R45" s="1209" t="n"/>
-      <c r="S45" s="1209" t="n"/>
-      <c r="T45" s="631" t="inlineStr">
+      <c r="O45" s="1269" t="n"/>
+      <c r="P45" s="1272" t="n"/>
+      <c r="Q45" s="1269" t="n"/>
+      <c r="R45" s="1269" t="n"/>
+      <c r="S45" s="1269" t="n"/>
+      <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1208" t="n"/>
-      <c r="V45" s="632" t="inlineStr">
+      <c r="U45" s="1268" t="n"/>
+      <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1213" t="inlineStr">
+      <c r="A46" s="1243" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B46" s="1244" t="inlineStr">
+        <is>
+          <t>night</t>
+        </is>
+      </c>
+      <c r="C46" s="1244" t="inlineStr">
+        <is>
+          <t>EVENT - Clean</t>
+        </is>
+      </c>
+      <c r="D46" s="1245" t="n"/>
+      <c r="E46" s="1245" t="n"/>
+      <c r="F46" s="1245" t="n"/>
+      <c r="G46" s="1245" t="n"/>
+      <c r="H46" s="1245" t="n"/>
+      <c r="I46" s="1246" t="n"/>
+      <c r="J46" s="1247" t="n"/>
+      <c r="K46" s="1247" t="n"/>
+      <c r="L46" s="1247" t="n"/>
+      <c r="M46" s="1245" t="n"/>
+      <c r="N46" s="1245" t="n"/>
+      <c r="O46" s="1245" t="n"/>
+      <c r="P46" s="1248" t="n"/>
+      <c r="Q46" s="1245" t="n"/>
+      <c r="R46" s="1245" t="n"/>
+      <c r="S46" s="1245" t="n"/>
+      <c r="T46" s="631" t="n"/>
+      <c r="U46" s="1244" t="n"/>
+      <c r="V46" s="632" t="inlineStr">
+        <is>
+          <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="1249" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B46" s="1214" t="inlineStr">
+      <c r="B47" s="1250" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C46" s="1214" t="inlineStr">
+      <c r="C47" s="1250" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D46" s="1215" t="n"/>
-      <c r="E46" s="1215" t="n">
+      <c r="D47" s="1251" t="n"/>
+      <c r="E47" s="1251" t="n">
         <v>16.6</v>
       </c>
-      <c r="F46" s="1215" t="n">
+      <c r="F47" s="1251" t="n">
         <v>0.6</v>
       </c>
-      <c r="G46" s="1215" t="n">
+      <c r="G47" s="1251" t="n">
         <v>4.1</v>
       </c>
-      <c r="H46" s="1215" t="n"/>
-      <c r="I46" s="1216" t="n">
+      <c r="H47" s="1251" t="n"/>
+      <c r="I47" s="1252" t="n">
         <v>0.9</v>
       </c>
-      <c r="J46" s="1217" t="n"/>
-      <c r="K46" s="1217" t="n"/>
-      <c r="L46" s="1217" t="n"/>
-      <c r="M46" s="1215" t="n"/>
-      <c r="N46" s="1215" t="n"/>
-      <c r="O46" s="1215" t="n">
+      <c r="J47" s="1253" t="n"/>
+      <c r="K47" s="1253" t="n"/>
+      <c r="L47" s="1253" t="n"/>
+      <c r="M47" s="1251" t="n"/>
+      <c r="N47" s="1251" t="n"/>
+      <c r="O47" s="1251" t="n">
         <v>13.2</v>
       </c>
-      <c r="P46" s="1218" t="n">
+      <c r="P47" s="1254" t="n">
         <v>0</v>
       </c>
-      <c r="Q46" s="1215" t="n"/>
-      <c r="R46" s="1215" t="n">
+      <c r="Q47" s="1251" t="n"/>
+      <c r="R47" s="1251" t="n">
         <v>84.5</v>
       </c>
-      <c r="S46" s="1215" t="n">
+      <c r="S47" s="1251" t="n">
         <v>11.8</v>
       </c>
-      <c r="T46" s="813" t="inlineStr">
+      <c r="T47" s="813" t="inlineStr">
         <is>
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U46" s="1214" t="inlineStr">
+      <c r="U47" s="1250" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
       </c>
-      <c r="V46" s="814" t="inlineStr">
+      <c r="V47" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 16.6, CC 0.6. (John wrote 'CC=16.6' but that's FC; a 16.6 combined chlorine is implausible -- logged as FC.) FC loss 4.1 ppm/24h = 17.2 (7/2 NOON) + 1.0gal x3.5 - 16.6, computed noon-to-noon; NOT the 2.3 daily_calc.py reported (it used the 7/2 evening recheck 15.4 as baseline -&gt; ~16.5h window, non-comparable). WATCH: CC creeping 0.0 -&gt; 0.4 -&gt; 0.6 over ~24h; still a trace, and higher FC should oxidize it away, but note the direction -- flag if it climbs past ~1.0. Pred error +0.9 (actual 16.6 vs 7/2 dose's 15.7 projection): model over-predicted loss again but by less than 7/2's +2.1 -- two straight hot/sunny days where real loss ran under the L24=5.0 estimate; watch a 3rd before nudging dose.py's l24_hot_sunny down. Water level 11.8 cm (was 11.9 on 7/2; -0.1 within ruler/reading noise, ruler adhesion still iffy). Hot day: high 94F, water 84.5F, ~13 sun hrs.</t>
         </is>
       </c>
     </row>
-    <row r="47">
-      <c r="A47" s="1225" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="1261" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1226" t="inlineStr">
+      <c r="B48" s="1262" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C47" s="1226" t="inlineStr">
+      <c r="C48" s="1262" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D47" s="1227" t="n"/>
-      <c r="E47" s="1227" t="n"/>
-      <c r="F47" s="1227" t="n"/>
-      <c r="G47" s="1227" t="n"/>
-      <c r="H47" s="1227" t="n">
+      <c r="D48" s="1263" t="n"/>
+      <c r="E48" s="1263" t="n"/>
+      <c r="F48" s="1263" t="n"/>
+      <c r="G48" s="1263" t="n"/>
+      <c r="H48" s="1263" t="n">
         <v>15.1</v>
       </c>
-      <c r="I47" s="1228" t="n"/>
-      <c r="J47" s="1229" t="n"/>
-      <c r="K47" s="1229" t="n"/>
-      <c r="L47" s="1229" t="n"/>
-      <c r="M47" s="1227" t="n">
+      <c r="I48" s="1264" t="n"/>
+      <c r="J48" s="1265" t="n"/>
+      <c r="K48" s="1265" t="n"/>
+      <c r="L48" s="1265" t="n"/>
+      <c r="M48" s="1263" t="n">
         <v>1</v>
       </c>
-      <c r="N47" s="1227" t="n">
+      <c r="N48" s="1263" t="n">
         <v>20</v>
       </c>
-      <c r="O47" s="1227" t="n"/>
-      <c r="P47" s="1230" t="n"/>
-      <c r="Q47" s="1227" t="n"/>
-      <c r="R47" s="1227" t="n"/>
-      <c r="S47" s="1227" t="n"/>
-      <c r="T47" s="827" t="inlineStr">
+      <c r="O48" s="1263" t="n"/>
+      <c r="P48" s="1266" t="n"/>
+      <c r="Q48" s="1263" t="n"/>
+      <c r="R48" s="1263" t="n"/>
+      <c r="S48" s="1263" t="n"/>
+      <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1226" t="n"/>
-      <c r="V47" s="828" t="inlineStr">
+      <c r="U48" s="1262" t="n"/>
+      <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
         </is>

</xml_diff>

<commit_message>
Log 2026-07-04 noon (FC 16.8, CC 0.2); retune hot-sunny loss constant 5.0->4.0
Third straight hot-day over-prediction (+1.7) confirms the L24 model
over-estimates loss on hot/sunny days -- actual losses ~2.9/4.1/3.3 vs
modeled 5.0. Lowered l24_hot_sunny to 4.0. Also: CC creep fully cleared
(0.6->0.2, confirms the benign debris+Magic-Eraser explanation), water
level slow-evaporation trend (11.9->11.8->11.65). Party prep: recommending
just 0.5 gal tonight so FC doesn't overshoot into the high teens.
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1273">
+  <cellXfs count="1315">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -4346,6 +4346,132 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4607,7 +4733,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V48"/>
+  <dimension ref="A1:V49"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -4784,35 +4910,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1237" t="inlineStr">
+      <c r="A3" s="1273" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1238" t="n"/>
-      <c r="C3" s="1238" t="inlineStr">
+      <c r="B3" s="1274" t="n"/>
+      <c r="C3" s="1274" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1239" t="n"/>
-      <c r="E3" s="1239" t="n"/>
-      <c r="F3" s="1239" t="n"/>
-      <c r="G3" s="1239" t="n"/>
-      <c r="H3" s="1239" t="n"/>
-      <c r="I3" s="1240" t="n"/>
-      <c r="J3" s="1241" t="n"/>
-      <c r="K3" s="1241" t="n"/>
-      <c r="L3" s="1241" t="n"/>
-      <c r="M3" s="1239" t="n"/>
-      <c r="N3" s="1239" t="n"/>
-      <c r="O3" s="1239" t="n"/>
-      <c r="P3" s="1242" t="n"/>
-      <c r="Q3" s="1239" t="n"/>
-      <c r="R3" s="1239" t="n"/>
-      <c r="S3" s="1239" t="n"/>
+      <c r="D3" s="1275" t="n"/>
+      <c r="E3" s="1275" t="n"/>
+      <c r="F3" s="1275" t="n"/>
+      <c r="G3" s="1275" t="n"/>
+      <c r="H3" s="1275" t="n"/>
+      <c r="I3" s="1276" t="n"/>
+      <c r="J3" s="1277" t="n"/>
+      <c r="K3" s="1277" t="n"/>
+      <c r="L3" s="1277" t="n"/>
+      <c r="M3" s="1275" t="n"/>
+      <c r="N3" s="1275" t="n"/>
+      <c r="O3" s="1275" t="n"/>
+      <c r="P3" s="1278" t="n"/>
+      <c r="Q3" s="1275" t="n"/>
+      <c r="R3" s="1275" t="n"/>
+      <c r="S3" s="1275" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1238" t="n"/>
+      <c r="U3" s="1274" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -4820,43 +4946,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1243" t="inlineStr">
+      <c r="A4" s="1279" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1244" t="inlineStr">
+      <c r="B4" s="1280" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1244" t="inlineStr">
+      <c r="C4" s="1280" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1245" t="n"/>
-      <c r="E4" s="1245" t="n"/>
-      <c r="F4" s="1245" t="n"/>
-      <c r="G4" s="1245" t="n"/>
-      <c r="H4" s="1245" t="n"/>
-      <c r="I4" s="1246" t="n"/>
-      <c r="J4" s="1247" t="n"/>
-      <c r="K4" s="1247" t="n"/>
-      <c r="L4" s="1247" t="n"/>
-      <c r="M4" s="1245" t="n">
+      <c r="D4" s="1281" t="n"/>
+      <c r="E4" s="1281" t="n"/>
+      <c r="F4" s="1281" t="n"/>
+      <c r="G4" s="1281" t="n"/>
+      <c r="H4" s="1281" t="n"/>
+      <c r="I4" s="1282" t="n"/>
+      <c r="J4" s="1283" t="n"/>
+      <c r="K4" s="1283" t="n"/>
+      <c r="L4" s="1283" t="n"/>
+      <c r="M4" s="1281" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1245" t="n">
+      <c r="N4" s="1281" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1245" t="n"/>
-      <c r="P4" s="1248" t="n"/>
-      <c r="Q4" s="1245" t="n"/>
-      <c r="R4" s="1245" t="n"/>
-      <c r="S4" s="1245" t="n"/>
+      <c r="O4" s="1281" t="n"/>
+      <c r="P4" s="1284" t="n"/>
+      <c r="Q4" s="1281" t="n"/>
+      <c r="R4" s="1281" t="n"/>
+      <c r="S4" s="1281" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1244" t="n"/>
+      <c r="U4" s="1280" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -4864,57 +4990,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1249" t="inlineStr">
+      <c r="A5" s="1285" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1250" t="inlineStr">
+      <c r="B5" s="1286" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1250" t="inlineStr">
+      <c r="C5" s="1286" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1251" t="n">
+      <c r="D5" s="1287" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1251" t="n">
+      <c r="E5" s="1287" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1251" t="n">
+      <c r="F5" s="1287" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1251" t="n"/>
-      <c r="H5" s="1251" t="n"/>
-      <c r="I5" s="1252" t="n"/>
-      <c r="J5" s="1253" t="n">
+      <c r="G5" s="1287" t="n"/>
+      <c r="H5" s="1287" t="n"/>
+      <c r="I5" s="1288" t="n"/>
+      <c r="J5" s="1289" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1253" t="n">
+      <c r="K5" s="1289" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1253" t="inlineStr">
+      <c r="L5" s="1289" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1251" t="n"/>
-      <c r="N5" s="1251" t="n"/>
-      <c r="O5" s="1251" t="n">
+      <c r="M5" s="1287" t="n"/>
+      <c r="N5" s="1287" t="n"/>
+      <c r="O5" s="1287" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1254" t="n">
+      <c r="P5" s="1290" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1251" t="n"/>
-      <c r="R5" s="1251" t="n"/>
-      <c r="S5" s="1251" t="n"/>
+      <c r="Q5" s="1287" t="n"/>
+      <c r="R5" s="1287" t="n"/>
+      <c r="S5" s="1287" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1250" t="n"/>
+      <c r="U5" s="1286" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -4922,43 +5048,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1255" t="inlineStr">
+      <c r="A6" s="1291" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1256" t="inlineStr">
+      <c r="B6" s="1292" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1256" t="inlineStr">
+      <c r="C6" s="1292" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1257" t="n"/>
-      <c r="E6" s="1257" t="n"/>
-      <c r="F6" s="1257" t="n"/>
-      <c r="G6" s="1257" t="n"/>
-      <c r="H6" s="1257" t="n"/>
-      <c r="I6" s="1258" t="n"/>
-      <c r="J6" s="1259" t="n"/>
-      <c r="K6" s="1259" t="n"/>
-      <c r="L6" s="1259" t="n"/>
-      <c r="M6" s="1257" t="n">
+      <c r="D6" s="1293" t="n"/>
+      <c r="E6" s="1293" t="n"/>
+      <c r="F6" s="1293" t="n"/>
+      <c r="G6" s="1293" t="n"/>
+      <c r="H6" s="1293" t="n"/>
+      <c r="I6" s="1294" t="n"/>
+      <c r="J6" s="1295" t="n"/>
+      <c r="K6" s="1295" t="n"/>
+      <c r="L6" s="1295" t="n"/>
+      <c r="M6" s="1293" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1257" t="n">
+      <c r="N6" s="1293" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1257" t="n"/>
-      <c r="P6" s="1260" t="n"/>
-      <c r="Q6" s="1257" t="n"/>
-      <c r="R6" s="1257" t="n"/>
-      <c r="S6" s="1257" t="n"/>
+      <c r="O6" s="1293" t="n"/>
+      <c r="P6" s="1296" t="n"/>
+      <c r="Q6" s="1293" t="n"/>
+      <c r="R6" s="1293" t="n"/>
+      <c r="S6" s="1293" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1256" t="n"/>
+      <c r="U6" s="1292" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -4966,39 +5092,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1261" t="inlineStr">
+      <c r="A7" s="1297" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1262" t="inlineStr">
+      <c r="B7" s="1298" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1262" t="inlineStr">
+      <c r="C7" s="1298" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1263" t="n"/>
-      <c r="E7" s="1263" t="n"/>
-      <c r="F7" s="1263" t="n"/>
-      <c r="G7" s="1263" t="n"/>
-      <c r="H7" s="1263" t="n"/>
-      <c r="I7" s="1264" t="n"/>
-      <c r="J7" s="1265" t="n"/>
-      <c r="K7" s="1265" t="n"/>
-      <c r="L7" s="1265" t="n"/>
-      <c r="M7" s="1263" t="n"/>
-      <c r="N7" s="1263" t="n"/>
-      <c r="O7" s="1263" t="n"/>
-      <c r="P7" s="1266" t="n"/>
-      <c r="Q7" s="1263" t="n"/>
-      <c r="R7" s="1263" t="n"/>
-      <c r="S7" s="1263" t="n"/>
+      <c r="D7" s="1299" t="n"/>
+      <c r="E7" s="1299" t="n"/>
+      <c r="F7" s="1299" t="n"/>
+      <c r="G7" s="1299" t="n"/>
+      <c r="H7" s="1299" t="n"/>
+      <c r="I7" s="1300" t="n"/>
+      <c r="J7" s="1301" t="n"/>
+      <c r="K7" s="1301" t="n"/>
+      <c r="L7" s="1301" t="n"/>
+      <c r="M7" s="1299" t="n"/>
+      <c r="N7" s="1299" t="n"/>
+      <c r="O7" s="1299" t="n"/>
+      <c r="P7" s="1302" t="n"/>
+      <c r="Q7" s="1299" t="n"/>
+      <c r="R7" s="1299" t="n"/>
+      <c r="S7" s="1299" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1262" t="n"/>
+      <c r="U7" s="1298" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5006,39 +5132,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1237" t="inlineStr">
+      <c r="A8" s="1273" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1238" t="inlineStr">
+      <c r="B8" s="1274" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1238" t="inlineStr">
+      <c r="C8" s="1274" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1239" t="n"/>
-      <c r="E8" s="1239" t="n"/>
-      <c r="F8" s="1239" t="n"/>
-      <c r="G8" s="1239" t="n"/>
-      <c r="H8" s="1239" t="n"/>
-      <c r="I8" s="1240" t="n"/>
-      <c r="J8" s="1241" t="n"/>
-      <c r="K8" s="1241" t="n"/>
-      <c r="L8" s="1241" t="n"/>
-      <c r="M8" s="1239" t="n"/>
-      <c r="N8" s="1239" t="n"/>
-      <c r="O8" s="1239" t="n"/>
-      <c r="P8" s="1242" t="n"/>
-      <c r="Q8" s="1239" t="n"/>
-      <c r="R8" s="1239" t="n"/>
-      <c r="S8" s="1239" t="n"/>
+      <c r="D8" s="1275" t="n"/>
+      <c r="E8" s="1275" t="n"/>
+      <c r="F8" s="1275" t="n"/>
+      <c r="G8" s="1275" t="n"/>
+      <c r="H8" s="1275" t="n"/>
+      <c r="I8" s="1276" t="n"/>
+      <c r="J8" s="1277" t="n"/>
+      <c r="K8" s="1277" t="n"/>
+      <c r="L8" s="1277" t="n"/>
+      <c r="M8" s="1275" t="n"/>
+      <c r="N8" s="1275" t="n"/>
+      <c r="O8" s="1275" t="n"/>
+      <c r="P8" s="1278" t="n"/>
+      <c r="Q8" s="1275" t="n"/>
+      <c r="R8" s="1275" t="n"/>
+      <c r="S8" s="1275" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1238" t="n"/>
+      <c r="U8" s="1274" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -5046,63 +5172,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1267" t="inlineStr">
+      <c r="A9" s="1303" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1268" t="inlineStr">
+      <c r="B9" s="1304" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1268" t="inlineStr">
+      <c r="C9" s="1304" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1269" t="n">
+      <c r="D9" s="1305" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1269" t="n">
+      <c r="E9" s="1305" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1269" t="n">
+      <c r="F9" s="1305" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1269" t="n">
+      <c r="G9" s="1305" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1269" t="n"/>
-      <c r="I9" s="1270" t="n"/>
-      <c r="J9" s="1271" t="n">
+      <c r="H9" s="1305" t="n"/>
+      <c r="I9" s="1306" t="n"/>
+      <c r="J9" s="1307" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1271" t="n">
+      <c r="K9" s="1307" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1271" t="inlineStr">
+      <c r="L9" s="1307" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1269" t="n"/>
-      <c r="N9" s="1269" t="n"/>
-      <c r="O9" s="1269" t="n">
+      <c r="M9" s="1305" t="n"/>
+      <c r="N9" s="1305" t="n"/>
+      <c r="O9" s="1305" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1272" t="n">
+      <c r="P9" s="1308" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1269" t="n"/>
-      <c r="R9" s="1269" t="n"/>
-      <c r="S9" s="1269" t="n"/>
+      <c r="Q9" s="1305" t="n"/>
+      <c r="R9" s="1305" t="n"/>
+      <c r="S9" s="1305" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1268" t="n"/>
+      <c r="U9" s="1304" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -5110,43 +5236,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1267" t="inlineStr">
+      <c r="A10" s="1303" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1268" t="inlineStr">
+      <c r="B10" s="1304" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1268" t="inlineStr">
+      <c r="C10" s="1304" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1269" t="n"/>
-      <c r="E10" s="1269" t="n"/>
-      <c r="F10" s="1269" t="n"/>
-      <c r="G10" s="1269" t="n"/>
-      <c r="H10" s="1269" t="n"/>
-      <c r="I10" s="1270" t="n"/>
-      <c r="J10" s="1271" t="n"/>
-      <c r="K10" s="1271" t="n"/>
-      <c r="L10" s="1271" t="inlineStr">
+      <c r="D10" s="1305" t="n"/>
+      <c r="E10" s="1305" t="n"/>
+      <c r="F10" s="1305" t="n"/>
+      <c r="G10" s="1305" t="n"/>
+      <c r="H10" s="1305" t="n"/>
+      <c r="I10" s="1306" t="n"/>
+      <c r="J10" s="1307" t="n"/>
+      <c r="K10" s="1307" t="n"/>
+      <c r="L10" s="1307" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1269" t="n"/>
-      <c r="N10" s="1269" t="n"/>
-      <c r="O10" s="1269" t="n"/>
-      <c r="P10" s="1272" t="n"/>
-      <c r="Q10" s="1269" t="n"/>
-      <c r="R10" s="1269" t="n"/>
-      <c r="S10" s="1269" t="n"/>
+      <c r="M10" s="1305" t="n"/>
+      <c r="N10" s="1305" t="n"/>
+      <c r="O10" s="1305" t="n"/>
+      <c r="P10" s="1308" t="n"/>
+      <c r="Q10" s="1305" t="n"/>
+      <c r="R10" s="1305" t="n"/>
+      <c r="S10" s="1305" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1268" t="n"/>
+      <c r="U10" s="1304" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -5154,43 +5280,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1267" t="inlineStr">
+      <c r="A11" s="1303" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1268" t="inlineStr">
+      <c r="B11" s="1304" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1268" t="inlineStr">
+      <c r="C11" s="1304" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1269" t="n"/>
-      <c r="E11" s="1269" t="n"/>
-      <c r="F11" s="1269" t="n"/>
-      <c r="G11" s="1269" t="n"/>
-      <c r="H11" s="1269" t="n"/>
-      <c r="I11" s="1270" t="n"/>
-      <c r="J11" s="1271" t="n"/>
-      <c r="K11" s="1271" t="n"/>
-      <c r="L11" s="1271" t="n"/>
-      <c r="M11" s="1269" t="n">
+      <c r="D11" s="1305" t="n"/>
+      <c r="E11" s="1305" t="n"/>
+      <c r="F11" s="1305" t="n"/>
+      <c r="G11" s="1305" t="n"/>
+      <c r="H11" s="1305" t="n"/>
+      <c r="I11" s="1306" t="n"/>
+      <c r="J11" s="1307" t="n"/>
+      <c r="K11" s="1307" t="n"/>
+      <c r="L11" s="1307" t="n"/>
+      <c r="M11" s="1305" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1269" t="n">
+      <c r="N11" s="1305" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1269" t="n"/>
-      <c r="P11" s="1272" t="n"/>
-      <c r="Q11" s="1269" t="n"/>
-      <c r="R11" s="1269" t="n"/>
-      <c r="S11" s="1269" t="n"/>
+      <c r="O11" s="1305" t="n"/>
+      <c r="P11" s="1308" t="n"/>
+      <c r="Q11" s="1305" t="n"/>
+      <c r="R11" s="1305" t="n"/>
+      <c r="S11" s="1305" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1268" t="n"/>
+      <c r="U11" s="1304" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -5198,39 +5324,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1243" t="inlineStr">
+      <c r="A12" s="1279" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1244" t="inlineStr">
+      <c r="B12" s="1280" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1244" t="inlineStr">
+      <c r="C12" s="1280" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1245" t="n"/>
-      <c r="E12" s="1245" t="n"/>
-      <c r="F12" s="1245" t="n"/>
-      <c r="G12" s="1245" t="n"/>
-      <c r="H12" s="1245" t="n"/>
-      <c r="I12" s="1246" t="n"/>
-      <c r="J12" s="1247" t="n"/>
-      <c r="K12" s="1247" t="n"/>
-      <c r="L12" s="1247" t="n"/>
-      <c r="M12" s="1245" t="n"/>
-      <c r="N12" s="1245" t="n"/>
-      <c r="O12" s="1245" t="n"/>
-      <c r="P12" s="1248" t="n"/>
-      <c r="Q12" s="1245" t="n"/>
-      <c r="R12" s="1245" t="n"/>
-      <c r="S12" s="1245" t="n"/>
+      <c r="D12" s="1281" t="n"/>
+      <c r="E12" s="1281" t="n"/>
+      <c r="F12" s="1281" t="n"/>
+      <c r="G12" s="1281" t="n"/>
+      <c r="H12" s="1281" t="n"/>
+      <c r="I12" s="1282" t="n"/>
+      <c r="J12" s="1283" t="n"/>
+      <c r="K12" s="1283" t="n"/>
+      <c r="L12" s="1283" t="n"/>
+      <c r="M12" s="1281" t="n"/>
+      <c r="N12" s="1281" t="n"/>
+      <c r="O12" s="1281" t="n"/>
+      <c r="P12" s="1284" t="n"/>
+      <c r="Q12" s="1281" t="n"/>
+      <c r="R12" s="1281" t="n"/>
+      <c r="S12" s="1281" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1244" t="n"/>
+      <c r="U12" s="1280" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5238,35 +5364,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1249" t="inlineStr">
+      <c r="A13" s="1285" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1250" t="n"/>
-      <c r="C13" s="1250" t="inlineStr">
+      <c r="B13" s="1286" t="n"/>
+      <c r="C13" s="1286" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1251" t="n"/>
-      <c r="E13" s="1251" t="n"/>
-      <c r="F13" s="1251" t="n"/>
-      <c r="G13" s="1251" t="n"/>
-      <c r="H13" s="1251" t="n"/>
-      <c r="I13" s="1252" t="n"/>
-      <c r="J13" s="1253" t="n"/>
-      <c r="K13" s="1253" t="n"/>
-      <c r="L13" s="1253" t="n"/>
-      <c r="M13" s="1251" t="n"/>
-      <c r="N13" s="1251" t="n"/>
-      <c r="O13" s="1251" t="n"/>
-      <c r="P13" s="1254" t="n"/>
-      <c r="Q13" s="1251" t="n"/>
-      <c r="R13" s="1251" t="n"/>
-      <c r="S13" s="1251" t="n"/>
+      <c r="D13" s="1287" t="n"/>
+      <c r="E13" s="1287" t="n"/>
+      <c r="F13" s="1287" t="n"/>
+      <c r="G13" s="1287" t="n"/>
+      <c r="H13" s="1287" t="n"/>
+      <c r="I13" s="1288" t="n"/>
+      <c r="J13" s="1289" t="n"/>
+      <c r="K13" s="1289" t="n"/>
+      <c r="L13" s="1289" t="n"/>
+      <c r="M13" s="1287" t="n"/>
+      <c r="N13" s="1287" t="n"/>
+      <c r="O13" s="1287" t="n"/>
+      <c r="P13" s="1290" t="n"/>
+      <c r="Q13" s="1287" t="n"/>
+      <c r="R13" s="1287" t="n"/>
+      <c r="S13" s="1287" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1250" t="n"/>
+      <c r="U13" s="1286" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -5274,53 +5400,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1255" t="inlineStr">
+      <c r="A14" s="1291" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1256" t="inlineStr">
+      <c r="B14" s="1292" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1256" t="inlineStr">
+      <c r="C14" s="1292" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1257" t="n"/>
-      <c r="E14" s="1257" t="n">
+      <c r="D14" s="1293" t="n"/>
+      <c r="E14" s="1293" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1257" t="n">
+      <c r="F14" s="1293" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1257" t="n">
+      <c r="G14" s="1293" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1257" t="n"/>
-      <c r="I14" s="1258" t="n"/>
-      <c r="J14" s="1259" t="n"/>
-      <c r="K14" s="1259" t="n"/>
-      <c r="L14" s="1259" t="n"/>
-      <c r="M14" s="1257" t="n"/>
-      <c r="N14" s="1257" t="n"/>
-      <c r="O14" s="1257" t="n">
+      <c r="H14" s="1293" t="n"/>
+      <c r="I14" s="1294" t="n"/>
+      <c r="J14" s="1295" t="n"/>
+      <c r="K14" s="1295" t="n"/>
+      <c r="L14" s="1295" t="n"/>
+      <c r="M14" s="1293" t="n"/>
+      <c r="N14" s="1293" t="n"/>
+      <c r="O14" s="1293" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1260" t="n">
+      <c r="P14" s="1296" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1257" t="n"/>
-      <c r="R14" s="1257" t="n"/>
-      <c r="S14" s="1257" t="n"/>
+      <c r="Q14" s="1293" t="n"/>
+      <c r="R14" s="1293" t="n"/>
+      <c r="S14" s="1293" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1256" t="n"/>
+      <c r="U14" s="1292" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -5328,43 +5454,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1255" t="inlineStr">
+      <c r="A15" s="1291" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1256" t="inlineStr">
+      <c r="B15" s="1292" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1256" t="inlineStr">
+      <c r="C15" s="1292" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1257" t="n"/>
-      <c r="E15" s="1257" t="n"/>
-      <c r="F15" s="1257" t="n"/>
-      <c r="G15" s="1257" t="n"/>
-      <c r="H15" s="1257" t="n"/>
-      <c r="I15" s="1258" t="n"/>
-      <c r="J15" s="1259" t="n"/>
-      <c r="K15" s="1259" t="n"/>
-      <c r="L15" s="1259" t="n"/>
-      <c r="M15" s="1257" t="n">
+      <c r="D15" s="1293" t="n"/>
+      <c r="E15" s="1293" t="n"/>
+      <c r="F15" s="1293" t="n"/>
+      <c r="G15" s="1293" t="n"/>
+      <c r="H15" s="1293" t="n"/>
+      <c r="I15" s="1294" t="n"/>
+      <c r="J15" s="1295" t="n"/>
+      <c r="K15" s="1295" t="n"/>
+      <c r="L15" s="1295" t="n"/>
+      <c r="M15" s="1293" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1257" t="n">
+      <c r="N15" s="1293" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1257" t="n"/>
-      <c r="P15" s="1260" t="n"/>
-      <c r="Q15" s="1257" t="n"/>
-      <c r="R15" s="1257" t="n"/>
-      <c r="S15" s="1257" t="n"/>
+      <c r="O15" s="1293" t="n"/>
+      <c r="P15" s="1296" t="n"/>
+      <c r="Q15" s="1293" t="n"/>
+      <c r="R15" s="1293" t="n"/>
+      <c r="S15" s="1293" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1256" t="n"/>
+      <c r="U15" s="1292" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -5372,39 +5498,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1261" t="inlineStr">
+      <c r="A16" s="1297" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1262" t="inlineStr">
+      <c r="B16" s="1298" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1262" t="inlineStr">
+      <c r="C16" s="1298" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1263" t="n"/>
-      <c r="E16" s="1263" t="n"/>
-      <c r="F16" s="1263" t="n"/>
-      <c r="G16" s="1263" t="n"/>
-      <c r="H16" s="1263" t="n"/>
-      <c r="I16" s="1264" t="n"/>
-      <c r="J16" s="1265" t="n"/>
-      <c r="K16" s="1265" t="n"/>
-      <c r="L16" s="1265" t="n"/>
-      <c r="M16" s="1263" t="n"/>
-      <c r="N16" s="1263" t="n"/>
-      <c r="O16" s="1263" t="n"/>
-      <c r="P16" s="1266" t="n"/>
-      <c r="Q16" s="1263" t="n"/>
-      <c r="R16" s="1263" t="n"/>
-      <c r="S16" s="1263" t="n"/>
+      <c r="D16" s="1299" t="n"/>
+      <c r="E16" s="1299" t="n"/>
+      <c r="F16" s="1299" t="n"/>
+      <c r="G16" s="1299" t="n"/>
+      <c r="H16" s="1299" t="n"/>
+      <c r="I16" s="1300" t="n"/>
+      <c r="J16" s="1301" t="n"/>
+      <c r="K16" s="1301" t="n"/>
+      <c r="L16" s="1301" t="n"/>
+      <c r="M16" s="1299" t="n"/>
+      <c r="N16" s="1299" t="n"/>
+      <c r="O16" s="1299" t="n"/>
+      <c r="P16" s="1302" t="n"/>
+      <c r="Q16" s="1299" t="n"/>
+      <c r="R16" s="1299" t="n"/>
+      <c r="S16" s="1299" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1262" t="n"/>
+      <c r="U16" s="1298" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -5412,39 +5538,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1237" t="inlineStr">
+      <c r="A17" s="1273" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1238" t="inlineStr">
+      <c r="B17" s="1274" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1238" t="inlineStr">
+      <c r="C17" s="1274" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1239" t="n"/>
-      <c r="E17" s="1239" t="n"/>
-      <c r="F17" s="1239" t="n"/>
-      <c r="G17" s="1239" t="n"/>
-      <c r="H17" s="1239" t="n"/>
-      <c r="I17" s="1240" t="n"/>
-      <c r="J17" s="1241" t="n"/>
-      <c r="K17" s="1241" t="n"/>
-      <c r="L17" s="1241" t="n"/>
-      <c r="M17" s="1239" t="n"/>
-      <c r="N17" s="1239" t="n"/>
-      <c r="O17" s="1239" t="n"/>
-      <c r="P17" s="1242" t="n"/>
-      <c r="Q17" s="1239" t="n"/>
-      <c r="R17" s="1239" t="n"/>
-      <c r="S17" s="1239" t="n"/>
+      <c r="D17" s="1275" t="n"/>
+      <c r="E17" s="1275" t="n"/>
+      <c r="F17" s="1275" t="n"/>
+      <c r="G17" s="1275" t="n"/>
+      <c r="H17" s="1275" t="n"/>
+      <c r="I17" s="1276" t="n"/>
+      <c r="J17" s="1277" t="n"/>
+      <c r="K17" s="1277" t="n"/>
+      <c r="L17" s="1277" t="n"/>
+      <c r="M17" s="1275" t="n"/>
+      <c r="N17" s="1275" t="n"/>
+      <c r="O17" s="1275" t="n"/>
+      <c r="P17" s="1278" t="n"/>
+      <c r="Q17" s="1275" t="n"/>
+      <c r="R17" s="1275" t="n"/>
+      <c r="S17" s="1275" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1238" t="n"/>
+      <c r="U17" s="1274" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -5452,53 +5578,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1267" t="inlineStr">
+      <c r="A18" s="1303" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1268" t="inlineStr">
+      <c r="B18" s="1304" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1268" t="inlineStr">
+      <c r="C18" s="1304" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1269" t="n"/>
-      <c r="E18" s="1269" t="n">
+      <c r="D18" s="1305" t="n"/>
+      <c r="E18" s="1305" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1269" t="n">
+      <c r="F18" s="1305" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1269" t="n">
+      <c r="G18" s="1305" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1269" t="n"/>
-      <c r="I18" s="1270" t="n"/>
-      <c r="J18" s="1271" t="n"/>
-      <c r="K18" s="1271" t="n"/>
-      <c r="L18" s="1271" t="n"/>
-      <c r="M18" s="1269" t="n"/>
-      <c r="N18" s="1269" t="n"/>
-      <c r="O18" s="1269" t="n">
+      <c r="H18" s="1305" t="n"/>
+      <c r="I18" s="1306" t="n"/>
+      <c r="J18" s="1307" t="n"/>
+      <c r="K18" s="1307" t="n"/>
+      <c r="L18" s="1307" t="n"/>
+      <c r="M18" s="1305" t="n"/>
+      <c r="N18" s="1305" t="n"/>
+      <c r="O18" s="1305" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1272" t="n">
+      <c r="P18" s="1308" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1269" t="n"/>
-      <c r="R18" s="1269" t="n"/>
-      <c r="S18" s="1269" t="n"/>
+      <c r="Q18" s="1305" t="n"/>
+      <c r="R18" s="1305" t="n"/>
+      <c r="S18" s="1305" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1268" t="n"/>
+      <c r="U18" s="1304" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -5506,47 +5632,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1267" t="inlineStr">
+      <c r="A19" s="1303" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1268" t="inlineStr">
+      <c r="B19" s="1304" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1268" t="inlineStr">
+      <c r="C19" s="1304" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1269" t="n"/>
-      <c r="E19" s="1269" t="n"/>
-      <c r="F19" s="1269" t="n"/>
-      <c r="G19" s="1269" t="n"/>
-      <c r="H19" s="1269" t="n"/>
-      <c r="I19" s="1270" t="n"/>
-      <c r="J19" s="1271" t="n"/>
-      <c r="K19" s="1271" t="n"/>
-      <c r="L19" s="1271" t="n"/>
-      <c r="M19" s="1269" t="n">
+      <c r="D19" s="1305" t="n"/>
+      <c r="E19" s="1305" t="n"/>
+      <c r="F19" s="1305" t="n"/>
+      <c r="G19" s="1305" t="n"/>
+      <c r="H19" s="1305" t="n"/>
+      <c r="I19" s="1306" t="n"/>
+      <c r="J19" s="1307" t="n"/>
+      <c r="K19" s="1307" t="n"/>
+      <c r="L19" s="1307" t="n"/>
+      <c r="M19" s="1305" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1269" t="n">
+      <c r="N19" s="1305" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1269" t="n"/>
-      <c r="P19" s="1272" t="n"/>
-      <c r="Q19" s="1269" t="n"/>
-      <c r="R19" s="1269" t="n"/>
-      <c r="S19" s="1269" t="n"/>
+      <c r="O19" s="1305" t="n"/>
+      <c r="P19" s="1308" t="n"/>
+      <c r="Q19" s="1305" t="n"/>
+      <c r="R19" s="1305" t="n"/>
+      <c r="S19" s="1305" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1268" t="n"/>
+      <c r="U19" s="1304" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -5554,43 +5680,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1267" t="inlineStr">
+      <c r="A20" s="1303" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1268" t="inlineStr">
+      <c r="B20" s="1304" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1268" t="inlineStr">
+      <c r="C20" s="1304" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1269" t="n"/>
-      <c r="E20" s="1269" t="n"/>
-      <c r="F20" s="1269" t="n"/>
-      <c r="G20" s="1269" t="n"/>
-      <c r="H20" s="1269" t="n"/>
-      <c r="I20" s="1270" t="n"/>
-      <c r="J20" s="1271" t="n"/>
-      <c r="K20" s="1271" t="n"/>
-      <c r="L20" s="1271" t="n"/>
-      <c r="M20" s="1269" t="n"/>
-      <c r="N20" s="1269" t="n"/>
-      <c r="O20" s="1269" t="n"/>
-      <c r="P20" s="1272" t="n"/>
-      <c r="Q20" s="1269" t="n"/>
-      <c r="R20" s="1269" t="n"/>
-      <c r="S20" s="1269" t="n"/>
+      <c r="D20" s="1305" t="n"/>
+      <c r="E20" s="1305" t="n"/>
+      <c r="F20" s="1305" t="n"/>
+      <c r="G20" s="1305" t="n"/>
+      <c r="H20" s="1305" t="n"/>
+      <c r="I20" s="1306" t="n"/>
+      <c r="J20" s="1307" t="n"/>
+      <c r="K20" s="1307" t="n"/>
+      <c r="L20" s="1307" t="n"/>
+      <c r="M20" s="1305" t="n"/>
+      <c r="N20" s="1305" t="n"/>
+      <c r="O20" s="1305" t="n"/>
+      <c r="P20" s="1308" t="n"/>
+      <c r="Q20" s="1305" t="n"/>
+      <c r="R20" s="1305" t="n"/>
+      <c r="S20" s="1305" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1268" t="n"/>
+      <c r="U20" s="1304" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -5598,39 +5724,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1243" t="inlineStr">
+      <c r="A21" s="1279" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1244" t="inlineStr">
+      <c r="B21" s="1280" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1244" t="inlineStr">
+      <c r="C21" s="1280" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1245" t="n"/>
-      <c r="E21" s="1245" t="n"/>
-      <c r="F21" s="1245" t="n"/>
-      <c r="G21" s="1245" t="n"/>
-      <c r="H21" s="1245" t="n"/>
-      <c r="I21" s="1246" t="n"/>
-      <c r="J21" s="1247" t="n"/>
-      <c r="K21" s="1247" t="n"/>
-      <c r="L21" s="1247" t="n"/>
-      <c r="M21" s="1245" t="n"/>
-      <c r="N21" s="1245" t="n"/>
-      <c r="O21" s="1245" t="n"/>
-      <c r="P21" s="1248" t="n"/>
-      <c r="Q21" s="1245" t="n"/>
-      <c r="R21" s="1245" t="n"/>
-      <c r="S21" s="1245" t="n"/>
+      <c r="D21" s="1281" t="n"/>
+      <c r="E21" s="1281" t="n"/>
+      <c r="F21" s="1281" t="n"/>
+      <c r="G21" s="1281" t="n"/>
+      <c r="H21" s="1281" t="n"/>
+      <c r="I21" s="1282" t="n"/>
+      <c r="J21" s="1283" t="n"/>
+      <c r="K21" s="1283" t="n"/>
+      <c r="L21" s="1283" t="n"/>
+      <c r="M21" s="1281" t="n"/>
+      <c r="N21" s="1281" t="n"/>
+      <c r="O21" s="1281" t="n"/>
+      <c r="P21" s="1284" t="n"/>
+      <c r="Q21" s="1281" t="n"/>
+      <c r="R21" s="1281" t="n"/>
+      <c r="S21" s="1281" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1244" t="n"/>
+      <c r="U21" s="1280" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -5638,39 +5764,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1249" t="inlineStr">
+      <c r="A22" s="1285" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1250" t="inlineStr">
+      <c r="B22" s="1286" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1250" t="inlineStr">
+      <c r="C22" s="1286" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1251" t="n"/>
-      <c r="E22" s="1251" t="n"/>
-      <c r="F22" s="1251" t="n"/>
-      <c r="G22" s="1251" t="n"/>
-      <c r="H22" s="1251" t="n"/>
-      <c r="I22" s="1252" t="n"/>
-      <c r="J22" s="1253" t="n"/>
-      <c r="K22" s="1253" t="n"/>
-      <c r="L22" s="1253" t="n"/>
-      <c r="M22" s="1251" t="n"/>
-      <c r="N22" s="1251" t="n"/>
-      <c r="O22" s="1251" t="n"/>
-      <c r="P22" s="1254" t="n"/>
-      <c r="Q22" s="1251" t="n"/>
-      <c r="R22" s="1251" t="n"/>
-      <c r="S22" s="1251" t="n"/>
+      <c r="D22" s="1287" t="n"/>
+      <c r="E22" s="1287" t="n"/>
+      <c r="F22" s="1287" t="n"/>
+      <c r="G22" s="1287" t="n"/>
+      <c r="H22" s="1287" t="n"/>
+      <c r="I22" s="1288" t="n"/>
+      <c r="J22" s="1289" t="n"/>
+      <c r="K22" s="1289" t="n"/>
+      <c r="L22" s="1289" t="n"/>
+      <c r="M22" s="1287" t="n"/>
+      <c r="N22" s="1287" t="n"/>
+      <c r="O22" s="1287" t="n"/>
+      <c r="P22" s="1290" t="n"/>
+      <c r="Q22" s="1287" t="n"/>
+      <c r="R22" s="1287" t="n"/>
+      <c r="S22" s="1287" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1250" t="n"/>
+      <c r="U22" s="1286" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -5678,53 +5804,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1255" t="inlineStr">
+      <c r="A23" s="1291" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1256" t="inlineStr">
+      <c r="B23" s="1292" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1256" t="inlineStr">
+      <c r="C23" s="1292" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1257" t="n"/>
-      <c r="E23" s="1257" t="n">
+      <c r="D23" s="1293" t="n"/>
+      <c r="E23" s="1293" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1257" t="n">
+      <c r="F23" s="1293" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1257" t="n">
+      <c r="G23" s="1293" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1257" t="n"/>
-      <c r="I23" s="1258" t="n"/>
-      <c r="J23" s="1259" t="n"/>
-      <c r="K23" s="1259" t="n"/>
-      <c r="L23" s="1259" t="n"/>
-      <c r="M23" s="1257" t="n"/>
-      <c r="N23" s="1257" t="n"/>
-      <c r="O23" s="1257" t="n">
+      <c r="H23" s="1293" t="n"/>
+      <c r="I23" s="1294" t="n"/>
+      <c r="J23" s="1295" t="n"/>
+      <c r="K23" s="1295" t="n"/>
+      <c r="L23" s="1295" t="n"/>
+      <c r="M23" s="1293" t="n"/>
+      <c r="N23" s="1293" t="n"/>
+      <c r="O23" s="1293" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1260" t="n">
+      <c r="P23" s="1296" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1257" t="n"/>
-      <c r="R23" s="1257" t="n"/>
-      <c r="S23" s="1257" t="n"/>
+      <c r="Q23" s="1293" t="n"/>
+      <c r="R23" s="1293" t="n"/>
+      <c r="S23" s="1293" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1256" t="n"/>
+      <c r="U23" s="1292" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -5732,47 +5858,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1261" t="inlineStr">
+      <c r="A24" s="1297" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1262" t="inlineStr">
+      <c r="B24" s="1298" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1262" t="inlineStr">
+      <c r="C24" s="1298" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1263" t="n"/>
-      <c r="E24" s="1263" t="n"/>
-      <c r="F24" s="1263" t="n"/>
-      <c r="G24" s="1263" t="n"/>
-      <c r="H24" s="1263" t="n"/>
-      <c r="I24" s="1264" t="n"/>
-      <c r="J24" s="1265" t="n"/>
-      <c r="K24" s="1265" t="n"/>
-      <c r="L24" s="1265" t="n"/>
-      <c r="M24" s="1263" t="n">
+      <c r="D24" s="1299" t="n"/>
+      <c r="E24" s="1299" t="n"/>
+      <c r="F24" s="1299" t="n"/>
+      <c r="G24" s="1299" t="n"/>
+      <c r="H24" s="1299" t="n"/>
+      <c r="I24" s="1300" t="n"/>
+      <c r="J24" s="1301" t="n"/>
+      <c r="K24" s="1301" t="n"/>
+      <c r="L24" s="1301" t="n"/>
+      <c r="M24" s="1299" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1263" t="n">
+      <c r="N24" s="1299" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1263" t="n"/>
-      <c r="P24" s="1266" t="n"/>
-      <c r="Q24" s="1263" t="n"/>
-      <c r="R24" s="1263" t="n"/>
-      <c r="S24" s="1263" t="n"/>
+      <c r="O24" s="1299" t="n"/>
+      <c r="P24" s="1302" t="n"/>
+      <c r="Q24" s="1299" t="n"/>
+      <c r="R24" s="1299" t="n"/>
+      <c r="S24" s="1299" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1262" t="n"/>
+      <c r="U24" s="1298" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -5780,61 +5906,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1237" t="inlineStr">
+      <c r="A25" s="1273" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1238" t="inlineStr">
+      <c r="B25" s="1274" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1238" t="inlineStr">
+      <c r="C25" s="1274" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1239" t="n">
+      <c r="D25" s="1275" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1239" t="n">
+      <c r="E25" s="1275" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1239" t="n">
+      <c r="F25" s="1275" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1239" t="n">
+      <c r="G25" s="1275" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1239" t="n"/>
-      <c r="I25" s="1240" t="n"/>
-      <c r="J25" s="1241" t="n">
+      <c r="H25" s="1275" t="n"/>
+      <c r="I25" s="1276" t="n"/>
+      <c r="J25" s="1277" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1241" t="n">
+      <c r="K25" s="1277" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1241" t="n">
+      <c r="L25" s="1277" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1239" t="n"/>
-      <c r="N25" s="1239" t="n"/>
-      <c r="O25" s="1239" t="n">
+      <c r="M25" s="1275" t="n"/>
+      <c r="N25" s="1275" t="n"/>
+      <c r="O25" s="1275" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1242" t="n">
+      <c r="P25" s="1278" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1239" t="n"/>
-      <c r="R25" s="1239" t="n"/>
-      <c r="S25" s="1239" t="n"/>
+      <c r="Q25" s="1275" t="n"/>
+      <c r="R25" s="1275" t="n"/>
+      <c r="S25" s="1275" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1238" t="n"/>
+      <c r="U25" s="1274" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -5842,47 +5968,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1243" t="inlineStr">
+      <c r="A26" s="1279" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1244" t="inlineStr">
+      <c r="B26" s="1280" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1244" t="inlineStr">
+      <c r="C26" s="1280" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1245" t="n"/>
-      <c r="E26" s="1245" t="n"/>
-      <c r="F26" s="1245" t="n"/>
-      <c r="G26" s="1245" t="n"/>
-      <c r="H26" s="1245" t="n"/>
-      <c r="I26" s="1246" t="n"/>
-      <c r="J26" s="1247" t="n"/>
-      <c r="K26" s="1247" t="n"/>
-      <c r="L26" s="1247" t="n"/>
-      <c r="M26" s="1245" t="n">
+      <c r="D26" s="1281" t="n"/>
+      <c r="E26" s="1281" t="n"/>
+      <c r="F26" s="1281" t="n"/>
+      <c r="G26" s="1281" t="n"/>
+      <c r="H26" s="1281" t="n"/>
+      <c r="I26" s="1282" t="n"/>
+      <c r="J26" s="1283" t="n"/>
+      <c r="K26" s="1283" t="n"/>
+      <c r="L26" s="1283" t="n"/>
+      <c r="M26" s="1281" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1245" t="n">
+      <c r="N26" s="1281" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1245" t="n"/>
-      <c r="P26" s="1248" t="n"/>
-      <c r="Q26" s="1245" t="n"/>
-      <c r="R26" s="1245" t="n"/>
-      <c r="S26" s="1245" t="n"/>
+      <c r="O26" s="1281" t="n"/>
+      <c r="P26" s="1284" t="n"/>
+      <c r="Q26" s="1281" t="n"/>
+      <c r="R26" s="1281" t="n"/>
+      <c r="S26" s="1281" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1244" t="n"/>
+      <c r="U26" s="1280" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -5890,53 +6016,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1249" t="inlineStr">
+      <c r="A27" s="1285" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1250" t="inlineStr">
+      <c r="B27" s="1286" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1250" t="inlineStr">
+      <c r="C27" s="1286" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1251" t="n"/>
-      <c r="E27" s="1251" t="n">
+      <c r="D27" s="1287" t="n"/>
+      <c r="E27" s="1287" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1251" t="n">
+      <c r="F27" s="1287" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1251" t="n">
+      <c r="G27" s="1287" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1251" t="n"/>
-      <c r="I27" s="1252" t="n"/>
-      <c r="J27" s="1253" t="n"/>
-      <c r="K27" s="1253" t="n"/>
-      <c r="L27" s="1253" t="n"/>
-      <c r="M27" s="1251" t="n"/>
-      <c r="N27" s="1251" t="n"/>
-      <c r="O27" s="1251" t="n">
+      <c r="H27" s="1287" t="n"/>
+      <c r="I27" s="1288" t="n"/>
+      <c r="J27" s="1289" t="n"/>
+      <c r="K27" s="1289" t="n"/>
+      <c r="L27" s="1289" t="n"/>
+      <c r="M27" s="1287" t="n"/>
+      <c r="N27" s="1287" t="n"/>
+      <c r="O27" s="1287" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1254" t="n">
+      <c r="P27" s="1290" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1251" t="n"/>
-      <c r="R27" s="1251" t="n"/>
-      <c r="S27" s="1251" t="n"/>
+      <c r="Q27" s="1287" t="n"/>
+      <c r="R27" s="1287" t="n"/>
+      <c r="S27" s="1287" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1250" t="n"/>
+      <c r="U27" s="1286" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -5944,47 +6070,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1261" t="inlineStr">
+      <c r="A28" s="1297" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1262" t="inlineStr">
+      <c r="B28" s="1298" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1262" t="inlineStr">
+      <c r="C28" s="1298" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1263" t="n"/>
-      <c r="E28" s="1263" t="n"/>
-      <c r="F28" s="1263" t="n"/>
-      <c r="G28" s="1263" t="n"/>
-      <c r="H28" s="1263" t="n"/>
-      <c r="I28" s="1264" t="n"/>
-      <c r="J28" s="1265" t="n"/>
-      <c r="K28" s="1265" t="n"/>
-      <c r="L28" s="1265" t="n"/>
-      <c r="M28" s="1263" t="n">
+      <c r="D28" s="1299" t="n"/>
+      <c r="E28" s="1299" t="n"/>
+      <c r="F28" s="1299" t="n"/>
+      <c r="G28" s="1299" t="n"/>
+      <c r="H28" s="1299" t="n"/>
+      <c r="I28" s="1300" t="n"/>
+      <c r="J28" s="1301" t="n"/>
+      <c r="K28" s="1301" t="n"/>
+      <c r="L28" s="1301" t="n"/>
+      <c r="M28" s="1299" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1263" t="n">
+      <c r="N28" s="1299" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1263" t="n"/>
-      <c r="P28" s="1266" t="n"/>
-      <c r="Q28" s="1263" t="n"/>
-      <c r="R28" s="1263" t="n"/>
-      <c r="S28" s="1263" t="n"/>
+      <c r="O28" s="1299" t="n"/>
+      <c r="P28" s="1302" t="n"/>
+      <c r="Q28" s="1299" t="n"/>
+      <c r="R28" s="1299" t="n"/>
+      <c r="S28" s="1299" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1262" t="n"/>
+      <c r="U28" s="1298" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -5992,53 +6118,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1237" t="inlineStr">
+      <c r="A29" s="1273" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1238" t="inlineStr">
+      <c r="B29" s="1274" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1238" t="inlineStr">
+      <c r="C29" s="1274" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1239" t="n"/>
-      <c r="E29" s="1239" t="n">
+      <c r="D29" s="1275" t="n"/>
+      <c r="E29" s="1275" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1239" t="n">
+      <c r="F29" s="1275" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1239" t="n">
+      <c r="G29" s="1275" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1239" t="n"/>
-      <c r="I29" s="1240" t="n"/>
-      <c r="J29" s="1241" t="n"/>
-      <c r="K29" s="1241" t="n"/>
-      <c r="L29" s="1241" t="n"/>
-      <c r="M29" s="1239" t="n"/>
-      <c r="N29" s="1239" t="n"/>
-      <c r="O29" s="1239" t="n">
+      <c r="H29" s="1275" t="n"/>
+      <c r="I29" s="1276" t="n"/>
+      <c r="J29" s="1277" t="n"/>
+      <c r="K29" s="1277" t="n"/>
+      <c r="L29" s="1277" t="n"/>
+      <c r="M29" s="1275" t="n"/>
+      <c r="N29" s="1275" t="n"/>
+      <c r="O29" s="1275" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1242" t="n">
+      <c r="P29" s="1278" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1239" t="n"/>
-      <c r="R29" s="1239" t="n"/>
-      <c r="S29" s="1239" t="n"/>
+      <c r="Q29" s="1275" t="n"/>
+      <c r="R29" s="1275" t="n"/>
+      <c r="S29" s="1275" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1238" t="n"/>
+      <c r="U29" s="1274" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -6046,43 +6172,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1243" t="inlineStr">
+      <c r="A30" s="1279" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1244" t="inlineStr">
+      <c r="B30" s="1280" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1244" t="inlineStr">
+      <c r="C30" s="1280" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1245" t="n"/>
-      <c r="E30" s="1245" t="n"/>
-      <c r="F30" s="1245" t="n"/>
-      <c r="G30" s="1245" t="n"/>
-      <c r="H30" s="1245" t="n"/>
-      <c r="I30" s="1246" t="n"/>
-      <c r="J30" s="1247" t="n"/>
-      <c r="K30" s="1247" t="n"/>
-      <c r="L30" s="1247" t="n"/>
-      <c r="M30" s="1245" t="n"/>
-      <c r="N30" s="1245" t="n"/>
-      <c r="O30" s="1245" t="n"/>
-      <c r="P30" s="1248" t="n"/>
-      <c r="Q30" s="1245" t="n"/>
-      <c r="R30" s="1245" t="n"/>
-      <c r="S30" s="1245" t="n"/>
+      <c r="D30" s="1281" t="n"/>
+      <c r="E30" s="1281" t="n"/>
+      <c r="F30" s="1281" t="n"/>
+      <c r="G30" s="1281" t="n"/>
+      <c r="H30" s="1281" t="n"/>
+      <c r="I30" s="1282" t="n"/>
+      <c r="J30" s="1283" t="n"/>
+      <c r="K30" s="1283" t="n"/>
+      <c r="L30" s="1283" t="n"/>
+      <c r="M30" s="1281" t="n"/>
+      <c r="N30" s="1281" t="n"/>
+      <c r="O30" s="1281" t="n"/>
+      <c r="P30" s="1284" t="n"/>
+      <c r="Q30" s="1281" t="n"/>
+      <c r="R30" s="1281" t="n"/>
+      <c r="S30" s="1281" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1244" t="n"/>
+      <c r="U30" s="1280" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -6090,53 +6216,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1249" t="inlineStr">
+      <c r="A31" s="1285" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1250" t="inlineStr">
+      <c r="B31" s="1286" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1250" t="inlineStr">
+      <c r="C31" s="1286" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1251" t="n"/>
-      <c r="E31" s="1251" t="n">
+      <c r="D31" s="1287" t="n"/>
+      <c r="E31" s="1287" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1251" t="n">
+      <c r="F31" s="1287" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1251" t="n">
+      <c r="G31" s="1287" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1251" t="n"/>
-      <c r="I31" s="1252" t="n"/>
-      <c r="J31" s="1253" t="n"/>
-      <c r="K31" s="1253" t="n"/>
-      <c r="L31" s="1253" t="n"/>
-      <c r="M31" s="1251" t="n"/>
-      <c r="N31" s="1251" t="n"/>
-      <c r="O31" s="1251" t="n">
+      <c r="H31" s="1287" t="n"/>
+      <c r="I31" s="1288" t="n"/>
+      <c r="J31" s="1289" t="n"/>
+      <c r="K31" s="1289" t="n"/>
+      <c r="L31" s="1289" t="n"/>
+      <c r="M31" s="1287" t="n"/>
+      <c r="N31" s="1287" t="n"/>
+      <c r="O31" s="1287" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1254" t="n">
+      <c r="P31" s="1290" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1251" t="n"/>
-      <c r="R31" s="1251" t="n"/>
-      <c r="S31" s="1251" t="n"/>
+      <c r="Q31" s="1287" t="n"/>
+      <c r="R31" s="1287" t="n"/>
+      <c r="S31" s="1287" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1250" t="inlineStr">
+      <c r="U31" s="1286" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -6148,49 +6274,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1261" t="inlineStr">
+      <c r="A32" s="1297" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1262" t="inlineStr">
+      <c r="B32" s="1298" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1262" t="inlineStr">
+      <c r="C32" s="1298" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1263" t="n"/>
-      <c r="E32" s="1263" t="n"/>
-      <c r="F32" s="1263" t="n"/>
-      <c r="G32" s="1263" t="n"/>
-      <c r="H32" s="1263" t="n">
+      <c r="D32" s="1299" t="n"/>
+      <c r="E32" s="1299" t="n"/>
+      <c r="F32" s="1299" t="n"/>
+      <c r="G32" s="1299" t="n"/>
+      <c r="H32" s="1299" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1264" t="n"/>
-      <c r="J32" s="1265" t="n"/>
-      <c r="K32" s="1265" t="n"/>
-      <c r="L32" s="1265" t="n"/>
-      <c r="M32" s="1263" t="n">
+      <c r="I32" s="1300" t="n"/>
+      <c r="J32" s="1301" t="n"/>
+      <c r="K32" s="1301" t="n"/>
+      <c r="L32" s="1301" t="n"/>
+      <c r="M32" s="1299" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1263" t="n">
+      <c r="N32" s="1299" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1263" t="n"/>
-      <c r="P32" s="1266" t="n"/>
-      <c r="Q32" s="1263" t="n"/>
-      <c r="R32" s="1263" t="n"/>
-      <c r="S32" s="1263" t="n"/>
+      <c r="O32" s="1299" t="n"/>
+      <c r="P32" s="1302" t="n"/>
+      <c r="Q32" s="1299" t="n"/>
+      <c r="R32" s="1299" t="n"/>
+      <c r="S32" s="1299" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1262" t="n"/>
+      <c r="U32" s="1298" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -6198,57 +6324,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1237" t="inlineStr">
+      <c r="A33" s="1273" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1238" t="inlineStr">
+      <c r="B33" s="1274" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1238" t="inlineStr">
+      <c r="C33" s="1274" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1239" t="n"/>
-      <c r="E33" s="1239" t="n">
+      <c r="D33" s="1275" t="n"/>
+      <c r="E33" s="1275" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1239" t="n">
+      <c r="F33" s="1275" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1239" t="n">
+      <c r="G33" s="1275" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1239" t="n"/>
-      <c r="I33" s="1240" t="n">
+      <c r="H33" s="1275" t="n"/>
+      <c r="I33" s="1276" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1241" t="n"/>
-      <c r="K33" s="1241" t="n"/>
-      <c r="L33" s="1241" t="n"/>
-      <c r="M33" s="1239" t="n"/>
-      <c r="N33" s="1239" t="n"/>
-      <c r="O33" s="1239" t="n">
+      <c r="J33" s="1277" t="n"/>
+      <c r="K33" s="1277" t="n"/>
+      <c r="L33" s="1277" t="n"/>
+      <c r="M33" s="1275" t="n"/>
+      <c r="N33" s="1275" t="n"/>
+      <c r="O33" s="1275" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1242" t="n">
+      <c r="P33" s="1278" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1239" t="n"/>
-      <c r="R33" s="1239" t="n">
+      <c r="Q33" s="1275" t="n"/>
+      <c r="R33" s="1275" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1239" t="n"/>
+      <c r="S33" s="1275" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1238" t="inlineStr">
+      <c r="U33" s="1274" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -6260,49 +6386,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1243" t="inlineStr">
+      <c r="A34" s="1279" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1244" t="inlineStr">
+      <c r="B34" s="1280" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1244" t="inlineStr">
+      <c r="C34" s="1280" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1245" t="n"/>
-      <c r="E34" s="1245" t="n"/>
-      <c r="F34" s="1245" t="n"/>
-      <c r="G34" s="1245" t="n"/>
-      <c r="H34" s="1245" t="n">
+      <c r="D34" s="1281" t="n"/>
+      <c r="E34" s="1281" t="n"/>
+      <c r="F34" s="1281" t="n"/>
+      <c r="G34" s="1281" t="n"/>
+      <c r="H34" s="1281" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1246" t="n"/>
-      <c r="J34" s="1247" t="n"/>
-      <c r="K34" s="1247" t="n"/>
-      <c r="L34" s="1247" t="n"/>
-      <c r="M34" s="1245" t="n">
+      <c r="I34" s="1282" t="n"/>
+      <c r="J34" s="1283" t="n"/>
+      <c r="K34" s="1283" t="n"/>
+      <c r="L34" s="1283" t="n"/>
+      <c r="M34" s="1281" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1245" t="n">
+      <c r="N34" s="1281" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1245" t="n"/>
-      <c r="P34" s="1248" t="n"/>
-      <c r="Q34" s="1245" t="n"/>
-      <c r="R34" s="1245" t="n"/>
-      <c r="S34" s="1245" t="n"/>
+      <c r="O34" s="1281" t="n"/>
+      <c r="P34" s="1284" t="n"/>
+      <c r="Q34" s="1281" t="n"/>
+      <c r="R34" s="1281" t="n"/>
+      <c r="S34" s="1281" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1244" t="n"/>
+      <c r="U34" s="1280" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -6310,57 +6436,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1249" t="inlineStr">
+      <c r="A35" s="1285" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1250" t="inlineStr">
+      <c r="B35" s="1286" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1250" t="inlineStr">
+      <c r="C35" s="1286" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1251" t="n"/>
-      <c r="E35" s="1251" t="n">
+      <c r="D35" s="1287" t="n"/>
+      <c r="E35" s="1287" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1251" t="n">
+      <c r="F35" s="1287" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1251" t="n">
+      <c r="G35" s="1287" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1251" t="n"/>
-      <c r="I35" s="1252" t="n">
+      <c r="H35" s="1287" t="n"/>
+      <c r="I35" s="1288" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1253" t="n"/>
-      <c r="K35" s="1253" t="n"/>
-      <c r="L35" s="1253" t="n"/>
-      <c r="M35" s="1251" t="n"/>
-      <c r="N35" s="1251" t="n"/>
-      <c r="O35" s="1251" t="n">
+      <c r="J35" s="1289" t="n"/>
+      <c r="K35" s="1289" t="n"/>
+      <c r="L35" s="1289" t="n"/>
+      <c r="M35" s="1287" t="n"/>
+      <c r="N35" s="1287" t="n"/>
+      <c r="O35" s="1287" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1254" t="n">
+      <c r="P35" s="1290" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1251" t="n"/>
-      <c r="R35" s="1251" t="n">
+      <c r="Q35" s="1287" t="n"/>
+      <c r="R35" s="1287" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1251" t="n"/>
+      <c r="S35" s="1287" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1250" t="inlineStr">
+      <c r="U35" s="1286" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -6372,49 +6498,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1255" t="inlineStr">
+      <c r="A36" s="1291" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1256" t="inlineStr">
+      <c r="B36" s="1292" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1256" t="inlineStr">
+      <c r="C36" s="1292" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1257" t="n"/>
-      <c r="E36" s="1257" t="n"/>
-      <c r="F36" s="1257" t="n"/>
-      <c r="G36" s="1257" t="n"/>
-      <c r="H36" s="1257" t="n">
+      <c r="D36" s="1293" t="n"/>
+      <c r="E36" s="1293" t="n"/>
+      <c r="F36" s="1293" t="n"/>
+      <c r="G36" s="1293" t="n"/>
+      <c r="H36" s="1293" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1258" t="n"/>
-      <c r="J36" s="1259" t="n"/>
-      <c r="K36" s="1259" t="n"/>
-      <c r="L36" s="1259" t="n"/>
-      <c r="M36" s="1257" t="n">
+      <c r="I36" s="1294" t="n"/>
+      <c r="J36" s="1295" t="n"/>
+      <c r="K36" s="1295" t="n"/>
+      <c r="L36" s="1295" t="n"/>
+      <c r="M36" s="1293" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1257" t="n">
+      <c r="N36" s="1293" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1257" t="n"/>
-      <c r="P36" s="1260" t="n"/>
-      <c r="Q36" s="1257" t="n"/>
-      <c r="R36" s="1257" t="n"/>
-      <c r="S36" s="1257" t="n"/>
+      <c r="O36" s="1293" t="n"/>
+      <c r="P36" s="1296" t="n"/>
+      <c r="Q36" s="1293" t="n"/>
+      <c r="R36" s="1293" t="n"/>
+      <c r="S36" s="1293" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1256" t="n"/>
+      <c r="U36" s="1292" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -6422,41 +6548,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1261" t="inlineStr">
+      <c r="A37" s="1297" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1262" t="inlineStr">
+      <c r="B37" s="1298" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1262" t="inlineStr">
+      <c r="C37" s="1298" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1263" t="n"/>
-      <c r="E37" s="1263" t="n"/>
-      <c r="F37" s="1263" t="n"/>
-      <c r="G37" s="1263" t="n"/>
-      <c r="H37" s="1263" t="n"/>
-      <c r="I37" s="1264" t="n"/>
-      <c r="J37" s="1265" t="n"/>
-      <c r="K37" s="1265" t="n"/>
-      <c r="L37" s="1265" t="n"/>
-      <c r="M37" s="1263" t="n"/>
-      <c r="N37" s="1263" t="n"/>
-      <c r="O37" s="1263" t="n"/>
-      <c r="P37" s="1266" t="n"/>
-      <c r="Q37" s="1263" t="n">
+      <c r="D37" s="1299" t="n"/>
+      <c r="E37" s="1299" t="n"/>
+      <c r="F37" s="1299" t="n"/>
+      <c r="G37" s="1299" t="n"/>
+      <c r="H37" s="1299" t="n"/>
+      <c r="I37" s="1300" t="n"/>
+      <c r="J37" s="1301" t="n"/>
+      <c r="K37" s="1301" t="n"/>
+      <c r="L37" s="1301" t="n"/>
+      <c r="M37" s="1299" t="n"/>
+      <c r="N37" s="1299" t="n"/>
+      <c r="O37" s="1299" t="n"/>
+      <c r="P37" s="1302" t="n"/>
+      <c r="Q37" s="1299" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1263" t="n"/>
-      <c r="S37" s="1263" t="n"/>
+      <c r="R37" s="1299" t="n"/>
+      <c r="S37" s="1299" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1262" t="n"/>
+      <c r="U37" s="1298" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -6464,57 +6590,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1237" t="inlineStr">
+      <c r="A38" s="1273" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1238" t="inlineStr">
+      <c r="B38" s="1274" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1238" t="inlineStr">
+      <c r="C38" s="1274" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1239" t="n"/>
-      <c r="E38" s="1239" t="n">
+      <c r="D38" s="1275" t="n"/>
+      <c r="E38" s="1275" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1239" t="n">
+      <c r="F38" s="1275" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1239" t="n">
+      <c r="G38" s="1275" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1239" t="n"/>
-      <c r="I38" s="1240" t="n">
+      <c r="H38" s="1275" t="n"/>
+      <c r="I38" s="1276" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1241" t="n"/>
-      <c r="K38" s="1241" t="n"/>
-      <c r="L38" s="1241" t="n"/>
-      <c r="M38" s="1239" t="n"/>
-      <c r="N38" s="1239" t="n"/>
-      <c r="O38" s="1239" t="n">
+      <c r="J38" s="1277" t="n"/>
+      <c r="K38" s="1277" t="n"/>
+      <c r="L38" s="1277" t="n"/>
+      <c r="M38" s="1275" t="n"/>
+      <c r="N38" s="1275" t="n"/>
+      <c r="O38" s="1275" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1242" t="n">
+      <c r="P38" s="1278" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1239" t="n"/>
-      <c r="R38" s="1239" t="n">
+      <c r="Q38" s="1275" t="n"/>
+      <c r="R38" s="1275" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1239" t="n"/>
+      <c r="S38" s="1275" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1238" t="inlineStr">
+      <c r="U38" s="1274" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -6526,49 +6652,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1267" t="inlineStr">
+      <c r="A39" s="1303" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1268" t="inlineStr">
+      <c r="B39" s="1304" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1268" t="inlineStr">
+      <c r="C39" s="1304" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1269" t="n"/>
-      <c r="E39" s="1269" t="n"/>
-      <c r="F39" s="1269" t="n"/>
-      <c r="G39" s="1269" t="n"/>
-      <c r="H39" s="1269" t="n">
+      <c r="D39" s="1305" t="n"/>
+      <c r="E39" s="1305" t="n"/>
+      <c r="F39" s="1305" t="n"/>
+      <c r="G39" s="1305" t="n"/>
+      <c r="H39" s="1305" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1270" t="n"/>
-      <c r="J39" s="1271" t="n"/>
-      <c r="K39" s="1271" t="n"/>
-      <c r="L39" s="1271" t="n"/>
-      <c r="M39" s="1269" t="n">
+      <c r="I39" s="1306" t="n"/>
+      <c r="J39" s="1307" t="n"/>
+      <c r="K39" s="1307" t="n"/>
+      <c r="L39" s="1307" t="n"/>
+      <c r="M39" s="1305" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1269" t="n">
+      <c r="N39" s="1305" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1269" t="n"/>
-      <c r="P39" s="1272" t="n"/>
-      <c r="Q39" s="1269" t="n"/>
-      <c r="R39" s="1269" t="n"/>
-      <c r="S39" s="1269" t="n"/>
+      <c r="O39" s="1305" t="n"/>
+      <c r="P39" s="1308" t="n"/>
+      <c r="Q39" s="1305" t="n"/>
+      <c r="R39" s="1305" t="n"/>
+      <c r="S39" s="1305" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1268" t="n"/>
+      <c r="U39" s="1304" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -6576,41 +6702,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1243" t="inlineStr">
+      <c r="A40" s="1279" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1244" t="inlineStr">
+      <c r="B40" s="1280" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1244" t="inlineStr">
+      <c r="C40" s="1280" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1245" t="n"/>
-      <c r="E40" s="1245" t="n"/>
-      <c r="F40" s="1245" t="n"/>
-      <c r="G40" s="1245" t="n"/>
-      <c r="H40" s="1245" t="n"/>
-      <c r="I40" s="1246" t="n"/>
-      <c r="J40" s="1247" t="n"/>
-      <c r="K40" s="1247" t="n"/>
-      <c r="L40" s="1247" t="n"/>
-      <c r="M40" s="1245" t="n"/>
-      <c r="N40" s="1245" t="n"/>
-      <c r="O40" s="1245" t="n"/>
-      <c r="P40" s="1248" t="n"/>
-      <c r="Q40" s="1245" t="n">
+      <c r="D40" s="1281" t="n"/>
+      <c r="E40" s="1281" t="n"/>
+      <c r="F40" s="1281" t="n"/>
+      <c r="G40" s="1281" t="n"/>
+      <c r="H40" s="1281" t="n"/>
+      <c r="I40" s="1282" t="n"/>
+      <c r="J40" s="1283" t="n"/>
+      <c r="K40" s="1283" t="n"/>
+      <c r="L40" s="1283" t="n"/>
+      <c r="M40" s="1281" t="n"/>
+      <c r="N40" s="1281" t="n"/>
+      <c r="O40" s="1281" t="n"/>
+      <c r="P40" s="1284" t="n"/>
+      <c r="Q40" s="1281" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1245" t="n"/>
-      <c r="S40" s="1245" t="n"/>
+      <c r="R40" s="1281" t="n"/>
+      <c r="S40" s="1281" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1244" t="n"/>
+      <c r="U40" s="1280" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -6618,57 +6744,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1249" t="inlineStr">
+      <c r="A41" s="1285" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1250" t="inlineStr">
+      <c r="B41" s="1286" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1250" t="inlineStr">
+      <c r="C41" s="1286" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1251" t="n"/>
-      <c r="E41" s="1251" t="n">
+      <c r="D41" s="1287" t="n"/>
+      <c r="E41" s="1287" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1251" t="n">
+      <c r="F41" s="1287" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1251" t="n">
+      <c r="G41" s="1287" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1251" t="n"/>
-      <c r="I41" s="1252" t="n">
+      <c r="H41" s="1287" t="n"/>
+      <c r="I41" s="1288" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1253" t="n"/>
-      <c r="K41" s="1253" t="n"/>
-      <c r="L41" s="1253" t="n"/>
-      <c r="M41" s="1251" t="n"/>
-      <c r="N41" s="1251" t="n"/>
-      <c r="O41" s="1251" t="n">
+      <c r="J41" s="1289" t="n"/>
+      <c r="K41" s="1289" t="n"/>
+      <c r="L41" s="1289" t="n"/>
+      <c r="M41" s="1287" t="n"/>
+      <c r="N41" s="1287" t="n"/>
+      <c r="O41" s="1287" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1254" t="n">
+      <c r="P41" s="1290" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1251" t="n"/>
-      <c r="R41" s="1251" t="n">
+      <c r="Q41" s="1287" t="n"/>
+      <c r="R41" s="1287" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1251" t="n"/>
+      <c r="S41" s="1287" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1250" t="inlineStr">
+      <c r="U41" s="1286" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -6680,49 +6806,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1261" t="inlineStr">
+      <c r="A42" s="1297" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1262" t="inlineStr">
+      <c r="B42" s="1298" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1262" t="inlineStr">
+      <c r="C42" s="1298" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1263" t="n"/>
-      <c r="E42" s="1263" t="n"/>
-      <c r="F42" s="1263" t="n"/>
-      <c r="G42" s="1263" t="n"/>
-      <c r="H42" s="1263" t="n">
+      <c r="D42" s="1299" t="n"/>
+      <c r="E42" s="1299" t="n"/>
+      <c r="F42" s="1299" t="n"/>
+      <c r="G42" s="1299" t="n"/>
+      <c r="H42" s="1299" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1264" t="n"/>
-      <c r="J42" s="1265" t="n"/>
-      <c r="K42" s="1265" t="n"/>
-      <c r="L42" s="1265" t="n"/>
-      <c r="M42" s="1263" t="n">
+      <c r="I42" s="1300" t="n"/>
+      <c r="J42" s="1301" t="n"/>
+      <c r="K42" s="1301" t="n"/>
+      <c r="L42" s="1301" t="n"/>
+      <c r="M42" s="1299" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1263" t="n">
+      <c r="N42" s="1299" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1263" t="n"/>
-      <c r="P42" s="1266" t="n"/>
-      <c r="Q42" s="1263" t="n"/>
-      <c r="R42" s="1263" t="n"/>
-      <c r="S42" s="1263" t="n"/>
+      <c r="O42" s="1299" t="n"/>
+      <c r="P42" s="1302" t="n"/>
+      <c r="Q42" s="1299" t="n"/>
+      <c r="R42" s="1299" t="n"/>
+      <c r="S42" s="1299" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1262" t="n"/>
+      <c r="U42" s="1298" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -6730,57 +6856,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1237" t="inlineStr">
+      <c r="A43" s="1273" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1238" t="inlineStr">
+      <c r="B43" s="1274" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1238" t="inlineStr">
+      <c r="C43" s="1274" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1239" t="n"/>
-      <c r="E43" s="1239" t="n">
+      <c r="D43" s="1275" t="n"/>
+      <c r="E43" s="1275" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1239" t="n">
+      <c r="F43" s="1275" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1239" t="n">
+      <c r="G43" s="1275" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1239" t="n"/>
-      <c r="I43" s="1240" t="n">
+      <c r="H43" s="1275" t="n"/>
+      <c r="I43" s="1276" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1241" t="n"/>
-      <c r="K43" s="1241" t="n"/>
-      <c r="L43" s="1241" t="n"/>
-      <c r="M43" s="1239" t="n"/>
-      <c r="N43" s="1239" t="n"/>
-      <c r="O43" s="1239" t="n">
+      <c r="J43" s="1277" t="n"/>
+      <c r="K43" s="1277" t="n"/>
+      <c r="L43" s="1277" t="n"/>
+      <c r="M43" s="1275" t="n"/>
+      <c r="N43" s="1275" t="n"/>
+      <c r="O43" s="1275" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1242" t="n">
+      <c r="P43" s="1278" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1239" t="n"/>
-      <c r="R43" s="1239" t="n">
+      <c r="Q43" s="1275" t="n"/>
+      <c r="R43" s="1275" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1239" t="n"/>
+      <c r="S43" s="1275" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1238" t="n"/>
+      <c r="U43" s="1274" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -6788,45 +6914,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1267" t="inlineStr">
+      <c r="A44" s="1303" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1268" t="inlineStr">
+      <c r="B44" s="1304" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1268" t="inlineStr">
+      <c r="C44" s="1304" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1269" t="n"/>
-      <c r="E44" s="1269" t="n">
+      <c r="D44" s="1305" t="n"/>
+      <c r="E44" s="1305" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1269" t="n">
+      <c r="F44" s="1305" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1269" t="n"/>
-      <c r="H44" s="1269" t="n"/>
-      <c r="I44" s="1270" t="n"/>
-      <c r="J44" s="1271" t="n"/>
-      <c r="K44" s="1271" t="n"/>
-      <c r="L44" s="1271" t="n"/>
-      <c r="M44" s="1269" t="n"/>
-      <c r="N44" s="1269" t="n"/>
-      <c r="O44" s="1269" t="n"/>
-      <c r="P44" s="1272" t="n"/>
-      <c r="Q44" s="1269" t="n"/>
-      <c r="R44" s="1269" t="n"/>
-      <c r="S44" s="1269" t="n">
+      <c r="G44" s="1305" t="n"/>
+      <c r="H44" s="1305" t="n"/>
+      <c r="I44" s="1306" t="n"/>
+      <c r="J44" s="1307" t="n"/>
+      <c r="K44" s="1307" t="n"/>
+      <c r="L44" s="1307" t="n"/>
+      <c r="M44" s="1305" t="n"/>
+      <c r="N44" s="1305" t="n"/>
+      <c r="O44" s="1305" t="n"/>
+      <c r="P44" s="1308" t="n"/>
+      <c r="Q44" s="1305" t="n"/>
+      <c r="R44" s="1305" t="n"/>
+      <c r="S44" s="1305" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1268" t="inlineStr">
+      <c r="U44" s="1304" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -6838,49 +6964,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1267" t="inlineStr">
+      <c r="A45" s="1303" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1268" t="inlineStr">
+      <c r="B45" s="1304" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1268" t="inlineStr">
+      <c r="C45" s="1304" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1269" t="n"/>
-      <c r="E45" s="1269" t="n"/>
-      <c r="F45" s="1269" t="n"/>
-      <c r="G45" s="1269" t="n"/>
-      <c r="H45" s="1269" t="n">
+      <c r="D45" s="1305" t="n"/>
+      <c r="E45" s="1305" t="n"/>
+      <c r="F45" s="1305" t="n"/>
+      <c r="G45" s="1305" t="n"/>
+      <c r="H45" s="1305" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1270" t="n"/>
-      <c r="J45" s="1271" t="n"/>
-      <c r="K45" s="1271" t="n"/>
-      <c r="L45" s="1271" t="n"/>
-      <c r="M45" s="1269" t="n">
+      <c r="I45" s="1306" t="n"/>
+      <c r="J45" s="1307" t="n"/>
+      <c r="K45" s="1307" t="n"/>
+      <c r="L45" s="1307" t="n"/>
+      <c r="M45" s="1305" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1269" t="n">
+      <c r="N45" s="1305" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1269" t="n"/>
-      <c r="P45" s="1272" t="n"/>
-      <c r="Q45" s="1269" t="n"/>
-      <c r="R45" s="1269" t="n"/>
-      <c r="S45" s="1269" t="n"/>
+      <c r="O45" s="1305" t="n"/>
+      <c r="P45" s="1308" t="n"/>
+      <c r="Q45" s="1305" t="n"/>
+      <c r="R45" s="1305" t="n"/>
+      <c r="S45" s="1305" t="n"/>
       <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1268" t="n"/>
+      <c r="U45" s="1304" t="n"/>
       <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -6888,39 +7014,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1243" t="inlineStr">
+      <c r="A46" s="1279" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B46" s="1244" t="inlineStr">
+      <c r="B46" s="1280" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="C46" s="1244" t="inlineStr">
+      <c r="C46" s="1280" t="inlineStr">
         <is>
           <t>EVENT - Clean</t>
         </is>
       </c>
-      <c r="D46" s="1245" t="n"/>
-      <c r="E46" s="1245" t="n"/>
-      <c r="F46" s="1245" t="n"/>
-      <c r="G46" s="1245" t="n"/>
-      <c r="H46" s="1245" t="n"/>
-      <c r="I46" s="1246" t="n"/>
-      <c r="J46" s="1247" t="n"/>
-      <c r="K46" s="1247" t="n"/>
-      <c r="L46" s="1247" t="n"/>
-      <c r="M46" s="1245" t="n"/>
-      <c r="N46" s="1245" t="n"/>
-      <c r="O46" s="1245" t="n"/>
-      <c r="P46" s="1248" t="n"/>
-      <c r="Q46" s="1245" t="n"/>
-      <c r="R46" s="1245" t="n"/>
-      <c r="S46" s="1245" t="n"/>
+      <c r="D46" s="1281" t="n"/>
+      <c r="E46" s="1281" t="n"/>
+      <c r="F46" s="1281" t="n"/>
+      <c r="G46" s="1281" t="n"/>
+      <c r="H46" s="1281" t="n"/>
+      <c r="I46" s="1282" t="n"/>
+      <c r="J46" s="1283" t="n"/>
+      <c r="K46" s="1283" t="n"/>
+      <c r="L46" s="1283" t="n"/>
+      <c r="M46" s="1281" t="n"/>
+      <c r="N46" s="1281" t="n"/>
+      <c r="O46" s="1281" t="n"/>
+      <c r="P46" s="1284" t="n"/>
+      <c r="Q46" s="1281" t="n"/>
+      <c r="R46" s="1281" t="n"/>
+      <c r="S46" s="1281" t="n"/>
       <c r="T46" s="631" t="n"/>
-      <c r="U46" s="1244" t="n"/>
+      <c r="U46" s="1280" t="n"/>
       <c r="V46" s="632" t="inlineStr">
         <is>
           <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
@@ -6928,51 +7054,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1249" t="inlineStr">
+      <c r="A47" s="1285" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1250" t="inlineStr">
+      <c r="B47" s="1286" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C47" s="1250" t="inlineStr">
+      <c r="C47" s="1286" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D47" s="1251" t="n"/>
-      <c r="E47" s="1251" t="n">
+      <c r="D47" s="1287" t="n"/>
+      <c r="E47" s="1287" t="n">
         <v>16.6</v>
       </c>
-      <c r="F47" s="1251" t="n">
+      <c r="F47" s="1287" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="1251" t="n">
+      <c r="G47" s="1287" t="n">
         <v>4.1</v>
       </c>
-      <c r="H47" s="1251" t="n"/>
-      <c r="I47" s="1252" t="n">
+      <c r="H47" s="1287" t="n"/>
+      <c r="I47" s="1288" t="n">
         <v>0.9</v>
       </c>
-      <c r="J47" s="1253" t="n"/>
-      <c r="K47" s="1253" t="n"/>
-      <c r="L47" s="1253" t="n"/>
-      <c r="M47" s="1251" t="n"/>
-      <c r="N47" s="1251" t="n"/>
-      <c r="O47" s="1251" t="n">
+      <c r="J47" s="1289" t="n"/>
+      <c r="K47" s="1289" t="n"/>
+      <c r="L47" s="1289" t="n"/>
+      <c r="M47" s="1287" t="n"/>
+      <c r="N47" s="1287" t="n"/>
+      <c r="O47" s="1287" t="n">
         <v>13.2</v>
       </c>
-      <c r="P47" s="1254" t="n">
+      <c r="P47" s="1290" t="n">
         <v>0</v>
       </c>
-      <c r="Q47" s="1251" t="n"/>
-      <c r="R47" s="1251" t="n">
+      <c r="Q47" s="1287" t="n"/>
+      <c r="R47" s="1287" t="n">
         <v>84.5</v>
       </c>
-      <c r="S47" s="1251" t="n">
+      <c r="S47" s="1287" t="n">
         <v>11.8</v>
       </c>
       <c r="T47" s="813" t="inlineStr">
@@ -6980,7 +7106,7 @@
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1250" t="inlineStr">
+      <c r="U47" s="1286" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
@@ -6992,52 +7118,112 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1261" t="inlineStr">
+      <c r="A48" s="1297" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B48" s="1262" t="inlineStr">
+      <c r="B48" s="1298" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C48" s="1262" t="inlineStr">
+      <c r="C48" s="1298" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D48" s="1263" t="n"/>
-      <c r="E48" s="1263" t="n"/>
-      <c r="F48" s="1263" t="n"/>
-      <c r="G48" s="1263" t="n"/>
-      <c r="H48" s="1263" t="n">
+      <c r="D48" s="1299" t="n"/>
+      <c r="E48" s="1299" t="n"/>
+      <c r="F48" s="1299" t="n"/>
+      <c r="G48" s="1299" t="n"/>
+      <c r="H48" s="1299" t="n">
         <v>15.1</v>
       </c>
-      <c r="I48" s="1264" t="n"/>
-      <c r="J48" s="1265" t="n"/>
-      <c r="K48" s="1265" t="n"/>
-      <c r="L48" s="1265" t="n"/>
-      <c r="M48" s="1263" t="n">
+      <c r="I48" s="1300" t="n"/>
+      <c r="J48" s="1301" t="n"/>
+      <c r="K48" s="1301" t="n"/>
+      <c r="L48" s="1301" t="n"/>
+      <c r="M48" s="1299" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="1263" t="n">
+      <c r="N48" s="1299" t="n">
         <v>20</v>
       </c>
-      <c r="O48" s="1263" t="n"/>
-      <c r="P48" s="1266" t="n"/>
-      <c r="Q48" s="1263" t="n"/>
-      <c r="R48" s="1263" t="n"/>
-      <c r="S48" s="1263" t="n"/>
+      <c r="O48" s="1299" t="n"/>
+      <c r="P48" s="1302" t="n"/>
+      <c r="Q48" s="1299" t="n"/>
+      <c r="R48" s="1299" t="n"/>
+      <c r="S48" s="1299" t="n"/>
       <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U48" s="1262" t="n"/>
+      <c r="U48" s="1298" t="n"/>
       <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="1309" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B49" s="1310" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="C49" s="1310" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="D49" s="1311" t="n"/>
+      <c r="E49" s="1311" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="F49" s="1311" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G49" s="1311" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="H49" s="1311" t="n"/>
+      <c r="I49" s="1312" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J49" s="1313" t="n"/>
+      <c r="K49" s="1313" t="n"/>
+      <c r="L49" s="1313" t="n"/>
+      <c r="M49" s="1311" t="n"/>
+      <c r="N49" s="1311" t="n"/>
+      <c r="O49" s="1311" t="n">
+        <v>13</v>
+      </c>
+      <c r="P49" s="1314" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="Q49" s="1311" t="n"/>
+      <c r="R49" s="1311" t="n">
+        <v>86</v>
+      </c>
+      <c r="S49" s="1311" t="n">
+        <v>11.65</v>
+      </c>
+      <c r="T49" s="1047" t="inlineStr">
+        <is>
+          <t>Clear now, 88F, 67% RH; sun so far 6.4h of 7h daylight (91%); today high 90F, 0.87in precip, UV max 7.9</t>
+        </is>
+      </c>
+      <c r="U49" s="1310" t="n"/>
+      <c r="V49" s="1048" t="inlineStr">
+        <is>
+          <t>25mL x0.2. FC 16.8, CC 0.2. CC CREEP CLEARED: 0.0-&gt;0.4-&gt;0.6-&gt;0.2 -- confirms the benign explanation (floating debris + 7/2 Magic Eraser residue), oxidized away by the high FC. Auto weather bucket said 'rain' (0.87in daily precip, likely the incoming 7/6 system's leading edge) but midday was clearly sunny (91% sun so far) -&gt; overrode to sunny for the loss model. fc_loss 3.3 ppm/24h (16.6 + 1.0gal x3.5 - 16.8), clean noon-to-noon (no recheck yesterday). PREDICTION RESOLVED: pred error +1.7 (actual 16.8 vs 7/3 dose's 15.1) = THIRD straight hot-day over-prediction (+2.1, +0.9, +1.7); the clean case -- landed high DESPITE today's extra CC-clearing demand. Actual hot-day losses ran ~2.9/4.1/3.3 (avg ~3.4), not the modeled 5.0. -&gt; Recalibrated dose.py l24_hot_sunny 5.0-&gt;4.0 (small cushion above the 3.4 mean). Water level 11.65 cm (11.9-&gt;11.8-&gt;11.65: steady slow evaporation decline over 3 hot dry days, ~0.1/day; the 7/6 rain will reverse it). PARTY PREP (Sun 7/5 1PM): recommending only 0.5 gal tonight -- FC already high at 16.8 and tomorrow's cooler/drizzly, so a full gal would overshoot into the high teens (John: don't go overboard). 0.5 gal -&gt; ~15-16 at party = comfortable top-of-band with cushion for bather load, not overboard.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log 2026-07-04 evening: party pre-load 0.5 gal @ 7:40pm (season 20.5), add 4 photos
Half the usual dose to avoid overshooting FC into the high teens before
the 7/5 party. Water clear/healthy, debris cleared, no stain progression.
Model projects 14.6 but storm-overnight means real loss is lower -> flagged
tomorrow's likely "high" reading as a weather mismatch, not the retune.
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1315">
+  <cellXfs count="1351">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -4472,6 +4472,114 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4733,7 +4841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V49"/>
+  <dimension ref="A1:V50"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -4910,35 +5018,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1273" t="inlineStr">
+      <c r="A3" s="1315" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1274" t="n"/>
-      <c r="C3" s="1274" t="inlineStr">
+      <c r="B3" s="1316" t="n"/>
+      <c r="C3" s="1316" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1275" t="n"/>
-      <c r="E3" s="1275" t="n"/>
-      <c r="F3" s="1275" t="n"/>
-      <c r="G3" s="1275" t="n"/>
-      <c r="H3" s="1275" t="n"/>
-      <c r="I3" s="1276" t="n"/>
-      <c r="J3" s="1277" t="n"/>
-      <c r="K3" s="1277" t="n"/>
-      <c r="L3" s="1277" t="n"/>
-      <c r="M3" s="1275" t="n"/>
-      <c r="N3" s="1275" t="n"/>
-      <c r="O3" s="1275" t="n"/>
-      <c r="P3" s="1278" t="n"/>
-      <c r="Q3" s="1275" t="n"/>
-      <c r="R3" s="1275" t="n"/>
-      <c r="S3" s="1275" t="n"/>
+      <c r="D3" s="1317" t="n"/>
+      <c r="E3" s="1317" t="n"/>
+      <c r="F3" s="1317" t="n"/>
+      <c r="G3" s="1317" t="n"/>
+      <c r="H3" s="1317" t="n"/>
+      <c r="I3" s="1318" t="n"/>
+      <c r="J3" s="1319" t="n"/>
+      <c r="K3" s="1319" t="n"/>
+      <c r="L3" s="1319" t="n"/>
+      <c r="M3" s="1317" t="n"/>
+      <c r="N3" s="1317" t="n"/>
+      <c r="O3" s="1317" t="n"/>
+      <c r="P3" s="1320" t="n"/>
+      <c r="Q3" s="1317" t="n"/>
+      <c r="R3" s="1317" t="n"/>
+      <c r="S3" s="1317" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1274" t="n"/>
+      <c r="U3" s="1316" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -4946,43 +5054,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1279" t="inlineStr">
+      <c r="A4" s="1321" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1280" t="inlineStr">
+      <c r="B4" s="1322" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1280" t="inlineStr">
+      <c r="C4" s="1322" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1281" t="n"/>
-      <c r="E4" s="1281" t="n"/>
-      <c r="F4" s="1281" t="n"/>
-      <c r="G4" s="1281" t="n"/>
-      <c r="H4" s="1281" t="n"/>
-      <c r="I4" s="1282" t="n"/>
-      <c r="J4" s="1283" t="n"/>
-      <c r="K4" s="1283" t="n"/>
-      <c r="L4" s="1283" t="n"/>
-      <c r="M4" s="1281" t="n">
+      <c r="D4" s="1323" t="n"/>
+      <c r="E4" s="1323" t="n"/>
+      <c r="F4" s="1323" t="n"/>
+      <c r="G4" s="1323" t="n"/>
+      <c r="H4" s="1323" t="n"/>
+      <c r="I4" s="1324" t="n"/>
+      <c r="J4" s="1325" t="n"/>
+      <c r="K4" s="1325" t="n"/>
+      <c r="L4" s="1325" t="n"/>
+      <c r="M4" s="1323" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1281" t="n">
+      <c r="N4" s="1323" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1281" t="n"/>
-      <c r="P4" s="1284" t="n"/>
-      <c r="Q4" s="1281" t="n"/>
-      <c r="R4" s="1281" t="n"/>
-      <c r="S4" s="1281" t="n"/>
+      <c r="O4" s="1323" t="n"/>
+      <c r="P4" s="1326" t="n"/>
+      <c r="Q4" s="1323" t="n"/>
+      <c r="R4" s="1323" t="n"/>
+      <c r="S4" s="1323" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1280" t="n"/>
+      <c r="U4" s="1322" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -4990,57 +5098,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1285" t="inlineStr">
+      <c r="A5" s="1327" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1286" t="inlineStr">
+      <c r="B5" s="1328" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1286" t="inlineStr">
+      <c r="C5" s="1328" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1287" t="n">
+      <c r="D5" s="1329" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1287" t="n">
+      <c r="E5" s="1329" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1287" t="n">
+      <c r="F5" s="1329" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1287" t="n"/>
-      <c r="H5" s="1287" t="n"/>
-      <c r="I5" s="1288" t="n"/>
-      <c r="J5" s="1289" t="n">
+      <c r="G5" s="1329" t="n"/>
+      <c r="H5" s="1329" t="n"/>
+      <c r="I5" s="1330" t="n"/>
+      <c r="J5" s="1331" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1289" t="n">
+      <c r="K5" s="1331" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1289" t="inlineStr">
+      <c r="L5" s="1331" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1287" t="n"/>
-      <c r="N5" s="1287" t="n"/>
-      <c r="O5" s="1287" t="n">
+      <c r="M5" s="1329" t="n"/>
+      <c r="N5" s="1329" t="n"/>
+      <c r="O5" s="1329" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1290" t="n">
+      <c r="P5" s="1332" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1287" t="n"/>
-      <c r="R5" s="1287" t="n"/>
-      <c r="S5" s="1287" t="n"/>
+      <c r="Q5" s="1329" t="n"/>
+      <c r="R5" s="1329" t="n"/>
+      <c r="S5" s="1329" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1286" t="n"/>
+      <c r="U5" s="1328" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -5048,43 +5156,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1291" t="inlineStr">
+      <c r="A6" s="1333" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1292" t="inlineStr">
+      <c r="B6" s="1334" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1292" t="inlineStr">
+      <c r="C6" s="1334" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1293" t="n"/>
-      <c r="E6" s="1293" t="n"/>
-      <c r="F6" s="1293" t="n"/>
-      <c r="G6" s="1293" t="n"/>
-      <c r="H6" s="1293" t="n"/>
-      <c r="I6" s="1294" t="n"/>
-      <c r="J6" s="1295" t="n"/>
-      <c r="K6" s="1295" t="n"/>
-      <c r="L6" s="1295" t="n"/>
-      <c r="M6" s="1293" t="n">
+      <c r="D6" s="1335" t="n"/>
+      <c r="E6" s="1335" t="n"/>
+      <c r="F6" s="1335" t="n"/>
+      <c r="G6" s="1335" t="n"/>
+      <c r="H6" s="1335" t="n"/>
+      <c r="I6" s="1336" t="n"/>
+      <c r="J6" s="1337" t="n"/>
+      <c r="K6" s="1337" t="n"/>
+      <c r="L6" s="1337" t="n"/>
+      <c r="M6" s="1335" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1293" t="n">
+      <c r="N6" s="1335" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1293" t="n"/>
-      <c r="P6" s="1296" t="n"/>
-      <c r="Q6" s="1293" t="n"/>
-      <c r="R6" s="1293" t="n"/>
-      <c r="S6" s="1293" t="n"/>
+      <c r="O6" s="1335" t="n"/>
+      <c r="P6" s="1338" t="n"/>
+      <c r="Q6" s="1335" t="n"/>
+      <c r="R6" s="1335" t="n"/>
+      <c r="S6" s="1335" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1292" t="n"/>
+      <c r="U6" s="1334" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -5092,39 +5200,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1297" t="inlineStr">
+      <c r="A7" s="1339" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1298" t="inlineStr">
+      <c r="B7" s="1340" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1298" t="inlineStr">
+      <c r="C7" s="1340" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1299" t="n"/>
-      <c r="E7" s="1299" t="n"/>
-      <c r="F7" s="1299" t="n"/>
-      <c r="G7" s="1299" t="n"/>
-      <c r="H7" s="1299" t="n"/>
-      <c r="I7" s="1300" t="n"/>
-      <c r="J7" s="1301" t="n"/>
-      <c r="K7" s="1301" t="n"/>
-      <c r="L7" s="1301" t="n"/>
-      <c r="M7" s="1299" t="n"/>
-      <c r="N7" s="1299" t="n"/>
-      <c r="O7" s="1299" t="n"/>
-      <c r="P7" s="1302" t="n"/>
-      <c r="Q7" s="1299" t="n"/>
-      <c r="R7" s="1299" t="n"/>
-      <c r="S7" s="1299" t="n"/>
+      <c r="D7" s="1341" t="n"/>
+      <c r="E7" s="1341" t="n"/>
+      <c r="F7" s="1341" t="n"/>
+      <c r="G7" s="1341" t="n"/>
+      <c r="H7" s="1341" t="n"/>
+      <c r="I7" s="1342" t="n"/>
+      <c r="J7" s="1343" t="n"/>
+      <c r="K7" s="1343" t="n"/>
+      <c r="L7" s="1343" t="n"/>
+      <c r="M7" s="1341" t="n"/>
+      <c r="N7" s="1341" t="n"/>
+      <c r="O7" s="1341" t="n"/>
+      <c r="P7" s="1344" t="n"/>
+      <c r="Q7" s="1341" t="n"/>
+      <c r="R7" s="1341" t="n"/>
+      <c r="S7" s="1341" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1298" t="n"/>
+      <c r="U7" s="1340" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5132,39 +5240,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1273" t="inlineStr">
+      <c r="A8" s="1315" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1274" t="inlineStr">
+      <c r="B8" s="1316" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1274" t="inlineStr">
+      <c r="C8" s="1316" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1275" t="n"/>
-      <c r="E8" s="1275" t="n"/>
-      <c r="F8" s="1275" t="n"/>
-      <c r="G8" s="1275" t="n"/>
-      <c r="H8" s="1275" t="n"/>
-      <c r="I8" s="1276" t="n"/>
-      <c r="J8" s="1277" t="n"/>
-      <c r="K8" s="1277" t="n"/>
-      <c r="L8" s="1277" t="n"/>
-      <c r="M8" s="1275" t="n"/>
-      <c r="N8" s="1275" t="n"/>
-      <c r="O8" s="1275" t="n"/>
-      <c r="P8" s="1278" t="n"/>
-      <c r="Q8" s="1275" t="n"/>
-      <c r="R8" s="1275" t="n"/>
-      <c r="S8" s="1275" t="n"/>
+      <c r="D8" s="1317" t="n"/>
+      <c r="E8" s="1317" t="n"/>
+      <c r="F8" s="1317" t="n"/>
+      <c r="G8" s="1317" t="n"/>
+      <c r="H8" s="1317" t="n"/>
+      <c r="I8" s="1318" t="n"/>
+      <c r="J8" s="1319" t="n"/>
+      <c r="K8" s="1319" t="n"/>
+      <c r="L8" s="1319" t="n"/>
+      <c r="M8" s="1317" t="n"/>
+      <c r="N8" s="1317" t="n"/>
+      <c r="O8" s="1317" t="n"/>
+      <c r="P8" s="1320" t="n"/>
+      <c r="Q8" s="1317" t="n"/>
+      <c r="R8" s="1317" t="n"/>
+      <c r="S8" s="1317" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1274" t="n"/>
+      <c r="U8" s="1316" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -5172,63 +5280,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1303" t="inlineStr">
+      <c r="A9" s="1345" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1304" t="inlineStr">
+      <c r="B9" s="1346" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1304" t="inlineStr">
+      <c r="C9" s="1346" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1305" t="n">
+      <c r="D9" s="1347" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1305" t="n">
+      <c r="E9" s="1347" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1305" t="n">
+      <c r="F9" s="1347" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1305" t="n">
+      <c r="G9" s="1347" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1305" t="n"/>
-      <c r="I9" s="1306" t="n"/>
-      <c r="J9" s="1307" t="n">
+      <c r="H9" s="1347" t="n"/>
+      <c r="I9" s="1348" t="n"/>
+      <c r="J9" s="1349" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1307" t="n">
+      <c r="K9" s="1349" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1307" t="inlineStr">
+      <c r="L9" s="1349" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1305" t="n"/>
-      <c r="N9" s="1305" t="n"/>
-      <c r="O9" s="1305" t="n">
+      <c r="M9" s="1347" t="n"/>
+      <c r="N9" s="1347" t="n"/>
+      <c r="O9" s="1347" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1308" t="n">
+      <c r="P9" s="1350" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1305" t="n"/>
-      <c r="R9" s="1305" t="n"/>
-      <c r="S9" s="1305" t="n"/>
+      <c r="Q9" s="1347" t="n"/>
+      <c r="R9" s="1347" t="n"/>
+      <c r="S9" s="1347" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1304" t="n"/>
+      <c r="U9" s="1346" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -5236,43 +5344,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1303" t="inlineStr">
+      <c r="A10" s="1345" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1304" t="inlineStr">
+      <c r="B10" s="1346" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1304" t="inlineStr">
+      <c r="C10" s="1346" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1305" t="n"/>
-      <c r="E10" s="1305" t="n"/>
-      <c r="F10" s="1305" t="n"/>
-      <c r="G10" s="1305" t="n"/>
-      <c r="H10" s="1305" t="n"/>
-      <c r="I10" s="1306" t="n"/>
-      <c r="J10" s="1307" t="n"/>
-      <c r="K10" s="1307" t="n"/>
-      <c r="L10" s="1307" t="inlineStr">
+      <c r="D10" s="1347" t="n"/>
+      <c r="E10" s="1347" t="n"/>
+      <c r="F10" s="1347" t="n"/>
+      <c r="G10" s="1347" t="n"/>
+      <c r="H10" s="1347" t="n"/>
+      <c r="I10" s="1348" t="n"/>
+      <c r="J10" s="1349" t="n"/>
+      <c r="K10" s="1349" t="n"/>
+      <c r="L10" s="1349" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1305" t="n"/>
-      <c r="N10" s="1305" t="n"/>
-      <c r="O10" s="1305" t="n"/>
-      <c r="P10" s="1308" t="n"/>
-      <c r="Q10" s="1305" t="n"/>
-      <c r="R10" s="1305" t="n"/>
-      <c r="S10" s="1305" t="n"/>
+      <c r="M10" s="1347" t="n"/>
+      <c r="N10" s="1347" t="n"/>
+      <c r="O10" s="1347" t="n"/>
+      <c r="P10" s="1350" t="n"/>
+      <c r="Q10" s="1347" t="n"/>
+      <c r="R10" s="1347" t="n"/>
+      <c r="S10" s="1347" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1304" t="n"/>
+      <c r="U10" s="1346" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -5280,43 +5388,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1303" t="inlineStr">
+      <c r="A11" s="1345" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1304" t="inlineStr">
+      <c r="B11" s="1346" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1304" t="inlineStr">
+      <c r="C11" s="1346" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1305" t="n"/>
-      <c r="E11" s="1305" t="n"/>
-      <c r="F11" s="1305" t="n"/>
-      <c r="G11" s="1305" t="n"/>
-      <c r="H11" s="1305" t="n"/>
-      <c r="I11" s="1306" t="n"/>
-      <c r="J11" s="1307" t="n"/>
-      <c r="K11" s="1307" t="n"/>
-      <c r="L11" s="1307" t="n"/>
-      <c r="M11" s="1305" t="n">
+      <c r="D11" s="1347" t="n"/>
+      <c r="E11" s="1347" t="n"/>
+      <c r="F11" s="1347" t="n"/>
+      <c r="G11" s="1347" t="n"/>
+      <c r="H11" s="1347" t="n"/>
+      <c r="I11" s="1348" t="n"/>
+      <c r="J11" s="1349" t="n"/>
+      <c r="K11" s="1349" t="n"/>
+      <c r="L11" s="1349" t="n"/>
+      <c r="M11" s="1347" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1305" t="n">
+      <c r="N11" s="1347" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1305" t="n"/>
-      <c r="P11" s="1308" t="n"/>
-      <c r="Q11" s="1305" t="n"/>
-      <c r="R11" s="1305" t="n"/>
-      <c r="S11" s="1305" t="n"/>
+      <c r="O11" s="1347" t="n"/>
+      <c r="P11" s="1350" t="n"/>
+      <c r="Q11" s="1347" t="n"/>
+      <c r="R11" s="1347" t="n"/>
+      <c r="S11" s="1347" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1304" t="n"/>
+      <c r="U11" s="1346" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -5324,39 +5432,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1279" t="inlineStr">
+      <c r="A12" s="1321" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1280" t="inlineStr">
+      <c r="B12" s="1322" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1280" t="inlineStr">
+      <c r="C12" s="1322" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1281" t="n"/>
-      <c r="E12" s="1281" t="n"/>
-      <c r="F12" s="1281" t="n"/>
-      <c r="G12" s="1281" t="n"/>
-      <c r="H12" s="1281" t="n"/>
-      <c r="I12" s="1282" t="n"/>
-      <c r="J12" s="1283" t="n"/>
-      <c r="K12" s="1283" t="n"/>
-      <c r="L12" s="1283" t="n"/>
-      <c r="M12" s="1281" t="n"/>
-      <c r="N12" s="1281" t="n"/>
-      <c r="O12" s="1281" t="n"/>
-      <c r="P12" s="1284" t="n"/>
-      <c r="Q12" s="1281" t="n"/>
-      <c r="R12" s="1281" t="n"/>
-      <c r="S12" s="1281" t="n"/>
+      <c r="D12" s="1323" t="n"/>
+      <c r="E12" s="1323" t="n"/>
+      <c r="F12" s="1323" t="n"/>
+      <c r="G12" s="1323" t="n"/>
+      <c r="H12" s="1323" t="n"/>
+      <c r="I12" s="1324" t="n"/>
+      <c r="J12" s="1325" t="n"/>
+      <c r="K12" s="1325" t="n"/>
+      <c r="L12" s="1325" t="n"/>
+      <c r="M12" s="1323" t="n"/>
+      <c r="N12" s="1323" t="n"/>
+      <c r="O12" s="1323" t="n"/>
+      <c r="P12" s="1326" t="n"/>
+      <c r="Q12" s="1323" t="n"/>
+      <c r="R12" s="1323" t="n"/>
+      <c r="S12" s="1323" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1280" t="n"/>
+      <c r="U12" s="1322" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5364,35 +5472,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1285" t="inlineStr">
+      <c r="A13" s="1327" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1286" t="n"/>
-      <c r="C13" s="1286" t="inlineStr">
+      <c r="B13" s="1328" t="n"/>
+      <c r="C13" s="1328" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1287" t="n"/>
-      <c r="E13" s="1287" t="n"/>
-      <c r="F13" s="1287" t="n"/>
-      <c r="G13" s="1287" t="n"/>
-      <c r="H13" s="1287" t="n"/>
-      <c r="I13" s="1288" t="n"/>
-      <c r="J13" s="1289" t="n"/>
-      <c r="K13" s="1289" t="n"/>
-      <c r="L13" s="1289" t="n"/>
-      <c r="M13" s="1287" t="n"/>
-      <c r="N13" s="1287" t="n"/>
-      <c r="O13" s="1287" t="n"/>
-      <c r="P13" s="1290" t="n"/>
-      <c r="Q13" s="1287" t="n"/>
-      <c r="R13" s="1287" t="n"/>
-      <c r="S13" s="1287" t="n"/>
+      <c r="D13" s="1329" t="n"/>
+      <c r="E13" s="1329" t="n"/>
+      <c r="F13" s="1329" t="n"/>
+      <c r="G13" s="1329" t="n"/>
+      <c r="H13" s="1329" t="n"/>
+      <c r="I13" s="1330" t="n"/>
+      <c r="J13" s="1331" t="n"/>
+      <c r="K13" s="1331" t="n"/>
+      <c r="L13" s="1331" t="n"/>
+      <c r="M13" s="1329" t="n"/>
+      <c r="N13" s="1329" t="n"/>
+      <c r="O13" s="1329" t="n"/>
+      <c r="P13" s="1332" t="n"/>
+      <c r="Q13" s="1329" t="n"/>
+      <c r="R13" s="1329" t="n"/>
+      <c r="S13" s="1329" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1286" t="n"/>
+      <c r="U13" s="1328" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -5400,53 +5508,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1291" t="inlineStr">
+      <c r="A14" s="1333" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1292" t="inlineStr">
+      <c r="B14" s="1334" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1292" t="inlineStr">
+      <c r="C14" s="1334" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1293" t="n"/>
-      <c r="E14" s="1293" t="n">
+      <c r="D14" s="1335" t="n"/>
+      <c r="E14" s="1335" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1293" t="n">
+      <c r="F14" s="1335" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1293" t="n">
+      <c r="G14" s="1335" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1293" t="n"/>
-      <c r="I14" s="1294" t="n"/>
-      <c r="J14" s="1295" t="n"/>
-      <c r="K14" s="1295" t="n"/>
-      <c r="L14" s="1295" t="n"/>
-      <c r="M14" s="1293" t="n"/>
-      <c r="N14" s="1293" t="n"/>
-      <c r="O14" s="1293" t="n">
+      <c r="H14" s="1335" t="n"/>
+      <c r="I14" s="1336" t="n"/>
+      <c r="J14" s="1337" t="n"/>
+      <c r="K14" s="1337" t="n"/>
+      <c r="L14" s="1337" t="n"/>
+      <c r="M14" s="1335" t="n"/>
+      <c r="N14" s="1335" t="n"/>
+      <c r="O14" s="1335" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1296" t="n">
+      <c r="P14" s="1338" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1293" t="n"/>
-      <c r="R14" s="1293" t="n"/>
-      <c r="S14" s="1293" t="n"/>
+      <c r="Q14" s="1335" t="n"/>
+      <c r="R14" s="1335" t="n"/>
+      <c r="S14" s="1335" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1292" t="n"/>
+      <c r="U14" s="1334" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -5454,43 +5562,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1291" t="inlineStr">
+      <c r="A15" s="1333" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1292" t="inlineStr">
+      <c r="B15" s="1334" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1292" t="inlineStr">
+      <c r="C15" s="1334" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1293" t="n"/>
-      <c r="E15" s="1293" t="n"/>
-      <c r="F15" s="1293" t="n"/>
-      <c r="G15" s="1293" t="n"/>
-      <c r="H15" s="1293" t="n"/>
-      <c r="I15" s="1294" t="n"/>
-      <c r="J15" s="1295" t="n"/>
-      <c r="K15" s="1295" t="n"/>
-      <c r="L15" s="1295" t="n"/>
-      <c r="M15" s="1293" t="n">
+      <c r="D15" s="1335" t="n"/>
+      <c r="E15" s="1335" t="n"/>
+      <c r="F15" s="1335" t="n"/>
+      <c r="G15" s="1335" t="n"/>
+      <c r="H15" s="1335" t="n"/>
+      <c r="I15" s="1336" t="n"/>
+      <c r="J15" s="1337" t="n"/>
+      <c r="K15" s="1337" t="n"/>
+      <c r="L15" s="1337" t="n"/>
+      <c r="M15" s="1335" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1293" t="n">
+      <c r="N15" s="1335" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1293" t="n"/>
-      <c r="P15" s="1296" t="n"/>
-      <c r="Q15" s="1293" t="n"/>
-      <c r="R15" s="1293" t="n"/>
-      <c r="S15" s="1293" t="n"/>
+      <c r="O15" s="1335" t="n"/>
+      <c r="P15" s="1338" t="n"/>
+      <c r="Q15" s="1335" t="n"/>
+      <c r="R15" s="1335" t="n"/>
+      <c r="S15" s="1335" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1292" t="n"/>
+      <c r="U15" s="1334" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -5498,39 +5606,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1297" t="inlineStr">
+      <c r="A16" s="1339" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1298" t="inlineStr">
+      <c r="B16" s="1340" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1298" t="inlineStr">
+      <c r="C16" s="1340" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1299" t="n"/>
-      <c r="E16" s="1299" t="n"/>
-      <c r="F16" s="1299" t="n"/>
-      <c r="G16" s="1299" t="n"/>
-      <c r="H16" s="1299" t="n"/>
-      <c r="I16" s="1300" t="n"/>
-      <c r="J16" s="1301" t="n"/>
-      <c r="K16" s="1301" t="n"/>
-      <c r="L16" s="1301" t="n"/>
-      <c r="M16" s="1299" t="n"/>
-      <c r="N16" s="1299" t="n"/>
-      <c r="O16" s="1299" t="n"/>
-      <c r="P16" s="1302" t="n"/>
-      <c r="Q16" s="1299" t="n"/>
-      <c r="R16" s="1299" t="n"/>
-      <c r="S16" s="1299" t="n"/>
+      <c r="D16" s="1341" t="n"/>
+      <c r="E16" s="1341" t="n"/>
+      <c r="F16" s="1341" t="n"/>
+      <c r="G16" s="1341" t="n"/>
+      <c r="H16" s="1341" t="n"/>
+      <c r="I16" s="1342" t="n"/>
+      <c r="J16" s="1343" t="n"/>
+      <c r="K16" s="1343" t="n"/>
+      <c r="L16" s="1343" t="n"/>
+      <c r="M16" s="1341" t="n"/>
+      <c r="N16" s="1341" t="n"/>
+      <c r="O16" s="1341" t="n"/>
+      <c r="P16" s="1344" t="n"/>
+      <c r="Q16" s="1341" t="n"/>
+      <c r="R16" s="1341" t="n"/>
+      <c r="S16" s="1341" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1298" t="n"/>
+      <c r="U16" s="1340" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -5538,39 +5646,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1273" t="inlineStr">
+      <c r="A17" s="1315" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1274" t="inlineStr">
+      <c r="B17" s="1316" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1274" t="inlineStr">
+      <c r="C17" s="1316" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1275" t="n"/>
-      <c r="E17" s="1275" t="n"/>
-      <c r="F17" s="1275" t="n"/>
-      <c r="G17" s="1275" t="n"/>
-      <c r="H17" s="1275" t="n"/>
-      <c r="I17" s="1276" t="n"/>
-      <c r="J17" s="1277" t="n"/>
-      <c r="K17" s="1277" t="n"/>
-      <c r="L17" s="1277" t="n"/>
-      <c r="M17" s="1275" t="n"/>
-      <c r="N17" s="1275" t="n"/>
-      <c r="O17" s="1275" t="n"/>
-      <c r="P17" s="1278" t="n"/>
-      <c r="Q17" s="1275" t="n"/>
-      <c r="R17" s="1275" t="n"/>
-      <c r="S17" s="1275" t="n"/>
+      <c r="D17" s="1317" t="n"/>
+      <c r="E17" s="1317" t="n"/>
+      <c r="F17" s="1317" t="n"/>
+      <c r="G17" s="1317" t="n"/>
+      <c r="H17" s="1317" t="n"/>
+      <c r="I17" s="1318" t="n"/>
+      <c r="J17" s="1319" t="n"/>
+      <c r="K17" s="1319" t="n"/>
+      <c r="L17" s="1319" t="n"/>
+      <c r="M17" s="1317" t="n"/>
+      <c r="N17" s="1317" t="n"/>
+      <c r="O17" s="1317" t="n"/>
+      <c r="P17" s="1320" t="n"/>
+      <c r="Q17" s="1317" t="n"/>
+      <c r="R17" s="1317" t="n"/>
+      <c r="S17" s="1317" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1274" t="n"/>
+      <c r="U17" s="1316" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -5578,53 +5686,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1303" t="inlineStr">
+      <c r="A18" s="1345" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1304" t="inlineStr">
+      <c r="B18" s="1346" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1304" t="inlineStr">
+      <c r="C18" s="1346" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1305" t="n"/>
-      <c r="E18" s="1305" t="n">
+      <c r="D18" s="1347" t="n"/>
+      <c r="E18" s="1347" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1305" t="n">
+      <c r="F18" s="1347" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1305" t="n">
+      <c r="G18" s="1347" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1305" t="n"/>
-      <c r="I18" s="1306" t="n"/>
-      <c r="J18" s="1307" t="n"/>
-      <c r="K18" s="1307" t="n"/>
-      <c r="L18" s="1307" t="n"/>
-      <c r="M18" s="1305" t="n"/>
-      <c r="N18" s="1305" t="n"/>
-      <c r="O18" s="1305" t="n">
+      <c r="H18" s="1347" t="n"/>
+      <c r="I18" s="1348" t="n"/>
+      <c r="J18" s="1349" t="n"/>
+      <c r="K18" s="1349" t="n"/>
+      <c r="L18" s="1349" t="n"/>
+      <c r="M18" s="1347" t="n"/>
+      <c r="N18" s="1347" t="n"/>
+      <c r="O18" s="1347" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1308" t="n">
+      <c r="P18" s="1350" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1305" t="n"/>
-      <c r="R18" s="1305" t="n"/>
-      <c r="S18" s="1305" t="n"/>
+      <c r="Q18" s="1347" t="n"/>
+      <c r="R18" s="1347" t="n"/>
+      <c r="S18" s="1347" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1304" t="n"/>
+      <c r="U18" s="1346" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -5632,47 +5740,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1303" t="inlineStr">
+      <c r="A19" s="1345" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1304" t="inlineStr">
+      <c r="B19" s="1346" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1304" t="inlineStr">
+      <c r="C19" s="1346" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1305" t="n"/>
-      <c r="E19" s="1305" t="n"/>
-      <c r="F19" s="1305" t="n"/>
-      <c r="G19" s="1305" t="n"/>
-      <c r="H19" s="1305" t="n"/>
-      <c r="I19" s="1306" t="n"/>
-      <c r="J19" s="1307" t="n"/>
-      <c r="K19" s="1307" t="n"/>
-      <c r="L19" s="1307" t="n"/>
-      <c r="M19" s="1305" t="n">
+      <c r="D19" s="1347" t="n"/>
+      <c r="E19" s="1347" t="n"/>
+      <c r="F19" s="1347" t="n"/>
+      <c r="G19" s="1347" t="n"/>
+      <c r="H19" s="1347" t="n"/>
+      <c r="I19" s="1348" t="n"/>
+      <c r="J19" s="1349" t="n"/>
+      <c r="K19" s="1349" t="n"/>
+      <c r="L19" s="1349" t="n"/>
+      <c r="M19" s="1347" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1305" t="n">
+      <c r="N19" s="1347" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1305" t="n"/>
-      <c r="P19" s="1308" t="n"/>
-      <c r="Q19" s="1305" t="n"/>
-      <c r="R19" s="1305" t="n"/>
-      <c r="S19" s="1305" t="n"/>
+      <c r="O19" s="1347" t="n"/>
+      <c r="P19" s="1350" t="n"/>
+      <c r="Q19" s="1347" t="n"/>
+      <c r="R19" s="1347" t="n"/>
+      <c r="S19" s="1347" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1304" t="n"/>
+      <c r="U19" s="1346" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -5680,43 +5788,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1303" t="inlineStr">
+      <c r="A20" s="1345" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1304" t="inlineStr">
+      <c r="B20" s="1346" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1304" t="inlineStr">
+      <c r="C20" s="1346" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1305" t="n"/>
-      <c r="E20" s="1305" t="n"/>
-      <c r="F20" s="1305" t="n"/>
-      <c r="G20" s="1305" t="n"/>
-      <c r="H20" s="1305" t="n"/>
-      <c r="I20" s="1306" t="n"/>
-      <c r="J20" s="1307" t="n"/>
-      <c r="K20" s="1307" t="n"/>
-      <c r="L20" s="1307" t="n"/>
-      <c r="M20" s="1305" t="n"/>
-      <c r="N20" s="1305" t="n"/>
-      <c r="O20" s="1305" t="n"/>
-      <c r="P20" s="1308" t="n"/>
-      <c r="Q20" s="1305" t="n"/>
-      <c r="R20" s="1305" t="n"/>
-      <c r="S20" s="1305" t="n"/>
+      <c r="D20" s="1347" t="n"/>
+      <c r="E20" s="1347" t="n"/>
+      <c r="F20" s="1347" t="n"/>
+      <c r="G20" s="1347" t="n"/>
+      <c r="H20" s="1347" t="n"/>
+      <c r="I20" s="1348" t="n"/>
+      <c r="J20" s="1349" t="n"/>
+      <c r="K20" s="1349" t="n"/>
+      <c r="L20" s="1349" t="n"/>
+      <c r="M20" s="1347" t="n"/>
+      <c r="N20" s="1347" t="n"/>
+      <c r="O20" s="1347" t="n"/>
+      <c r="P20" s="1350" t="n"/>
+      <c r="Q20" s="1347" t="n"/>
+      <c r="R20" s="1347" t="n"/>
+      <c r="S20" s="1347" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1304" t="n"/>
+      <c r="U20" s="1346" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -5724,39 +5832,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1279" t="inlineStr">
+      <c r="A21" s="1321" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1280" t="inlineStr">
+      <c r="B21" s="1322" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1280" t="inlineStr">
+      <c r="C21" s="1322" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1281" t="n"/>
-      <c r="E21" s="1281" t="n"/>
-      <c r="F21" s="1281" t="n"/>
-      <c r="G21" s="1281" t="n"/>
-      <c r="H21" s="1281" t="n"/>
-      <c r="I21" s="1282" t="n"/>
-      <c r="J21" s="1283" t="n"/>
-      <c r="K21" s="1283" t="n"/>
-      <c r="L21" s="1283" t="n"/>
-      <c r="M21" s="1281" t="n"/>
-      <c r="N21" s="1281" t="n"/>
-      <c r="O21" s="1281" t="n"/>
-      <c r="P21" s="1284" t="n"/>
-      <c r="Q21" s="1281" t="n"/>
-      <c r="R21" s="1281" t="n"/>
-      <c r="S21" s="1281" t="n"/>
+      <c r="D21" s="1323" t="n"/>
+      <c r="E21" s="1323" t="n"/>
+      <c r="F21" s="1323" t="n"/>
+      <c r="G21" s="1323" t="n"/>
+      <c r="H21" s="1323" t="n"/>
+      <c r="I21" s="1324" t="n"/>
+      <c r="J21" s="1325" t="n"/>
+      <c r="K21" s="1325" t="n"/>
+      <c r="L21" s="1325" t="n"/>
+      <c r="M21" s="1323" t="n"/>
+      <c r="N21" s="1323" t="n"/>
+      <c r="O21" s="1323" t="n"/>
+      <c r="P21" s="1326" t="n"/>
+      <c r="Q21" s="1323" t="n"/>
+      <c r="R21" s="1323" t="n"/>
+      <c r="S21" s="1323" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1280" t="n"/>
+      <c r="U21" s="1322" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -5764,39 +5872,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1285" t="inlineStr">
+      <c r="A22" s="1327" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1286" t="inlineStr">
+      <c r="B22" s="1328" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1286" t="inlineStr">
+      <c r="C22" s="1328" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1287" t="n"/>
-      <c r="E22" s="1287" t="n"/>
-      <c r="F22" s="1287" t="n"/>
-      <c r="G22" s="1287" t="n"/>
-      <c r="H22" s="1287" t="n"/>
-      <c r="I22" s="1288" t="n"/>
-      <c r="J22" s="1289" t="n"/>
-      <c r="K22" s="1289" t="n"/>
-      <c r="L22" s="1289" t="n"/>
-      <c r="M22" s="1287" t="n"/>
-      <c r="N22" s="1287" t="n"/>
-      <c r="O22" s="1287" t="n"/>
-      <c r="P22" s="1290" t="n"/>
-      <c r="Q22" s="1287" t="n"/>
-      <c r="R22" s="1287" t="n"/>
-      <c r="S22" s="1287" t="n"/>
+      <c r="D22" s="1329" t="n"/>
+      <c r="E22" s="1329" t="n"/>
+      <c r="F22" s="1329" t="n"/>
+      <c r="G22" s="1329" t="n"/>
+      <c r="H22" s="1329" t="n"/>
+      <c r="I22" s="1330" t="n"/>
+      <c r="J22" s="1331" t="n"/>
+      <c r="K22" s="1331" t="n"/>
+      <c r="L22" s="1331" t="n"/>
+      <c r="M22" s="1329" t="n"/>
+      <c r="N22" s="1329" t="n"/>
+      <c r="O22" s="1329" t="n"/>
+      <c r="P22" s="1332" t="n"/>
+      <c r="Q22" s="1329" t="n"/>
+      <c r="R22" s="1329" t="n"/>
+      <c r="S22" s="1329" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1286" t="n"/>
+      <c r="U22" s="1328" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -5804,53 +5912,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1291" t="inlineStr">
+      <c r="A23" s="1333" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1292" t="inlineStr">
+      <c r="B23" s="1334" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1292" t="inlineStr">
+      <c r="C23" s="1334" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1293" t="n"/>
-      <c r="E23" s="1293" t="n">
+      <c r="D23" s="1335" t="n"/>
+      <c r="E23" s="1335" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1293" t="n">
+      <c r="F23" s="1335" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1293" t="n">
+      <c r="G23" s="1335" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1293" t="n"/>
-      <c r="I23" s="1294" t="n"/>
-      <c r="J23" s="1295" t="n"/>
-      <c r="K23" s="1295" t="n"/>
-      <c r="L23" s="1295" t="n"/>
-      <c r="M23" s="1293" t="n"/>
-      <c r="N23" s="1293" t="n"/>
-      <c r="O23" s="1293" t="n">
+      <c r="H23" s="1335" t="n"/>
+      <c r="I23" s="1336" t="n"/>
+      <c r="J23" s="1337" t="n"/>
+      <c r="K23" s="1337" t="n"/>
+      <c r="L23" s="1337" t="n"/>
+      <c r="M23" s="1335" t="n"/>
+      <c r="N23" s="1335" t="n"/>
+      <c r="O23" s="1335" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1296" t="n">
+      <c r="P23" s="1338" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1293" t="n"/>
-      <c r="R23" s="1293" t="n"/>
-      <c r="S23" s="1293" t="n"/>
+      <c r="Q23" s="1335" t="n"/>
+      <c r="R23" s="1335" t="n"/>
+      <c r="S23" s="1335" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1292" t="n"/>
+      <c r="U23" s="1334" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -5858,47 +5966,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1297" t="inlineStr">
+      <c r="A24" s="1339" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1298" t="inlineStr">
+      <c r="B24" s="1340" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1298" t="inlineStr">
+      <c r="C24" s="1340" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1299" t="n"/>
-      <c r="E24" s="1299" t="n"/>
-      <c r="F24" s="1299" t="n"/>
-      <c r="G24" s="1299" t="n"/>
-      <c r="H24" s="1299" t="n"/>
-      <c r="I24" s="1300" t="n"/>
-      <c r="J24" s="1301" t="n"/>
-      <c r="K24" s="1301" t="n"/>
-      <c r="L24" s="1301" t="n"/>
-      <c r="M24" s="1299" t="n">
+      <c r="D24" s="1341" t="n"/>
+      <c r="E24" s="1341" t="n"/>
+      <c r="F24" s="1341" t="n"/>
+      <c r="G24" s="1341" t="n"/>
+      <c r="H24" s="1341" t="n"/>
+      <c r="I24" s="1342" t="n"/>
+      <c r="J24" s="1343" t="n"/>
+      <c r="K24" s="1343" t="n"/>
+      <c r="L24" s="1343" t="n"/>
+      <c r="M24" s="1341" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1299" t="n">
+      <c r="N24" s="1341" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1299" t="n"/>
-      <c r="P24" s="1302" t="n"/>
-      <c r="Q24" s="1299" t="n"/>
-      <c r="R24" s="1299" t="n"/>
-      <c r="S24" s="1299" t="n"/>
+      <c r="O24" s="1341" t="n"/>
+      <c r="P24" s="1344" t="n"/>
+      <c r="Q24" s="1341" t="n"/>
+      <c r="R24" s="1341" t="n"/>
+      <c r="S24" s="1341" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1298" t="n"/>
+      <c r="U24" s="1340" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -5906,61 +6014,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1273" t="inlineStr">
+      <c r="A25" s="1315" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1274" t="inlineStr">
+      <c r="B25" s="1316" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1274" t="inlineStr">
+      <c r="C25" s="1316" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1275" t="n">
+      <c r="D25" s="1317" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1275" t="n">
+      <c r="E25" s="1317" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1275" t="n">
+      <c r="F25" s="1317" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1275" t="n">
+      <c r="G25" s="1317" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1275" t="n"/>
-      <c r="I25" s="1276" t="n"/>
-      <c r="J25" s="1277" t="n">
+      <c r="H25" s="1317" t="n"/>
+      <c r="I25" s="1318" t="n"/>
+      <c r="J25" s="1319" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1277" t="n">
+      <c r="K25" s="1319" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1277" t="n">
+      <c r="L25" s="1319" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1275" t="n"/>
-      <c r="N25" s="1275" t="n"/>
-      <c r="O25" s="1275" t="n">
+      <c r="M25" s="1317" t="n"/>
+      <c r="N25" s="1317" t="n"/>
+      <c r="O25" s="1317" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1278" t="n">
+      <c r="P25" s="1320" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1275" t="n"/>
-      <c r="R25" s="1275" t="n"/>
-      <c r="S25" s="1275" t="n"/>
+      <c r="Q25" s="1317" t="n"/>
+      <c r="R25" s="1317" t="n"/>
+      <c r="S25" s="1317" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1274" t="n"/>
+      <c r="U25" s="1316" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -5968,47 +6076,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1279" t="inlineStr">
+      <c r="A26" s="1321" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1280" t="inlineStr">
+      <c r="B26" s="1322" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1280" t="inlineStr">
+      <c r="C26" s="1322" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1281" t="n"/>
-      <c r="E26" s="1281" t="n"/>
-      <c r="F26" s="1281" t="n"/>
-      <c r="G26" s="1281" t="n"/>
-      <c r="H26" s="1281" t="n"/>
-      <c r="I26" s="1282" t="n"/>
-      <c r="J26" s="1283" t="n"/>
-      <c r="K26" s="1283" t="n"/>
-      <c r="L26" s="1283" t="n"/>
-      <c r="M26" s="1281" t="n">
+      <c r="D26" s="1323" t="n"/>
+      <c r="E26" s="1323" t="n"/>
+      <c r="F26" s="1323" t="n"/>
+      <c r="G26" s="1323" t="n"/>
+      <c r="H26" s="1323" t="n"/>
+      <c r="I26" s="1324" t="n"/>
+      <c r="J26" s="1325" t="n"/>
+      <c r="K26" s="1325" t="n"/>
+      <c r="L26" s="1325" t="n"/>
+      <c r="M26" s="1323" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1281" t="n">
+      <c r="N26" s="1323" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1281" t="n"/>
-      <c r="P26" s="1284" t="n"/>
-      <c r="Q26" s="1281" t="n"/>
-      <c r="R26" s="1281" t="n"/>
-      <c r="S26" s="1281" t="n"/>
+      <c r="O26" s="1323" t="n"/>
+      <c r="P26" s="1326" t="n"/>
+      <c r="Q26" s="1323" t="n"/>
+      <c r="R26" s="1323" t="n"/>
+      <c r="S26" s="1323" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1280" t="n"/>
+      <c r="U26" s="1322" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -6016,53 +6124,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1285" t="inlineStr">
+      <c r="A27" s="1327" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1286" t="inlineStr">
+      <c r="B27" s="1328" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1286" t="inlineStr">
+      <c r="C27" s="1328" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1287" t="n"/>
-      <c r="E27" s="1287" t="n">
+      <c r="D27" s="1329" t="n"/>
+      <c r="E27" s="1329" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1287" t="n">
+      <c r="F27" s="1329" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1287" t="n">
+      <c r="G27" s="1329" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1287" t="n"/>
-      <c r="I27" s="1288" t="n"/>
-      <c r="J27" s="1289" t="n"/>
-      <c r="K27" s="1289" t="n"/>
-      <c r="L27" s="1289" t="n"/>
-      <c r="M27" s="1287" t="n"/>
-      <c r="N27" s="1287" t="n"/>
-      <c r="O27" s="1287" t="n">
+      <c r="H27" s="1329" t="n"/>
+      <c r="I27" s="1330" t="n"/>
+      <c r="J27" s="1331" t="n"/>
+      <c r="K27" s="1331" t="n"/>
+      <c r="L27" s="1331" t="n"/>
+      <c r="M27" s="1329" t="n"/>
+      <c r="N27" s="1329" t="n"/>
+      <c r="O27" s="1329" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1290" t="n">
+      <c r="P27" s="1332" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1287" t="n"/>
-      <c r="R27" s="1287" t="n"/>
-      <c r="S27" s="1287" t="n"/>
+      <c r="Q27" s="1329" t="n"/>
+      <c r="R27" s="1329" t="n"/>
+      <c r="S27" s="1329" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1286" t="n"/>
+      <c r="U27" s="1328" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -6070,47 +6178,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1297" t="inlineStr">
+      <c r="A28" s="1339" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1298" t="inlineStr">
+      <c r="B28" s="1340" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1298" t="inlineStr">
+      <c r="C28" s="1340" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1299" t="n"/>
-      <c r="E28" s="1299" t="n"/>
-      <c r="F28" s="1299" t="n"/>
-      <c r="G28" s="1299" t="n"/>
-      <c r="H28" s="1299" t="n"/>
-      <c r="I28" s="1300" t="n"/>
-      <c r="J28" s="1301" t="n"/>
-      <c r="K28" s="1301" t="n"/>
-      <c r="L28" s="1301" t="n"/>
-      <c r="M28" s="1299" t="n">
+      <c r="D28" s="1341" t="n"/>
+      <c r="E28" s="1341" t="n"/>
+      <c r="F28" s="1341" t="n"/>
+      <c r="G28" s="1341" t="n"/>
+      <c r="H28" s="1341" t="n"/>
+      <c r="I28" s="1342" t="n"/>
+      <c r="J28" s="1343" t="n"/>
+      <c r="K28" s="1343" t="n"/>
+      <c r="L28" s="1343" t="n"/>
+      <c r="M28" s="1341" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1299" t="n">
+      <c r="N28" s="1341" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1299" t="n"/>
-      <c r="P28" s="1302" t="n"/>
-      <c r="Q28" s="1299" t="n"/>
-      <c r="R28" s="1299" t="n"/>
-      <c r="S28" s="1299" t="n"/>
+      <c r="O28" s="1341" t="n"/>
+      <c r="P28" s="1344" t="n"/>
+      <c r="Q28" s="1341" t="n"/>
+      <c r="R28" s="1341" t="n"/>
+      <c r="S28" s="1341" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1298" t="n"/>
+      <c r="U28" s="1340" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -6118,53 +6226,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1273" t="inlineStr">
+      <c r="A29" s="1315" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1274" t="inlineStr">
+      <c r="B29" s="1316" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1274" t="inlineStr">
+      <c r="C29" s="1316" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1275" t="n"/>
-      <c r="E29" s="1275" t="n">
+      <c r="D29" s="1317" t="n"/>
+      <c r="E29" s="1317" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1275" t="n">
+      <c r="F29" s="1317" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1275" t="n">
+      <c r="G29" s="1317" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1275" t="n"/>
-      <c r="I29" s="1276" t="n"/>
-      <c r="J29" s="1277" t="n"/>
-      <c r="K29" s="1277" t="n"/>
-      <c r="L29" s="1277" t="n"/>
-      <c r="M29" s="1275" t="n"/>
-      <c r="N29" s="1275" t="n"/>
-      <c r="O29" s="1275" t="n">
+      <c r="H29" s="1317" t="n"/>
+      <c r="I29" s="1318" t="n"/>
+      <c r="J29" s="1319" t="n"/>
+      <c r="K29" s="1319" t="n"/>
+      <c r="L29" s="1319" t="n"/>
+      <c r="M29" s="1317" t="n"/>
+      <c r="N29" s="1317" t="n"/>
+      <c r="O29" s="1317" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1278" t="n">
+      <c r="P29" s="1320" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1275" t="n"/>
-      <c r="R29" s="1275" t="n"/>
-      <c r="S29" s="1275" t="n"/>
+      <c r="Q29" s="1317" t="n"/>
+      <c r="R29" s="1317" t="n"/>
+      <c r="S29" s="1317" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1274" t="n"/>
+      <c r="U29" s="1316" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -6172,43 +6280,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1279" t="inlineStr">
+      <c r="A30" s="1321" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1280" t="inlineStr">
+      <c r="B30" s="1322" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1280" t="inlineStr">
+      <c r="C30" s="1322" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1281" t="n"/>
-      <c r="E30" s="1281" t="n"/>
-      <c r="F30" s="1281" t="n"/>
-      <c r="G30" s="1281" t="n"/>
-      <c r="H30" s="1281" t="n"/>
-      <c r="I30" s="1282" t="n"/>
-      <c r="J30" s="1283" t="n"/>
-      <c r="K30" s="1283" t="n"/>
-      <c r="L30" s="1283" t="n"/>
-      <c r="M30" s="1281" t="n"/>
-      <c r="N30" s="1281" t="n"/>
-      <c r="O30" s="1281" t="n"/>
-      <c r="P30" s="1284" t="n"/>
-      <c r="Q30" s="1281" t="n"/>
-      <c r="R30" s="1281" t="n"/>
-      <c r="S30" s="1281" t="n"/>
+      <c r="D30" s="1323" t="n"/>
+      <c r="E30" s="1323" t="n"/>
+      <c r="F30" s="1323" t="n"/>
+      <c r="G30" s="1323" t="n"/>
+      <c r="H30" s="1323" t="n"/>
+      <c r="I30" s="1324" t="n"/>
+      <c r="J30" s="1325" t="n"/>
+      <c r="K30" s="1325" t="n"/>
+      <c r="L30" s="1325" t="n"/>
+      <c r="M30" s="1323" t="n"/>
+      <c r="N30" s="1323" t="n"/>
+      <c r="O30" s="1323" t="n"/>
+      <c r="P30" s="1326" t="n"/>
+      <c r="Q30" s="1323" t="n"/>
+      <c r="R30" s="1323" t="n"/>
+      <c r="S30" s="1323" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1280" t="n"/>
+      <c r="U30" s="1322" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -6216,53 +6324,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1285" t="inlineStr">
+      <c r="A31" s="1327" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1286" t="inlineStr">
+      <c r="B31" s="1328" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1286" t="inlineStr">
+      <c r="C31" s="1328" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1287" t="n"/>
-      <c r="E31" s="1287" t="n">
+      <c r="D31" s="1329" t="n"/>
+      <c r="E31" s="1329" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1287" t="n">
+      <c r="F31" s="1329" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1287" t="n">
+      <c r="G31" s="1329" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1287" t="n"/>
-      <c r="I31" s="1288" t="n"/>
-      <c r="J31" s="1289" t="n"/>
-      <c r="K31" s="1289" t="n"/>
-      <c r="L31" s="1289" t="n"/>
-      <c r="M31" s="1287" t="n"/>
-      <c r="N31" s="1287" t="n"/>
-      <c r="O31" s="1287" t="n">
+      <c r="H31" s="1329" t="n"/>
+      <c r="I31" s="1330" t="n"/>
+      <c r="J31" s="1331" t="n"/>
+      <c r="K31" s="1331" t="n"/>
+      <c r="L31" s="1331" t="n"/>
+      <c r="M31" s="1329" t="n"/>
+      <c r="N31" s="1329" t="n"/>
+      <c r="O31" s="1329" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1290" t="n">
+      <c r="P31" s="1332" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1287" t="n"/>
-      <c r="R31" s="1287" t="n"/>
-      <c r="S31" s="1287" t="n"/>
+      <c r="Q31" s="1329" t="n"/>
+      <c r="R31" s="1329" t="n"/>
+      <c r="S31" s="1329" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1286" t="inlineStr">
+      <c r="U31" s="1328" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -6274,49 +6382,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1297" t="inlineStr">
+      <c r="A32" s="1339" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1298" t="inlineStr">
+      <c r="B32" s="1340" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1298" t="inlineStr">
+      <c r="C32" s="1340" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1299" t="n"/>
-      <c r="E32" s="1299" t="n"/>
-      <c r="F32" s="1299" t="n"/>
-      <c r="G32" s="1299" t="n"/>
-      <c r="H32" s="1299" t="n">
+      <c r="D32" s="1341" t="n"/>
+      <c r="E32" s="1341" t="n"/>
+      <c r="F32" s="1341" t="n"/>
+      <c r="G32" s="1341" t="n"/>
+      <c r="H32" s="1341" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1300" t="n"/>
-      <c r="J32" s="1301" t="n"/>
-      <c r="K32" s="1301" t="n"/>
-      <c r="L32" s="1301" t="n"/>
-      <c r="M32" s="1299" t="n">
+      <c r="I32" s="1342" t="n"/>
+      <c r="J32" s="1343" t="n"/>
+      <c r="K32" s="1343" t="n"/>
+      <c r="L32" s="1343" t="n"/>
+      <c r="M32" s="1341" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1299" t="n">
+      <c r="N32" s="1341" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1299" t="n"/>
-      <c r="P32" s="1302" t="n"/>
-      <c r="Q32" s="1299" t="n"/>
-      <c r="R32" s="1299" t="n"/>
-      <c r="S32" s="1299" t="n"/>
+      <c r="O32" s="1341" t="n"/>
+      <c r="P32" s="1344" t="n"/>
+      <c r="Q32" s="1341" t="n"/>
+      <c r="R32" s="1341" t="n"/>
+      <c r="S32" s="1341" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1298" t="n"/>
+      <c r="U32" s="1340" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -6324,57 +6432,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1273" t="inlineStr">
+      <c r="A33" s="1315" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1274" t="inlineStr">
+      <c r="B33" s="1316" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1274" t="inlineStr">
+      <c r="C33" s="1316" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1275" t="n"/>
-      <c r="E33" s="1275" t="n">
+      <c r="D33" s="1317" t="n"/>
+      <c r="E33" s="1317" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1275" t="n">
+      <c r="F33" s="1317" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1275" t="n">
+      <c r="G33" s="1317" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1275" t="n"/>
-      <c r="I33" s="1276" t="n">
+      <c r="H33" s="1317" t="n"/>
+      <c r="I33" s="1318" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1277" t="n"/>
-      <c r="K33" s="1277" t="n"/>
-      <c r="L33" s="1277" t="n"/>
-      <c r="M33" s="1275" t="n"/>
-      <c r="N33" s="1275" t="n"/>
-      <c r="O33" s="1275" t="n">
+      <c r="J33" s="1319" t="n"/>
+      <c r="K33" s="1319" t="n"/>
+      <c r="L33" s="1319" t="n"/>
+      <c r="M33" s="1317" t="n"/>
+      <c r="N33" s="1317" t="n"/>
+      <c r="O33" s="1317" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1278" t="n">
+      <c r="P33" s="1320" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1275" t="n"/>
-      <c r="R33" s="1275" t="n">
+      <c r="Q33" s="1317" t="n"/>
+      <c r="R33" s="1317" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1275" t="n"/>
+      <c r="S33" s="1317" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1274" t="inlineStr">
+      <c r="U33" s="1316" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -6386,49 +6494,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1279" t="inlineStr">
+      <c r="A34" s="1321" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1280" t="inlineStr">
+      <c r="B34" s="1322" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1280" t="inlineStr">
+      <c r="C34" s="1322" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1281" t="n"/>
-      <c r="E34" s="1281" t="n"/>
-      <c r="F34" s="1281" t="n"/>
-      <c r="G34" s="1281" t="n"/>
-      <c r="H34" s="1281" t="n">
+      <c r="D34" s="1323" t="n"/>
+      <c r="E34" s="1323" t="n"/>
+      <c r="F34" s="1323" t="n"/>
+      <c r="G34" s="1323" t="n"/>
+      <c r="H34" s="1323" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1282" t="n"/>
-      <c r="J34" s="1283" t="n"/>
-      <c r="K34" s="1283" t="n"/>
-      <c r="L34" s="1283" t="n"/>
-      <c r="M34" s="1281" t="n">
+      <c r="I34" s="1324" t="n"/>
+      <c r="J34" s="1325" t="n"/>
+      <c r="K34" s="1325" t="n"/>
+      <c r="L34" s="1325" t="n"/>
+      <c r="M34" s="1323" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1281" t="n">
+      <c r="N34" s="1323" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1281" t="n"/>
-      <c r="P34" s="1284" t="n"/>
-      <c r="Q34" s="1281" t="n"/>
-      <c r="R34" s="1281" t="n"/>
-      <c r="S34" s="1281" t="n"/>
+      <c r="O34" s="1323" t="n"/>
+      <c r="P34" s="1326" t="n"/>
+      <c r="Q34" s="1323" t="n"/>
+      <c r="R34" s="1323" t="n"/>
+      <c r="S34" s="1323" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1280" t="n"/>
+      <c r="U34" s="1322" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -6436,57 +6544,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1285" t="inlineStr">
+      <c r="A35" s="1327" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1286" t="inlineStr">
+      <c r="B35" s="1328" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1286" t="inlineStr">
+      <c r="C35" s="1328" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1287" t="n"/>
-      <c r="E35" s="1287" t="n">
+      <c r="D35" s="1329" t="n"/>
+      <c r="E35" s="1329" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1287" t="n">
+      <c r="F35" s="1329" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1287" t="n">
+      <c r="G35" s="1329" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1287" t="n"/>
-      <c r="I35" s="1288" t="n">
+      <c r="H35" s="1329" t="n"/>
+      <c r="I35" s="1330" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1289" t="n"/>
-      <c r="K35" s="1289" t="n"/>
-      <c r="L35" s="1289" t="n"/>
-      <c r="M35" s="1287" t="n"/>
-      <c r="N35" s="1287" t="n"/>
-      <c r="O35" s="1287" t="n">
+      <c r="J35" s="1331" t="n"/>
+      <c r="K35" s="1331" t="n"/>
+      <c r="L35" s="1331" t="n"/>
+      <c r="M35" s="1329" t="n"/>
+      <c r="N35" s="1329" t="n"/>
+      <c r="O35" s="1329" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1290" t="n">
+      <c r="P35" s="1332" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1287" t="n"/>
-      <c r="R35" s="1287" t="n">
+      <c r="Q35" s="1329" t="n"/>
+      <c r="R35" s="1329" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1287" t="n"/>
+      <c r="S35" s="1329" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1286" t="inlineStr">
+      <c r="U35" s="1328" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -6498,49 +6606,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1291" t="inlineStr">
+      <c r="A36" s="1333" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1292" t="inlineStr">
+      <c r="B36" s="1334" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1292" t="inlineStr">
+      <c r="C36" s="1334" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1293" t="n"/>
-      <c r="E36" s="1293" t="n"/>
-      <c r="F36" s="1293" t="n"/>
-      <c r="G36" s="1293" t="n"/>
-      <c r="H36" s="1293" t="n">
+      <c r="D36" s="1335" t="n"/>
+      <c r="E36" s="1335" t="n"/>
+      <c r="F36" s="1335" t="n"/>
+      <c r="G36" s="1335" t="n"/>
+      <c r="H36" s="1335" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1294" t="n"/>
-      <c r="J36" s="1295" t="n"/>
-      <c r="K36" s="1295" t="n"/>
-      <c r="L36" s="1295" t="n"/>
-      <c r="M36" s="1293" t="n">
+      <c r="I36" s="1336" t="n"/>
+      <c r="J36" s="1337" t="n"/>
+      <c r="K36" s="1337" t="n"/>
+      <c r="L36" s="1337" t="n"/>
+      <c r="M36" s="1335" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1293" t="n">
+      <c r="N36" s="1335" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1293" t="n"/>
-      <c r="P36" s="1296" t="n"/>
-      <c r="Q36" s="1293" t="n"/>
-      <c r="R36" s="1293" t="n"/>
-      <c r="S36" s="1293" t="n"/>
+      <c r="O36" s="1335" t="n"/>
+      <c r="P36" s="1338" t="n"/>
+      <c r="Q36" s="1335" t="n"/>
+      <c r="R36" s="1335" t="n"/>
+      <c r="S36" s="1335" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1292" t="n"/>
+      <c r="U36" s="1334" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -6548,41 +6656,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1297" t="inlineStr">
+      <c r="A37" s="1339" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1298" t="inlineStr">
+      <c r="B37" s="1340" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1298" t="inlineStr">
+      <c r="C37" s="1340" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1299" t="n"/>
-      <c r="E37" s="1299" t="n"/>
-      <c r="F37" s="1299" t="n"/>
-      <c r="G37" s="1299" t="n"/>
-      <c r="H37" s="1299" t="n"/>
-      <c r="I37" s="1300" t="n"/>
-      <c r="J37" s="1301" t="n"/>
-      <c r="K37" s="1301" t="n"/>
-      <c r="L37" s="1301" t="n"/>
-      <c r="M37" s="1299" t="n"/>
-      <c r="N37" s="1299" t="n"/>
-      <c r="O37" s="1299" t="n"/>
-      <c r="P37" s="1302" t="n"/>
-      <c r="Q37" s="1299" t="n">
+      <c r="D37" s="1341" t="n"/>
+      <c r="E37" s="1341" t="n"/>
+      <c r="F37" s="1341" t="n"/>
+      <c r="G37" s="1341" t="n"/>
+      <c r="H37" s="1341" t="n"/>
+      <c r="I37" s="1342" t="n"/>
+      <c r="J37" s="1343" t="n"/>
+      <c r="K37" s="1343" t="n"/>
+      <c r="L37" s="1343" t="n"/>
+      <c r="M37" s="1341" t="n"/>
+      <c r="N37" s="1341" t="n"/>
+      <c r="O37" s="1341" t="n"/>
+      <c r="P37" s="1344" t="n"/>
+      <c r="Q37" s="1341" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1299" t="n"/>
-      <c r="S37" s="1299" t="n"/>
+      <c r="R37" s="1341" t="n"/>
+      <c r="S37" s="1341" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1298" t="n"/>
+      <c r="U37" s="1340" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -6590,57 +6698,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1273" t="inlineStr">
+      <c r="A38" s="1315" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1274" t="inlineStr">
+      <c r="B38" s="1316" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1274" t="inlineStr">
+      <c r="C38" s="1316" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1275" t="n"/>
-      <c r="E38" s="1275" t="n">
+      <c r="D38" s="1317" t="n"/>
+      <c r="E38" s="1317" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1275" t="n">
+      <c r="F38" s="1317" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1275" t="n">
+      <c r="G38" s="1317" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1275" t="n"/>
-      <c r="I38" s="1276" t="n">
+      <c r="H38" s="1317" t="n"/>
+      <c r="I38" s="1318" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1277" t="n"/>
-      <c r="K38" s="1277" t="n"/>
-      <c r="L38" s="1277" t="n"/>
-      <c r="M38" s="1275" t="n"/>
-      <c r="N38" s="1275" t="n"/>
-      <c r="O38" s="1275" t="n">
+      <c r="J38" s="1319" t="n"/>
+      <c r="K38" s="1319" t="n"/>
+      <c r="L38" s="1319" t="n"/>
+      <c r="M38" s="1317" t="n"/>
+      <c r="N38" s="1317" t="n"/>
+      <c r="O38" s="1317" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1278" t="n">
+      <c r="P38" s="1320" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1275" t="n"/>
-      <c r="R38" s="1275" t="n">
+      <c r="Q38" s="1317" t="n"/>
+      <c r="R38" s="1317" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1275" t="n"/>
+      <c r="S38" s="1317" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1274" t="inlineStr">
+      <c r="U38" s="1316" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -6652,49 +6760,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1303" t="inlineStr">
+      <c r="A39" s="1345" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1304" t="inlineStr">
+      <c r="B39" s="1346" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1304" t="inlineStr">
+      <c r="C39" s="1346" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1305" t="n"/>
-      <c r="E39" s="1305" t="n"/>
-      <c r="F39" s="1305" t="n"/>
-      <c r="G39" s="1305" t="n"/>
-      <c r="H39" s="1305" t="n">
+      <c r="D39" s="1347" t="n"/>
+      <c r="E39" s="1347" t="n"/>
+      <c r="F39" s="1347" t="n"/>
+      <c r="G39" s="1347" t="n"/>
+      <c r="H39" s="1347" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1306" t="n"/>
-      <c r="J39" s="1307" t="n"/>
-      <c r="K39" s="1307" t="n"/>
-      <c r="L39" s="1307" t="n"/>
-      <c r="M39" s="1305" t="n">
+      <c r="I39" s="1348" t="n"/>
+      <c r="J39" s="1349" t="n"/>
+      <c r="K39" s="1349" t="n"/>
+      <c r="L39" s="1349" t="n"/>
+      <c r="M39" s="1347" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1305" t="n">
+      <c r="N39" s="1347" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1305" t="n"/>
-      <c r="P39" s="1308" t="n"/>
-      <c r="Q39" s="1305" t="n"/>
-      <c r="R39" s="1305" t="n"/>
-      <c r="S39" s="1305" t="n"/>
+      <c r="O39" s="1347" t="n"/>
+      <c r="P39" s="1350" t="n"/>
+      <c r="Q39" s="1347" t="n"/>
+      <c r="R39" s="1347" t="n"/>
+      <c r="S39" s="1347" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1304" t="n"/>
+      <c r="U39" s="1346" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -6702,41 +6810,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1279" t="inlineStr">
+      <c r="A40" s="1321" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1280" t="inlineStr">
+      <c r="B40" s="1322" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1280" t="inlineStr">
+      <c r="C40" s="1322" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1281" t="n"/>
-      <c r="E40" s="1281" t="n"/>
-      <c r="F40" s="1281" t="n"/>
-      <c r="G40" s="1281" t="n"/>
-      <c r="H40" s="1281" t="n"/>
-      <c r="I40" s="1282" t="n"/>
-      <c r="J40" s="1283" t="n"/>
-      <c r="K40" s="1283" t="n"/>
-      <c r="L40" s="1283" t="n"/>
-      <c r="M40" s="1281" t="n"/>
-      <c r="N40" s="1281" t="n"/>
-      <c r="O40" s="1281" t="n"/>
-      <c r="P40" s="1284" t="n"/>
-      <c r="Q40" s="1281" t="n">
+      <c r="D40" s="1323" t="n"/>
+      <c r="E40" s="1323" t="n"/>
+      <c r="F40" s="1323" t="n"/>
+      <c r="G40" s="1323" t="n"/>
+      <c r="H40" s="1323" t="n"/>
+      <c r="I40" s="1324" t="n"/>
+      <c r="J40" s="1325" t="n"/>
+      <c r="K40" s="1325" t="n"/>
+      <c r="L40" s="1325" t="n"/>
+      <c r="M40" s="1323" t="n"/>
+      <c r="N40" s="1323" t="n"/>
+      <c r="O40" s="1323" t="n"/>
+      <c r="P40" s="1326" t="n"/>
+      <c r="Q40" s="1323" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1281" t="n"/>
-      <c r="S40" s="1281" t="n"/>
+      <c r="R40" s="1323" t="n"/>
+      <c r="S40" s="1323" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1280" t="n"/>
+      <c r="U40" s="1322" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -6744,57 +6852,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1285" t="inlineStr">
+      <c r="A41" s="1327" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1286" t="inlineStr">
+      <c r="B41" s="1328" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1286" t="inlineStr">
+      <c r="C41" s="1328" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1287" t="n"/>
-      <c r="E41" s="1287" t="n">
+      <c r="D41" s="1329" t="n"/>
+      <c r="E41" s="1329" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1287" t="n">
+      <c r="F41" s="1329" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1287" t="n">
+      <c r="G41" s="1329" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1287" t="n"/>
-      <c r="I41" s="1288" t="n">
+      <c r="H41" s="1329" t="n"/>
+      <c r="I41" s="1330" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1289" t="n"/>
-      <c r="K41" s="1289" t="n"/>
-      <c r="L41" s="1289" t="n"/>
-      <c r="M41" s="1287" t="n"/>
-      <c r="N41" s="1287" t="n"/>
-      <c r="O41" s="1287" t="n">
+      <c r="J41" s="1331" t="n"/>
+      <c r="K41" s="1331" t="n"/>
+      <c r="L41" s="1331" t="n"/>
+      <c r="M41" s="1329" t="n"/>
+      <c r="N41" s="1329" t="n"/>
+      <c r="O41" s="1329" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1290" t="n">
+      <c r="P41" s="1332" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1287" t="n"/>
-      <c r="R41" s="1287" t="n">
+      <c r="Q41" s="1329" t="n"/>
+      <c r="R41" s="1329" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1287" t="n"/>
+      <c r="S41" s="1329" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1286" t="inlineStr">
+      <c r="U41" s="1328" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -6806,49 +6914,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1297" t="inlineStr">
+      <c r="A42" s="1339" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1298" t="inlineStr">
+      <c r="B42" s="1340" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1298" t="inlineStr">
+      <c r="C42" s="1340" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1299" t="n"/>
-      <c r="E42" s="1299" t="n"/>
-      <c r="F42" s="1299" t="n"/>
-      <c r="G42" s="1299" t="n"/>
-      <c r="H42" s="1299" t="n">
+      <c r="D42" s="1341" t="n"/>
+      <c r="E42" s="1341" t="n"/>
+      <c r="F42" s="1341" t="n"/>
+      <c r="G42" s="1341" t="n"/>
+      <c r="H42" s="1341" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1300" t="n"/>
-      <c r="J42" s="1301" t="n"/>
-      <c r="K42" s="1301" t="n"/>
-      <c r="L42" s="1301" t="n"/>
-      <c r="M42" s="1299" t="n">
+      <c r="I42" s="1342" t="n"/>
+      <c r="J42" s="1343" t="n"/>
+      <c r="K42" s="1343" t="n"/>
+      <c r="L42" s="1343" t="n"/>
+      <c r="M42" s="1341" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1299" t="n">
+      <c r="N42" s="1341" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1299" t="n"/>
-      <c r="P42" s="1302" t="n"/>
-      <c r="Q42" s="1299" t="n"/>
-      <c r="R42" s="1299" t="n"/>
-      <c r="S42" s="1299" t="n"/>
+      <c r="O42" s="1341" t="n"/>
+      <c r="P42" s="1344" t="n"/>
+      <c r="Q42" s="1341" t="n"/>
+      <c r="R42" s="1341" t="n"/>
+      <c r="S42" s="1341" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1298" t="n"/>
+      <c r="U42" s="1340" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -6856,57 +6964,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1273" t="inlineStr">
+      <c r="A43" s="1315" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1274" t="inlineStr">
+      <c r="B43" s="1316" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1274" t="inlineStr">
+      <c r="C43" s="1316" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1275" t="n"/>
-      <c r="E43" s="1275" t="n">
+      <c r="D43" s="1317" t="n"/>
+      <c r="E43" s="1317" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1275" t="n">
+      <c r="F43" s="1317" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1275" t="n">
+      <c r="G43" s="1317" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1275" t="n"/>
-      <c r="I43" s="1276" t="n">
+      <c r="H43" s="1317" t="n"/>
+      <c r="I43" s="1318" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1277" t="n"/>
-      <c r="K43" s="1277" t="n"/>
-      <c r="L43" s="1277" t="n"/>
-      <c r="M43" s="1275" t="n"/>
-      <c r="N43" s="1275" t="n"/>
-      <c r="O43" s="1275" t="n">
+      <c r="J43" s="1319" t="n"/>
+      <c r="K43" s="1319" t="n"/>
+      <c r="L43" s="1319" t="n"/>
+      <c r="M43" s="1317" t="n"/>
+      <c r="N43" s="1317" t="n"/>
+      <c r="O43" s="1317" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1278" t="n">
+      <c r="P43" s="1320" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1275" t="n"/>
-      <c r="R43" s="1275" t="n">
+      <c r="Q43" s="1317" t="n"/>
+      <c r="R43" s="1317" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1275" t="n"/>
+      <c r="S43" s="1317" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1274" t="n"/>
+      <c r="U43" s="1316" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -6914,45 +7022,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1303" t="inlineStr">
+      <c r="A44" s="1345" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1304" t="inlineStr">
+      <c r="B44" s="1346" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1304" t="inlineStr">
+      <c r="C44" s="1346" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1305" t="n"/>
-      <c r="E44" s="1305" t="n">
+      <c r="D44" s="1347" t="n"/>
+      <c r="E44" s="1347" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1305" t="n">
+      <c r="F44" s="1347" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1305" t="n"/>
-      <c r="H44" s="1305" t="n"/>
-      <c r="I44" s="1306" t="n"/>
-      <c r="J44" s="1307" t="n"/>
-      <c r="K44" s="1307" t="n"/>
-      <c r="L44" s="1307" t="n"/>
-      <c r="M44" s="1305" t="n"/>
-      <c r="N44" s="1305" t="n"/>
-      <c r="O44" s="1305" t="n"/>
-      <c r="P44" s="1308" t="n"/>
-      <c r="Q44" s="1305" t="n"/>
-      <c r="R44" s="1305" t="n"/>
-      <c r="S44" s="1305" t="n">
+      <c r="G44" s="1347" t="n"/>
+      <c r="H44" s="1347" t="n"/>
+      <c r="I44" s="1348" t="n"/>
+      <c r="J44" s="1349" t="n"/>
+      <c r="K44" s="1349" t="n"/>
+      <c r="L44" s="1349" t="n"/>
+      <c r="M44" s="1347" t="n"/>
+      <c r="N44" s="1347" t="n"/>
+      <c r="O44" s="1347" t="n"/>
+      <c r="P44" s="1350" t="n"/>
+      <c r="Q44" s="1347" t="n"/>
+      <c r="R44" s="1347" t="n"/>
+      <c r="S44" s="1347" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1304" t="inlineStr">
+      <c r="U44" s="1346" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -6964,49 +7072,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1303" t="inlineStr">
+      <c r="A45" s="1345" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1304" t="inlineStr">
+      <c r="B45" s="1346" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1304" t="inlineStr">
+      <c r="C45" s="1346" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1305" t="n"/>
-      <c r="E45" s="1305" t="n"/>
-      <c r="F45" s="1305" t="n"/>
-      <c r="G45" s="1305" t="n"/>
-      <c r="H45" s="1305" t="n">
+      <c r="D45" s="1347" t="n"/>
+      <c r="E45" s="1347" t="n"/>
+      <c r="F45" s="1347" t="n"/>
+      <c r="G45" s="1347" t="n"/>
+      <c r="H45" s="1347" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1306" t="n"/>
-      <c r="J45" s="1307" t="n"/>
-      <c r="K45" s="1307" t="n"/>
-      <c r="L45" s="1307" t="n"/>
-      <c r="M45" s="1305" t="n">
+      <c r="I45" s="1348" t="n"/>
+      <c r="J45" s="1349" t="n"/>
+      <c r="K45" s="1349" t="n"/>
+      <c r="L45" s="1349" t="n"/>
+      <c r="M45" s="1347" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1305" t="n">
+      <c r="N45" s="1347" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1305" t="n"/>
-      <c r="P45" s="1308" t="n"/>
-      <c r="Q45" s="1305" t="n"/>
-      <c r="R45" s="1305" t="n"/>
-      <c r="S45" s="1305" t="n"/>
+      <c r="O45" s="1347" t="n"/>
+      <c r="P45" s="1350" t="n"/>
+      <c r="Q45" s="1347" t="n"/>
+      <c r="R45" s="1347" t="n"/>
+      <c r="S45" s="1347" t="n"/>
       <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1304" t="n"/>
+      <c r="U45" s="1346" t="n"/>
       <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -7014,39 +7122,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1279" t="inlineStr">
+      <c r="A46" s="1321" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B46" s="1280" t="inlineStr">
+      <c r="B46" s="1322" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="C46" s="1280" t="inlineStr">
+      <c r="C46" s="1322" t="inlineStr">
         <is>
           <t>EVENT - Clean</t>
         </is>
       </c>
-      <c r="D46" s="1281" t="n"/>
-      <c r="E46" s="1281" t="n"/>
-      <c r="F46" s="1281" t="n"/>
-      <c r="G46" s="1281" t="n"/>
-      <c r="H46" s="1281" t="n"/>
-      <c r="I46" s="1282" t="n"/>
-      <c r="J46" s="1283" t="n"/>
-      <c r="K46" s="1283" t="n"/>
-      <c r="L46" s="1283" t="n"/>
-      <c r="M46" s="1281" t="n"/>
-      <c r="N46" s="1281" t="n"/>
-      <c r="O46" s="1281" t="n"/>
-      <c r="P46" s="1284" t="n"/>
-      <c r="Q46" s="1281" t="n"/>
-      <c r="R46" s="1281" t="n"/>
-      <c r="S46" s="1281" t="n"/>
+      <c r="D46" s="1323" t="n"/>
+      <c r="E46" s="1323" t="n"/>
+      <c r="F46" s="1323" t="n"/>
+      <c r="G46" s="1323" t="n"/>
+      <c r="H46" s="1323" t="n"/>
+      <c r="I46" s="1324" t="n"/>
+      <c r="J46" s="1325" t="n"/>
+      <c r="K46" s="1325" t="n"/>
+      <c r="L46" s="1325" t="n"/>
+      <c r="M46" s="1323" t="n"/>
+      <c r="N46" s="1323" t="n"/>
+      <c r="O46" s="1323" t="n"/>
+      <c r="P46" s="1326" t="n"/>
+      <c r="Q46" s="1323" t="n"/>
+      <c r="R46" s="1323" t="n"/>
+      <c r="S46" s="1323" t="n"/>
       <c r="T46" s="631" t="n"/>
-      <c r="U46" s="1280" t="n"/>
+      <c r="U46" s="1322" t="n"/>
       <c r="V46" s="632" t="inlineStr">
         <is>
           <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
@@ -7054,51 +7162,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1285" t="inlineStr">
+      <c r="A47" s="1327" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1286" t="inlineStr">
+      <c r="B47" s="1328" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C47" s="1286" t="inlineStr">
+      <c r="C47" s="1328" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D47" s="1287" t="n"/>
-      <c r="E47" s="1287" t="n">
+      <c r="D47" s="1329" t="n"/>
+      <c r="E47" s="1329" t="n">
         <v>16.6</v>
       </c>
-      <c r="F47" s="1287" t="n">
+      <c r="F47" s="1329" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="1287" t="n">
+      <c r="G47" s="1329" t="n">
         <v>4.1</v>
       </c>
-      <c r="H47" s="1287" t="n"/>
-      <c r="I47" s="1288" t="n">
+      <c r="H47" s="1329" t="n"/>
+      <c r="I47" s="1330" t="n">
         <v>0.9</v>
       </c>
-      <c r="J47" s="1289" t="n"/>
-      <c r="K47" s="1289" t="n"/>
-      <c r="L47" s="1289" t="n"/>
-      <c r="M47" s="1287" t="n"/>
-      <c r="N47" s="1287" t="n"/>
-      <c r="O47" s="1287" t="n">
+      <c r="J47" s="1331" t="n"/>
+      <c r="K47" s="1331" t="n"/>
+      <c r="L47" s="1331" t="n"/>
+      <c r="M47" s="1329" t="n"/>
+      <c r="N47" s="1329" t="n"/>
+      <c r="O47" s="1329" t="n">
         <v>13.2</v>
       </c>
-      <c r="P47" s="1290" t="n">
+      <c r="P47" s="1332" t="n">
         <v>0</v>
       </c>
-      <c r="Q47" s="1287" t="n"/>
-      <c r="R47" s="1287" t="n">
+      <c r="Q47" s="1329" t="n"/>
+      <c r="R47" s="1329" t="n">
         <v>84.5</v>
       </c>
-      <c r="S47" s="1287" t="n">
+      <c r="S47" s="1329" t="n">
         <v>11.8</v>
       </c>
       <c r="T47" s="813" t="inlineStr">
@@ -7106,7 +7214,7 @@
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1286" t="inlineStr">
+      <c r="U47" s="1328" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
@@ -7118,49 +7226,49 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1297" t="inlineStr">
+      <c r="A48" s="1339" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B48" s="1298" t="inlineStr">
+      <c r="B48" s="1340" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C48" s="1298" t="inlineStr">
+      <c r="C48" s="1340" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D48" s="1299" t="n"/>
-      <c r="E48" s="1299" t="n"/>
-      <c r="F48" s="1299" t="n"/>
-      <c r="G48" s="1299" t="n"/>
-      <c r="H48" s="1299" t="n">
+      <c r="D48" s="1341" t="n"/>
+      <c r="E48" s="1341" t="n"/>
+      <c r="F48" s="1341" t="n"/>
+      <c r="G48" s="1341" t="n"/>
+      <c r="H48" s="1341" t="n">
         <v>15.1</v>
       </c>
-      <c r="I48" s="1300" t="n"/>
-      <c r="J48" s="1301" t="n"/>
-      <c r="K48" s="1301" t="n"/>
-      <c r="L48" s="1301" t="n"/>
-      <c r="M48" s="1299" t="n">
+      <c r="I48" s="1342" t="n"/>
+      <c r="J48" s="1343" t="n"/>
+      <c r="K48" s="1343" t="n"/>
+      <c r="L48" s="1343" t="n"/>
+      <c r="M48" s="1341" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="1299" t="n">
+      <c r="N48" s="1341" t="n">
         <v>20</v>
       </c>
-      <c r="O48" s="1299" t="n"/>
-      <c r="P48" s="1302" t="n"/>
-      <c r="Q48" s="1299" t="n"/>
-      <c r="R48" s="1299" t="n"/>
-      <c r="S48" s="1299" t="n"/>
+      <c r="O48" s="1341" t="n"/>
+      <c r="P48" s="1344" t="n"/>
+      <c r="Q48" s="1341" t="n"/>
+      <c r="R48" s="1341" t="n"/>
+      <c r="S48" s="1341" t="n"/>
       <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U48" s="1298" t="n"/>
+      <c r="U48" s="1340" t="n"/>
       <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
@@ -7168,62 +7276,116 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1309" t="inlineStr">
+      <c r="A49" s="1315" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B49" s="1310" t="inlineStr">
+      <c r="B49" s="1316" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C49" s="1310" t="inlineStr">
+      <c r="C49" s="1316" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D49" s="1311" t="n"/>
-      <c r="E49" s="1311" t="n">
+      <c r="D49" s="1317" t="n"/>
+      <c r="E49" s="1317" t="n">
         <v>16.8</v>
       </c>
-      <c r="F49" s="1311" t="n">
+      <c r="F49" s="1317" t="n">
         <v>0.2</v>
       </c>
-      <c r="G49" s="1311" t="n">
+      <c r="G49" s="1317" t="n">
         <v>3.3</v>
       </c>
-      <c r="H49" s="1311" t="n"/>
-      <c r="I49" s="1312" t="n">
+      <c r="H49" s="1317" t="n"/>
+      <c r="I49" s="1318" t="n">
         <v>1.7</v>
       </c>
-      <c r="J49" s="1313" t="n"/>
-      <c r="K49" s="1313" t="n"/>
-      <c r="L49" s="1313" t="n"/>
-      <c r="M49" s="1311" t="n"/>
-      <c r="N49" s="1311" t="n"/>
-      <c r="O49" s="1311" t="n">
+      <c r="J49" s="1319" t="n"/>
+      <c r="K49" s="1319" t="n"/>
+      <c r="L49" s="1319" t="n"/>
+      <c r="M49" s="1317" t="n"/>
+      <c r="N49" s="1317" t="n"/>
+      <c r="O49" s="1317" t="n">
         <v>13</v>
       </c>
-      <c r="P49" s="1314" t="n">
+      <c r="P49" s="1320" t="n">
         <v>0.87</v>
       </c>
-      <c r="Q49" s="1311" t="n"/>
-      <c r="R49" s="1311" t="n">
+      <c r="Q49" s="1317" t="n"/>
+      <c r="R49" s="1317" t="n">
         <v>86</v>
       </c>
-      <c r="S49" s="1311" t="n">
+      <c r="S49" s="1317" t="n">
         <v>11.65</v>
       </c>
-      <c r="T49" s="1047" t="inlineStr">
+      <c r="T49" s="624" t="inlineStr">
         <is>
           <t>Clear now, 88F, 67% RH; sun so far 6.4h of 7h daylight (91%); today high 90F, 0.87in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U49" s="1310" t="n"/>
-      <c r="V49" s="1048" t="inlineStr">
+      <c r="U49" s="1316" t="inlineStr">
+        <is>
+          <t>2026-07-04_1.jpeg;2026-07-04_2.jpeg;2026-07-04_3.jpeg;2026-07-04_4.jpeg</t>
+        </is>
+      </c>
+      <c r="V49" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 16.8, CC 0.2. CC CREEP CLEARED: 0.0-&gt;0.4-&gt;0.6-&gt;0.2 -- confirms the benign explanation (floating debris + 7/2 Magic Eraser residue), oxidized away by the high FC. Auto weather bucket said 'rain' (0.87in daily precip, likely the incoming 7/6 system's leading edge) but midday was clearly sunny (91% sun so far) -&gt; overrode to sunny for the loss model. fc_loss 3.3 ppm/24h (16.6 + 1.0gal x3.5 - 16.8), clean noon-to-noon (no recheck yesterday). PREDICTION RESOLVED: pred error +1.7 (actual 16.8 vs 7/3 dose's 15.1) = THIRD straight hot-day over-prediction (+2.1, +0.9, +1.7); the clean case -- landed high DESPITE today's extra CC-clearing demand. Actual hot-day losses ran ~2.9/4.1/3.3 (avg ~3.4), not the modeled 5.0. -&gt; Recalibrated dose.py l24_hot_sunny 5.0-&gt;4.0 (small cushion above the 3.4 mean). Water level 11.65 cm (11.9-&gt;11.8-&gt;11.65: steady slow evaporation decline over 3 hot dry days, ~0.1/day; the 7/6 rain will reverse it). PARTY PREP (Sun 7/5 1PM): recommending only 0.5 gal tonight -- FC already high at 16.8 and tomorrow's cooler/drizzly, so a full gal would overshoot into the high teens (John: don't go overboard). 0.5 gal -&gt; ~15-16 at party = comfortable top-of-band with cushion for bather load, not overboard.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="1321" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B50" s="1322" t="inlineStr">
+        <is>
+          <t>19:40</t>
+        </is>
+      </c>
+      <c r="C50" s="1322" t="inlineStr">
+        <is>
+          <t>DOSE</t>
+        </is>
+      </c>
+      <c r="D50" s="1323" t="n"/>
+      <c r="E50" s="1323" t="n"/>
+      <c r="F50" s="1323" t="n"/>
+      <c r="G50" s="1323" t="n"/>
+      <c r="H50" s="1323" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="I50" s="1324" t="n"/>
+      <c r="J50" s="1325" t="n"/>
+      <c r="K50" s="1325" t="n"/>
+      <c r="L50" s="1325" t="n"/>
+      <c r="M50" s="1323" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N50" s="1323" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="O50" s="1323" t="n"/>
+      <c r="P50" s="1326" t="n"/>
+      <c r="Q50" s="1323" t="n"/>
+      <c r="R50" s="1323" t="n"/>
+      <c r="S50" s="1323" t="n"/>
+      <c r="T50" s="631" t="inlineStr">
+        <is>
+          <t>Hot/sunny day (high 90F, water 86F); storm forecast overnight</t>
+        </is>
+      </c>
+      <c r="U50" s="1322" t="n"/>
+      <c r="V50" s="632" t="inlineStr">
+        <is>
+          <t>0.5 gal added 7:40 PM. PARTY PRE-LOAD (Sun 7/5 1PM picnic): deliberately HALF the usual dose -- FC already high at 16.8, and John didn't want to overshoot into the high teens for guests. Sized on the retuned model (l24_hot_sunny now 4.0). Model projects ~14.6 next noon, BUT this is a known weather-mismatch case: model keys L24 off today's hot/sunny weather, while the actual loss window is a storm overnight (no UV) + cooler/cloudy Sun morning -&gt; real loss will be LOWER, so FC likely lands ~15-16 at the party (comfortable top-of-band, cushion for bather load, not overboard). =&gt; If tomorrow's noon comes in ABOVE 14.6, that's the weather mismatch, NOT the freshly-retuned constant; don't chase it. Plan: dose back up Sun evening after the crowd's out (expect a bather-load FC drop). Season total 20.5 gal. PHOTOS(4): water clear/healthy blue, bottom fully visible, no cloudiness/algae; yesterday's surface debris now gone (tracks with CC clearing to 0.2); liner step close-up normal speckled blue, no rust/stain progression. Ruler photo documents the ~11.65 cm level.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log 2026-07-05 7:45AM (party day): FC 16.0, CC 0.5, level 13.9 (storm +2.25cm)
Early test before the 1PM picnic -- FC 16.0 is great, no morning top-up
needed. Confirms the weather mismatch flagged last night: overcast/cool
75F day means FC ran high vs the hot-sunny prediction (not the retune).
Overnight storm jumped the water level 11.65->13.9. CC ticked to 0.5
(rain-washed organic load, still a trace).
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1351">
+  <cellXfs count="1393">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -4580,6 +4580,132 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4841,7 +4967,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V50"/>
+  <dimension ref="A1:V51"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -5018,35 +5144,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1315" t="inlineStr">
+      <c r="A3" s="1351" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1316" t="n"/>
-      <c r="C3" s="1316" t="inlineStr">
+      <c r="B3" s="1352" t="n"/>
+      <c r="C3" s="1352" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1317" t="n"/>
-      <c r="E3" s="1317" t="n"/>
-      <c r="F3" s="1317" t="n"/>
-      <c r="G3" s="1317" t="n"/>
-      <c r="H3" s="1317" t="n"/>
-      <c r="I3" s="1318" t="n"/>
-      <c r="J3" s="1319" t="n"/>
-      <c r="K3" s="1319" t="n"/>
-      <c r="L3" s="1319" t="n"/>
-      <c r="M3" s="1317" t="n"/>
-      <c r="N3" s="1317" t="n"/>
-      <c r="O3" s="1317" t="n"/>
-      <c r="P3" s="1320" t="n"/>
-      <c r="Q3" s="1317" t="n"/>
-      <c r="R3" s="1317" t="n"/>
-      <c r="S3" s="1317" t="n"/>
+      <c r="D3" s="1353" t="n"/>
+      <c r="E3" s="1353" t="n"/>
+      <c r="F3" s="1353" t="n"/>
+      <c r="G3" s="1353" t="n"/>
+      <c r="H3" s="1353" t="n"/>
+      <c r="I3" s="1354" t="n"/>
+      <c r="J3" s="1355" t="n"/>
+      <c r="K3" s="1355" t="n"/>
+      <c r="L3" s="1355" t="n"/>
+      <c r="M3" s="1353" t="n"/>
+      <c r="N3" s="1353" t="n"/>
+      <c r="O3" s="1353" t="n"/>
+      <c r="P3" s="1356" t="n"/>
+      <c r="Q3" s="1353" t="n"/>
+      <c r="R3" s="1353" t="n"/>
+      <c r="S3" s="1353" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1316" t="n"/>
+      <c r="U3" s="1352" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -5054,43 +5180,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1321" t="inlineStr">
+      <c r="A4" s="1357" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1322" t="inlineStr">
+      <c r="B4" s="1358" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1322" t="inlineStr">
+      <c r="C4" s="1358" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1323" t="n"/>
-      <c r="E4" s="1323" t="n"/>
-      <c r="F4" s="1323" t="n"/>
-      <c r="G4" s="1323" t="n"/>
-      <c r="H4" s="1323" t="n"/>
-      <c r="I4" s="1324" t="n"/>
-      <c r="J4" s="1325" t="n"/>
-      <c r="K4" s="1325" t="n"/>
-      <c r="L4" s="1325" t="n"/>
-      <c r="M4" s="1323" t="n">
+      <c r="D4" s="1359" t="n"/>
+      <c r="E4" s="1359" t="n"/>
+      <c r="F4" s="1359" t="n"/>
+      <c r="G4" s="1359" t="n"/>
+      <c r="H4" s="1359" t="n"/>
+      <c r="I4" s="1360" t="n"/>
+      <c r="J4" s="1361" t="n"/>
+      <c r="K4" s="1361" t="n"/>
+      <c r="L4" s="1361" t="n"/>
+      <c r="M4" s="1359" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1323" t="n">
+      <c r="N4" s="1359" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1323" t="n"/>
-      <c r="P4" s="1326" t="n"/>
-      <c r="Q4" s="1323" t="n"/>
-      <c r="R4" s="1323" t="n"/>
-      <c r="S4" s="1323" t="n"/>
+      <c r="O4" s="1359" t="n"/>
+      <c r="P4" s="1362" t="n"/>
+      <c r="Q4" s="1359" t="n"/>
+      <c r="R4" s="1359" t="n"/>
+      <c r="S4" s="1359" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1322" t="n"/>
+      <c r="U4" s="1358" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -5098,57 +5224,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1327" t="inlineStr">
+      <c r="A5" s="1363" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1328" t="inlineStr">
+      <c r="B5" s="1364" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1328" t="inlineStr">
+      <c r="C5" s="1364" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1329" t="n">
+      <c r="D5" s="1365" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1329" t="n">
+      <c r="E5" s="1365" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1329" t="n">
+      <c r="F5" s="1365" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1329" t="n"/>
-      <c r="H5" s="1329" t="n"/>
-      <c r="I5" s="1330" t="n"/>
-      <c r="J5" s="1331" t="n">
+      <c r="G5" s="1365" t="n"/>
+      <c r="H5" s="1365" t="n"/>
+      <c r="I5" s="1366" t="n"/>
+      <c r="J5" s="1367" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1331" t="n">
+      <c r="K5" s="1367" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1331" t="inlineStr">
+      <c r="L5" s="1367" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1329" t="n"/>
-      <c r="N5" s="1329" t="n"/>
-      <c r="O5" s="1329" t="n">
+      <c r="M5" s="1365" t="n"/>
+      <c r="N5" s="1365" t="n"/>
+      <c r="O5" s="1365" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1332" t="n">
+      <c r="P5" s="1368" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1329" t="n"/>
-      <c r="R5" s="1329" t="n"/>
-      <c r="S5" s="1329" t="n"/>
+      <c r="Q5" s="1365" t="n"/>
+      <c r="R5" s="1365" t="n"/>
+      <c r="S5" s="1365" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1328" t="n"/>
+      <c r="U5" s="1364" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -5156,43 +5282,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1333" t="inlineStr">
+      <c r="A6" s="1369" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1334" t="inlineStr">
+      <c r="B6" s="1370" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1334" t="inlineStr">
+      <c r="C6" s="1370" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1335" t="n"/>
-      <c r="E6" s="1335" t="n"/>
-      <c r="F6" s="1335" t="n"/>
-      <c r="G6" s="1335" t="n"/>
-      <c r="H6" s="1335" t="n"/>
-      <c r="I6" s="1336" t="n"/>
-      <c r="J6" s="1337" t="n"/>
-      <c r="K6" s="1337" t="n"/>
-      <c r="L6" s="1337" t="n"/>
-      <c r="M6" s="1335" t="n">
+      <c r="D6" s="1371" t="n"/>
+      <c r="E6" s="1371" t="n"/>
+      <c r="F6" s="1371" t="n"/>
+      <c r="G6" s="1371" t="n"/>
+      <c r="H6" s="1371" t="n"/>
+      <c r="I6" s="1372" t="n"/>
+      <c r="J6" s="1373" t="n"/>
+      <c r="K6" s="1373" t="n"/>
+      <c r="L6" s="1373" t="n"/>
+      <c r="M6" s="1371" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1335" t="n">
+      <c r="N6" s="1371" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1335" t="n"/>
-      <c r="P6" s="1338" t="n"/>
-      <c r="Q6" s="1335" t="n"/>
-      <c r="R6" s="1335" t="n"/>
-      <c r="S6" s="1335" t="n"/>
+      <c r="O6" s="1371" t="n"/>
+      <c r="P6" s="1374" t="n"/>
+      <c r="Q6" s="1371" t="n"/>
+      <c r="R6" s="1371" t="n"/>
+      <c r="S6" s="1371" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1334" t="n"/>
+      <c r="U6" s="1370" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -5200,39 +5326,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1339" t="inlineStr">
+      <c r="A7" s="1375" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1340" t="inlineStr">
+      <c r="B7" s="1376" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1340" t="inlineStr">
+      <c r="C7" s="1376" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1341" t="n"/>
-      <c r="E7" s="1341" t="n"/>
-      <c r="F7" s="1341" t="n"/>
-      <c r="G7" s="1341" t="n"/>
-      <c r="H7" s="1341" t="n"/>
-      <c r="I7" s="1342" t="n"/>
-      <c r="J7" s="1343" t="n"/>
-      <c r="K7" s="1343" t="n"/>
-      <c r="L7" s="1343" t="n"/>
-      <c r="M7" s="1341" t="n"/>
-      <c r="N7" s="1341" t="n"/>
-      <c r="O7" s="1341" t="n"/>
-      <c r="P7" s="1344" t="n"/>
-      <c r="Q7" s="1341" t="n"/>
-      <c r="R7" s="1341" t="n"/>
-      <c r="S7" s="1341" t="n"/>
+      <c r="D7" s="1377" t="n"/>
+      <c r="E7" s="1377" t="n"/>
+      <c r="F7" s="1377" t="n"/>
+      <c r="G7" s="1377" t="n"/>
+      <c r="H7" s="1377" t="n"/>
+      <c r="I7" s="1378" t="n"/>
+      <c r="J7" s="1379" t="n"/>
+      <c r="K7" s="1379" t="n"/>
+      <c r="L7" s="1379" t="n"/>
+      <c r="M7" s="1377" t="n"/>
+      <c r="N7" s="1377" t="n"/>
+      <c r="O7" s="1377" t="n"/>
+      <c r="P7" s="1380" t="n"/>
+      <c r="Q7" s="1377" t="n"/>
+      <c r="R7" s="1377" t="n"/>
+      <c r="S7" s="1377" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1340" t="n"/>
+      <c r="U7" s="1376" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5240,39 +5366,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1315" t="inlineStr">
+      <c r="A8" s="1351" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1316" t="inlineStr">
+      <c r="B8" s="1352" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1316" t="inlineStr">
+      <c r="C8" s="1352" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1317" t="n"/>
-      <c r="E8" s="1317" t="n"/>
-      <c r="F8" s="1317" t="n"/>
-      <c r="G8" s="1317" t="n"/>
-      <c r="H8" s="1317" t="n"/>
-      <c r="I8" s="1318" t="n"/>
-      <c r="J8" s="1319" t="n"/>
-      <c r="K8" s="1319" t="n"/>
-      <c r="L8" s="1319" t="n"/>
-      <c r="M8" s="1317" t="n"/>
-      <c r="N8" s="1317" t="n"/>
-      <c r="O8" s="1317" t="n"/>
-      <c r="P8" s="1320" t="n"/>
-      <c r="Q8" s="1317" t="n"/>
-      <c r="R8" s="1317" t="n"/>
-      <c r="S8" s="1317" t="n"/>
+      <c r="D8" s="1353" t="n"/>
+      <c r="E8" s="1353" t="n"/>
+      <c r="F8" s="1353" t="n"/>
+      <c r="G8" s="1353" t="n"/>
+      <c r="H8" s="1353" t="n"/>
+      <c r="I8" s="1354" t="n"/>
+      <c r="J8" s="1355" t="n"/>
+      <c r="K8" s="1355" t="n"/>
+      <c r="L8" s="1355" t="n"/>
+      <c r="M8" s="1353" t="n"/>
+      <c r="N8" s="1353" t="n"/>
+      <c r="O8" s="1353" t="n"/>
+      <c r="P8" s="1356" t="n"/>
+      <c r="Q8" s="1353" t="n"/>
+      <c r="R8" s="1353" t="n"/>
+      <c r="S8" s="1353" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1316" t="n"/>
+      <c r="U8" s="1352" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -5280,63 +5406,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1345" t="inlineStr">
+      <c r="A9" s="1381" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1346" t="inlineStr">
+      <c r="B9" s="1382" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1346" t="inlineStr">
+      <c r="C9" s="1382" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1347" t="n">
+      <c r="D9" s="1383" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1347" t="n">
+      <c r="E9" s="1383" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1347" t="n">
+      <c r="F9" s="1383" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1347" t="n">
+      <c r="G9" s="1383" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1347" t="n"/>
-      <c r="I9" s="1348" t="n"/>
-      <c r="J9" s="1349" t="n">
+      <c r="H9" s="1383" t="n"/>
+      <c r="I9" s="1384" t="n"/>
+      <c r="J9" s="1385" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1349" t="n">
+      <c r="K9" s="1385" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1349" t="inlineStr">
+      <c r="L9" s="1385" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1347" t="n"/>
-      <c r="N9" s="1347" t="n"/>
-      <c r="O9" s="1347" t="n">
+      <c r="M9" s="1383" t="n"/>
+      <c r="N9" s="1383" t="n"/>
+      <c r="O9" s="1383" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1350" t="n">
+      <c r="P9" s="1386" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1347" t="n"/>
-      <c r="R9" s="1347" t="n"/>
-      <c r="S9" s="1347" t="n"/>
+      <c r="Q9" s="1383" t="n"/>
+      <c r="R9" s="1383" t="n"/>
+      <c r="S9" s="1383" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1346" t="n"/>
+      <c r="U9" s="1382" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -5344,43 +5470,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1345" t="inlineStr">
+      <c r="A10" s="1381" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1346" t="inlineStr">
+      <c r="B10" s="1382" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1346" t="inlineStr">
+      <c r="C10" s="1382" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1347" t="n"/>
-      <c r="E10" s="1347" t="n"/>
-      <c r="F10" s="1347" t="n"/>
-      <c r="G10" s="1347" t="n"/>
-      <c r="H10" s="1347" t="n"/>
-      <c r="I10" s="1348" t="n"/>
-      <c r="J10" s="1349" t="n"/>
-      <c r="K10" s="1349" t="n"/>
-      <c r="L10" s="1349" t="inlineStr">
+      <c r="D10" s="1383" t="n"/>
+      <c r="E10" s="1383" t="n"/>
+      <c r="F10" s="1383" t="n"/>
+      <c r="G10" s="1383" t="n"/>
+      <c r="H10" s="1383" t="n"/>
+      <c r="I10" s="1384" t="n"/>
+      <c r="J10" s="1385" t="n"/>
+      <c r="K10" s="1385" t="n"/>
+      <c r="L10" s="1385" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1347" t="n"/>
-      <c r="N10" s="1347" t="n"/>
-      <c r="O10" s="1347" t="n"/>
-      <c r="P10" s="1350" t="n"/>
-      <c r="Q10" s="1347" t="n"/>
-      <c r="R10" s="1347" t="n"/>
-      <c r="S10" s="1347" t="n"/>
+      <c r="M10" s="1383" t="n"/>
+      <c r="N10" s="1383" t="n"/>
+      <c r="O10" s="1383" t="n"/>
+      <c r="P10" s="1386" t="n"/>
+      <c r="Q10" s="1383" t="n"/>
+      <c r="R10" s="1383" t="n"/>
+      <c r="S10" s="1383" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1346" t="n"/>
+      <c r="U10" s="1382" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -5388,43 +5514,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1345" t="inlineStr">
+      <c r="A11" s="1381" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1346" t="inlineStr">
+      <c r="B11" s="1382" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1346" t="inlineStr">
+      <c r="C11" s="1382" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1347" t="n"/>
-      <c r="E11" s="1347" t="n"/>
-      <c r="F11" s="1347" t="n"/>
-      <c r="G11" s="1347" t="n"/>
-      <c r="H11" s="1347" t="n"/>
-      <c r="I11" s="1348" t="n"/>
-      <c r="J11" s="1349" t="n"/>
-      <c r="K11" s="1349" t="n"/>
-      <c r="L11" s="1349" t="n"/>
-      <c r="M11" s="1347" t="n">
+      <c r="D11" s="1383" t="n"/>
+      <c r="E11" s="1383" t="n"/>
+      <c r="F11" s="1383" t="n"/>
+      <c r="G11" s="1383" t="n"/>
+      <c r="H11" s="1383" t="n"/>
+      <c r="I11" s="1384" t="n"/>
+      <c r="J11" s="1385" t="n"/>
+      <c r="K11" s="1385" t="n"/>
+      <c r="L11" s="1385" t="n"/>
+      <c r="M11" s="1383" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1347" t="n">
+      <c r="N11" s="1383" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1347" t="n"/>
-      <c r="P11" s="1350" t="n"/>
-      <c r="Q11" s="1347" t="n"/>
-      <c r="R11" s="1347" t="n"/>
-      <c r="S11" s="1347" t="n"/>
+      <c r="O11" s="1383" t="n"/>
+      <c r="P11" s="1386" t="n"/>
+      <c r="Q11" s="1383" t="n"/>
+      <c r="R11" s="1383" t="n"/>
+      <c r="S11" s="1383" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1346" t="n"/>
+      <c r="U11" s="1382" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -5432,39 +5558,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1321" t="inlineStr">
+      <c r="A12" s="1357" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1322" t="inlineStr">
+      <c r="B12" s="1358" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1322" t="inlineStr">
+      <c r="C12" s="1358" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1323" t="n"/>
-      <c r="E12" s="1323" t="n"/>
-      <c r="F12" s="1323" t="n"/>
-      <c r="G12" s="1323" t="n"/>
-      <c r="H12" s="1323" t="n"/>
-      <c r="I12" s="1324" t="n"/>
-      <c r="J12" s="1325" t="n"/>
-      <c r="K12" s="1325" t="n"/>
-      <c r="L12" s="1325" t="n"/>
-      <c r="M12" s="1323" t="n"/>
-      <c r="N12" s="1323" t="n"/>
-      <c r="O12" s="1323" t="n"/>
-      <c r="P12" s="1326" t="n"/>
-      <c r="Q12" s="1323" t="n"/>
-      <c r="R12" s="1323" t="n"/>
-      <c r="S12" s="1323" t="n"/>
+      <c r="D12" s="1359" t="n"/>
+      <c r="E12" s="1359" t="n"/>
+      <c r="F12" s="1359" t="n"/>
+      <c r="G12" s="1359" t="n"/>
+      <c r="H12" s="1359" t="n"/>
+      <c r="I12" s="1360" t="n"/>
+      <c r="J12" s="1361" t="n"/>
+      <c r="K12" s="1361" t="n"/>
+      <c r="L12" s="1361" t="n"/>
+      <c r="M12" s="1359" t="n"/>
+      <c r="N12" s="1359" t="n"/>
+      <c r="O12" s="1359" t="n"/>
+      <c r="P12" s="1362" t="n"/>
+      <c r="Q12" s="1359" t="n"/>
+      <c r="R12" s="1359" t="n"/>
+      <c r="S12" s="1359" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1322" t="n"/>
+      <c r="U12" s="1358" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5472,35 +5598,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1327" t="inlineStr">
+      <c r="A13" s="1363" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1328" t="n"/>
-      <c r="C13" s="1328" t="inlineStr">
+      <c r="B13" s="1364" t="n"/>
+      <c r="C13" s="1364" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1329" t="n"/>
-      <c r="E13" s="1329" t="n"/>
-      <c r="F13" s="1329" t="n"/>
-      <c r="G13" s="1329" t="n"/>
-      <c r="H13" s="1329" t="n"/>
-      <c r="I13" s="1330" t="n"/>
-      <c r="J13" s="1331" t="n"/>
-      <c r="K13" s="1331" t="n"/>
-      <c r="L13" s="1331" t="n"/>
-      <c r="M13" s="1329" t="n"/>
-      <c r="N13" s="1329" t="n"/>
-      <c r="O13" s="1329" t="n"/>
-      <c r="P13" s="1332" t="n"/>
-      <c r="Q13" s="1329" t="n"/>
-      <c r="R13" s="1329" t="n"/>
-      <c r="S13" s="1329" t="n"/>
+      <c r="D13" s="1365" t="n"/>
+      <c r="E13" s="1365" t="n"/>
+      <c r="F13" s="1365" t="n"/>
+      <c r="G13" s="1365" t="n"/>
+      <c r="H13" s="1365" t="n"/>
+      <c r="I13" s="1366" t="n"/>
+      <c r="J13" s="1367" t="n"/>
+      <c r="K13" s="1367" t="n"/>
+      <c r="L13" s="1367" t="n"/>
+      <c r="M13" s="1365" t="n"/>
+      <c r="N13" s="1365" t="n"/>
+      <c r="O13" s="1365" t="n"/>
+      <c r="P13" s="1368" t="n"/>
+      <c r="Q13" s="1365" t="n"/>
+      <c r="R13" s="1365" t="n"/>
+      <c r="S13" s="1365" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1328" t="n"/>
+      <c r="U13" s="1364" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -5508,53 +5634,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1333" t="inlineStr">
+      <c r="A14" s="1369" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1334" t="inlineStr">
+      <c r="B14" s="1370" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1334" t="inlineStr">
+      <c r="C14" s="1370" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1335" t="n"/>
-      <c r="E14" s="1335" t="n">
+      <c r="D14" s="1371" t="n"/>
+      <c r="E14" s="1371" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1335" t="n">
+      <c r="F14" s="1371" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1335" t="n">
+      <c r="G14" s="1371" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1335" t="n"/>
-      <c r="I14" s="1336" t="n"/>
-      <c r="J14" s="1337" t="n"/>
-      <c r="K14" s="1337" t="n"/>
-      <c r="L14" s="1337" t="n"/>
-      <c r="M14" s="1335" t="n"/>
-      <c r="N14" s="1335" t="n"/>
-      <c r="O14" s="1335" t="n">
+      <c r="H14" s="1371" t="n"/>
+      <c r="I14" s="1372" t="n"/>
+      <c r="J14" s="1373" t="n"/>
+      <c r="K14" s="1373" t="n"/>
+      <c r="L14" s="1373" t="n"/>
+      <c r="M14" s="1371" t="n"/>
+      <c r="N14" s="1371" t="n"/>
+      <c r="O14" s="1371" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1338" t="n">
+      <c r="P14" s="1374" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1335" t="n"/>
-      <c r="R14" s="1335" t="n"/>
-      <c r="S14" s="1335" t="n"/>
+      <c r="Q14" s="1371" t="n"/>
+      <c r="R14" s="1371" t="n"/>
+      <c r="S14" s="1371" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1334" t="n"/>
+      <c r="U14" s="1370" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -5562,43 +5688,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1333" t="inlineStr">
+      <c r="A15" s="1369" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1334" t="inlineStr">
+      <c r="B15" s="1370" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1334" t="inlineStr">
+      <c r="C15" s="1370" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1335" t="n"/>
-      <c r="E15" s="1335" t="n"/>
-      <c r="F15" s="1335" t="n"/>
-      <c r="G15" s="1335" t="n"/>
-      <c r="H15" s="1335" t="n"/>
-      <c r="I15" s="1336" t="n"/>
-      <c r="J15" s="1337" t="n"/>
-      <c r="K15" s="1337" t="n"/>
-      <c r="L15" s="1337" t="n"/>
-      <c r="M15" s="1335" t="n">
+      <c r="D15" s="1371" t="n"/>
+      <c r="E15" s="1371" t="n"/>
+      <c r="F15" s="1371" t="n"/>
+      <c r="G15" s="1371" t="n"/>
+      <c r="H15" s="1371" t="n"/>
+      <c r="I15" s="1372" t="n"/>
+      <c r="J15" s="1373" t="n"/>
+      <c r="K15" s="1373" t="n"/>
+      <c r="L15" s="1373" t="n"/>
+      <c r="M15" s="1371" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1335" t="n">
+      <c r="N15" s="1371" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1335" t="n"/>
-      <c r="P15" s="1338" t="n"/>
-      <c r="Q15" s="1335" t="n"/>
-      <c r="R15" s="1335" t="n"/>
-      <c r="S15" s="1335" t="n"/>
+      <c r="O15" s="1371" t="n"/>
+      <c r="P15" s="1374" t="n"/>
+      <c r="Q15" s="1371" t="n"/>
+      <c r="R15" s="1371" t="n"/>
+      <c r="S15" s="1371" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1334" t="n"/>
+      <c r="U15" s="1370" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -5606,39 +5732,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1339" t="inlineStr">
+      <c r="A16" s="1375" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1340" t="inlineStr">
+      <c r="B16" s="1376" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1340" t="inlineStr">
+      <c r="C16" s="1376" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1341" t="n"/>
-      <c r="E16" s="1341" t="n"/>
-      <c r="F16" s="1341" t="n"/>
-      <c r="G16" s="1341" t="n"/>
-      <c r="H16" s="1341" t="n"/>
-      <c r="I16" s="1342" t="n"/>
-      <c r="J16" s="1343" t="n"/>
-      <c r="K16" s="1343" t="n"/>
-      <c r="L16" s="1343" t="n"/>
-      <c r="M16" s="1341" t="n"/>
-      <c r="N16" s="1341" t="n"/>
-      <c r="O16" s="1341" t="n"/>
-      <c r="P16" s="1344" t="n"/>
-      <c r="Q16" s="1341" t="n"/>
-      <c r="R16" s="1341" t="n"/>
-      <c r="S16" s="1341" t="n"/>
+      <c r="D16" s="1377" t="n"/>
+      <c r="E16" s="1377" t="n"/>
+      <c r="F16" s="1377" t="n"/>
+      <c r="G16" s="1377" t="n"/>
+      <c r="H16" s="1377" t="n"/>
+      <c r="I16" s="1378" t="n"/>
+      <c r="J16" s="1379" t="n"/>
+      <c r="K16" s="1379" t="n"/>
+      <c r="L16" s="1379" t="n"/>
+      <c r="M16" s="1377" t="n"/>
+      <c r="N16" s="1377" t="n"/>
+      <c r="O16" s="1377" t="n"/>
+      <c r="P16" s="1380" t="n"/>
+      <c r="Q16" s="1377" t="n"/>
+      <c r="R16" s="1377" t="n"/>
+      <c r="S16" s="1377" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1340" t="n"/>
+      <c r="U16" s="1376" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -5646,39 +5772,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1315" t="inlineStr">
+      <c r="A17" s="1351" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1316" t="inlineStr">
+      <c r="B17" s="1352" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1316" t="inlineStr">
+      <c r="C17" s="1352" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1317" t="n"/>
-      <c r="E17" s="1317" t="n"/>
-      <c r="F17" s="1317" t="n"/>
-      <c r="G17" s="1317" t="n"/>
-      <c r="H17" s="1317" t="n"/>
-      <c r="I17" s="1318" t="n"/>
-      <c r="J17" s="1319" t="n"/>
-      <c r="K17" s="1319" t="n"/>
-      <c r="L17" s="1319" t="n"/>
-      <c r="M17" s="1317" t="n"/>
-      <c r="N17" s="1317" t="n"/>
-      <c r="O17" s="1317" t="n"/>
-      <c r="P17" s="1320" t="n"/>
-      <c r="Q17" s="1317" t="n"/>
-      <c r="R17" s="1317" t="n"/>
-      <c r="S17" s="1317" t="n"/>
+      <c r="D17" s="1353" t="n"/>
+      <c r="E17" s="1353" t="n"/>
+      <c r="F17" s="1353" t="n"/>
+      <c r="G17" s="1353" t="n"/>
+      <c r="H17" s="1353" t="n"/>
+      <c r="I17" s="1354" t="n"/>
+      <c r="J17" s="1355" t="n"/>
+      <c r="K17" s="1355" t="n"/>
+      <c r="L17" s="1355" t="n"/>
+      <c r="M17" s="1353" t="n"/>
+      <c r="N17" s="1353" t="n"/>
+      <c r="O17" s="1353" t="n"/>
+      <c r="P17" s="1356" t="n"/>
+      <c r="Q17" s="1353" t="n"/>
+      <c r="R17" s="1353" t="n"/>
+      <c r="S17" s="1353" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1316" t="n"/>
+      <c r="U17" s="1352" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -5686,53 +5812,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1345" t="inlineStr">
+      <c r="A18" s="1381" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1346" t="inlineStr">
+      <c r="B18" s="1382" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1346" t="inlineStr">
+      <c r="C18" s="1382" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1347" t="n"/>
-      <c r="E18" s="1347" t="n">
+      <c r="D18" s="1383" t="n"/>
+      <c r="E18" s="1383" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1347" t="n">
+      <c r="F18" s="1383" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1347" t="n">
+      <c r="G18" s="1383" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1347" t="n"/>
-      <c r="I18" s="1348" t="n"/>
-      <c r="J18" s="1349" t="n"/>
-      <c r="K18" s="1349" t="n"/>
-      <c r="L18" s="1349" t="n"/>
-      <c r="M18" s="1347" t="n"/>
-      <c r="N18" s="1347" t="n"/>
-      <c r="O18" s="1347" t="n">
+      <c r="H18" s="1383" t="n"/>
+      <c r="I18" s="1384" t="n"/>
+      <c r="J18" s="1385" t="n"/>
+      <c r="K18" s="1385" t="n"/>
+      <c r="L18" s="1385" t="n"/>
+      <c r="M18" s="1383" t="n"/>
+      <c r="N18" s="1383" t="n"/>
+      <c r="O18" s="1383" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1350" t="n">
+      <c r="P18" s="1386" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1347" t="n"/>
-      <c r="R18" s="1347" t="n"/>
-      <c r="S18" s="1347" t="n"/>
+      <c r="Q18" s="1383" t="n"/>
+      <c r="R18" s="1383" t="n"/>
+      <c r="S18" s="1383" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1346" t="n"/>
+      <c r="U18" s="1382" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -5740,47 +5866,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1345" t="inlineStr">
+      <c r="A19" s="1381" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1346" t="inlineStr">
+      <c r="B19" s="1382" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1346" t="inlineStr">
+      <c r="C19" s="1382" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1347" t="n"/>
-      <c r="E19" s="1347" t="n"/>
-      <c r="F19" s="1347" t="n"/>
-      <c r="G19" s="1347" t="n"/>
-      <c r="H19" s="1347" t="n"/>
-      <c r="I19" s="1348" t="n"/>
-      <c r="J19" s="1349" t="n"/>
-      <c r="K19" s="1349" t="n"/>
-      <c r="L19" s="1349" t="n"/>
-      <c r="M19" s="1347" t="n">
+      <c r="D19" s="1383" t="n"/>
+      <c r="E19" s="1383" t="n"/>
+      <c r="F19" s="1383" t="n"/>
+      <c r="G19" s="1383" t="n"/>
+      <c r="H19" s="1383" t="n"/>
+      <c r="I19" s="1384" t="n"/>
+      <c r="J19" s="1385" t="n"/>
+      <c r="K19" s="1385" t="n"/>
+      <c r="L19" s="1385" t="n"/>
+      <c r="M19" s="1383" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1347" t="n">
+      <c r="N19" s="1383" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1347" t="n"/>
-      <c r="P19" s="1350" t="n"/>
-      <c r="Q19" s="1347" t="n"/>
-      <c r="R19" s="1347" t="n"/>
-      <c r="S19" s="1347" t="n"/>
+      <c r="O19" s="1383" t="n"/>
+      <c r="P19" s="1386" t="n"/>
+      <c r="Q19" s="1383" t="n"/>
+      <c r="R19" s="1383" t="n"/>
+      <c r="S19" s="1383" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1346" t="n"/>
+      <c r="U19" s="1382" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -5788,43 +5914,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1345" t="inlineStr">
+      <c r="A20" s="1381" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1346" t="inlineStr">
+      <c r="B20" s="1382" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1346" t="inlineStr">
+      <c r="C20" s="1382" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1347" t="n"/>
-      <c r="E20" s="1347" t="n"/>
-      <c r="F20" s="1347" t="n"/>
-      <c r="G20" s="1347" t="n"/>
-      <c r="H20" s="1347" t="n"/>
-      <c r="I20" s="1348" t="n"/>
-      <c r="J20" s="1349" t="n"/>
-      <c r="K20" s="1349" t="n"/>
-      <c r="L20" s="1349" t="n"/>
-      <c r="M20" s="1347" t="n"/>
-      <c r="N20" s="1347" t="n"/>
-      <c r="O20" s="1347" t="n"/>
-      <c r="P20" s="1350" t="n"/>
-      <c r="Q20" s="1347" t="n"/>
-      <c r="R20" s="1347" t="n"/>
-      <c r="S20" s="1347" t="n"/>
+      <c r="D20" s="1383" t="n"/>
+      <c r="E20" s="1383" t="n"/>
+      <c r="F20" s="1383" t="n"/>
+      <c r="G20" s="1383" t="n"/>
+      <c r="H20" s="1383" t="n"/>
+      <c r="I20" s="1384" t="n"/>
+      <c r="J20" s="1385" t="n"/>
+      <c r="K20" s="1385" t="n"/>
+      <c r="L20" s="1385" t="n"/>
+      <c r="M20" s="1383" t="n"/>
+      <c r="N20" s="1383" t="n"/>
+      <c r="O20" s="1383" t="n"/>
+      <c r="P20" s="1386" t="n"/>
+      <c r="Q20" s="1383" t="n"/>
+      <c r="R20" s="1383" t="n"/>
+      <c r="S20" s="1383" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1346" t="n"/>
+      <c r="U20" s="1382" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -5832,39 +5958,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1321" t="inlineStr">
+      <c r="A21" s="1357" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1322" t="inlineStr">
+      <c r="B21" s="1358" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1322" t="inlineStr">
+      <c r="C21" s="1358" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1323" t="n"/>
-      <c r="E21" s="1323" t="n"/>
-      <c r="F21" s="1323" t="n"/>
-      <c r="G21" s="1323" t="n"/>
-      <c r="H21" s="1323" t="n"/>
-      <c r="I21" s="1324" t="n"/>
-      <c r="J21" s="1325" t="n"/>
-      <c r="K21" s="1325" t="n"/>
-      <c r="L21" s="1325" t="n"/>
-      <c r="M21" s="1323" t="n"/>
-      <c r="N21" s="1323" t="n"/>
-      <c r="O21" s="1323" t="n"/>
-      <c r="P21" s="1326" t="n"/>
-      <c r="Q21" s="1323" t="n"/>
-      <c r="R21" s="1323" t="n"/>
-      <c r="S21" s="1323" t="n"/>
+      <c r="D21" s="1359" t="n"/>
+      <c r="E21" s="1359" t="n"/>
+      <c r="F21" s="1359" t="n"/>
+      <c r="G21" s="1359" t="n"/>
+      <c r="H21" s="1359" t="n"/>
+      <c r="I21" s="1360" t="n"/>
+      <c r="J21" s="1361" t="n"/>
+      <c r="K21" s="1361" t="n"/>
+      <c r="L21" s="1361" t="n"/>
+      <c r="M21" s="1359" t="n"/>
+      <c r="N21" s="1359" t="n"/>
+      <c r="O21" s="1359" t="n"/>
+      <c r="P21" s="1362" t="n"/>
+      <c r="Q21" s="1359" t="n"/>
+      <c r="R21" s="1359" t="n"/>
+      <c r="S21" s="1359" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1322" t="n"/>
+      <c r="U21" s="1358" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -5872,39 +5998,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1327" t="inlineStr">
+      <c r="A22" s="1363" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1328" t="inlineStr">
+      <c r="B22" s="1364" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1328" t="inlineStr">
+      <c r="C22" s="1364" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1329" t="n"/>
-      <c r="E22" s="1329" t="n"/>
-      <c r="F22" s="1329" t="n"/>
-      <c r="G22" s="1329" t="n"/>
-      <c r="H22" s="1329" t="n"/>
-      <c r="I22" s="1330" t="n"/>
-      <c r="J22" s="1331" t="n"/>
-      <c r="K22" s="1331" t="n"/>
-      <c r="L22" s="1331" t="n"/>
-      <c r="M22" s="1329" t="n"/>
-      <c r="N22" s="1329" t="n"/>
-      <c r="O22" s="1329" t="n"/>
-      <c r="P22" s="1332" t="n"/>
-      <c r="Q22" s="1329" t="n"/>
-      <c r="R22" s="1329" t="n"/>
-      <c r="S22" s="1329" t="n"/>
+      <c r="D22" s="1365" t="n"/>
+      <c r="E22" s="1365" t="n"/>
+      <c r="F22" s="1365" t="n"/>
+      <c r="G22" s="1365" t="n"/>
+      <c r="H22" s="1365" t="n"/>
+      <c r="I22" s="1366" t="n"/>
+      <c r="J22" s="1367" t="n"/>
+      <c r="K22" s="1367" t="n"/>
+      <c r="L22" s="1367" t="n"/>
+      <c r="M22" s="1365" t="n"/>
+      <c r="N22" s="1365" t="n"/>
+      <c r="O22" s="1365" t="n"/>
+      <c r="P22" s="1368" t="n"/>
+      <c r="Q22" s="1365" t="n"/>
+      <c r="R22" s="1365" t="n"/>
+      <c r="S22" s="1365" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1328" t="n"/>
+      <c r="U22" s="1364" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -5912,53 +6038,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1333" t="inlineStr">
+      <c r="A23" s="1369" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1334" t="inlineStr">
+      <c r="B23" s="1370" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1334" t="inlineStr">
+      <c r="C23" s="1370" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1335" t="n"/>
-      <c r="E23" s="1335" t="n">
+      <c r="D23" s="1371" t="n"/>
+      <c r="E23" s="1371" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1335" t="n">
+      <c r="F23" s="1371" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1335" t="n">
+      <c r="G23" s="1371" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1335" t="n"/>
-      <c r="I23" s="1336" t="n"/>
-      <c r="J23" s="1337" t="n"/>
-      <c r="K23" s="1337" t="n"/>
-      <c r="L23" s="1337" t="n"/>
-      <c r="M23" s="1335" t="n"/>
-      <c r="N23" s="1335" t="n"/>
-      <c r="O23" s="1335" t="n">
+      <c r="H23" s="1371" t="n"/>
+      <c r="I23" s="1372" t="n"/>
+      <c r="J23" s="1373" t="n"/>
+      <c r="K23" s="1373" t="n"/>
+      <c r="L23" s="1373" t="n"/>
+      <c r="M23" s="1371" t="n"/>
+      <c r="N23" s="1371" t="n"/>
+      <c r="O23" s="1371" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1338" t="n">
+      <c r="P23" s="1374" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1335" t="n"/>
-      <c r="R23" s="1335" t="n"/>
-      <c r="S23" s="1335" t="n"/>
+      <c r="Q23" s="1371" t="n"/>
+      <c r="R23" s="1371" t="n"/>
+      <c r="S23" s="1371" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1334" t="n"/>
+      <c r="U23" s="1370" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -5966,47 +6092,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1339" t="inlineStr">
+      <c r="A24" s="1375" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1340" t="inlineStr">
+      <c r="B24" s="1376" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1340" t="inlineStr">
+      <c r="C24" s="1376" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1341" t="n"/>
-      <c r="E24" s="1341" t="n"/>
-      <c r="F24" s="1341" t="n"/>
-      <c r="G24" s="1341" t="n"/>
-      <c r="H24" s="1341" t="n"/>
-      <c r="I24" s="1342" t="n"/>
-      <c r="J24" s="1343" t="n"/>
-      <c r="K24" s="1343" t="n"/>
-      <c r="L24" s="1343" t="n"/>
-      <c r="M24" s="1341" t="n">
+      <c r="D24" s="1377" t="n"/>
+      <c r="E24" s="1377" t="n"/>
+      <c r="F24" s="1377" t="n"/>
+      <c r="G24" s="1377" t="n"/>
+      <c r="H24" s="1377" t="n"/>
+      <c r="I24" s="1378" t="n"/>
+      <c r="J24" s="1379" t="n"/>
+      <c r="K24" s="1379" t="n"/>
+      <c r="L24" s="1379" t="n"/>
+      <c r="M24" s="1377" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1341" t="n">
+      <c r="N24" s="1377" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1341" t="n"/>
-      <c r="P24" s="1344" t="n"/>
-      <c r="Q24" s="1341" t="n"/>
-      <c r="R24" s="1341" t="n"/>
-      <c r="S24" s="1341" t="n"/>
+      <c r="O24" s="1377" t="n"/>
+      <c r="P24" s="1380" t="n"/>
+      <c r="Q24" s="1377" t="n"/>
+      <c r="R24" s="1377" t="n"/>
+      <c r="S24" s="1377" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1340" t="n"/>
+      <c r="U24" s="1376" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -6014,61 +6140,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1315" t="inlineStr">
+      <c r="A25" s="1351" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1316" t="inlineStr">
+      <c r="B25" s="1352" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1316" t="inlineStr">
+      <c r="C25" s="1352" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1317" t="n">
+      <c r="D25" s="1353" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1317" t="n">
+      <c r="E25" s="1353" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1317" t="n">
+      <c r="F25" s="1353" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1317" t="n">
+      <c r="G25" s="1353" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1317" t="n"/>
-      <c r="I25" s="1318" t="n"/>
-      <c r="J25" s="1319" t="n">
+      <c r="H25" s="1353" t="n"/>
+      <c r="I25" s="1354" t="n"/>
+      <c r="J25" s="1355" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1319" t="n">
+      <c r="K25" s="1355" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1319" t="n">
+      <c r="L25" s="1355" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1317" t="n"/>
-      <c r="N25" s="1317" t="n"/>
-      <c r="O25" s="1317" t="n">
+      <c r="M25" s="1353" t="n"/>
+      <c r="N25" s="1353" t="n"/>
+      <c r="O25" s="1353" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1320" t="n">
+      <c r="P25" s="1356" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1317" t="n"/>
-      <c r="R25" s="1317" t="n"/>
-      <c r="S25" s="1317" t="n"/>
+      <c r="Q25" s="1353" t="n"/>
+      <c r="R25" s="1353" t="n"/>
+      <c r="S25" s="1353" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1316" t="n"/>
+      <c r="U25" s="1352" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -6076,47 +6202,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1321" t="inlineStr">
+      <c r="A26" s="1357" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1322" t="inlineStr">
+      <c r="B26" s="1358" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1322" t="inlineStr">
+      <c r="C26" s="1358" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1323" t="n"/>
-      <c r="E26" s="1323" t="n"/>
-      <c r="F26" s="1323" t="n"/>
-      <c r="G26" s="1323" t="n"/>
-      <c r="H26" s="1323" t="n"/>
-      <c r="I26" s="1324" t="n"/>
-      <c r="J26" s="1325" t="n"/>
-      <c r="K26" s="1325" t="n"/>
-      <c r="L26" s="1325" t="n"/>
-      <c r="M26" s="1323" t="n">
+      <c r="D26" s="1359" t="n"/>
+      <c r="E26" s="1359" t="n"/>
+      <c r="F26" s="1359" t="n"/>
+      <c r="G26" s="1359" t="n"/>
+      <c r="H26" s="1359" t="n"/>
+      <c r="I26" s="1360" t="n"/>
+      <c r="J26" s="1361" t="n"/>
+      <c r="K26" s="1361" t="n"/>
+      <c r="L26" s="1361" t="n"/>
+      <c r="M26" s="1359" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1323" t="n">
+      <c r="N26" s="1359" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1323" t="n"/>
-      <c r="P26" s="1326" t="n"/>
-      <c r="Q26" s="1323" t="n"/>
-      <c r="R26" s="1323" t="n"/>
-      <c r="S26" s="1323" t="n"/>
+      <c r="O26" s="1359" t="n"/>
+      <c r="P26" s="1362" t="n"/>
+      <c r="Q26" s="1359" t="n"/>
+      <c r="R26" s="1359" t="n"/>
+      <c r="S26" s="1359" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1322" t="n"/>
+      <c r="U26" s="1358" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -6124,53 +6250,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1327" t="inlineStr">
+      <c r="A27" s="1363" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1328" t="inlineStr">
+      <c r="B27" s="1364" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1328" t="inlineStr">
+      <c r="C27" s="1364" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1329" t="n"/>
-      <c r="E27" s="1329" t="n">
+      <c r="D27" s="1365" t="n"/>
+      <c r="E27" s="1365" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1329" t="n">
+      <c r="F27" s="1365" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1329" t="n">
+      <c r="G27" s="1365" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1329" t="n"/>
-      <c r="I27" s="1330" t="n"/>
-      <c r="J27" s="1331" t="n"/>
-      <c r="K27" s="1331" t="n"/>
-      <c r="L27" s="1331" t="n"/>
-      <c r="M27" s="1329" t="n"/>
-      <c r="N27" s="1329" t="n"/>
-      <c r="O27" s="1329" t="n">
+      <c r="H27" s="1365" t="n"/>
+      <c r="I27" s="1366" t="n"/>
+      <c r="J27" s="1367" t="n"/>
+      <c r="K27" s="1367" t="n"/>
+      <c r="L27" s="1367" t="n"/>
+      <c r="M27" s="1365" t="n"/>
+      <c r="N27" s="1365" t="n"/>
+      <c r="O27" s="1365" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1332" t="n">
+      <c r="P27" s="1368" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1329" t="n"/>
-      <c r="R27" s="1329" t="n"/>
-      <c r="S27" s="1329" t="n"/>
+      <c r="Q27" s="1365" t="n"/>
+      <c r="R27" s="1365" t="n"/>
+      <c r="S27" s="1365" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1328" t="n"/>
+      <c r="U27" s="1364" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -6178,47 +6304,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1339" t="inlineStr">
+      <c r="A28" s="1375" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1340" t="inlineStr">
+      <c r="B28" s="1376" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1340" t="inlineStr">
+      <c r="C28" s="1376" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1341" t="n"/>
-      <c r="E28" s="1341" t="n"/>
-      <c r="F28" s="1341" t="n"/>
-      <c r="G28" s="1341" t="n"/>
-      <c r="H28" s="1341" t="n"/>
-      <c r="I28" s="1342" t="n"/>
-      <c r="J28" s="1343" t="n"/>
-      <c r="K28" s="1343" t="n"/>
-      <c r="L28" s="1343" t="n"/>
-      <c r="M28" s="1341" t="n">
+      <c r="D28" s="1377" t="n"/>
+      <c r="E28" s="1377" t="n"/>
+      <c r="F28" s="1377" t="n"/>
+      <c r="G28" s="1377" t="n"/>
+      <c r="H28" s="1377" t="n"/>
+      <c r="I28" s="1378" t="n"/>
+      <c r="J28" s="1379" t="n"/>
+      <c r="K28" s="1379" t="n"/>
+      <c r="L28" s="1379" t="n"/>
+      <c r="M28" s="1377" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1341" t="n">
+      <c r="N28" s="1377" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1341" t="n"/>
-      <c r="P28" s="1344" t="n"/>
-      <c r="Q28" s="1341" t="n"/>
-      <c r="R28" s="1341" t="n"/>
-      <c r="S28" s="1341" t="n"/>
+      <c r="O28" s="1377" t="n"/>
+      <c r="P28" s="1380" t="n"/>
+      <c r="Q28" s="1377" t="n"/>
+      <c r="R28" s="1377" t="n"/>
+      <c r="S28" s="1377" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1340" t="n"/>
+      <c r="U28" s="1376" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -6226,53 +6352,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1315" t="inlineStr">
+      <c r="A29" s="1351" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1316" t="inlineStr">
+      <c r="B29" s="1352" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1316" t="inlineStr">
+      <c r="C29" s="1352" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1317" t="n"/>
-      <c r="E29" s="1317" t="n">
+      <c r="D29" s="1353" t="n"/>
+      <c r="E29" s="1353" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1317" t="n">
+      <c r="F29" s="1353" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1317" t="n">
+      <c r="G29" s="1353" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1317" t="n"/>
-      <c r="I29" s="1318" t="n"/>
-      <c r="J29" s="1319" t="n"/>
-      <c r="K29" s="1319" t="n"/>
-      <c r="L29" s="1319" t="n"/>
-      <c r="M29" s="1317" t="n"/>
-      <c r="N29" s="1317" t="n"/>
-      <c r="O29" s="1317" t="n">
+      <c r="H29" s="1353" t="n"/>
+      <c r="I29" s="1354" t="n"/>
+      <c r="J29" s="1355" t="n"/>
+      <c r="K29" s="1355" t="n"/>
+      <c r="L29" s="1355" t="n"/>
+      <c r="M29" s="1353" t="n"/>
+      <c r="N29" s="1353" t="n"/>
+      <c r="O29" s="1353" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1320" t="n">
+      <c r="P29" s="1356" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1317" t="n"/>
-      <c r="R29" s="1317" t="n"/>
-      <c r="S29" s="1317" t="n"/>
+      <c r="Q29" s="1353" t="n"/>
+      <c r="R29" s="1353" t="n"/>
+      <c r="S29" s="1353" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1316" t="n"/>
+      <c r="U29" s="1352" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -6280,43 +6406,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1321" t="inlineStr">
+      <c r="A30" s="1357" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1322" t="inlineStr">
+      <c r="B30" s="1358" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1322" t="inlineStr">
+      <c r="C30" s="1358" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1323" t="n"/>
-      <c r="E30" s="1323" t="n"/>
-      <c r="F30" s="1323" t="n"/>
-      <c r="G30" s="1323" t="n"/>
-      <c r="H30" s="1323" t="n"/>
-      <c r="I30" s="1324" t="n"/>
-      <c r="J30" s="1325" t="n"/>
-      <c r="K30" s="1325" t="n"/>
-      <c r="L30" s="1325" t="n"/>
-      <c r="M30" s="1323" t="n"/>
-      <c r="N30" s="1323" t="n"/>
-      <c r="O30" s="1323" t="n"/>
-      <c r="P30" s="1326" t="n"/>
-      <c r="Q30" s="1323" t="n"/>
-      <c r="R30" s="1323" t="n"/>
-      <c r="S30" s="1323" t="n"/>
+      <c r="D30" s="1359" t="n"/>
+      <c r="E30" s="1359" t="n"/>
+      <c r="F30" s="1359" t="n"/>
+      <c r="G30" s="1359" t="n"/>
+      <c r="H30" s="1359" t="n"/>
+      <c r="I30" s="1360" t="n"/>
+      <c r="J30" s="1361" t="n"/>
+      <c r="K30" s="1361" t="n"/>
+      <c r="L30" s="1361" t="n"/>
+      <c r="M30" s="1359" t="n"/>
+      <c r="N30" s="1359" t="n"/>
+      <c r="O30" s="1359" t="n"/>
+      <c r="P30" s="1362" t="n"/>
+      <c r="Q30" s="1359" t="n"/>
+      <c r="R30" s="1359" t="n"/>
+      <c r="S30" s="1359" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1322" t="n"/>
+      <c r="U30" s="1358" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -6324,53 +6450,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1327" t="inlineStr">
+      <c r="A31" s="1363" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1328" t="inlineStr">
+      <c r="B31" s="1364" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1328" t="inlineStr">
+      <c r="C31" s="1364" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1329" t="n"/>
-      <c r="E31" s="1329" t="n">
+      <c r="D31" s="1365" t="n"/>
+      <c r="E31" s="1365" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1329" t="n">
+      <c r="F31" s="1365" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1329" t="n">
+      <c r="G31" s="1365" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1329" t="n"/>
-      <c r="I31" s="1330" t="n"/>
-      <c r="J31" s="1331" t="n"/>
-      <c r="K31" s="1331" t="n"/>
-      <c r="L31" s="1331" t="n"/>
-      <c r="M31" s="1329" t="n"/>
-      <c r="N31" s="1329" t="n"/>
-      <c r="O31" s="1329" t="n">
+      <c r="H31" s="1365" t="n"/>
+      <c r="I31" s="1366" t="n"/>
+      <c r="J31" s="1367" t="n"/>
+      <c r="K31" s="1367" t="n"/>
+      <c r="L31" s="1367" t="n"/>
+      <c r="M31" s="1365" t="n"/>
+      <c r="N31" s="1365" t="n"/>
+      <c r="O31" s="1365" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1332" t="n">
+      <c r="P31" s="1368" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1329" t="n"/>
-      <c r="R31" s="1329" t="n"/>
-      <c r="S31" s="1329" t="n"/>
+      <c r="Q31" s="1365" t="n"/>
+      <c r="R31" s="1365" t="n"/>
+      <c r="S31" s="1365" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1328" t="inlineStr">
+      <c r="U31" s="1364" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -6382,49 +6508,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1339" t="inlineStr">
+      <c r="A32" s="1375" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1340" t="inlineStr">
+      <c r="B32" s="1376" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1340" t="inlineStr">
+      <c r="C32" s="1376" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1341" t="n"/>
-      <c r="E32" s="1341" t="n"/>
-      <c r="F32" s="1341" t="n"/>
-      <c r="G32" s="1341" t="n"/>
-      <c r="H32" s="1341" t="n">
+      <c r="D32" s="1377" t="n"/>
+      <c r="E32" s="1377" t="n"/>
+      <c r="F32" s="1377" t="n"/>
+      <c r="G32" s="1377" t="n"/>
+      <c r="H32" s="1377" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1342" t="n"/>
-      <c r="J32" s="1343" t="n"/>
-      <c r="K32" s="1343" t="n"/>
-      <c r="L32" s="1343" t="n"/>
-      <c r="M32" s="1341" t="n">
+      <c r="I32" s="1378" t="n"/>
+      <c r="J32" s="1379" t="n"/>
+      <c r="K32" s="1379" t="n"/>
+      <c r="L32" s="1379" t="n"/>
+      <c r="M32" s="1377" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1341" t="n">
+      <c r="N32" s="1377" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1341" t="n"/>
-      <c r="P32" s="1344" t="n"/>
-      <c r="Q32" s="1341" t="n"/>
-      <c r="R32" s="1341" t="n"/>
-      <c r="S32" s="1341" t="n"/>
+      <c r="O32" s="1377" t="n"/>
+      <c r="P32" s="1380" t="n"/>
+      <c r="Q32" s="1377" t="n"/>
+      <c r="R32" s="1377" t="n"/>
+      <c r="S32" s="1377" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1340" t="n"/>
+      <c r="U32" s="1376" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -6432,57 +6558,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1315" t="inlineStr">
+      <c r="A33" s="1351" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1316" t="inlineStr">
+      <c r="B33" s="1352" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1316" t="inlineStr">
+      <c r="C33" s="1352" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1317" t="n"/>
-      <c r="E33" s="1317" t="n">
+      <c r="D33" s="1353" t="n"/>
+      <c r="E33" s="1353" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1317" t="n">
+      <c r="F33" s="1353" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1317" t="n">
+      <c r="G33" s="1353" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1317" t="n"/>
-      <c r="I33" s="1318" t="n">
+      <c r="H33" s="1353" t="n"/>
+      <c r="I33" s="1354" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1319" t="n"/>
-      <c r="K33" s="1319" t="n"/>
-      <c r="L33" s="1319" t="n"/>
-      <c r="M33" s="1317" t="n"/>
-      <c r="N33" s="1317" t="n"/>
-      <c r="O33" s="1317" t="n">
+      <c r="J33" s="1355" t="n"/>
+      <c r="K33" s="1355" t="n"/>
+      <c r="L33" s="1355" t="n"/>
+      <c r="M33" s="1353" t="n"/>
+      <c r="N33" s="1353" t="n"/>
+      <c r="O33" s="1353" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1320" t="n">
+      <c r="P33" s="1356" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1317" t="n"/>
-      <c r="R33" s="1317" t="n">
+      <c r="Q33" s="1353" t="n"/>
+      <c r="R33" s="1353" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1317" t="n"/>
+      <c r="S33" s="1353" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1316" t="inlineStr">
+      <c r="U33" s="1352" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -6494,49 +6620,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1321" t="inlineStr">
+      <c r="A34" s="1357" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1322" t="inlineStr">
+      <c r="B34" s="1358" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1322" t="inlineStr">
+      <c r="C34" s="1358" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1323" t="n"/>
-      <c r="E34" s="1323" t="n"/>
-      <c r="F34" s="1323" t="n"/>
-      <c r="G34" s="1323" t="n"/>
-      <c r="H34" s="1323" t="n">
+      <c r="D34" s="1359" t="n"/>
+      <c r="E34" s="1359" t="n"/>
+      <c r="F34" s="1359" t="n"/>
+      <c r="G34" s="1359" t="n"/>
+      <c r="H34" s="1359" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1324" t="n"/>
-      <c r="J34" s="1325" t="n"/>
-      <c r="K34" s="1325" t="n"/>
-      <c r="L34" s="1325" t="n"/>
-      <c r="M34" s="1323" t="n">
+      <c r="I34" s="1360" t="n"/>
+      <c r="J34" s="1361" t="n"/>
+      <c r="K34" s="1361" t="n"/>
+      <c r="L34" s="1361" t="n"/>
+      <c r="M34" s="1359" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1323" t="n">
+      <c r="N34" s="1359" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1323" t="n"/>
-      <c r="P34" s="1326" t="n"/>
-      <c r="Q34" s="1323" t="n"/>
-      <c r="R34" s="1323" t="n"/>
-      <c r="S34" s="1323" t="n"/>
+      <c r="O34" s="1359" t="n"/>
+      <c r="P34" s="1362" t="n"/>
+      <c r="Q34" s="1359" t="n"/>
+      <c r="R34" s="1359" t="n"/>
+      <c r="S34" s="1359" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1322" t="n"/>
+      <c r="U34" s="1358" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -6544,57 +6670,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1327" t="inlineStr">
+      <c r="A35" s="1363" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1328" t="inlineStr">
+      <c r="B35" s="1364" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1328" t="inlineStr">
+      <c r="C35" s="1364" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1329" t="n"/>
-      <c r="E35" s="1329" t="n">
+      <c r="D35" s="1365" t="n"/>
+      <c r="E35" s="1365" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1329" t="n">
+      <c r="F35" s="1365" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1329" t="n">
+      <c r="G35" s="1365" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1329" t="n"/>
-      <c r="I35" s="1330" t="n">
+      <c r="H35" s="1365" t="n"/>
+      <c r="I35" s="1366" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1331" t="n"/>
-      <c r="K35" s="1331" t="n"/>
-      <c r="L35" s="1331" t="n"/>
-      <c r="M35" s="1329" t="n"/>
-      <c r="N35" s="1329" t="n"/>
-      <c r="O35" s="1329" t="n">
+      <c r="J35" s="1367" t="n"/>
+      <c r="K35" s="1367" t="n"/>
+      <c r="L35" s="1367" t="n"/>
+      <c r="M35" s="1365" t="n"/>
+      <c r="N35" s="1365" t="n"/>
+      <c r="O35" s="1365" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1332" t="n">
+      <c r="P35" s="1368" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1329" t="n"/>
-      <c r="R35" s="1329" t="n">
+      <c r="Q35" s="1365" t="n"/>
+      <c r="R35" s="1365" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1329" t="n"/>
+      <c r="S35" s="1365" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1328" t="inlineStr">
+      <c r="U35" s="1364" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -6606,49 +6732,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1333" t="inlineStr">
+      <c r="A36" s="1369" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1334" t="inlineStr">
+      <c r="B36" s="1370" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1334" t="inlineStr">
+      <c r="C36" s="1370" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1335" t="n"/>
-      <c r="E36" s="1335" t="n"/>
-      <c r="F36" s="1335" t="n"/>
-      <c r="G36" s="1335" t="n"/>
-      <c r="H36" s="1335" t="n">
+      <c r="D36" s="1371" t="n"/>
+      <c r="E36" s="1371" t="n"/>
+      <c r="F36" s="1371" t="n"/>
+      <c r="G36" s="1371" t="n"/>
+      <c r="H36" s="1371" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1336" t="n"/>
-      <c r="J36" s="1337" t="n"/>
-      <c r="K36" s="1337" t="n"/>
-      <c r="L36" s="1337" t="n"/>
-      <c r="M36" s="1335" t="n">
+      <c r="I36" s="1372" t="n"/>
+      <c r="J36" s="1373" t="n"/>
+      <c r="K36" s="1373" t="n"/>
+      <c r="L36" s="1373" t="n"/>
+      <c r="M36" s="1371" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1335" t="n">
+      <c r="N36" s="1371" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1335" t="n"/>
-      <c r="P36" s="1338" t="n"/>
-      <c r="Q36" s="1335" t="n"/>
-      <c r="R36" s="1335" t="n"/>
-      <c r="S36" s="1335" t="n"/>
+      <c r="O36" s="1371" t="n"/>
+      <c r="P36" s="1374" t="n"/>
+      <c r="Q36" s="1371" t="n"/>
+      <c r="R36" s="1371" t="n"/>
+      <c r="S36" s="1371" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1334" t="n"/>
+      <c r="U36" s="1370" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -6656,41 +6782,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1339" t="inlineStr">
+      <c r="A37" s="1375" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1340" t="inlineStr">
+      <c r="B37" s="1376" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1340" t="inlineStr">
+      <c r="C37" s="1376" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1341" t="n"/>
-      <c r="E37" s="1341" t="n"/>
-      <c r="F37" s="1341" t="n"/>
-      <c r="G37" s="1341" t="n"/>
-      <c r="H37" s="1341" t="n"/>
-      <c r="I37" s="1342" t="n"/>
-      <c r="J37" s="1343" t="n"/>
-      <c r="K37" s="1343" t="n"/>
-      <c r="L37" s="1343" t="n"/>
-      <c r="M37" s="1341" t="n"/>
-      <c r="N37" s="1341" t="n"/>
-      <c r="O37" s="1341" t="n"/>
-      <c r="P37" s="1344" t="n"/>
-      <c r="Q37" s="1341" t="n">
+      <c r="D37" s="1377" t="n"/>
+      <c r="E37" s="1377" t="n"/>
+      <c r="F37" s="1377" t="n"/>
+      <c r="G37" s="1377" t="n"/>
+      <c r="H37" s="1377" t="n"/>
+      <c r="I37" s="1378" t="n"/>
+      <c r="J37" s="1379" t="n"/>
+      <c r="K37" s="1379" t="n"/>
+      <c r="L37" s="1379" t="n"/>
+      <c r="M37" s="1377" t="n"/>
+      <c r="N37" s="1377" t="n"/>
+      <c r="O37" s="1377" t="n"/>
+      <c r="P37" s="1380" t="n"/>
+      <c r="Q37" s="1377" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1341" t="n"/>
-      <c r="S37" s="1341" t="n"/>
+      <c r="R37" s="1377" t="n"/>
+      <c r="S37" s="1377" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1340" t="n"/>
+      <c r="U37" s="1376" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -6698,57 +6824,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1315" t="inlineStr">
+      <c r="A38" s="1351" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1316" t="inlineStr">
+      <c r="B38" s="1352" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1316" t="inlineStr">
+      <c r="C38" s="1352" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1317" t="n"/>
-      <c r="E38" s="1317" t="n">
+      <c r="D38" s="1353" t="n"/>
+      <c r="E38" s="1353" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1317" t="n">
+      <c r="F38" s="1353" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1317" t="n">
+      <c r="G38" s="1353" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1317" t="n"/>
-      <c r="I38" s="1318" t="n">
+      <c r="H38" s="1353" t="n"/>
+      <c r="I38" s="1354" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1319" t="n"/>
-      <c r="K38" s="1319" t="n"/>
-      <c r="L38" s="1319" t="n"/>
-      <c r="M38" s="1317" t="n"/>
-      <c r="N38" s="1317" t="n"/>
-      <c r="O38" s="1317" t="n">
+      <c r="J38" s="1355" t="n"/>
+      <c r="K38" s="1355" t="n"/>
+      <c r="L38" s="1355" t="n"/>
+      <c r="M38" s="1353" t="n"/>
+      <c r="N38" s="1353" t="n"/>
+      <c r="O38" s="1353" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1320" t="n">
+      <c r="P38" s="1356" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1317" t="n"/>
-      <c r="R38" s="1317" t="n">
+      <c r="Q38" s="1353" t="n"/>
+      <c r="R38" s="1353" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1317" t="n"/>
+      <c r="S38" s="1353" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1316" t="inlineStr">
+      <c r="U38" s="1352" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -6760,49 +6886,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1345" t="inlineStr">
+      <c r="A39" s="1381" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1346" t="inlineStr">
+      <c r="B39" s="1382" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1346" t="inlineStr">
+      <c r="C39" s="1382" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1347" t="n"/>
-      <c r="E39" s="1347" t="n"/>
-      <c r="F39" s="1347" t="n"/>
-      <c r="G39" s="1347" t="n"/>
-      <c r="H39" s="1347" t="n">
+      <c r="D39" s="1383" t="n"/>
+      <c r="E39" s="1383" t="n"/>
+      <c r="F39" s="1383" t="n"/>
+      <c r="G39" s="1383" t="n"/>
+      <c r="H39" s="1383" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1348" t="n"/>
-      <c r="J39" s="1349" t="n"/>
-      <c r="K39" s="1349" t="n"/>
-      <c r="L39" s="1349" t="n"/>
-      <c r="M39" s="1347" t="n">
+      <c r="I39" s="1384" t="n"/>
+      <c r="J39" s="1385" t="n"/>
+      <c r="K39" s="1385" t="n"/>
+      <c r="L39" s="1385" t="n"/>
+      <c r="M39" s="1383" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1347" t="n">
+      <c r="N39" s="1383" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1347" t="n"/>
-      <c r="P39" s="1350" t="n"/>
-      <c r="Q39" s="1347" t="n"/>
-      <c r="R39" s="1347" t="n"/>
-      <c r="S39" s="1347" t="n"/>
+      <c r="O39" s="1383" t="n"/>
+      <c r="P39" s="1386" t="n"/>
+      <c r="Q39" s="1383" t="n"/>
+      <c r="R39" s="1383" t="n"/>
+      <c r="S39" s="1383" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1346" t="n"/>
+      <c r="U39" s="1382" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -6810,41 +6936,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1321" t="inlineStr">
+      <c r="A40" s="1357" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1322" t="inlineStr">
+      <c r="B40" s="1358" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1322" t="inlineStr">
+      <c r="C40" s="1358" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1323" t="n"/>
-      <c r="E40" s="1323" t="n"/>
-      <c r="F40" s="1323" t="n"/>
-      <c r="G40" s="1323" t="n"/>
-      <c r="H40" s="1323" t="n"/>
-      <c r="I40" s="1324" t="n"/>
-      <c r="J40" s="1325" t="n"/>
-      <c r="K40" s="1325" t="n"/>
-      <c r="L40" s="1325" t="n"/>
-      <c r="M40" s="1323" t="n"/>
-      <c r="N40" s="1323" t="n"/>
-      <c r="O40" s="1323" t="n"/>
-      <c r="P40" s="1326" t="n"/>
-      <c r="Q40" s="1323" t="n">
+      <c r="D40" s="1359" t="n"/>
+      <c r="E40" s="1359" t="n"/>
+      <c r="F40" s="1359" t="n"/>
+      <c r="G40" s="1359" t="n"/>
+      <c r="H40" s="1359" t="n"/>
+      <c r="I40" s="1360" t="n"/>
+      <c r="J40" s="1361" t="n"/>
+      <c r="K40" s="1361" t="n"/>
+      <c r="L40" s="1361" t="n"/>
+      <c r="M40" s="1359" t="n"/>
+      <c r="N40" s="1359" t="n"/>
+      <c r="O40" s="1359" t="n"/>
+      <c r="P40" s="1362" t="n"/>
+      <c r="Q40" s="1359" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1323" t="n"/>
-      <c r="S40" s="1323" t="n"/>
+      <c r="R40" s="1359" t="n"/>
+      <c r="S40" s="1359" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1322" t="n"/>
+      <c r="U40" s="1358" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -6852,57 +6978,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1327" t="inlineStr">
+      <c r="A41" s="1363" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1328" t="inlineStr">
+      <c r="B41" s="1364" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1328" t="inlineStr">
+      <c r="C41" s="1364" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1329" t="n"/>
-      <c r="E41" s="1329" t="n">
+      <c r="D41" s="1365" t="n"/>
+      <c r="E41" s="1365" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1329" t="n">
+      <c r="F41" s="1365" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1329" t="n">
+      <c r="G41" s="1365" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1329" t="n"/>
-      <c r="I41" s="1330" t="n">
+      <c r="H41" s="1365" t="n"/>
+      <c r="I41" s="1366" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1331" t="n"/>
-      <c r="K41" s="1331" t="n"/>
-      <c r="L41" s="1331" t="n"/>
-      <c r="M41" s="1329" t="n"/>
-      <c r="N41" s="1329" t="n"/>
-      <c r="O41" s="1329" t="n">
+      <c r="J41" s="1367" t="n"/>
+      <c r="K41" s="1367" t="n"/>
+      <c r="L41" s="1367" t="n"/>
+      <c r="M41" s="1365" t="n"/>
+      <c r="N41" s="1365" t="n"/>
+      <c r="O41" s="1365" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1332" t="n">
+      <c r="P41" s="1368" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1329" t="n"/>
-      <c r="R41" s="1329" t="n">
+      <c r="Q41" s="1365" t="n"/>
+      <c r="R41" s="1365" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1329" t="n"/>
+      <c r="S41" s="1365" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1328" t="inlineStr">
+      <c r="U41" s="1364" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -6914,49 +7040,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1339" t="inlineStr">
+      <c r="A42" s="1375" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1340" t="inlineStr">
+      <c r="B42" s="1376" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1340" t="inlineStr">
+      <c r="C42" s="1376" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1341" t="n"/>
-      <c r="E42" s="1341" t="n"/>
-      <c r="F42" s="1341" t="n"/>
-      <c r="G42" s="1341" t="n"/>
-      <c r="H42" s="1341" t="n">
+      <c r="D42" s="1377" t="n"/>
+      <c r="E42" s="1377" t="n"/>
+      <c r="F42" s="1377" t="n"/>
+      <c r="G42" s="1377" t="n"/>
+      <c r="H42" s="1377" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1342" t="n"/>
-      <c r="J42" s="1343" t="n"/>
-      <c r="K42" s="1343" t="n"/>
-      <c r="L42" s="1343" t="n"/>
-      <c r="M42" s="1341" t="n">
+      <c r="I42" s="1378" t="n"/>
+      <c r="J42" s="1379" t="n"/>
+      <c r="K42" s="1379" t="n"/>
+      <c r="L42" s="1379" t="n"/>
+      <c r="M42" s="1377" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1341" t="n">
+      <c r="N42" s="1377" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1341" t="n"/>
-      <c r="P42" s="1344" t="n"/>
-      <c r="Q42" s="1341" t="n"/>
-      <c r="R42" s="1341" t="n"/>
-      <c r="S42" s="1341" t="n"/>
+      <c r="O42" s="1377" t="n"/>
+      <c r="P42" s="1380" t="n"/>
+      <c r="Q42" s="1377" t="n"/>
+      <c r="R42" s="1377" t="n"/>
+      <c r="S42" s="1377" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1340" t="n"/>
+      <c r="U42" s="1376" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -6964,57 +7090,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1315" t="inlineStr">
+      <c r="A43" s="1351" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1316" t="inlineStr">
+      <c r="B43" s="1352" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1316" t="inlineStr">
+      <c r="C43" s="1352" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1317" t="n"/>
-      <c r="E43" s="1317" t="n">
+      <c r="D43" s="1353" t="n"/>
+      <c r="E43" s="1353" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1317" t="n">
+      <c r="F43" s="1353" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1317" t="n">
+      <c r="G43" s="1353" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1317" t="n"/>
-      <c r="I43" s="1318" t="n">
+      <c r="H43" s="1353" t="n"/>
+      <c r="I43" s="1354" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1319" t="n"/>
-      <c r="K43" s="1319" t="n"/>
-      <c r="L43" s="1319" t="n"/>
-      <c r="M43" s="1317" t="n"/>
-      <c r="N43" s="1317" t="n"/>
-      <c r="O43" s="1317" t="n">
+      <c r="J43" s="1355" t="n"/>
+      <c r="K43" s="1355" t="n"/>
+      <c r="L43" s="1355" t="n"/>
+      <c r="M43" s="1353" t="n"/>
+      <c r="N43" s="1353" t="n"/>
+      <c r="O43" s="1353" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1320" t="n">
+      <c r="P43" s="1356" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1317" t="n"/>
-      <c r="R43" s="1317" t="n">
+      <c r="Q43" s="1353" t="n"/>
+      <c r="R43" s="1353" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1317" t="n"/>
+      <c r="S43" s="1353" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1316" t="n"/>
+      <c r="U43" s="1352" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -7022,45 +7148,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1345" t="inlineStr">
+      <c r="A44" s="1381" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1346" t="inlineStr">
+      <c r="B44" s="1382" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1346" t="inlineStr">
+      <c r="C44" s="1382" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1347" t="n"/>
-      <c r="E44" s="1347" t="n">
+      <c r="D44" s="1383" t="n"/>
+      <c r="E44" s="1383" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1347" t="n">
+      <c r="F44" s="1383" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1347" t="n"/>
-      <c r="H44" s="1347" t="n"/>
-      <c r="I44" s="1348" t="n"/>
-      <c r="J44" s="1349" t="n"/>
-      <c r="K44" s="1349" t="n"/>
-      <c r="L44" s="1349" t="n"/>
-      <c r="M44" s="1347" t="n"/>
-      <c r="N44" s="1347" t="n"/>
-      <c r="O44" s="1347" t="n"/>
-      <c r="P44" s="1350" t="n"/>
-      <c r="Q44" s="1347" t="n"/>
-      <c r="R44" s="1347" t="n"/>
-      <c r="S44" s="1347" t="n">
+      <c r="G44" s="1383" t="n"/>
+      <c r="H44" s="1383" t="n"/>
+      <c r="I44" s="1384" t="n"/>
+      <c r="J44" s="1385" t="n"/>
+      <c r="K44" s="1385" t="n"/>
+      <c r="L44" s="1385" t="n"/>
+      <c r="M44" s="1383" t="n"/>
+      <c r="N44" s="1383" t="n"/>
+      <c r="O44" s="1383" t="n"/>
+      <c r="P44" s="1386" t="n"/>
+      <c r="Q44" s="1383" t="n"/>
+      <c r="R44" s="1383" t="n"/>
+      <c r="S44" s="1383" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1346" t="inlineStr">
+      <c r="U44" s="1382" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -7072,49 +7198,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1345" t="inlineStr">
+      <c r="A45" s="1381" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1346" t="inlineStr">
+      <c r="B45" s="1382" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1346" t="inlineStr">
+      <c r="C45" s="1382" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1347" t="n"/>
-      <c r="E45" s="1347" t="n"/>
-      <c r="F45" s="1347" t="n"/>
-      <c r="G45" s="1347" t="n"/>
-      <c r="H45" s="1347" t="n">
+      <c r="D45" s="1383" t="n"/>
+      <c r="E45" s="1383" t="n"/>
+      <c r="F45" s="1383" t="n"/>
+      <c r="G45" s="1383" t="n"/>
+      <c r="H45" s="1383" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1348" t="n"/>
-      <c r="J45" s="1349" t="n"/>
-      <c r="K45" s="1349" t="n"/>
-      <c r="L45" s="1349" t="n"/>
-      <c r="M45" s="1347" t="n">
+      <c r="I45" s="1384" t="n"/>
+      <c r="J45" s="1385" t="n"/>
+      <c r="K45" s="1385" t="n"/>
+      <c r="L45" s="1385" t="n"/>
+      <c r="M45" s="1383" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1347" t="n">
+      <c r="N45" s="1383" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1347" t="n"/>
-      <c r="P45" s="1350" t="n"/>
-      <c r="Q45" s="1347" t="n"/>
-      <c r="R45" s="1347" t="n"/>
-      <c r="S45" s="1347" t="n"/>
+      <c r="O45" s="1383" t="n"/>
+      <c r="P45" s="1386" t="n"/>
+      <c r="Q45" s="1383" t="n"/>
+      <c r="R45" s="1383" t="n"/>
+      <c r="S45" s="1383" t="n"/>
       <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1346" t="n"/>
+      <c r="U45" s="1382" t="n"/>
       <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -7122,39 +7248,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1321" t="inlineStr">
+      <c r="A46" s="1357" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B46" s="1322" t="inlineStr">
+      <c r="B46" s="1358" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="C46" s="1322" t="inlineStr">
+      <c r="C46" s="1358" t="inlineStr">
         <is>
           <t>EVENT - Clean</t>
         </is>
       </c>
-      <c r="D46" s="1323" t="n"/>
-      <c r="E46" s="1323" t="n"/>
-      <c r="F46" s="1323" t="n"/>
-      <c r="G46" s="1323" t="n"/>
-      <c r="H46" s="1323" t="n"/>
-      <c r="I46" s="1324" t="n"/>
-      <c r="J46" s="1325" t="n"/>
-      <c r="K46" s="1325" t="n"/>
-      <c r="L46" s="1325" t="n"/>
-      <c r="M46" s="1323" t="n"/>
-      <c r="N46" s="1323" t="n"/>
-      <c r="O46" s="1323" t="n"/>
-      <c r="P46" s="1326" t="n"/>
-      <c r="Q46" s="1323" t="n"/>
-      <c r="R46" s="1323" t="n"/>
-      <c r="S46" s="1323" t="n"/>
+      <c r="D46" s="1359" t="n"/>
+      <c r="E46" s="1359" t="n"/>
+      <c r="F46" s="1359" t="n"/>
+      <c r="G46" s="1359" t="n"/>
+      <c r="H46" s="1359" t="n"/>
+      <c r="I46" s="1360" t="n"/>
+      <c r="J46" s="1361" t="n"/>
+      <c r="K46" s="1361" t="n"/>
+      <c r="L46" s="1361" t="n"/>
+      <c r="M46" s="1359" t="n"/>
+      <c r="N46" s="1359" t="n"/>
+      <c r="O46" s="1359" t="n"/>
+      <c r="P46" s="1362" t="n"/>
+      <c r="Q46" s="1359" t="n"/>
+      <c r="R46" s="1359" t="n"/>
+      <c r="S46" s="1359" t="n"/>
       <c r="T46" s="631" t="n"/>
-      <c r="U46" s="1322" t="n"/>
+      <c r="U46" s="1358" t="n"/>
       <c r="V46" s="632" t="inlineStr">
         <is>
           <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
@@ -7162,51 +7288,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1327" t="inlineStr">
+      <c r="A47" s="1363" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1328" t="inlineStr">
+      <c r="B47" s="1364" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C47" s="1328" t="inlineStr">
+      <c r="C47" s="1364" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D47" s="1329" t="n"/>
-      <c r="E47" s="1329" t="n">
+      <c r="D47" s="1365" t="n"/>
+      <c r="E47" s="1365" t="n">
         <v>16.6</v>
       </c>
-      <c r="F47" s="1329" t="n">
+      <c r="F47" s="1365" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="1329" t="n">
+      <c r="G47" s="1365" t="n">
         <v>4.1</v>
       </c>
-      <c r="H47" s="1329" t="n"/>
-      <c r="I47" s="1330" t="n">
+      <c r="H47" s="1365" t="n"/>
+      <c r="I47" s="1366" t="n">
         <v>0.9</v>
       </c>
-      <c r="J47" s="1331" t="n"/>
-      <c r="K47" s="1331" t="n"/>
-      <c r="L47" s="1331" t="n"/>
-      <c r="M47" s="1329" t="n"/>
-      <c r="N47" s="1329" t="n"/>
-      <c r="O47" s="1329" t="n">
+      <c r="J47" s="1367" t="n"/>
+      <c r="K47" s="1367" t="n"/>
+      <c r="L47" s="1367" t="n"/>
+      <c r="M47" s="1365" t="n"/>
+      <c r="N47" s="1365" t="n"/>
+      <c r="O47" s="1365" t="n">
         <v>13.2</v>
       </c>
-      <c r="P47" s="1332" t="n">
+      <c r="P47" s="1368" t="n">
         <v>0</v>
       </c>
-      <c r="Q47" s="1329" t="n"/>
-      <c r="R47" s="1329" t="n">
+      <c r="Q47" s="1365" t="n"/>
+      <c r="R47" s="1365" t="n">
         <v>84.5</v>
       </c>
-      <c r="S47" s="1329" t="n">
+      <c r="S47" s="1365" t="n">
         <v>11.8</v>
       </c>
       <c r="T47" s="813" t="inlineStr">
@@ -7214,7 +7340,7 @@
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1328" t="inlineStr">
+      <c r="U47" s="1364" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
@@ -7226,49 +7352,49 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1339" t="inlineStr">
+      <c r="A48" s="1375" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B48" s="1340" t="inlineStr">
+      <c r="B48" s="1376" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C48" s="1340" t="inlineStr">
+      <c r="C48" s="1376" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D48" s="1341" t="n"/>
-      <c r="E48" s="1341" t="n"/>
-      <c r="F48" s="1341" t="n"/>
-      <c r="G48" s="1341" t="n"/>
-      <c r="H48" s="1341" t="n">
+      <c r="D48" s="1377" t="n"/>
+      <c r="E48" s="1377" t="n"/>
+      <c r="F48" s="1377" t="n"/>
+      <c r="G48" s="1377" t="n"/>
+      <c r="H48" s="1377" t="n">
         <v>15.1</v>
       </c>
-      <c r="I48" s="1342" t="n"/>
-      <c r="J48" s="1343" t="n"/>
-      <c r="K48" s="1343" t="n"/>
-      <c r="L48" s="1343" t="n"/>
-      <c r="M48" s="1341" t="n">
+      <c r="I48" s="1378" t="n"/>
+      <c r="J48" s="1379" t="n"/>
+      <c r="K48" s="1379" t="n"/>
+      <c r="L48" s="1379" t="n"/>
+      <c r="M48" s="1377" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="1341" t="n">
+      <c r="N48" s="1377" t="n">
         <v>20</v>
       </c>
-      <c r="O48" s="1341" t="n"/>
-      <c r="P48" s="1344" t="n"/>
-      <c r="Q48" s="1341" t="n"/>
-      <c r="R48" s="1341" t="n"/>
-      <c r="S48" s="1341" t="n"/>
+      <c r="O48" s="1377" t="n"/>
+      <c r="P48" s="1380" t="n"/>
+      <c r="Q48" s="1377" t="n"/>
+      <c r="R48" s="1377" t="n"/>
+      <c r="S48" s="1377" t="n"/>
       <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U48" s="1340" t="n"/>
+      <c r="U48" s="1376" t="n"/>
       <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
@@ -7276,51 +7402,51 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1315" t="inlineStr">
+      <c r="A49" s="1351" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B49" s="1316" t="inlineStr">
+      <c r="B49" s="1352" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C49" s="1316" t="inlineStr">
+      <c r="C49" s="1352" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D49" s="1317" t="n"/>
-      <c r="E49" s="1317" t="n">
+      <c r="D49" s="1353" t="n"/>
+      <c r="E49" s="1353" t="n">
         <v>16.8</v>
       </c>
-      <c r="F49" s="1317" t="n">
+      <c r="F49" s="1353" t="n">
         <v>0.2</v>
       </c>
-      <c r="G49" s="1317" t="n">
+      <c r="G49" s="1353" t="n">
         <v>3.3</v>
       </c>
-      <c r="H49" s="1317" t="n"/>
-      <c r="I49" s="1318" t="n">
+      <c r="H49" s="1353" t="n"/>
+      <c r="I49" s="1354" t="n">
         <v>1.7</v>
       </c>
-      <c r="J49" s="1319" t="n"/>
-      <c r="K49" s="1319" t="n"/>
-      <c r="L49" s="1319" t="n"/>
-      <c r="M49" s="1317" t="n"/>
-      <c r="N49" s="1317" t="n"/>
-      <c r="O49" s="1317" t="n">
+      <c r="J49" s="1355" t="n"/>
+      <c r="K49" s="1355" t="n"/>
+      <c r="L49" s="1355" t="n"/>
+      <c r="M49" s="1353" t="n"/>
+      <c r="N49" s="1353" t="n"/>
+      <c r="O49" s="1353" t="n">
         <v>13</v>
       </c>
-      <c r="P49" s="1320" t="n">
+      <c r="P49" s="1356" t="n">
         <v>0.87</v>
       </c>
-      <c r="Q49" s="1317" t="n"/>
-      <c r="R49" s="1317" t="n">
+      <c r="Q49" s="1353" t="n"/>
+      <c r="R49" s="1353" t="n">
         <v>86</v>
       </c>
-      <c r="S49" s="1317" t="n">
+      <c r="S49" s="1353" t="n">
         <v>11.65</v>
       </c>
       <c r="T49" s="624" t="inlineStr">
@@ -7328,7 +7454,7 @@
           <t>Clear now, 88F, 67% RH; sun so far 6.4h of 7h daylight (91%); today high 90F, 0.87in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U49" s="1316" t="inlineStr">
+      <c r="U49" s="1352" t="inlineStr">
         <is>
           <t>2026-07-04_1.jpeg;2026-07-04_2.jpeg;2026-07-04_3.jpeg;2026-07-04_4.jpeg</t>
         </is>
@@ -7340,52 +7466,108 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1321" t="inlineStr">
+      <c r="A50" s="1357" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B50" s="1322" t="inlineStr">
+      <c r="B50" s="1358" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C50" s="1322" t="inlineStr">
+      <c r="C50" s="1358" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D50" s="1323" t="n"/>
-      <c r="E50" s="1323" t="n"/>
-      <c r="F50" s="1323" t="n"/>
-      <c r="G50" s="1323" t="n"/>
-      <c r="H50" s="1323" t="n">
+      <c r="D50" s="1359" t="n"/>
+      <c r="E50" s="1359" t="n"/>
+      <c r="F50" s="1359" t="n"/>
+      <c r="G50" s="1359" t="n"/>
+      <c r="H50" s="1359" t="n">
         <v>14.6</v>
       </c>
-      <c r="I50" s="1324" t="n"/>
-      <c r="J50" s="1325" t="n"/>
-      <c r="K50" s="1325" t="n"/>
-      <c r="L50" s="1325" t="n"/>
-      <c r="M50" s="1323" t="n">
+      <c r="I50" s="1360" t="n"/>
+      <c r="J50" s="1361" t="n"/>
+      <c r="K50" s="1361" t="n"/>
+      <c r="L50" s="1361" t="n"/>
+      <c r="M50" s="1359" t="n">
         <v>0.5</v>
       </c>
-      <c r="N50" s="1323" t="n">
+      <c r="N50" s="1359" t="n">
         <v>20.5</v>
       </c>
-      <c r="O50" s="1323" t="n"/>
-      <c r="P50" s="1326" t="n"/>
-      <c r="Q50" s="1323" t="n"/>
-      <c r="R50" s="1323" t="n"/>
-      <c r="S50" s="1323" t="n"/>
+      <c r="O50" s="1359" t="n"/>
+      <c r="P50" s="1362" t="n"/>
+      <c r="Q50" s="1359" t="n"/>
+      <c r="R50" s="1359" t="n"/>
+      <c r="S50" s="1359" t="n"/>
       <c r="T50" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny day (high 90F, water 86F); storm forecast overnight</t>
         </is>
       </c>
-      <c r="U50" s="1322" t="n"/>
+      <c r="U50" s="1358" t="n"/>
       <c r="V50" s="632" t="inlineStr">
         <is>
           <t>0.5 gal added 7:40 PM. PARTY PRE-LOAD (Sun 7/5 1PM picnic): deliberately HALF the usual dose -- FC already high at 16.8, and John didn't want to overshoot into the high teens for guests. Sized on the retuned model (l24_hot_sunny now 4.0). Model projects ~14.6 next noon, BUT this is a known weather-mismatch case: model keys L24 off today's hot/sunny weather, while the actual loss window is a storm overnight (no UV) + cooler/cloudy Sun morning -&gt; real loss will be LOWER, so FC likely lands ~15-16 at the party (comfortable top-of-band, cushion for bather load, not overboard). =&gt; If tomorrow's noon comes in ABOVE 14.6, that's the weather mismatch, NOT the freshly-retuned constant; don't chase it. Plan: dose back up Sun evening after the crowd's out (expect a bather-load FC drop). Season total 20.5 gal. PHOTOS(4): water clear/healthy blue, bottom fully visible, no cloudiness/algae; yesterday's surface debris now gone (tracks with CC clearing to 0.2); liner step close-up normal speckled blue, no rust/stain progression. Ruler photo documents the ~11.65 cm level.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="1387" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B51" s="1388" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="C51" s="1388" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="D51" s="1389" t="n"/>
+      <c r="E51" s="1389" t="n">
+        <v>16</v>
+      </c>
+      <c r="F51" s="1389" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G51" s="1389" t="n"/>
+      <c r="H51" s="1389" t="n"/>
+      <c r="I51" s="1390" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="J51" s="1391" t="n"/>
+      <c r="K51" s="1391" t="n"/>
+      <c r="L51" s="1391" t="n"/>
+      <c r="M51" s="1389" t="n"/>
+      <c r="N51" s="1389" t="n"/>
+      <c r="O51" s="1389" t="n"/>
+      <c r="P51" s="1392" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="Q51" s="1389" t="n"/>
+      <c r="R51" s="1389" t="n">
+        <v>84</v>
+      </c>
+      <c r="S51" s="1389" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="T51" s="1199" t="inlineStr">
+        <is>
+          <t>Overcast now, 75F, 90% RH; sun so far 0.0h of 3h daylight (0%); today high 75F, 0.04in precip, UV max 6.5</t>
+        </is>
+      </c>
+      <c r="U51" s="1388" t="n"/>
+      <c r="V51" s="1200" t="inlineStr">
+        <is>
+          <t>25mL x0.2. Early test (7:45 AM, party day 1PM, John busy) -- off the usual noon cadence, fine. PARTY CALL: FC 16.0 is great; NO morning top-up needed (plan only called for one 'if FC slipped' -- it didn't). Cloudy/cool day (75F, 0 sun) means it'll hold through the party. WEATHER-MISMATCH CONFIRMED (as flagged on last night's dose): 7/4 dose predicted 14.6 for today assuming hot/sunny loss, but today is overcast/cool -&gt; FC ran high at 16.0 (pred error +1.4). This is the weather mismatch, NOT the freshly-retuned l24_hot_sunny=4.0; the constant still gets validated by future clean HOT-day noon readings (mid-week, after Mon rain). fc_loss left blank: off-cadence (~19h not 24h), 0.5gal dose in between, plus rain dilution -&gt; non-comparable. WATER LEVEL 11.65 -&gt; 13.9 (+2.25 cm) from the overnight storm (~0.9in rain, ~445 gal) -- ruler tracked the storm perfectly. CC ticked 0.2 -&gt; 0.5 (rain-driven organic/N load washed in by the storm; still a trace, high FC clears it -- not a party concern). Water temp 86 -&gt; 84 (cool front). NOTE: the BIG rain is still Mon 7/6 (~5.7in) -&gt; watch for overflow then, possible backwash-down after (bonus CYA lowering).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log 2026-07-05 evening (post-party): FC 14.8, CC 0.3, add 2 photos
Party outcome excellent -- FC only dropped 1.2 across the day (16.0->14.8,
right at aim) and CC actually fell (0.5->0.3) despite the crowd. Water
crystal-clear. Recommending 0.5 gal tonight, sized on tomorrow's rainy
forecast (real loss window) -> projects ~15.1 Mon noon.
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1393">
+  <cellXfs count="1429">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -4706,6 +4706,114 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -4967,7 +5075,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V51"/>
+  <dimension ref="A1:V52"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -5144,35 +5252,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1351" t="inlineStr">
+      <c r="A3" s="1393" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1352" t="n"/>
-      <c r="C3" s="1352" t="inlineStr">
+      <c r="B3" s="1394" t="n"/>
+      <c r="C3" s="1394" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1353" t="n"/>
-      <c r="E3" s="1353" t="n"/>
-      <c r="F3" s="1353" t="n"/>
-      <c r="G3" s="1353" t="n"/>
-      <c r="H3" s="1353" t="n"/>
-      <c r="I3" s="1354" t="n"/>
-      <c r="J3" s="1355" t="n"/>
-      <c r="K3" s="1355" t="n"/>
-      <c r="L3" s="1355" t="n"/>
-      <c r="M3" s="1353" t="n"/>
-      <c r="N3" s="1353" t="n"/>
-      <c r="O3" s="1353" t="n"/>
-      <c r="P3" s="1356" t="n"/>
-      <c r="Q3" s="1353" t="n"/>
-      <c r="R3" s="1353" t="n"/>
-      <c r="S3" s="1353" t="n"/>
+      <c r="D3" s="1395" t="n"/>
+      <c r="E3" s="1395" t="n"/>
+      <c r="F3" s="1395" t="n"/>
+      <c r="G3" s="1395" t="n"/>
+      <c r="H3" s="1395" t="n"/>
+      <c r="I3" s="1396" t="n"/>
+      <c r="J3" s="1397" t="n"/>
+      <c r="K3" s="1397" t="n"/>
+      <c r="L3" s="1397" t="n"/>
+      <c r="M3" s="1395" t="n"/>
+      <c r="N3" s="1395" t="n"/>
+      <c r="O3" s="1395" t="n"/>
+      <c r="P3" s="1398" t="n"/>
+      <c r="Q3" s="1395" t="n"/>
+      <c r="R3" s="1395" t="n"/>
+      <c r="S3" s="1395" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1352" t="n"/>
+      <c r="U3" s="1394" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -5180,43 +5288,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1357" t="inlineStr">
+      <c r="A4" s="1399" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1358" t="inlineStr">
+      <c r="B4" s="1400" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1358" t="inlineStr">
+      <c r="C4" s="1400" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1359" t="n"/>
-      <c r="E4" s="1359" t="n"/>
-      <c r="F4" s="1359" t="n"/>
-      <c r="G4" s="1359" t="n"/>
-      <c r="H4" s="1359" t="n"/>
-      <c r="I4" s="1360" t="n"/>
-      <c r="J4" s="1361" t="n"/>
-      <c r="K4" s="1361" t="n"/>
-      <c r="L4" s="1361" t="n"/>
-      <c r="M4" s="1359" t="n">
+      <c r="D4" s="1401" t="n"/>
+      <c r="E4" s="1401" t="n"/>
+      <c r="F4" s="1401" t="n"/>
+      <c r="G4" s="1401" t="n"/>
+      <c r="H4" s="1401" t="n"/>
+      <c r="I4" s="1402" t="n"/>
+      <c r="J4" s="1403" t="n"/>
+      <c r="K4" s="1403" t="n"/>
+      <c r="L4" s="1403" t="n"/>
+      <c r="M4" s="1401" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1359" t="n">
+      <c r="N4" s="1401" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1359" t="n"/>
-      <c r="P4" s="1362" t="n"/>
-      <c r="Q4" s="1359" t="n"/>
-      <c r="R4" s="1359" t="n"/>
-      <c r="S4" s="1359" t="n"/>
+      <c r="O4" s="1401" t="n"/>
+      <c r="P4" s="1404" t="n"/>
+      <c r="Q4" s="1401" t="n"/>
+      <c r="R4" s="1401" t="n"/>
+      <c r="S4" s="1401" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1358" t="n"/>
+      <c r="U4" s="1400" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -5224,57 +5332,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1363" t="inlineStr">
+      <c r="A5" s="1405" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1364" t="inlineStr">
+      <c r="B5" s="1406" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1364" t="inlineStr">
+      <c r="C5" s="1406" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1365" t="n">
+      <c r="D5" s="1407" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1365" t="n">
+      <c r="E5" s="1407" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1365" t="n">
+      <c r="F5" s="1407" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1365" t="n"/>
-      <c r="H5" s="1365" t="n"/>
-      <c r="I5" s="1366" t="n"/>
-      <c r="J5" s="1367" t="n">
+      <c r="G5" s="1407" t="n"/>
+      <c r="H5" s="1407" t="n"/>
+      <c r="I5" s="1408" t="n"/>
+      <c r="J5" s="1409" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1367" t="n">
+      <c r="K5" s="1409" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1367" t="inlineStr">
+      <c r="L5" s="1409" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1365" t="n"/>
-      <c r="N5" s="1365" t="n"/>
-      <c r="O5" s="1365" t="n">
+      <c r="M5" s="1407" t="n"/>
+      <c r="N5" s="1407" t="n"/>
+      <c r="O5" s="1407" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1368" t="n">
+      <c r="P5" s="1410" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1365" t="n"/>
-      <c r="R5" s="1365" t="n"/>
-      <c r="S5" s="1365" t="n"/>
+      <c r="Q5" s="1407" t="n"/>
+      <c r="R5" s="1407" t="n"/>
+      <c r="S5" s="1407" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1364" t="n"/>
+      <c r="U5" s="1406" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -5282,43 +5390,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1369" t="inlineStr">
+      <c r="A6" s="1411" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1370" t="inlineStr">
+      <c r="B6" s="1412" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1370" t="inlineStr">
+      <c r="C6" s="1412" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1371" t="n"/>
-      <c r="E6" s="1371" t="n"/>
-      <c r="F6" s="1371" t="n"/>
-      <c r="G6" s="1371" t="n"/>
-      <c r="H6" s="1371" t="n"/>
-      <c r="I6" s="1372" t="n"/>
-      <c r="J6" s="1373" t="n"/>
-      <c r="K6" s="1373" t="n"/>
-      <c r="L6" s="1373" t="n"/>
-      <c r="M6" s="1371" t="n">
+      <c r="D6" s="1413" t="n"/>
+      <c r="E6" s="1413" t="n"/>
+      <c r="F6" s="1413" t="n"/>
+      <c r="G6" s="1413" t="n"/>
+      <c r="H6" s="1413" t="n"/>
+      <c r="I6" s="1414" t="n"/>
+      <c r="J6" s="1415" t="n"/>
+      <c r="K6" s="1415" t="n"/>
+      <c r="L6" s="1415" t="n"/>
+      <c r="M6" s="1413" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1371" t="n">
+      <c r="N6" s="1413" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1371" t="n"/>
-      <c r="P6" s="1374" t="n"/>
-      <c r="Q6" s="1371" t="n"/>
-      <c r="R6" s="1371" t="n"/>
-      <c r="S6" s="1371" t="n"/>
+      <c r="O6" s="1413" t="n"/>
+      <c r="P6" s="1416" t="n"/>
+      <c r="Q6" s="1413" t="n"/>
+      <c r="R6" s="1413" t="n"/>
+      <c r="S6" s="1413" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1370" t="n"/>
+      <c r="U6" s="1412" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -5326,39 +5434,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1375" t="inlineStr">
+      <c r="A7" s="1417" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1376" t="inlineStr">
+      <c r="B7" s="1418" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1376" t="inlineStr">
+      <c r="C7" s="1418" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1377" t="n"/>
-      <c r="E7" s="1377" t="n"/>
-      <c r="F7" s="1377" t="n"/>
-      <c r="G7" s="1377" t="n"/>
-      <c r="H7" s="1377" t="n"/>
-      <c r="I7" s="1378" t="n"/>
-      <c r="J7" s="1379" t="n"/>
-      <c r="K7" s="1379" t="n"/>
-      <c r="L7" s="1379" t="n"/>
-      <c r="M7" s="1377" t="n"/>
-      <c r="N7" s="1377" t="n"/>
-      <c r="O7" s="1377" t="n"/>
-      <c r="P7" s="1380" t="n"/>
-      <c r="Q7" s="1377" t="n"/>
-      <c r="R7" s="1377" t="n"/>
-      <c r="S7" s="1377" t="n"/>
+      <c r="D7" s="1419" t="n"/>
+      <c r="E7" s="1419" t="n"/>
+      <c r="F7" s="1419" t="n"/>
+      <c r="G7" s="1419" t="n"/>
+      <c r="H7" s="1419" t="n"/>
+      <c r="I7" s="1420" t="n"/>
+      <c r="J7" s="1421" t="n"/>
+      <c r="K7" s="1421" t="n"/>
+      <c r="L7" s="1421" t="n"/>
+      <c r="M7" s="1419" t="n"/>
+      <c r="N7" s="1419" t="n"/>
+      <c r="O7" s="1419" t="n"/>
+      <c r="P7" s="1422" t="n"/>
+      <c r="Q7" s="1419" t="n"/>
+      <c r="R7" s="1419" t="n"/>
+      <c r="S7" s="1419" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1376" t="n"/>
+      <c r="U7" s="1418" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5366,39 +5474,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1351" t="inlineStr">
+      <c r="A8" s="1393" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1352" t="inlineStr">
+      <c r="B8" s="1394" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1352" t="inlineStr">
+      <c r="C8" s="1394" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1353" t="n"/>
-      <c r="E8" s="1353" t="n"/>
-      <c r="F8" s="1353" t="n"/>
-      <c r="G8" s="1353" t="n"/>
-      <c r="H8" s="1353" t="n"/>
-      <c r="I8" s="1354" t="n"/>
-      <c r="J8" s="1355" t="n"/>
-      <c r="K8" s="1355" t="n"/>
-      <c r="L8" s="1355" t="n"/>
-      <c r="M8" s="1353" t="n"/>
-      <c r="N8" s="1353" t="n"/>
-      <c r="O8" s="1353" t="n"/>
-      <c r="P8" s="1356" t="n"/>
-      <c r="Q8" s="1353" t="n"/>
-      <c r="R8" s="1353" t="n"/>
-      <c r="S8" s="1353" t="n"/>
+      <c r="D8" s="1395" t="n"/>
+      <c r="E8" s="1395" t="n"/>
+      <c r="F8" s="1395" t="n"/>
+      <c r="G8" s="1395" t="n"/>
+      <c r="H8" s="1395" t="n"/>
+      <c r="I8" s="1396" t="n"/>
+      <c r="J8" s="1397" t="n"/>
+      <c r="K8" s="1397" t="n"/>
+      <c r="L8" s="1397" t="n"/>
+      <c r="M8" s="1395" t="n"/>
+      <c r="N8" s="1395" t="n"/>
+      <c r="O8" s="1395" t="n"/>
+      <c r="P8" s="1398" t="n"/>
+      <c r="Q8" s="1395" t="n"/>
+      <c r="R8" s="1395" t="n"/>
+      <c r="S8" s="1395" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1352" t="n"/>
+      <c r="U8" s="1394" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -5406,63 +5514,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1381" t="inlineStr">
+      <c r="A9" s="1423" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1382" t="inlineStr">
+      <c r="B9" s="1424" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1382" t="inlineStr">
+      <c r="C9" s="1424" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1383" t="n">
+      <c r="D9" s="1425" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1383" t="n">
+      <c r="E9" s="1425" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1383" t="n">
+      <c r="F9" s="1425" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1383" t="n">
+      <c r="G9" s="1425" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1383" t="n"/>
-      <c r="I9" s="1384" t="n"/>
-      <c r="J9" s="1385" t="n">
+      <c r="H9" s="1425" t="n"/>
+      <c r="I9" s="1426" t="n"/>
+      <c r="J9" s="1427" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1385" t="n">
+      <c r="K9" s="1427" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1385" t="inlineStr">
+      <c r="L9" s="1427" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1383" t="n"/>
-      <c r="N9" s="1383" t="n"/>
-      <c r="O9" s="1383" t="n">
+      <c r="M9" s="1425" t="n"/>
+      <c r="N9" s="1425" t="n"/>
+      <c r="O9" s="1425" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1386" t="n">
+      <c r="P9" s="1428" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1383" t="n"/>
-      <c r="R9" s="1383" t="n"/>
-      <c r="S9" s="1383" t="n"/>
+      <c r="Q9" s="1425" t="n"/>
+      <c r="R9" s="1425" t="n"/>
+      <c r="S9" s="1425" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1382" t="n"/>
+      <c r="U9" s="1424" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -5470,43 +5578,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1381" t="inlineStr">
+      <c r="A10" s="1423" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1382" t="inlineStr">
+      <c r="B10" s="1424" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1382" t="inlineStr">
+      <c r="C10" s="1424" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1383" t="n"/>
-      <c r="E10" s="1383" t="n"/>
-      <c r="F10" s="1383" t="n"/>
-      <c r="G10" s="1383" t="n"/>
-      <c r="H10" s="1383" t="n"/>
-      <c r="I10" s="1384" t="n"/>
-      <c r="J10" s="1385" t="n"/>
-      <c r="K10" s="1385" t="n"/>
-      <c r="L10" s="1385" t="inlineStr">
+      <c r="D10" s="1425" t="n"/>
+      <c r="E10" s="1425" t="n"/>
+      <c r="F10" s="1425" t="n"/>
+      <c r="G10" s="1425" t="n"/>
+      <c r="H10" s="1425" t="n"/>
+      <c r="I10" s="1426" t="n"/>
+      <c r="J10" s="1427" t="n"/>
+      <c r="K10" s="1427" t="n"/>
+      <c r="L10" s="1427" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1383" t="n"/>
-      <c r="N10" s="1383" t="n"/>
-      <c r="O10" s="1383" t="n"/>
-      <c r="P10" s="1386" t="n"/>
-      <c r="Q10" s="1383" t="n"/>
-      <c r="R10" s="1383" t="n"/>
-      <c r="S10" s="1383" t="n"/>
+      <c r="M10" s="1425" t="n"/>
+      <c r="N10" s="1425" t="n"/>
+      <c r="O10" s="1425" t="n"/>
+      <c r="P10" s="1428" t="n"/>
+      <c r="Q10" s="1425" t="n"/>
+      <c r="R10" s="1425" t="n"/>
+      <c r="S10" s="1425" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1382" t="n"/>
+      <c r="U10" s="1424" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -5514,43 +5622,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1381" t="inlineStr">
+      <c r="A11" s="1423" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1382" t="inlineStr">
+      <c r="B11" s="1424" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1382" t="inlineStr">
+      <c r="C11" s="1424" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1383" t="n"/>
-      <c r="E11" s="1383" t="n"/>
-      <c r="F11" s="1383" t="n"/>
-      <c r="G11" s="1383" t="n"/>
-      <c r="H11" s="1383" t="n"/>
-      <c r="I11" s="1384" t="n"/>
-      <c r="J11" s="1385" t="n"/>
-      <c r="K11" s="1385" t="n"/>
-      <c r="L11" s="1385" t="n"/>
-      <c r="M11" s="1383" t="n">
+      <c r="D11" s="1425" t="n"/>
+      <c r="E11" s="1425" t="n"/>
+      <c r="F11" s="1425" t="n"/>
+      <c r="G11" s="1425" t="n"/>
+      <c r="H11" s="1425" t="n"/>
+      <c r="I11" s="1426" t="n"/>
+      <c r="J11" s="1427" t="n"/>
+      <c r="K11" s="1427" t="n"/>
+      <c r="L11" s="1427" t="n"/>
+      <c r="M11" s="1425" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1383" t="n">
+      <c r="N11" s="1425" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1383" t="n"/>
-      <c r="P11" s="1386" t="n"/>
-      <c r="Q11" s="1383" t="n"/>
-      <c r="R11" s="1383" t="n"/>
-      <c r="S11" s="1383" t="n"/>
+      <c r="O11" s="1425" t="n"/>
+      <c r="P11" s="1428" t="n"/>
+      <c r="Q11" s="1425" t="n"/>
+      <c r="R11" s="1425" t="n"/>
+      <c r="S11" s="1425" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1382" t="n"/>
+      <c r="U11" s="1424" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -5558,39 +5666,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1357" t="inlineStr">
+      <c r="A12" s="1399" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1358" t="inlineStr">
+      <c r="B12" s="1400" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1358" t="inlineStr">
+      <c r="C12" s="1400" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1359" t="n"/>
-      <c r="E12" s="1359" t="n"/>
-      <c r="F12" s="1359" t="n"/>
-      <c r="G12" s="1359" t="n"/>
-      <c r="H12" s="1359" t="n"/>
-      <c r="I12" s="1360" t="n"/>
-      <c r="J12" s="1361" t="n"/>
-      <c r="K12" s="1361" t="n"/>
-      <c r="L12" s="1361" t="n"/>
-      <c r="M12" s="1359" t="n"/>
-      <c r="N12" s="1359" t="n"/>
-      <c r="O12" s="1359" t="n"/>
-      <c r="P12" s="1362" t="n"/>
-      <c r="Q12" s="1359" t="n"/>
-      <c r="R12" s="1359" t="n"/>
-      <c r="S12" s="1359" t="n"/>
+      <c r="D12" s="1401" t="n"/>
+      <c r="E12" s="1401" t="n"/>
+      <c r="F12" s="1401" t="n"/>
+      <c r="G12" s="1401" t="n"/>
+      <c r="H12" s="1401" t="n"/>
+      <c r="I12" s="1402" t="n"/>
+      <c r="J12" s="1403" t="n"/>
+      <c r="K12" s="1403" t="n"/>
+      <c r="L12" s="1403" t="n"/>
+      <c r="M12" s="1401" t="n"/>
+      <c r="N12" s="1401" t="n"/>
+      <c r="O12" s="1401" t="n"/>
+      <c r="P12" s="1404" t="n"/>
+      <c r="Q12" s="1401" t="n"/>
+      <c r="R12" s="1401" t="n"/>
+      <c r="S12" s="1401" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1358" t="n"/>
+      <c r="U12" s="1400" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5598,35 +5706,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1363" t="inlineStr">
+      <c r="A13" s="1405" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1364" t="n"/>
-      <c r="C13" s="1364" t="inlineStr">
+      <c r="B13" s="1406" t="n"/>
+      <c r="C13" s="1406" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1365" t="n"/>
-      <c r="E13" s="1365" t="n"/>
-      <c r="F13" s="1365" t="n"/>
-      <c r="G13" s="1365" t="n"/>
-      <c r="H13" s="1365" t="n"/>
-      <c r="I13" s="1366" t="n"/>
-      <c r="J13" s="1367" t="n"/>
-      <c r="K13" s="1367" t="n"/>
-      <c r="L13" s="1367" t="n"/>
-      <c r="M13" s="1365" t="n"/>
-      <c r="N13" s="1365" t="n"/>
-      <c r="O13" s="1365" t="n"/>
-      <c r="P13" s="1368" t="n"/>
-      <c r="Q13" s="1365" t="n"/>
-      <c r="R13" s="1365" t="n"/>
-      <c r="S13" s="1365" t="n"/>
+      <c r="D13" s="1407" t="n"/>
+      <c r="E13" s="1407" t="n"/>
+      <c r="F13" s="1407" t="n"/>
+      <c r="G13" s="1407" t="n"/>
+      <c r="H13" s="1407" t="n"/>
+      <c r="I13" s="1408" t="n"/>
+      <c r="J13" s="1409" t="n"/>
+      <c r="K13" s="1409" t="n"/>
+      <c r="L13" s="1409" t="n"/>
+      <c r="M13" s="1407" t="n"/>
+      <c r="N13" s="1407" t="n"/>
+      <c r="O13" s="1407" t="n"/>
+      <c r="P13" s="1410" t="n"/>
+      <c r="Q13" s="1407" t="n"/>
+      <c r="R13" s="1407" t="n"/>
+      <c r="S13" s="1407" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1364" t="n"/>
+      <c r="U13" s="1406" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -5634,53 +5742,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1369" t="inlineStr">
+      <c r="A14" s="1411" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1370" t="inlineStr">
+      <c r="B14" s="1412" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1370" t="inlineStr">
+      <c r="C14" s="1412" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1371" t="n"/>
-      <c r="E14" s="1371" t="n">
+      <c r="D14" s="1413" t="n"/>
+      <c r="E14" s="1413" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1371" t="n">
+      <c r="F14" s="1413" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1371" t="n">
+      <c r="G14" s="1413" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1371" t="n"/>
-      <c r="I14" s="1372" t="n"/>
-      <c r="J14" s="1373" t="n"/>
-      <c r="K14" s="1373" t="n"/>
-      <c r="L14" s="1373" t="n"/>
-      <c r="M14" s="1371" t="n"/>
-      <c r="N14" s="1371" t="n"/>
-      <c r="O14" s="1371" t="n">
+      <c r="H14" s="1413" t="n"/>
+      <c r="I14" s="1414" t="n"/>
+      <c r="J14" s="1415" t="n"/>
+      <c r="K14" s="1415" t="n"/>
+      <c r="L14" s="1415" t="n"/>
+      <c r="M14" s="1413" t="n"/>
+      <c r="N14" s="1413" t="n"/>
+      <c r="O14" s="1413" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1374" t="n">
+      <c r="P14" s="1416" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1371" t="n"/>
-      <c r="R14" s="1371" t="n"/>
-      <c r="S14" s="1371" t="n"/>
+      <c r="Q14" s="1413" t="n"/>
+      <c r="R14" s="1413" t="n"/>
+      <c r="S14" s="1413" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1370" t="n"/>
+      <c r="U14" s="1412" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -5688,43 +5796,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1369" t="inlineStr">
+      <c r="A15" s="1411" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1370" t="inlineStr">
+      <c r="B15" s="1412" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1370" t="inlineStr">
+      <c r="C15" s="1412" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1371" t="n"/>
-      <c r="E15" s="1371" t="n"/>
-      <c r="F15" s="1371" t="n"/>
-      <c r="G15" s="1371" t="n"/>
-      <c r="H15" s="1371" t="n"/>
-      <c r="I15" s="1372" t="n"/>
-      <c r="J15" s="1373" t="n"/>
-      <c r="K15" s="1373" t="n"/>
-      <c r="L15" s="1373" t="n"/>
-      <c r="M15" s="1371" t="n">
+      <c r="D15" s="1413" t="n"/>
+      <c r="E15" s="1413" t="n"/>
+      <c r="F15" s="1413" t="n"/>
+      <c r="G15" s="1413" t="n"/>
+      <c r="H15" s="1413" t="n"/>
+      <c r="I15" s="1414" t="n"/>
+      <c r="J15" s="1415" t="n"/>
+      <c r="K15" s="1415" t="n"/>
+      <c r="L15" s="1415" t="n"/>
+      <c r="M15" s="1413" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1371" t="n">
+      <c r="N15" s="1413" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1371" t="n"/>
-      <c r="P15" s="1374" t="n"/>
-      <c r="Q15" s="1371" t="n"/>
-      <c r="R15" s="1371" t="n"/>
-      <c r="S15" s="1371" t="n"/>
+      <c r="O15" s="1413" t="n"/>
+      <c r="P15" s="1416" t="n"/>
+      <c r="Q15" s="1413" t="n"/>
+      <c r="R15" s="1413" t="n"/>
+      <c r="S15" s="1413" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1370" t="n"/>
+      <c r="U15" s="1412" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -5732,39 +5840,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1375" t="inlineStr">
+      <c r="A16" s="1417" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1376" t="inlineStr">
+      <c r="B16" s="1418" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1376" t="inlineStr">
+      <c r="C16" s="1418" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1377" t="n"/>
-      <c r="E16" s="1377" t="n"/>
-      <c r="F16" s="1377" t="n"/>
-      <c r="G16" s="1377" t="n"/>
-      <c r="H16" s="1377" t="n"/>
-      <c r="I16" s="1378" t="n"/>
-      <c r="J16" s="1379" t="n"/>
-      <c r="K16" s="1379" t="n"/>
-      <c r="L16" s="1379" t="n"/>
-      <c r="M16" s="1377" t="n"/>
-      <c r="N16" s="1377" t="n"/>
-      <c r="O16" s="1377" t="n"/>
-      <c r="P16" s="1380" t="n"/>
-      <c r="Q16" s="1377" t="n"/>
-      <c r="R16" s="1377" t="n"/>
-      <c r="S16" s="1377" t="n"/>
+      <c r="D16" s="1419" t="n"/>
+      <c r="E16" s="1419" t="n"/>
+      <c r="F16" s="1419" t="n"/>
+      <c r="G16" s="1419" t="n"/>
+      <c r="H16" s="1419" t="n"/>
+      <c r="I16" s="1420" t="n"/>
+      <c r="J16" s="1421" t="n"/>
+      <c r="K16" s="1421" t="n"/>
+      <c r="L16" s="1421" t="n"/>
+      <c r="M16" s="1419" t="n"/>
+      <c r="N16" s="1419" t="n"/>
+      <c r="O16" s="1419" t="n"/>
+      <c r="P16" s="1422" t="n"/>
+      <c r="Q16" s="1419" t="n"/>
+      <c r="R16" s="1419" t="n"/>
+      <c r="S16" s="1419" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1376" t="n"/>
+      <c r="U16" s="1418" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -5772,39 +5880,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1351" t="inlineStr">
+      <c r="A17" s="1393" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1352" t="inlineStr">
+      <c r="B17" s="1394" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1352" t="inlineStr">
+      <c r="C17" s="1394" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1353" t="n"/>
-      <c r="E17" s="1353" t="n"/>
-      <c r="F17" s="1353" t="n"/>
-      <c r="G17" s="1353" t="n"/>
-      <c r="H17" s="1353" t="n"/>
-      <c r="I17" s="1354" t="n"/>
-      <c r="J17" s="1355" t="n"/>
-      <c r="K17" s="1355" t="n"/>
-      <c r="L17" s="1355" t="n"/>
-      <c r="M17" s="1353" t="n"/>
-      <c r="N17" s="1353" t="n"/>
-      <c r="O17" s="1353" t="n"/>
-      <c r="P17" s="1356" t="n"/>
-      <c r="Q17" s="1353" t="n"/>
-      <c r="R17" s="1353" t="n"/>
-      <c r="S17" s="1353" t="n"/>
+      <c r="D17" s="1395" t="n"/>
+      <c r="E17" s="1395" t="n"/>
+      <c r="F17" s="1395" t="n"/>
+      <c r="G17" s="1395" t="n"/>
+      <c r="H17" s="1395" t="n"/>
+      <c r="I17" s="1396" t="n"/>
+      <c r="J17" s="1397" t="n"/>
+      <c r="K17" s="1397" t="n"/>
+      <c r="L17" s="1397" t="n"/>
+      <c r="M17" s="1395" t="n"/>
+      <c r="N17" s="1395" t="n"/>
+      <c r="O17" s="1395" t="n"/>
+      <c r="P17" s="1398" t="n"/>
+      <c r="Q17" s="1395" t="n"/>
+      <c r="R17" s="1395" t="n"/>
+      <c r="S17" s="1395" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1352" t="n"/>
+      <c r="U17" s="1394" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -5812,53 +5920,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1381" t="inlineStr">
+      <c r="A18" s="1423" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1382" t="inlineStr">
+      <c r="B18" s="1424" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1382" t="inlineStr">
+      <c r="C18" s="1424" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1383" t="n"/>
-      <c r="E18" s="1383" t="n">
+      <c r="D18" s="1425" t="n"/>
+      <c r="E18" s="1425" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1383" t="n">
+      <c r="F18" s="1425" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1383" t="n">
+      <c r="G18" s="1425" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1383" t="n"/>
-      <c r="I18" s="1384" t="n"/>
-      <c r="J18" s="1385" t="n"/>
-      <c r="K18" s="1385" t="n"/>
-      <c r="L18" s="1385" t="n"/>
-      <c r="M18" s="1383" t="n"/>
-      <c r="N18" s="1383" t="n"/>
-      <c r="O18" s="1383" t="n">
+      <c r="H18" s="1425" t="n"/>
+      <c r="I18" s="1426" t="n"/>
+      <c r="J18" s="1427" t="n"/>
+      <c r="K18" s="1427" t="n"/>
+      <c r="L18" s="1427" t="n"/>
+      <c r="M18" s="1425" t="n"/>
+      <c r="N18" s="1425" t="n"/>
+      <c r="O18" s="1425" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1386" t="n">
+      <c r="P18" s="1428" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1383" t="n"/>
-      <c r="R18" s="1383" t="n"/>
-      <c r="S18" s="1383" t="n"/>
+      <c r="Q18" s="1425" t="n"/>
+      <c r="R18" s="1425" t="n"/>
+      <c r="S18" s="1425" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1382" t="n"/>
+      <c r="U18" s="1424" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -5866,47 +5974,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1381" t="inlineStr">
+      <c r="A19" s="1423" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1382" t="inlineStr">
+      <c r="B19" s="1424" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1382" t="inlineStr">
+      <c r="C19" s="1424" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1383" t="n"/>
-      <c r="E19" s="1383" t="n"/>
-      <c r="F19" s="1383" t="n"/>
-      <c r="G19" s="1383" t="n"/>
-      <c r="H19" s="1383" t="n"/>
-      <c r="I19" s="1384" t="n"/>
-      <c r="J19" s="1385" t="n"/>
-      <c r="K19" s="1385" t="n"/>
-      <c r="L19" s="1385" t="n"/>
-      <c r="M19" s="1383" t="n">
+      <c r="D19" s="1425" t="n"/>
+      <c r="E19" s="1425" t="n"/>
+      <c r="F19" s="1425" t="n"/>
+      <c r="G19" s="1425" t="n"/>
+      <c r="H19" s="1425" t="n"/>
+      <c r="I19" s="1426" t="n"/>
+      <c r="J19" s="1427" t="n"/>
+      <c r="K19" s="1427" t="n"/>
+      <c r="L19" s="1427" t="n"/>
+      <c r="M19" s="1425" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1383" t="n">
+      <c r="N19" s="1425" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1383" t="n"/>
-      <c r="P19" s="1386" t="n"/>
-      <c r="Q19" s="1383" t="n"/>
-      <c r="R19" s="1383" t="n"/>
-      <c r="S19" s="1383" t="n"/>
+      <c r="O19" s="1425" t="n"/>
+      <c r="P19" s="1428" t="n"/>
+      <c r="Q19" s="1425" t="n"/>
+      <c r="R19" s="1425" t="n"/>
+      <c r="S19" s="1425" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1382" t="n"/>
+      <c r="U19" s="1424" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -5914,43 +6022,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1381" t="inlineStr">
+      <c r="A20" s="1423" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1382" t="inlineStr">
+      <c r="B20" s="1424" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1382" t="inlineStr">
+      <c r="C20" s="1424" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1383" t="n"/>
-      <c r="E20" s="1383" t="n"/>
-      <c r="F20" s="1383" t="n"/>
-      <c r="G20" s="1383" t="n"/>
-      <c r="H20" s="1383" t="n"/>
-      <c r="I20" s="1384" t="n"/>
-      <c r="J20" s="1385" t="n"/>
-      <c r="K20" s="1385" t="n"/>
-      <c r="L20" s="1385" t="n"/>
-      <c r="M20" s="1383" t="n"/>
-      <c r="N20" s="1383" t="n"/>
-      <c r="O20" s="1383" t="n"/>
-      <c r="P20" s="1386" t="n"/>
-      <c r="Q20" s="1383" t="n"/>
-      <c r="R20" s="1383" t="n"/>
-      <c r="S20" s="1383" t="n"/>
+      <c r="D20" s="1425" t="n"/>
+      <c r="E20" s="1425" t="n"/>
+      <c r="F20" s="1425" t="n"/>
+      <c r="G20" s="1425" t="n"/>
+      <c r="H20" s="1425" t="n"/>
+      <c r="I20" s="1426" t="n"/>
+      <c r="J20" s="1427" t="n"/>
+      <c r="K20" s="1427" t="n"/>
+      <c r="L20" s="1427" t="n"/>
+      <c r="M20" s="1425" t="n"/>
+      <c r="N20" s="1425" t="n"/>
+      <c r="O20" s="1425" t="n"/>
+      <c r="P20" s="1428" t="n"/>
+      <c r="Q20" s="1425" t="n"/>
+      <c r="R20" s="1425" t="n"/>
+      <c r="S20" s="1425" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1382" t="n"/>
+      <c r="U20" s="1424" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -5958,39 +6066,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1357" t="inlineStr">
+      <c r="A21" s="1399" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1358" t="inlineStr">
+      <c r="B21" s="1400" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1358" t="inlineStr">
+      <c r="C21" s="1400" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1359" t="n"/>
-      <c r="E21" s="1359" t="n"/>
-      <c r="F21" s="1359" t="n"/>
-      <c r="G21" s="1359" t="n"/>
-      <c r="H21" s="1359" t="n"/>
-      <c r="I21" s="1360" t="n"/>
-      <c r="J21" s="1361" t="n"/>
-      <c r="K21" s="1361" t="n"/>
-      <c r="L21" s="1361" t="n"/>
-      <c r="M21" s="1359" t="n"/>
-      <c r="N21" s="1359" t="n"/>
-      <c r="O21" s="1359" t="n"/>
-      <c r="P21" s="1362" t="n"/>
-      <c r="Q21" s="1359" t="n"/>
-      <c r="R21" s="1359" t="n"/>
-      <c r="S21" s="1359" t="n"/>
+      <c r="D21" s="1401" t="n"/>
+      <c r="E21" s="1401" t="n"/>
+      <c r="F21" s="1401" t="n"/>
+      <c r="G21" s="1401" t="n"/>
+      <c r="H21" s="1401" t="n"/>
+      <c r="I21" s="1402" t="n"/>
+      <c r="J21" s="1403" t="n"/>
+      <c r="K21" s="1403" t="n"/>
+      <c r="L21" s="1403" t="n"/>
+      <c r="M21" s="1401" t="n"/>
+      <c r="N21" s="1401" t="n"/>
+      <c r="O21" s="1401" t="n"/>
+      <c r="P21" s="1404" t="n"/>
+      <c r="Q21" s="1401" t="n"/>
+      <c r="R21" s="1401" t="n"/>
+      <c r="S21" s="1401" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1358" t="n"/>
+      <c r="U21" s="1400" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -5998,39 +6106,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1363" t="inlineStr">
+      <c r="A22" s="1405" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1364" t="inlineStr">
+      <c r="B22" s="1406" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1364" t="inlineStr">
+      <c r="C22" s="1406" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1365" t="n"/>
-      <c r="E22" s="1365" t="n"/>
-      <c r="F22" s="1365" t="n"/>
-      <c r="G22" s="1365" t="n"/>
-      <c r="H22" s="1365" t="n"/>
-      <c r="I22" s="1366" t="n"/>
-      <c r="J22" s="1367" t="n"/>
-      <c r="K22" s="1367" t="n"/>
-      <c r="L22" s="1367" t="n"/>
-      <c r="M22" s="1365" t="n"/>
-      <c r="N22" s="1365" t="n"/>
-      <c r="O22" s="1365" t="n"/>
-      <c r="P22" s="1368" t="n"/>
-      <c r="Q22" s="1365" t="n"/>
-      <c r="R22" s="1365" t="n"/>
-      <c r="S22" s="1365" t="n"/>
+      <c r="D22" s="1407" t="n"/>
+      <c r="E22" s="1407" t="n"/>
+      <c r="F22" s="1407" t="n"/>
+      <c r="G22" s="1407" t="n"/>
+      <c r="H22" s="1407" t="n"/>
+      <c r="I22" s="1408" t="n"/>
+      <c r="J22" s="1409" t="n"/>
+      <c r="K22" s="1409" t="n"/>
+      <c r="L22" s="1409" t="n"/>
+      <c r="M22" s="1407" t="n"/>
+      <c r="N22" s="1407" t="n"/>
+      <c r="O22" s="1407" t="n"/>
+      <c r="P22" s="1410" t="n"/>
+      <c r="Q22" s="1407" t="n"/>
+      <c r="R22" s="1407" t="n"/>
+      <c r="S22" s="1407" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1364" t="n"/>
+      <c r="U22" s="1406" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -6038,53 +6146,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1369" t="inlineStr">
+      <c r="A23" s="1411" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1370" t="inlineStr">
+      <c r="B23" s="1412" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1370" t="inlineStr">
+      <c r="C23" s="1412" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1371" t="n"/>
-      <c r="E23" s="1371" t="n">
+      <c r="D23" s="1413" t="n"/>
+      <c r="E23" s="1413" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1371" t="n">
+      <c r="F23" s="1413" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1371" t="n">
+      <c r="G23" s="1413" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1371" t="n"/>
-      <c r="I23" s="1372" t="n"/>
-      <c r="J23" s="1373" t="n"/>
-      <c r="K23" s="1373" t="n"/>
-      <c r="L23" s="1373" t="n"/>
-      <c r="M23" s="1371" t="n"/>
-      <c r="N23" s="1371" t="n"/>
-      <c r="O23" s="1371" t="n">
+      <c r="H23" s="1413" t="n"/>
+      <c r="I23" s="1414" t="n"/>
+      <c r="J23" s="1415" t="n"/>
+      <c r="K23" s="1415" t="n"/>
+      <c r="L23" s="1415" t="n"/>
+      <c r="M23" s="1413" t="n"/>
+      <c r="N23" s="1413" t="n"/>
+      <c r="O23" s="1413" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1374" t="n">
+      <c r="P23" s="1416" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1371" t="n"/>
-      <c r="R23" s="1371" t="n"/>
-      <c r="S23" s="1371" t="n"/>
+      <c r="Q23" s="1413" t="n"/>
+      <c r="R23" s="1413" t="n"/>
+      <c r="S23" s="1413" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1370" t="n"/>
+      <c r="U23" s="1412" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -6092,47 +6200,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1375" t="inlineStr">
+      <c r="A24" s="1417" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1376" t="inlineStr">
+      <c r="B24" s="1418" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1376" t="inlineStr">
+      <c r="C24" s="1418" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1377" t="n"/>
-      <c r="E24" s="1377" t="n"/>
-      <c r="F24" s="1377" t="n"/>
-      <c r="G24" s="1377" t="n"/>
-      <c r="H24" s="1377" t="n"/>
-      <c r="I24" s="1378" t="n"/>
-      <c r="J24" s="1379" t="n"/>
-      <c r="K24" s="1379" t="n"/>
-      <c r="L24" s="1379" t="n"/>
-      <c r="M24" s="1377" t="n">
+      <c r="D24" s="1419" t="n"/>
+      <c r="E24" s="1419" t="n"/>
+      <c r="F24" s="1419" t="n"/>
+      <c r="G24" s="1419" t="n"/>
+      <c r="H24" s="1419" t="n"/>
+      <c r="I24" s="1420" t="n"/>
+      <c r="J24" s="1421" t="n"/>
+      <c r="K24" s="1421" t="n"/>
+      <c r="L24" s="1421" t="n"/>
+      <c r="M24" s="1419" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1377" t="n">
+      <c r="N24" s="1419" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1377" t="n"/>
-      <c r="P24" s="1380" t="n"/>
-      <c r="Q24" s="1377" t="n"/>
-      <c r="R24" s="1377" t="n"/>
-      <c r="S24" s="1377" t="n"/>
+      <c r="O24" s="1419" t="n"/>
+      <c r="P24" s="1422" t="n"/>
+      <c r="Q24" s="1419" t="n"/>
+      <c r="R24" s="1419" t="n"/>
+      <c r="S24" s="1419" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1376" t="n"/>
+      <c r="U24" s="1418" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -6140,61 +6248,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1351" t="inlineStr">
+      <c r="A25" s="1393" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1352" t="inlineStr">
+      <c r="B25" s="1394" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1352" t="inlineStr">
+      <c r="C25" s="1394" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1353" t="n">
+      <c r="D25" s="1395" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1353" t="n">
+      <c r="E25" s="1395" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1353" t="n">
+      <c r="F25" s="1395" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1353" t="n">
+      <c r="G25" s="1395" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1353" t="n"/>
-      <c r="I25" s="1354" t="n"/>
-      <c r="J25" s="1355" t="n">
+      <c r="H25" s="1395" t="n"/>
+      <c r="I25" s="1396" t="n"/>
+      <c r="J25" s="1397" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1355" t="n">
+      <c r="K25" s="1397" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1355" t="n">
+      <c r="L25" s="1397" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1353" t="n"/>
-      <c r="N25" s="1353" t="n"/>
-      <c r="O25" s="1353" t="n">
+      <c r="M25" s="1395" t="n"/>
+      <c r="N25" s="1395" t="n"/>
+      <c r="O25" s="1395" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1356" t="n">
+      <c r="P25" s="1398" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1353" t="n"/>
-      <c r="R25" s="1353" t="n"/>
-      <c r="S25" s="1353" t="n"/>
+      <c r="Q25" s="1395" t="n"/>
+      <c r="R25" s="1395" t="n"/>
+      <c r="S25" s="1395" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1352" t="n"/>
+      <c r="U25" s="1394" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -6202,47 +6310,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1357" t="inlineStr">
+      <c r="A26" s="1399" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1358" t="inlineStr">
+      <c r="B26" s="1400" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1358" t="inlineStr">
+      <c r="C26" s="1400" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1359" t="n"/>
-      <c r="E26" s="1359" t="n"/>
-      <c r="F26" s="1359" t="n"/>
-      <c r="G26" s="1359" t="n"/>
-      <c r="H26" s="1359" t="n"/>
-      <c r="I26" s="1360" t="n"/>
-      <c r="J26" s="1361" t="n"/>
-      <c r="K26" s="1361" t="n"/>
-      <c r="L26" s="1361" t="n"/>
-      <c r="M26" s="1359" t="n">
+      <c r="D26" s="1401" t="n"/>
+      <c r="E26" s="1401" t="n"/>
+      <c r="F26" s="1401" t="n"/>
+      <c r="G26" s="1401" t="n"/>
+      <c r="H26" s="1401" t="n"/>
+      <c r="I26" s="1402" t="n"/>
+      <c r="J26" s="1403" t="n"/>
+      <c r="K26" s="1403" t="n"/>
+      <c r="L26" s="1403" t="n"/>
+      <c r="M26" s="1401" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1359" t="n">
+      <c r="N26" s="1401" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1359" t="n"/>
-      <c r="P26" s="1362" t="n"/>
-      <c r="Q26" s="1359" t="n"/>
-      <c r="R26" s="1359" t="n"/>
-      <c r="S26" s="1359" t="n"/>
+      <c r="O26" s="1401" t="n"/>
+      <c r="P26" s="1404" t="n"/>
+      <c r="Q26" s="1401" t="n"/>
+      <c r="R26" s="1401" t="n"/>
+      <c r="S26" s="1401" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1358" t="n"/>
+      <c r="U26" s="1400" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -6250,53 +6358,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1363" t="inlineStr">
+      <c r="A27" s="1405" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1364" t="inlineStr">
+      <c r="B27" s="1406" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1364" t="inlineStr">
+      <c r="C27" s="1406" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1365" t="n"/>
-      <c r="E27" s="1365" t="n">
+      <c r="D27" s="1407" t="n"/>
+      <c r="E27" s="1407" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1365" t="n">
+      <c r="F27" s="1407" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1365" t="n">
+      <c r="G27" s="1407" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1365" t="n"/>
-      <c r="I27" s="1366" t="n"/>
-      <c r="J27" s="1367" t="n"/>
-      <c r="K27" s="1367" t="n"/>
-      <c r="L27" s="1367" t="n"/>
-      <c r="M27" s="1365" t="n"/>
-      <c r="N27" s="1365" t="n"/>
-      <c r="O27" s="1365" t="n">
+      <c r="H27" s="1407" t="n"/>
+      <c r="I27" s="1408" t="n"/>
+      <c r="J27" s="1409" t="n"/>
+      <c r="K27" s="1409" t="n"/>
+      <c r="L27" s="1409" t="n"/>
+      <c r="M27" s="1407" t="n"/>
+      <c r="N27" s="1407" t="n"/>
+      <c r="O27" s="1407" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1368" t="n">
+      <c r="P27" s="1410" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1365" t="n"/>
-      <c r="R27" s="1365" t="n"/>
-      <c r="S27" s="1365" t="n"/>
+      <c r="Q27" s="1407" t="n"/>
+      <c r="R27" s="1407" t="n"/>
+      <c r="S27" s="1407" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1364" t="n"/>
+      <c r="U27" s="1406" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -6304,47 +6412,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1375" t="inlineStr">
+      <c r="A28" s="1417" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1376" t="inlineStr">
+      <c r="B28" s="1418" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1376" t="inlineStr">
+      <c r="C28" s="1418" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1377" t="n"/>
-      <c r="E28" s="1377" t="n"/>
-      <c r="F28" s="1377" t="n"/>
-      <c r="G28" s="1377" t="n"/>
-      <c r="H28" s="1377" t="n"/>
-      <c r="I28" s="1378" t="n"/>
-      <c r="J28" s="1379" t="n"/>
-      <c r="K28" s="1379" t="n"/>
-      <c r="L28" s="1379" t="n"/>
-      <c r="M28" s="1377" t="n">
+      <c r="D28" s="1419" t="n"/>
+      <c r="E28" s="1419" t="n"/>
+      <c r="F28" s="1419" t="n"/>
+      <c r="G28" s="1419" t="n"/>
+      <c r="H28" s="1419" t="n"/>
+      <c r="I28" s="1420" t="n"/>
+      <c r="J28" s="1421" t="n"/>
+      <c r="K28" s="1421" t="n"/>
+      <c r="L28" s="1421" t="n"/>
+      <c r="M28" s="1419" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1377" t="n">
+      <c r="N28" s="1419" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1377" t="n"/>
-      <c r="P28" s="1380" t="n"/>
-      <c r="Q28" s="1377" t="n"/>
-      <c r="R28" s="1377" t="n"/>
-      <c r="S28" s="1377" t="n"/>
+      <c r="O28" s="1419" t="n"/>
+      <c r="P28" s="1422" t="n"/>
+      <c r="Q28" s="1419" t="n"/>
+      <c r="R28" s="1419" t="n"/>
+      <c r="S28" s="1419" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1376" t="n"/>
+      <c r="U28" s="1418" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -6352,53 +6460,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1351" t="inlineStr">
+      <c r="A29" s="1393" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1352" t="inlineStr">
+      <c r="B29" s="1394" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1352" t="inlineStr">
+      <c r="C29" s="1394" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1353" t="n"/>
-      <c r="E29" s="1353" t="n">
+      <c r="D29" s="1395" t="n"/>
+      <c r="E29" s="1395" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1353" t="n">
+      <c r="F29" s="1395" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1353" t="n">
+      <c r="G29" s="1395" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1353" t="n"/>
-      <c r="I29" s="1354" t="n"/>
-      <c r="J29" s="1355" t="n"/>
-      <c r="K29" s="1355" t="n"/>
-      <c r="L29" s="1355" t="n"/>
-      <c r="M29" s="1353" t="n"/>
-      <c r="N29" s="1353" t="n"/>
-      <c r="O29" s="1353" t="n">
+      <c r="H29" s="1395" t="n"/>
+      <c r="I29" s="1396" t="n"/>
+      <c r="J29" s="1397" t="n"/>
+      <c r="K29" s="1397" t="n"/>
+      <c r="L29" s="1397" t="n"/>
+      <c r="M29" s="1395" t="n"/>
+      <c r="N29" s="1395" t="n"/>
+      <c r="O29" s="1395" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1356" t="n">
+      <c r="P29" s="1398" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1353" t="n"/>
-      <c r="R29" s="1353" t="n"/>
-      <c r="S29" s="1353" t="n"/>
+      <c r="Q29" s="1395" t="n"/>
+      <c r="R29" s="1395" t="n"/>
+      <c r="S29" s="1395" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1352" t="n"/>
+      <c r="U29" s="1394" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -6406,43 +6514,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1357" t="inlineStr">
+      <c r="A30" s="1399" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1358" t="inlineStr">
+      <c r="B30" s="1400" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1358" t="inlineStr">
+      <c r="C30" s="1400" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1359" t="n"/>
-      <c r="E30" s="1359" t="n"/>
-      <c r="F30" s="1359" t="n"/>
-      <c r="G30" s="1359" t="n"/>
-      <c r="H30" s="1359" t="n"/>
-      <c r="I30" s="1360" t="n"/>
-      <c r="J30" s="1361" t="n"/>
-      <c r="K30" s="1361" t="n"/>
-      <c r="L30" s="1361" t="n"/>
-      <c r="M30" s="1359" t="n"/>
-      <c r="N30" s="1359" t="n"/>
-      <c r="O30" s="1359" t="n"/>
-      <c r="P30" s="1362" t="n"/>
-      <c r="Q30" s="1359" t="n"/>
-      <c r="R30" s="1359" t="n"/>
-      <c r="S30" s="1359" t="n"/>
+      <c r="D30" s="1401" t="n"/>
+      <c r="E30" s="1401" t="n"/>
+      <c r="F30" s="1401" t="n"/>
+      <c r="G30" s="1401" t="n"/>
+      <c r="H30" s="1401" t="n"/>
+      <c r="I30" s="1402" t="n"/>
+      <c r="J30" s="1403" t="n"/>
+      <c r="K30" s="1403" t="n"/>
+      <c r="L30" s="1403" t="n"/>
+      <c r="M30" s="1401" t="n"/>
+      <c r="N30" s="1401" t="n"/>
+      <c r="O30" s="1401" t="n"/>
+      <c r="P30" s="1404" t="n"/>
+      <c r="Q30" s="1401" t="n"/>
+      <c r="R30" s="1401" t="n"/>
+      <c r="S30" s="1401" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1358" t="n"/>
+      <c r="U30" s="1400" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -6450,53 +6558,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1363" t="inlineStr">
+      <c r="A31" s="1405" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1364" t="inlineStr">
+      <c r="B31" s="1406" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1364" t="inlineStr">
+      <c r="C31" s="1406" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1365" t="n"/>
-      <c r="E31" s="1365" t="n">
+      <c r="D31" s="1407" t="n"/>
+      <c r="E31" s="1407" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1365" t="n">
+      <c r="F31" s="1407" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1365" t="n">
+      <c r="G31" s="1407" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1365" t="n"/>
-      <c r="I31" s="1366" t="n"/>
-      <c r="J31" s="1367" t="n"/>
-      <c r="K31" s="1367" t="n"/>
-      <c r="L31" s="1367" t="n"/>
-      <c r="M31" s="1365" t="n"/>
-      <c r="N31" s="1365" t="n"/>
-      <c r="O31" s="1365" t="n">
+      <c r="H31" s="1407" t="n"/>
+      <c r="I31" s="1408" t="n"/>
+      <c r="J31" s="1409" t="n"/>
+      <c r="K31" s="1409" t="n"/>
+      <c r="L31" s="1409" t="n"/>
+      <c r="M31" s="1407" t="n"/>
+      <c r="N31" s="1407" t="n"/>
+      <c r="O31" s="1407" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1368" t="n">
+      <c r="P31" s="1410" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1365" t="n"/>
-      <c r="R31" s="1365" t="n"/>
-      <c r="S31" s="1365" t="n"/>
+      <c r="Q31" s="1407" t="n"/>
+      <c r="R31" s="1407" t="n"/>
+      <c r="S31" s="1407" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1364" t="inlineStr">
+      <c r="U31" s="1406" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -6508,49 +6616,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1375" t="inlineStr">
+      <c r="A32" s="1417" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1376" t="inlineStr">
+      <c r="B32" s="1418" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1376" t="inlineStr">
+      <c r="C32" s="1418" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1377" t="n"/>
-      <c r="E32" s="1377" t="n"/>
-      <c r="F32" s="1377" t="n"/>
-      <c r="G32" s="1377" t="n"/>
-      <c r="H32" s="1377" t="n">
+      <c r="D32" s="1419" t="n"/>
+      <c r="E32" s="1419" t="n"/>
+      <c r="F32" s="1419" t="n"/>
+      <c r="G32" s="1419" t="n"/>
+      <c r="H32" s="1419" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1378" t="n"/>
-      <c r="J32" s="1379" t="n"/>
-      <c r="K32" s="1379" t="n"/>
-      <c r="L32" s="1379" t="n"/>
-      <c r="M32" s="1377" t="n">
+      <c r="I32" s="1420" t="n"/>
+      <c r="J32" s="1421" t="n"/>
+      <c r="K32" s="1421" t="n"/>
+      <c r="L32" s="1421" t="n"/>
+      <c r="M32" s="1419" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1377" t="n">
+      <c r="N32" s="1419" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1377" t="n"/>
-      <c r="P32" s="1380" t="n"/>
-      <c r="Q32" s="1377" t="n"/>
-      <c r="R32" s="1377" t="n"/>
-      <c r="S32" s="1377" t="n"/>
+      <c r="O32" s="1419" t="n"/>
+      <c r="P32" s="1422" t="n"/>
+      <c r="Q32" s="1419" t="n"/>
+      <c r="R32" s="1419" t="n"/>
+      <c r="S32" s="1419" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1376" t="n"/>
+      <c r="U32" s="1418" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -6558,57 +6666,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1351" t="inlineStr">
+      <c r="A33" s="1393" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1352" t="inlineStr">
+      <c r="B33" s="1394" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1352" t="inlineStr">
+      <c r="C33" s="1394" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1353" t="n"/>
-      <c r="E33" s="1353" t="n">
+      <c r="D33" s="1395" t="n"/>
+      <c r="E33" s="1395" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1353" t="n">
+      <c r="F33" s="1395" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1353" t="n">
+      <c r="G33" s="1395" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1353" t="n"/>
-      <c r="I33" s="1354" t="n">
+      <c r="H33" s="1395" t="n"/>
+      <c r="I33" s="1396" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1355" t="n"/>
-      <c r="K33" s="1355" t="n"/>
-      <c r="L33" s="1355" t="n"/>
-      <c r="M33" s="1353" t="n"/>
-      <c r="N33" s="1353" t="n"/>
-      <c r="O33" s="1353" t="n">
+      <c r="J33" s="1397" t="n"/>
+      <c r="K33" s="1397" t="n"/>
+      <c r="L33" s="1397" t="n"/>
+      <c r="M33" s="1395" t="n"/>
+      <c r="N33" s="1395" t="n"/>
+      <c r="O33" s="1395" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1356" t="n">
+      <c r="P33" s="1398" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1353" t="n"/>
-      <c r="R33" s="1353" t="n">
+      <c r="Q33" s="1395" t="n"/>
+      <c r="R33" s="1395" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1353" t="n"/>
+      <c r="S33" s="1395" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1352" t="inlineStr">
+      <c r="U33" s="1394" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -6620,49 +6728,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1357" t="inlineStr">
+      <c r="A34" s="1399" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1358" t="inlineStr">
+      <c r="B34" s="1400" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1358" t="inlineStr">
+      <c r="C34" s="1400" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1359" t="n"/>
-      <c r="E34" s="1359" t="n"/>
-      <c r="F34" s="1359" t="n"/>
-      <c r="G34" s="1359" t="n"/>
-      <c r="H34" s="1359" t="n">
+      <c r="D34" s="1401" t="n"/>
+      <c r="E34" s="1401" t="n"/>
+      <c r="F34" s="1401" t="n"/>
+      <c r="G34" s="1401" t="n"/>
+      <c r="H34" s="1401" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1360" t="n"/>
-      <c r="J34" s="1361" t="n"/>
-      <c r="K34" s="1361" t="n"/>
-      <c r="L34" s="1361" t="n"/>
-      <c r="M34" s="1359" t="n">
+      <c r="I34" s="1402" t="n"/>
+      <c r="J34" s="1403" t="n"/>
+      <c r="K34" s="1403" t="n"/>
+      <c r="L34" s="1403" t="n"/>
+      <c r="M34" s="1401" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1359" t="n">
+      <c r="N34" s="1401" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1359" t="n"/>
-      <c r="P34" s="1362" t="n"/>
-      <c r="Q34" s="1359" t="n"/>
-      <c r="R34" s="1359" t="n"/>
-      <c r="S34" s="1359" t="n"/>
+      <c r="O34" s="1401" t="n"/>
+      <c r="P34" s="1404" t="n"/>
+      <c r="Q34" s="1401" t="n"/>
+      <c r="R34" s="1401" t="n"/>
+      <c r="S34" s="1401" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1358" t="n"/>
+      <c r="U34" s="1400" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -6670,57 +6778,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1363" t="inlineStr">
+      <c r="A35" s="1405" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1364" t="inlineStr">
+      <c r="B35" s="1406" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1364" t="inlineStr">
+      <c r="C35" s="1406" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1365" t="n"/>
-      <c r="E35" s="1365" t="n">
+      <c r="D35" s="1407" t="n"/>
+      <c r="E35" s="1407" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1365" t="n">
+      <c r="F35" s="1407" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1365" t="n">
+      <c r="G35" s="1407" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1365" t="n"/>
-      <c r="I35" s="1366" t="n">
+      <c r="H35" s="1407" t="n"/>
+      <c r="I35" s="1408" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1367" t="n"/>
-      <c r="K35" s="1367" t="n"/>
-      <c r="L35" s="1367" t="n"/>
-      <c r="M35" s="1365" t="n"/>
-      <c r="N35" s="1365" t="n"/>
-      <c r="O35" s="1365" t="n">
+      <c r="J35" s="1409" t="n"/>
+      <c r="K35" s="1409" t="n"/>
+      <c r="L35" s="1409" t="n"/>
+      <c r="M35" s="1407" t="n"/>
+      <c r="N35" s="1407" t="n"/>
+      <c r="O35" s="1407" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1368" t="n">
+      <c r="P35" s="1410" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1365" t="n"/>
-      <c r="R35" s="1365" t="n">
+      <c r="Q35" s="1407" t="n"/>
+      <c r="R35" s="1407" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1365" t="n"/>
+      <c r="S35" s="1407" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1364" t="inlineStr">
+      <c r="U35" s="1406" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -6732,49 +6840,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1369" t="inlineStr">
+      <c r="A36" s="1411" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1370" t="inlineStr">
+      <c r="B36" s="1412" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1370" t="inlineStr">
+      <c r="C36" s="1412" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1371" t="n"/>
-      <c r="E36" s="1371" t="n"/>
-      <c r="F36" s="1371" t="n"/>
-      <c r="G36" s="1371" t="n"/>
-      <c r="H36" s="1371" t="n">
+      <c r="D36" s="1413" t="n"/>
+      <c r="E36" s="1413" t="n"/>
+      <c r="F36" s="1413" t="n"/>
+      <c r="G36" s="1413" t="n"/>
+      <c r="H36" s="1413" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1372" t="n"/>
-      <c r="J36" s="1373" t="n"/>
-      <c r="K36" s="1373" t="n"/>
-      <c r="L36" s="1373" t="n"/>
-      <c r="M36" s="1371" t="n">
+      <c r="I36" s="1414" t="n"/>
+      <c r="J36" s="1415" t="n"/>
+      <c r="K36" s="1415" t="n"/>
+      <c r="L36" s="1415" t="n"/>
+      <c r="M36" s="1413" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1371" t="n">
+      <c r="N36" s="1413" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1371" t="n"/>
-      <c r="P36" s="1374" t="n"/>
-      <c r="Q36" s="1371" t="n"/>
-      <c r="R36" s="1371" t="n"/>
-      <c r="S36" s="1371" t="n"/>
+      <c r="O36" s="1413" t="n"/>
+      <c r="P36" s="1416" t="n"/>
+      <c r="Q36" s="1413" t="n"/>
+      <c r="R36" s="1413" t="n"/>
+      <c r="S36" s="1413" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1370" t="n"/>
+      <c r="U36" s="1412" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -6782,41 +6890,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1375" t="inlineStr">
+      <c r="A37" s="1417" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1376" t="inlineStr">
+      <c r="B37" s="1418" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1376" t="inlineStr">
+      <c r="C37" s="1418" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1377" t="n"/>
-      <c r="E37" s="1377" t="n"/>
-      <c r="F37" s="1377" t="n"/>
-      <c r="G37" s="1377" t="n"/>
-      <c r="H37" s="1377" t="n"/>
-      <c r="I37" s="1378" t="n"/>
-      <c r="J37" s="1379" t="n"/>
-      <c r="K37" s="1379" t="n"/>
-      <c r="L37" s="1379" t="n"/>
-      <c r="M37" s="1377" t="n"/>
-      <c r="N37" s="1377" t="n"/>
-      <c r="O37" s="1377" t="n"/>
-      <c r="P37" s="1380" t="n"/>
-      <c r="Q37" s="1377" t="n">
+      <c r="D37" s="1419" t="n"/>
+      <c r="E37" s="1419" t="n"/>
+      <c r="F37" s="1419" t="n"/>
+      <c r="G37" s="1419" t="n"/>
+      <c r="H37" s="1419" t="n"/>
+      <c r="I37" s="1420" t="n"/>
+      <c r="J37" s="1421" t="n"/>
+      <c r="K37" s="1421" t="n"/>
+      <c r="L37" s="1421" t="n"/>
+      <c r="M37" s="1419" t="n"/>
+      <c r="N37" s="1419" t="n"/>
+      <c r="O37" s="1419" t="n"/>
+      <c r="P37" s="1422" t="n"/>
+      <c r="Q37" s="1419" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1377" t="n"/>
-      <c r="S37" s="1377" t="n"/>
+      <c r="R37" s="1419" t="n"/>
+      <c r="S37" s="1419" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1376" t="n"/>
+      <c r="U37" s="1418" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -6824,57 +6932,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1351" t="inlineStr">
+      <c r="A38" s="1393" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1352" t="inlineStr">
+      <c r="B38" s="1394" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1352" t="inlineStr">
+      <c r="C38" s="1394" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1353" t="n"/>
-      <c r="E38" s="1353" t="n">
+      <c r="D38" s="1395" t="n"/>
+      <c r="E38" s="1395" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1353" t="n">
+      <c r="F38" s="1395" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1353" t="n">
+      <c r="G38" s="1395" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1353" t="n"/>
-      <c r="I38" s="1354" t="n">
+      <c r="H38" s="1395" t="n"/>
+      <c r="I38" s="1396" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1355" t="n"/>
-      <c r="K38" s="1355" t="n"/>
-      <c r="L38" s="1355" t="n"/>
-      <c r="M38" s="1353" t="n"/>
-      <c r="N38" s="1353" t="n"/>
-      <c r="O38" s="1353" t="n">
+      <c r="J38" s="1397" t="n"/>
+      <c r="K38" s="1397" t="n"/>
+      <c r="L38" s="1397" t="n"/>
+      <c r="M38" s="1395" t="n"/>
+      <c r="N38" s="1395" t="n"/>
+      <c r="O38" s="1395" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1356" t="n">
+      <c r="P38" s="1398" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1353" t="n"/>
-      <c r="R38" s="1353" t="n">
+      <c r="Q38" s="1395" t="n"/>
+      <c r="R38" s="1395" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1353" t="n"/>
+      <c r="S38" s="1395" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1352" t="inlineStr">
+      <c r="U38" s="1394" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -6886,49 +6994,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1381" t="inlineStr">
+      <c r="A39" s="1423" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1382" t="inlineStr">
+      <c r="B39" s="1424" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1382" t="inlineStr">
+      <c r="C39" s="1424" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1383" t="n"/>
-      <c r="E39" s="1383" t="n"/>
-      <c r="F39" s="1383" t="n"/>
-      <c r="G39" s="1383" t="n"/>
-      <c r="H39" s="1383" t="n">
+      <c r="D39" s="1425" t="n"/>
+      <c r="E39" s="1425" t="n"/>
+      <c r="F39" s="1425" t="n"/>
+      <c r="G39" s="1425" t="n"/>
+      <c r="H39" s="1425" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1384" t="n"/>
-      <c r="J39" s="1385" t="n"/>
-      <c r="K39" s="1385" t="n"/>
-      <c r="L39" s="1385" t="n"/>
-      <c r="M39" s="1383" t="n">
+      <c r="I39" s="1426" t="n"/>
+      <c r="J39" s="1427" t="n"/>
+      <c r="K39" s="1427" t="n"/>
+      <c r="L39" s="1427" t="n"/>
+      <c r="M39" s="1425" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1383" t="n">
+      <c r="N39" s="1425" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1383" t="n"/>
-      <c r="P39" s="1386" t="n"/>
-      <c r="Q39" s="1383" t="n"/>
-      <c r="R39" s="1383" t="n"/>
-      <c r="S39" s="1383" t="n"/>
+      <c r="O39" s="1425" t="n"/>
+      <c r="P39" s="1428" t="n"/>
+      <c r="Q39" s="1425" t="n"/>
+      <c r="R39" s="1425" t="n"/>
+      <c r="S39" s="1425" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1382" t="n"/>
+      <c r="U39" s="1424" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -6936,41 +7044,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1357" t="inlineStr">
+      <c r="A40" s="1399" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1358" t="inlineStr">
+      <c r="B40" s="1400" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1358" t="inlineStr">
+      <c r="C40" s="1400" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1359" t="n"/>
-      <c r="E40" s="1359" t="n"/>
-      <c r="F40" s="1359" t="n"/>
-      <c r="G40" s="1359" t="n"/>
-      <c r="H40" s="1359" t="n"/>
-      <c r="I40" s="1360" t="n"/>
-      <c r="J40" s="1361" t="n"/>
-      <c r="K40" s="1361" t="n"/>
-      <c r="L40" s="1361" t="n"/>
-      <c r="M40" s="1359" t="n"/>
-      <c r="N40" s="1359" t="n"/>
-      <c r="O40" s="1359" t="n"/>
-      <c r="P40" s="1362" t="n"/>
-      <c r="Q40" s="1359" t="n">
+      <c r="D40" s="1401" t="n"/>
+      <c r="E40" s="1401" t="n"/>
+      <c r="F40" s="1401" t="n"/>
+      <c r="G40" s="1401" t="n"/>
+      <c r="H40" s="1401" t="n"/>
+      <c r="I40" s="1402" t="n"/>
+      <c r="J40" s="1403" t="n"/>
+      <c r="K40" s="1403" t="n"/>
+      <c r="L40" s="1403" t="n"/>
+      <c r="M40" s="1401" t="n"/>
+      <c r="N40" s="1401" t="n"/>
+      <c r="O40" s="1401" t="n"/>
+      <c r="P40" s="1404" t="n"/>
+      <c r="Q40" s="1401" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1359" t="n"/>
-      <c r="S40" s="1359" t="n"/>
+      <c r="R40" s="1401" t="n"/>
+      <c r="S40" s="1401" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1358" t="n"/>
+      <c r="U40" s="1400" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -6978,57 +7086,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1363" t="inlineStr">
+      <c r="A41" s="1405" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1364" t="inlineStr">
+      <c r="B41" s="1406" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1364" t="inlineStr">
+      <c r="C41" s="1406" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1365" t="n"/>
-      <c r="E41" s="1365" t="n">
+      <c r="D41" s="1407" t="n"/>
+      <c r="E41" s="1407" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1365" t="n">
+      <c r="F41" s="1407" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1365" t="n">
+      <c r="G41" s="1407" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1365" t="n"/>
-      <c r="I41" s="1366" t="n">
+      <c r="H41" s="1407" t="n"/>
+      <c r="I41" s="1408" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1367" t="n"/>
-      <c r="K41" s="1367" t="n"/>
-      <c r="L41" s="1367" t="n"/>
-      <c r="M41" s="1365" t="n"/>
-      <c r="N41" s="1365" t="n"/>
-      <c r="O41" s="1365" t="n">
+      <c r="J41" s="1409" t="n"/>
+      <c r="K41" s="1409" t="n"/>
+      <c r="L41" s="1409" t="n"/>
+      <c r="M41" s="1407" t="n"/>
+      <c r="N41" s="1407" t="n"/>
+      <c r="O41" s="1407" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1368" t="n">
+      <c r="P41" s="1410" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1365" t="n"/>
-      <c r="R41" s="1365" t="n">
+      <c r="Q41" s="1407" t="n"/>
+      <c r="R41" s="1407" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1365" t="n"/>
+      <c r="S41" s="1407" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1364" t="inlineStr">
+      <c r="U41" s="1406" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -7040,49 +7148,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1375" t="inlineStr">
+      <c r="A42" s="1417" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1376" t="inlineStr">
+      <c r="B42" s="1418" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1376" t="inlineStr">
+      <c r="C42" s="1418" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1377" t="n"/>
-      <c r="E42" s="1377" t="n"/>
-      <c r="F42" s="1377" t="n"/>
-      <c r="G42" s="1377" t="n"/>
-      <c r="H42" s="1377" t="n">
+      <c r="D42" s="1419" t="n"/>
+      <c r="E42" s="1419" t="n"/>
+      <c r="F42" s="1419" t="n"/>
+      <c r="G42" s="1419" t="n"/>
+      <c r="H42" s="1419" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1378" t="n"/>
-      <c r="J42" s="1379" t="n"/>
-      <c r="K42" s="1379" t="n"/>
-      <c r="L42" s="1379" t="n"/>
-      <c r="M42" s="1377" t="n">
+      <c r="I42" s="1420" t="n"/>
+      <c r="J42" s="1421" t="n"/>
+      <c r="K42" s="1421" t="n"/>
+      <c r="L42" s="1421" t="n"/>
+      <c r="M42" s="1419" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1377" t="n">
+      <c r="N42" s="1419" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1377" t="n"/>
-      <c r="P42" s="1380" t="n"/>
-      <c r="Q42" s="1377" t="n"/>
-      <c r="R42" s="1377" t="n"/>
-      <c r="S42" s="1377" t="n"/>
+      <c r="O42" s="1419" t="n"/>
+      <c r="P42" s="1422" t="n"/>
+      <c r="Q42" s="1419" t="n"/>
+      <c r="R42" s="1419" t="n"/>
+      <c r="S42" s="1419" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1376" t="n"/>
+      <c r="U42" s="1418" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -7090,57 +7198,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1351" t="inlineStr">
+      <c r="A43" s="1393" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1352" t="inlineStr">
+      <c r="B43" s="1394" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1352" t="inlineStr">
+      <c r="C43" s="1394" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1353" t="n"/>
-      <c r="E43" s="1353" t="n">
+      <c r="D43" s="1395" t="n"/>
+      <c r="E43" s="1395" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1353" t="n">
+      <c r="F43" s="1395" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1353" t="n">
+      <c r="G43" s="1395" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1353" t="n"/>
-      <c r="I43" s="1354" t="n">
+      <c r="H43" s="1395" t="n"/>
+      <c r="I43" s="1396" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1355" t="n"/>
-      <c r="K43" s="1355" t="n"/>
-      <c r="L43" s="1355" t="n"/>
-      <c r="M43" s="1353" t="n"/>
-      <c r="N43" s="1353" t="n"/>
-      <c r="O43" s="1353" t="n">
+      <c r="J43" s="1397" t="n"/>
+      <c r="K43" s="1397" t="n"/>
+      <c r="L43" s="1397" t="n"/>
+      <c r="M43" s="1395" t="n"/>
+      <c r="N43" s="1395" t="n"/>
+      <c r="O43" s="1395" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1356" t="n">
+      <c r="P43" s="1398" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1353" t="n"/>
-      <c r="R43" s="1353" t="n">
+      <c r="Q43" s="1395" t="n"/>
+      <c r="R43" s="1395" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1353" t="n"/>
+      <c r="S43" s="1395" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1352" t="n"/>
+      <c r="U43" s="1394" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -7148,45 +7256,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1381" t="inlineStr">
+      <c r="A44" s="1423" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1382" t="inlineStr">
+      <c r="B44" s="1424" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1382" t="inlineStr">
+      <c r="C44" s="1424" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1383" t="n"/>
-      <c r="E44" s="1383" t="n">
+      <c r="D44" s="1425" t="n"/>
+      <c r="E44" s="1425" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1383" t="n">
+      <c r="F44" s="1425" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1383" t="n"/>
-      <c r="H44" s="1383" t="n"/>
-      <c r="I44" s="1384" t="n"/>
-      <c r="J44" s="1385" t="n"/>
-      <c r="K44" s="1385" t="n"/>
-      <c r="L44" s="1385" t="n"/>
-      <c r="M44" s="1383" t="n"/>
-      <c r="N44" s="1383" t="n"/>
-      <c r="O44" s="1383" t="n"/>
-      <c r="P44" s="1386" t="n"/>
-      <c r="Q44" s="1383" t="n"/>
-      <c r="R44" s="1383" t="n"/>
-      <c r="S44" s="1383" t="n">
+      <c r="G44" s="1425" t="n"/>
+      <c r="H44" s="1425" t="n"/>
+      <c r="I44" s="1426" t="n"/>
+      <c r="J44" s="1427" t="n"/>
+      <c r="K44" s="1427" t="n"/>
+      <c r="L44" s="1427" t="n"/>
+      <c r="M44" s="1425" t="n"/>
+      <c r="N44" s="1425" t="n"/>
+      <c r="O44" s="1425" t="n"/>
+      <c r="P44" s="1428" t="n"/>
+      <c r="Q44" s="1425" t="n"/>
+      <c r="R44" s="1425" t="n"/>
+      <c r="S44" s="1425" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1382" t="inlineStr">
+      <c r="U44" s="1424" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -7198,49 +7306,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1381" t="inlineStr">
+      <c r="A45" s="1423" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1382" t="inlineStr">
+      <c r="B45" s="1424" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1382" t="inlineStr">
+      <c r="C45" s="1424" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1383" t="n"/>
-      <c r="E45" s="1383" t="n"/>
-      <c r="F45" s="1383" t="n"/>
-      <c r="G45" s="1383" t="n"/>
-      <c r="H45" s="1383" t="n">
+      <c r="D45" s="1425" t="n"/>
+      <c r="E45" s="1425" t="n"/>
+      <c r="F45" s="1425" t="n"/>
+      <c r="G45" s="1425" t="n"/>
+      <c r="H45" s="1425" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1384" t="n"/>
-      <c r="J45" s="1385" t="n"/>
-      <c r="K45" s="1385" t="n"/>
-      <c r="L45" s="1385" t="n"/>
-      <c r="M45" s="1383" t="n">
+      <c r="I45" s="1426" t="n"/>
+      <c r="J45" s="1427" t="n"/>
+      <c r="K45" s="1427" t="n"/>
+      <c r="L45" s="1427" t="n"/>
+      <c r="M45" s="1425" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1383" t="n">
+      <c r="N45" s="1425" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1383" t="n"/>
-      <c r="P45" s="1386" t="n"/>
-      <c r="Q45" s="1383" t="n"/>
-      <c r="R45" s="1383" t="n"/>
-      <c r="S45" s="1383" t="n"/>
+      <c r="O45" s="1425" t="n"/>
+      <c r="P45" s="1428" t="n"/>
+      <c r="Q45" s="1425" t="n"/>
+      <c r="R45" s="1425" t="n"/>
+      <c r="S45" s="1425" t="n"/>
       <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1382" t="n"/>
+      <c r="U45" s="1424" t="n"/>
       <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -7248,39 +7356,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1357" t="inlineStr">
+      <c r="A46" s="1399" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B46" s="1358" t="inlineStr">
+      <c r="B46" s="1400" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="C46" s="1358" t="inlineStr">
+      <c r="C46" s="1400" t="inlineStr">
         <is>
           <t>EVENT - Clean</t>
         </is>
       </c>
-      <c r="D46" s="1359" t="n"/>
-      <c r="E46" s="1359" t="n"/>
-      <c r="F46" s="1359" t="n"/>
-      <c r="G46" s="1359" t="n"/>
-      <c r="H46" s="1359" t="n"/>
-      <c r="I46" s="1360" t="n"/>
-      <c r="J46" s="1361" t="n"/>
-      <c r="K46" s="1361" t="n"/>
-      <c r="L46" s="1361" t="n"/>
-      <c r="M46" s="1359" t="n"/>
-      <c r="N46" s="1359" t="n"/>
-      <c r="O46" s="1359" t="n"/>
-      <c r="P46" s="1362" t="n"/>
-      <c r="Q46" s="1359" t="n"/>
-      <c r="R46" s="1359" t="n"/>
-      <c r="S46" s="1359" t="n"/>
+      <c r="D46" s="1401" t="n"/>
+      <c r="E46" s="1401" t="n"/>
+      <c r="F46" s="1401" t="n"/>
+      <c r="G46" s="1401" t="n"/>
+      <c r="H46" s="1401" t="n"/>
+      <c r="I46" s="1402" t="n"/>
+      <c r="J46" s="1403" t="n"/>
+      <c r="K46" s="1403" t="n"/>
+      <c r="L46" s="1403" t="n"/>
+      <c r="M46" s="1401" t="n"/>
+      <c r="N46" s="1401" t="n"/>
+      <c r="O46" s="1401" t="n"/>
+      <c r="P46" s="1404" t="n"/>
+      <c r="Q46" s="1401" t="n"/>
+      <c r="R46" s="1401" t="n"/>
+      <c r="S46" s="1401" t="n"/>
       <c r="T46" s="631" t="n"/>
-      <c r="U46" s="1358" t="n"/>
+      <c r="U46" s="1400" t="n"/>
       <c r="V46" s="632" t="inlineStr">
         <is>
           <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
@@ -7288,51 +7396,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1363" t="inlineStr">
+      <c r="A47" s="1405" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1364" t="inlineStr">
+      <c r="B47" s="1406" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C47" s="1364" t="inlineStr">
+      <c r="C47" s="1406" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D47" s="1365" t="n"/>
-      <c r="E47" s="1365" t="n">
+      <c r="D47" s="1407" t="n"/>
+      <c r="E47" s="1407" t="n">
         <v>16.6</v>
       </c>
-      <c r="F47" s="1365" t="n">
+      <c r="F47" s="1407" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="1365" t="n">
+      <c r="G47" s="1407" t="n">
         <v>4.1</v>
       </c>
-      <c r="H47" s="1365" t="n"/>
-      <c r="I47" s="1366" t="n">
+      <c r="H47" s="1407" t="n"/>
+      <c r="I47" s="1408" t="n">
         <v>0.9</v>
       </c>
-      <c r="J47" s="1367" t="n"/>
-      <c r="K47" s="1367" t="n"/>
-      <c r="L47" s="1367" t="n"/>
-      <c r="M47" s="1365" t="n"/>
-      <c r="N47" s="1365" t="n"/>
-      <c r="O47" s="1365" t="n">
+      <c r="J47" s="1409" t="n"/>
+      <c r="K47" s="1409" t="n"/>
+      <c r="L47" s="1409" t="n"/>
+      <c r="M47" s="1407" t="n"/>
+      <c r="N47" s="1407" t="n"/>
+      <c r="O47" s="1407" t="n">
         <v>13.2</v>
       </c>
-      <c r="P47" s="1368" t="n">
+      <c r="P47" s="1410" t="n">
         <v>0</v>
       </c>
-      <c r="Q47" s="1365" t="n"/>
-      <c r="R47" s="1365" t="n">
+      <c r="Q47" s="1407" t="n"/>
+      <c r="R47" s="1407" t="n">
         <v>84.5</v>
       </c>
-      <c r="S47" s="1365" t="n">
+      <c r="S47" s="1407" t="n">
         <v>11.8</v>
       </c>
       <c r="T47" s="813" t="inlineStr">
@@ -7340,7 +7448,7 @@
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1364" t="inlineStr">
+      <c r="U47" s="1406" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
@@ -7352,49 +7460,49 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1375" t="inlineStr">
+      <c r="A48" s="1417" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B48" s="1376" t="inlineStr">
+      <c r="B48" s="1418" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C48" s="1376" t="inlineStr">
+      <c r="C48" s="1418" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D48" s="1377" t="n"/>
-      <c r="E48" s="1377" t="n"/>
-      <c r="F48" s="1377" t="n"/>
-      <c r="G48" s="1377" t="n"/>
-      <c r="H48" s="1377" t="n">
+      <c r="D48" s="1419" t="n"/>
+      <c r="E48" s="1419" t="n"/>
+      <c r="F48" s="1419" t="n"/>
+      <c r="G48" s="1419" t="n"/>
+      <c r="H48" s="1419" t="n">
         <v>15.1</v>
       </c>
-      <c r="I48" s="1378" t="n"/>
-      <c r="J48" s="1379" t="n"/>
-      <c r="K48" s="1379" t="n"/>
-      <c r="L48" s="1379" t="n"/>
-      <c r="M48" s="1377" t="n">
+      <c r="I48" s="1420" t="n"/>
+      <c r="J48" s="1421" t="n"/>
+      <c r="K48" s="1421" t="n"/>
+      <c r="L48" s="1421" t="n"/>
+      <c r="M48" s="1419" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="1377" t="n">
+      <c r="N48" s="1419" t="n">
         <v>20</v>
       </c>
-      <c r="O48" s="1377" t="n"/>
-      <c r="P48" s="1380" t="n"/>
-      <c r="Q48" s="1377" t="n"/>
-      <c r="R48" s="1377" t="n"/>
-      <c r="S48" s="1377" t="n"/>
+      <c r="O48" s="1419" t="n"/>
+      <c r="P48" s="1422" t="n"/>
+      <c r="Q48" s="1419" t="n"/>
+      <c r="R48" s="1419" t="n"/>
+      <c r="S48" s="1419" t="n"/>
       <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U48" s="1376" t="n"/>
+      <c r="U48" s="1418" t="n"/>
       <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
@@ -7402,51 +7510,51 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1351" t="inlineStr">
+      <c r="A49" s="1393" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B49" s="1352" t="inlineStr">
+      <c r="B49" s="1394" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C49" s="1352" t="inlineStr">
+      <c r="C49" s="1394" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D49" s="1353" t="n"/>
-      <c r="E49" s="1353" t="n">
+      <c r="D49" s="1395" t="n"/>
+      <c r="E49" s="1395" t="n">
         <v>16.8</v>
       </c>
-      <c r="F49" s="1353" t="n">
+      <c r="F49" s="1395" t="n">
         <v>0.2</v>
       </c>
-      <c r="G49" s="1353" t="n">
+      <c r="G49" s="1395" t="n">
         <v>3.3</v>
       </c>
-      <c r="H49" s="1353" t="n"/>
-      <c r="I49" s="1354" t="n">
+      <c r="H49" s="1395" t="n"/>
+      <c r="I49" s="1396" t="n">
         <v>1.7</v>
       </c>
-      <c r="J49" s="1355" t="n"/>
-      <c r="K49" s="1355" t="n"/>
-      <c r="L49" s="1355" t="n"/>
-      <c r="M49" s="1353" t="n"/>
-      <c r="N49" s="1353" t="n"/>
-      <c r="O49" s="1353" t="n">
+      <c r="J49" s="1397" t="n"/>
+      <c r="K49" s="1397" t="n"/>
+      <c r="L49" s="1397" t="n"/>
+      <c r="M49" s="1395" t="n"/>
+      <c r="N49" s="1395" t="n"/>
+      <c r="O49" s="1395" t="n">
         <v>13</v>
       </c>
-      <c r="P49" s="1356" t="n">
+      <c r="P49" s="1398" t="n">
         <v>0.87</v>
       </c>
-      <c r="Q49" s="1353" t="n"/>
-      <c r="R49" s="1353" t="n">
+      <c r="Q49" s="1395" t="n"/>
+      <c r="R49" s="1395" t="n">
         <v>86</v>
       </c>
-      <c r="S49" s="1353" t="n">
+      <c r="S49" s="1395" t="n">
         <v>11.65</v>
       </c>
       <c r="T49" s="624" t="inlineStr">
@@ -7454,7 +7562,7 @@
           <t>Clear now, 88F, 67% RH; sun so far 6.4h of 7h daylight (91%); today high 90F, 0.87in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U49" s="1352" t="inlineStr">
+      <c r="U49" s="1394" t="inlineStr">
         <is>
           <t>2026-07-04_1.jpeg;2026-07-04_2.jpeg;2026-07-04_3.jpeg;2026-07-04_4.jpeg</t>
         </is>
@@ -7466,49 +7574,49 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1357" t="inlineStr">
+      <c r="A50" s="1399" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B50" s="1358" t="inlineStr">
+      <c r="B50" s="1400" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C50" s="1358" t="inlineStr">
+      <c r="C50" s="1400" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D50" s="1359" t="n"/>
-      <c r="E50" s="1359" t="n"/>
-      <c r="F50" s="1359" t="n"/>
-      <c r="G50" s="1359" t="n"/>
-      <c r="H50" s="1359" t="n">
+      <c r="D50" s="1401" t="n"/>
+      <c r="E50" s="1401" t="n"/>
+      <c r="F50" s="1401" t="n"/>
+      <c r="G50" s="1401" t="n"/>
+      <c r="H50" s="1401" t="n">
         <v>14.6</v>
       </c>
-      <c r="I50" s="1360" t="n"/>
-      <c r="J50" s="1361" t="n"/>
-      <c r="K50" s="1361" t="n"/>
-      <c r="L50" s="1361" t="n"/>
-      <c r="M50" s="1359" t="n">
+      <c r="I50" s="1402" t="n"/>
+      <c r="J50" s="1403" t="n"/>
+      <c r="K50" s="1403" t="n"/>
+      <c r="L50" s="1403" t="n"/>
+      <c r="M50" s="1401" t="n">
         <v>0.5</v>
       </c>
-      <c r="N50" s="1359" t="n">
+      <c r="N50" s="1401" t="n">
         <v>20.5</v>
       </c>
-      <c r="O50" s="1359" t="n"/>
-      <c r="P50" s="1362" t="n"/>
-      <c r="Q50" s="1359" t="n"/>
-      <c r="R50" s="1359" t="n"/>
-      <c r="S50" s="1359" t="n"/>
+      <c r="O50" s="1401" t="n"/>
+      <c r="P50" s="1404" t="n"/>
+      <c r="Q50" s="1401" t="n"/>
+      <c r="R50" s="1401" t="n"/>
+      <c r="S50" s="1401" t="n"/>
       <c r="T50" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny day (high 90F, water 86F); storm forecast overnight</t>
         </is>
       </c>
-      <c r="U50" s="1358" t="n"/>
+      <c r="U50" s="1400" t="n"/>
       <c r="V50" s="632" t="inlineStr">
         <is>
           <t>0.5 gal added 7:40 PM. PARTY PRE-LOAD (Sun 7/5 1PM picnic): deliberately HALF the usual dose -- FC already high at 16.8, and John didn't want to overshoot into the high teens for guests. Sized on the retuned model (l24_hot_sunny now 4.0). Model projects ~14.6 next noon, BUT this is a known weather-mismatch case: model keys L24 off today's hot/sunny weather, while the actual loss window is a storm overnight (no UV) + cooler/cloudy Sun morning -&gt; real loss will be LOWER, so FC likely lands ~15-16 at the party (comfortable top-of-band, cushion for bather load, not overboard). =&gt; If tomorrow's noon comes in ABOVE 14.6, that's the weather mismatch, NOT the freshly-retuned constant; don't chase it. Plan: dose back up Sun evening after the crowd's out (expect a bather-load FC drop). Season total 20.5 gal. PHOTOS(4): water clear/healthy blue, bottom fully visible, no cloudiness/algae; yesterday's surface debris now gone (tracks with CC clearing to 0.2); liner step close-up normal speckled blue, no rust/stain progression. Ruler photo documents the ~11.65 cm level.</t>
@@ -7516,58 +7624,110 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1387" t="inlineStr">
+      <c r="A51" s="1405" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B51" s="1388" t="inlineStr">
+      <c r="B51" s="1406" t="inlineStr">
         <is>
           <t>07:45</t>
         </is>
       </c>
-      <c r="C51" s="1388" t="inlineStr">
+      <c r="C51" s="1406" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D51" s="1389" t="n"/>
-      <c r="E51" s="1389" t="n">
+      <c r="D51" s="1407" t="n"/>
+      <c r="E51" s="1407" t="n">
         <v>16</v>
       </c>
-      <c r="F51" s="1389" t="n">
+      <c r="F51" s="1407" t="n">
         <v>0.5</v>
       </c>
-      <c r="G51" s="1389" t="n"/>
-      <c r="H51" s="1389" t="n"/>
-      <c r="I51" s="1390" t="n">
+      <c r="G51" s="1407" t="n"/>
+      <c r="H51" s="1407" t="n"/>
+      <c r="I51" s="1408" t="n">
         <v>1.4</v>
       </c>
-      <c r="J51" s="1391" t="n"/>
-      <c r="K51" s="1391" t="n"/>
-      <c r="L51" s="1391" t="n"/>
-      <c r="M51" s="1389" t="n"/>
-      <c r="N51" s="1389" t="n"/>
-      <c r="O51" s="1389" t="n"/>
-      <c r="P51" s="1392" t="n">
+      <c r="J51" s="1409" t="n"/>
+      <c r="K51" s="1409" t="n"/>
+      <c r="L51" s="1409" t="n"/>
+      <c r="M51" s="1407" t="n"/>
+      <c r="N51" s="1407" t="n"/>
+      <c r="O51" s="1407" t="n"/>
+      <c r="P51" s="1410" t="n">
         <v>0.04</v>
       </c>
-      <c r="Q51" s="1389" t="n"/>
-      <c r="R51" s="1389" t="n">
+      <c r="Q51" s="1407" t="n"/>
+      <c r="R51" s="1407" t="n">
         <v>84</v>
       </c>
-      <c r="S51" s="1389" t="n">
+      <c r="S51" s="1407" t="n">
         <v>13.9</v>
       </c>
-      <c r="T51" s="1199" t="inlineStr">
+      <c r="T51" s="813" t="inlineStr">
         <is>
           <t>Overcast now, 75F, 90% RH; sun so far 0.0h of 3h daylight (0%); today high 75F, 0.04in precip, UV max 6.5</t>
         </is>
       </c>
-      <c r="U51" s="1388" t="n"/>
-      <c r="V51" s="1200" t="inlineStr">
+      <c r="U51" s="1406" t="n"/>
+      <c r="V51" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. Early test (7:45 AM, party day 1PM, John busy) -- off the usual noon cadence, fine. PARTY CALL: FC 16.0 is great; NO morning top-up needed (plan only called for one 'if FC slipped' -- it didn't). Cloudy/cool day (75F, 0 sun) means it'll hold through the party. WEATHER-MISMATCH CONFIRMED (as flagged on last night's dose): 7/4 dose predicted 14.6 for today assuming hot/sunny loss, but today is overcast/cool -&gt; FC ran high at 16.0 (pred error +1.4). This is the weather mismatch, NOT the freshly-retuned l24_hot_sunny=4.0; the constant still gets validated by future clean HOT-day noon readings (mid-week, after Mon rain). fc_loss left blank: off-cadence (~19h not 24h), 0.5gal dose in between, plus rain dilution -&gt; non-comparable. WATER LEVEL 11.65 -&gt; 13.9 (+2.25 cm) from the overnight storm (~0.9in rain, ~445 gal) -- ruler tracked the storm perfectly. CC ticked 0.2 -&gt; 0.5 (rain-driven organic/N load washed in by the storm; still a trace, high FC clears it -- not a party concern). Water temp 86 -&gt; 84 (cool front). NOTE: the BIG rain is still Mon 7/6 (~5.7in) -&gt; watch for overflow then, possible backwash-down after (bonus CYA lowering).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="1417" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B52" s="1418" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C52" s="1418" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="D52" s="1419" t="n"/>
+      <c r="E52" s="1419" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="F52" s="1419" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="G52" s="1419" t="n"/>
+      <c r="H52" s="1419" t="n"/>
+      <c r="I52" s="1420" t="n"/>
+      <c r="J52" s="1421" t="n"/>
+      <c r="K52" s="1421" t="n"/>
+      <c r="L52" s="1421" t="n"/>
+      <c r="M52" s="1419" t="n"/>
+      <c r="N52" s="1419" t="n"/>
+      <c r="O52" s="1419" t="n"/>
+      <c r="P52" s="1422" t="n"/>
+      <c r="Q52" s="1419" t="n"/>
+      <c r="R52" s="1419" t="n"/>
+      <c r="S52" s="1419" t="n"/>
+      <c r="T52" s="827" t="inlineStr">
+        <is>
+          <t>Overcast now, 72F, 76% RH; sun so far 8.4h of 13h daylight (65%); today high 80F, 0.00in precip, UV max 6.0</t>
+        </is>
+      </c>
+      <c r="U52" s="1418" t="inlineStr">
+        <is>
+          <t>2026-07-05_1.jpeg;2026-07-05_2.jpeg</t>
+        </is>
+      </c>
+      <c r="V52" s="828" t="inlineStr">
+        <is>
+          <t>Post-party evening test (2nd test of the day; morning 7:45AM was 16.0). PARTY OUTCOME -- EXCELLENT: FC 16.0(AM) -&gt; 14.8(now), only -1.2 ppm across the whole party (landed right at aim 15); CC 0.5 -&gt; 0.3, i.e. CC DROPPED even after a crowd -- the high FC oxidized bather-load chloramines faster than they formed. The pre-load-modestly strategy worked perfectly (didn't overshoot, didn't crash). PHOTOS(2): wide shot shows crystal-clear water, bottom fully visible, no cloudiness/debris/algae -- pool sailed through. Evening dose recommended 0.5 gal, sized on TOMORROW's rainy forecast (the real loss window: wet/overcast 7/6, ~0.9in rain, low UV) rather than today's sun -&gt; projects ~15.1 at Mon noon. (Day actually cleared to 8.4 sun hrs vs the overcast 7:45AM read.) fc_loss/pred_error blank: off-cadence 2nd test; the 7/4 dose's prediction was already scored against this morning's reading. No water level/temp reported this eve -- ruler photo taken (2026-07-05_2) but no number given; will log if John reads it off.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log 2026-07-05 evening water level 13.6 cm; add evening ruler photo; fix photo attribution
Evening level 13.6 (down from the morning's post-storm 13.9 -- daytime
evaporation + party splashout, no daytime rain). Moved the morning ruler
photo to the morning row and put the evening wide+ruler shots on the
evening row for honest per-reading attribution.
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1429">
+  <cellXfs count="1465">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -4706,6 +4706,114 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -5252,35 +5360,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1393" t="inlineStr">
+      <c r="A3" s="1429" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1394" t="n"/>
-      <c r="C3" s="1394" t="inlineStr">
+      <c r="B3" s="1430" t="n"/>
+      <c r="C3" s="1430" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1395" t="n"/>
-      <c r="E3" s="1395" t="n"/>
-      <c r="F3" s="1395" t="n"/>
-      <c r="G3" s="1395" t="n"/>
-      <c r="H3" s="1395" t="n"/>
-      <c r="I3" s="1396" t="n"/>
-      <c r="J3" s="1397" t="n"/>
-      <c r="K3" s="1397" t="n"/>
-      <c r="L3" s="1397" t="n"/>
-      <c r="M3" s="1395" t="n"/>
-      <c r="N3" s="1395" t="n"/>
-      <c r="O3" s="1395" t="n"/>
-      <c r="P3" s="1398" t="n"/>
-      <c r="Q3" s="1395" t="n"/>
-      <c r="R3" s="1395" t="n"/>
-      <c r="S3" s="1395" t="n"/>
+      <c r="D3" s="1431" t="n"/>
+      <c r="E3" s="1431" t="n"/>
+      <c r="F3" s="1431" t="n"/>
+      <c r="G3" s="1431" t="n"/>
+      <c r="H3" s="1431" t="n"/>
+      <c r="I3" s="1432" t="n"/>
+      <c r="J3" s="1433" t="n"/>
+      <c r="K3" s="1433" t="n"/>
+      <c r="L3" s="1433" t="n"/>
+      <c r="M3" s="1431" t="n"/>
+      <c r="N3" s="1431" t="n"/>
+      <c r="O3" s="1431" t="n"/>
+      <c r="P3" s="1434" t="n"/>
+      <c r="Q3" s="1431" t="n"/>
+      <c r="R3" s="1431" t="n"/>
+      <c r="S3" s="1431" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1394" t="n"/>
+      <c r="U3" s="1430" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -5288,43 +5396,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1399" t="inlineStr">
+      <c r="A4" s="1435" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1400" t="inlineStr">
+      <c r="B4" s="1436" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1400" t="inlineStr">
+      <c r="C4" s="1436" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1401" t="n"/>
-      <c r="E4" s="1401" t="n"/>
-      <c r="F4" s="1401" t="n"/>
-      <c r="G4" s="1401" t="n"/>
-      <c r="H4" s="1401" t="n"/>
-      <c r="I4" s="1402" t="n"/>
-      <c r="J4" s="1403" t="n"/>
-      <c r="K4" s="1403" t="n"/>
-      <c r="L4" s="1403" t="n"/>
-      <c r="M4" s="1401" t="n">
+      <c r="D4" s="1437" t="n"/>
+      <c r="E4" s="1437" t="n"/>
+      <c r="F4" s="1437" t="n"/>
+      <c r="G4" s="1437" t="n"/>
+      <c r="H4" s="1437" t="n"/>
+      <c r="I4" s="1438" t="n"/>
+      <c r="J4" s="1439" t="n"/>
+      <c r="K4" s="1439" t="n"/>
+      <c r="L4" s="1439" t="n"/>
+      <c r="M4" s="1437" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1401" t="n">
+      <c r="N4" s="1437" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1401" t="n"/>
-      <c r="P4" s="1404" t="n"/>
-      <c r="Q4" s="1401" t="n"/>
-      <c r="R4" s="1401" t="n"/>
-      <c r="S4" s="1401" t="n"/>
+      <c r="O4" s="1437" t="n"/>
+      <c r="P4" s="1440" t="n"/>
+      <c r="Q4" s="1437" t="n"/>
+      <c r="R4" s="1437" t="n"/>
+      <c r="S4" s="1437" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1400" t="n"/>
+      <c r="U4" s="1436" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -5332,57 +5440,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1405" t="inlineStr">
+      <c r="A5" s="1441" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1406" t="inlineStr">
+      <c r="B5" s="1442" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1406" t="inlineStr">
+      <c r="C5" s="1442" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1407" t="n">
+      <c r="D5" s="1443" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1407" t="n">
+      <c r="E5" s="1443" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1407" t="n">
+      <c r="F5" s="1443" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1407" t="n"/>
-      <c r="H5" s="1407" t="n"/>
-      <c r="I5" s="1408" t="n"/>
-      <c r="J5" s="1409" t="n">
+      <c r="G5" s="1443" t="n"/>
+      <c r="H5" s="1443" t="n"/>
+      <c r="I5" s="1444" t="n"/>
+      <c r="J5" s="1445" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1409" t="n">
+      <c r="K5" s="1445" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1409" t="inlineStr">
+      <c r="L5" s="1445" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1407" t="n"/>
-      <c r="N5" s="1407" t="n"/>
-      <c r="O5" s="1407" t="n">
+      <c r="M5" s="1443" t="n"/>
+      <c r="N5" s="1443" t="n"/>
+      <c r="O5" s="1443" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1410" t="n">
+      <c r="P5" s="1446" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1407" t="n"/>
-      <c r="R5" s="1407" t="n"/>
-      <c r="S5" s="1407" t="n"/>
+      <c r="Q5" s="1443" t="n"/>
+      <c r="R5" s="1443" t="n"/>
+      <c r="S5" s="1443" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1406" t="n"/>
+      <c r="U5" s="1442" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -5390,43 +5498,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1411" t="inlineStr">
+      <c r="A6" s="1447" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1412" t="inlineStr">
+      <c r="B6" s="1448" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1412" t="inlineStr">
+      <c r="C6" s="1448" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1413" t="n"/>
-      <c r="E6" s="1413" t="n"/>
-      <c r="F6" s="1413" t="n"/>
-      <c r="G6" s="1413" t="n"/>
-      <c r="H6" s="1413" t="n"/>
-      <c r="I6" s="1414" t="n"/>
-      <c r="J6" s="1415" t="n"/>
-      <c r="K6" s="1415" t="n"/>
-      <c r="L6" s="1415" t="n"/>
-      <c r="M6" s="1413" t="n">
+      <c r="D6" s="1449" t="n"/>
+      <c r="E6" s="1449" t="n"/>
+      <c r="F6" s="1449" t="n"/>
+      <c r="G6" s="1449" t="n"/>
+      <c r="H6" s="1449" t="n"/>
+      <c r="I6" s="1450" t="n"/>
+      <c r="J6" s="1451" t="n"/>
+      <c r="K6" s="1451" t="n"/>
+      <c r="L6" s="1451" t="n"/>
+      <c r="M6" s="1449" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1413" t="n">
+      <c r="N6" s="1449" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1413" t="n"/>
-      <c r="P6" s="1416" t="n"/>
-      <c r="Q6" s="1413" t="n"/>
-      <c r="R6" s="1413" t="n"/>
-      <c r="S6" s="1413" t="n"/>
+      <c r="O6" s="1449" t="n"/>
+      <c r="P6" s="1452" t="n"/>
+      <c r="Q6" s="1449" t="n"/>
+      <c r="R6" s="1449" t="n"/>
+      <c r="S6" s="1449" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1412" t="n"/>
+      <c r="U6" s="1448" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -5434,39 +5542,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1417" t="inlineStr">
+      <c r="A7" s="1453" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1418" t="inlineStr">
+      <c r="B7" s="1454" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1418" t="inlineStr">
+      <c r="C7" s="1454" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1419" t="n"/>
-      <c r="E7" s="1419" t="n"/>
-      <c r="F7" s="1419" t="n"/>
-      <c r="G7" s="1419" t="n"/>
-      <c r="H7" s="1419" t="n"/>
-      <c r="I7" s="1420" t="n"/>
-      <c r="J7" s="1421" t="n"/>
-      <c r="K7" s="1421" t="n"/>
-      <c r="L7" s="1421" t="n"/>
-      <c r="M7" s="1419" t="n"/>
-      <c r="N7" s="1419" t="n"/>
-      <c r="O7" s="1419" t="n"/>
-      <c r="P7" s="1422" t="n"/>
-      <c r="Q7" s="1419" t="n"/>
-      <c r="R7" s="1419" t="n"/>
-      <c r="S7" s="1419" t="n"/>
+      <c r="D7" s="1455" t="n"/>
+      <c r="E7" s="1455" t="n"/>
+      <c r="F7" s="1455" t="n"/>
+      <c r="G7" s="1455" t="n"/>
+      <c r="H7" s="1455" t="n"/>
+      <c r="I7" s="1456" t="n"/>
+      <c r="J7" s="1457" t="n"/>
+      <c r="K7" s="1457" t="n"/>
+      <c r="L7" s="1457" t="n"/>
+      <c r="M7" s="1455" t="n"/>
+      <c r="N7" s="1455" t="n"/>
+      <c r="O7" s="1455" t="n"/>
+      <c r="P7" s="1458" t="n"/>
+      <c r="Q7" s="1455" t="n"/>
+      <c r="R7" s="1455" t="n"/>
+      <c r="S7" s="1455" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1418" t="n"/>
+      <c r="U7" s="1454" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5474,39 +5582,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1393" t="inlineStr">
+      <c r="A8" s="1429" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1394" t="inlineStr">
+      <c r="B8" s="1430" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1394" t="inlineStr">
+      <c r="C8" s="1430" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1395" t="n"/>
-      <c r="E8" s="1395" t="n"/>
-      <c r="F8" s="1395" t="n"/>
-      <c r="G8" s="1395" t="n"/>
-      <c r="H8" s="1395" t="n"/>
-      <c r="I8" s="1396" t="n"/>
-      <c r="J8" s="1397" t="n"/>
-      <c r="K8" s="1397" t="n"/>
-      <c r="L8" s="1397" t="n"/>
-      <c r="M8" s="1395" t="n"/>
-      <c r="N8" s="1395" t="n"/>
-      <c r="O8" s="1395" t="n"/>
-      <c r="P8" s="1398" t="n"/>
-      <c r="Q8" s="1395" t="n"/>
-      <c r="R8" s="1395" t="n"/>
-      <c r="S8" s="1395" t="n"/>
+      <c r="D8" s="1431" t="n"/>
+      <c r="E8" s="1431" t="n"/>
+      <c r="F8" s="1431" t="n"/>
+      <c r="G8" s="1431" t="n"/>
+      <c r="H8" s="1431" t="n"/>
+      <c r="I8" s="1432" t="n"/>
+      <c r="J8" s="1433" t="n"/>
+      <c r="K8" s="1433" t="n"/>
+      <c r="L8" s="1433" t="n"/>
+      <c r="M8" s="1431" t="n"/>
+      <c r="N8" s="1431" t="n"/>
+      <c r="O8" s="1431" t="n"/>
+      <c r="P8" s="1434" t="n"/>
+      <c r="Q8" s="1431" t="n"/>
+      <c r="R8" s="1431" t="n"/>
+      <c r="S8" s="1431" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1394" t="n"/>
+      <c r="U8" s="1430" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -5514,63 +5622,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1423" t="inlineStr">
+      <c r="A9" s="1459" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1424" t="inlineStr">
+      <c r="B9" s="1460" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1424" t="inlineStr">
+      <c r="C9" s="1460" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1425" t="n">
+      <c r="D9" s="1461" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1425" t="n">
+      <c r="E9" s="1461" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1425" t="n">
+      <c r="F9" s="1461" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1425" t="n">
+      <c r="G9" s="1461" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1425" t="n"/>
-      <c r="I9" s="1426" t="n"/>
-      <c r="J9" s="1427" t="n">
+      <c r="H9" s="1461" t="n"/>
+      <c r="I9" s="1462" t="n"/>
+      <c r="J9" s="1463" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1427" t="n">
+      <c r="K9" s="1463" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1427" t="inlineStr">
+      <c r="L9" s="1463" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1425" t="n"/>
-      <c r="N9" s="1425" t="n"/>
-      <c r="O9" s="1425" t="n">
+      <c r="M9" s="1461" t="n"/>
+      <c r="N9" s="1461" t="n"/>
+      <c r="O9" s="1461" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1428" t="n">
+      <c r="P9" s="1464" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1425" t="n"/>
-      <c r="R9" s="1425" t="n"/>
-      <c r="S9" s="1425" t="n"/>
+      <c r="Q9" s="1461" t="n"/>
+      <c r="R9" s="1461" t="n"/>
+      <c r="S9" s="1461" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1424" t="n"/>
+      <c r="U9" s="1460" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -5578,43 +5686,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1423" t="inlineStr">
+      <c r="A10" s="1459" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1424" t="inlineStr">
+      <c r="B10" s="1460" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1424" t="inlineStr">
+      <c r="C10" s="1460" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1425" t="n"/>
-      <c r="E10" s="1425" t="n"/>
-      <c r="F10" s="1425" t="n"/>
-      <c r="G10" s="1425" t="n"/>
-      <c r="H10" s="1425" t="n"/>
-      <c r="I10" s="1426" t="n"/>
-      <c r="J10" s="1427" t="n"/>
-      <c r="K10" s="1427" t="n"/>
-      <c r="L10" s="1427" t="inlineStr">
+      <c r="D10" s="1461" t="n"/>
+      <c r="E10" s="1461" t="n"/>
+      <c r="F10" s="1461" t="n"/>
+      <c r="G10" s="1461" t="n"/>
+      <c r="H10" s="1461" t="n"/>
+      <c r="I10" s="1462" t="n"/>
+      <c r="J10" s="1463" t="n"/>
+      <c r="K10" s="1463" t="n"/>
+      <c r="L10" s="1463" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1425" t="n"/>
-      <c r="N10" s="1425" t="n"/>
-      <c r="O10" s="1425" t="n"/>
-      <c r="P10" s="1428" t="n"/>
-      <c r="Q10" s="1425" t="n"/>
-      <c r="R10" s="1425" t="n"/>
-      <c r="S10" s="1425" t="n"/>
+      <c r="M10" s="1461" t="n"/>
+      <c r="N10" s="1461" t="n"/>
+      <c r="O10" s="1461" t="n"/>
+      <c r="P10" s="1464" t="n"/>
+      <c r="Q10" s="1461" t="n"/>
+      <c r="R10" s="1461" t="n"/>
+      <c r="S10" s="1461" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1424" t="n"/>
+      <c r="U10" s="1460" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -5622,43 +5730,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1423" t="inlineStr">
+      <c r="A11" s="1459" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1424" t="inlineStr">
+      <c r="B11" s="1460" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1424" t="inlineStr">
+      <c r="C11" s="1460" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1425" t="n"/>
-      <c r="E11" s="1425" t="n"/>
-      <c r="F11" s="1425" t="n"/>
-      <c r="G11" s="1425" t="n"/>
-      <c r="H11" s="1425" t="n"/>
-      <c r="I11" s="1426" t="n"/>
-      <c r="J11" s="1427" t="n"/>
-      <c r="K11" s="1427" t="n"/>
-      <c r="L11" s="1427" t="n"/>
-      <c r="M11" s="1425" t="n">
+      <c r="D11" s="1461" t="n"/>
+      <c r="E11" s="1461" t="n"/>
+      <c r="F11" s="1461" t="n"/>
+      <c r="G11" s="1461" t="n"/>
+      <c r="H11" s="1461" t="n"/>
+      <c r="I11" s="1462" t="n"/>
+      <c r="J11" s="1463" t="n"/>
+      <c r="K11" s="1463" t="n"/>
+      <c r="L11" s="1463" t="n"/>
+      <c r="M11" s="1461" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1425" t="n">
+      <c r="N11" s="1461" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1425" t="n"/>
-      <c r="P11" s="1428" t="n"/>
-      <c r="Q11" s="1425" t="n"/>
-      <c r="R11" s="1425" t="n"/>
-      <c r="S11" s="1425" t="n"/>
+      <c r="O11" s="1461" t="n"/>
+      <c r="P11" s="1464" t="n"/>
+      <c r="Q11" s="1461" t="n"/>
+      <c r="R11" s="1461" t="n"/>
+      <c r="S11" s="1461" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1424" t="n"/>
+      <c r="U11" s="1460" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -5666,39 +5774,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1399" t="inlineStr">
+      <c r="A12" s="1435" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1400" t="inlineStr">
+      <c r="B12" s="1436" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1400" t="inlineStr">
+      <c r="C12" s="1436" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1401" t="n"/>
-      <c r="E12" s="1401" t="n"/>
-      <c r="F12" s="1401" t="n"/>
-      <c r="G12" s="1401" t="n"/>
-      <c r="H12" s="1401" t="n"/>
-      <c r="I12" s="1402" t="n"/>
-      <c r="J12" s="1403" t="n"/>
-      <c r="K12" s="1403" t="n"/>
-      <c r="L12" s="1403" t="n"/>
-      <c r="M12" s="1401" t="n"/>
-      <c r="N12" s="1401" t="n"/>
-      <c r="O12" s="1401" t="n"/>
-      <c r="P12" s="1404" t="n"/>
-      <c r="Q12" s="1401" t="n"/>
-      <c r="R12" s="1401" t="n"/>
-      <c r="S12" s="1401" t="n"/>
+      <c r="D12" s="1437" t="n"/>
+      <c r="E12" s="1437" t="n"/>
+      <c r="F12" s="1437" t="n"/>
+      <c r="G12" s="1437" t="n"/>
+      <c r="H12" s="1437" t="n"/>
+      <c r="I12" s="1438" t="n"/>
+      <c r="J12" s="1439" t="n"/>
+      <c r="K12" s="1439" t="n"/>
+      <c r="L12" s="1439" t="n"/>
+      <c r="M12" s="1437" t="n"/>
+      <c r="N12" s="1437" t="n"/>
+      <c r="O12" s="1437" t="n"/>
+      <c r="P12" s="1440" t="n"/>
+      <c r="Q12" s="1437" t="n"/>
+      <c r="R12" s="1437" t="n"/>
+      <c r="S12" s="1437" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1400" t="n"/>
+      <c r="U12" s="1436" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5706,35 +5814,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1405" t="inlineStr">
+      <c r="A13" s="1441" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1406" t="n"/>
-      <c r="C13" s="1406" t="inlineStr">
+      <c r="B13" s="1442" t="n"/>
+      <c r="C13" s="1442" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1407" t="n"/>
-      <c r="E13" s="1407" t="n"/>
-      <c r="F13" s="1407" t="n"/>
-      <c r="G13" s="1407" t="n"/>
-      <c r="H13" s="1407" t="n"/>
-      <c r="I13" s="1408" t="n"/>
-      <c r="J13" s="1409" t="n"/>
-      <c r="K13" s="1409" t="n"/>
-      <c r="L13" s="1409" t="n"/>
-      <c r="M13" s="1407" t="n"/>
-      <c r="N13" s="1407" t="n"/>
-      <c r="O13" s="1407" t="n"/>
-      <c r="P13" s="1410" t="n"/>
-      <c r="Q13" s="1407" t="n"/>
-      <c r="R13" s="1407" t="n"/>
-      <c r="S13" s="1407" t="n"/>
+      <c r="D13" s="1443" t="n"/>
+      <c r="E13" s="1443" t="n"/>
+      <c r="F13" s="1443" t="n"/>
+      <c r="G13" s="1443" t="n"/>
+      <c r="H13" s="1443" t="n"/>
+      <c r="I13" s="1444" t="n"/>
+      <c r="J13" s="1445" t="n"/>
+      <c r="K13" s="1445" t="n"/>
+      <c r="L13" s="1445" t="n"/>
+      <c r="M13" s="1443" t="n"/>
+      <c r="N13" s="1443" t="n"/>
+      <c r="O13" s="1443" t="n"/>
+      <c r="P13" s="1446" t="n"/>
+      <c r="Q13" s="1443" t="n"/>
+      <c r="R13" s="1443" t="n"/>
+      <c r="S13" s="1443" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1406" t="n"/>
+      <c r="U13" s="1442" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -5742,53 +5850,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1411" t="inlineStr">
+      <c r="A14" s="1447" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1412" t="inlineStr">
+      <c r="B14" s="1448" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1412" t="inlineStr">
+      <c r="C14" s="1448" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1413" t="n"/>
-      <c r="E14" s="1413" t="n">
+      <c r="D14" s="1449" t="n"/>
+      <c r="E14" s="1449" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1413" t="n">
+      <c r="F14" s="1449" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1413" t="n">
+      <c r="G14" s="1449" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1413" t="n"/>
-      <c r="I14" s="1414" t="n"/>
-      <c r="J14" s="1415" t="n"/>
-      <c r="K14" s="1415" t="n"/>
-      <c r="L14" s="1415" t="n"/>
-      <c r="M14" s="1413" t="n"/>
-      <c r="N14" s="1413" t="n"/>
-      <c r="O14" s="1413" t="n">
+      <c r="H14" s="1449" t="n"/>
+      <c r="I14" s="1450" t="n"/>
+      <c r="J14" s="1451" t="n"/>
+      <c r="K14" s="1451" t="n"/>
+      <c r="L14" s="1451" t="n"/>
+      <c r="M14" s="1449" t="n"/>
+      <c r="N14" s="1449" t="n"/>
+      <c r="O14" s="1449" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1416" t="n">
+      <c r="P14" s="1452" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1413" t="n"/>
-      <c r="R14" s="1413" t="n"/>
-      <c r="S14" s="1413" t="n"/>
+      <c r="Q14" s="1449" t="n"/>
+      <c r="R14" s="1449" t="n"/>
+      <c r="S14" s="1449" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1412" t="n"/>
+      <c r="U14" s="1448" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -5796,43 +5904,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1411" t="inlineStr">
+      <c r="A15" s="1447" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1412" t="inlineStr">
+      <c r="B15" s="1448" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1412" t="inlineStr">
+      <c r="C15" s="1448" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1413" t="n"/>
-      <c r="E15" s="1413" t="n"/>
-      <c r="F15" s="1413" t="n"/>
-      <c r="G15" s="1413" t="n"/>
-      <c r="H15" s="1413" t="n"/>
-      <c r="I15" s="1414" t="n"/>
-      <c r="J15" s="1415" t="n"/>
-      <c r="K15" s="1415" t="n"/>
-      <c r="L15" s="1415" t="n"/>
-      <c r="M15" s="1413" t="n">
+      <c r="D15" s="1449" t="n"/>
+      <c r="E15" s="1449" t="n"/>
+      <c r="F15" s="1449" t="n"/>
+      <c r="G15" s="1449" t="n"/>
+      <c r="H15" s="1449" t="n"/>
+      <c r="I15" s="1450" t="n"/>
+      <c r="J15" s="1451" t="n"/>
+      <c r="K15" s="1451" t="n"/>
+      <c r="L15" s="1451" t="n"/>
+      <c r="M15" s="1449" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1413" t="n">
+      <c r="N15" s="1449" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1413" t="n"/>
-      <c r="P15" s="1416" t="n"/>
-      <c r="Q15" s="1413" t="n"/>
-      <c r="R15" s="1413" t="n"/>
-      <c r="S15" s="1413" t="n"/>
+      <c r="O15" s="1449" t="n"/>
+      <c r="P15" s="1452" t="n"/>
+      <c r="Q15" s="1449" t="n"/>
+      <c r="R15" s="1449" t="n"/>
+      <c r="S15" s="1449" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1412" t="n"/>
+      <c r="U15" s="1448" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -5840,39 +5948,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1417" t="inlineStr">
+      <c r="A16" s="1453" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1418" t="inlineStr">
+      <c r="B16" s="1454" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1418" t="inlineStr">
+      <c r="C16" s="1454" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1419" t="n"/>
-      <c r="E16" s="1419" t="n"/>
-      <c r="F16" s="1419" t="n"/>
-      <c r="G16" s="1419" t="n"/>
-      <c r="H16" s="1419" t="n"/>
-      <c r="I16" s="1420" t="n"/>
-      <c r="J16" s="1421" t="n"/>
-      <c r="K16" s="1421" t="n"/>
-      <c r="L16" s="1421" t="n"/>
-      <c r="M16" s="1419" t="n"/>
-      <c r="N16" s="1419" t="n"/>
-      <c r="O16" s="1419" t="n"/>
-      <c r="P16" s="1422" t="n"/>
-      <c r="Q16" s="1419" t="n"/>
-      <c r="R16" s="1419" t="n"/>
-      <c r="S16" s="1419" t="n"/>
+      <c r="D16" s="1455" t="n"/>
+      <c r="E16" s="1455" t="n"/>
+      <c r="F16" s="1455" t="n"/>
+      <c r="G16" s="1455" t="n"/>
+      <c r="H16" s="1455" t="n"/>
+      <c r="I16" s="1456" t="n"/>
+      <c r="J16" s="1457" t="n"/>
+      <c r="K16" s="1457" t="n"/>
+      <c r="L16" s="1457" t="n"/>
+      <c r="M16" s="1455" t="n"/>
+      <c r="N16" s="1455" t="n"/>
+      <c r="O16" s="1455" t="n"/>
+      <c r="P16" s="1458" t="n"/>
+      <c r="Q16" s="1455" t="n"/>
+      <c r="R16" s="1455" t="n"/>
+      <c r="S16" s="1455" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1418" t="n"/>
+      <c r="U16" s="1454" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -5880,39 +5988,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1393" t="inlineStr">
+      <c r="A17" s="1429" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1394" t="inlineStr">
+      <c r="B17" s="1430" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1394" t="inlineStr">
+      <c r="C17" s="1430" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1395" t="n"/>
-      <c r="E17" s="1395" t="n"/>
-      <c r="F17" s="1395" t="n"/>
-      <c r="G17" s="1395" t="n"/>
-      <c r="H17" s="1395" t="n"/>
-      <c r="I17" s="1396" t="n"/>
-      <c r="J17" s="1397" t="n"/>
-      <c r="K17" s="1397" t="n"/>
-      <c r="L17" s="1397" t="n"/>
-      <c r="M17" s="1395" t="n"/>
-      <c r="N17" s="1395" t="n"/>
-      <c r="O17" s="1395" t="n"/>
-      <c r="P17" s="1398" t="n"/>
-      <c r="Q17" s="1395" t="n"/>
-      <c r="R17" s="1395" t="n"/>
-      <c r="S17" s="1395" t="n"/>
+      <c r="D17" s="1431" t="n"/>
+      <c r="E17" s="1431" t="n"/>
+      <c r="F17" s="1431" t="n"/>
+      <c r="G17" s="1431" t="n"/>
+      <c r="H17" s="1431" t="n"/>
+      <c r="I17" s="1432" t="n"/>
+      <c r="J17" s="1433" t="n"/>
+      <c r="K17" s="1433" t="n"/>
+      <c r="L17" s="1433" t="n"/>
+      <c r="M17" s="1431" t="n"/>
+      <c r="N17" s="1431" t="n"/>
+      <c r="O17" s="1431" t="n"/>
+      <c r="P17" s="1434" t="n"/>
+      <c r="Q17" s="1431" t="n"/>
+      <c r="R17" s="1431" t="n"/>
+      <c r="S17" s="1431" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1394" t="n"/>
+      <c r="U17" s="1430" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -5920,53 +6028,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1423" t="inlineStr">
+      <c r="A18" s="1459" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1424" t="inlineStr">
+      <c r="B18" s="1460" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1424" t="inlineStr">
+      <c r="C18" s="1460" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1425" t="n"/>
-      <c r="E18" s="1425" t="n">
+      <c r="D18" s="1461" t="n"/>
+      <c r="E18" s="1461" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1425" t="n">
+      <c r="F18" s="1461" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1425" t="n">
+      <c r="G18" s="1461" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1425" t="n"/>
-      <c r="I18" s="1426" t="n"/>
-      <c r="J18" s="1427" t="n"/>
-      <c r="K18" s="1427" t="n"/>
-      <c r="L18" s="1427" t="n"/>
-      <c r="M18" s="1425" t="n"/>
-      <c r="N18" s="1425" t="n"/>
-      <c r="O18" s="1425" t="n">
+      <c r="H18" s="1461" t="n"/>
+      <c r="I18" s="1462" t="n"/>
+      <c r="J18" s="1463" t="n"/>
+      <c r="K18" s="1463" t="n"/>
+      <c r="L18" s="1463" t="n"/>
+      <c r="M18" s="1461" t="n"/>
+      <c r="N18" s="1461" t="n"/>
+      <c r="O18" s="1461" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1428" t="n">
+      <c r="P18" s="1464" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1425" t="n"/>
-      <c r="R18" s="1425" t="n"/>
-      <c r="S18" s="1425" t="n"/>
+      <c r="Q18" s="1461" t="n"/>
+      <c r="R18" s="1461" t="n"/>
+      <c r="S18" s="1461" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1424" t="n"/>
+      <c r="U18" s="1460" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -5974,47 +6082,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1423" t="inlineStr">
+      <c r="A19" s="1459" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1424" t="inlineStr">
+      <c r="B19" s="1460" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1424" t="inlineStr">
+      <c r="C19" s="1460" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1425" t="n"/>
-      <c r="E19" s="1425" t="n"/>
-      <c r="F19" s="1425" t="n"/>
-      <c r="G19" s="1425" t="n"/>
-      <c r="H19" s="1425" t="n"/>
-      <c r="I19" s="1426" t="n"/>
-      <c r="J19" s="1427" t="n"/>
-      <c r="K19" s="1427" t="n"/>
-      <c r="L19" s="1427" t="n"/>
-      <c r="M19" s="1425" t="n">
+      <c r="D19" s="1461" t="n"/>
+      <c r="E19" s="1461" t="n"/>
+      <c r="F19" s="1461" t="n"/>
+      <c r="G19" s="1461" t="n"/>
+      <c r="H19" s="1461" t="n"/>
+      <c r="I19" s="1462" t="n"/>
+      <c r="J19" s="1463" t="n"/>
+      <c r="K19" s="1463" t="n"/>
+      <c r="L19" s="1463" t="n"/>
+      <c r="M19" s="1461" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1425" t="n">
+      <c r="N19" s="1461" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1425" t="n"/>
-      <c r="P19" s="1428" t="n"/>
-      <c r="Q19" s="1425" t="n"/>
-      <c r="R19" s="1425" t="n"/>
-      <c r="S19" s="1425" t="n"/>
+      <c r="O19" s="1461" t="n"/>
+      <c r="P19" s="1464" t="n"/>
+      <c r="Q19" s="1461" t="n"/>
+      <c r="R19" s="1461" t="n"/>
+      <c r="S19" s="1461" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1424" t="n"/>
+      <c r="U19" s="1460" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -6022,43 +6130,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1423" t="inlineStr">
+      <c r="A20" s="1459" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1424" t="inlineStr">
+      <c r="B20" s="1460" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1424" t="inlineStr">
+      <c r="C20" s="1460" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1425" t="n"/>
-      <c r="E20" s="1425" t="n"/>
-      <c r="F20" s="1425" t="n"/>
-      <c r="G20" s="1425" t="n"/>
-      <c r="H20" s="1425" t="n"/>
-      <c r="I20" s="1426" t="n"/>
-      <c r="J20" s="1427" t="n"/>
-      <c r="K20" s="1427" t="n"/>
-      <c r="L20" s="1427" t="n"/>
-      <c r="M20" s="1425" t="n"/>
-      <c r="N20" s="1425" t="n"/>
-      <c r="O20" s="1425" t="n"/>
-      <c r="P20" s="1428" t="n"/>
-      <c r="Q20" s="1425" t="n"/>
-      <c r="R20" s="1425" t="n"/>
-      <c r="S20" s="1425" t="n"/>
+      <c r="D20" s="1461" t="n"/>
+      <c r="E20" s="1461" t="n"/>
+      <c r="F20" s="1461" t="n"/>
+      <c r="G20" s="1461" t="n"/>
+      <c r="H20" s="1461" t="n"/>
+      <c r="I20" s="1462" t="n"/>
+      <c r="J20" s="1463" t="n"/>
+      <c r="K20" s="1463" t="n"/>
+      <c r="L20" s="1463" t="n"/>
+      <c r="M20" s="1461" t="n"/>
+      <c r="N20" s="1461" t="n"/>
+      <c r="O20" s="1461" t="n"/>
+      <c r="P20" s="1464" t="n"/>
+      <c r="Q20" s="1461" t="n"/>
+      <c r="R20" s="1461" t="n"/>
+      <c r="S20" s="1461" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1424" t="n"/>
+      <c r="U20" s="1460" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -6066,39 +6174,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1399" t="inlineStr">
+      <c r="A21" s="1435" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1400" t="inlineStr">
+      <c r="B21" s="1436" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1400" t="inlineStr">
+      <c r="C21" s="1436" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1401" t="n"/>
-      <c r="E21" s="1401" t="n"/>
-      <c r="F21" s="1401" t="n"/>
-      <c r="G21" s="1401" t="n"/>
-      <c r="H21" s="1401" t="n"/>
-      <c r="I21" s="1402" t="n"/>
-      <c r="J21" s="1403" t="n"/>
-      <c r="K21" s="1403" t="n"/>
-      <c r="L21" s="1403" t="n"/>
-      <c r="M21" s="1401" t="n"/>
-      <c r="N21" s="1401" t="n"/>
-      <c r="O21" s="1401" t="n"/>
-      <c r="P21" s="1404" t="n"/>
-      <c r="Q21" s="1401" t="n"/>
-      <c r="R21" s="1401" t="n"/>
-      <c r="S21" s="1401" t="n"/>
+      <c r="D21" s="1437" t="n"/>
+      <c r="E21" s="1437" t="n"/>
+      <c r="F21" s="1437" t="n"/>
+      <c r="G21" s="1437" t="n"/>
+      <c r="H21" s="1437" t="n"/>
+      <c r="I21" s="1438" t="n"/>
+      <c r="J21" s="1439" t="n"/>
+      <c r="K21" s="1439" t="n"/>
+      <c r="L21" s="1439" t="n"/>
+      <c r="M21" s="1437" t="n"/>
+      <c r="N21" s="1437" t="n"/>
+      <c r="O21" s="1437" t="n"/>
+      <c r="P21" s="1440" t="n"/>
+      <c r="Q21" s="1437" t="n"/>
+      <c r="R21" s="1437" t="n"/>
+      <c r="S21" s="1437" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1400" t="n"/>
+      <c r="U21" s="1436" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -6106,39 +6214,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1405" t="inlineStr">
+      <c r="A22" s="1441" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1406" t="inlineStr">
+      <c r="B22" s="1442" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1406" t="inlineStr">
+      <c r="C22" s="1442" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1407" t="n"/>
-      <c r="E22" s="1407" t="n"/>
-      <c r="F22" s="1407" t="n"/>
-      <c r="G22" s="1407" t="n"/>
-      <c r="H22" s="1407" t="n"/>
-      <c r="I22" s="1408" t="n"/>
-      <c r="J22" s="1409" t="n"/>
-      <c r="K22" s="1409" t="n"/>
-      <c r="L22" s="1409" t="n"/>
-      <c r="M22" s="1407" t="n"/>
-      <c r="N22" s="1407" t="n"/>
-      <c r="O22" s="1407" t="n"/>
-      <c r="P22" s="1410" t="n"/>
-      <c r="Q22" s="1407" t="n"/>
-      <c r="R22" s="1407" t="n"/>
-      <c r="S22" s="1407" t="n"/>
+      <c r="D22" s="1443" t="n"/>
+      <c r="E22" s="1443" t="n"/>
+      <c r="F22" s="1443" t="n"/>
+      <c r="G22" s="1443" t="n"/>
+      <c r="H22" s="1443" t="n"/>
+      <c r="I22" s="1444" t="n"/>
+      <c r="J22" s="1445" t="n"/>
+      <c r="K22" s="1445" t="n"/>
+      <c r="L22" s="1445" t="n"/>
+      <c r="M22" s="1443" t="n"/>
+      <c r="N22" s="1443" t="n"/>
+      <c r="O22" s="1443" t="n"/>
+      <c r="P22" s="1446" t="n"/>
+      <c r="Q22" s="1443" t="n"/>
+      <c r="R22" s="1443" t="n"/>
+      <c r="S22" s="1443" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1406" t="n"/>
+      <c r="U22" s="1442" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -6146,53 +6254,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1411" t="inlineStr">
+      <c r="A23" s="1447" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1412" t="inlineStr">
+      <c r="B23" s="1448" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1412" t="inlineStr">
+      <c r="C23" s="1448" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1413" t="n"/>
-      <c r="E23" s="1413" t="n">
+      <c r="D23" s="1449" t="n"/>
+      <c r="E23" s="1449" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1413" t="n">
+      <c r="F23" s="1449" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1413" t="n">
+      <c r="G23" s="1449" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1413" t="n"/>
-      <c r="I23" s="1414" t="n"/>
-      <c r="J23" s="1415" t="n"/>
-      <c r="K23" s="1415" t="n"/>
-      <c r="L23" s="1415" t="n"/>
-      <c r="M23" s="1413" t="n"/>
-      <c r="N23" s="1413" t="n"/>
-      <c r="O23" s="1413" t="n">
+      <c r="H23" s="1449" t="n"/>
+      <c r="I23" s="1450" t="n"/>
+      <c r="J23" s="1451" t="n"/>
+      <c r="K23" s="1451" t="n"/>
+      <c r="L23" s="1451" t="n"/>
+      <c r="M23" s="1449" t="n"/>
+      <c r="N23" s="1449" t="n"/>
+      <c r="O23" s="1449" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1416" t="n">
+      <c r="P23" s="1452" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1413" t="n"/>
-      <c r="R23" s="1413" t="n"/>
-      <c r="S23" s="1413" t="n"/>
+      <c r="Q23" s="1449" t="n"/>
+      <c r="R23" s="1449" t="n"/>
+      <c r="S23" s="1449" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1412" t="n"/>
+      <c r="U23" s="1448" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -6200,47 +6308,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1417" t="inlineStr">
+      <c r="A24" s="1453" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1418" t="inlineStr">
+      <c r="B24" s="1454" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1418" t="inlineStr">
+      <c r="C24" s="1454" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1419" t="n"/>
-      <c r="E24" s="1419" t="n"/>
-      <c r="F24" s="1419" t="n"/>
-      <c r="G24" s="1419" t="n"/>
-      <c r="H24" s="1419" t="n"/>
-      <c r="I24" s="1420" t="n"/>
-      <c r="J24" s="1421" t="n"/>
-      <c r="K24" s="1421" t="n"/>
-      <c r="L24" s="1421" t="n"/>
-      <c r="M24" s="1419" t="n">
+      <c r="D24" s="1455" t="n"/>
+      <c r="E24" s="1455" t="n"/>
+      <c r="F24" s="1455" t="n"/>
+      <c r="G24" s="1455" t="n"/>
+      <c r="H24" s="1455" t="n"/>
+      <c r="I24" s="1456" t="n"/>
+      <c r="J24" s="1457" t="n"/>
+      <c r="K24" s="1457" t="n"/>
+      <c r="L24" s="1457" t="n"/>
+      <c r="M24" s="1455" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1419" t="n">
+      <c r="N24" s="1455" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1419" t="n"/>
-      <c r="P24" s="1422" t="n"/>
-      <c r="Q24" s="1419" t="n"/>
-      <c r="R24" s="1419" t="n"/>
-      <c r="S24" s="1419" t="n"/>
+      <c r="O24" s="1455" t="n"/>
+      <c r="P24" s="1458" t="n"/>
+      <c r="Q24" s="1455" t="n"/>
+      <c r="R24" s="1455" t="n"/>
+      <c r="S24" s="1455" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1418" t="n"/>
+      <c r="U24" s="1454" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -6248,61 +6356,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1393" t="inlineStr">
+      <c r="A25" s="1429" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1394" t="inlineStr">
+      <c r="B25" s="1430" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1394" t="inlineStr">
+      <c r="C25" s="1430" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1395" t="n">
+      <c r="D25" s="1431" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1395" t="n">
+      <c r="E25" s="1431" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1395" t="n">
+      <c r="F25" s="1431" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1395" t="n">
+      <c r="G25" s="1431" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1395" t="n"/>
-      <c r="I25" s="1396" t="n"/>
-      <c r="J25" s="1397" t="n">
+      <c r="H25" s="1431" t="n"/>
+      <c r="I25" s="1432" t="n"/>
+      <c r="J25" s="1433" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1397" t="n">
+      <c r="K25" s="1433" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1397" t="n">
+      <c r="L25" s="1433" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1395" t="n"/>
-      <c r="N25" s="1395" t="n"/>
-      <c r="O25" s="1395" t="n">
+      <c r="M25" s="1431" t="n"/>
+      <c r="N25" s="1431" t="n"/>
+      <c r="O25" s="1431" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1398" t="n">
+      <c r="P25" s="1434" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1395" t="n"/>
-      <c r="R25" s="1395" t="n"/>
-      <c r="S25" s="1395" t="n"/>
+      <c r="Q25" s="1431" t="n"/>
+      <c r="R25" s="1431" t="n"/>
+      <c r="S25" s="1431" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1394" t="n"/>
+      <c r="U25" s="1430" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -6310,47 +6418,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1399" t="inlineStr">
+      <c r="A26" s="1435" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1400" t="inlineStr">
+      <c r="B26" s="1436" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1400" t="inlineStr">
+      <c r="C26" s="1436" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1401" t="n"/>
-      <c r="E26" s="1401" t="n"/>
-      <c r="F26" s="1401" t="n"/>
-      <c r="G26" s="1401" t="n"/>
-      <c r="H26" s="1401" t="n"/>
-      <c r="I26" s="1402" t="n"/>
-      <c r="J26" s="1403" t="n"/>
-      <c r="K26" s="1403" t="n"/>
-      <c r="L26" s="1403" t="n"/>
-      <c r="M26" s="1401" t="n">
+      <c r="D26" s="1437" t="n"/>
+      <c r="E26" s="1437" t="n"/>
+      <c r="F26" s="1437" t="n"/>
+      <c r="G26" s="1437" t="n"/>
+      <c r="H26" s="1437" t="n"/>
+      <c r="I26" s="1438" t="n"/>
+      <c r="J26" s="1439" t="n"/>
+      <c r="K26" s="1439" t="n"/>
+      <c r="L26" s="1439" t="n"/>
+      <c r="M26" s="1437" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1401" t="n">
+      <c r="N26" s="1437" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1401" t="n"/>
-      <c r="P26" s="1404" t="n"/>
-      <c r="Q26" s="1401" t="n"/>
-      <c r="R26" s="1401" t="n"/>
-      <c r="S26" s="1401" t="n"/>
+      <c r="O26" s="1437" t="n"/>
+      <c r="P26" s="1440" t="n"/>
+      <c r="Q26" s="1437" t="n"/>
+      <c r="R26" s="1437" t="n"/>
+      <c r="S26" s="1437" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1400" t="n"/>
+      <c r="U26" s="1436" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -6358,53 +6466,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1405" t="inlineStr">
+      <c r="A27" s="1441" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1406" t="inlineStr">
+      <c r="B27" s="1442" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1406" t="inlineStr">
+      <c r="C27" s="1442" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1407" t="n"/>
-      <c r="E27" s="1407" t="n">
+      <c r="D27" s="1443" t="n"/>
+      <c r="E27" s="1443" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1407" t="n">
+      <c r="F27" s="1443" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1407" t="n">
+      <c r="G27" s="1443" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1407" t="n"/>
-      <c r="I27" s="1408" t="n"/>
-      <c r="J27" s="1409" t="n"/>
-      <c r="K27" s="1409" t="n"/>
-      <c r="L27" s="1409" t="n"/>
-      <c r="M27" s="1407" t="n"/>
-      <c r="N27" s="1407" t="n"/>
-      <c r="O27" s="1407" t="n">
+      <c r="H27" s="1443" t="n"/>
+      <c r="I27" s="1444" t="n"/>
+      <c r="J27" s="1445" t="n"/>
+      <c r="K27" s="1445" t="n"/>
+      <c r="L27" s="1445" t="n"/>
+      <c r="M27" s="1443" t="n"/>
+      <c r="N27" s="1443" t="n"/>
+      <c r="O27" s="1443" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1410" t="n">
+      <c r="P27" s="1446" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1407" t="n"/>
-      <c r="R27" s="1407" t="n"/>
-      <c r="S27" s="1407" t="n"/>
+      <c r="Q27" s="1443" t="n"/>
+      <c r="R27" s="1443" t="n"/>
+      <c r="S27" s="1443" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1406" t="n"/>
+      <c r="U27" s="1442" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -6412,47 +6520,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1417" t="inlineStr">
+      <c r="A28" s="1453" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1418" t="inlineStr">
+      <c r="B28" s="1454" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1418" t="inlineStr">
+      <c r="C28" s="1454" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1419" t="n"/>
-      <c r="E28" s="1419" t="n"/>
-      <c r="F28" s="1419" t="n"/>
-      <c r="G28" s="1419" t="n"/>
-      <c r="H28" s="1419" t="n"/>
-      <c r="I28" s="1420" t="n"/>
-      <c r="J28" s="1421" t="n"/>
-      <c r="K28" s="1421" t="n"/>
-      <c r="L28" s="1421" t="n"/>
-      <c r="M28" s="1419" t="n">
+      <c r="D28" s="1455" t="n"/>
+      <c r="E28" s="1455" t="n"/>
+      <c r="F28" s="1455" t="n"/>
+      <c r="G28" s="1455" t="n"/>
+      <c r="H28" s="1455" t="n"/>
+      <c r="I28" s="1456" t="n"/>
+      <c r="J28" s="1457" t="n"/>
+      <c r="K28" s="1457" t="n"/>
+      <c r="L28" s="1457" t="n"/>
+      <c r="M28" s="1455" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1419" t="n">
+      <c r="N28" s="1455" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1419" t="n"/>
-      <c r="P28" s="1422" t="n"/>
-      <c r="Q28" s="1419" t="n"/>
-      <c r="R28" s="1419" t="n"/>
-      <c r="S28" s="1419" t="n"/>
+      <c r="O28" s="1455" t="n"/>
+      <c r="P28" s="1458" t="n"/>
+      <c r="Q28" s="1455" t="n"/>
+      <c r="R28" s="1455" t="n"/>
+      <c r="S28" s="1455" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1418" t="n"/>
+      <c r="U28" s="1454" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -6460,53 +6568,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1393" t="inlineStr">
+      <c r="A29" s="1429" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1394" t="inlineStr">
+      <c r="B29" s="1430" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1394" t="inlineStr">
+      <c r="C29" s="1430" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1395" t="n"/>
-      <c r="E29" s="1395" t="n">
+      <c r="D29" s="1431" t="n"/>
+      <c r="E29" s="1431" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1395" t="n">
+      <c r="F29" s="1431" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1395" t="n">
+      <c r="G29" s="1431" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1395" t="n"/>
-      <c r="I29" s="1396" t="n"/>
-      <c r="J29" s="1397" t="n"/>
-      <c r="K29" s="1397" t="n"/>
-      <c r="L29" s="1397" t="n"/>
-      <c r="M29" s="1395" t="n"/>
-      <c r="N29" s="1395" t="n"/>
-      <c r="O29" s="1395" t="n">
+      <c r="H29" s="1431" t="n"/>
+      <c r="I29" s="1432" t="n"/>
+      <c r="J29" s="1433" t="n"/>
+      <c r="K29" s="1433" t="n"/>
+      <c r="L29" s="1433" t="n"/>
+      <c r="M29" s="1431" t="n"/>
+      <c r="N29" s="1431" t="n"/>
+      <c r="O29" s="1431" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1398" t="n">
+      <c r="P29" s="1434" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1395" t="n"/>
-      <c r="R29" s="1395" t="n"/>
-      <c r="S29" s="1395" t="n"/>
+      <c r="Q29" s="1431" t="n"/>
+      <c r="R29" s="1431" t="n"/>
+      <c r="S29" s="1431" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1394" t="n"/>
+      <c r="U29" s="1430" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -6514,43 +6622,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1399" t="inlineStr">
+      <c r="A30" s="1435" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1400" t="inlineStr">
+      <c r="B30" s="1436" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1400" t="inlineStr">
+      <c r="C30" s="1436" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1401" t="n"/>
-      <c r="E30" s="1401" t="n"/>
-      <c r="F30" s="1401" t="n"/>
-      <c r="G30" s="1401" t="n"/>
-      <c r="H30" s="1401" t="n"/>
-      <c r="I30" s="1402" t="n"/>
-      <c r="J30" s="1403" t="n"/>
-      <c r="K30" s="1403" t="n"/>
-      <c r="L30" s="1403" t="n"/>
-      <c r="M30" s="1401" t="n"/>
-      <c r="N30" s="1401" t="n"/>
-      <c r="O30" s="1401" t="n"/>
-      <c r="P30" s="1404" t="n"/>
-      <c r="Q30" s="1401" t="n"/>
-      <c r="R30" s="1401" t="n"/>
-      <c r="S30" s="1401" t="n"/>
+      <c r="D30" s="1437" t="n"/>
+      <c r="E30" s="1437" t="n"/>
+      <c r="F30" s="1437" t="n"/>
+      <c r="G30" s="1437" t="n"/>
+      <c r="H30" s="1437" t="n"/>
+      <c r="I30" s="1438" t="n"/>
+      <c r="J30" s="1439" t="n"/>
+      <c r="K30" s="1439" t="n"/>
+      <c r="L30" s="1439" t="n"/>
+      <c r="M30" s="1437" t="n"/>
+      <c r="N30" s="1437" t="n"/>
+      <c r="O30" s="1437" t="n"/>
+      <c r="P30" s="1440" t="n"/>
+      <c r="Q30" s="1437" t="n"/>
+      <c r="R30" s="1437" t="n"/>
+      <c r="S30" s="1437" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1400" t="n"/>
+      <c r="U30" s="1436" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -6558,53 +6666,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1405" t="inlineStr">
+      <c r="A31" s="1441" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1406" t="inlineStr">
+      <c r="B31" s="1442" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1406" t="inlineStr">
+      <c r="C31" s="1442" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1407" t="n"/>
-      <c r="E31" s="1407" t="n">
+      <c r="D31" s="1443" t="n"/>
+      <c r="E31" s="1443" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1407" t="n">
+      <c r="F31" s="1443" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1407" t="n">
+      <c r="G31" s="1443" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1407" t="n"/>
-      <c r="I31" s="1408" t="n"/>
-      <c r="J31" s="1409" t="n"/>
-      <c r="K31" s="1409" t="n"/>
-      <c r="L31" s="1409" t="n"/>
-      <c r="M31" s="1407" t="n"/>
-      <c r="N31" s="1407" t="n"/>
-      <c r="O31" s="1407" t="n">
+      <c r="H31" s="1443" t="n"/>
+      <c r="I31" s="1444" t="n"/>
+      <c r="J31" s="1445" t="n"/>
+      <c r="K31" s="1445" t="n"/>
+      <c r="L31" s="1445" t="n"/>
+      <c r="M31" s="1443" t="n"/>
+      <c r="N31" s="1443" t="n"/>
+      <c r="O31" s="1443" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1410" t="n">
+      <c r="P31" s="1446" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1407" t="n"/>
-      <c r="R31" s="1407" t="n"/>
-      <c r="S31" s="1407" t="n"/>
+      <c r="Q31" s="1443" t="n"/>
+      <c r="R31" s="1443" t="n"/>
+      <c r="S31" s="1443" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1406" t="inlineStr">
+      <c r="U31" s="1442" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -6616,49 +6724,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1417" t="inlineStr">
+      <c r="A32" s="1453" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1418" t="inlineStr">
+      <c r="B32" s="1454" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1418" t="inlineStr">
+      <c r="C32" s="1454" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1419" t="n"/>
-      <c r="E32" s="1419" t="n"/>
-      <c r="F32" s="1419" t="n"/>
-      <c r="G32" s="1419" t="n"/>
-      <c r="H32" s="1419" t="n">
+      <c r="D32" s="1455" t="n"/>
+      <c r="E32" s="1455" t="n"/>
+      <c r="F32" s="1455" t="n"/>
+      <c r="G32" s="1455" t="n"/>
+      <c r="H32" s="1455" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1420" t="n"/>
-      <c r="J32" s="1421" t="n"/>
-      <c r="K32" s="1421" t="n"/>
-      <c r="L32" s="1421" t="n"/>
-      <c r="M32" s="1419" t="n">
+      <c r="I32" s="1456" t="n"/>
+      <c r="J32" s="1457" t="n"/>
+      <c r="K32" s="1457" t="n"/>
+      <c r="L32" s="1457" t="n"/>
+      <c r="M32" s="1455" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1419" t="n">
+      <c r="N32" s="1455" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1419" t="n"/>
-      <c r="P32" s="1422" t="n"/>
-      <c r="Q32" s="1419" t="n"/>
-      <c r="R32" s="1419" t="n"/>
-      <c r="S32" s="1419" t="n"/>
+      <c r="O32" s="1455" t="n"/>
+      <c r="P32" s="1458" t="n"/>
+      <c r="Q32" s="1455" t="n"/>
+      <c r="R32" s="1455" t="n"/>
+      <c r="S32" s="1455" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1418" t="n"/>
+      <c r="U32" s="1454" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -6666,57 +6774,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1393" t="inlineStr">
+      <c r="A33" s="1429" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1394" t="inlineStr">
+      <c r="B33" s="1430" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1394" t="inlineStr">
+      <c r="C33" s="1430" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1395" t="n"/>
-      <c r="E33" s="1395" t="n">
+      <c r="D33" s="1431" t="n"/>
+      <c r="E33" s="1431" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1395" t="n">
+      <c r="F33" s="1431" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1395" t="n">
+      <c r="G33" s="1431" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1395" t="n"/>
-      <c r="I33" s="1396" t="n">
+      <c r="H33" s="1431" t="n"/>
+      <c r="I33" s="1432" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1397" t="n"/>
-      <c r="K33" s="1397" t="n"/>
-      <c r="L33" s="1397" t="n"/>
-      <c r="M33" s="1395" t="n"/>
-      <c r="N33" s="1395" t="n"/>
-      <c r="O33" s="1395" t="n">
+      <c r="J33" s="1433" t="n"/>
+      <c r="K33" s="1433" t="n"/>
+      <c r="L33" s="1433" t="n"/>
+      <c r="M33" s="1431" t="n"/>
+      <c r="N33" s="1431" t="n"/>
+      <c r="O33" s="1431" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1398" t="n">
+      <c r="P33" s="1434" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1395" t="n"/>
-      <c r="R33" s="1395" t="n">
+      <c r="Q33" s="1431" t="n"/>
+      <c r="R33" s="1431" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1395" t="n"/>
+      <c r="S33" s="1431" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1394" t="inlineStr">
+      <c r="U33" s="1430" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -6728,49 +6836,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1399" t="inlineStr">
+      <c r="A34" s="1435" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1400" t="inlineStr">
+      <c r="B34" s="1436" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1400" t="inlineStr">
+      <c r="C34" s="1436" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1401" t="n"/>
-      <c r="E34" s="1401" t="n"/>
-      <c r="F34" s="1401" t="n"/>
-      <c r="G34" s="1401" t="n"/>
-      <c r="H34" s="1401" t="n">
+      <c r="D34" s="1437" t="n"/>
+      <c r="E34" s="1437" t="n"/>
+      <c r="F34" s="1437" t="n"/>
+      <c r="G34" s="1437" t="n"/>
+      <c r="H34" s="1437" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1402" t="n"/>
-      <c r="J34" s="1403" t="n"/>
-      <c r="K34" s="1403" t="n"/>
-      <c r="L34" s="1403" t="n"/>
-      <c r="M34" s="1401" t="n">
+      <c r="I34" s="1438" t="n"/>
+      <c r="J34" s="1439" t="n"/>
+      <c r="K34" s="1439" t="n"/>
+      <c r="L34" s="1439" t="n"/>
+      <c r="M34" s="1437" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1401" t="n">
+      <c r="N34" s="1437" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1401" t="n"/>
-      <c r="P34" s="1404" t="n"/>
-      <c r="Q34" s="1401" t="n"/>
-      <c r="R34" s="1401" t="n"/>
-      <c r="S34" s="1401" t="n"/>
+      <c r="O34" s="1437" t="n"/>
+      <c r="P34" s="1440" t="n"/>
+      <c r="Q34" s="1437" t="n"/>
+      <c r="R34" s="1437" t="n"/>
+      <c r="S34" s="1437" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1400" t="n"/>
+      <c r="U34" s="1436" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -6778,57 +6886,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1405" t="inlineStr">
+      <c r="A35" s="1441" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1406" t="inlineStr">
+      <c r="B35" s="1442" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1406" t="inlineStr">
+      <c r="C35" s="1442" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1407" t="n"/>
-      <c r="E35" s="1407" t="n">
+      <c r="D35" s="1443" t="n"/>
+      <c r="E35" s="1443" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1407" t="n">
+      <c r="F35" s="1443" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1407" t="n">
+      <c r="G35" s="1443" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1407" t="n"/>
-      <c r="I35" s="1408" t="n">
+      <c r="H35" s="1443" t="n"/>
+      <c r="I35" s="1444" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1409" t="n"/>
-      <c r="K35" s="1409" t="n"/>
-      <c r="L35" s="1409" t="n"/>
-      <c r="M35" s="1407" t="n"/>
-      <c r="N35" s="1407" t="n"/>
-      <c r="O35" s="1407" t="n">
+      <c r="J35" s="1445" t="n"/>
+      <c r="K35" s="1445" t="n"/>
+      <c r="L35" s="1445" t="n"/>
+      <c r="M35" s="1443" t="n"/>
+      <c r="N35" s="1443" t="n"/>
+      <c r="O35" s="1443" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1410" t="n">
+      <c r="P35" s="1446" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1407" t="n"/>
-      <c r="R35" s="1407" t="n">
+      <c r="Q35" s="1443" t="n"/>
+      <c r="R35" s="1443" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1407" t="n"/>
+      <c r="S35" s="1443" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1406" t="inlineStr">
+      <c r="U35" s="1442" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -6840,49 +6948,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1411" t="inlineStr">
+      <c r="A36" s="1447" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1412" t="inlineStr">
+      <c r="B36" s="1448" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1412" t="inlineStr">
+      <c r="C36" s="1448" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1413" t="n"/>
-      <c r="E36" s="1413" t="n"/>
-      <c r="F36" s="1413" t="n"/>
-      <c r="G36" s="1413" t="n"/>
-      <c r="H36" s="1413" t="n">
+      <c r="D36" s="1449" t="n"/>
+      <c r="E36" s="1449" t="n"/>
+      <c r="F36" s="1449" t="n"/>
+      <c r="G36" s="1449" t="n"/>
+      <c r="H36" s="1449" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1414" t="n"/>
-      <c r="J36" s="1415" t="n"/>
-      <c r="K36" s="1415" t="n"/>
-      <c r="L36" s="1415" t="n"/>
-      <c r="M36" s="1413" t="n">
+      <c r="I36" s="1450" t="n"/>
+      <c r="J36" s="1451" t="n"/>
+      <c r="K36" s="1451" t="n"/>
+      <c r="L36" s="1451" t="n"/>
+      <c r="M36" s="1449" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1413" t="n">
+      <c r="N36" s="1449" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1413" t="n"/>
-      <c r="P36" s="1416" t="n"/>
-      <c r="Q36" s="1413" t="n"/>
-      <c r="R36" s="1413" t="n"/>
-      <c r="S36" s="1413" t="n"/>
+      <c r="O36" s="1449" t="n"/>
+      <c r="P36" s="1452" t="n"/>
+      <c r="Q36" s="1449" t="n"/>
+      <c r="R36" s="1449" t="n"/>
+      <c r="S36" s="1449" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1412" t="n"/>
+      <c r="U36" s="1448" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -6890,41 +6998,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1417" t="inlineStr">
+      <c r="A37" s="1453" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1418" t="inlineStr">
+      <c r="B37" s="1454" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1418" t="inlineStr">
+      <c r="C37" s="1454" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1419" t="n"/>
-      <c r="E37" s="1419" t="n"/>
-      <c r="F37" s="1419" t="n"/>
-      <c r="G37" s="1419" t="n"/>
-      <c r="H37" s="1419" t="n"/>
-      <c r="I37" s="1420" t="n"/>
-      <c r="J37" s="1421" t="n"/>
-      <c r="K37" s="1421" t="n"/>
-      <c r="L37" s="1421" t="n"/>
-      <c r="M37" s="1419" t="n"/>
-      <c r="N37" s="1419" t="n"/>
-      <c r="O37" s="1419" t="n"/>
-      <c r="P37" s="1422" t="n"/>
-      <c r="Q37" s="1419" t="n">
+      <c r="D37" s="1455" t="n"/>
+      <c r="E37" s="1455" t="n"/>
+      <c r="F37" s="1455" t="n"/>
+      <c r="G37" s="1455" t="n"/>
+      <c r="H37" s="1455" t="n"/>
+      <c r="I37" s="1456" t="n"/>
+      <c r="J37" s="1457" t="n"/>
+      <c r="K37" s="1457" t="n"/>
+      <c r="L37" s="1457" t="n"/>
+      <c r="M37" s="1455" t="n"/>
+      <c r="N37" s="1455" t="n"/>
+      <c r="O37" s="1455" t="n"/>
+      <c r="P37" s="1458" t="n"/>
+      <c r="Q37" s="1455" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1419" t="n"/>
-      <c r="S37" s="1419" t="n"/>
+      <c r="R37" s="1455" t="n"/>
+      <c r="S37" s="1455" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1418" t="n"/>
+      <c r="U37" s="1454" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -6932,57 +7040,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1393" t="inlineStr">
+      <c r="A38" s="1429" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1394" t="inlineStr">
+      <c r="B38" s="1430" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1394" t="inlineStr">
+      <c r="C38" s="1430" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1395" t="n"/>
-      <c r="E38" s="1395" t="n">
+      <c r="D38" s="1431" t="n"/>
+      <c r="E38" s="1431" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1395" t="n">
+      <c r="F38" s="1431" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1395" t="n">
+      <c r="G38" s="1431" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1395" t="n"/>
-      <c r="I38" s="1396" t="n">
+      <c r="H38" s="1431" t="n"/>
+      <c r="I38" s="1432" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1397" t="n"/>
-      <c r="K38" s="1397" t="n"/>
-      <c r="L38" s="1397" t="n"/>
-      <c r="M38" s="1395" t="n"/>
-      <c r="N38" s="1395" t="n"/>
-      <c r="O38" s="1395" t="n">
+      <c r="J38" s="1433" t="n"/>
+      <c r="K38" s="1433" t="n"/>
+      <c r="L38" s="1433" t="n"/>
+      <c r="M38" s="1431" t="n"/>
+      <c r="N38" s="1431" t="n"/>
+      <c r="O38" s="1431" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1398" t="n">
+      <c r="P38" s="1434" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1395" t="n"/>
-      <c r="R38" s="1395" t="n">
+      <c r="Q38" s="1431" t="n"/>
+      <c r="R38" s="1431" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1395" t="n"/>
+      <c r="S38" s="1431" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1394" t="inlineStr">
+      <c r="U38" s="1430" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -6994,49 +7102,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1423" t="inlineStr">
+      <c r="A39" s="1459" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1424" t="inlineStr">
+      <c r="B39" s="1460" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1424" t="inlineStr">
+      <c r="C39" s="1460" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1425" t="n"/>
-      <c r="E39" s="1425" t="n"/>
-      <c r="F39" s="1425" t="n"/>
-      <c r="G39" s="1425" t="n"/>
-      <c r="H39" s="1425" t="n">
+      <c r="D39" s="1461" t="n"/>
+      <c r="E39" s="1461" t="n"/>
+      <c r="F39" s="1461" t="n"/>
+      <c r="G39" s="1461" t="n"/>
+      <c r="H39" s="1461" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1426" t="n"/>
-      <c r="J39" s="1427" t="n"/>
-      <c r="K39" s="1427" t="n"/>
-      <c r="L39" s="1427" t="n"/>
-      <c r="M39" s="1425" t="n">
+      <c r="I39" s="1462" t="n"/>
+      <c r="J39" s="1463" t="n"/>
+      <c r="K39" s="1463" t="n"/>
+      <c r="L39" s="1463" t="n"/>
+      <c r="M39" s="1461" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1425" t="n">
+      <c r="N39" s="1461" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1425" t="n"/>
-      <c r="P39" s="1428" t="n"/>
-      <c r="Q39" s="1425" t="n"/>
-      <c r="R39" s="1425" t="n"/>
-      <c r="S39" s="1425" t="n"/>
+      <c r="O39" s="1461" t="n"/>
+      <c r="P39" s="1464" t="n"/>
+      <c r="Q39" s="1461" t="n"/>
+      <c r="R39" s="1461" t="n"/>
+      <c r="S39" s="1461" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1424" t="n"/>
+      <c r="U39" s="1460" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -7044,41 +7152,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1399" t="inlineStr">
+      <c r="A40" s="1435" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1400" t="inlineStr">
+      <c r="B40" s="1436" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1400" t="inlineStr">
+      <c r="C40" s="1436" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1401" t="n"/>
-      <c r="E40" s="1401" t="n"/>
-      <c r="F40" s="1401" t="n"/>
-      <c r="G40" s="1401" t="n"/>
-      <c r="H40" s="1401" t="n"/>
-      <c r="I40" s="1402" t="n"/>
-      <c r="J40" s="1403" t="n"/>
-      <c r="K40" s="1403" t="n"/>
-      <c r="L40" s="1403" t="n"/>
-      <c r="M40" s="1401" t="n"/>
-      <c r="N40" s="1401" t="n"/>
-      <c r="O40" s="1401" t="n"/>
-      <c r="P40" s="1404" t="n"/>
-      <c r="Q40" s="1401" t="n">
+      <c r="D40" s="1437" t="n"/>
+      <c r="E40" s="1437" t="n"/>
+      <c r="F40" s="1437" t="n"/>
+      <c r="G40" s="1437" t="n"/>
+      <c r="H40" s="1437" t="n"/>
+      <c r="I40" s="1438" t="n"/>
+      <c r="J40" s="1439" t="n"/>
+      <c r="K40" s="1439" t="n"/>
+      <c r="L40" s="1439" t="n"/>
+      <c r="M40" s="1437" t="n"/>
+      <c r="N40" s="1437" t="n"/>
+      <c r="O40" s="1437" t="n"/>
+      <c r="P40" s="1440" t="n"/>
+      <c r="Q40" s="1437" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1401" t="n"/>
-      <c r="S40" s="1401" t="n"/>
+      <c r="R40" s="1437" t="n"/>
+      <c r="S40" s="1437" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1400" t="n"/>
+      <c r="U40" s="1436" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -7086,57 +7194,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1405" t="inlineStr">
+      <c r="A41" s="1441" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1406" t="inlineStr">
+      <c r="B41" s="1442" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1406" t="inlineStr">
+      <c r="C41" s="1442" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1407" t="n"/>
-      <c r="E41" s="1407" t="n">
+      <c r="D41" s="1443" t="n"/>
+      <c r="E41" s="1443" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1407" t="n">
+      <c r="F41" s="1443" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1407" t="n">
+      <c r="G41" s="1443" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1407" t="n"/>
-      <c r="I41" s="1408" t="n">
+      <c r="H41" s="1443" t="n"/>
+      <c r="I41" s="1444" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1409" t="n"/>
-      <c r="K41" s="1409" t="n"/>
-      <c r="L41" s="1409" t="n"/>
-      <c r="M41" s="1407" t="n"/>
-      <c r="N41" s="1407" t="n"/>
-      <c r="O41" s="1407" t="n">
+      <c r="J41" s="1445" t="n"/>
+      <c r="K41" s="1445" t="n"/>
+      <c r="L41" s="1445" t="n"/>
+      <c r="M41" s="1443" t="n"/>
+      <c r="N41" s="1443" t="n"/>
+      <c r="O41" s="1443" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1410" t="n">
+      <c r="P41" s="1446" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1407" t="n"/>
-      <c r="R41" s="1407" t="n">
+      <c r="Q41" s="1443" t="n"/>
+      <c r="R41" s="1443" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1407" t="n"/>
+      <c r="S41" s="1443" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1406" t="inlineStr">
+      <c r="U41" s="1442" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -7148,49 +7256,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1417" t="inlineStr">
+      <c r="A42" s="1453" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1418" t="inlineStr">
+      <c r="B42" s="1454" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1418" t="inlineStr">
+      <c r="C42" s="1454" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1419" t="n"/>
-      <c r="E42" s="1419" t="n"/>
-      <c r="F42" s="1419" t="n"/>
-      <c r="G42" s="1419" t="n"/>
-      <c r="H42" s="1419" t="n">
+      <c r="D42" s="1455" t="n"/>
+      <c r="E42" s="1455" t="n"/>
+      <c r="F42" s="1455" t="n"/>
+      <c r="G42" s="1455" t="n"/>
+      <c r="H42" s="1455" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1420" t="n"/>
-      <c r="J42" s="1421" t="n"/>
-      <c r="K42" s="1421" t="n"/>
-      <c r="L42" s="1421" t="n"/>
-      <c r="M42" s="1419" t="n">
+      <c r="I42" s="1456" t="n"/>
+      <c r="J42" s="1457" t="n"/>
+      <c r="K42" s="1457" t="n"/>
+      <c r="L42" s="1457" t="n"/>
+      <c r="M42" s="1455" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1419" t="n">
+      <c r="N42" s="1455" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1419" t="n"/>
-      <c r="P42" s="1422" t="n"/>
-      <c r="Q42" s="1419" t="n"/>
-      <c r="R42" s="1419" t="n"/>
-      <c r="S42" s="1419" t="n"/>
+      <c r="O42" s="1455" t="n"/>
+      <c r="P42" s="1458" t="n"/>
+      <c r="Q42" s="1455" t="n"/>
+      <c r="R42" s="1455" t="n"/>
+      <c r="S42" s="1455" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1418" t="n"/>
+      <c r="U42" s="1454" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -7198,57 +7306,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1393" t="inlineStr">
+      <c r="A43" s="1429" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1394" t="inlineStr">
+      <c r="B43" s="1430" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1394" t="inlineStr">
+      <c r="C43" s="1430" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1395" t="n"/>
-      <c r="E43" s="1395" t="n">
+      <c r="D43" s="1431" t="n"/>
+      <c r="E43" s="1431" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1395" t="n">
+      <c r="F43" s="1431" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1395" t="n">
+      <c r="G43" s="1431" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1395" t="n"/>
-      <c r="I43" s="1396" t="n">
+      <c r="H43" s="1431" t="n"/>
+      <c r="I43" s="1432" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1397" t="n"/>
-      <c r="K43" s="1397" t="n"/>
-      <c r="L43" s="1397" t="n"/>
-      <c r="M43" s="1395" t="n"/>
-      <c r="N43" s="1395" t="n"/>
-      <c r="O43" s="1395" t="n">
+      <c r="J43" s="1433" t="n"/>
+      <c r="K43" s="1433" t="n"/>
+      <c r="L43" s="1433" t="n"/>
+      <c r="M43" s="1431" t="n"/>
+      <c r="N43" s="1431" t="n"/>
+      <c r="O43" s="1431" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1398" t="n">
+      <c r="P43" s="1434" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1395" t="n"/>
-      <c r="R43" s="1395" t="n">
+      <c r="Q43" s="1431" t="n"/>
+      <c r="R43" s="1431" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1395" t="n"/>
+      <c r="S43" s="1431" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1394" t="n"/>
+      <c r="U43" s="1430" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -7256,45 +7364,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1423" t="inlineStr">
+      <c r="A44" s="1459" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1424" t="inlineStr">
+      <c r="B44" s="1460" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1424" t="inlineStr">
+      <c r="C44" s="1460" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1425" t="n"/>
-      <c r="E44" s="1425" t="n">
+      <c r="D44" s="1461" t="n"/>
+      <c r="E44" s="1461" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1425" t="n">
+      <c r="F44" s="1461" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1425" t="n"/>
-      <c r="H44" s="1425" t="n"/>
-      <c r="I44" s="1426" t="n"/>
-      <c r="J44" s="1427" t="n"/>
-      <c r="K44" s="1427" t="n"/>
-      <c r="L44" s="1427" t="n"/>
-      <c r="M44" s="1425" t="n"/>
-      <c r="N44" s="1425" t="n"/>
-      <c r="O44" s="1425" t="n"/>
-      <c r="P44" s="1428" t="n"/>
-      <c r="Q44" s="1425" t="n"/>
-      <c r="R44" s="1425" t="n"/>
-      <c r="S44" s="1425" t="n">
+      <c r="G44" s="1461" t="n"/>
+      <c r="H44" s="1461" t="n"/>
+      <c r="I44" s="1462" t="n"/>
+      <c r="J44" s="1463" t="n"/>
+      <c r="K44" s="1463" t="n"/>
+      <c r="L44" s="1463" t="n"/>
+      <c r="M44" s="1461" t="n"/>
+      <c r="N44" s="1461" t="n"/>
+      <c r="O44" s="1461" t="n"/>
+      <c r="P44" s="1464" t="n"/>
+      <c r="Q44" s="1461" t="n"/>
+      <c r="R44" s="1461" t="n"/>
+      <c r="S44" s="1461" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1424" t="inlineStr">
+      <c r="U44" s="1460" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -7306,49 +7414,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1423" t="inlineStr">
+      <c r="A45" s="1459" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1424" t="inlineStr">
+      <c r="B45" s="1460" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1424" t="inlineStr">
+      <c r="C45" s="1460" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1425" t="n"/>
-      <c r="E45" s="1425" t="n"/>
-      <c r="F45" s="1425" t="n"/>
-      <c r="G45" s="1425" t="n"/>
-      <c r="H45" s="1425" t="n">
+      <c r="D45" s="1461" t="n"/>
+      <c r="E45" s="1461" t="n"/>
+      <c r="F45" s="1461" t="n"/>
+      <c r="G45" s="1461" t="n"/>
+      <c r="H45" s="1461" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1426" t="n"/>
-      <c r="J45" s="1427" t="n"/>
-      <c r="K45" s="1427" t="n"/>
-      <c r="L45" s="1427" t="n"/>
-      <c r="M45" s="1425" t="n">
+      <c r="I45" s="1462" t="n"/>
+      <c r="J45" s="1463" t="n"/>
+      <c r="K45" s="1463" t="n"/>
+      <c r="L45" s="1463" t="n"/>
+      <c r="M45" s="1461" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1425" t="n">
+      <c r="N45" s="1461" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1425" t="n"/>
-      <c r="P45" s="1428" t="n"/>
-      <c r="Q45" s="1425" t="n"/>
-      <c r="R45" s="1425" t="n"/>
-      <c r="S45" s="1425" t="n"/>
+      <c r="O45" s="1461" t="n"/>
+      <c r="P45" s="1464" t="n"/>
+      <c r="Q45" s="1461" t="n"/>
+      <c r="R45" s="1461" t="n"/>
+      <c r="S45" s="1461" t="n"/>
       <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1424" t="n"/>
+      <c r="U45" s="1460" t="n"/>
       <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -7356,39 +7464,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1399" t="inlineStr">
+      <c r="A46" s="1435" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B46" s="1400" t="inlineStr">
+      <c r="B46" s="1436" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="C46" s="1400" t="inlineStr">
+      <c r="C46" s="1436" t="inlineStr">
         <is>
           <t>EVENT - Clean</t>
         </is>
       </c>
-      <c r="D46" s="1401" t="n"/>
-      <c r="E46" s="1401" t="n"/>
-      <c r="F46" s="1401" t="n"/>
-      <c r="G46" s="1401" t="n"/>
-      <c r="H46" s="1401" t="n"/>
-      <c r="I46" s="1402" t="n"/>
-      <c r="J46" s="1403" t="n"/>
-      <c r="K46" s="1403" t="n"/>
-      <c r="L46" s="1403" t="n"/>
-      <c r="M46" s="1401" t="n"/>
-      <c r="N46" s="1401" t="n"/>
-      <c r="O46" s="1401" t="n"/>
-      <c r="P46" s="1404" t="n"/>
-      <c r="Q46" s="1401" t="n"/>
-      <c r="R46" s="1401" t="n"/>
-      <c r="S46" s="1401" t="n"/>
+      <c r="D46" s="1437" t="n"/>
+      <c r="E46" s="1437" t="n"/>
+      <c r="F46" s="1437" t="n"/>
+      <c r="G46" s="1437" t="n"/>
+      <c r="H46" s="1437" t="n"/>
+      <c r="I46" s="1438" t="n"/>
+      <c r="J46" s="1439" t="n"/>
+      <c r="K46" s="1439" t="n"/>
+      <c r="L46" s="1439" t="n"/>
+      <c r="M46" s="1437" t="n"/>
+      <c r="N46" s="1437" t="n"/>
+      <c r="O46" s="1437" t="n"/>
+      <c r="P46" s="1440" t="n"/>
+      <c r="Q46" s="1437" t="n"/>
+      <c r="R46" s="1437" t="n"/>
+      <c r="S46" s="1437" t="n"/>
       <c r="T46" s="631" t="n"/>
-      <c r="U46" s="1400" t="n"/>
+      <c r="U46" s="1436" t="n"/>
       <c r="V46" s="632" t="inlineStr">
         <is>
           <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
@@ -7396,51 +7504,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1405" t="inlineStr">
+      <c r="A47" s="1441" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1406" t="inlineStr">
+      <c r="B47" s="1442" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C47" s="1406" t="inlineStr">
+      <c r="C47" s="1442" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D47" s="1407" t="n"/>
-      <c r="E47" s="1407" t="n">
+      <c r="D47" s="1443" t="n"/>
+      <c r="E47" s="1443" t="n">
         <v>16.6</v>
       </c>
-      <c r="F47" s="1407" t="n">
+      <c r="F47" s="1443" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="1407" t="n">
+      <c r="G47" s="1443" t="n">
         <v>4.1</v>
       </c>
-      <c r="H47" s="1407" t="n"/>
-      <c r="I47" s="1408" t="n">
+      <c r="H47" s="1443" t="n"/>
+      <c r="I47" s="1444" t="n">
         <v>0.9</v>
       </c>
-      <c r="J47" s="1409" t="n"/>
-      <c r="K47" s="1409" t="n"/>
-      <c r="L47" s="1409" t="n"/>
-      <c r="M47" s="1407" t="n"/>
-      <c r="N47" s="1407" t="n"/>
-      <c r="O47" s="1407" t="n">
+      <c r="J47" s="1445" t="n"/>
+      <c r="K47" s="1445" t="n"/>
+      <c r="L47" s="1445" t="n"/>
+      <c r="M47" s="1443" t="n"/>
+      <c r="N47" s="1443" t="n"/>
+      <c r="O47" s="1443" t="n">
         <v>13.2</v>
       </c>
-      <c r="P47" s="1410" t="n">
+      <c r="P47" s="1446" t="n">
         <v>0</v>
       </c>
-      <c r="Q47" s="1407" t="n"/>
-      <c r="R47" s="1407" t="n">
+      <c r="Q47" s="1443" t="n"/>
+      <c r="R47" s="1443" t="n">
         <v>84.5</v>
       </c>
-      <c r="S47" s="1407" t="n">
+      <c r="S47" s="1443" t="n">
         <v>11.8</v>
       </c>
       <c r="T47" s="813" t="inlineStr">
@@ -7448,7 +7556,7 @@
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1406" t="inlineStr">
+      <c r="U47" s="1442" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
@@ -7460,49 +7568,49 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1417" t="inlineStr">
+      <c r="A48" s="1453" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B48" s="1418" t="inlineStr">
+      <c r="B48" s="1454" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C48" s="1418" t="inlineStr">
+      <c r="C48" s="1454" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D48" s="1419" t="n"/>
-      <c r="E48" s="1419" t="n"/>
-      <c r="F48" s="1419" t="n"/>
-      <c r="G48" s="1419" t="n"/>
-      <c r="H48" s="1419" t="n">
+      <c r="D48" s="1455" t="n"/>
+      <c r="E48" s="1455" t="n"/>
+      <c r="F48" s="1455" t="n"/>
+      <c r="G48" s="1455" t="n"/>
+      <c r="H48" s="1455" t="n">
         <v>15.1</v>
       </c>
-      <c r="I48" s="1420" t="n"/>
-      <c r="J48" s="1421" t="n"/>
-      <c r="K48" s="1421" t="n"/>
-      <c r="L48" s="1421" t="n"/>
-      <c r="M48" s="1419" t="n">
+      <c r="I48" s="1456" t="n"/>
+      <c r="J48" s="1457" t="n"/>
+      <c r="K48" s="1457" t="n"/>
+      <c r="L48" s="1457" t="n"/>
+      <c r="M48" s="1455" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="1419" t="n">
+      <c r="N48" s="1455" t="n">
         <v>20</v>
       </c>
-      <c r="O48" s="1419" t="n"/>
-      <c r="P48" s="1422" t="n"/>
-      <c r="Q48" s="1419" t="n"/>
-      <c r="R48" s="1419" t="n"/>
-      <c r="S48" s="1419" t="n"/>
+      <c r="O48" s="1455" t="n"/>
+      <c r="P48" s="1458" t="n"/>
+      <c r="Q48" s="1455" t="n"/>
+      <c r="R48" s="1455" t="n"/>
+      <c r="S48" s="1455" t="n"/>
       <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U48" s="1418" t="n"/>
+      <c r="U48" s="1454" t="n"/>
       <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
@@ -7510,51 +7618,51 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1393" t="inlineStr">
+      <c r="A49" s="1429" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B49" s="1394" t="inlineStr">
+      <c r="B49" s="1430" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C49" s="1394" t="inlineStr">
+      <c r="C49" s="1430" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D49" s="1395" t="n"/>
-      <c r="E49" s="1395" t="n">
+      <c r="D49" s="1431" t="n"/>
+      <c r="E49" s="1431" t="n">
         <v>16.8</v>
       </c>
-      <c r="F49" s="1395" t="n">
+      <c r="F49" s="1431" t="n">
         <v>0.2</v>
       </c>
-      <c r="G49" s="1395" t="n">
+      <c r="G49" s="1431" t="n">
         <v>3.3</v>
       </c>
-      <c r="H49" s="1395" t="n"/>
-      <c r="I49" s="1396" t="n">
+      <c r="H49" s="1431" t="n"/>
+      <c r="I49" s="1432" t="n">
         <v>1.7</v>
       </c>
-      <c r="J49" s="1397" t="n"/>
-      <c r="K49" s="1397" t="n"/>
-      <c r="L49" s="1397" t="n"/>
-      <c r="M49" s="1395" t="n"/>
-      <c r="N49" s="1395" t="n"/>
-      <c r="O49" s="1395" t="n">
+      <c r="J49" s="1433" t="n"/>
+      <c r="K49" s="1433" t="n"/>
+      <c r="L49" s="1433" t="n"/>
+      <c r="M49" s="1431" t="n"/>
+      <c r="N49" s="1431" t="n"/>
+      <c r="O49" s="1431" t="n">
         <v>13</v>
       </c>
-      <c r="P49" s="1398" t="n">
+      <c r="P49" s="1434" t="n">
         <v>0.87</v>
       </c>
-      <c r="Q49" s="1395" t="n"/>
-      <c r="R49" s="1395" t="n">
+      <c r="Q49" s="1431" t="n"/>
+      <c r="R49" s="1431" t="n">
         <v>86</v>
       </c>
-      <c r="S49" s="1395" t="n">
+      <c r="S49" s="1431" t="n">
         <v>11.65</v>
       </c>
       <c r="T49" s="624" t="inlineStr">
@@ -7562,7 +7670,7 @@
           <t>Clear now, 88F, 67% RH; sun so far 6.4h of 7h daylight (91%); today high 90F, 0.87in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U49" s="1394" t="inlineStr">
+      <c r="U49" s="1430" t="inlineStr">
         <is>
           <t>2026-07-04_1.jpeg;2026-07-04_2.jpeg;2026-07-04_3.jpeg;2026-07-04_4.jpeg</t>
         </is>
@@ -7574,49 +7682,49 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1399" t="inlineStr">
+      <c r="A50" s="1435" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B50" s="1400" t="inlineStr">
+      <c r="B50" s="1436" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C50" s="1400" t="inlineStr">
+      <c r="C50" s="1436" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D50" s="1401" t="n"/>
-      <c r="E50" s="1401" t="n"/>
-      <c r="F50" s="1401" t="n"/>
-      <c r="G50" s="1401" t="n"/>
-      <c r="H50" s="1401" t="n">
+      <c r="D50" s="1437" t="n"/>
+      <c r="E50" s="1437" t="n"/>
+      <c r="F50" s="1437" t="n"/>
+      <c r="G50" s="1437" t="n"/>
+      <c r="H50" s="1437" t="n">
         <v>14.6</v>
       </c>
-      <c r="I50" s="1402" t="n"/>
-      <c r="J50" s="1403" t="n"/>
-      <c r="K50" s="1403" t="n"/>
-      <c r="L50" s="1403" t="n"/>
-      <c r="M50" s="1401" t="n">
+      <c r="I50" s="1438" t="n"/>
+      <c r="J50" s="1439" t="n"/>
+      <c r="K50" s="1439" t="n"/>
+      <c r="L50" s="1439" t="n"/>
+      <c r="M50" s="1437" t="n">
         <v>0.5</v>
       </c>
-      <c r="N50" s="1401" t="n">
+      <c r="N50" s="1437" t="n">
         <v>20.5</v>
       </c>
-      <c r="O50" s="1401" t="n"/>
-      <c r="P50" s="1404" t="n"/>
-      <c r="Q50" s="1401" t="n"/>
-      <c r="R50" s="1401" t="n"/>
-      <c r="S50" s="1401" t="n"/>
+      <c r="O50" s="1437" t="n"/>
+      <c r="P50" s="1440" t="n"/>
+      <c r="Q50" s="1437" t="n"/>
+      <c r="R50" s="1437" t="n"/>
+      <c r="S50" s="1437" t="n"/>
       <c r="T50" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny day (high 90F, water 86F); storm forecast overnight</t>
         </is>
       </c>
-      <c r="U50" s="1400" t="n"/>
+      <c r="U50" s="1436" t="n"/>
       <c r="V50" s="632" t="inlineStr">
         <is>
           <t>0.5 gal added 7:40 PM. PARTY PRE-LOAD (Sun 7/5 1PM picnic): deliberately HALF the usual dose -- FC already high at 16.8, and John didn't want to overshoot into the high teens for guests. Sized on the retuned model (l24_hot_sunny now 4.0). Model projects ~14.6 next noon, BUT this is a known weather-mismatch case: model keys L24 off today's hot/sunny weather, while the actual loss window is a storm overnight (no UV) + cooler/cloudy Sun morning -&gt; real loss will be LOWER, so FC likely lands ~15-16 at the party (comfortable top-of-band, cushion for bather load, not overboard). =&gt; If tomorrow's noon comes in ABOVE 14.6, that's the weather mismatch, NOT the freshly-retuned constant; don't chase it. Plan: dose back up Sun evening after the crowd's out (expect a bather-load FC drop). Season total 20.5 gal. PHOTOS(4): water clear/healthy blue, bottom fully visible, no cloudiness/algae; yesterday's surface debris now gone (tracks with CC clearing to 0.2); liner step close-up normal speckled blue, no rust/stain progression. Ruler photo documents the ~11.65 cm level.</t>
@@ -7624,47 +7732,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1405" t="inlineStr">
+      <c r="A51" s="1441" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B51" s="1406" t="inlineStr">
+      <c r="B51" s="1442" t="inlineStr">
         <is>
           <t>07:45</t>
         </is>
       </c>
-      <c r="C51" s="1406" t="inlineStr">
+      <c r="C51" s="1442" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D51" s="1407" t="n"/>
-      <c r="E51" s="1407" t="n">
+      <c r="D51" s="1443" t="n"/>
+      <c r="E51" s="1443" t="n">
         <v>16</v>
       </c>
-      <c r="F51" s="1407" t="n">
+      <c r="F51" s="1443" t="n">
         <v>0.5</v>
       </c>
-      <c r="G51" s="1407" t="n"/>
-      <c r="H51" s="1407" t="n"/>
-      <c r="I51" s="1408" t="n">
+      <c r="G51" s="1443" t="n"/>
+      <c r="H51" s="1443" t="n"/>
+      <c r="I51" s="1444" t="n">
         <v>1.4</v>
       </c>
-      <c r="J51" s="1409" t="n"/>
-      <c r="K51" s="1409" t="n"/>
-      <c r="L51" s="1409" t="n"/>
-      <c r="M51" s="1407" t="n"/>
-      <c r="N51" s="1407" t="n"/>
-      <c r="O51" s="1407" t="n"/>
-      <c r="P51" s="1410" t="n">
+      <c r="J51" s="1445" t="n"/>
+      <c r="K51" s="1445" t="n"/>
+      <c r="L51" s="1445" t="n"/>
+      <c r="M51" s="1443" t="n"/>
+      <c r="N51" s="1443" t="n"/>
+      <c r="O51" s="1443" t="n"/>
+      <c r="P51" s="1446" t="n">
         <v>0.04</v>
       </c>
-      <c r="Q51" s="1407" t="n"/>
-      <c r="R51" s="1407" t="n">
+      <c r="Q51" s="1443" t="n"/>
+      <c r="R51" s="1443" t="n">
         <v>84</v>
       </c>
-      <c r="S51" s="1407" t="n">
+      <c r="S51" s="1443" t="n">
         <v>13.9</v>
       </c>
       <c r="T51" s="813" t="inlineStr">
@@ -7672,7 +7780,11 @@
           <t>Overcast now, 75F, 90% RH; sun so far 0.0h of 3h daylight (0%); today high 75F, 0.04in precip, UV max 6.5</t>
         </is>
       </c>
-      <c r="U51" s="1406" t="n"/>
+      <c r="U51" s="1442" t="inlineStr">
+        <is>
+          <t>2026-07-05_2.jpeg</t>
+        </is>
+      </c>
       <c r="V51" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. Early test (7:45 AM, party day 1PM, John busy) -- off the usual noon cadence, fine. PARTY CALL: FC 16.0 is great; NO morning top-up needed (plan only called for one 'if FC slipped' -- it didn't). Cloudy/cool day (75F, 0 sun) means it'll hold through the party. WEATHER-MISMATCH CONFIRMED (as flagged on last night's dose): 7/4 dose predicted 14.6 for today assuming hot/sunny loss, but today is overcast/cool -&gt; FC ran high at 16.0 (pred error +1.4). This is the weather mismatch, NOT the freshly-retuned l24_hot_sunny=4.0; the constant still gets validated by future clean HOT-day noon readings (mid-week, after Mon rain). fc_loss left blank: off-cadence (~19h not 24h), 0.5gal dose in between, plus rain dilution -&gt; non-comparable. WATER LEVEL 11.65 -&gt; 13.9 (+2.25 cm) from the overnight storm (~0.9in rain, ~445 gal) -- ruler tracked the storm perfectly. CC ticked 0.2 -&gt; 0.5 (rain-driven organic/N load washed in by the storm; still a trace, high FC clears it -- not a party concern). Water temp 86 -&gt; 84 (cool front). NOTE: the BIG rain is still Mon 7/6 (~5.7in) -&gt; watch for overflow then, possible backwash-down after (bonus CYA lowering).</t>
@@ -7680,49 +7792,51 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1417" t="inlineStr">
+      <c r="A52" s="1453" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B52" s="1418" t="inlineStr">
+      <c r="B52" s="1454" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C52" s="1418" t="inlineStr">
+      <c r="C52" s="1454" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D52" s="1419" t="n"/>
-      <c r="E52" s="1419" t="n">
+      <c r="D52" s="1455" t="n"/>
+      <c r="E52" s="1455" t="n">
         <v>14.8</v>
       </c>
-      <c r="F52" s="1419" t="n">
+      <c r="F52" s="1455" t="n">
         <v>0.3</v>
       </c>
-      <c r="G52" s="1419" t="n"/>
-      <c r="H52" s="1419" t="n"/>
-      <c r="I52" s="1420" t="n"/>
-      <c r="J52" s="1421" t="n"/>
-      <c r="K52" s="1421" t="n"/>
-      <c r="L52" s="1421" t="n"/>
-      <c r="M52" s="1419" t="n"/>
-      <c r="N52" s="1419" t="n"/>
-      <c r="O52" s="1419" t="n"/>
-      <c r="P52" s="1422" t="n"/>
-      <c r="Q52" s="1419" t="n"/>
-      <c r="R52" s="1419" t="n"/>
-      <c r="S52" s="1419" t="n"/>
+      <c r="G52" s="1455" t="n"/>
+      <c r="H52" s="1455" t="n"/>
+      <c r="I52" s="1456" t="n"/>
+      <c r="J52" s="1457" t="n"/>
+      <c r="K52" s="1457" t="n"/>
+      <c r="L52" s="1457" t="n"/>
+      <c r="M52" s="1455" t="n"/>
+      <c r="N52" s="1455" t="n"/>
+      <c r="O52" s="1455" t="n"/>
+      <c r="P52" s="1458" t="n"/>
+      <c r="Q52" s="1455" t="n"/>
+      <c r="R52" s="1455" t="n"/>
+      <c r="S52" s="1455" t="n">
+        <v>13.6</v>
+      </c>
       <c r="T52" s="827" t="inlineStr">
         <is>
           <t>Overcast now, 72F, 76% RH; sun so far 8.4h of 13h daylight (65%); today high 80F, 0.00in precip, UV max 6.0</t>
         </is>
       </c>
-      <c r="U52" s="1418" t="inlineStr">
-        <is>
-          <t>2026-07-05_1.jpeg;2026-07-05_2.jpeg</t>
+      <c r="U52" s="1454" t="inlineStr">
+        <is>
+          <t>2026-07-05_1.jpeg;2026-07-05_3.jpeg</t>
         </is>
       </c>
       <c r="V52" s="828" t="inlineStr">

</xml_diff>

<commit_message>
Add video support to Photos page; log 2026-07-05 dose (0.5 gal, season 21.0)
Renders an HTML5 <video> player above each day's photos when a dated .mp4
is present. Phone .MOV originals are transcoded to a small web mp4 with
ffmpeg (960p/CRF30/faststart, ~40MB->8MB) and gitignored; only the mp4
is committed. build_site scans/copies .mp4 by date and build_photos
emits the player above the thumbs. Also logs tonight's party-recovery
dose (0.5 gal @ 7:25pm, cum 21.0, projecting ~15.1 Mon noon).
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1465">
+  <cellXfs count="1501">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -4706,6 +4706,114 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -5183,7 +5291,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V52"/>
+  <dimension ref="A1:V53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -5360,35 +5468,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1429" t="inlineStr">
+      <c r="A3" s="1465" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1430" t="n"/>
-      <c r="C3" s="1430" t="inlineStr">
+      <c r="B3" s="1466" t="n"/>
+      <c r="C3" s="1466" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1431" t="n"/>
-      <c r="E3" s="1431" t="n"/>
-      <c r="F3" s="1431" t="n"/>
-      <c r="G3" s="1431" t="n"/>
-      <c r="H3" s="1431" t="n"/>
-      <c r="I3" s="1432" t="n"/>
-      <c r="J3" s="1433" t="n"/>
-      <c r="K3" s="1433" t="n"/>
-      <c r="L3" s="1433" t="n"/>
-      <c r="M3" s="1431" t="n"/>
-      <c r="N3" s="1431" t="n"/>
-      <c r="O3" s="1431" t="n"/>
-      <c r="P3" s="1434" t="n"/>
-      <c r="Q3" s="1431" t="n"/>
-      <c r="R3" s="1431" t="n"/>
-      <c r="S3" s="1431" t="n"/>
+      <c r="D3" s="1467" t="n"/>
+      <c r="E3" s="1467" t="n"/>
+      <c r="F3" s="1467" t="n"/>
+      <c r="G3" s="1467" t="n"/>
+      <c r="H3" s="1467" t="n"/>
+      <c r="I3" s="1468" t="n"/>
+      <c r="J3" s="1469" t="n"/>
+      <c r="K3" s="1469" t="n"/>
+      <c r="L3" s="1469" t="n"/>
+      <c r="M3" s="1467" t="n"/>
+      <c r="N3" s="1467" t="n"/>
+      <c r="O3" s="1467" t="n"/>
+      <c r="P3" s="1470" t="n"/>
+      <c r="Q3" s="1467" t="n"/>
+      <c r="R3" s="1467" t="n"/>
+      <c r="S3" s="1467" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1430" t="n"/>
+      <c r="U3" s="1466" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -5396,43 +5504,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1435" t="inlineStr">
+      <c r="A4" s="1471" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1436" t="inlineStr">
+      <c r="B4" s="1472" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1436" t="inlineStr">
+      <c r="C4" s="1472" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1437" t="n"/>
-      <c r="E4" s="1437" t="n"/>
-      <c r="F4" s="1437" t="n"/>
-      <c r="G4" s="1437" t="n"/>
-      <c r="H4" s="1437" t="n"/>
-      <c r="I4" s="1438" t="n"/>
-      <c r="J4" s="1439" t="n"/>
-      <c r="K4" s="1439" t="n"/>
-      <c r="L4" s="1439" t="n"/>
-      <c r="M4" s="1437" t="n">
+      <c r="D4" s="1473" t="n"/>
+      <c r="E4" s="1473" t="n"/>
+      <c r="F4" s="1473" t="n"/>
+      <c r="G4" s="1473" t="n"/>
+      <c r="H4" s="1473" t="n"/>
+      <c r="I4" s="1474" t="n"/>
+      <c r="J4" s="1475" t="n"/>
+      <c r="K4" s="1475" t="n"/>
+      <c r="L4" s="1475" t="n"/>
+      <c r="M4" s="1473" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1437" t="n">
+      <c r="N4" s="1473" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1437" t="n"/>
-      <c r="P4" s="1440" t="n"/>
-      <c r="Q4" s="1437" t="n"/>
-      <c r="R4" s="1437" t="n"/>
-      <c r="S4" s="1437" t="n"/>
+      <c r="O4" s="1473" t="n"/>
+      <c r="P4" s="1476" t="n"/>
+      <c r="Q4" s="1473" t="n"/>
+      <c r="R4" s="1473" t="n"/>
+      <c r="S4" s="1473" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1436" t="n"/>
+      <c r="U4" s="1472" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -5440,57 +5548,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1441" t="inlineStr">
+      <c r="A5" s="1477" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1442" t="inlineStr">
+      <c r="B5" s="1478" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1442" t="inlineStr">
+      <c r="C5" s="1478" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1443" t="n">
+      <c r="D5" s="1479" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1443" t="n">
+      <c r="E5" s="1479" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1443" t="n">
+      <c r="F5" s="1479" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1443" t="n"/>
-      <c r="H5" s="1443" t="n"/>
-      <c r="I5" s="1444" t="n"/>
-      <c r="J5" s="1445" t="n">
+      <c r="G5" s="1479" t="n"/>
+      <c r="H5" s="1479" t="n"/>
+      <c r="I5" s="1480" t="n"/>
+      <c r="J5" s="1481" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1445" t="n">
+      <c r="K5" s="1481" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1445" t="inlineStr">
+      <c r="L5" s="1481" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1443" t="n"/>
-      <c r="N5" s="1443" t="n"/>
-      <c r="O5" s="1443" t="n">
+      <c r="M5" s="1479" t="n"/>
+      <c r="N5" s="1479" t="n"/>
+      <c r="O5" s="1479" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1446" t="n">
+      <c r="P5" s="1482" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1443" t="n"/>
-      <c r="R5" s="1443" t="n"/>
-      <c r="S5" s="1443" t="n"/>
+      <c r="Q5" s="1479" t="n"/>
+      <c r="R5" s="1479" t="n"/>
+      <c r="S5" s="1479" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1442" t="n"/>
+      <c r="U5" s="1478" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -5498,43 +5606,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1447" t="inlineStr">
+      <c r="A6" s="1483" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1448" t="inlineStr">
+      <c r="B6" s="1484" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1448" t="inlineStr">
+      <c r="C6" s="1484" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1449" t="n"/>
-      <c r="E6" s="1449" t="n"/>
-      <c r="F6" s="1449" t="n"/>
-      <c r="G6" s="1449" t="n"/>
-      <c r="H6" s="1449" t="n"/>
-      <c r="I6" s="1450" t="n"/>
-      <c r="J6" s="1451" t="n"/>
-      <c r="K6" s="1451" t="n"/>
-      <c r="L6" s="1451" t="n"/>
-      <c r="M6" s="1449" t="n">
+      <c r="D6" s="1485" t="n"/>
+      <c r="E6" s="1485" t="n"/>
+      <c r="F6" s="1485" t="n"/>
+      <c r="G6" s="1485" t="n"/>
+      <c r="H6" s="1485" t="n"/>
+      <c r="I6" s="1486" t="n"/>
+      <c r="J6" s="1487" t="n"/>
+      <c r="K6" s="1487" t="n"/>
+      <c r="L6" s="1487" t="n"/>
+      <c r="M6" s="1485" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1449" t="n">
+      <c r="N6" s="1485" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1449" t="n"/>
-      <c r="P6" s="1452" t="n"/>
-      <c r="Q6" s="1449" t="n"/>
-      <c r="R6" s="1449" t="n"/>
-      <c r="S6" s="1449" t="n"/>
+      <c r="O6" s="1485" t="n"/>
+      <c r="P6" s="1488" t="n"/>
+      <c r="Q6" s="1485" t="n"/>
+      <c r="R6" s="1485" t="n"/>
+      <c r="S6" s="1485" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1448" t="n"/>
+      <c r="U6" s="1484" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -5542,39 +5650,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1453" t="inlineStr">
+      <c r="A7" s="1489" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1454" t="inlineStr">
+      <c r="B7" s="1490" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1454" t="inlineStr">
+      <c r="C7" s="1490" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1455" t="n"/>
-      <c r="E7" s="1455" t="n"/>
-      <c r="F7" s="1455" t="n"/>
-      <c r="G7" s="1455" t="n"/>
-      <c r="H7" s="1455" t="n"/>
-      <c r="I7" s="1456" t="n"/>
-      <c r="J7" s="1457" t="n"/>
-      <c r="K7" s="1457" t="n"/>
-      <c r="L7" s="1457" t="n"/>
-      <c r="M7" s="1455" t="n"/>
-      <c r="N7" s="1455" t="n"/>
-      <c r="O7" s="1455" t="n"/>
-      <c r="P7" s="1458" t="n"/>
-      <c r="Q7" s="1455" t="n"/>
-      <c r="R7" s="1455" t="n"/>
-      <c r="S7" s="1455" t="n"/>
+      <c r="D7" s="1491" t="n"/>
+      <c r="E7" s="1491" t="n"/>
+      <c r="F7" s="1491" t="n"/>
+      <c r="G7" s="1491" t="n"/>
+      <c r="H7" s="1491" t="n"/>
+      <c r="I7" s="1492" t="n"/>
+      <c r="J7" s="1493" t="n"/>
+      <c r="K7" s="1493" t="n"/>
+      <c r="L7" s="1493" t="n"/>
+      <c r="M7" s="1491" t="n"/>
+      <c r="N7" s="1491" t="n"/>
+      <c r="O7" s="1491" t="n"/>
+      <c r="P7" s="1494" t="n"/>
+      <c r="Q7" s="1491" t="n"/>
+      <c r="R7" s="1491" t="n"/>
+      <c r="S7" s="1491" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1454" t="n"/>
+      <c r="U7" s="1490" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5582,39 +5690,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1429" t="inlineStr">
+      <c r="A8" s="1465" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1430" t="inlineStr">
+      <c r="B8" s="1466" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1430" t="inlineStr">
+      <c r="C8" s="1466" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1431" t="n"/>
-      <c r="E8" s="1431" t="n"/>
-      <c r="F8" s="1431" t="n"/>
-      <c r="G8" s="1431" t="n"/>
-      <c r="H8" s="1431" t="n"/>
-      <c r="I8" s="1432" t="n"/>
-      <c r="J8" s="1433" t="n"/>
-      <c r="K8" s="1433" t="n"/>
-      <c r="L8" s="1433" t="n"/>
-      <c r="M8" s="1431" t="n"/>
-      <c r="N8" s="1431" t="n"/>
-      <c r="O8" s="1431" t="n"/>
-      <c r="P8" s="1434" t="n"/>
-      <c r="Q8" s="1431" t="n"/>
-      <c r="R8" s="1431" t="n"/>
-      <c r="S8" s="1431" t="n"/>
+      <c r="D8" s="1467" t="n"/>
+      <c r="E8" s="1467" t="n"/>
+      <c r="F8" s="1467" t="n"/>
+      <c r="G8" s="1467" t="n"/>
+      <c r="H8" s="1467" t="n"/>
+      <c r="I8" s="1468" t="n"/>
+      <c r="J8" s="1469" t="n"/>
+      <c r="K8" s="1469" t="n"/>
+      <c r="L8" s="1469" t="n"/>
+      <c r="M8" s="1467" t="n"/>
+      <c r="N8" s="1467" t="n"/>
+      <c r="O8" s="1467" t="n"/>
+      <c r="P8" s="1470" t="n"/>
+      <c r="Q8" s="1467" t="n"/>
+      <c r="R8" s="1467" t="n"/>
+      <c r="S8" s="1467" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1430" t="n"/>
+      <c r="U8" s="1466" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -5622,63 +5730,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1459" t="inlineStr">
+      <c r="A9" s="1495" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1460" t="inlineStr">
+      <c r="B9" s="1496" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1460" t="inlineStr">
+      <c r="C9" s="1496" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1461" t="n">
+      <c r="D9" s="1497" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1461" t="n">
+      <c r="E9" s="1497" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1461" t="n">
+      <c r="F9" s="1497" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1461" t="n">
+      <c r="G9" s="1497" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1461" t="n"/>
-      <c r="I9" s="1462" t="n"/>
-      <c r="J9" s="1463" t="n">
+      <c r="H9" s="1497" t="n"/>
+      <c r="I9" s="1498" t="n"/>
+      <c r="J9" s="1499" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1463" t="n">
+      <c r="K9" s="1499" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1463" t="inlineStr">
+      <c r="L9" s="1499" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1461" t="n"/>
-      <c r="N9" s="1461" t="n"/>
-      <c r="O9" s="1461" t="n">
+      <c r="M9" s="1497" t="n"/>
+      <c r="N9" s="1497" t="n"/>
+      <c r="O9" s="1497" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1464" t="n">
+      <c r="P9" s="1500" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1461" t="n"/>
-      <c r="R9" s="1461" t="n"/>
-      <c r="S9" s="1461" t="n"/>
+      <c r="Q9" s="1497" t="n"/>
+      <c r="R9" s="1497" t="n"/>
+      <c r="S9" s="1497" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1460" t="n"/>
+      <c r="U9" s="1496" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -5686,43 +5794,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1459" t="inlineStr">
+      <c r="A10" s="1495" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1460" t="inlineStr">
+      <c r="B10" s="1496" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1460" t="inlineStr">
+      <c r="C10" s="1496" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1461" t="n"/>
-      <c r="E10" s="1461" t="n"/>
-      <c r="F10" s="1461" t="n"/>
-      <c r="G10" s="1461" t="n"/>
-      <c r="H10" s="1461" t="n"/>
-      <c r="I10" s="1462" t="n"/>
-      <c r="J10" s="1463" t="n"/>
-      <c r="K10" s="1463" t="n"/>
-      <c r="L10" s="1463" t="inlineStr">
+      <c r="D10" s="1497" t="n"/>
+      <c r="E10" s="1497" t="n"/>
+      <c r="F10" s="1497" t="n"/>
+      <c r="G10" s="1497" t="n"/>
+      <c r="H10" s="1497" t="n"/>
+      <c r="I10" s="1498" t="n"/>
+      <c r="J10" s="1499" t="n"/>
+      <c r="K10" s="1499" t="n"/>
+      <c r="L10" s="1499" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1461" t="n"/>
-      <c r="N10" s="1461" t="n"/>
-      <c r="O10" s="1461" t="n"/>
-      <c r="P10" s="1464" t="n"/>
-      <c r="Q10" s="1461" t="n"/>
-      <c r="R10" s="1461" t="n"/>
-      <c r="S10" s="1461" t="n"/>
+      <c r="M10" s="1497" t="n"/>
+      <c r="N10" s="1497" t="n"/>
+      <c r="O10" s="1497" t="n"/>
+      <c r="P10" s="1500" t="n"/>
+      <c r="Q10" s="1497" t="n"/>
+      <c r="R10" s="1497" t="n"/>
+      <c r="S10" s="1497" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1460" t="n"/>
+      <c r="U10" s="1496" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -5730,43 +5838,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1459" t="inlineStr">
+      <c r="A11" s="1495" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1460" t="inlineStr">
+      <c r="B11" s="1496" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1460" t="inlineStr">
+      <c r="C11" s="1496" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1461" t="n"/>
-      <c r="E11" s="1461" t="n"/>
-      <c r="F11" s="1461" t="n"/>
-      <c r="G11" s="1461" t="n"/>
-      <c r="H11" s="1461" t="n"/>
-      <c r="I11" s="1462" t="n"/>
-      <c r="J11" s="1463" t="n"/>
-      <c r="K11" s="1463" t="n"/>
-      <c r="L11" s="1463" t="n"/>
-      <c r="M11" s="1461" t="n">
+      <c r="D11" s="1497" t="n"/>
+      <c r="E11" s="1497" t="n"/>
+      <c r="F11" s="1497" t="n"/>
+      <c r="G11" s="1497" t="n"/>
+      <c r="H11" s="1497" t="n"/>
+      <c r="I11" s="1498" t="n"/>
+      <c r="J11" s="1499" t="n"/>
+      <c r="K11" s="1499" t="n"/>
+      <c r="L11" s="1499" t="n"/>
+      <c r="M11" s="1497" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1461" t="n">
+      <c r="N11" s="1497" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1461" t="n"/>
-      <c r="P11" s="1464" t="n"/>
-      <c r="Q11" s="1461" t="n"/>
-      <c r="R11" s="1461" t="n"/>
-      <c r="S11" s="1461" t="n"/>
+      <c r="O11" s="1497" t="n"/>
+      <c r="P11" s="1500" t="n"/>
+      <c r="Q11" s="1497" t="n"/>
+      <c r="R11" s="1497" t="n"/>
+      <c r="S11" s="1497" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1460" t="n"/>
+      <c r="U11" s="1496" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -5774,39 +5882,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1435" t="inlineStr">
+      <c r="A12" s="1471" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1436" t="inlineStr">
+      <c r="B12" s="1472" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1436" t="inlineStr">
+      <c r="C12" s="1472" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1437" t="n"/>
-      <c r="E12" s="1437" t="n"/>
-      <c r="F12" s="1437" t="n"/>
-      <c r="G12" s="1437" t="n"/>
-      <c r="H12" s="1437" t="n"/>
-      <c r="I12" s="1438" t="n"/>
-      <c r="J12" s="1439" t="n"/>
-      <c r="K12" s="1439" t="n"/>
-      <c r="L12" s="1439" t="n"/>
-      <c r="M12" s="1437" t="n"/>
-      <c r="N12" s="1437" t="n"/>
-      <c r="O12" s="1437" t="n"/>
-      <c r="P12" s="1440" t="n"/>
-      <c r="Q12" s="1437" t="n"/>
-      <c r="R12" s="1437" t="n"/>
-      <c r="S12" s="1437" t="n"/>
+      <c r="D12" s="1473" t="n"/>
+      <c r="E12" s="1473" t="n"/>
+      <c r="F12" s="1473" t="n"/>
+      <c r="G12" s="1473" t="n"/>
+      <c r="H12" s="1473" t="n"/>
+      <c r="I12" s="1474" t="n"/>
+      <c r="J12" s="1475" t="n"/>
+      <c r="K12" s="1475" t="n"/>
+      <c r="L12" s="1475" t="n"/>
+      <c r="M12" s="1473" t="n"/>
+      <c r="N12" s="1473" t="n"/>
+      <c r="O12" s="1473" t="n"/>
+      <c r="P12" s="1476" t="n"/>
+      <c r="Q12" s="1473" t="n"/>
+      <c r="R12" s="1473" t="n"/>
+      <c r="S12" s="1473" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1436" t="n"/>
+      <c r="U12" s="1472" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5814,35 +5922,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1441" t="inlineStr">
+      <c r="A13" s="1477" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1442" t="n"/>
-      <c r="C13" s="1442" t="inlineStr">
+      <c r="B13" s="1478" t="n"/>
+      <c r="C13" s="1478" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1443" t="n"/>
-      <c r="E13" s="1443" t="n"/>
-      <c r="F13" s="1443" t="n"/>
-      <c r="G13" s="1443" t="n"/>
-      <c r="H13" s="1443" t="n"/>
-      <c r="I13" s="1444" t="n"/>
-      <c r="J13" s="1445" t="n"/>
-      <c r="K13" s="1445" t="n"/>
-      <c r="L13" s="1445" t="n"/>
-      <c r="M13" s="1443" t="n"/>
-      <c r="N13" s="1443" t="n"/>
-      <c r="O13" s="1443" t="n"/>
-      <c r="P13" s="1446" t="n"/>
-      <c r="Q13" s="1443" t="n"/>
-      <c r="R13" s="1443" t="n"/>
-      <c r="S13" s="1443" t="n"/>
+      <c r="D13" s="1479" t="n"/>
+      <c r="E13" s="1479" t="n"/>
+      <c r="F13" s="1479" t="n"/>
+      <c r="G13" s="1479" t="n"/>
+      <c r="H13" s="1479" t="n"/>
+      <c r="I13" s="1480" t="n"/>
+      <c r="J13" s="1481" t="n"/>
+      <c r="K13" s="1481" t="n"/>
+      <c r="L13" s="1481" t="n"/>
+      <c r="M13" s="1479" t="n"/>
+      <c r="N13" s="1479" t="n"/>
+      <c r="O13" s="1479" t="n"/>
+      <c r="P13" s="1482" t="n"/>
+      <c r="Q13" s="1479" t="n"/>
+      <c r="R13" s="1479" t="n"/>
+      <c r="S13" s="1479" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1442" t="n"/>
+      <c r="U13" s="1478" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -5850,53 +5958,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1447" t="inlineStr">
+      <c r="A14" s="1483" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1448" t="inlineStr">
+      <c r="B14" s="1484" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1448" t="inlineStr">
+      <c r="C14" s="1484" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1449" t="n"/>
-      <c r="E14" s="1449" t="n">
+      <c r="D14" s="1485" t="n"/>
+      <c r="E14" s="1485" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1449" t="n">
+      <c r="F14" s="1485" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1449" t="n">
+      <c r="G14" s="1485" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1449" t="n"/>
-      <c r="I14" s="1450" t="n"/>
-      <c r="J14" s="1451" t="n"/>
-      <c r="K14" s="1451" t="n"/>
-      <c r="L14" s="1451" t="n"/>
-      <c r="M14" s="1449" t="n"/>
-      <c r="N14" s="1449" t="n"/>
-      <c r="O14" s="1449" t="n">
+      <c r="H14" s="1485" t="n"/>
+      <c r="I14" s="1486" t="n"/>
+      <c r="J14" s="1487" t="n"/>
+      <c r="K14" s="1487" t="n"/>
+      <c r="L14" s="1487" t="n"/>
+      <c r="M14" s="1485" t="n"/>
+      <c r="N14" s="1485" t="n"/>
+      <c r="O14" s="1485" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1452" t="n">
+      <c r="P14" s="1488" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1449" t="n"/>
-      <c r="R14" s="1449" t="n"/>
-      <c r="S14" s="1449" t="n"/>
+      <c r="Q14" s="1485" t="n"/>
+      <c r="R14" s="1485" t="n"/>
+      <c r="S14" s="1485" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1448" t="n"/>
+      <c r="U14" s="1484" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -5904,43 +6012,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1447" t="inlineStr">
+      <c r="A15" s="1483" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1448" t="inlineStr">
+      <c r="B15" s="1484" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1448" t="inlineStr">
+      <c r="C15" s="1484" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1449" t="n"/>
-      <c r="E15" s="1449" t="n"/>
-      <c r="F15" s="1449" t="n"/>
-      <c r="G15" s="1449" t="n"/>
-      <c r="H15" s="1449" t="n"/>
-      <c r="I15" s="1450" t="n"/>
-      <c r="J15" s="1451" t="n"/>
-      <c r="K15" s="1451" t="n"/>
-      <c r="L15" s="1451" t="n"/>
-      <c r="M15" s="1449" t="n">
+      <c r="D15" s="1485" t="n"/>
+      <c r="E15" s="1485" t="n"/>
+      <c r="F15" s="1485" t="n"/>
+      <c r="G15" s="1485" t="n"/>
+      <c r="H15" s="1485" t="n"/>
+      <c r="I15" s="1486" t="n"/>
+      <c r="J15" s="1487" t="n"/>
+      <c r="K15" s="1487" t="n"/>
+      <c r="L15" s="1487" t="n"/>
+      <c r="M15" s="1485" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1449" t="n">
+      <c r="N15" s="1485" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1449" t="n"/>
-      <c r="P15" s="1452" t="n"/>
-      <c r="Q15" s="1449" t="n"/>
-      <c r="R15" s="1449" t="n"/>
-      <c r="S15" s="1449" t="n"/>
+      <c r="O15" s="1485" t="n"/>
+      <c r="P15" s="1488" t="n"/>
+      <c r="Q15" s="1485" t="n"/>
+      <c r="R15" s="1485" t="n"/>
+      <c r="S15" s="1485" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1448" t="n"/>
+      <c r="U15" s="1484" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -5948,39 +6056,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1453" t="inlineStr">
+      <c r="A16" s="1489" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1454" t="inlineStr">
+      <c r="B16" s="1490" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1454" t="inlineStr">
+      <c r="C16" s="1490" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1455" t="n"/>
-      <c r="E16" s="1455" t="n"/>
-      <c r="F16" s="1455" t="n"/>
-      <c r="G16" s="1455" t="n"/>
-      <c r="H16" s="1455" t="n"/>
-      <c r="I16" s="1456" t="n"/>
-      <c r="J16" s="1457" t="n"/>
-      <c r="K16" s="1457" t="n"/>
-      <c r="L16" s="1457" t="n"/>
-      <c r="M16" s="1455" t="n"/>
-      <c r="N16" s="1455" t="n"/>
-      <c r="O16" s="1455" t="n"/>
-      <c r="P16" s="1458" t="n"/>
-      <c r="Q16" s="1455" t="n"/>
-      <c r="R16" s="1455" t="n"/>
-      <c r="S16" s="1455" t="n"/>
+      <c r="D16" s="1491" t="n"/>
+      <c r="E16" s="1491" t="n"/>
+      <c r="F16" s="1491" t="n"/>
+      <c r="G16" s="1491" t="n"/>
+      <c r="H16" s="1491" t="n"/>
+      <c r="I16" s="1492" t="n"/>
+      <c r="J16" s="1493" t="n"/>
+      <c r="K16" s="1493" t="n"/>
+      <c r="L16" s="1493" t="n"/>
+      <c r="M16" s="1491" t="n"/>
+      <c r="N16" s="1491" t="n"/>
+      <c r="O16" s="1491" t="n"/>
+      <c r="P16" s="1494" t="n"/>
+      <c r="Q16" s="1491" t="n"/>
+      <c r="R16" s="1491" t="n"/>
+      <c r="S16" s="1491" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1454" t="n"/>
+      <c r="U16" s="1490" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -5988,39 +6096,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1429" t="inlineStr">
+      <c r="A17" s="1465" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1430" t="inlineStr">
+      <c r="B17" s="1466" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1430" t="inlineStr">
+      <c r="C17" s="1466" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1431" t="n"/>
-      <c r="E17" s="1431" t="n"/>
-      <c r="F17" s="1431" t="n"/>
-      <c r="G17" s="1431" t="n"/>
-      <c r="H17" s="1431" t="n"/>
-      <c r="I17" s="1432" t="n"/>
-      <c r="J17" s="1433" t="n"/>
-      <c r="K17" s="1433" t="n"/>
-      <c r="L17" s="1433" t="n"/>
-      <c r="M17" s="1431" t="n"/>
-      <c r="N17" s="1431" t="n"/>
-      <c r="O17" s="1431" t="n"/>
-      <c r="P17" s="1434" t="n"/>
-      <c r="Q17" s="1431" t="n"/>
-      <c r="R17" s="1431" t="n"/>
-      <c r="S17" s="1431" t="n"/>
+      <c r="D17" s="1467" t="n"/>
+      <c r="E17" s="1467" t="n"/>
+      <c r="F17" s="1467" t="n"/>
+      <c r="G17" s="1467" t="n"/>
+      <c r="H17" s="1467" t="n"/>
+      <c r="I17" s="1468" t="n"/>
+      <c r="J17" s="1469" t="n"/>
+      <c r="K17" s="1469" t="n"/>
+      <c r="L17" s="1469" t="n"/>
+      <c r="M17" s="1467" t="n"/>
+      <c r="N17" s="1467" t="n"/>
+      <c r="O17" s="1467" t="n"/>
+      <c r="P17" s="1470" t="n"/>
+      <c r="Q17" s="1467" t="n"/>
+      <c r="R17" s="1467" t="n"/>
+      <c r="S17" s="1467" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1430" t="n"/>
+      <c r="U17" s="1466" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -6028,53 +6136,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1459" t="inlineStr">
+      <c r="A18" s="1495" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1460" t="inlineStr">
+      <c r="B18" s="1496" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1460" t="inlineStr">
+      <c r="C18" s="1496" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1461" t="n"/>
-      <c r="E18" s="1461" t="n">
+      <c r="D18" s="1497" t="n"/>
+      <c r="E18" s="1497" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1461" t="n">
+      <c r="F18" s="1497" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1461" t="n">
+      <c r="G18" s="1497" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1461" t="n"/>
-      <c r="I18" s="1462" t="n"/>
-      <c r="J18" s="1463" t="n"/>
-      <c r="K18" s="1463" t="n"/>
-      <c r="L18" s="1463" t="n"/>
-      <c r="M18" s="1461" t="n"/>
-      <c r="N18" s="1461" t="n"/>
-      <c r="O18" s="1461" t="n">
+      <c r="H18" s="1497" t="n"/>
+      <c r="I18" s="1498" t="n"/>
+      <c r="J18" s="1499" t="n"/>
+      <c r="K18" s="1499" t="n"/>
+      <c r="L18" s="1499" t="n"/>
+      <c r="M18" s="1497" t="n"/>
+      <c r="N18" s="1497" t="n"/>
+      <c r="O18" s="1497" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1464" t="n">
+      <c r="P18" s="1500" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1461" t="n"/>
-      <c r="R18" s="1461" t="n"/>
-      <c r="S18" s="1461" t="n"/>
+      <c r="Q18" s="1497" t="n"/>
+      <c r="R18" s="1497" t="n"/>
+      <c r="S18" s="1497" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1460" t="n"/>
+      <c r="U18" s="1496" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -6082,47 +6190,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1459" t="inlineStr">
+      <c r="A19" s="1495" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1460" t="inlineStr">
+      <c r="B19" s="1496" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1460" t="inlineStr">
+      <c r="C19" s="1496" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1461" t="n"/>
-      <c r="E19" s="1461" t="n"/>
-      <c r="F19" s="1461" t="n"/>
-      <c r="G19" s="1461" t="n"/>
-      <c r="H19" s="1461" t="n"/>
-      <c r="I19" s="1462" t="n"/>
-      <c r="J19" s="1463" t="n"/>
-      <c r="K19" s="1463" t="n"/>
-      <c r="L19" s="1463" t="n"/>
-      <c r="M19" s="1461" t="n">
+      <c r="D19" s="1497" t="n"/>
+      <c r="E19" s="1497" t="n"/>
+      <c r="F19" s="1497" t="n"/>
+      <c r="G19" s="1497" t="n"/>
+      <c r="H19" s="1497" t="n"/>
+      <c r="I19" s="1498" t="n"/>
+      <c r="J19" s="1499" t="n"/>
+      <c r="K19" s="1499" t="n"/>
+      <c r="L19" s="1499" t="n"/>
+      <c r="M19" s="1497" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1461" t="n">
+      <c r="N19" s="1497" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1461" t="n"/>
-      <c r="P19" s="1464" t="n"/>
-      <c r="Q19" s="1461" t="n"/>
-      <c r="R19" s="1461" t="n"/>
-      <c r="S19" s="1461" t="n"/>
+      <c r="O19" s="1497" t="n"/>
+      <c r="P19" s="1500" t="n"/>
+      <c r="Q19" s="1497" t="n"/>
+      <c r="R19" s="1497" t="n"/>
+      <c r="S19" s="1497" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1460" t="n"/>
+      <c r="U19" s="1496" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -6130,43 +6238,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1459" t="inlineStr">
+      <c r="A20" s="1495" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1460" t="inlineStr">
+      <c r="B20" s="1496" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1460" t="inlineStr">
+      <c r="C20" s="1496" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1461" t="n"/>
-      <c r="E20" s="1461" t="n"/>
-      <c r="F20" s="1461" t="n"/>
-      <c r="G20" s="1461" t="n"/>
-      <c r="H20" s="1461" t="n"/>
-      <c r="I20" s="1462" t="n"/>
-      <c r="J20" s="1463" t="n"/>
-      <c r="K20" s="1463" t="n"/>
-      <c r="L20" s="1463" t="n"/>
-      <c r="M20" s="1461" t="n"/>
-      <c r="N20" s="1461" t="n"/>
-      <c r="O20" s="1461" t="n"/>
-      <c r="P20" s="1464" t="n"/>
-      <c r="Q20" s="1461" t="n"/>
-      <c r="R20" s="1461" t="n"/>
-      <c r="S20" s="1461" t="n"/>
+      <c r="D20" s="1497" t="n"/>
+      <c r="E20" s="1497" t="n"/>
+      <c r="F20" s="1497" t="n"/>
+      <c r="G20" s="1497" t="n"/>
+      <c r="H20" s="1497" t="n"/>
+      <c r="I20" s="1498" t="n"/>
+      <c r="J20" s="1499" t="n"/>
+      <c r="K20" s="1499" t="n"/>
+      <c r="L20" s="1499" t="n"/>
+      <c r="M20" s="1497" t="n"/>
+      <c r="N20" s="1497" t="n"/>
+      <c r="O20" s="1497" t="n"/>
+      <c r="P20" s="1500" t="n"/>
+      <c r="Q20" s="1497" t="n"/>
+      <c r="R20" s="1497" t="n"/>
+      <c r="S20" s="1497" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1460" t="n"/>
+      <c r="U20" s="1496" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -6174,39 +6282,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1435" t="inlineStr">
+      <c r="A21" s="1471" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1436" t="inlineStr">
+      <c r="B21" s="1472" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1436" t="inlineStr">
+      <c r="C21" s="1472" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1437" t="n"/>
-      <c r="E21" s="1437" t="n"/>
-      <c r="F21" s="1437" t="n"/>
-      <c r="G21" s="1437" t="n"/>
-      <c r="H21" s="1437" t="n"/>
-      <c r="I21" s="1438" t="n"/>
-      <c r="J21" s="1439" t="n"/>
-      <c r="K21" s="1439" t="n"/>
-      <c r="L21" s="1439" t="n"/>
-      <c r="M21" s="1437" t="n"/>
-      <c r="N21" s="1437" t="n"/>
-      <c r="O21" s="1437" t="n"/>
-      <c r="P21" s="1440" t="n"/>
-      <c r="Q21" s="1437" t="n"/>
-      <c r="R21" s="1437" t="n"/>
-      <c r="S21" s="1437" t="n"/>
+      <c r="D21" s="1473" t="n"/>
+      <c r="E21" s="1473" t="n"/>
+      <c r="F21" s="1473" t="n"/>
+      <c r="G21" s="1473" t="n"/>
+      <c r="H21" s="1473" t="n"/>
+      <c r="I21" s="1474" t="n"/>
+      <c r="J21" s="1475" t="n"/>
+      <c r="K21" s="1475" t="n"/>
+      <c r="L21" s="1475" t="n"/>
+      <c r="M21" s="1473" t="n"/>
+      <c r="N21" s="1473" t="n"/>
+      <c r="O21" s="1473" t="n"/>
+      <c r="P21" s="1476" t="n"/>
+      <c r="Q21" s="1473" t="n"/>
+      <c r="R21" s="1473" t="n"/>
+      <c r="S21" s="1473" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1436" t="n"/>
+      <c r="U21" s="1472" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -6214,39 +6322,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1441" t="inlineStr">
+      <c r="A22" s="1477" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1442" t="inlineStr">
+      <c r="B22" s="1478" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1442" t="inlineStr">
+      <c r="C22" s="1478" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1443" t="n"/>
-      <c r="E22" s="1443" t="n"/>
-      <c r="F22" s="1443" t="n"/>
-      <c r="G22" s="1443" t="n"/>
-      <c r="H22" s="1443" t="n"/>
-      <c r="I22" s="1444" t="n"/>
-      <c r="J22" s="1445" t="n"/>
-      <c r="K22" s="1445" t="n"/>
-      <c r="L22" s="1445" t="n"/>
-      <c r="M22" s="1443" t="n"/>
-      <c r="N22" s="1443" t="n"/>
-      <c r="O22" s="1443" t="n"/>
-      <c r="P22" s="1446" t="n"/>
-      <c r="Q22" s="1443" t="n"/>
-      <c r="R22" s="1443" t="n"/>
-      <c r="S22" s="1443" t="n"/>
+      <c r="D22" s="1479" t="n"/>
+      <c r="E22" s="1479" t="n"/>
+      <c r="F22" s="1479" t="n"/>
+      <c r="G22" s="1479" t="n"/>
+      <c r="H22" s="1479" t="n"/>
+      <c r="I22" s="1480" t="n"/>
+      <c r="J22" s="1481" t="n"/>
+      <c r="K22" s="1481" t="n"/>
+      <c r="L22" s="1481" t="n"/>
+      <c r="M22" s="1479" t="n"/>
+      <c r="N22" s="1479" t="n"/>
+      <c r="O22" s="1479" t="n"/>
+      <c r="P22" s="1482" t="n"/>
+      <c r="Q22" s="1479" t="n"/>
+      <c r="R22" s="1479" t="n"/>
+      <c r="S22" s="1479" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1442" t="n"/>
+      <c r="U22" s="1478" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -6254,53 +6362,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1447" t="inlineStr">
+      <c r="A23" s="1483" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1448" t="inlineStr">
+      <c r="B23" s="1484" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1448" t="inlineStr">
+      <c r="C23" s="1484" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1449" t="n"/>
-      <c r="E23" s="1449" t="n">
+      <c r="D23" s="1485" t="n"/>
+      <c r="E23" s="1485" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1449" t="n">
+      <c r="F23" s="1485" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1449" t="n">
+      <c r="G23" s="1485" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1449" t="n"/>
-      <c r="I23" s="1450" t="n"/>
-      <c r="J23" s="1451" t="n"/>
-      <c r="K23" s="1451" t="n"/>
-      <c r="L23" s="1451" t="n"/>
-      <c r="M23" s="1449" t="n"/>
-      <c r="N23" s="1449" t="n"/>
-      <c r="O23" s="1449" t="n">
+      <c r="H23" s="1485" t="n"/>
+      <c r="I23" s="1486" t="n"/>
+      <c r="J23" s="1487" t="n"/>
+      <c r="K23" s="1487" t="n"/>
+      <c r="L23" s="1487" t="n"/>
+      <c r="M23" s="1485" t="n"/>
+      <c r="N23" s="1485" t="n"/>
+      <c r="O23" s="1485" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1452" t="n">
+      <c r="P23" s="1488" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1449" t="n"/>
-      <c r="R23" s="1449" t="n"/>
-      <c r="S23" s="1449" t="n"/>
+      <c r="Q23" s="1485" t="n"/>
+      <c r="R23" s="1485" t="n"/>
+      <c r="S23" s="1485" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1448" t="n"/>
+      <c r="U23" s="1484" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -6308,47 +6416,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1453" t="inlineStr">
+      <c r="A24" s="1489" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1454" t="inlineStr">
+      <c r="B24" s="1490" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1454" t="inlineStr">
+      <c r="C24" s="1490" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1455" t="n"/>
-      <c r="E24" s="1455" t="n"/>
-      <c r="F24" s="1455" t="n"/>
-      <c r="G24" s="1455" t="n"/>
-      <c r="H24" s="1455" t="n"/>
-      <c r="I24" s="1456" t="n"/>
-      <c r="J24" s="1457" t="n"/>
-      <c r="K24" s="1457" t="n"/>
-      <c r="L24" s="1457" t="n"/>
-      <c r="M24" s="1455" t="n">
+      <c r="D24" s="1491" t="n"/>
+      <c r="E24" s="1491" t="n"/>
+      <c r="F24" s="1491" t="n"/>
+      <c r="G24" s="1491" t="n"/>
+      <c r="H24" s="1491" t="n"/>
+      <c r="I24" s="1492" t="n"/>
+      <c r="J24" s="1493" t="n"/>
+      <c r="K24" s="1493" t="n"/>
+      <c r="L24" s="1493" t="n"/>
+      <c r="M24" s="1491" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1455" t="n">
+      <c r="N24" s="1491" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1455" t="n"/>
-      <c r="P24" s="1458" t="n"/>
-      <c r="Q24" s="1455" t="n"/>
-      <c r="R24" s="1455" t="n"/>
-      <c r="S24" s="1455" t="n"/>
+      <c r="O24" s="1491" t="n"/>
+      <c r="P24" s="1494" t="n"/>
+      <c r="Q24" s="1491" t="n"/>
+      <c r="R24" s="1491" t="n"/>
+      <c r="S24" s="1491" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1454" t="n"/>
+      <c r="U24" s="1490" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -6356,61 +6464,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1429" t="inlineStr">
+      <c r="A25" s="1465" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1430" t="inlineStr">
+      <c r="B25" s="1466" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1430" t="inlineStr">
+      <c r="C25" s="1466" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1431" t="n">
+      <c r="D25" s="1467" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1431" t="n">
+      <c r="E25" s="1467" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1431" t="n">
+      <c r="F25" s="1467" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1431" t="n">
+      <c r="G25" s="1467" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1431" t="n"/>
-      <c r="I25" s="1432" t="n"/>
-      <c r="J25" s="1433" t="n">
+      <c r="H25" s="1467" t="n"/>
+      <c r="I25" s="1468" t="n"/>
+      <c r="J25" s="1469" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1433" t="n">
+      <c r="K25" s="1469" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1433" t="n">
+      <c r="L25" s="1469" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1431" t="n"/>
-      <c r="N25" s="1431" t="n"/>
-      <c r="O25" s="1431" t="n">
+      <c r="M25" s="1467" t="n"/>
+      <c r="N25" s="1467" t="n"/>
+      <c r="O25" s="1467" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1434" t="n">
+      <c r="P25" s="1470" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1431" t="n"/>
-      <c r="R25" s="1431" t="n"/>
-      <c r="S25" s="1431" t="n"/>
+      <c r="Q25" s="1467" t="n"/>
+      <c r="R25" s="1467" t="n"/>
+      <c r="S25" s="1467" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1430" t="n"/>
+      <c r="U25" s="1466" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -6418,47 +6526,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1435" t="inlineStr">
+      <c r="A26" s="1471" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1436" t="inlineStr">
+      <c r="B26" s="1472" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1436" t="inlineStr">
+      <c r="C26" s="1472" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1437" t="n"/>
-      <c r="E26" s="1437" t="n"/>
-      <c r="F26" s="1437" t="n"/>
-      <c r="G26" s="1437" t="n"/>
-      <c r="H26" s="1437" t="n"/>
-      <c r="I26" s="1438" t="n"/>
-      <c r="J26" s="1439" t="n"/>
-      <c r="K26" s="1439" t="n"/>
-      <c r="L26" s="1439" t="n"/>
-      <c r="M26" s="1437" t="n">
+      <c r="D26" s="1473" t="n"/>
+      <c r="E26" s="1473" t="n"/>
+      <c r="F26" s="1473" t="n"/>
+      <c r="G26" s="1473" t="n"/>
+      <c r="H26" s="1473" t="n"/>
+      <c r="I26" s="1474" t="n"/>
+      <c r="J26" s="1475" t="n"/>
+      <c r="K26" s="1475" t="n"/>
+      <c r="L26" s="1475" t="n"/>
+      <c r="M26" s="1473" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1437" t="n">
+      <c r="N26" s="1473" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1437" t="n"/>
-      <c r="P26" s="1440" t="n"/>
-      <c r="Q26" s="1437" t="n"/>
-      <c r="R26" s="1437" t="n"/>
-      <c r="S26" s="1437" t="n"/>
+      <c r="O26" s="1473" t="n"/>
+      <c r="P26" s="1476" t="n"/>
+      <c r="Q26" s="1473" t="n"/>
+      <c r="R26" s="1473" t="n"/>
+      <c r="S26" s="1473" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1436" t="n"/>
+      <c r="U26" s="1472" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -6466,53 +6574,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1441" t="inlineStr">
+      <c r="A27" s="1477" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1442" t="inlineStr">
+      <c r="B27" s="1478" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1442" t="inlineStr">
+      <c r="C27" s="1478" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1443" t="n"/>
-      <c r="E27" s="1443" t="n">
+      <c r="D27" s="1479" t="n"/>
+      <c r="E27" s="1479" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1443" t="n">
+      <c r="F27" s="1479" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1443" t="n">
+      <c r="G27" s="1479" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1443" t="n"/>
-      <c r="I27" s="1444" t="n"/>
-      <c r="J27" s="1445" t="n"/>
-      <c r="K27" s="1445" t="n"/>
-      <c r="L27" s="1445" t="n"/>
-      <c r="M27" s="1443" t="n"/>
-      <c r="N27" s="1443" t="n"/>
-      <c r="O27" s="1443" t="n">
+      <c r="H27" s="1479" t="n"/>
+      <c r="I27" s="1480" t="n"/>
+      <c r="J27" s="1481" t="n"/>
+      <c r="K27" s="1481" t="n"/>
+      <c r="L27" s="1481" t="n"/>
+      <c r="M27" s="1479" t="n"/>
+      <c r="N27" s="1479" t="n"/>
+      <c r="O27" s="1479" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1446" t="n">
+      <c r="P27" s="1482" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1443" t="n"/>
-      <c r="R27" s="1443" t="n"/>
-      <c r="S27" s="1443" t="n"/>
+      <c r="Q27" s="1479" t="n"/>
+      <c r="R27" s="1479" t="n"/>
+      <c r="S27" s="1479" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1442" t="n"/>
+      <c r="U27" s="1478" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -6520,47 +6628,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1453" t="inlineStr">
+      <c r="A28" s="1489" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1454" t="inlineStr">
+      <c r="B28" s="1490" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1454" t="inlineStr">
+      <c r="C28" s="1490" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1455" t="n"/>
-      <c r="E28" s="1455" t="n"/>
-      <c r="F28" s="1455" t="n"/>
-      <c r="G28" s="1455" t="n"/>
-      <c r="H28" s="1455" t="n"/>
-      <c r="I28" s="1456" t="n"/>
-      <c r="J28" s="1457" t="n"/>
-      <c r="K28" s="1457" t="n"/>
-      <c r="L28" s="1457" t="n"/>
-      <c r="M28" s="1455" t="n">
+      <c r="D28" s="1491" t="n"/>
+      <c r="E28" s="1491" t="n"/>
+      <c r="F28" s="1491" t="n"/>
+      <c r="G28" s="1491" t="n"/>
+      <c r="H28" s="1491" t="n"/>
+      <c r="I28" s="1492" t="n"/>
+      <c r="J28" s="1493" t="n"/>
+      <c r="K28" s="1493" t="n"/>
+      <c r="L28" s="1493" t="n"/>
+      <c r="M28" s="1491" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1455" t="n">
+      <c r="N28" s="1491" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1455" t="n"/>
-      <c r="P28" s="1458" t="n"/>
-      <c r="Q28" s="1455" t="n"/>
-      <c r="R28" s="1455" t="n"/>
-      <c r="S28" s="1455" t="n"/>
+      <c r="O28" s="1491" t="n"/>
+      <c r="P28" s="1494" t="n"/>
+      <c r="Q28" s="1491" t="n"/>
+      <c r="R28" s="1491" t="n"/>
+      <c r="S28" s="1491" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1454" t="n"/>
+      <c r="U28" s="1490" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -6568,53 +6676,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1429" t="inlineStr">
+      <c r="A29" s="1465" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1430" t="inlineStr">
+      <c r="B29" s="1466" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1430" t="inlineStr">
+      <c r="C29" s="1466" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1431" t="n"/>
-      <c r="E29" s="1431" t="n">
+      <c r="D29" s="1467" t="n"/>
+      <c r="E29" s="1467" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1431" t="n">
+      <c r="F29" s="1467" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1431" t="n">
+      <c r="G29" s="1467" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1431" t="n"/>
-      <c r="I29" s="1432" t="n"/>
-      <c r="J29" s="1433" t="n"/>
-      <c r="K29" s="1433" t="n"/>
-      <c r="L29" s="1433" t="n"/>
-      <c r="M29" s="1431" t="n"/>
-      <c r="N29" s="1431" t="n"/>
-      <c r="O29" s="1431" t="n">
+      <c r="H29" s="1467" t="n"/>
+      <c r="I29" s="1468" t="n"/>
+      <c r="J29" s="1469" t="n"/>
+      <c r="K29" s="1469" t="n"/>
+      <c r="L29" s="1469" t="n"/>
+      <c r="M29" s="1467" t="n"/>
+      <c r="N29" s="1467" t="n"/>
+      <c r="O29" s="1467" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1434" t="n">
+      <c r="P29" s="1470" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1431" t="n"/>
-      <c r="R29" s="1431" t="n"/>
-      <c r="S29" s="1431" t="n"/>
+      <c r="Q29" s="1467" t="n"/>
+      <c r="R29" s="1467" t="n"/>
+      <c r="S29" s="1467" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1430" t="n"/>
+      <c r="U29" s="1466" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -6622,43 +6730,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1435" t="inlineStr">
+      <c r="A30" s="1471" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1436" t="inlineStr">
+      <c r="B30" s="1472" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1436" t="inlineStr">
+      <c r="C30" s="1472" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1437" t="n"/>
-      <c r="E30" s="1437" t="n"/>
-      <c r="F30" s="1437" t="n"/>
-      <c r="G30" s="1437" t="n"/>
-      <c r="H30" s="1437" t="n"/>
-      <c r="I30" s="1438" t="n"/>
-      <c r="J30" s="1439" t="n"/>
-      <c r="K30" s="1439" t="n"/>
-      <c r="L30" s="1439" t="n"/>
-      <c r="M30" s="1437" t="n"/>
-      <c r="N30" s="1437" t="n"/>
-      <c r="O30" s="1437" t="n"/>
-      <c r="P30" s="1440" t="n"/>
-      <c r="Q30" s="1437" t="n"/>
-      <c r="R30" s="1437" t="n"/>
-      <c r="S30" s="1437" t="n"/>
+      <c r="D30" s="1473" t="n"/>
+      <c r="E30" s="1473" t="n"/>
+      <c r="F30" s="1473" t="n"/>
+      <c r="G30" s="1473" t="n"/>
+      <c r="H30" s="1473" t="n"/>
+      <c r="I30" s="1474" t="n"/>
+      <c r="J30" s="1475" t="n"/>
+      <c r="K30" s="1475" t="n"/>
+      <c r="L30" s="1475" t="n"/>
+      <c r="M30" s="1473" t="n"/>
+      <c r="N30" s="1473" t="n"/>
+      <c r="O30" s="1473" t="n"/>
+      <c r="P30" s="1476" t="n"/>
+      <c r="Q30" s="1473" t="n"/>
+      <c r="R30" s="1473" t="n"/>
+      <c r="S30" s="1473" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1436" t="n"/>
+      <c r="U30" s="1472" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -6666,53 +6774,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1441" t="inlineStr">
+      <c r="A31" s="1477" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1442" t="inlineStr">
+      <c r="B31" s="1478" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1442" t="inlineStr">
+      <c r="C31" s="1478" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1443" t="n"/>
-      <c r="E31" s="1443" t="n">
+      <c r="D31" s="1479" t="n"/>
+      <c r="E31" s="1479" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1443" t="n">
+      <c r="F31" s="1479" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1443" t="n">
+      <c r="G31" s="1479" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1443" t="n"/>
-      <c r="I31" s="1444" t="n"/>
-      <c r="J31" s="1445" t="n"/>
-      <c r="K31" s="1445" t="n"/>
-      <c r="L31" s="1445" t="n"/>
-      <c r="M31" s="1443" t="n"/>
-      <c r="N31" s="1443" t="n"/>
-      <c r="O31" s="1443" t="n">
+      <c r="H31" s="1479" t="n"/>
+      <c r="I31" s="1480" t="n"/>
+      <c r="J31" s="1481" t="n"/>
+      <c r="K31" s="1481" t="n"/>
+      <c r="L31" s="1481" t="n"/>
+      <c r="M31" s="1479" t="n"/>
+      <c r="N31" s="1479" t="n"/>
+      <c r="O31" s="1479" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1446" t="n">
+      <c r="P31" s="1482" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1443" t="n"/>
-      <c r="R31" s="1443" t="n"/>
-      <c r="S31" s="1443" t="n"/>
+      <c r="Q31" s="1479" t="n"/>
+      <c r="R31" s="1479" t="n"/>
+      <c r="S31" s="1479" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1442" t="inlineStr">
+      <c r="U31" s="1478" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -6724,49 +6832,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1453" t="inlineStr">
+      <c r="A32" s="1489" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1454" t="inlineStr">
+      <c r="B32" s="1490" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1454" t="inlineStr">
+      <c r="C32" s="1490" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1455" t="n"/>
-      <c r="E32" s="1455" t="n"/>
-      <c r="F32" s="1455" t="n"/>
-      <c r="G32" s="1455" t="n"/>
-      <c r="H32" s="1455" t="n">
+      <c r="D32" s="1491" t="n"/>
+      <c r="E32" s="1491" t="n"/>
+      <c r="F32" s="1491" t="n"/>
+      <c r="G32" s="1491" t="n"/>
+      <c r="H32" s="1491" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1456" t="n"/>
-      <c r="J32" s="1457" t="n"/>
-      <c r="K32" s="1457" t="n"/>
-      <c r="L32" s="1457" t="n"/>
-      <c r="M32" s="1455" t="n">
+      <c r="I32" s="1492" t="n"/>
+      <c r="J32" s="1493" t="n"/>
+      <c r="K32" s="1493" t="n"/>
+      <c r="L32" s="1493" t="n"/>
+      <c r="M32" s="1491" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1455" t="n">
+      <c r="N32" s="1491" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1455" t="n"/>
-      <c r="P32" s="1458" t="n"/>
-      <c r="Q32" s="1455" t="n"/>
-      <c r="R32" s="1455" t="n"/>
-      <c r="S32" s="1455" t="n"/>
+      <c r="O32" s="1491" t="n"/>
+      <c r="P32" s="1494" t="n"/>
+      <c r="Q32" s="1491" t="n"/>
+      <c r="R32" s="1491" t="n"/>
+      <c r="S32" s="1491" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1454" t="n"/>
+      <c r="U32" s="1490" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -6774,57 +6882,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1429" t="inlineStr">
+      <c r="A33" s="1465" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1430" t="inlineStr">
+      <c r="B33" s="1466" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1430" t="inlineStr">
+      <c r="C33" s="1466" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1431" t="n"/>
-      <c r="E33" s="1431" t="n">
+      <c r="D33" s="1467" t="n"/>
+      <c r="E33" s="1467" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1431" t="n">
+      <c r="F33" s="1467" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1431" t="n">
+      <c r="G33" s="1467" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1431" t="n"/>
-      <c r="I33" s="1432" t="n">
+      <c r="H33" s="1467" t="n"/>
+      <c r="I33" s="1468" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1433" t="n"/>
-      <c r="K33" s="1433" t="n"/>
-      <c r="L33" s="1433" t="n"/>
-      <c r="M33" s="1431" t="n"/>
-      <c r="N33" s="1431" t="n"/>
-      <c r="O33" s="1431" t="n">
+      <c r="J33" s="1469" t="n"/>
+      <c r="K33" s="1469" t="n"/>
+      <c r="L33" s="1469" t="n"/>
+      <c r="M33" s="1467" t="n"/>
+      <c r="N33" s="1467" t="n"/>
+      <c r="O33" s="1467" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1434" t="n">
+      <c r="P33" s="1470" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1431" t="n"/>
-      <c r="R33" s="1431" t="n">
+      <c r="Q33" s="1467" t="n"/>
+      <c r="R33" s="1467" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1431" t="n"/>
+      <c r="S33" s="1467" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1430" t="inlineStr">
+      <c r="U33" s="1466" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -6836,49 +6944,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1435" t="inlineStr">
+      <c r="A34" s="1471" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1436" t="inlineStr">
+      <c r="B34" s="1472" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1436" t="inlineStr">
+      <c r="C34" s="1472" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1437" t="n"/>
-      <c r="E34" s="1437" t="n"/>
-      <c r="F34" s="1437" t="n"/>
-      <c r="G34" s="1437" t="n"/>
-      <c r="H34" s="1437" t="n">
+      <c r="D34" s="1473" t="n"/>
+      <c r="E34" s="1473" t="n"/>
+      <c r="F34" s="1473" t="n"/>
+      <c r="G34" s="1473" t="n"/>
+      <c r="H34" s="1473" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1438" t="n"/>
-      <c r="J34" s="1439" t="n"/>
-      <c r="K34" s="1439" t="n"/>
-      <c r="L34" s="1439" t="n"/>
-      <c r="M34" s="1437" t="n">
+      <c r="I34" s="1474" t="n"/>
+      <c r="J34" s="1475" t="n"/>
+      <c r="K34" s="1475" t="n"/>
+      <c r="L34" s="1475" t="n"/>
+      <c r="M34" s="1473" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1437" t="n">
+      <c r="N34" s="1473" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1437" t="n"/>
-      <c r="P34" s="1440" t="n"/>
-      <c r="Q34" s="1437" t="n"/>
-      <c r="R34" s="1437" t="n"/>
-      <c r="S34" s="1437" t="n"/>
+      <c r="O34" s="1473" t="n"/>
+      <c r="P34" s="1476" t="n"/>
+      <c r="Q34" s="1473" t="n"/>
+      <c r="R34" s="1473" t="n"/>
+      <c r="S34" s="1473" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1436" t="n"/>
+      <c r="U34" s="1472" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -6886,57 +6994,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1441" t="inlineStr">
+      <c r="A35" s="1477" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1442" t="inlineStr">
+      <c r="B35" s="1478" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1442" t="inlineStr">
+      <c r="C35" s="1478" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1443" t="n"/>
-      <c r="E35" s="1443" t="n">
+      <c r="D35" s="1479" t="n"/>
+      <c r="E35" s="1479" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1443" t="n">
+      <c r="F35" s="1479" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1443" t="n">
+      <c r="G35" s="1479" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1443" t="n"/>
-      <c r="I35" s="1444" t="n">
+      <c r="H35" s="1479" t="n"/>
+      <c r="I35" s="1480" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1445" t="n"/>
-      <c r="K35" s="1445" t="n"/>
-      <c r="L35" s="1445" t="n"/>
-      <c r="M35" s="1443" t="n"/>
-      <c r="N35" s="1443" t="n"/>
-      <c r="O35" s="1443" t="n">
+      <c r="J35" s="1481" t="n"/>
+      <c r="K35" s="1481" t="n"/>
+      <c r="L35" s="1481" t="n"/>
+      <c r="M35" s="1479" t="n"/>
+      <c r="N35" s="1479" t="n"/>
+      <c r="O35" s="1479" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1446" t="n">
+      <c r="P35" s="1482" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1443" t="n"/>
-      <c r="R35" s="1443" t="n">
+      <c r="Q35" s="1479" t="n"/>
+      <c r="R35" s="1479" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1443" t="n"/>
+      <c r="S35" s="1479" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1442" t="inlineStr">
+      <c r="U35" s="1478" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -6948,49 +7056,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1447" t="inlineStr">
+      <c r="A36" s="1483" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1448" t="inlineStr">
+      <c r="B36" s="1484" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1448" t="inlineStr">
+      <c r="C36" s="1484" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1449" t="n"/>
-      <c r="E36" s="1449" t="n"/>
-      <c r="F36" s="1449" t="n"/>
-      <c r="G36" s="1449" t="n"/>
-      <c r="H36" s="1449" t="n">
+      <c r="D36" s="1485" t="n"/>
+      <c r="E36" s="1485" t="n"/>
+      <c r="F36" s="1485" t="n"/>
+      <c r="G36" s="1485" t="n"/>
+      <c r="H36" s="1485" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1450" t="n"/>
-      <c r="J36" s="1451" t="n"/>
-      <c r="K36" s="1451" t="n"/>
-      <c r="L36" s="1451" t="n"/>
-      <c r="M36" s="1449" t="n">
+      <c r="I36" s="1486" t="n"/>
+      <c r="J36" s="1487" t="n"/>
+      <c r="K36" s="1487" t="n"/>
+      <c r="L36" s="1487" t="n"/>
+      <c r="M36" s="1485" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1449" t="n">
+      <c r="N36" s="1485" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1449" t="n"/>
-      <c r="P36" s="1452" t="n"/>
-      <c r="Q36" s="1449" t="n"/>
-      <c r="R36" s="1449" t="n"/>
-      <c r="S36" s="1449" t="n"/>
+      <c r="O36" s="1485" t="n"/>
+      <c r="P36" s="1488" t="n"/>
+      <c r="Q36" s="1485" t="n"/>
+      <c r="R36" s="1485" t="n"/>
+      <c r="S36" s="1485" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1448" t="n"/>
+      <c r="U36" s="1484" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -6998,41 +7106,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1453" t="inlineStr">
+      <c r="A37" s="1489" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1454" t="inlineStr">
+      <c r="B37" s="1490" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1454" t="inlineStr">
+      <c r="C37" s="1490" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1455" t="n"/>
-      <c r="E37" s="1455" t="n"/>
-      <c r="F37" s="1455" t="n"/>
-      <c r="G37" s="1455" t="n"/>
-      <c r="H37" s="1455" t="n"/>
-      <c r="I37" s="1456" t="n"/>
-      <c r="J37" s="1457" t="n"/>
-      <c r="K37" s="1457" t="n"/>
-      <c r="L37" s="1457" t="n"/>
-      <c r="M37" s="1455" t="n"/>
-      <c r="N37" s="1455" t="n"/>
-      <c r="O37" s="1455" t="n"/>
-      <c r="P37" s="1458" t="n"/>
-      <c r="Q37" s="1455" t="n">
+      <c r="D37" s="1491" t="n"/>
+      <c r="E37" s="1491" t="n"/>
+      <c r="F37" s="1491" t="n"/>
+      <c r="G37" s="1491" t="n"/>
+      <c r="H37" s="1491" t="n"/>
+      <c r="I37" s="1492" t="n"/>
+      <c r="J37" s="1493" t="n"/>
+      <c r="K37" s="1493" t="n"/>
+      <c r="L37" s="1493" t="n"/>
+      <c r="M37" s="1491" t="n"/>
+      <c r="N37" s="1491" t="n"/>
+      <c r="O37" s="1491" t="n"/>
+      <c r="P37" s="1494" t="n"/>
+      <c r="Q37" s="1491" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1455" t="n"/>
-      <c r="S37" s="1455" t="n"/>
+      <c r="R37" s="1491" t="n"/>
+      <c r="S37" s="1491" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1454" t="n"/>
+      <c r="U37" s="1490" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -7040,57 +7148,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1429" t="inlineStr">
+      <c r="A38" s="1465" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1430" t="inlineStr">
+      <c r="B38" s="1466" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1430" t="inlineStr">
+      <c r="C38" s="1466" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1431" t="n"/>
-      <c r="E38" s="1431" t="n">
+      <c r="D38" s="1467" t="n"/>
+      <c r="E38" s="1467" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1431" t="n">
+      <c r="F38" s="1467" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1431" t="n">
+      <c r="G38" s="1467" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1431" t="n"/>
-      <c r="I38" s="1432" t="n">
+      <c r="H38" s="1467" t="n"/>
+      <c r="I38" s="1468" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1433" t="n"/>
-      <c r="K38" s="1433" t="n"/>
-      <c r="L38" s="1433" t="n"/>
-      <c r="M38" s="1431" t="n"/>
-      <c r="N38" s="1431" t="n"/>
-      <c r="O38" s="1431" t="n">
+      <c r="J38" s="1469" t="n"/>
+      <c r="K38" s="1469" t="n"/>
+      <c r="L38" s="1469" t="n"/>
+      <c r="M38" s="1467" t="n"/>
+      <c r="N38" s="1467" t="n"/>
+      <c r="O38" s="1467" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1434" t="n">
+      <c r="P38" s="1470" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1431" t="n"/>
-      <c r="R38" s="1431" t="n">
+      <c r="Q38" s="1467" t="n"/>
+      <c r="R38" s="1467" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1431" t="n"/>
+      <c r="S38" s="1467" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1430" t="inlineStr">
+      <c r="U38" s="1466" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -7102,49 +7210,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1459" t="inlineStr">
+      <c r="A39" s="1495" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1460" t="inlineStr">
+      <c r="B39" s="1496" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1460" t="inlineStr">
+      <c r="C39" s="1496" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1461" t="n"/>
-      <c r="E39" s="1461" t="n"/>
-      <c r="F39" s="1461" t="n"/>
-      <c r="G39" s="1461" t="n"/>
-      <c r="H39" s="1461" t="n">
+      <c r="D39" s="1497" t="n"/>
+      <c r="E39" s="1497" t="n"/>
+      <c r="F39" s="1497" t="n"/>
+      <c r="G39" s="1497" t="n"/>
+      <c r="H39" s="1497" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1462" t="n"/>
-      <c r="J39" s="1463" t="n"/>
-      <c r="K39" s="1463" t="n"/>
-      <c r="L39" s="1463" t="n"/>
-      <c r="M39" s="1461" t="n">
+      <c r="I39" s="1498" t="n"/>
+      <c r="J39" s="1499" t="n"/>
+      <c r="K39" s="1499" t="n"/>
+      <c r="L39" s="1499" t="n"/>
+      <c r="M39" s="1497" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1461" t="n">
+      <c r="N39" s="1497" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1461" t="n"/>
-      <c r="P39" s="1464" t="n"/>
-      <c r="Q39" s="1461" t="n"/>
-      <c r="R39" s="1461" t="n"/>
-      <c r="S39" s="1461" t="n"/>
+      <c r="O39" s="1497" t="n"/>
+      <c r="P39" s="1500" t="n"/>
+      <c r="Q39" s="1497" t="n"/>
+      <c r="R39" s="1497" t="n"/>
+      <c r="S39" s="1497" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1460" t="n"/>
+      <c r="U39" s="1496" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -7152,41 +7260,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1435" t="inlineStr">
+      <c r="A40" s="1471" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1436" t="inlineStr">
+      <c r="B40" s="1472" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1436" t="inlineStr">
+      <c r="C40" s="1472" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1437" t="n"/>
-      <c r="E40" s="1437" t="n"/>
-      <c r="F40" s="1437" t="n"/>
-      <c r="G40" s="1437" t="n"/>
-      <c r="H40" s="1437" t="n"/>
-      <c r="I40" s="1438" t="n"/>
-      <c r="J40" s="1439" t="n"/>
-      <c r="K40" s="1439" t="n"/>
-      <c r="L40" s="1439" t="n"/>
-      <c r="M40" s="1437" t="n"/>
-      <c r="N40" s="1437" t="n"/>
-      <c r="O40" s="1437" t="n"/>
-      <c r="P40" s="1440" t="n"/>
-      <c r="Q40" s="1437" t="n">
+      <c r="D40" s="1473" t="n"/>
+      <c r="E40" s="1473" t="n"/>
+      <c r="F40" s="1473" t="n"/>
+      <c r="G40" s="1473" t="n"/>
+      <c r="H40" s="1473" t="n"/>
+      <c r="I40" s="1474" t="n"/>
+      <c r="J40" s="1475" t="n"/>
+      <c r="K40" s="1475" t="n"/>
+      <c r="L40" s="1475" t="n"/>
+      <c r="M40" s="1473" t="n"/>
+      <c r="N40" s="1473" t="n"/>
+      <c r="O40" s="1473" t="n"/>
+      <c r="P40" s="1476" t="n"/>
+      <c r="Q40" s="1473" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1437" t="n"/>
-      <c r="S40" s="1437" t="n"/>
+      <c r="R40" s="1473" t="n"/>
+      <c r="S40" s="1473" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1436" t="n"/>
+      <c r="U40" s="1472" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -7194,57 +7302,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1441" t="inlineStr">
+      <c r="A41" s="1477" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1442" t="inlineStr">
+      <c r="B41" s="1478" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1442" t="inlineStr">
+      <c r="C41" s="1478" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1443" t="n"/>
-      <c r="E41" s="1443" t="n">
+      <c r="D41" s="1479" t="n"/>
+      <c r="E41" s="1479" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1443" t="n">
+      <c r="F41" s="1479" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1443" t="n">
+      <c r="G41" s="1479" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1443" t="n"/>
-      <c r="I41" s="1444" t="n">
+      <c r="H41" s="1479" t="n"/>
+      <c r="I41" s="1480" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1445" t="n"/>
-      <c r="K41" s="1445" t="n"/>
-      <c r="L41" s="1445" t="n"/>
-      <c r="M41" s="1443" t="n"/>
-      <c r="N41" s="1443" t="n"/>
-      <c r="O41" s="1443" t="n">
+      <c r="J41" s="1481" t="n"/>
+      <c r="K41" s="1481" t="n"/>
+      <c r="L41" s="1481" t="n"/>
+      <c r="M41" s="1479" t="n"/>
+      <c r="N41" s="1479" t="n"/>
+      <c r="O41" s="1479" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1446" t="n">
+      <c r="P41" s="1482" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1443" t="n"/>
-      <c r="R41" s="1443" t="n">
+      <c r="Q41" s="1479" t="n"/>
+      <c r="R41" s="1479" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1443" t="n"/>
+      <c r="S41" s="1479" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1442" t="inlineStr">
+      <c r="U41" s="1478" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -7256,49 +7364,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1453" t="inlineStr">
+      <c r="A42" s="1489" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1454" t="inlineStr">
+      <c r="B42" s="1490" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1454" t="inlineStr">
+      <c r="C42" s="1490" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1455" t="n"/>
-      <c r="E42" s="1455" t="n"/>
-      <c r="F42" s="1455" t="n"/>
-      <c r="G42" s="1455" t="n"/>
-      <c r="H42" s="1455" t="n">
+      <c r="D42" s="1491" t="n"/>
+      <c r="E42" s="1491" t="n"/>
+      <c r="F42" s="1491" t="n"/>
+      <c r="G42" s="1491" t="n"/>
+      <c r="H42" s="1491" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1456" t="n"/>
-      <c r="J42" s="1457" t="n"/>
-      <c r="K42" s="1457" t="n"/>
-      <c r="L42" s="1457" t="n"/>
-      <c r="M42" s="1455" t="n">
+      <c r="I42" s="1492" t="n"/>
+      <c r="J42" s="1493" t="n"/>
+      <c r="K42" s="1493" t="n"/>
+      <c r="L42" s="1493" t="n"/>
+      <c r="M42" s="1491" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1455" t="n">
+      <c r="N42" s="1491" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1455" t="n"/>
-      <c r="P42" s="1458" t="n"/>
-      <c r="Q42" s="1455" t="n"/>
-      <c r="R42" s="1455" t="n"/>
-      <c r="S42" s="1455" t="n"/>
+      <c r="O42" s="1491" t="n"/>
+      <c r="P42" s="1494" t="n"/>
+      <c r="Q42" s="1491" t="n"/>
+      <c r="R42" s="1491" t="n"/>
+      <c r="S42" s="1491" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1454" t="n"/>
+      <c r="U42" s="1490" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -7306,57 +7414,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1429" t="inlineStr">
+      <c r="A43" s="1465" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1430" t="inlineStr">
+      <c r="B43" s="1466" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1430" t="inlineStr">
+      <c r="C43" s="1466" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1431" t="n"/>
-      <c r="E43" s="1431" t="n">
+      <c r="D43" s="1467" t="n"/>
+      <c r="E43" s="1467" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1431" t="n">
+      <c r="F43" s="1467" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1431" t="n">
+      <c r="G43" s="1467" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1431" t="n"/>
-      <c r="I43" s="1432" t="n">
+      <c r="H43" s="1467" t="n"/>
+      <c r="I43" s="1468" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1433" t="n"/>
-      <c r="K43" s="1433" t="n"/>
-      <c r="L43" s="1433" t="n"/>
-      <c r="M43" s="1431" t="n"/>
-      <c r="N43" s="1431" t="n"/>
-      <c r="O43" s="1431" t="n">
+      <c r="J43" s="1469" t="n"/>
+      <c r="K43" s="1469" t="n"/>
+      <c r="L43" s="1469" t="n"/>
+      <c r="M43" s="1467" t="n"/>
+      <c r="N43" s="1467" t="n"/>
+      <c r="O43" s="1467" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1434" t="n">
+      <c r="P43" s="1470" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1431" t="n"/>
-      <c r="R43" s="1431" t="n">
+      <c r="Q43" s="1467" t="n"/>
+      <c r="R43" s="1467" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1431" t="n"/>
+      <c r="S43" s="1467" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1430" t="n"/>
+      <c r="U43" s="1466" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -7364,45 +7472,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1459" t="inlineStr">
+      <c r="A44" s="1495" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1460" t="inlineStr">
+      <c r="B44" s="1496" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1460" t="inlineStr">
+      <c r="C44" s="1496" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1461" t="n"/>
-      <c r="E44" s="1461" t="n">
+      <c r="D44" s="1497" t="n"/>
+      <c r="E44" s="1497" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1461" t="n">
+      <c r="F44" s="1497" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1461" t="n"/>
-      <c r="H44" s="1461" t="n"/>
-      <c r="I44" s="1462" t="n"/>
-      <c r="J44" s="1463" t="n"/>
-      <c r="K44" s="1463" t="n"/>
-      <c r="L44" s="1463" t="n"/>
-      <c r="M44" s="1461" t="n"/>
-      <c r="N44" s="1461" t="n"/>
-      <c r="O44" s="1461" t="n"/>
-      <c r="P44" s="1464" t="n"/>
-      <c r="Q44" s="1461" t="n"/>
-      <c r="R44" s="1461" t="n"/>
-      <c r="S44" s="1461" t="n">
+      <c r="G44" s="1497" t="n"/>
+      <c r="H44" s="1497" t="n"/>
+      <c r="I44" s="1498" t="n"/>
+      <c r="J44" s="1499" t="n"/>
+      <c r="K44" s="1499" t="n"/>
+      <c r="L44" s="1499" t="n"/>
+      <c r="M44" s="1497" t="n"/>
+      <c r="N44" s="1497" t="n"/>
+      <c r="O44" s="1497" t="n"/>
+      <c r="P44" s="1500" t="n"/>
+      <c r="Q44" s="1497" t="n"/>
+      <c r="R44" s="1497" t="n"/>
+      <c r="S44" s="1497" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1460" t="inlineStr">
+      <c r="U44" s="1496" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -7414,49 +7522,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1459" t="inlineStr">
+      <c r="A45" s="1495" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1460" t="inlineStr">
+      <c r="B45" s="1496" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1460" t="inlineStr">
+      <c r="C45" s="1496" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1461" t="n"/>
-      <c r="E45" s="1461" t="n"/>
-      <c r="F45" s="1461" t="n"/>
-      <c r="G45" s="1461" t="n"/>
-      <c r="H45" s="1461" t="n">
+      <c r="D45" s="1497" t="n"/>
+      <c r="E45" s="1497" t="n"/>
+      <c r="F45" s="1497" t="n"/>
+      <c r="G45" s="1497" t="n"/>
+      <c r="H45" s="1497" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1462" t="n"/>
-      <c r="J45" s="1463" t="n"/>
-      <c r="K45" s="1463" t="n"/>
-      <c r="L45" s="1463" t="n"/>
-      <c r="M45" s="1461" t="n">
+      <c r="I45" s="1498" t="n"/>
+      <c r="J45" s="1499" t="n"/>
+      <c r="K45" s="1499" t="n"/>
+      <c r="L45" s="1499" t="n"/>
+      <c r="M45" s="1497" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1461" t="n">
+      <c r="N45" s="1497" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1461" t="n"/>
-      <c r="P45" s="1464" t="n"/>
-      <c r="Q45" s="1461" t="n"/>
-      <c r="R45" s="1461" t="n"/>
-      <c r="S45" s="1461" t="n"/>
+      <c r="O45" s="1497" t="n"/>
+      <c r="P45" s="1500" t="n"/>
+      <c r="Q45" s="1497" t="n"/>
+      <c r="R45" s="1497" t="n"/>
+      <c r="S45" s="1497" t="n"/>
       <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1460" t="n"/>
+      <c r="U45" s="1496" t="n"/>
       <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -7464,39 +7572,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1435" t="inlineStr">
+      <c r="A46" s="1471" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B46" s="1436" t="inlineStr">
+      <c r="B46" s="1472" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="C46" s="1436" t="inlineStr">
+      <c r="C46" s="1472" t="inlineStr">
         <is>
           <t>EVENT - Clean</t>
         </is>
       </c>
-      <c r="D46" s="1437" t="n"/>
-      <c r="E46" s="1437" t="n"/>
-      <c r="F46" s="1437" t="n"/>
-      <c r="G46" s="1437" t="n"/>
-      <c r="H46" s="1437" t="n"/>
-      <c r="I46" s="1438" t="n"/>
-      <c r="J46" s="1439" t="n"/>
-      <c r="K46" s="1439" t="n"/>
-      <c r="L46" s="1439" t="n"/>
-      <c r="M46" s="1437" t="n"/>
-      <c r="N46" s="1437" t="n"/>
-      <c r="O46" s="1437" t="n"/>
-      <c r="P46" s="1440" t="n"/>
-      <c r="Q46" s="1437" t="n"/>
-      <c r="R46" s="1437" t="n"/>
-      <c r="S46" s="1437" t="n"/>
+      <c r="D46" s="1473" t="n"/>
+      <c r="E46" s="1473" t="n"/>
+      <c r="F46" s="1473" t="n"/>
+      <c r="G46" s="1473" t="n"/>
+      <c r="H46" s="1473" t="n"/>
+      <c r="I46" s="1474" t="n"/>
+      <c r="J46" s="1475" t="n"/>
+      <c r="K46" s="1475" t="n"/>
+      <c r="L46" s="1475" t="n"/>
+      <c r="M46" s="1473" t="n"/>
+      <c r="N46" s="1473" t="n"/>
+      <c r="O46" s="1473" t="n"/>
+      <c r="P46" s="1476" t="n"/>
+      <c r="Q46" s="1473" t="n"/>
+      <c r="R46" s="1473" t="n"/>
+      <c r="S46" s="1473" t="n"/>
       <c r="T46" s="631" t="n"/>
-      <c r="U46" s="1436" t="n"/>
+      <c r="U46" s="1472" t="n"/>
       <c r="V46" s="632" t="inlineStr">
         <is>
           <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
@@ -7504,51 +7612,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1441" t="inlineStr">
+      <c r="A47" s="1477" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1442" t="inlineStr">
+      <c r="B47" s="1478" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C47" s="1442" t="inlineStr">
+      <c r="C47" s="1478" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D47" s="1443" t="n"/>
-      <c r="E47" s="1443" t="n">
+      <c r="D47" s="1479" t="n"/>
+      <c r="E47" s="1479" t="n">
         <v>16.6</v>
       </c>
-      <c r="F47" s="1443" t="n">
+      <c r="F47" s="1479" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="1443" t="n">
+      <c r="G47" s="1479" t="n">
         <v>4.1</v>
       </c>
-      <c r="H47" s="1443" t="n"/>
-      <c r="I47" s="1444" t="n">
+      <c r="H47" s="1479" t="n"/>
+      <c r="I47" s="1480" t="n">
         <v>0.9</v>
       </c>
-      <c r="J47" s="1445" t="n"/>
-      <c r="K47" s="1445" t="n"/>
-      <c r="L47" s="1445" t="n"/>
-      <c r="M47" s="1443" t="n"/>
-      <c r="N47" s="1443" t="n"/>
-      <c r="O47" s="1443" t="n">
+      <c r="J47" s="1481" t="n"/>
+      <c r="K47" s="1481" t="n"/>
+      <c r="L47" s="1481" t="n"/>
+      <c r="M47" s="1479" t="n"/>
+      <c r="N47" s="1479" t="n"/>
+      <c r="O47" s="1479" t="n">
         <v>13.2</v>
       </c>
-      <c r="P47" s="1446" t="n">
+      <c r="P47" s="1482" t="n">
         <v>0</v>
       </c>
-      <c r="Q47" s="1443" t="n"/>
-      <c r="R47" s="1443" t="n">
+      <c r="Q47" s="1479" t="n"/>
+      <c r="R47" s="1479" t="n">
         <v>84.5</v>
       </c>
-      <c r="S47" s="1443" t="n">
+      <c r="S47" s="1479" t="n">
         <v>11.8</v>
       </c>
       <c r="T47" s="813" t="inlineStr">
@@ -7556,7 +7664,7 @@
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1442" t="inlineStr">
+      <c r="U47" s="1478" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
@@ -7568,49 +7676,49 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1453" t="inlineStr">
+      <c r="A48" s="1489" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B48" s="1454" t="inlineStr">
+      <c r="B48" s="1490" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C48" s="1454" t="inlineStr">
+      <c r="C48" s="1490" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D48" s="1455" t="n"/>
-      <c r="E48" s="1455" t="n"/>
-      <c r="F48" s="1455" t="n"/>
-      <c r="G48" s="1455" t="n"/>
-      <c r="H48" s="1455" t="n">
+      <c r="D48" s="1491" t="n"/>
+      <c r="E48" s="1491" t="n"/>
+      <c r="F48" s="1491" t="n"/>
+      <c r="G48" s="1491" t="n"/>
+      <c r="H48" s="1491" t="n">
         <v>15.1</v>
       </c>
-      <c r="I48" s="1456" t="n"/>
-      <c r="J48" s="1457" t="n"/>
-      <c r="K48" s="1457" t="n"/>
-      <c r="L48" s="1457" t="n"/>
-      <c r="M48" s="1455" t="n">
+      <c r="I48" s="1492" t="n"/>
+      <c r="J48" s="1493" t="n"/>
+      <c r="K48" s="1493" t="n"/>
+      <c r="L48" s="1493" t="n"/>
+      <c r="M48" s="1491" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="1455" t="n">
+      <c r="N48" s="1491" t="n">
         <v>20</v>
       </c>
-      <c r="O48" s="1455" t="n"/>
-      <c r="P48" s="1458" t="n"/>
-      <c r="Q48" s="1455" t="n"/>
-      <c r="R48" s="1455" t="n"/>
-      <c r="S48" s="1455" t="n"/>
+      <c r="O48" s="1491" t="n"/>
+      <c r="P48" s="1494" t="n"/>
+      <c r="Q48" s="1491" t="n"/>
+      <c r="R48" s="1491" t="n"/>
+      <c r="S48" s="1491" t="n"/>
       <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U48" s="1454" t="n"/>
+      <c r="U48" s="1490" t="n"/>
       <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
@@ -7618,51 +7726,51 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1429" t="inlineStr">
+      <c r="A49" s="1465" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B49" s="1430" t="inlineStr">
+      <c r="B49" s="1466" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C49" s="1430" t="inlineStr">
+      <c r="C49" s="1466" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D49" s="1431" t="n"/>
-      <c r="E49" s="1431" t="n">
+      <c r="D49" s="1467" t="n"/>
+      <c r="E49" s="1467" t="n">
         <v>16.8</v>
       </c>
-      <c r="F49" s="1431" t="n">
+      <c r="F49" s="1467" t="n">
         <v>0.2</v>
       </c>
-      <c r="G49" s="1431" t="n">
+      <c r="G49" s="1467" t="n">
         <v>3.3</v>
       </c>
-      <c r="H49" s="1431" t="n"/>
-      <c r="I49" s="1432" t="n">
+      <c r="H49" s="1467" t="n"/>
+      <c r="I49" s="1468" t="n">
         <v>1.7</v>
       </c>
-      <c r="J49" s="1433" t="n"/>
-      <c r="K49" s="1433" t="n"/>
-      <c r="L49" s="1433" t="n"/>
-      <c r="M49" s="1431" t="n"/>
-      <c r="N49" s="1431" t="n"/>
-      <c r="O49" s="1431" t="n">
+      <c r="J49" s="1469" t="n"/>
+      <c r="K49" s="1469" t="n"/>
+      <c r="L49" s="1469" t="n"/>
+      <c r="M49" s="1467" t="n"/>
+      <c r="N49" s="1467" t="n"/>
+      <c r="O49" s="1467" t="n">
         <v>13</v>
       </c>
-      <c r="P49" s="1434" t="n">
+      <c r="P49" s="1470" t="n">
         <v>0.87</v>
       </c>
-      <c r="Q49" s="1431" t="n"/>
-      <c r="R49" s="1431" t="n">
+      <c r="Q49" s="1467" t="n"/>
+      <c r="R49" s="1467" t="n">
         <v>86</v>
       </c>
-      <c r="S49" s="1431" t="n">
+      <c r="S49" s="1467" t="n">
         <v>11.65</v>
       </c>
       <c r="T49" s="624" t="inlineStr">
@@ -7670,7 +7778,7 @@
           <t>Clear now, 88F, 67% RH; sun so far 6.4h of 7h daylight (91%); today high 90F, 0.87in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U49" s="1430" t="inlineStr">
+      <c r="U49" s="1466" t="inlineStr">
         <is>
           <t>2026-07-04_1.jpeg;2026-07-04_2.jpeg;2026-07-04_3.jpeg;2026-07-04_4.jpeg</t>
         </is>
@@ -7682,49 +7790,49 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1435" t="inlineStr">
+      <c r="A50" s="1471" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B50" s="1436" t="inlineStr">
+      <c r="B50" s="1472" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C50" s="1436" t="inlineStr">
+      <c r="C50" s="1472" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D50" s="1437" t="n"/>
-      <c r="E50" s="1437" t="n"/>
-      <c r="F50" s="1437" t="n"/>
-      <c r="G50" s="1437" t="n"/>
-      <c r="H50" s="1437" t="n">
+      <c r="D50" s="1473" t="n"/>
+      <c r="E50" s="1473" t="n"/>
+      <c r="F50" s="1473" t="n"/>
+      <c r="G50" s="1473" t="n"/>
+      <c r="H50" s="1473" t="n">
         <v>14.6</v>
       </c>
-      <c r="I50" s="1438" t="n"/>
-      <c r="J50" s="1439" t="n"/>
-      <c r="K50" s="1439" t="n"/>
-      <c r="L50" s="1439" t="n"/>
-      <c r="M50" s="1437" t="n">
+      <c r="I50" s="1474" t="n"/>
+      <c r="J50" s="1475" t="n"/>
+      <c r="K50" s="1475" t="n"/>
+      <c r="L50" s="1475" t="n"/>
+      <c r="M50" s="1473" t="n">
         <v>0.5</v>
       </c>
-      <c r="N50" s="1437" t="n">
+      <c r="N50" s="1473" t="n">
         <v>20.5</v>
       </c>
-      <c r="O50" s="1437" t="n"/>
-      <c r="P50" s="1440" t="n"/>
-      <c r="Q50" s="1437" t="n"/>
-      <c r="R50" s="1437" t="n"/>
-      <c r="S50" s="1437" t="n"/>
+      <c r="O50" s="1473" t="n"/>
+      <c r="P50" s="1476" t="n"/>
+      <c r="Q50" s="1473" t="n"/>
+      <c r="R50" s="1473" t="n"/>
+      <c r="S50" s="1473" t="n"/>
       <c r="T50" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny day (high 90F, water 86F); storm forecast overnight</t>
         </is>
       </c>
-      <c r="U50" s="1436" t="n"/>
+      <c r="U50" s="1472" t="n"/>
       <c r="V50" s="632" t="inlineStr">
         <is>
           <t>0.5 gal added 7:40 PM. PARTY PRE-LOAD (Sun 7/5 1PM picnic): deliberately HALF the usual dose -- FC already high at 16.8, and John didn't want to overshoot into the high teens for guests. Sized on the retuned model (l24_hot_sunny now 4.0). Model projects ~14.6 next noon, BUT this is a known weather-mismatch case: model keys L24 off today's hot/sunny weather, while the actual loss window is a storm overnight (no UV) + cooler/cloudy Sun morning -&gt; real loss will be LOWER, so FC likely lands ~15-16 at the party (comfortable top-of-band, cushion for bather load, not overboard). =&gt; If tomorrow's noon comes in ABOVE 14.6, that's the weather mismatch, NOT the freshly-retuned constant; don't chase it. Plan: dose back up Sun evening after the crowd's out (expect a bather-load FC drop). Season total 20.5 gal. PHOTOS(4): water clear/healthy blue, bottom fully visible, no cloudiness/algae; yesterday's surface debris now gone (tracks with CC clearing to 0.2); liner step close-up normal speckled blue, no rust/stain progression. Ruler photo documents the ~11.65 cm level.</t>
@@ -7732,47 +7840,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1441" t="inlineStr">
+      <c r="A51" s="1477" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B51" s="1442" t="inlineStr">
+      <c r="B51" s="1478" t="inlineStr">
         <is>
           <t>07:45</t>
         </is>
       </c>
-      <c r="C51" s="1442" t="inlineStr">
+      <c r="C51" s="1478" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D51" s="1443" t="n"/>
-      <c r="E51" s="1443" t="n">
+      <c r="D51" s="1479" t="n"/>
+      <c r="E51" s="1479" t="n">
         <v>16</v>
       </c>
-      <c r="F51" s="1443" t="n">
+      <c r="F51" s="1479" t="n">
         <v>0.5</v>
       </c>
-      <c r="G51" s="1443" t="n"/>
-      <c r="H51" s="1443" t="n"/>
-      <c r="I51" s="1444" t="n">
+      <c r="G51" s="1479" t="n"/>
+      <c r="H51" s="1479" t="n"/>
+      <c r="I51" s="1480" t="n">
         <v>1.4</v>
       </c>
-      <c r="J51" s="1445" t="n"/>
-      <c r="K51" s="1445" t="n"/>
-      <c r="L51" s="1445" t="n"/>
-      <c r="M51" s="1443" t="n"/>
-      <c r="N51" s="1443" t="n"/>
-      <c r="O51" s="1443" t="n"/>
-      <c r="P51" s="1446" t="n">
+      <c r="J51" s="1481" t="n"/>
+      <c r="K51" s="1481" t="n"/>
+      <c r="L51" s="1481" t="n"/>
+      <c r="M51" s="1479" t="n"/>
+      <c r="N51" s="1479" t="n"/>
+      <c r="O51" s="1479" t="n"/>
+      <c r="P51" s="1482" t="n">
         <v>0.04</v>
       </c>
-      <c r="Q51" s="1443" t="n"/>
-      <c r="R51" s="1443" t="n">
+      <c r="Q51" s="1479" t="n"/>
+      <c r="R51" s="1479" t="n">
         <v>84</v>
       </c>
-      <c r="S51" s="1443" t="n">
+      <c r="S51" s="1479" t="n">
         <v>13.9</v>
       </c>
       <c r="T51" s="813" t="inlineStr">
@@ -7780,7 +7888,7 @@
           <t>Overcast now, 75F, 90% RH; sun so far 0.0h of 3h daylight (0%); today high 75F, 0.04in precip, UV max 6.5</t>
         </is>
       </c>
-      <c r="U51" s="1442" t="inlineStr">
+      <c r="U51" s="1478" t="inlineStr">
         <is>
           <t>2026-07-05_2.jpeg</t>
         </is>
@@ -7792,56 +7900,106 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1453" t="inlineStr">
+      <c r="A52" s="1483" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B52" s="1454" t="inlineStr">
+      <c r="B52" s="1484" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C52" s="1454" t="inlineStr">
+      <c r="C52" s="1484" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D52" s="1455" t="n"/>
-      <c r="E52" s="1455" t="n">
+      <c r="D52" s="1485" t="n"/>
+      <c r="E52" s="1485" t="n">
         <v>14.8</v>
       </c>
-      <c r="F52" s="1455" t="n">
+      <c r="F52" s="1485" t="n">
         <v>0.3</v>
       </c>
-      <c r="G52" s="1455" t="n"/>
-      <c r="H52" s="1455" t="n"/>
-      <c r="I52" s="1456" t="n"/>
-      <c r="J52" s="1457" t="n"/>
-      <c r="K52" s="1457" t="n"/>
-      <c r="L52" s="1457" t="n"/>
-      <c r="M52" s="1455" t="n"/>
-      <c r="N52" s="1455" t="n"/>
-      <c r="O52" s="1455" t="n"/>
-      <c r="P52" s="1458" t="n"/>
-      <c r="Q52" s="1455" t="n"/>
-      <c r="R52" s="1455" t="n"/>
-      <c r="S52" s="1455" t="n">
+      <c r="G52" s="1485" t="n"/>
+      <c r="H52" s="1485" t="n"/>
+      <c r="I52" s="1486" t="n"/>
+      <c r="J52" s="1487" t="n"/>
+      <c r="K52" s="1487" t="n"/>
+      <c r="L52" s="1487" t="n"/>
+      <c r="M52" s="1485" t="n"/>
+      <c r="N52" s="1485" t="n"/>
+      <c r="O52" s="1485" t="n"/>
+      <c r="P52" s="1488" t="n"/>
+      <c r="Q52" s="1485" t="n"/>
+      <c r="R52" s="1485" t="n"/>
+      <c r="S52" s="1485" t="n">
         <v>13.6</v>
       </c>
-      <c r="T52" s="827" t="inlineStr">
+      <c r="T52" s="820" t="inlineStr">
         <is>
           <t>Overcast now, 72F, 76% RH; sun so far 8.4h of 13h daylight (65%); today high 80F, 0.00in precip, UV max 6.0</t>
         </is>
       </c>
-      <c r="U52" s="1454" t="inlineStr">
+      <c r="U52" s="1484" t="inlineStr">
         <is>
           <t>2026-07-05_1.jpeg;2026-07-05_3.jpeg</t>
         </is>
       </c>
-      <c r="V52" s="828" t="inlineStr">
+      <c r="V52" s="821" t="inlineStr">
         <is>
           <t>Post-party evening test (2nd test of the day; morning 7:45AM was 16.0). PARTY OUTCOME -- EXCELLENT: FC 16.0(AM) -&gt; 14.8(now), only -1.2 ppm across the whole party (landed right at aim 15); CC 0.5 -&gt; 0.3, i.e. CC DROPPED even after a crowd -- the high FC oxidized bather-load chloramines faster than they formed. The pre-load-modestly strategy worked perfectly (didn't overshoot, didn't crash). PHOTOS(2): wide shot shows crystal-clear water, bottom fully visible, no cloudiness/debris/algae -- pool sailed through. Evening dose recommended 0.5 gal, sized on TOMORROW's rainy forecast (the real loss window: wet/overcast 7/6, ~0.9in rain, low UV) rather than today's sun -&gt; projects ~15.1 at Mon noon. (Day actually cleared to 8.4 sun hrs vs the overcast 7:45AM read.) fc_loss/pred_error blank: off-cadence 2nd test; the 7/4 dose's prediction was already scored against this morning's reading. No water level/temp reported this eve -- ruler photo taken (2026-07-05_2) but no number given; will log if John reads it off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="1489" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B53" s="1490" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="C53" s="1490" t="inlineStr">
+        <is>
+          <t>DOSE</t>
+        </is>
+      </c>
+      <c r="D53" s="1491" t="n"/>
+      <c r="E53" s="1491" t="n"/>
+      <c r="F53" s="1491" t="n"/>
+      <c r="G53" s="1491" t="n"/>
+      <c r="H53" s="1491" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="I53" s="1492" t="n"/>
+      <c r="J53" s="1493" t="n"/>
+      <c r="K53" s="1493" t="n"/>
+      <c r="L53" s="1493" t="n"/>
+      <c r="M53" s="1491" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="N53" s="1491" t="n">
+        <v>21</v>
+      </c>
+      <c r="O53" s="1491" t="n"/>
+      <c r="P53" s="1494" t="n"/>
+      <c r="Q53" s="1491" t="n"/>
+      <c r="R53" s="1491" t="n"/>
+      <c r="S53" s="1491" t="n"/>
+      <c r="T53" s="827" t="inlineStr">
+        <is>
+          <t>Cleared to partly sunny (8.4 sun hrs, high 80F, water 84F); all-day rain forecast Mon 7/6</t>
+        </is>
+      </c>
+      <c r="U53" s="1490" t="n"/>
+      <c r="V53" s="828" t="inlineStr">
+        <is>
+          <t>0.5 gal added 7:25 PM (post-party recovery dose). Sized on TOMORROW's rainy forecast (the real loss window: overcast/wet 7/6, ~0.9in rain, low UV) not today's sun -&gt; projects ~15.1 at Mon noon. Party went great (FC held 16.0-&gt;14.8, CC dropped 0.5-&gt;0.3). Season total 21.0 gal. This is the first prediction that deliberately used the next-day forecast for L24 instead of the model's default (today's weather as proxy) -- if it lands near 15.1 tomorrow, that validates feeding the forecast on weather-change days.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log 2026-07-06 noon (rain): FC 13.8, CC 0.2, level 15.1 (overflowing)
First negative prediction error (-1.3): heavy rain (2in) overflowed the
pool, carrying FC+CYA out beyond what the UV-only rain bucket models.
fc_loss blank (overflow/dilution confound). Overflow is passively lowering
CYA -- good. Recommending HOLD on dosing tonight (overflow wastes it,
FC fine, chlorine low till refill).
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1501">
+  <cellXfs count="1543">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -5030,6 +5030,132 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5291,7 +5417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V53"/>
+  <dimension ref="A1:V54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -5468,35 +5594,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1465" t="inlineStr">
+      <c r="A3" s="1501" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1466" t="n"/>
-      <c r="C3" s="1466" t="inlineStr">
+      <c r="B3" s="1502" t="n"/>
+      <c r="C3" s="1502" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1467" t="n"/>
-      <c r="E3" s="1467" t="n"/>
-      <c r="F3" s="1467" t="n"/>
-      <c r="G3" s="1467" t="n"/>
-      <c r="H3" s="1467" t="n"/>
-      <c r="I3" s="1468" t="n"/>
-      <c r="J3" s="1469" t="n"/>
-      <c r="K3" s="1469" t="n"/>
-      <c r="L3" s="1469" t="n"/>
-      <c r="M3" s="1467" t="n"/>
-      <c r="N3" s="1467" t="n"/>
-      <c r="O3" s="1467" t="n"/>
-      <c r="P3" s="1470" t="n"/>
-      <c r="Q3" s="1467" t="n"/>
-      <c r="R3" s="1467" t="n"/>
-      <c r="S3" s="1467" t="n"/>
+      <c r="D3" s="1503" t="n"/>
+      <c r="E3" s="1503" t="n"/>
+      <c r="F3" s="1503" t="n"/>
+      <c r="G3" s="1503" t="n"/>
+      <c r="H3" s="1503" t="n"/>
+      <c r="I3" s="1504" t="n"/>
+      <c r="J3" s="1505" t="n"/>
+      <c r="K3" s="1505" t="n"/>
+      <c r="L3" s="1505" t="n"/>
+      <c r="M3" s="1503" t="n"/>
+      <c r="N3" s="1503" t="n"/>
+      <c r="O3" s="1503" t="n"/>
+      <c r="P3" s="1506" t="n"/>
+      <c r="Q3" s="1503" t="n"/>
+      <c r="R3" s="1503" t="n"/>
+      <c r="S3" s="1503" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1466" t="n"/>
+      <c r="U3" s="1502" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -5504,43 +5630,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1471" t="inlineStr">
+      <c r="A4" s="1507" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1472" t="inlineStr">
+      <c r="B4" s="1508" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1472" t="inlineStr">
+      <c r="C4" s="1508" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1473" t="n"/>
-      <c r="E4" s="1473" t="n"/>
-      <c r="F4" s="1473" t="n"/>
-      <c r="G4" s="1473" t="n"/>
-      <c r="H4" s="1473" t="n"/>
-      <c r="I4" s="1474" t="n"/>
-      <c r="J4" s="1475" t="n"/>
-      <c r="K4" s="1475" t="n"/>
-      <c r="L4" s="1475" t="n"/>
-      <c r="M4" s="1473" t="n">
+      <c r="D4" s="1509" t="n"/>
+      <c r="E4" s="1509" t="n"/>
+      <c r="F4" s="1509" t="n"/>
+      <c r="G4" s="1509" t="n"/>
+      <c r="H4" s="1509" t="n"/>
+      <c r="I4" s="1510" t="n"/>
+      <c r="J4" s="1511" t="n"/>
+      <c r="K4" s="1511" t="n"/>
+      <c r="L4" s="1511" t="n"/>
+      <c r="M4" s="1509" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1473" t="n">
+      <c r="N4" s="1509" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1473" t="n"/>
-      <c r="P4" s="1476" t="n"/>
-      <c r="Q4" s="1473" t="n"/>
-      <c r="R4" s="1473" t="n"/>
-      <c r="S4" s="1473" t="n"/>
+      <c r="O4" s="1509" t="n"/>
+      <c r="P4" s="1512" t="n"/>
+      <c r="Q4" s="1509" t="n"/>
+      <c r="R4" s="1509" t="n"/>
+      <c r="S4" s="1509" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1472" t="n"/>
+      <c r="U4" s="1508" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -5548,57 +5674,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1477" t="inlineStr">
+      <c r="A5" s="1513" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1478" t="inlineStr">
+      <c r="B5" s="1514" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1478" t="inlineStr">
+      <c r="C5" s="1514" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1479" t="n">
+      <c r="D5" s="1515" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1479" t="n">
+      <c r="E5" s="1515" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1479" t="n">
+      <c r="F5" s="1515" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1479" t="n"/>
-      <c r="H5" s="1479" t="n"/>
-      <c r="I5" s="1480" t="n"/>
-      <c r="J5" s="1481" t="n">
+      <c r="G5" s="1515" t="n"/>
+      <c r="H5" s="1515" t="n"/>
+      <c r="I5" s="1516" t="n"/>
+      <c r="J5" s="1517" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1481" t="n">
+      <c r="K5" s="1517" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1481" t="inlineStr">
+      <c r="L5" s="1517" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1479" t="n"/>
-      <c r="N5" s="1479" t="n"/>
-      <c r="O5" s="1479" t="n">
+      <c r="M5" s="1515" t="n"/>
+      <c r="N5" s="1515" t="n"/>
+      <c r="O5" s="1515" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1482" t="n">
+      <c r="P5" s="1518" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1479" t="n"/>
-      <c r="R5" s="1479" t="n"/>
-      <c r="S5" s="1479" t="n"/>
+      <c r="Q5" s="1515" t="n"/>
+      <c r="R5" s="1515" t="n"/>
+      <c r="S5" s="1515" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1478" t="n"/>
+      <c r="U5" s="1514" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -5606,43 +5732,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1483" t="inlineStr">
+      <c r="A6" s="1519" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1484" t="inlineStr">
+      <c r="B6" s="1520" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1484" t="inlineStr">
+      <c r="C6" s="1520" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1485" t="n"/>
-      <c r="E6" s="1485" t="n"/>
-      <c r="F6" s="1485" t="n"/>
-      <c r="G6" s="1485" t="n"/>
-      <c r="H6" s="1485" t="n"/>
-      <c r="I6" s="1486" t="n"/>
-      <c r="J6" s="1487" t="n"/>
-      <c r="K6" s="1487" t="n"/>
-      <c r="L6" s="1487" t="n"/>
-      <c r="M6" s="1485" t="n">
+      <c r="D6" s="1521" t="n"/>
+      <c r="E6" s="1521" t="n"/>
+      <c r="F6" s="1521" t="n"/>
+      <c r="G6" s="1521" t="n"/>
+      <c r="H6" s="1521" t="n"/>
+      <c r="I6" s="1522" t="n"/>
+      <c r="J6" s="1523" t="n"/>
+      <c r="K6" s="1523" t="n"/>
+      <c r="L6" s="1523" t="n"/>
+      <c r="M6" s="1521" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1485" t="n">
+      <c r="N6" s="1521" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1485" t="n"/>
-      <c r="P6" s="1488" t="n"/>
-      <c r="Q6" s="1485" t="n"/>
-      <c r="R6" s="1485" t="n"/>
-      <c r="S6" s="1485" t="n"/>
+      <c r="O6" s="1521" t="n"/>
+      <c r="P6" s="1524" t="n"/>
+      <c r="Q6" s="1521" t="n"/>
+      <c r="R6" s="1521" t="n"/>
+      <c r="S6" s="1521" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1484" t="n"/>
+      <c r="U6" s="1520" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -5650,39 +5776,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1489" t="inlineStr">
+      <c r="A7" s="1525" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1490" t="inlineStr">
+      <c r="B7" s="1526" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1490" t="inlineStr">
+      <c r="C7" s="1526" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1491" t="n"/>
-      <c r="E7" s="1491" t="n"/>
-      <c r="F7" s="1491" t="n"/>
-      <c r="G7" s="1491" t="n"/>
-      <c r="H7" s="1491" t="n"/>
-      <c r="I7" s="1492" t="n"/>
-      <c r="J7" s="1493" t="n"/>
-      <c r="K7" s="1493" t="n"/>
-      <c r="L7" s="1493" t="n"/>
-      <c r="M7" s="1491" t="n"/>
-      <c r="N7" s="1491" t="n"/>
-      <c r="O7" s="1491" t="n"/>
-      <c r="P7" s="1494" t="n"/>
-      <c r="Q7" s="1491" t="n"/>
-      <c r="R7" s="1491" t="n"/>
-      <c r="S7" s="1491" t="n"/>
+      <c r="D7" s="1527" t="n"/>
+      <c r="E7" s="1527" t="n"/>
+      <c r="F7" s="1527" t="n"/>
+      <c r="G7" s="1527" t="n"/>
+      <c r="H7" s="1527" t="n"/>
+      <c r="I7" s="1528" t="n"/>
+      <c r="J7" s="1529" t="n"/>
+      <c r="K7" s="1529" t="n"/>
+      <c r="L7" s="1529" t="n"/>
+      <c r="M7" s="1527" t="n"/>
+      <c r="N7" s="1527" t="n"/>
+      <c r="O7" s="1527" t="n"/>
+      <c r="P7" s="1530" t="n"/>
+      <c r="Q7" s="1527" t="n"/>
+      <c r="R7" s="1527" t="n"/>
+      <c r="S7" s="1527" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1490" t="n"/>
+      <c r="U7" s="1526" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5690,39 +5816,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1465" t="inlineStr">
+      <c r="A8" s="1501" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1466" t="inlineStr">
+      <c r="B8" s="1502" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1466" t="inlineStr">
+      <c r="C8" s="1502" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1467" t="n"/>
-      <c r="E8" s="1467" t="n"/>
-      <c r="F8" s="1467" t="n"/>
-      <c r="G8" s="1467" t="n"/>
-      <c r="H8" s="1467" t="n"/>
-      <c r="I8" s="1468" t="n"/>
-      <c r="J8" s="1469" t="n"/>
-      <c r="K8" s="1469" t="n"/>
-      <c r="L8" s="1469" t="n"/>
-      <c r="M8" s="1467" t="n"/>
-      <c r="N8" s="1467" t="n"/>
-      <c r="O8" s="1467" t="n"/>
-      <c r="P8" s="1470" t="n"/>
-      <c r="Q8" s="1467" t="n"/>
-      <c r="R8" s="1467" t="n"/>
-      <c r="S8" s="1467" t="n"/>
+      <c r="D8" s="1503" t="n"/>
+      <c r="E8" s="1503" t="n"/>
+      <c r="F8" s="1503" t="n"/>
+      <c r="G8" s="1503" t="n"/>
+      <c r="H8" s="1503" t="n"/>
+      <c r="I8" s="1504" t="n"/>
+      <c r="J8" s="1505" t="n"/>
+      <c r="K8" s="1505" t="n"/>
+      <c r="L8" s="1505" t="n"/>
+      <c r="M8" s="1503" t="n"/>
+      <c r="N8" s="1503" t="n"/>
+      <c r="O8" s="1503" t="n"/>
+      <c r="P8" s="1506" t="n"/>
+      <c r="Q8" s="1503" t="n"/>
+      <c r="R8" s="1503" t="n"/>
+      <c r="S8" s="1503" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1466" t="n"/>
+      <c r="U8" s="1502" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -5730,63 +5856,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1495" t="inlineStr">
+      <c r="A9" s="1531" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1496" t="inlineStr">
+      <c r="B9" s="1532" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1496" t="inlineStr">
+      <c r="C9" s="1532" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1497" t="n">
+      <c r="D9" s="1533" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1497" t="n">
+      <c r="E9" s="1533" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1497" t="n">
+      <c r="F9" s="1533" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1497" t="n">
+      <c r="G9" s="1533" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1497" t="n"/>
-      <c r="I9" s="1498" t="n"/>
-      <c r="J9" s="1499" t="n">
+      <c r="H9" s="1533" t="n"/>
+      <c r="I9" s="1534" t="n"/>
+      <c r="J9" s="1535" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1499" t="n">
+      <c r="K9" s="1535" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1499" t="inlineStr">
+      <c r="L9" s="1535" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1497" t="n"/>
-      <c r="N9" s="1497" t="n"/>
-      <c r="O9" s="1497" t="n">
+      <c r="M9" s="1533" t="n"/>
+      <c r="N9" s="1533" t="n"/>
+      <c r="O9" s="1533" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1500" t="n">
+      <c r="P9" s="1536" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1497" t="n"/>
-      <c r="R9" s="1497" t="n"/>
-      <c r="S9" s="1497" t="n"/>
+      <c r="Q9" s="1533" t="n"/>
+      <c r="R9" s="1533" t="n"/>
+      <c r="S9" s="1533" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1496" t="n"/>
+      <c r="U9" s="1532" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -5794,43 +5920,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1495" t="inlineStr">
+      <c r="A10" s="1531" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1496" t="inlineStr">
+      <c r="B10" s="1532" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1496" t="inlineStr">
+      <c r="C10" s="1532" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1497" t="n"/>
-      <c r="E10" s="1497" t="n"/>
-      <c r="F10" s="1497" t="n"/>
-      <c r="G10" s="1497" t="n"/>
-      <c r="H10" s="1497" t="n"/>
-      <c r="I10" s="1498" t="n"/>
-      <c r="J10" s="1499" t="n"/>
-      <c r="K10" s="1499" t="n"/>
-      <c r="L10" s="1499" t="inlineStr">
+      <c r="D10" s="1533" t="n"/>
+      <c r="E10" s="1533" t="n"/>
+      <c r="F10" s="1533" t="n"/>
+      <c r="G10" s="1533" t="n"/>
+      <c r="H10" s="1533" t="n"/>
+      <c r="I10" s="1534" t="n"/>
+      <c r="J10" s="1535" t="n"/>
+      <c r="K10" s="1535" t="n"/>
+      <c r="L10" s="1535" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1497" t="n"/>
-      <c r="N10" s="1497" t="n"/>
-      <c r="O10" s="1497" t="n"/>
-      <c r="P10" s="1500" t="n"/>
-      <c r="Q10" s="1497" t="n"/>
-      <c r="R10" s="1497" t="n"/>
-      <c r="S10" s="1497" t="n"/>
+      <c r="M10" s="1533" t="n"/>
+      <c r="N10" s="1533" t="n"/>
+      <c r="O10" s="1533" t="n"/>
+      <c r="P10" s="1536" t="n"/>
+      <c r="Q10" s="1533" t="n"/>
+      <c r="R10" s="1533" t="n"/>
+      <c r="S10" s="1533" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1496" t="n"/>
+      <c r="U10" s="1532" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -5838,43 +5964,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1495" t="inlineStr">
+      <c r="A11" s="1531" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1496" t="inlineStr">
+      <c r="B11" s="1532" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1496" t="inlineStr">
+      <c r="C11" s="1532" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1497" t="n"/>
-      <c r="E11" s="1497" t="n"/>
-      <c r="F11" s="1497" t="n"/>
-      <c r="G11" s="1497" t="n"/>
-      <c r="H11" s="1497" t="n"/>
-      <c r="I11" s="1498" t="n"/>
-      <c r="J11" s="1499" t="n"/>
-      <c r="K11" s="1499" t="n"/>
-      <c r="L11" s="1499" t="n"/>
-      <c r="M11" s="1497" t="n">
+      <c r="D11" s="1533" t="n"/>
+      <c r="E11" s="1533" t="n"/>
+      <c r="F11" s="1533" t="n"/>
+      <c r="G11" s="1533" t="n"/>
+      <c r="H11" s="1533" t="n"/>
+      <c r="I11" s="1534" t="n"/>
+      <c r="J11" s="1535" t="n"/>
+      <c r="K11" s="1535" t="n"/>
+      <c r="L11" s="1535" t="n"/>
+      <c r="M11" s="1533" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1497" t="n">
+      <c r="N11" s="1533" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1497" t="n"/>
-      <c r="P11" s="1500" t="n"/>
-      <c r="Q11" s="1497" t="n"/>
-      <c r="R11" s="1497" t="n"/>
-      <c r="S11" s="1497" t="n"/>
+      <c r="O11" s="1533" t="n"/>
+      <c r="P11" s="1536" t="n"/>
+      <c r="Q11" s="1533" t="n"/>
+      <c r="R11" s="1533" t="n"/>
+      <c r="S11" s="1533" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1496" t="n"/>
+      <c r="U11" s="1532" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -5882,39 +6008,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1471" t="inlineStr">
+      <c r="A12" s="1507" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1472" t="inlineStr">
+      <c r="B12" s="1508" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1472" t="inlineStr">
+      <c r="C12" s="1508" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1473" t="n"/>
-      <c r="E12" s="1473" t="n"/>
-      <c r="F12" s="1473" t="n"/>
-      <c r="G12" s="1473" t="n"/>
-      <c r="H12" s="1473" t="n"/>
-      <c r="I12" s="1474" t="n"/>
-      <c r="J12" s="1475" t="n"/>
-      <c r="K12" s="1475" t="n"/>
-      <c r="L12" s="1475" t="n"/>
-      <c r="M12" s="1473" t="n"/>
-      <c r="N12" s="1473" t="n"/>
-      <c r="O12" s="1473" t="n"/>
-      <c r="P12" s="1476" t="n"/>
-      <c r="Q12" s="1473" t="n"/>
-      <c r="R12" s="1473" t="n"/>
-      <c r="S12" s="1473" t="n"/>
+      <c r="D12" s="1509" t="n"/>
+      <c r="E12" s="1509" t="n"/>
+      <c r="F12" s="1509" t="n"/>
+      <c r="G12" s="1509" t="n"/>
+      <c r="H12" s="1509" t="n"/>
+      <c r="I12" s="1510" t="n"/>
+      <c r="J12" s="1511" t="n"/>
+      <c r="K12" s="1511" t="n"/>
+      <c r="L12" s="1511" t="n"/>
+      <c r="M12" s="1509" t="n"/>
+      <c r="N12" s="1509" t="n"/>
+      <c r="O12" s="1509" t="n"/>
+      <c r="P12" s="1512" t="n"/>
+      <c r="Q12" s="1509" t="n"/>
+      <c r="R12" s="1509" t="n"/>
+      <c r="S12" s="1509" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1472" t="n"/>
+      <c r="U12" s="1508" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5922,35 +6048,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1477" t="inlineStr">
+      <c r="A13" s="1513" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1478" t="n"/>
-      <c r="C13" s="1478" t="inlineStr">
+      <c r="B13" s="1514" t="n"/>
+      <c r="C13" s="1514" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1479" t="n"/>
-      <c r="E13" s="1479" t="n"/>
-      <c r="F13" s="1479" t="n"/>
-      <c r="G13" s="1479" t="n"/>
-      <c r="H13" s="1479" t="n"/>
-      <c r="I13" s="1480" t="n"/>
-      <c r="J13" s="1481" t="n"/>
-      <c r="K13" s="1481" t="n"/>
-      <c r="L13" s="1481" t="n"/>
-      <c r="M13" s="1479" t="n"/>
-      <c r="N13" s="1479" t="n"/>
-      <c r="O13" s="1479" t="n"/>
-      <c r="P13" s="1482" t="n"/>
-      <c r="Q13" s="1479" t="n"/>
-      <c r="R13" s="1479" t="n"/>
-      <c r="S13" s="1479" t="n"/>
+      <c r="D13" s="1515" t="n"/>
+      <c r="E13" s="1515" t="n"/>
+      <c r="F13" s="1515" t="n"/>
+      <c r="G13" s="1515" t="n"/>
+      <c r="H13" s="1515" t="n"/>
+      <c r="I13" s="1516" t="n"/>
+      <c r="J13" s="1517" t="n"/>
+      <c r="K13" s="1517" t="n"/>
+      <c r="L13" s="1517" t="n"/>
+      <c r="M13" s="1515" t="n"/>
+      <c r="N13" s="1515" t="n"/>
+      <c r="O13" s="1515" t="n"/>
+      <c r="P13" s="1518" t="n"/>
+      <c r="Q13" s="1515" t="n"/>
+      <c r="R13" s="1515" t="n"/>
+      <c r="S13" s="1515" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1478" t="n"/>
+      <c r="U13" s="1514" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -5958,53 +6084,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1483" t="inlineStr">
+      <c r="A14" s="1519" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1484" t="inlineStr">
+      <c r="B14" s="1520" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1484" t="inlineStr">
+      <c r="C14" s="1520" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1485" t="n"/>
-      <c r="E14" s="1485" t="n">
+      <c r="D14" s="1521" t="n"/>
+      <c r="E14" s="1521" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1485" t="n">
+      <c r="F14" s="1521" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1485" t="n">
+      <c r="G14" s="1521" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1485" t="n"/>
-      <c r="I14" s="1486" t="n"/>
-      <c r="J14" s="1487" t="n"/>
-      <c r="K14" s="1487" t="n"/>
-      <c r="L14" s="1487" t="n"/>
-      <c r="M14" s="1485" t="n"/>
-      <c r="N14" s="1485" t="n"/>
-      <c r="O14" s="1485" t="n">
+      <c r="H14" s="1521" t="n"/>
+      <c r="I14" s="1522" t="n"/>
+      <c r="J14" s="1523" t="n"/>
+      <c r="K14" s="1523" t="n"/>
+      <c r="L14" s="1523" t="n"/>
+      <c r="M14" s="1521" t="n"/>
+      <c r="N14" s="1521" t="n"/>
+      <c r="O14" s="1521" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1488" t="n">
+      <c r="P14" s="1524" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1485" t="n"/>
-      <c r="R14" s="1485" t="n"/>
-      <c r="S14" s="1485" t="n"/>
+      <c r="Q14" s="1521" t="n"/>
+      <c r="R14" s="1521" t="n"/>
+      <c r="S14" s="1521" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1484" t="n"/>
+      <c r="U14" s="1520" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -6012,43 +6138,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1483" t="inlineStr">
+      <c r="A15" s="1519" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1484" t="inlineStr">
+      <c r="B15" s="1520" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1484" t="inlineStr">
+      <c r="C15" s="1520" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1485" t="n"/>
-      <c r="E15" s="1485" t="n"/>
-      <c r="F15" s="1485" t="n"/>
-      <c r="G15" s="1485" t="n"/>
-      <c r="H15" s="1485" t="n"/>
-      <c r="I15" s="1486" t="n"/>
-      <c r="J15" s="1487" t="n"/>
-      <c r="K15" s="1487" t="n"/>
-      <c r="L15" s="1487" t="n"/>
-      <c r="M15" s="1485" t="n">
+      <c r="D15" s="1521" t="n"/>
+      <c r="E15" s="1521" t="n"/>
+      <c r="F15" s="1521" t="n"/>
+      <c r="G15" s="1521" t="n"/>
+      <c r="H15" s="1521" t="n"/>
+      <c r="I15" s="1522" t="n"/>
+      <c r="J15" s="1523" t="n"/>
+      <c r="K15" s="1523" t="n"/>
+      <c r="L15" s="1523" t="n"/>
+      <c r="M15" s="1521" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1485" t="n">
+      <c r="N15" s="1521" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1485" t="n"/>
-      <c r="P15" s="1488" t="n"/>
-      <c r="Q15" s="1485" t="n"/>
-      <c r="R15" s="1485" t="n"/>
-      <c r="S15" s="1485" t="n"/>
+      <c r="O15" s="1521" t="n"/>
+      <c r="P15" s="1524" t="n"/>
+      <c r="Q15" s="1521" t="n"/>
+      <c r="R15" s="1521" t="n"/>
+      <c r="S15" s="1521" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1484" t="n"/>
+      <c r="U15" s="1520" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -6056,39 +6182,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1489" t="inlineStr">
+      <c r="A16" s="1525" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1490" t="inlineStr">
+      <c r="B16" s="1526" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1490" t="inlineStr">
+      <c r="C16" s="1526" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1491" t="n"/>
-      <c r="E16" s="1491" t="n"/>
-      <c r="F16" s="1491" t="n"/>
-      <c r="G16" s="1491" t="n"/>
-      <c r="H16" s="1491" t="n"/>
-      <c r="I16" s="1492" t="n"/>
-      <c r="J16" s="1493" t="n"/>
-      <c r="K16" s="1493" t="n"/>
-      <c r="L16" s="1493" t="n"/>
-      <c r="M16" s="1491" t="n"/>
-      <c r="N16" s="1491" t="n"/>
-      <c r="O16" s="1491" t="n"/>
-      <c r="P16" s="1494" t="n"/>
-      <c r="Q16" s="1491" t="n"/>
-      <c r="R16" s="1491" t="n"/>
-      <c r="S16" s="1491" t="n"/>
+      <c r="D16" s="1527" t="n"/>
+      <c r="E16" s="1527" t="n"/>
+      <c r="F16" s="1527" t="n"/>
+      <c r="G16" s="1527" t="n"/>
+      <c r="H16" s="1527" t="n"/>
+      <c r="I16" s="1528" t="n"/>
+      <c r="J16" s="1529" t="n"/>
+      <c r="K16" s="1529" t="n"/>
+      <c r="L16" s="1529" t="n"/>
+      <c r="M16" s="1527" t="n"/>
+      <c r="N16" s="1527" t="n"/>
+      <c r="O16" s="1527" t="n"/>
+      <c r="P16" s="1530" t="n"/>
+      <c r="Q16" s="1527" t="n"/>
+      <c r="R16" s="1527" t="n"/>
+      <c r="S16" s="1527" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1490" t="n"/>
+      <c r="U16" s="1526" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -6096,39 +6222,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1465" t="inlineStr">
+      <c r="A17" s="1501" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1466" t="inlineStr">
+      <c r="B17" s="1502" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1466" t="inlineStr">
+      <c r="C17" s="1502" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1467" t="n"/>
-      <c r="E17" s="1467" t="n"/>
-      <c r="F17" s="1467" t="n"/>
-      <c r="G17" s="1467" t="n"/>
-      <c r="H17" s="1467" t="n"/>
-      <c r="I17" s="1468" t="n"/>
-      <c r="J17" s="1469" t="n"/>
-      <c r="K17" s="1469" t="n"/>
-      <c r="L17" s="1469" t="n"/>
-      <c r="M17" s="1467" t="n"/>
-      <c r="N17" s="1467" t="n"/>
-      <c r="O17" s="1467" t="n"/>
-      <c r="P17" s="1470" t="n"/>
-      <c r="Q17" s="1467" t="n"/>
-      <c r="R17" s="1467" t="n"/>
-      <c r="S17" s="1467" t="n"/>
+      <c r="D17" s="1503" t="n"/>
+      <c r="E17" s="1503" t="n"/>
+      <c r="F17" s="1503" t="n"/>
+      <c r="G17" s="1503" t="n"/>
+      <c r="H17" s="1503" t="n"/>
+      <c r="I17" s="1504" t="n"/>
+      <c r="J17" s="1505" t="n"/>
+      <c r="K17" s="1505" t="n"/>
+      <c r="L17" s="1505" t="n"/>
+      <c r="M17" s="1503" t="n"/>
+      <c r="N17" s="1503" t="n"/>
+      <c r="O17" s="1503" t="n"/>
+      <c r="P17" s="1506" t="n"/>
+      <c r="Q17" s="1503" t="n"/>
+      <c r="R17" s="1503" t="n"/>
+      <c r="S17" s="1503" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1466" t="n"/>
+      <c r="U17" s="1502" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -6136,53 +6262,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1495" t="inlineStr">
+      <c r="A18" s="1531" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1496" t="inlineStr">
+      <c r="B18" s="1532" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1496" t="inlineStr">
+      <c r="C18" s="1532" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1497" t="n"/>
-      <c r="E18" s="1497" t="n">
+      <c r="D18" s="1533" t="n"/>
+      <c r="E18" s="1533" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1497" t="n">
+      <c r="F18" s="1533" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1497" t="n">
+      <c r="G18" s="1533" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1497" t="n"/>
-      <c r="I18" s="1498" t="n"/>
-      <c r="J18" s="1499" t="n"/>
-      <c r="K18" s="1499" t="n"/>
-      <c r="L18" s="1499" t="n"/>
-      <c r="M18" s="1497" t="n"/>
-      <c r="N18" s="1497" t="n"/>
-      <c r="O18" s="1497" t="n">
+      <c r="H18" s="1533" t="n"/>
+      <c r="I18" s="1534" t="n"/>
+      <c r="J18" s="1535" t="n"/>
+      <c r="K18" s="1535" t="n"/>
+      <c r="L18" s="1535" t="n"/>
+      <c r="M18" s="1533" t="n"/>
+      <c r="N18" s="1533" t="n"/>
+      <c r="O18" s="1533" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1500" t="n">
+      <c r="P18" s="1536" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1497" t="n"/>
-      <c r="R18" s="1497" t="n"/>
-      <c r="S18" s="1497" t="n"/>
+      <c r="Q18" s="1533" t="n"/>
+      <c r="R18" s="1533" t="n"/>
+      <c r="S18" s="1533" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1496" t="n"/>
+      <c r="U18" s="1532" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -6190,47 +6316,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1495" t="inlineStr">
+      <c r="A19" s="1531" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1496" t="inlineStr">
+      <c r="B19" s="1532" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1496" t="inlineStr">
+      <c r="C19" s="1532" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1497" t="n"/>
-      <c r="E19" s="1497" t="n"/>
-      <c r="F19" s="1497" t="n"/>
-      <c r="G19" s="1497" t="n"/>
-      <c r="H19" s="1497" t="n"/>
-      <c r="I19" s="1498" t="n"/>
-      <c r="J19" s="1499" t="n"/>
-      <c r="K19" s="1499" t="n"/>
-      <c r="L19" s="1499" t="n"/>
-      <c r="M19" s="1497" t="n">
+      <c r="D19" s="1533" t="n"/>
+      <c r="E19" s="1533" t="n"/>
+      <c r="F19" s="1533" t="n"/>
+      <c r="G19" s="1533" t="n"/>
+      <c r="H19" s="1533" t="n"/>
+      <c r="I19" s="1534" t="n"/>
+      <c r="J19" s="1535" t="n"/>
+      <c r="K19" s="1535" t="n"/>
+      <c r="L19" s="1535" t="n"/>
+      <c r="M19" s="1533" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1497" t="n">
+      <c r="N19" s="1533" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1497" t="n"/>
-      <c r="P19" s="1500" t="n"/>
-      <c r="Q19" s="1497" t="n"/>
-      <c r="R19" s="1497" t="n"/>
-      <c r="S19" s="1497" t="n"/>
+      <c r="O19" s="1533" t="n"/>
+      <c r="P19" s="1536" t="n"/>
+      <c r="Q19" s="1533" t="n"/>
+      <c r="R19" s="1533" t="n"/>
+      <c r="S19" s="1533" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1496" t="n"/>
+      <c r="U19" s="1532" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -6238,43 +6364,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1495" t="inlineStr">
+      <c r="A20" s="1531" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1496" t="inlineStr">
+      <c r="B20" s="1532" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1496" t="inlineStr">
+      <c r="C20" s="1532" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1497" t="n"/>
-      <c r="E20" s="1497" t="n"/>
-      <c r="F20" s="1497" t="n"/>
-      <c r="G20" s="1497" t="n"/>
-      <c r="H20" s="1497" t="n"/>
-      <c r="I20" s="1498" t="n"/>
-      <c r="J20" s="1499" t="n"/>
-      <c r="K20" s="1499" t="n"/>
-      <c r="L20" s="1499" t="n"/>
-      <c r="M20" s="1497" t="n"/>
-      <c r="N20" s="1497" t="n"/>
-      <c r="O20" s="1497" t="n"/>
-      <c r="P20" s="1500" t="n"/>
-      <c r="Q20" s="1497" t="n"/>
-      <c r="R20" s="1497" t="n"/>
-      <c r="S20" s="1497" t="n"/>
+      <c r="D20" s="1533" t="n"/>
+      <c r="E20" s="1533" t="n"/>
+      <c r="F20" s="1533" t="n"/>
+      <c r="G20" s="1533" t="n"/>
+      <c r="H20" s="1533" t="n"/>
+      <c r="I20" s="1534" t="n"/>
+      <c r="J20" s="1535" t="n"/>
+      <c r="K20" s="1535" t="n"/>
+      <c r="L20" s="1535" t="n"/>
+      <c r="M20" s="1533" t="n"/>
+      <c r="N20" s="1533" t="n"/>
+      <c r="O20" s="1533" t="n"/>
+      <c r="P20" s="1536" t="n"/>
+      <c r="Q20" s="1533" t="n"/>
+      <c r="R20" s="1533" t="n"/>
+      <c r="S20" s="1533" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1496" t="n"/>
+      <c r="U20" s="1532" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -6282,39 +6408,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1471" t="inlineStr">
+      <c r="A21" s="1507" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1472" t="inlineStr">
+      <c r="B21" s="1508" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1472" t="inlineStr">
+      <c r="C21" s="1508" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1473" t="n"/>
-      <c r="E21" s="1473" t="n"/>
-      <c r="F21" s="1473" t="n"/>
-      <c r="G21" s="1473" t="n"/>
-      <c r="H21" s="1473" t="n"/>
-      <c r="I21" s="1474" t="n"/>
-      <c r="J21" s="1475" t="n"/>
-      <c r="K21" s="1475" t="n"/>
-      <c r="L21" s="1475" t="n"/>
-      <c r="M21" s="1473" t="n"/>
-      <c r="N21" s="1473" t="n"/>
-      <c r="O21" s="1473" t="n"/>
-      <c r="P21" s="1476" t="n"/>
-      <c r="Q21" s="1473" t="n"/>
-      <c r="R21" s="1473" t="n"/>
-      <c r="S21" s="1473" t="n"/>
+      <c r="D21" s="1509" t="n"/>
+      <c r="E21" s="1509" t="n"/>
+      <c r="F21" s="1509" t="n"/>
+      <c r="G21" s="1509" t="n"/>
+      <c r="H21" s="1509" t="n"/>
+      <c r="I21" s="1510" t="n"/>
+      <c r="J21" s="1511" t="n"/>
+      <c r="K21" s="1511" t="n"/>
+      <c r="L21" s="1511" t="n"/>
+      <c r="M21" s="1509" t="n"/>
+      <c r="N21" s="1509" t="n"/>
+      <c r="O21" s="1509" t="n"/>
+      <c r="P21" s="1512" t="n"/>
+      <c r="Q21" s="1509" t="n"/>
+      <c r="R21" s="1509" t="n"/>
+      <c r="S21" s="1509" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1472" t="n"/>
+      <c r="U21" s="1508" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -6322,39 +6448,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1477" t="inlineStr">
+      <c r="A22" s="1513" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1478" t="inlineStr">
+      <c r="B22" s="1514" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1478" t="inlineStr">
+      <c r="C22" s="1514" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1479" t="n"/>
-      <c r="E22" s="1479" t="n"/>
-      <c r="F22" s="1479" t="n"/>
-      <c r="G22" s="1479" t="n"/>
-      <c r="H22" s="1479" t="n"/>
-      <c r="I22" s="1480" t="n"/>
-      <c r="J22" s="1481" t="n"/>
-      <c r="K22" s="1481" t="n"/>
-      <c r="L22" s="1481" t="n"/>
-      <c r="M22" s="1479" t="n"/>
-      <c r="N22" s="1479" t="n"/>
-      <c r="O22" s="1479" t="n"/>
-      <c r="P22" s="1482" t="n"/>
-      <c r="Q22" s="1479" t="n"/>
-      <c r="R22" s="1479" t="n"/>
-      <c r="S22" s="1479" t="n"/>
+      <c r="D22" s="1515" t="n"/>
+      <c r="E22" s="1515" t="n"/>
+      <c r="F22" s="1515" t="n"/>
+      <c r="G22" s="1515" t="n"/>
+      <c r="H22" s="1515" t="n"/>
+      <c r="I22" s="1516" t="n"/>
+      <c r="J22" s="1517" t="n"/>
+      <c r="K22" s="1517" t="n"/>
+      <c r="L22" s="1517" t="n"/>
+      <c r="M22" s="1515" t="n"/>
+      <c r="N22" s="1515" t="n"/>
+      <c r="O22" s="1515" t="n"/>
+      <c r="P22" s="1518" t="n"/>
+      <c r="Q22" s="1515" t="n"/>
+      <c r="R22" s="1515" t="n"/>
+      <c r="S22" s="1515" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1478" t="n"/>
+      <c r="U22" s="1514" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -6362,53 +6488,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1483" t="inlineStr">
+      <c r="A23" s="1519" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1484" t="inlineStr">
+      <c r="B23" s="1520" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1484" t="inlineStr">
+      <c r="C23" s="1520" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1485" t="n"/>
-      <c r="E23" s="1485" t="n">
+      <c r="D23" s="1521" t="n"/>
+      <c r="E23" s="1521" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1485" t="n">
+      <c r="F23" s="1521" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1485" t="n">
+      <c r="G23" s="1521" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1485" t="n"/>
-      <c r="I23" s="1486" t="n"/>
-      <c r="J23" s="1487" t="n"/>
-      <c r="K23" s="1487" t="n"/>
-      <c r="L23" s="1487" t="n"/>
-      <c r="M23" s="1485" t="n"/>
-      <c r="N23" s="1485" t="n"/>
-      <c r="O23" s="1485" t="n">
+      <c r="H23" s="1521" t="n"/>
+      <c r="I23" s="1522" t="n"/>
+      <c r="J23" s="1523" t="n"/>
+      <c r="K23" s="1523" t="n"/>
+      <c r="L23" s="1523" t="n"/>
+      <c r="M23" s="1521" t="n"/>
+      <c r="N23" s="1521" t="n"/>
+      <c r="O23" s="1521" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1488" t="n">
+      <c r="P23" s="1524" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1485" t="n"/>
-      <c r="R23" s="1485" t="n"/>
-      <c r="S23" s="1485" t="n"/>
+      <c r="Q23" s="1521" t="n"/>
+      <c r="R23" s="1521" t="n"/>
+      <c r="S23" s="1521" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1484" t="n"/>
+      <c r="U23" s="1520" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -6416,47 +6542,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1489" t="inlineStr">
+      <c r="A24" s="1525" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1490" t="inlineStr">
+      <c r="B24" s="1526" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1490" t="inlineStr">
+      <c r="C24" s="1526" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1491" t="n"/>
-      <c r="E24" s="1491" t="n"/>
-      <c r="F24" s="1491" t="n"/>
-      <c r="G24" s="1491" t="n"/>
-      <c r="H24" s="1491" t="n"/>
-      <c r="I24" s="1492" t="n"/>
-      <c r="J24" s="1493" t="n"/>
-      <c r="K24" s="1493" t="n"/>
-      <c r="L24" s="1493" t="n"/>
-      <c r="M24" s="1491" t="n">
+      <c r="D24" s="1527" t="n"/>
+      <c r="E24" s="1527" t="n"/>
+      <c r="F24" s="1527" t="n"/>
+      <c r="G24" s="1527" t="n"/>
+      <c r="H24" s="1527" t="n"/>
+      <c r="I24" s="1528" t="n"/>
+      <c r="J24" s="1529" t="n"/>
+      <c r="K24" s="1529" t="n"/>
+      <c r="L24" s="1529" t="n"/>
+      <c r="M24" s="1527" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1491" t="n">
+      <c r="N24" s="1527" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1491" t="n"/>
-      <c r="P24" s="1494" t="n"/>
-      <c r="Q24" s="1491" t="n"/>
-      <c r="R24" s="1491" t="n"/>
-      <c r="S24" s="1491" t="n"/>
+      <c r="O24" s="1527" t="n"/>
+      <c r="P24" s="1530" t="n"/>
+      <c r="Q24" s="1527" t="n"/>
+      <c r="R24" s="1527" t="n"/>
+      <c r="S24" s="1527" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1490" t="n"/>
+      <c r="U24" s="1526" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -6464,61 +6590,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1465" t="inlineStr">
+      <c r="A25" s="1501" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1466" t="inlineStr">
+      <c r="B25" s="1502" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1466" t="inlineStr">
+      <c r="C25" s="1502" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1467" t="n">
+      <c r="D25" s="1503" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1467" t="n">
+      <c r="E25" s="1503" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1467" t="n">
+      <c r="F25" s="1503" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1467" t="n">
+      <c r="G25" s="1503" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1467" t="n"/>
-      <c r="I25" s="1468" t="n"/>
-      <c r="J25" s="1469" t="n">
+      <c r="H25" s="1503" t="n"/>
+      <c r="I25" s="1504" t="n"/>
+      <c r="J25" s="1505" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1469" t="n">
+      <c r="K25" s="1505" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1469" t="n">
+      <c r="L25" s="1505" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1467" t="n"/>
-      <c r="N25" s="1467" t="n"/>
-      <c r="O25" s="1467" t="n">
+      <c r="M25" s="1503" t="n"/>
+      <c r="N25" s="1503" t="n"/>
+      <c r="O25" s="1503" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1470" t="n">
+      <c r="P25" s="1506" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1467" t="n"/>
-      <c r="R25" s="1467" t="n"/>
-      <c r="S25" s="1467" t="n"/>
+      <c r="Q25" s="1503" t="n"/>
+      <c r="R25" s="1503" t="n"/>
+      <c r="S25" s="1503" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1466" t="n"/>
+      <c r="U25" s="1502" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -6526,47 +6652,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1471" t="inlineStr">
+      <c r="A26" s="1507" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1472" t="inlineStr">
+      <c r="B26" s="1508" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1472" t="inlineStr">
+      <c r="C26" s="1508" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1473" t="n"/>
-      <c r="E26" s="1473" t="n"/>
-      <c r="F26" s="1473" t="n"/>
-      <c r="G26" s="1473" t="n"/>
-      <c r="H26" s="1473" t="n"/>
-      <c r="I26" s="1474" t="n"/>
-      <c r="J26" s="1475" t="n"/>
-      <c r="K26" s="1475" t="n"/>
-      <c r="L26" s="1475" t="n"/>
-      <c r="M26" s="1473" t="n">
+      <c r="D26" s="1509" t="n"/>
+      <c r="E26" s="1509" t="n"/>
+      <c r="F26" s="1509" t="n"/>
+      <c r="G26" s="1509" t="n"/>
+      <c r="H26" s="1509" t="n"/>
+      <c r="I26" s="1510" t="n"/>
+      <c r="J26" s="1511" t="n"/>
+      <c r="K26" s="1511" t="n"/>
+      <c r="L26" s="1511" t="n"/>
+      <c r="M26" s="1509" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1473" t="n">
+      <c r="N26" s="1509" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1473" t="n"/>
-      <c r="P26" s="1476" t="n"/>
-      <c r="Q26" s="1473" t="n"/>
-      <c r="R26" s="1473" t="n"/>
-      <c r="S26" s="1473" t="n"/>
+      <c r="O26" s="1509" t="n"/>
+      <c r="P26" s="1512" t="n"/>
+      <c r="Q26" s="1509" t="n"/>
+      <c r="R26" s="1509" t="n"/>
+      <c r="S26" s="1509" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1472" t="n"/>
+      <c r="U26" s="1508" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -6574,53 +6700,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1477" t="inlineStr">
+      <c r="A27" s="1513" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1478" t="inlineStr">
+      <c r="B27" s="1514" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1478" t="inlineStr">
+      <c r="C27" s="1514" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1479" t="n"/>
-      <c r="E27" s="1479" t="n">
+      <c r="D27" s="1515" t="n"/>
+      <c r="E27" s="1515" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1479" t="n">
+      <c r="F27" s="1515" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1479" t="n">
+      <c r="G27" s="1515" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1479" t="n"/>
-      <c r="I27" s="1480" t="n"/>
-      <c r="J27" s="1481" t="n"/>
-      <c r="K27" s="1481" t="n"/>
-      <c r="L27" s="1481" t="n"/>
-      <c r="M27" s="1479" t="n"/>
-      <c r="N27" s="1479" t="n"/>
-      <c r="O27" s="1479" t="n">
+      <c r="H27" s="1515" t="n"/>
+      <c r="I27" s="1516" t="n"/>
+      <c r="J27" s="1517" t="n"/>
+      <c r="K27" s="1517" t="n"/>
+      <c r="L27" s="1517" t="n"/>
+      <c r="M27" s="1515" t="n"/>
+      <c r="N27" s="1515" t="n"/>
+      <c r="O27" s="1515" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1482" t="n">
+      <c r="P27" s="1518" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1479" t="n"/>
-      <c r="R27" s="1479" t="n"/>
-      <c r="S27" s="1479" t="n"/>
+      <c r="Q27" s="1515" t="n"/>
+      <c r="R27" s="1515" t="n"/>
+      <c r="S27" s="1515" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1478" t="n"/>
+      <c r="U27" s="1514" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -6628,47 +6754,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1489" t="inlineStr">
+      <c r="A28" s="1525" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1490" t="inlineStr">
+      <c r="B28" s="1526" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1490" t="inlineStr">
+      <c r="C28" s="1526" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1491" t="n"/>
-      <c r="E28" s="1491" t="n"/>
-      <c r="F28" s="1491" t="n"/>
-      <c r="G28" s="1491" t="n"/>
-      <c r="H28" s="1491" t="n"/>
-      <c r="I28" s="1492" t="n"/>
-      <c r="J28" s="1493" t="n"/>
-      <c r="K28" s="1493" t="n"/>
-      <c r="L28" s="1493" t="n"/>
-      <c r="M28" s="1491" t="n">
+      <c r="D28" s="1527" t="n"/>
+      <c r="E28" s="1527" t="n"/>
+      <c r="F28" s="1527" t="n"/>
+      <c r="G28" s="1527" t="n"/>
+      <c r="H28" s="1527" t="n"/>
+      <c r="I28" s="1528" t="n"/>
+      <c r="J28" s="1529" t="n"/>
+      <c r="K28" s="1529" t="n"/>
+      <c r="L28" s="1529" t="n"/>
+      <c r="M28" s="1527" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1491" t="n">
+      <c r="N28" s="1527" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1491" t="n"/>
-      <c r="P28" s="1494" t="n"/>
-      <c r="Q28" s="1491" t="n"/>
-      <c r="R28" s="1491" t="n"/>
-      <c r="S28" s="1491" t="n"/>
+      <c r="O28" s="1527" t="n"/>
+      <c r="P28" s="1530" t="n"/>
+      <c r="Q28" s="1527" t="n"/>
+      <c r="R28" s="1527" t="n"/>
+      <c r="S28" s="1527" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1490" t="n"/>
+      <c r="U28" s="1526" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -6676,53 +6802,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1465" t="inlineStr">
+      <c r="A29" s="1501" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1466" t="inlineStr">
+      <c r="B29" s="1502" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1466" t="inlineStr">
+      <c r="C29" s="1502" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1467" t="n"/>
-      <c r="E29" s="1467" t="n">
+      <c r="D29" s="1503" t="n"/>
+      <c r="E29" s="1503" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1467" t="n">
+      <c r="F29" s="1503" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1467" t="n">
+      <c r="G29" s="1503" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1467" t="n"/>
-      <c r="I29" s="1468" t="n"/>
-      <c r="J29" s="1469" t="n"/>
-      <c r="K29" s="1469" t="n"/>
-      <c r="L29" s="1469" t="n"/>
-      <c r="M29" s="1467" t="n"/>
-      <c r="N29" s="1467" t="n"/>
-      <c r="O29" s="1467" t="n">
+      <c r="H29" s="1503" t="n"/>
+      <c r="I29" s="1504" t="n"/>
+      <c r="J29" s="1505" t="n"/>
+      <c r="K29" s="1505" t="n"/>
+      <c r="L29" s="1505" t="n"/>
+      <c r="M29" s="1503" t="n"/>
+      <c r="N29" s="1503" t="n"/>
+      <c r="O29" s="1503" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1470" t="n">
+      <c r="P29" s="1506" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1467" t="n"/>
-      <c r="R29" s="1467" t="n"/>
-      <c r="S29" s="1467" t="n"/>
+      <c r="Q29" s="1503" t="n"/>
+      <c r="R29" s="1503" t="n"/>
+      <c r="S29" s="1503" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1466" t="n"/>
+      <c r="U29" s="1502" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -6730,43 +6856,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1471" t="inlineStr">
+      <c r="A30" s="1507" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1472" t="inlineStr">
+      <c r="B30" s="1508" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1472" t="inlineStr">
+      <c r="C30" s="1508" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1473" t="n"/>
-      <c r="E30" s="1473" t="n"/>
-      <c r="F30" s="1473" t="n"/>
-      <c r="G30" s="1473" t="n"/>
-      <c r="H30" s="1473" t="n"/>
-      <c r="I30" s="1474" t="n"/>
-      <c r="J30" s="1475" t="n"/>
-      <c r="K30" s="1475" t="n"/>
-      <c r="L30" s="1475" t="n"/>
-      <c r="M30" s="1473" t="n"/>
-      <c r="N30" s="1473" t="n"/>
-      <c r="O30" s="1473" t="n"/>
-      <c r="P30" s="1476" t="n"/>
-      <c r="Q30" s="1473" t="n"/>
-      <c r="R30" s="1473" t="n"/>
-      <c r="S30" s="1473" t="n"/>
+      <c r="D30" s="1509" t="n"/>
+      <c r="E30" s="1509" t="n"/>
+      <c r="F30" s="1509" t="n"/>
+      <c r="G30" s="1509" t="n"/>
+      <c r="H30" s="1509" t="n"/>
+      <c r="I30" s="1510" t="n"/>
+      <c r="J30" s="1511" t="n"/>
+      <c r="K30" s="1511" t="n"/>
+      <c r="L30" s="1511" t="n"/>
+      <c r="M30" s="1509" t="n"/>
+      <c r="N30" s="1509" t="n"/>
+      <c r="O30" s="1509" t="n"/>
+      <c r="P30" s="1512" t="n"/>
+      <c r="Q30" s="1509" t="n"/>
+      <c r="R30" s="1509" t="n"/>
+      <c r="S30" s="1509" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1472" t="n"/>
+      <c r="U30" s="1508" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -6774,53 +6900,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1477" t="inlineStr">
+      <c r="A31" s="1513" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1478" t="inlineStr">
+      <c r="B31" s="1514" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1478" t="inlineStr">
+      <c r="C31" s="1514" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1479" t="n"/>
-      <c r="E31" s="1479" t="n">
+      <c r="D31" s="1515" t="n"/>
+      <c r="E31" s="1515" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1479" t="n">
+      <c r="F31" s="1515" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1479" t="n">
+      <c r="G31" s="1515" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1479" t="n"/>
-      <c r="I31" s="1480" t="n"/>
-      <c r="J31" s="1481" t="n"/>
-      <c r="K31" s="1481" t="n"/>
-      <c r="L31" s="1481" t="n"/>
-      <c r="M31" s="1479" t="n"/>
-      <c r="N31" s="1479" t="n"/>
-      <c r="O31" s="1479" t="n">
+      <c r="H31" s="1515" t="n"/>
+      <c r="I31" s="1516" t="n"/>
+      <c r="J31" s="1517" t="n"/>
+      <c r="K31" s="1517" t="n"/>
+      <c r="L31" s="1517" t="n"/>
+      <c r="M31" s="1515" t="n"/>
+      <c r="N31" s="1515" t="n"/>
+      <c r="O31" s="1515" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1482" t="n">
+      <c r="P31" s="1518" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1479" t="n"/>
-      <c r="R31" s="1479" t="n"/>
-      <c r="S31" s="1479" t="n"/>
+      <c r="Q31" s="1515" t="n"/>
+      <c r="R31" s="1515" t="n"/>
+      <c r="S31" s="1515" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1478" t="inlineStr">
+      <c r="U31" s="1514" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -6832,49 +6958,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1489" t="inlineStr">
+      <c r="A32" s="1525" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1490" t="inlineStr">
+      <c r="B32" s="1526" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1490" t="inlineStr">
+      <c r="C32" s="1526" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1491" t="n"/>
-      <c r="E32" s="1491" t="n"/>
-      <c r="F32" s="1491" t="n"/>
-      <c r="G32" s="1491" t="n"/>
-      <c r="H32" s="1491" t="n">
+      <c r="D32" s="1527" t="n"/>
+      <c r="E32" s="1527" t="n"/>
+      <c r="F32" s="1527" t="n"/>
+      <c r="G32" s="1527" t="n"/>
+      <c r="H32" s="1527" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1492" t="n"/>
-      <c r="J32" s="1493" t="n"/>
-      <c r="K32" s="1493" t="n"/>
-      <c r="L32" s="1493" t="n"/>
-      <c r="M32" s="1491" t="n">
+      <c r="I32" s="1528" t="n"/>
+      <c r="J32" s="1529" t="n"/>
+      <c r="K32" s="1529" t="n"/>
+      <c r="L32" s="1529" t="n"/>
+      <c r="M32" s="1527" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1491" t="n">
+      <c r="N32" s="1527" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1491" t="n"/>
-      <c r="P32" s="1494" t="n"/>
-      <c r="Q32" s="1491" t="n"/>
-      <c r="R32" s="1491" t="n"/>
-      <c r="S32" s="1491" t="n"/>
+      <c r="O32" s="1527" t="n"/>
+      <c r="P32" s="1530" t="n"/>
+      <c r="Q32" s="1527" t="n"/>
+      <c r="R32" s="1527" t="n"/>
+      <c r="S32" s="1527" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1490" t="n"/>
+      <c r="U32" s="1526" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -6882,57 +7008,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1465" t="inlineStr">
+      <c r="A33" s="1501" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1466" t="inlineStr">
+      <c r="B33" s="1502" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1466" t="inlineStr">
+      <c r="C33" s="1502" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1467" t="n"/>
-      <c r="E33" s="1467" t="n">
+      <c r="D33" s="1503" t="n"/>
+      <c r="E33" s="1503" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1467" t="n">
+      <c r="F33" s="1503" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1467" t="n">
+      <c r="G33" s="1503" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1467" t="n"/>
-      <c r="I33" s="1468" t="n">
+      <c r="H33" s="1503" t="n"/>
+      <c r="I33" s="1504" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1469" t="n"/>
-      <c r="K33" s="1469" t="n"/>
-      <c r="L33" s="1469" t="n"/>
-      <c r="M33" s="1467" t="n"/>
-      <c r="N33" s="1467" t="n"/>
-      <c r="O33" s="1467" t="n">
+      <c r="J33" s="1505" t="n"/>
+      <c r="K33" s="1505" t="n"/>
+      <c r="L33" s="1505" t="n"/>
+      <c r="M33" s="1503" t="n"/>
+      <c r="N33" s="1503" t="n"/>
+      <c r="O33" s="1503" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1470" t="n">
+      <c r="P33" s="1506" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1467" t="n"/>
-      <c r="R33" s="1467" t="n">
+      <c r="Q33" s="1503" t="n"/>
+      <c r="R33" s="1503" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1467" t="n"/>
+      <c r="S33" s="1503" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1466" t="inlineStr">
+      <c r="U33" s="1502" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -6944,49 +7070,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1471" t="inlineStr">
+      <c r="A34" s="1507" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1472" t="inlineStr">
+      <c r="B34" s="1508" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1472" t="inlineStr">
+      <c r="C34" s="1508" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1473" t="n"/>
-      <c r="E34" s="1473" t="n"/>
-      <c r="F34" s="1473" t="n"/>
-      <c r="G34" s="1473" t="n"/>
-      <c r="H34" s="1473" t="n">
+      <c r="D34" s="1509" t="n"/>
+      <c r="E34" s="1509" t="n"/>
+      <c r="F34" s="1509" t="n"/>
+      <c r="G34" s="1509" t="n"/>
+      <c r="H34" s="1509" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1474" t="n"/>
-      <c r="J34" s="1475" t="n"/>
-      <c r="K34" s="1475" t="n"/>
-      <c r="L34" s="1475" t="n"/>
-      <c r="M34" s="1473" t="n">
+      <c r="I34" s="1510" t="n"/>
+      <c r="J34" s="1511" t="n"/>
+      <c r="K34" s="1511" t="n"/>
+      <c r="L34" s="1511" t="n"/>
+      <c r="M34" s="1509" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1473" t="n">
+      <c r="N34" s="1509" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1473" t="n"/>
-      <c r="P34" s="1476" t="n"/>
-      <c r="Q34" s="1473" t="n"/>
-      <c r="R34" s="1473" t="n"/>
-      <c r="S34" s="1473" t="n"/>
+      <c r="O34" s="1509" t="n"/>
+      <c r="P34" s="1512" t="n"/>
+      <c r="Q34" s="1509" t="n"/>
+      <c r="R34" s="1509" t="n"/>
+      <c r="S34" s="1509" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1472" t="n"/>
+      <c r="U34" s="1508" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -6994,57 +7120,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1477" t="inlineStr">
+      <c r="A35" s="1513" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1478" t="inlineStr">
+      <c r="B35" s="1514" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1478" t="inlineStr">
+      <c r="C35" s="1514" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1479" t="n"/>
-      <c r="E35" s="1479" t="n">
+      <c r="D35" s="1515" t="n"/>
+      <c r="E35" s="1515" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1479" t="n">
+      <c r="F35" s="1515" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1479" t="n">
+      <c r="G35" s="1515" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1479" t="n"/>
-      <c r="I35" s="1480" t="n">
+      <c r="H35" s="1515" t="n"/>
+      <c r="I35" s="1516" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1481" t="n"/>
-      <c r="K35" s="1481" t="n"/>
-      <c r="L35" s="1481" t="n"/>
-      <c r="M35" s="1479" t="n"/>
-      <c r="N35" s="1479" t="n"/>
-      <c r="O35" s="1479" t="n">
+      <c r="J35" s="1517" t="n"/>
+      <c r="K35" s="1517" t="n"/>
+      <c r="L35" s="1517" t="n"/>
+      <c r="M35" s="1515" t="n"/>
+      <c r="N35" s="1515" t="n"/>
+      <c r="O35" s="1515" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1482" t="n">
+      <c r="P35" s="1518" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1479" t="n"/>
-      <c r="R35" s="1479" t="n">
+      <c r="Q35" s="1515" t="n"/>
+      <c r="R35" s="1515" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1479" t="n"/>
+      <c r="S35" s="1515" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1478" t="inlineStr">
+      <c r="U35" s="1514" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -7056,49 +7182,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1483" t="inlineStr">
+      <c r="A36" s="1519" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1484" t="inlineStr">
+      <c r="B36" s="1520" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1484" t="inlineStr">
+      <c r="C36" s="1520" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1485" t="n"/>
-      <c r="E36" s="1485" t="n"/>
-      <c r="F36" s="1485" t="n"/>
-      <c r="G36" s="1485" t="n"/>
-      <c r="H36" s="1485" t="n">
+      <c r="D36" s="1521" t="n"/>
+      <c r="E36" s="1521" t="n"/>
+      <c r="F36" s="1521" t="n"/>
+      <c r="G36" s="1521" t="n"/>
+      <c r="H36" s="1521" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1486" t="n"/>
-      <c r="J36" s="1487" t="n"/>
-      <c r="K36" s="1487" t="n"/>
-      <c r="L36" s="1487" t="n"/>
-      <c r="M36" s="1485" t="n">
+      <c r="I36" s="1522" t="n"/>
+      <c r="J36" s="1523" t="n"/>
+      <c r="K36" s="1523" t="n"/>
+      <c r="L36" s="1523" t="n"/>
+      <c r="M36" s="1521" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1485" t="n">
+      <c r="N36" s="1521" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1485" t="n"/>
-      <c r="P36" s="1488" t="n"/>
-      <c r="Q36" s="1485" t="n"/>
-      <c r="R36" s="1485" t="n"/>
-      <c r="S36" s="1485" t="n"/>
+      <c r="O36" s="1521" t="n"/>
+      <c r="P36" s="1524" t="n"/>
+      <c r="Q36" s="1521" t="n"/>
+      <c r="R36" s="1521" t="n"/>
+      <c r="S36" s="1521" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1484" t="n"/>
+      <c r="U36" s="1520" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -7106,41 +7232,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1489" t="inlineStr">
+      <c r="A37" s="1525" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1490" t="inlineStr">
+      <c r="B37" s="1526" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1490" t="inlineStr">
+      <c r="C37" s="1526" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1491" t="n"/>
-      <c r="E37" s="1491" t="n"/>
-      <c r="F37" s="1491" t="n"/>
-      <c r="G37" s="1491" t="n"/>
-      <c r="H37" s="1491" t="n"/>
-      <c r="I37" s="1492" t="n"/>
-      <c r="J37" s="1493" t="n"/>
-      <c r="K37" s="1493" t="n"/>
-      <c r="L37" s="1493" t="n"/>
-      <c r="M37" s="1491" t="n"/>
-      <c r="N37" s="1491" t="n"/>
-      <c r="O37" s="1491" t="n"/>
-      <c r="P37" s="1494" t="n"/>
-      <c r="Q37" s="1491" t="n">
+      <c r="D37" s="1527" t="n"/>
+      <c r="E37" s="1527" t="n"/>
+      <c r="F37" s="1527" t="n"/>
+      <c r="G37" s="1527" t="n"/>
+      <c r="H37" s="1527" t="n"/>
+      <c r="I37" s="1528" t="n"/>
+      <c r="J37" s="1529" t="n"/>
+      <c r="K37" s="1529" t="n"/>
+      <c r="L37" s="1529" t="n"/>
+      <c r="M37" s="1527" t="n"/>
+      <c r="N37" s="1527" t="n"/>
+      <c r="O37" s="1527" t="n"/>
+      <c r="P37" s="1530" t="n"/>
+      <c r="Q37" s="1527" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1491" t="n"/>
-      <c r="S37" s="1491" t="n"/>
+      <c r="R37" s="1527" t="n"/>
+      <c r="S37" s="1527" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1490" t="n"/>
+      <c r="U37" s="1526" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -7148,57 +7274,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1465" t="inlineStr">
+      <c r="A38" s="1501" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1466" t="inlineStr">
+      <c r="B38" s="1502" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1466" t="inlineStr">
+      <c r="C38" s="1502" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1467" t="n"/>
-      <c r="E38" s="1467" t="n">
+      <c r="D38" s="1503" t="n"/>
+      <c r="E38" s="1503" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1467" t="n">
+      <c r="F38" s="1503" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1467" t="n">
+      <c r="G38" s="1503" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1467" t="n"/>
-      <c r="I38" s="1468" t="n">
+      <c r="H38" s="1503" t="n"/>
+      <c r="I38" s="1504" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1469" t="n"/>
-      <c r="K38" s="1469" t="n"/>
-      <c r="L38" s="1469" t="n"/>
-      <c r="M38" s="1467" t="n"/>
-      <c r="N38" s="1467" t="n"/>
-      <c r="O38" s="1467" t="n">
+      <c r="J38" s="1505" t="n"/>
+      <c r="K38" s="1505" t="n"/>
+      <c r="L38" s="1505" t="n"/>
+      <c r="M38" s="1503" t="n"/>
+      <c r="N38" s="1503" t="n"/>
+      <c r="O38" s="1503" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1470" t="n">
+      <c r="P38" s="1506" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1467" t="n"/>
-      <c r="R38" s="1467" t="n">
+      <c r="Q38" s="1503" t="n"/>
+      <c r="R38" s="1503" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1467" t="n"/>
+      <c r="S38" s="1503" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1466" t="inlineStr">
+      <c r="U38" s="1502" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -7210,49 +7336,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1495" t="inlineStr">
+      <c r="A39" s="1531" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1496" t="inlineStr">
+      <c r="B39" s="1532" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1496" t="inlineStr">
+      <c r="C39" s="1532" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1497" t="n"/>
-      <c r="E39" s="1497" t="n"/>
-      <c r="F39" s="1497" t="n"/>
-      <c r="G39" s="1497" t="n"/>
-      <c r="H39" s="1497" t="n">
+      <c r="D39" s="1533" t="n"/>
+      <c r="E39" s="1533" t="n"/>
+      <c r="F39" s="1533" t="n"/>
+      <c r="G39" s="1533" t="n"/>
+      <c r="H39" s="1533" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1498" t="n"/>
-      <c r="J39" s="1499" t="n"/>
-      <c r="K39" s="1499" t="n"/>
-      <c r="L39" s="1499" t="n"/>
-      <c r="M39" s="1497" t="n">
+      <c r="I39" s="1534" t="n"/>
+      <c r="J39" s="1535" t="n"/>
+      <c r="K39" s="1535" t="n"/>
+      <c r="L39" s="1535" t="n"/>
+      <c r="M39" s="1533" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1497" t="n">
+      <c r="N39" s="1533" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1497" t="n"/>
-      <c r="P39" s="1500" t="n"/>
-      <c r="Q39" s="1497" t="n"/>
-      <c r="R39" s="1497" t="n"/>
-      <c r="S39" s="1497" t="n"/>
+      <c r="O39" s="1533" t="n"/>
+      <c r="P39" s="1536" t="n"/>
+      <c r="Q39" s="1533" t="n"/>
+      <c r="R39" s="1533" t="n"/>
+      <c r="S39" s="1533" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1496" t="n"/>
+      <c r="U39" s="1532" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -7260,41 +7386,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1471" t="inlineStr">
+      <c r="A40" s="1507" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1472" t="inlineStr">
+      <c r="B40" s="1508" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1472" t="inlineStr">
+      <c r="C40" s="1508" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1473" t="n"/>
-      <c r="E40" s="1473" t="n"/>
-      <c r="F40" s="1473" t="n"/>
-      <c r="G40" s="1473" t="n"/>
-      <c r="H40" s="1473" t="n"/>
-      <c r="I40" s="1474" t="n"/>
-      <c r="J40" s="1475" t="n"/>
-      <c r="K40" s="1475" t="n"/>
-      <c r="L40" s="1475" t="n"/>
-      <c r="M40" s="1473" t="n"/>
-      <c r="N40" s="1473" t="n"/>
-      <c r="O40" s="1473" t="n"/>
-      <c r="P40" s="1476" t="n"/>
-      <c r="Q40" s="1473" t="n">
+      <c r="D40" s="1509" t="n"/>
+      <c r="E40" s="1509" t="n"/>
+      <c r="F40" s="1509" t="n"/>
+      <c r="G40" s="1509" t="n"/>
+      <c r="H40" s="1509" t="n"/>
+      <c r="I40" s="1510" t="n"/>
+      <c r="J40" s="1511" t="n"/>
+      <c r="K40" s="1511" t="n"/>
+      <c r="L40" s="1511" t="n"/>
+      <c r="M40" s="1509" t="n"/>
+      <c r="N40" s="1509" t="n"/>
+      <c r="O40" s="1509" t="n"/>
+      <c r="P40" s="1512" t="n"/>
+      <c r="Q40" s="1509" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1473" t="n"/>
-      <c r="S40" s="1473" t="n"/>
+      <c r="R40" s="1509" t="n"/>
+      <c r="S40" s="1509" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1472" t="n"/>
+      <c r="U40" s="1508" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -7302,57 +7428,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1477" t="inlineStr">
+      <c r="A41" s="1513" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1478" t="inlineStr">
+      <c r="B41" s="1514" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1478" t="inlineStr">
+      <c r="C41" s="1514" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1479" t="n"/>
-      <c r="E41" s="1479" t="n">
+      <c r="D41" s="1515" t="n"/>
+      <c r="E41" s="1515" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1479" t="n">
+      <c r="F41" s="1515" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1479" t="n">
+      <c r="G41" s="1515" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1479" t="n"/>
-      <c r="I41" s="1480" t="n">
+      <c r="H41" s="1515" t="n"/>
+      <c r="I41" s="1516" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1481" t="n"/>
-      <c r="K41" s="1481" t="n"/>
-      <c r="L41" s="1481" t="n"/>
-      <c r="M41" s="1479" t="n"/>
-      <c r="N41" s="1479" t="n"/>
-      <c r="O41" s="1479" t="n">
+      <c r="J41" s="1517" t="n"/>
+      <c r="K41" s="1517" t="n"/>
+      <c r="L41" s="1517" t="n"/>
+      <c r="M41" s="1515" t="n"/>
+      <c r="N41" s="1515" t="n"/>
+      <c r="O41" s="1515" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1482" t="n">
+      <c r="P41" s="1518" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1479" t="n"/>
-      <c r="R41" s="1479" t="n">
+      <c r="Q41" s="1515" t="n"/>
+      <c r="R41" s="1515" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1479" t="n"/>
+      <c r="S41" s="1515" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1478" t="inlineStr">
+      <c r="U41" s="1514" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -7364,49 +7490,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1489" t="inlineStr">
+      <c r="A42" s="1525" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1490" t="inlineStr">
+      <c r="B42" s="1526" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1490" t="inlineStr">
+      <c r="C42" s="1526" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1491" t="n"/>
-      <c r="E42" s="1491" t="n"/>
-      <c r="F42" s="1491" t="n"/>
-      <c r="G42" s="1491" t="n"/>
-      <c r="H42" s="1491" t="n">
+      <c r="D42" s="1527" t="n"/>
+      <c r="E42" s="1527" t="n"/>
+      <c r="F42" s="1527" t="n"/>
+      <c r="G42" s="1527" t="n"/>
+      <c r="H42" s="1527" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1492" t="n"/>
-      <c r="J42" s="1493" t="n"/>
-      <c r="K42" s="1493" t="n"/>
-      <c r="L42" s="1493" t="n"/>
-      <c r="M42" s="1491" t="n">
+      <c r="I42" s="1528" t="n"/>
+      <c r="J42" s="1529" t="n"/>
+      <c r="K42" s="1529" t="n"/>
+      <c r="L42" s="1529" t="n"/>
+      <c r="M42" s="1527" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1491" t="n">
+      <c r="N42" s="1527" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1491" t="n"/>
-      <c r="P42" s="1494" t="n"/>
-      <c r="Q42" s="1491" t="n"/>
-      <c r="R42" s="1491" t="n"/>
-      <c r="S42" s="1491" t="n"/>
+      <c r="O42" s="1527" t="n"/>
+      <c r="P42" s="1530" t="n"/>
+      <c r="Q42" s="1527" t="n"/>
+      <c r="R42" s="1527" t="n"/>
+      <c r="S42" s="1527" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1490" t="n"/>
+      <c r="U42" s="1526" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -7414,57 +7540,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1465" t="inlineStr">
+      <c r="A43" s="1501" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1466" t="inlineStr">
+      <c r="B43" s="1502" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1466" t="inlineStr">
+      <c r="C43" s="1502" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1467" t="n"/>
-      <c r="E43" s="1467" t="n">
+      <c r="D43" s="1503" t="n"/>
+      <c r="E43" s="1503" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1467" t="n">
+      <c r="F43" s="1503" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1467" t="n">
+      <c r="G43" s="1503" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1467" t="n"/>
-      <c r="I43" s="1468" t="n">
+      <c r="H43" s="1503" t="n"/>
+      <c r="I43" s="1504" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1469" t="n"/>
-      <c r="K43" s="1469" t="n"/>
-      <c r="L43" s="1469" t="n"/>
-      <c r="M43" s="1467" t="n"/>
-      <c r="N43" s="1467" t="n"/>
-      <c r="O43" s="1467" t="n">
+      <c r="J43" s="1505" t="n"/>
+      <c r="K43" s="1505" t="n"/>
+      <c r="L43" s="1505" t="n"/>
+      <c r="M43" s="1503" t="n"/>
+      <c r="N43" s="1503" t="n"/>
+      <c r="O43" s="1503" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1470" t="n">
+      <c r="P43" s="1506" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1467" t="n"/>
-      <c r="R43" s="1467" t="n">
+      <c r="Q43" s="1503" t="n"/>
+      <c r="R43" s="1503" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1467" t="n"/>
+      <c r="S43" s="1503" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1466" t="n"/>
+      <c r="U43" s="1502" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -7472,45 +7598,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1495" t="inlineStr">
+      <c r="A44" s="1531" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1496" t="inlineStr">
+      <c r="B44" s="1532" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1496" t="inlineStr">
+      <c r="C44" s="1532" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1497" t="n"/>
-      <c r="E44" s="1497" t="n">
+      <c r="D44" s="1533" t="n"/>
+      <c r="E44" s="1533" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1497" t="n">
+      <c r="F44" s="1533" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1497" t="n"/>
-      <c r="H44" s="1497" t="n"/>
-      <c r="I44" s="1498" t="n"/>
-      <c r="J44" s="1499" t="n"/>
-      <c r="K44" s="1499" t="n"/>
-      <c r="L44" s="1499" t="n"/>
-      <c r="M44" s="1497" t="n"/>
-      <c r="N44" s="1497" t="n"/>
-      <c r="O44" s="1497" t="n"/>
-      <c r="P44" s="1500" t="n"/>
-      <c r="Q44" s="1497" t="n"/>
-      <c r="R44" s="1497" t="n"/>
-      <c r="S44" s="1497" t="n">
+      <c r="G44" s="1533" t="n"/>
+      <c r="H44" s="1533" t="n"/>
+      <c r="I44" s="1534" t="n"/>
+      <c r="J44" s="1535" t="n"/>
+      <c r="K44" s="1535" t="n"/>
+      <c r="L44" s="1535" t="n"/>
+      <c r="M44" s="1533" t="n"/>
+      <c r="N44" s="1533" t="n"/>
+      <c r="O44" s="1533" t="n"/>
+      <c r="P44" s="1536" t="n"/>
+      <c r="Q44" s="1533" t="n"/>
+      <c r="R44" s="1533" t="n"/>
+      <c r="S44" s="1533" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1496" t="inlineStr">
+      <c r="U44" s="1532" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -7522,49 +7648,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1495" t="inlineStr">
+      <c r="A45" s="1531" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1496" t="inlineStr">
+      <c r="B45" s="1532" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1496" t="inlineStr">
+      <c r="C45" s="1532" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1497" t="n"/>
-      <c r="E45" s="1497" t="n"/>
-      <c r="F45" s="1497" t="n"/>
-      <c r="G45" s="1497" t="n"/>
-      <c r="H45" s="1497" t="n">
+      <c r="D45" s="1533" t="n"/>
+      <c r="E45" s="1533" t="n"/>
+      <c r="F45" s="1533" t="n"/>
+      <c r="G45" s="1533" t="n"/>
+      <c r="H45" s="1533" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1498" t="n"/>
-      <c r="J45" s="1499" t="n"/>
-      <c r="K45" s="1499" t="n"/>
-      <c r="L45" s="1499" t="n"/>
-      <c r="M45" s="1497" t="n">
+      <c r="I45" s="1534" t="n"/>
+      <c r="J45" s="1535" t="n"/>
+      <c r="K45" s="1535" t="n"/>
+      <c r="L45" s="1535" t="n"/>
+      <c r="M45" s="1533" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1497" t="n">
+      <c r="N45" s="1533" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1497" t="n"/>
-      <c r="P45" s="1500" t="n"/>
-      <c r="Q45" s="1497" t="n"/>
-      <c r="R45" s="1497" t="n"/>
-      <c r="S45" s="1497" t="n"/>
+      <c r="O45" s="1533" t="n"/>
+      <c r="P45" s="1536" t="n"/>
+      <c r="Q45" s="1533" t="n"/>
+      <c r="R45" s="1533" t="n"/>
+      <c r="S45" s="1533" t="n"/>
       <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1496" t="n"/>
+      <c r="U45" s="1532" t="n"/>
       <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -7572,39 +7698,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1471" t="inlineStr">
+      <c r="A46" s="1507" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B46" s="1472" t="inlineStr">
+      <c r="B46" s="1508" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="C46" s="1472" t="inlineStr">
+      <c r="C46" s="1508" t="inlineStr">
         <is>
           <t>EVENT - Clean</t>
         </is>
       </c>
-      <c r="D46" s="1473" t="n"/>
-      <c r="E46" s="1473" t="n"/>
-      <c r="F46" s="1473" t="n"/>
-      <c r="G46" s="1473" t="n"/>
-      <c r="H46" s="1473" t="n"/>
-      <c r="I46" s="1474" t="n"/>
-      <c r="J46" s="1475" t="n"/>
-      <c r="K46" s="1475" t="n"/>
-      <c r="L46" s="1475" t="n"/>
-      <c r="M46" s="1473" t="n"/>
-      <c r="N46" s="1473" t="n"/>
-      <c r="O46" s="1473" t="n"/>
-      <c r="P46" s="1476" t="n"/>
-      <c r="Q46" s="1473" t="n"/>
-      <c r="R46" s="1473" t="n"/>
-      <c r="S46" s="1473" t="n"/>
+      <c r="D46" s="1509" t="n"/>
+      <c r="E46" s="1509" t="n"/>
+      <c r="F46" s="1509" t="n"/>
+      <c r="G46" s="1509" t="n"/>
+      <c r="H46" s="1509" t="n"/>
+      <c r="I46" s="1510" t="n"/>
+      <c r="J46" s="1511" t="n"/>
+      <c r="K46" s="1511" t="n"/>
+      <c r="L46" s="1511" t="n"/>
+      <c r="M46" s="1509" t="n"/>
+      <c r="N46" s="1509" t="n"/>
+      <c r="O46" s="1509" t="n"/>
+      <c r="P46" s="1512" t="n"/>
+      <c r="Q46" s="1509" t="n"/>
+      <c r="R46" s="1509" t="n"/>
+      <c r="S46" s="1509" t="n"/>
       <c r="T46" s="631" t="n"/>
-      <c r="U46" s="1472" t="n"/>
+      <c r="U46" s="1508" t="n"/>
       <c r="V46" s="632" t="inlineStr">
         <is>
           <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
@@ -7612,51 +7738,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1477" t="inlineStr">
+      <c r="A47" s="1513" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1478" t="inlineStr">
+      <c r="B47" s="1514" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C47" s="1478" t="inlineStr">
+      <c r="C47" s="1514" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D47" s="1479" t="n"/>
-      <c r="E47" s="1479" t="n">
+      <c r="D47" s="1515" t="n"/>
+      <c r="E47" s="1515" t="n">
         <v>16.6</v>
       </c>
-      <c r="F47" s="1479" t="n">
+      <c r="F47" s="1515" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="1479" t="n">
+      <c r="G47" s="1515" t="n">
         <v>4.1</v>
       </c>
-      <c r="H47" s="1479" t="n"/>
-      <c r="I47" s="1480" t="n">
+      <c r="H47" s="1515" t="n"/>
+      <c r="I47" s="1516" t="n">
         <v>0.9</v>
       </c>
-      <c r="J47" s="1481" t="n"/>
-      <c r="K47" s="1481" t="n"/>
-      <c r="L47" s="1481" t="n"/>
-      <c r="M47" s="1479" t="n"/>
-      <c r="N47" s="1479" t="n"/>
-      <c r="O47" s="1479" t="n">
+      <c r="J47" s="1517" t="n"/>
+      <c r="K47" s="1517" t="n"/>
+      <c r="L47" s="1517" t="n"/>
+      <c r="M47" s="1515" t="n"/>
+      <c r="N47" s="1515" t="n"/>
+      <c r="O47" s="1515" t="n">
         <v>13.2</v>
       </c>
-      <c r="P47" s="1482" t="n">
+      <c r="P47" s="1518" t="n">
         <v>0</v>
       </c>
-      <c r="Q47" s="1479" t="n"/>
-      <c r="R47" s="1479" t="n">
+      <c r="Q47" s="1515" t="n"/>
+      <c r="R47" s="1515" t="n">
         <v>84.5</v>
       </c>
-      <c r="S47" s="1479" t="n">
+      <c r="S47" s="1515" t="n">
         <v>11.8</v>
       </c>
       <c r="T47" s="813" t="inlineStr">
@@ -7664,7 +7790,7 @@
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1478" t="inlineStr">
+      <c r="U47" s="1514" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
@@ -7676,49 +7802,49 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1489" t="inlineStr">
+      <c r="A48" s="1525" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B48" s="1490" t="inlineStr">
+      <c r="B48" s="1526" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C48" s="1490" t="inlineStr">
+      <c r="C48" s="1526" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D48" s="1491" t="n"/>
-      <c r="E48" s="1491" t="n"/>
-      <c r="F48" s="1491" t="n"/>
-      <c r="G48" s="1491" t="n"/>
-      <c r="H48" s="1491" t="n">
+      <c r="D48" s="1527" t="n"/>
+      <c r="E48" s="1527" t="n"/>
+      <c r="F48" s="1527" t="n"/>
+      <c r="G48" s="1527" t="n"/>
+      <c r="H48" s="1527" t="n">
         <v>15.1</v>
       </c>
-      <c r="I48" s="1492" t="n"/>
-      <c r="J48" s="1493" t="n"/>
-      <c r="K48" s="1493" t="n"/>
-      <c r="L48" s="1493" t="n"/>
-      <c r="M48" s="1491" t="n">
+      <c r="I48" s="1528" t="n"/>
+      <c r="J48" s="1529" t="n"/>
+      <c r="K48" s="1529" t="n"/>
+      <c r="L48" s="1529" t="n"/>
+      <c r="M48" s="1527" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="1491" t="n">
+      <c r="N48" s="1527" t="n">
         <v>20</v>
       </c>
-      <c r="O48" s="1491" t="n"/>
-      <c r="P48" s="1494" t="n"/>
-      <c r="Q48" s="1491" t="n"/>
-      <c r="R48" s="1491" t="n"/>
-      <c r="S48" s="1491" t="n"/>
+      <c r="O48" s="1527" t="n"/>
+      <c r="P48" s="1530" t="n"/>
+      <c r="Q48" s="1527" t="n"/>
+      <c r="R48" s="1527" t="n"/>
+      <c r="S48" s="1527" t="n"/>
       <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U48" s="1490" t="n"/>
+      <c r="U48" s="1526" t="n"/>
       <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
@@ -7726,51 +7852,51 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1465" t="inlineStr">
+      <c r="A49" s="1501" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B49" s="1466" t="inlineStr">
+      <c r="B49" s="1502" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C49" s="1466" t="inlineStr">
+      <c r="C49" s="1502" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D49" s="1467" t="n"/>
-      <c r="E49" s="1467" t="n">
+      <c r="D49" s="1503" t="n"/>
+      <c r="E49" s="1503" t="n">
         <v>16.8</v>
       </c>
-      <c r="F49" s="1467" t="n">
+      <c r="F49" s="1503" t="n">
         <v>0.2</v>
       </c>
-      <c r="G49" s="1467" t="n">
+      <c r="G49" s="1503" t="n">
         <v>3.3</v>
       </c>
-      <c r="H49" s="1467" t="n"/>
-      <c r="I49" s="1468" t="n">
+      <c r="H49" s="1503" t="n"/>
+      <c r="I49" s="1504" t="n">
         <v>1.7</v>
       </c>
-      <c r="J49" s="1469" t="n"/>
-      <c r="K49" s="1469" t="n"/>
-      <c r="L49" s="1469" t="n"/>
-      <c r="M49" s="1467" t="n"/>
-      <c r="N49" s="1467" t="n"/>
-      <c r="O49" s="1467" t="n">
+      <c r="J49" s="1505" t="n"/>
+      <c r="K49" s="1505" t="n"/>
+      <c r="L49" s="1505" t="n"/>
+      <c r="M49" s="1503" t="n"/>
+      <c r="N49" s="1503" t="n"/>
+      <c r="O49" s="1503" t="n">
         <v>13</v>
       </c>
-      <c r="P49" s="1470" t="n">
+      <c r="P49" s="1506" t="n">
         <v>0.87</v>
       </c>
-      <c r="Q49" s="1467" t="n"/>
-      <c r="R49" s="1467" t="n">
+      <c r="Q49" s="1503" t="n"/>
+      <c r="R49" s="1503" t="n">
         <v>86</v>
       </c>
-      <c r="S49" s="1467" t="n">
+      <c r="S49" s="1503" t="n">
         <v>11.65</v>
       </c>
       <c r="T49" s="624" t="inlineStr">
@@ -7778,7 +7904,7 @@
           <t>Clear now, 88F, 67% RH; sun so far 6.4h of 7h daylight (91%); today high 90F, 0.87in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U49" s="1466" t="inlineStr">
+      <c r="U49" s="1502" t="inlineStr">
         <is>
           <t>2026-07-04_1.jpeg;2026-07-04_2.jpeg;2026-07-04_3.jpeg;2026-07-04_4.jpeg</t>
         </is>
@@ -7790,49 +7916,49 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1471" t="inlineStr">
+      <c r="A50" s="1507" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B50" s="1472" t="inlineStr">
+      <c r="B50" s="1508" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C50" s="1472" t="inlineStr">
+      <c r="C50" s="1508" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D50" s="1473" t="n"/>
-      <c r="E50" s="1473" t="n"/>
-      <c r="F50" s="1473" t="n"/>
-      <c r="G50" s="1473" t="n"/>
-      <c r="H50" s="1473" t="n">
+      <c r="D50" s="1509" t="n"/>
+      <c r="E50" s="1509" t="n"/>
+      <c r="F50" s="1509" t="n"/>
+      <c r="G50" s="1509" t="n"/>
+      <c r="H50" s="1509" t="n">
         <v>14.6</v>
       </c>
-      <c r="I50" s="1474" t="n"/>
-      <c r="J50" s="1475" t="n"/>
-      <c r="K50" s="1475" t="n"/>
-      <c r="L50" s="1475" t="n"/>
-      <c r="M50" s="1473" t="n">
+      <c r="I50" s="1510" t="n"/>
+      <c r="J50" s="1511" t="n"/>
+      <c r="K50" s="1511" t="n"/>
+      <c r="L50" s="1511" t="n"/>
+      <c r="M50" s="1509" t="n">
         <v>0.5</v>
       </c>
-      <c r="N50" s="1473" t="n">
+      <c r="N50" s="1509" t="n">
         <v>20.5</v>
       </c>
-      <c r="O50" s="1473" t="n"/>
-      <c r="P50" s="1476" t="n"/>
-      <c r="Q50" s="1473" t="n"/>
-      <c r="R50" s="1473" t="n"/>
-      <c r="S50" s="1473" t="n"/>
+      <c r="O50" s="1509" t="n"/>
+      <c r="P50" s="1512" t="n"/>
+      <c r="Q50" s="1509" t="n"/>
+      <c r="R50" s="1509" t="n"/>
+      <c r="S50" s="1509" t="n"/>
       <c r="T50" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny day (high 90F, water 86F); storm forecast overnight</t>
         </is>
       </c>
-      <c r="U50" s="1472" t="n"/>
+      <c r="U50" s="1508" t="n"/>
       <c r="V50" s="632" t="inlineStr">
         <is>
           <t>0.5 gal added 7:40 PM. PARTY PRE-LOAD (Sun 7/5 1PM picnic): deliberately HALF the usual dose -- FC already high at 16.8, and John didn't want to overshoot into the high teens for guests. Sized on the retuned model (l24_hot_sunny now 4.0). Model projects ~14.6 next noon, BUT this is a known weather-mismatch case: model keys L24 off today's hot/sunny weather, while the actual loss window is a storm overnight (no UV) + cooler/cloudy Sun morning -&gt; real loss will be LOWER, so FC likely lands ~15-16 at the party (comfortable top-of-band, cushion for bather load, not overboard). =&gt; If tomorrow's noon comes in ABOVE 14.6, that's the weather mismatch, NOT the freshly-retuned constant; don't chase it. Plan: dose back up Sun evening after the crowd's out (expect a bather-load FC drop). Season total 20.5 gal. PHOTOS(4): water clear/healthy blue, bottom fully visible, no cloudiness/algae; yesterday's surface debris now gone (tracks with CC clearing to 0.2); liner step close-up normal speckled blue, no rust/stain progression. Ruler photo documents the ~11.65 cm level.</t>
@@ -7840,47 +7966,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1477" t="inlineStr">
+      <c r="A51" s="1513" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B51" s="1478" t="inlineStr">
+      <c r="B51" s="1514" t="inlineStr">
         <is>
           <t>07:45</t>
         </is>
       </c>
-      <c r="C51" s="1478" t="inlineStr">
+      <c r="C51" s="1514" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D51" s="1479" t="n"/>
-      <c r="E51" s="1479" t="n">
+      <c r="D51" s="1515" t="n"/>
+      <c r="E51" s="1515" t="n">
         <v>16</v>
       </c>
-      <c r="F51" s="1479" t="n">
+      <c r="F51" s="1515" t="n">
         <v>0.5</v>
       </c>
-      <c r="G51" s="1479" t="n"/>
-      <c r="H51" s="1479" t="n"/>
-      <c r="I51" s="1480" t="n">
+      <c r="G51" s="1515" t="n"/>
+      <c r="H51" s="1515" t="n"/>
+      <c r="I51" s="1516" t="n">
         <v>1.4</v>
       </c>
-      <c r="J51" s="1481" t="n"/>
-      <c r="K51" s="1481" t="n"/>
-      <c r="L51" s="1481" t="n"/>
-      <c r="M51" s="1479" t="n"/>
-      <c r="N51" s="1479" t="n"/>
-      <c r="O51" s="1479" t="n"/>
-      <c r="P51" s="1482" t="n">
+      <c r="J51" s="1517" t="n"/>
+      <c r="K51" s="1517" t="n"/>
+      <c r="L51" s="1517" t="n"/>
+      <c r="M51" s="1515" t="n"/>
+      <c r="N51" s="1515" t="n"/>
+      <c r="O51" s="1515" t="n"/>
+      <c r="P51" s="1518" t="n">
         <v>0.04</v>
       </c>
-      <c r="Q51" s="1479" t="n"/>
-      <c r="R51" s="1479" t="n">
+      <c r="Q51" s="1515" t="n"/>
+      <c r="R51" s="1515" t="n">
         <v>84</v>
       </c>
-      <c r="S51" s="1479" t="n">
+      <c r="S51" s="1515" t="n">
         <v>13.9</v>
       </c>
       <c r="T51" s="813" t="inlineStr">
@@ -7888,7 +8014,7 @@
           <t>Overcast now, 75F, 90% RH; sun so far 0.0h of 3h daylight (0%); today high 75F, 0.04in precip, UV max 6.5</t>
         </is>
       </c>
-      <c r="U51" s="1478" t="inlineStr">
+      <c r="U51" s="1514" t="inlineStr">
         <is>
           <t>2026-07-05_2.jpeg</t>
         </is>
@@ -7900,41 +8026,41 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1483" t="inlineStr">
+      <c r="A52" s="1519" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B52" s="1484" t="inlineStr">
+      <c r="B52" s="1520" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C52" s="1484" t="inlineStr">
+      <c r="C52" s="1520" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D52" s="1485" t="n"/>
-      <c r="E52" s="1485" t="n">
+      <c r="D52" s="1521" t="n"/>
+      <c r="E52" s="1521" t="n">
         <v>14.8</v>
       </c>
-      <c r="F52" s="1485" t="n">
+      <c r="F52" s="1521" t="n">
         <v>0.3</v>
       </c>
-      <c r="G52" s="1485" t="n"/>
-      <c r="H52" s="1485" t="n"/>
-      <c r="I52" s="1486" t="n"/>
-      <c r="J52" s="1487" t="n"/>
-      <c r="K52" s="1487" t="n"/>
-      <c r="L52" s="1487" t="n"/>
-      <c r="M52" s="1485" t="n"/>
-      <c r="N52" s="1485" t="n"/>
-      <c r="O52" s="1485" t="n"/>
-      <c r="P52" s="1488" t="n"/>
-      <c r="Q52" s="1485" t="n"/>
-      <c r="R52" s="1485" t="n"/>
-      <c r="S52" s="1485" t="n">
+      <c r="G52" s="1521" t="n"/>
+      <c r="H52" s="1521" t="n"/>
+      <c r="I52" s="1522" t="n"/>
+      <c r="J52" s="1523" t="n"/>
+      <c r="K52" s="1523" t="n"/>
+      <c r="L52" s="1523" t="n"/>
+      <c r="M52" s="1521" t="n"/>
+      <c r="N52" s="1521" t="n"/>
+      <c r="O52" s="1521" t="n"/>
+      <c r="P52" s="1524" t="n"/>
+      <c r="Q52" s="1521" t="n"/>
+      <c r="R52" s="1521" t="n"/>
+      <c r="S52" s="1521" t="n">
         <v>13.6</v>
       </c>
       <c r="T52" s="820" t="inlineStr">
@@ -7942,7 +8068,7 @@
           <t>Overcast now, 72F, 76% RH; sun so far 8.4h of 13h daylight (65%); today high 80F, 0.00in precip, UV max 6.0</t>
         </is>
       </c>
-      <c r="U52" s="1484" t="inlineStr">
+      <c r="U52" s="1520" t="inlineStr">
         <is>
           <t>2026-07-05_1.jpeg;2026-07-05_3.jpeg</t>
         </is>
@@ -7954,52 +8080,114 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1489" t="inlineStr">
+      <c r="A53" s="1525" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B53" s="1490" t="inlineStr">
+      <c r="B53" s="1526" t="inlineStr">
         <is>
           <t>19:25</t>
         </is>
       </c>
-      <c r="C53" s="1490" t="inlineStr">
+      <c r="C53" s="1526" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D53" s="1491" t="n"/>
-      <c r="E53" s="1491" t="n"/>
-      <c r="F53" s="1491" t="n"/>
-      <c r="G53" s="1491" t="n"/>
-      <c r="H53" s="1491" t="n">
+      <c r="D53" s="1527" t="n"/>
+      <c r="E53" s="1527" t="n"/>
+      <c r="F53" s="1527" t="n"/>
+      <c r="G53" s="1527" t="n"/>
+      <c r="H53" s="1527" t="n">
         <v>15.1</v>
       </c>
-      <c r="I53" s="1492" t="n"/>
-      <c r="J53" s="1493" t="n"/>
-      <c r="K53" s="1493" t="n"/>
-      <c r="L53" s="1493" t="n"/>
-      <c r="M53" s="1491" t="n">
+      <c r="I53" s="1528" t="n"/>
+      <c r="J53" s="1529" t="n"/>
+      <c r="K53" s="1529" t="n"/>
+      <c r="L53" s="1529" t="n"/>
+      <c r="M53" s="1527" t="n">
         <v>0.5</v>
       </c>
-      <c r="N53" s="1491" t="n">
+      <c r="N53" s="1527" t="n">
         <v>21</v>
       </c>
-      <c r="O53" s="1491" t="n"/>
-      <c r="P53" s="1494" t="n"/>
-      <c r="Q53" s="1491" t="n"/>
-      <c r="R53" s="1491" t="n"/>
-      <c r="S53" s="1491" t="n"/>
+      <c r="O53" s="1527" t="n"/>
+      <c r="P53" s="1530" t="n"/>
+      <c r="Q53" s="1527" t="n"/>
+      <c r="R53" s="1527" t="n"/>
+      <c r="S53" s="1527" t="n"/>
       <c r="T53" s="827" t="inlineStr">
         <is>
           <t>Cleared to partly sunny (8.4 sun hrs, high 80F, water 84F); all-day rain forecast Mon 7/6</t>
         </is>
       </c>
-      <c r="U53" s="1490" t="n"/>
+      <c r="U53" s="1526" t="n"/>
       <c r="V53" s="828" t="inlineStr">
         <is>
           <t>0.5 gal added 7:25 PM (post-party recovery dose). Sized on TOMORROW's rainy forecast (the real loss window: overcast/wet 7/6, ~0.9in rain, low UV) not today's sun -&gt; projects ~15.1 at Mon noon. Party went great (FC held 16.0-&gt;14.8, CC dropped 0.5-&gt;0.3). Season total 21.0 gal. This is the first prediction that deliberately used the next-day forecast for L24 instead of the model's default (today's weather as proxy) -- if it lands near 15.1 tomorrow, that validates feeding the forecast on weather-change days.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1537" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B54" s="1538" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="C54" s="1538" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="D54" s="1539" t="n"/>
+      <c r="E54" s="1539" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="F54" s="1539" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G54" s="1539" t="n"/>
+      <c r="H54" s="1539" t="n"/>
+      <c r="I54" s="1540" t="n">
+        <v>-1.3</v>
+      </c>
+      <c r="J54" s="1541" t="n"/>
+      <c r="K54" s="1541" t="n"/>
+      <c r="L54" s="1541" t="n"/>
+      <c r="M54" s="1539" t="n"/>
+      <c r="N54" s="1539" t="n"/>
+      <c r="O54" s="1539" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" s="1542" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q54" s="1539" t="n"/>
+      <c r="R54" s="1539" t="n">
+        <v>81</v>
+      </c>
+      <c r="S54" s="1539" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="T54" s="1047" t="inlineStr">
+        <is>
+          <t>Light rain now, 65F, 93% RH; sun so far 0.0h of 6h daylight (0%); today high 68F, 2.00in precip, UV max 0.5</t>
+        </is>
+      </c>
+      <c r="U54" s="1538" t="inlineStr">
+        <is>
+          <t>2026-07-06_1.jpeg</t>
+        </is>
+      </c>
+      <c r="V54" s="1048" t="inlineStr">
+        <is>
+          <t>25mL x0.2. FC 13.8, CC 0.2 -- in band, all healthy. FIRST NEGATIVE prediction error (-1.3): actual 13.8 vs the 7/5 dose's 15.1 (which used the rain bucket L24=1.5). i.e. the model UNDER-estimated loss on this heavy-rain day. WHY: 2.0in of rain fell but the level only rose 0.6in (13.6-&gt;15.1 cm) -&gt; the pool is OVERFLOWING, carrying FC (and CYA) over the edge, plus rain dilution -- neither of which the UV-only rain bucket models. So heavy-rain/overflow days lose MORE than the rain bucket predicts. This is the FIRST forward rainy-day point AND it's confounded by overflow -&gt; do NOT retune the rain bucket off it (it may still be fine for light/no-overflow drizzle); just note heavy-rain != low-loss. SILVER LINING: the overflow + dilution is passively lowering CYA (currently ~150) -- exactly what we want -&gt; good trigger for a CYA recheck once it clears. fc_loss left BLANK: overflow+dilution make today's drop not a clean chemical-loss measurement. Level 15.1 (near the top, overflowing). Water temp 81 (cooling). DOSE REC TONIGHT: HOLD (no dose) -- dosing into an overflowing pool just sends chlorine over the edge, FC 13.8 is comfortably in-band, nobody's swimming in the rain, and John's low on chlorine (refill 1-2 days out). Let it ride; dose Wed when the rain clears and the refill's here. If FC dips toward floor 11 faster than expected, reassess.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct 2026-07-06 log: pool is NOT overflowing
My prior note wrongly read overflow. The weather feed's 2.00in is the
day's FORECAST total, not fallen-yet; only ~0.6in has actually fallen,
which matches the 0.6in level rise -- no overflow, 6+ in freeboard.
Real cause of the -1.3 miss: a STORM (not calm rain) washing organic
load in and consuming FC, which the drizzle-tuned rain bucket
under-estimates. Revised dose rec to a modest 0.5 gal (storm is eating
FC, no overflow to waste it).
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1543">
+  <cellXfs count="1585">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -5030,6 +5030,132 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -5594,35 +5720,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1501" t="inlineStr">
+      <c r="A3" s="1543" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1502" t="n"/>
-      <c r="C3" s="1502" t="inlineStr">
+      <c r="B3" s="1544" t="n"/>
+      <c r="C3" s="1544" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1503" t="n"/>
-      <c r="E3" s="1503" t="n"/>
-      <c r="F3" s="1503" t="n"/>
-      <c r="G3" s="1503" t="n"/>
-      <c r="H3" s="1503" t="n"/>
-      <c r="I3" s="1504" t="n"/>
-      <c r="J3" s="1505" t="n"/>
-      <c r="K3" s="1505" t="n"/>
-      <c r="L3" s="1505" t="n"/>
-      <c r="M3" s="1503" t="n"/>
-      <c r="N3" s="1503" t="n"/>
-      <c r="O3" s="1503" t="n"/>
-      <c r="P3" s="1506" t="n"/>
-      <c r="Q3" s="1503" t="n"/>
-      <c r="R3" s="1503" t="n"/>
-      <c r="S3" s="1503" t="n"/>
+      <c r="D3" s="1545" t="n"/>
+      <c r="E3" s="1545" t="n"/>
+      <c r="F3" s="1545" t="n"/>
+      <c r="G3" s="1545" t="n"/>
+      <c r="H3" s="1545" t="n"/>
+      <c r="I3" s="1546" t="n"/>
+      <c r="J3" s="1547" t="n"/>
+      <c r="K3" s="1547" t="n"/>
+      <c r="L3" s="1547" t="n"/>
+      <c r="M3" s="1545" t="n"/>
+      <c r="N3" s="1545" t="n"/>
+      <c r="O3" s="1545" t="n"/>
+      <c r="P3" s="1548" t="n"/>
+      <c r="Q3" s="1545" t="n"/>
+      <c r="R3" s="1545" t="n"/>
+      <c r="S3" s="1545" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1502" t="n"/>
+      <c r="U3" s="1544" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -5630,43 +5756,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1507" t="inlineStr">
+      <c r="A4" s="1549" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1508" t="inlineStr">
+      <c r="B4" s="1550" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1508" t="inlineStr">
+      <c r="C4" s="1550" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1509" t="n"/>
-      <c r="E4" s="1509" t="n"/>
-      <c r="F4" s="1509" t="n"/>
-      <c r="G4" s="1509" t="n"/>
-      <c r="H4" s="1509" t="n"/>
-      <c r="I4" s="1510" t="n"/>
-      <c r="J4" s="1511" t="n"/>
-      <c r="K4" s="1511" t="n"/>
-      <c r="L4" s="1511" t="n"/>
-      <c r="M4" s="1509" t="n">
+      <c r="D4" s="1551" t="n"/>
+      <c r="E4" s="1551" t="n"/>
+      <c r="F4" s="1551" t="n"/>
+      <c r="G4" s="1551" t="n"/>
+      <c r="H4" s="1551" t="n"/>
+      <c r="I4" s="1552" t="n"/>
+      <c r="J4" s="1553" t="n"/>
+      <c r="K4" s="1553" t="n"/>
+      <c r="L4" s="1553" t="n"/>
+      <c r="M4" s="1551" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1509" t="n">
+      <c r="N4" s="1551" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1509" t="n"/>
-      <c r="P4" s="1512" t="n"/>
-      <c r="Q4" s="1509" t="n"/>
-      <c r="R4" s="1509" t="n"/>
-      <c r="S4" s="1509" t="n"/>
+      <c r="O4" s="1551" t="n"/>
+      <c r="P4" s="1554" t="n"/>
+      <c r="Q4" s="1551" t="n"/>
+      <c r="R4" s="1551" t="n"/>
+      <c r="S4" s="1551" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1508" t="n"/>
+      <c r="U4" s="1550" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -5674,57 +5800,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1513" t="inlineStr">
+      <c r="A5" s="1555" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1514" t="inlineStr">
+      <c r="B5" s="1556" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1514" t="inlineStr">
+      <c r="C5" s="1556" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1515" t="n">
+      <c r="D5" s="1557" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1515" t="n">
+      <c r="E5" s="1557" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1515" t="n">
+      <c r="F5" s="1557" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1515" t="n"/>
-      <c r="H5" s="1515" t="n"/>
-      <c r="I5" s="1516" t="n"/>
-      <c r="J5" s="1517" t="n">
+      <c r="G5" s="1557" t="n"/>
+      <c r="H5" s="1557" t="n"/>
+      <c r="I5" s="1558" t="n"/>
+      <c r="J5" s="1559" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1517" t="n">
+      <c r="K5" s="1559" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1517" t="inlineStr">
+      <c r="L5" s="1559" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1515" t="n"/>
-      <c r="N5" s="1515" t="n"/>
-      <c r="O5" s="1515" t="n">
+      <c r="M5" s="1557" t="n"/>
+      <c r="N5" s="1557" t="n"/>
+      <c r="O5" s="1557" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1518" t="n">
+      <c r="P5" s="1560" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1515" t="n"/>
-      <c r="R5" s="1515" t="n"/>
-      <c r="S5" s="1515" t="n"/>
+      <c r="Q5" s="1557" t="n"/>
+      <c r="R5" s="1557" t="n"/>
+      <c r="S5" s="1557" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1514" t="n"/>
+      <c r="U5" s="1556" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -5732,43 +5858,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1519" t="inlineStr">
+      <c r="A6" s="1561" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1520" t="inlineStr">
+      <c r="B6" s="1562" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1520" t="inlineStr">
+      <c r="C6" s="1562" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1521" t="n"/>
-      <c r="E6" s="1521" t="n"/>
-      <c r="F6" s="1521" t="n"/>
-      <c r="G6" s="1521" t="n"/>
-      <c r="H6" s="1521" t="n"/>
-      <c r="I6" s="1522" t="n"/>
-      <c r="J6" s="1523" t="n"/>
-      <c r="K6" s="1523" t="n"/>
-      <c r="L6" s="1523" t="n"/>
-      <c r="M6" s="1521" t="n">
+      <c r="D6" s="1563" t="n"/>
+      <c r="E6" s="1563" t="n"/>
+      <c r="F6" s="1563" t="n"/>
+      <c r="G6" s="1563" t="n"/>
+      <c r="H6" s="1563" t="n"/>
+      <c r="I6" s="1564" t="n"/>
+      <c r="J6" s="1565" t="n"/>
+      <c r="K6" s="1565" t="n"/>
+      <c r="L6" s="1565" t="n"/>
+      <c r="M6" s="1563" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1521" t="n">
+      <c r="N6" s="1563" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1521" t="n"/>
-      <c r="P6" s="1524" t="n"/>
-      <c r="Q6" s="1521" t="n"/>
-      <c r="R6" s="1521" t="n"/>
-      <c r="S6" s="1521" t="n"/>
+      <c r="O6" s="1563" t="n"/>
+      <c r="P6" s="1566" t="n"/>
+      <c r="Q6" s="1563" t="n"/>
+      <c r="R6" s="1563" t="n"/>
+      <c r="S6" s="1563" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1520" t="n"/>
+      <c r="U6" s="1562" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -5776,39 +5902,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1525" t="inlineStr">
+      <c r="A7" s="1567" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1526" t="inlineStr">
+      <c r="B7" s="1568" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1526" t="inlineStr">
+      <c r="C7" s="1568" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1527" t="n"/>
-      <c r="E7" s="1527" t="n"/>
-      <c r="F7" s="1527" t="n"/>
-      <c r="G7" s="1527" t="n"/>
-      <c r="H7" s="1527" t="n"/>
-      <c r="I7" s="1528" t="n"/>
-      <c r="J7" s="1529" t="n"/>
-      <c r="K7" s="1529" t="n"/>
-      <c r="L7" s="1529" t="n"/>
-      <c r="M7" s="1527" t="n"/>
-      <c r="N7" s="1527" t="n"/>
-      <c r="O7" s="1527" t="n"/>
-      <c r="P7" s="1530" t="n"/>
-      <c r="Q7" s="1527" t="n"/>
-      <c r="R7" s="1527" t="n"/>
-      <c r="S7" s="1527" t="n"/>
+      <c r="D7" s="1569" t="n"/>
+      <c r="E7" s="1569" t="n"/>
+      <c r="F7" s="1569" t="n"/>
+      <c r="G7" s="1569" t="n"/>
+      <c r="H7" s="1569" t="n"/>
+      <c r="I7" s="1570" t="n"/>
+      <c r="J7" s="1571" t="n"/>
+      <c r="K7" s="1571" t="n"/>
+      <c r="L7" s="1571" t="n"/>
+      <c r="M7" s="1569" t="n"/>
+      <c r="N7" s="1569" t="n"/>
+      <c r="O7" s="1569" t="n"/>
+      <c r="P7" s="1572" t="n"/>
+      <c r="Q7" s="1569" t="n"/>
+      <c r="R7" s="1569" t="n"/>
+      <c r="S7" s="1569" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1526" t="n"/>
+      <c r="U7" s="1568" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5816,39 +5942,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1501" t="inlineStr">
+      <c r="A8" s="1543" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1502" t="inlineStr">
+      <c r="B8" s="1544" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1502" t="inlineStr">
+      <c r="C8" s="1544" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1503" t="n"/>
-      <c r="E8" s="1503" t="n"/>
-      <c r="F8" s="1503" t="n"/>
-      <c r="G8" s="1503" t="n"/>
-      <c r="H8" s="1503" t="n"/>
-      <c r="I8" s="1504" t="n"/>
-      <c r="J8" s="1505" t="n"/>
-      <c r="K8" s="1505" t="n"/>
-      <c r="L8" s="1505" t="n"/>
-      <c r="M8" s="1503" t="n"/>
-      <c r="N8" s="1503" t="n"/>
-      <c r="O8" s="1503" t="n"/>
-      <c r="P8" s="1506" t="n"/>
-      <c r="Q8" s="1503" t="n"/>
-      <c r="R8" s="1503" t="n"/>
-      <c r="S8" s="1503" t="n"/>
+      <c r="D8" s="1545" t="n"/>
+      <c r="E8" s="1545" t="n"/>
+      <c r="F8" s="1545" t="n"/>
+      <c r="G8" s="1545" t="n"/>
+      <c r="H8" s="1545" t="n"/>
+      <c r="I8" s="1546" t="n"/>
+      <c r="J8" s="1547" t="n"/>
+      <c r="K8" s="1547" t="n"/>
+      <c r="L8" s="1547" t="n"/>
+      <c r="M8" s="1545" t="n"/>
+      <c r="N8" s="1545" t="n"/>
+      <c r="O8" s="1545" t="n"/>
+      <c r="P8" s="1548" t="n"/>
+      <c r="Q8" s="1545" t="n"/>
+      <c r="R8" s="1545" t="n"/>
+      <c r="S8" s="1545" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1502" t="n"/>
+      <c r="U8" s="1544" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -5856,63 +5982,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1531" t="inlineStr">
+      <c r="A9" s="1573" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1532" t="inlineStr">
+      <c r="B9" s="1574" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1532" t="inlineStr">
+      <c r="C9" s="1574" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1533" t="n">
+      <c r="D9" s="1575" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1533" t="n">
+      <c r="E9" s="1575" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1533" t="n">
+      <c r="F9" s="1575" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1533" t="n">
+      <c r="G9" s="1575" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1533" t="n"/>
-      <c r="I9" s="1534" t="n"/>
-      <c r="J9" s="1535" t="n">
+      <c r="H9" s="1575" t="n"/>
+      <c r="I9" s="1576" t="n"/>
+      <c r="J9" s="1577" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1535" t="n">
+      <c r="K9" s="1577" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1535" t="inlineStr">
+      <c r="L9" s="1577" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1533" t="n"/>
-      <c r="N9" s="1533" t="n"/>
-      <c r="O9" s="1533" t="n">
+      <c r="M9" s="1575" t="n"/>
+      <c r="N9" s="1575" t="n"/>
+      <c r="O9" s="1575" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1536" t="n">
+      <c r="P9" s="1578" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1533" t="n"/>
-      <c r="R9" s="1533" t="n"/>
-      <c r="S9" s="1533" t="n"/>
+      <c r="Q9" s="1575" t="n"/>
+      <c r="R9" s="1575" t="n"/>
+      <c r="S9" s="1575" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1532" t="n"/>
+      <c r="U9" s="1574" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -5920,43 +6046,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1531" t="inlineStr">
+      <c r="A10" s="1573" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1532" t="inlineStr">
+      <c r="B10" s="1574" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1532" t="inlineStr">
+      <c r="C10" s="1574" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1533" t="n"/>
-      <c r="E10" s="1533" t="n"/>
-      <c r="F10" s="1533" t="n"/>
-      <c r="G10" s="1533" t="n"/>
-      <c r="H10" s="1533" t="n"/>
-      <c r="I10" s="1534" t="n"/>
-      <c r="J10" s="1535" t="n"/>
-      <c r="K10" s="1535" t="n"/>
-      <c r="L10" s="1535" t="inlineStr">
+      <c r="D10" s="1575" t="n"/>
+      <c r="E10" s="1575" t="n"/>
+      <c r="F10" s="1575" t="n"/>
+      <c r="G10" s="1575" t="n"/>
+      <c r="H10" s="1575" t="n"/>
+      <c r="I10" s="1576" t="n"/>
+      <c r="J10" s="1577" t="n"/>
+      <c r="K10" s="1577" t="n"/>
+      <c r="L10" s="1577" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1533" t="n"/>
-      <c r="N10" s="1533" t="n"/>
-      <c r="O10" s="1533" t="n"/>
-      <c r="P10" s="1536" t="n"/>
-      <c r="Q10" s="1533" t="n"/>
-      <c r="R10" s="1533" t="n"/>
-      <c r="S10" s="1533" t="n"/>
+      <c r="M10" s="1575" t="n"/>
+      <c r="N10" s="1575" t="n"/>
+      <c r="O10" s="1575" t="n"/>
+      <c r="P10" s="1578" t="n"/>
+      <c r="Q10" s="1575" t="n"/>
+      <c r="R10" s="1575" t="n"/>
+      <c r="S10" s="1575" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1532" t="n"/>
+      <c r="U10" s="1574" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -5964,43 +6090,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1531" t="inlineStr">
+      <c r="A11" s="1573" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1532" t="inlineStr">
+      <c r="B11" s="1574" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1532" t="inlineStr">
+      <c r="C11" s="1574" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1533" t="n"/>
-      <c r="E11" s="1533" t="n"/>
-      <c r="F11" s="1533" t="n"/>
-      <c r="G11" s="1533" t="n"/>
-      <c r="H11" s="1533" t="n"/>
-      <c r="I11" s="1534" t="n"/>
-      <c r="J11" s="1535" t="n"/>
-      <c r="K11" s="1535" t="n"/>
-      <c r="L11" s="1535" t="n"/>
-      <c r="M11" s="1533" t="n">
+      <c r="D11" s="1575" t="n"/>
+      <c r="E11" s="1575" t="n"/>
+      <c r="F11" s="1575" t="n"/>
+      <c r="G11" s="1575" t="n"/>
+      <c r="H11" s="1575" t="n"/>
+      <c r="I11" s="1576" t="n"/>
+      <c r="J11" s="1577" t="n"/>
+      <c r="K11" s="1577" t="n"/>
+      <c r="L11" s="1577" t="n"/>
+      <c r="M11" s="1575" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1533" t="n">
+      <c r="N11" s="1575" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1533" t="n"/>
-      <c r="P11" s="1536" t="n"/>
-      <c r="Q11" s="1533" t="n"/>
-      <c r="R11" s="1533" t="n"/>
-      <c r="S11" s="1533" t="n"/>
+      <c r="O11" s="1575" t="n"/>
+      <c r="P11" s="1578" t="n"/>
+      <c r="Q11" s="1575" t="n"/>
+      <c r="R11" s="1575" t="n"/>
+      <c r="S11" s="1575" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1532" t="n"/>
+      <c r="U11" s="1574" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -6008,39 +6134,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1507" t="inlineStr">
+      <c r="A12" s="1549" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1508" t="inlineStr">
+      <c r="B12" s="1550" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1508" t="inlineStr">
+      <c r="C12" s="1550" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1509" t="n"/>
-      <c r="E12" s="1509" t="n"/>
-      <c r="F12" s="1509" t="n"/>
-      <c r="G12" s="1509" t="n"/>
-      <c r="H12" s="1509" t="n"/>
-      <c r="I12" s="1510" t="n"/>
-      <c r="J12" s="1511" t="n"/>
-      <c r="K12" s="1511" t="n"/>
-      <c r="L12" s="1511" t="n"/>
-      <c r="M12" s="1509" t="n"/>
-      <c r="N12" s="1509" t="n"/>
-      <c r="O12" s="1509" t="n"/>
-      <c r="P12" s="1512" t="n"/>
-      <c r="Q12" s="1509" t="n"/>
-      <c r="R12" s="1509" t="n"/>
-      <c r="S12" s="1509" t="n"/>
+      <c r="D12" s="1551" t="n"/>
+      <c r="E12" s="1551" t="n"/>
+      <c r="F12" s="1551" t="n"/>
+      <c r="G12" s="1551" t="n"/>
+      <c r="H12" s="1551" t="n"/>
+      <c r="I12" s="1552" t="n"/>
+      <c r="J12" s="1553" t="n"/>
+      <c r="K12" s="1553" t="n"/>
+      <c r="L12" s="1553" t="n"/>
+      <c r="M12" s="1551" t="n"/>
+      <c r="N12" s="1551" t="n"/>
+      <c r="O12" s="1551" t="n"/>
+      <c r="P12" s="1554" t="n"/>
+      <c r="Q12" s="1551" t="n"/>
+      <c r="R12" s="1551" t="n"/>
+      <c r="S12" s="1551" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1508" t="n"/>
+      <c r="U12" s="1550" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -6048,35 +6174,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1513" t="inlineStr">
+      <c r="A13" s="1555" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1514" t="n"/>
-      <c r="C13" s="1514" t="inlineStr">
+      <c r="B13" s="1556" t="n"/>
+      <c r="C13" s="1556" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1515" t="n"/>
-      <c r="E13" s="1515" t="n"/>
-      <c r="F13" s="1515" t="n"/>
-      <c r="G13" s="1515" t="n"/>
-      <c r="H13" s="1515" t="n"/>
-      <c r="I13" s="1516" t="n"/>
-      <c r="J13" s="1517" t="n"/>
-      <c r="K13" s="1517" t="n"/>
-      <c r="L13" s="1517" t="n"/>
-      <c r="M13" s="1515" t="n"/>
-      <c r="N13" s="1515" t="n"/>
-      <c r="O13" s="1515" t="n"/>
-      <c r="P13" s="1518" t="n"/>
-      <c r="Q13" s="1515" t="n"/>
-      <c r="R13" s="1515" t="n"/>
-      <c r="S13" s="1515" t="n"/>
+      <c r="D13" s="1557" t="n"/>
+      <c r="E13" s="1557" t="n"/>
+      <c r="F13" s="1557" t="n"/>
+      <c r="G13" s="1557" t="n"/>
+      <c r="H13" s="1557" t="n"/>
+      <c r="I13" s="1558" t="n"/>
+      <c r="J13" s="1559" t="n"/>
+      <c r="K13" s="1559" t="n"/>
+      <c r="L13" s="1559" t="n"/>
+      <c r="M13" s="1557" t="n"/>
+      <c r="N13" s="1557" t="n"/>
+      <c r="O13" s="1557" t="n"/>
+      <c r="P13" s="1560" t="n"/>
+      <c r="Q13" s="1557" t="n"/>
+      <c r="R13" s="1557" t="n"/>
+      <c r="S13" s="1557" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1514" t="n"/>
+      <c r="U13" s="1556" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -6084,53 +6210,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1519" t="inlineStr">
+      <c r="A14" s="1561" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1520" t="inlineStr">
+      <c r="B14" s="1562" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1520" t="inlineStr">
+      <c r="C14" s="1562" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1521" t="n"/>
-      <c r="E14" s="1521" t="n">
+      <c r="D14" s="1563" t="n"/>
+      <c r="E14" s="1563" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1521" t="n">
+      <c r="F14" s="1563" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1521" t="n">
+      <c r="G14" s="1563" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1521" t="n"/>
-      <c r="I14" s="1522" t="n"/>
-      <c r="J14" s="1523" t="n"/>
-      <c r="K14" s="1523" t="n"/>
-      <c r="L14" s="1523" t="n"/>
-      <c r="M14" s="1521" t="n"/>
-      <c r="N14" s="1521" t="n"/>
-      <c r="O14" s="1521" t="n">
+      <c r="H14" s="1563" t="n"/>
+      <c r="I14" s="1564" t="n"/>
+      <c r="J14" s="1565" t="n"/>
+      <c r="K14" s="1565" t="n"/>
+      <c r="L14" s="1565" t="n"/>
+      <c r="M14" s="1563" t="n"/>
+      <c r="N14" s="1563" t="n"/>
+      <c r="O14" s="1563" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1524" t="n">
+      <c r="P14" s="1566" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1521" t="n"/>
-      <c r="R14" s="1521" t="n"/>
-      <c r="S14" s="1521" t="n"/>
+      <c r="Q14" s="1563" t="n"/>
+      <c r="R14" s="1563" t="n"/>
+      <c r="S14" s="1563" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1520" t="n"/>
+      <c r="U14" s="1562" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -6138,43 +6264,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1519" t="inlineStr">
+      <c r="A15" s="1561" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1520" t="inlineStr">
+      <c r="B15" s="1562" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1520" t="inlineStr">
+      <c r="C15" s="1562" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1521" t="n"/>
-      <c r="E15" s="1521" t="n"/>
-      <c r="F15" s="1521" t="n"/>
-      <c r="G15" s="1521" t="n"/>
-      <c r="H15" s="1521" t="n"/>
-      <c r="I15" s="1522" t="n"/>
-      <c r="J15" s="1523" t="n"/>
-      <c r="K15" s="1523" t="n"/>
-      <c r="L15" s="1523" t="n"/>
-      <c r="M15" s="1521" t="n">
+      <c r="D15" s="1563" t="n"/>
+      <c r="E15" s="1563" t="n"/>
+      <c r="F15" s="1563" t="n"/>
+      <c r="G15" s="1563" t="n"/>
+      <c r="H15" s="1563" t="n"/>
+      <c r="I15" s="1564" t="n"/>
+      <c r="J15" s="1565" t="n"/>
+      <c r="K15" s="1565" t="n"/>
+      <c r="L15" s="1565" t="n"/>
+      <c r="M15" s="1563" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1521" t="n">
+      <c r="N15" s="1563" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1521" t="n"/>
-      <c r="P15" s="1524" t="n"/>
-      <c r="Q15" s="1521" t="n"/>
-      <c r="R15" s="1521" t="n"/>
-      <c r="S15" s="1521" t="n"/>
+      <c r="O15" s="1563" t="n"/>
+      <c r="P15" s="1566" t="n"/>
+      <c r="Q15" s="1563" t="n"/>
+      <c r="R15" s="1563" t="n"/>
+      <c r="S15" s="1563" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1520" t="n"/>
+      <c r="U15" s="1562" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -6182,39 +6308,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1525" t="inlineStr">
+      <c r="A16" s="1567" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1526" t="inlineStr">
+      <c r="B16" s="1568" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1526" t="inlineStr">
+      <c r="C16" s="1568" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1527" t="n"/>
-      <c r="E16" s="1527" t="n"/>
-      <c r="F16" s="1527" t="n"/>
-      <c r="G16" s="1527" t="n"/>
-      <c r="H16" s="1527" t="n"/>
-      <c r="I16" s="1528" t="n"/>
-      <c r="J16" s="1529" t="n"/>
-      <c r="K16" s="1529" t="n"/>
-      <c r="L16" s="1529" t="n"/>
-      <c r="M16" s="1527" t="n"/>
-      <c r="N16" s="1527" t="n"/>
-      <c r="O16" s="1527" t="n"/>
-      <c r="P16" s="1530" t="n"/>
-      <c r="Q16" s="1527" t="n"/>
-      <c r="R16" s="1527" t="n"/>
-      <c r="S16" s="1527" t="n"/>
+      <c r="D16" s="1569" t="n"/>
+      <c r="E16" s="1569" t="n"/>
+      <c r="F16" s="1569" t="n"/>
+      <c r="G16" s="1569" t="n"/>
+      <c r="H16" s="1569" t="n"/>
+      <c r="I16" s="1570" t="n"/>
+      <c r="J16" s="1571" t="n"/>
+      <c r="K16" s="1571" t="n"/>
+      <c r="L16" s="1571" t="n"/>
+      <c r="M16" s="1569" t="n"/>
+      <c r="N16" s="1569" t="n"/>
+      <c r="O16" s="1569" t="n"/>
+      <c r="P16" s="1572" t="n"/>
+      <c r="Q16" s="1569" t="n"/>
+      <c r="R16" s="1569" t="n"/>
+      <c r="S16" s="1569" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1526" t="n"/>
+      <c r="U16" s="1568" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -6222,39 +6348,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1501" t="inlineStr">
+      <c r="A17" s="1543" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1502" t="inlineStr">
+      <c r="B17" s="1544" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1502" t="inlineStr">
+      <c r="C17" s="1544" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1503" t="n"/>
-      <c r="E17" s="1503" t="n"/>
-      <c r="F17" s="1503" t="n"/>
-      <c r="G17" s="1503" t="n"/>
-      <c r="H17" s="1503" t="n"/>
-      <c r="I17" s="1504" t="n"/>
-      <c r="J17" s="1505" t="n"/>
-      <c r="K17" s="1505" t="n"/>
-      <c r="L17" s="1505" t="n"/>
-      <c r="M17" s="1503" t="n"/>
-      <c r="N17" s="1503" t="n"/>
-      <c r="O17" s="1503" t="n"/>
-      <c r="P17" s="1506" t="n"/>
-      <c r="Q17" s="1503" t="n"/>
-      <c r="R17" s="1503" t="n"/>
-      <c r="S17" s="1503" t="n"/>
+      <c r="D17" s="1545" t="n"/>
+      <c r="E17" s="1545" t="n"/>
+      <c r="F17" s="1545" t="n"/>
+      <c r="G17" s="1545" t="n"/>
+      <c r="H17" s="1545" t="n"/>
+      <c r="I17" s="1546" t="n"/>
+      <c r="J17" s="1547" t="n"/>
+      <c r="K17" s="1547" t="n"/>
+      <c r="L17" s="1547" t="n"/>
+      <c r="M17" s="1545" t="n"/>
+      <c r="N17" s="1545" t="n"/>
+      <c r="O17" s="1545" t="n"/>
+      <c r="P17" s="1548" t="n"/>
+      <c r="Q17" s="1545" t="n"/>
+      <c r="R17" s="1545" t="n"/>
+      <c r="S17" s="1545" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1502" t="n"/>
+      <c r="U17" s="1544" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -6262,53 +6388,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1531" t="inlineStr">
+      <c r="A18" s="1573" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1532" t="inlineStr">
+      <c r="B18" s="1574" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1532" t="inlineStr">
+      <c r="C18" s="1574" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1533" t="n"/>
-      <c r="E18" s="1533" t="n">
+      <c r="D18" s="1575" t="n"/>
+      <c r="E18" s="1575" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1533" t="n">
+      <c r="F18" s="1575" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1533" t="n">
+      <c r="G18" s="1575" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1533" t="n"/>
-      <c r="I18" s="1534" t="n"/>
-      <c r="J18" s="1535" t="n"/>
-      <c r="K18" s="1535" t="n"/>
-      <c r="L18" s="1535" t="n"/>
-      <c r="M18" s="1533" t="n"/>
-      <c r="N18" s="1533" t="n"/>
-      <c r="O18" s="1533" t="n">
+      <c r="H18" s="1575" t="n"/>
+      <c r="I18" s="1576" t="n"/>
+      <c r="J18" s="1577" t="n"/>
+      <c r="K18" s="1577" t="n"/>
+      <c r="L18" s="1577" t="n"/>
+      <c r="M18" s="1575" t="n"/>
+      <c r="N18" s="1575" t="n"/>
+      <c r="O18" s="1575" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1536" t="n">
+      <c r="P18" s="1578" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1533" t="n"/>
-      <c r="R18" s="1533" t="n"/>
-      <c r="S18" s="1533" t="n"/>
+      <c r="Q18" s="1575" t="n"/>
+      <c r="R18" s="1575" t="n"/>
+      <c r="S18" s="1575" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1532" t="n"/>
+      <c r="U18" s="1574" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -6316,47 +6442,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1531" t="inlineStr">
+      <c r="A19" s="1573" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1532" t="inlineStr">
+      <c r="B19" s="1574" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1532" t="inlineStr">
+      <c r="C19" s="1574" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1533" t="n"/>
-      <c r="E19" s="1533" t="n"/>
-      <c r="F19" s="1533" t="n"/>
-      <c r="G19" s="1533" t="n"/>
-      <c r="H19" s="1533" t="n"/>
-      <c r="I19" s="1534" t="n"/>
-      <c r="J19" s="1535" t="n"/>
-      <c r="K19" s="1535" t="n"/>
-      <c r="L19" s="1535" t="n"/>
-      <c r="M19" s="1533" t="n">
+      <c r="D19" s="1575" t="n"/>
+      <c r="E19" s="1575" t="n"/>
+      <c r="F19" s="1575" t="n"/>
+      <c r="G19" s="1575" t="n"/>
+      <c r="H19" s="1575" t="n"/>
+      <c r="I19" s="1576" t="n"/>
+      <c r="J19" s="1577" t="n"/>
+      <c r="K19" s="1577" t="n"/>
+      <c r="L19" s="1577" t="n"/>
+      <c r="M19" s="1575" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1533" t="n">
+      <c r="N19" s="1575" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1533" t="n"/>
-      <c r="P19" s="1536" t="n"/>
-      <c r="Q19" s="1533" t="n"/>
-      <c r="R19" s="1533" t="n"/>
-      <c r="S19" s="1533" t="n"/>
+      <c r="O19" s="1575" t="n"/>
+      <c r="P19" s="1578" t="n"/>
+      <c r="Q19" s="1575" t="n"/>
+      <c r="R19" s="1575" t="n"/>
+      <c r="S19" s="1575" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1532" t="n"/>
+      <c r="U19" s="1574" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -6364,43 +6490,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1531" t="inlineStr">
+      <c r="A20" s="1573" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1532" t="inlineStr">
+      <c r="B20" s="1574" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1532" t="inlineStr">
+      <c r="C20" s="1574" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1533" t="n"/>
-      <c r="E20" s="1533" t="n"/>
-      <c r="F20" s="1533" t="n"/>
-      <c r="G20" s="1533" t="n"/>
-      <c r="H20" s="1533" t="n"/>
-      <c r="I20" s="1534" t="n"/>
-      <c r="J20" s="1535" t="n"/>
-      <c r="K20" s="1535" t="n"/>
-      <c r="L20" s="1535" t="n"/>
-      <c r="M20" s="1533" t="n"/>
-      <c r="N20" s="1533" t="n"/>
-      <c r="O20" s="1533" t="n"/>
-      <c r="P20" s="1536" t="n"/>
-      <c r="Q20" s="1533" t="n"/>
-      <c r="R20" s="1533" t="n"/>
-      <c r="S20" s="1533" t="n"/>
+      <c r="D20" s="1575" t="n"/>
+      <c r="E20" s="1575" t="n"/>
+      <c r="F20" s="1575" t="n"/>
+      <c r="G20" s="1575" t="n"/>
+      <c r="H20" s="1575" t="n"/>
+      <c r="I20" s="1576" t="n"/>
+      <c r="J20" s="1577" t="n"/>
+      <c r="K20" s="1577" t="n"/>
+      <c r="L20" s="1577" t="n"/>
+      <c r="M20" s="1575" t="n"/>
+      <c r="N20" s="1575" t="n"/>
+      <c r="O20" s="1575" t="n"/>
+      <c r="P20" s="1578" t="n"/>
+      <c r="Q20" s="1575" t="n"/>
+      <c r="R20" s="1575" t="n"/>
+      <c r="S20" s="1575" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1532" t="n"/>
+      <c r="U20" s="1574" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -6408,39 +6534,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1507" t="inlineStr">
+      <c r="A21" s="1549" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1508" t="inlineStr">
+      <c r="B21" s="1550" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1508" t="inlineStr">
+      <c r="C21" s="1550" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1509" t="n"/>
-      <c r="E21" s="1509" t="n"/>
-      <c r="F21" s="1509" t="n"/>
-      <c r="G21" s="1509" t="n"/>
-      <c r="H21" s="1509" t="n"/>
-      <c r="I21" s="1510" t="n"/>
-      <c r="J21" s="1511" t="n"/>
-      <c r="K21" s="1511" t="n"/>
-      <c r="L21" s="1511" t="n"/>
-      <c r="M21" s="1509" t="n"/>
-      <c r="N21" s="1509" t="n"/>
-      <c r="O21" s="1509" t="n"/>
-      <c r="P21" s="1512" t="n"/>
-      <c r="Q21" s="1509" t="n"/>
-      <c r="R21" s="1509" t="n"/>
-      <c r="S21" s="1509" t="n"/>
+      <c r="D21" s="1551" t="n"/>
+      <c r="E21" s="1551" t="n"/>
+      <c r="F21" s="1551" t="n"/>
+      <c r="G21" s="1551" t="n"/>
+      <c r="H21" s="1551" t="n"/>
+      <c r="I21" s="1552" t="n"/>
+      <c r="J21" s="1553" t="n"/>
+      <c r="K21" s="1553" t="n"/>
+      <c r="L21" s="1553" t="n"/>
+      <c r="M21" s="1551" t="n"/>
+      <c r="N21" s="1551" t="n"/>
+      <c r="O21" s="1551" t="n"/>
+      <c r="P21" s="1554" t="n"/>
+      <c r="Q21" s="1551" t="n"/>
+      <c r="R21" s="1551" t="n"/>
+      <c r="S21" s="1551" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1508" t="n"/>
+      <c r="U21" s="1550" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -6448,39 +6574,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1513" t="inlineStr">
+      <c r="A22" s="1555" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1514" t="inlineStr">
+      <c r="B22" s="1556" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1514" t="inlineStr">
+      <c r="C22" s="1556" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1515" t="n"/>
-      <c r="E22" s="1515" t="n"/>
-      <c r="F22" s="1515" t="n"/>
-      <c r="G22" s="1515" t="n"/>
-      <c r="H22" s="1515" t="n"/>
-      <c r="I22" s="1516" t="n"/>
-      <c r="J22" s="1517" t="n"/>
-      <c r="K22" s="1517" t="n"/>
-      <c r="L22" s="1517" t="n"/>
-      <c r="M22" s="1515" t="n"/>
-      <c r="N22" s="1515" t="n"/>
-      <c r="O22" s="1515" t="n"/>
-      <c r="P22" s="1518" t="n"/>
-      <c r="Q22" s="1515" t="n"/>
-      <c r="R22" s="1515" t="n"/>
-      <c r="S22" s="1515" t="n"/>
+      <c r="D22" s="1557" t="n"/>
+      <c r="E22" s="1557" t="n"/>
+      <c r="F22" s="1557" t="n"/>
+      <c r="G22" s="1557" t="n"/>
+      <c r="H22" s="1557" t="n"/>
+      <c r="I22" s="1558" t="n"/>
+      <c r="J22" s="1559" t="n"/>
+      <c r="K22" s="1559" t="n"/>
+      <c r="L22" s="1559" t="n"/>
+      <c r="M22" s="1557" t="n"/>
+      <c r="N22" s="1557" t="n"/>
+      <c r="O22" s="1557" t="n"/>
+      <c r="P22" s="1560" t="n"/>
+      <c r="Q22" s="1557" t="n"/>
+      <c r="R22" s="1557" t="n"/>
+      <c r="S22" s="1557" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1514" t="n"/>
+      <c r="U22" s="1556" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -6488,53 +6614,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1519" t="inlineStr">
+      <c r="A23" s="1561" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1520" t="inlineStr">
+      <c r="B23" s="1562" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1520" t="inlineStr">
+      <c r="C23" s="1562" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1521" t="n"/>
-      <c r="E23" s="1521" t="n">
+      <c r="D23" s="1563" t="n"/>
+      <c r="E23" s="1563" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1521" t="n">
+      <c r="F23" s="1563" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1521" t="n">
+      <c r="G23" s="1563" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1521" t="n"/>
-      <c r="I23" s="1522" t="n"/>
-      <c r="J23" s="1523" t="n"/>
-      <c r="K23" s="1523" t="n"/>
-      <c r="L23" s="1523" t="n"/>
-      <c r="M23" s="1521" t="n"/>
-      <c r="N23" s="1521" t="n"/>
-      <c r="O23" s="1521" t="n">
+      <c r="H23" s="1563" t="n"/>
+      <c r="I23" s="1564" t="n"/>
+      <c r="J23" s="1565" t="n"/>
+      <c r="K23" s="1565" t="n"/>
+      <c r="L23" s="1565" t="n"/>
+      <c r="M23" s="1563" t="n"/>
+      <c r="N23" s="1563" t="n"/>
+      <c r="O23" s="1563" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1524" t="n">
+      <c r="P23" s="1566" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1521" t="n"/>
-      <c r="R23" s="1521" t="n"/>
-      <c r="S23" s="1521" t="n"/>
+      <c r="Q23" s="1563" t="n"/>
+      <c r="R23" s="1563" t="n"/>
+      <c r="S23" s="1563" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1520" t="n"/>
+      <c r="U23" s="1562" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -6542,47 +6668,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1525" t="inlineStr">
+      <c r="A24" s="1567" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1526" t="inlineStr">
+      <c r="B24" s="1568" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1526" t="inlineStr">
+      <c r="C24" s="1568" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1527" t="n"/>
-      <c r="E24" s="1527" t="n"/>
-      <c r="F24" s="1527" t="n"/>
-      <c r="G24" s="1527" t="n"/>
-      <c r="H24" s="1527" t="n"/>
-      <c r="I24" s="1528" t="n"/>
-      <c r="J24" s="1529" t="n"/>
-      <c r="K24" s="1529" t="n"/>
-      <c r="L24" s="1529" t="n"/>
-      <c r="M24" s="1527" t="n">
+      <c r="D24" s="1569" t="n"/>
+      <c r="E24" s="1569" t="n"/>
+      <c r="F24" s="1569" t="n"/>
+      <c r="G24" s="1569" t="n"/>
+      <c r="H24" s="1569" t="n"/>
+      <c r="I24" s="1570" t="n"/>
+      <c r="J24" s="1571" t="n"/>
+      <c r="K24" s="1571" t="n"/>
+      <c r="L24" s="1571" t="n"/>
+      <c r="M24" s="1569" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1527" t="n">
+      <c r="N24" s="1569" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1527" t="n"/>
-      <c r="P24" s="1530" t="n"/>
-      <c r="Q24" s="1527" t="n"/>
-      <c r="R24" s="1527" t="n"/>
-      <c r="S24" s="1527" t="n"/>
+      <c r="O24" s="1569" t="n"/>
+      <c r="P24" s="1572" t="n"/>
+      <c r="Q24" s="1569" t="n"/>
+      <c r="R24" s="1569" t="n"/>
+      <c r="S24" s="1569" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1526" t="n"/>
+      <c r="U24" s="1568" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -6590,61 +6716,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1501" t="inlineStr">
+      <c r="A25" s="1543" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1502" t="inlineStr">
+      <c r="B25" s="1544" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1502" t="inlineStr">
+      <c r="C25" s="1544" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1503" t="n">
+      <c r="D25" s="1545" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1503" t="n">
+      <c r="E25" s="1545" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1503" t="n">
+      <c r="F25" s="1545" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1503" t="n">
+      <c r="G25" s="1545" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1503" t="n"/>
-      <c r="I25" s="1504" t="n"/>
-      <c r="J25" s="1505" t="n">
+      <c r="H25" s="1545" t="n"/>
+      <c r="I25" s="1546" t="n"/>
+      <c r="J25" s="1547" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1505" t="n">
+      <c r="K25" s="1547" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1505" t="n">
+      <c r="L25" s="1547" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1503" t="n"/>
-      <c r="N25" s="1503" t="n"/>
-      <c r="O25" s="1503" t="n">
+      <c r="M25" s="1545" t="n"/>
+      <c r="N25" s="1545" t="n"/>
+      <c r="O25" s="1545" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1506" t="n">
+      <c r="P25" s="1548" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1503" t="n"/>
-      <c r="R25" s="1503" t="n"/>
-      <c r="S25" s="1503" t="n"/>
+      <c r="Q25" s="1545" t="n"/>
+      <c r="R25" s="1545" t="n"/>
+      <c r="S25" s="1545" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1502" t="n"/>
+      <c r="U25" s="1544" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -6652,47 +6778,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1507" t="inlineStr">
+      <c r="A26" s="1549" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1508" t="inlineStr">
+      <c r="B26" s="1550" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1508" t="inlineStr">
+      <c r="C26" s="1550" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1509" t="n"/>
-      <c r="E26" s="1509" t="n"/>
-      <c r="F26" s="1509" t="n"/>
-      <c r="G26" s="1509" t="n"/>
-      <c r="H26" s="1509" t="n"/>
-      <c r="I26" s="1510" t="n"/>
-      <c r="J26" s="1511" t="n"/>
-      <c r="K26" s="1511" t="n"/>
-      <c r="L26" s="1511" t="n"/>
-      <c r="M26" s="1509" t="n">
+      <c r="D26" s="1551" t="n"/>
+      <c r="E26" s="1551" t="n"/>
+      <c r="F26" s="1551" t="n"/>
+      <c r="G26" s="1551" t="n"/>
+      <c r="H26" s="1551" t="n"/>
+      <c r="I26" s="1552" t="n"/>
+      <c r="J26" s="1553" t="n"/>
+      <c r="K26" s="1553" t="n"/>
+      <c r="L26" s="1553" t="n"/>
+      <c r="M26" s="1551" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1509" t="n">
+      <c r="N26" s="1551" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1509" t="n"/>
-      <c r="P26" s="1512" t="n"/>
-      <c r="Q26" s="1509" t="n"/>
-      <c r="R26" s="1509" t="n"/>
-      <c r="S26" s="1509" t="n"/>
+      <c r="O26" s="1551" t="n"/>
+      <c r="P26" s="1554" t="n"/>
+      <c r="Q26" s="1551" t="n"/>
+      <c r="R26" s="1551" t="n"/>
+      <c r="S26" s="1551" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1508" t="n"/>
+      <c r="U26" s="1550" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -6700,53 +6826,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1513" t="inlineStr">
+      <c r="A27" s="1555" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1514" t="inlineStr">
+      <c r="B27" s="1556" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1514" t="inlineStr">
+      <c r="C27" s="1556" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1515" t="n"/>
-      <c r="E27" s="1515" t="n">
+      <c r="D27" s="1557" t="n"/>
+      <c r="E27" s="1557" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1515" t="n">
+      <c r="F27" s="1557" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1515" t="n">
+      <c r="G27" s="1557" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1515" t="n"/>
-      <c r="I27" s="1516" t="n"/>
-      <c r="J27" s="1517" t="n"/>
-      <c r="K27" s="1517" t="n"/>
-      <c r="L27" s="1517" t="n"/>
-      <c r="M27" s="1515" t="n"/>
-      <c r="N27" s="1515" t="n"/>
-      <c r="O27" s="1515" t="n">
+      <c r="H27" s="1557" t="n"/>
+      <c r="I27" s="1558" t="n"/>
+      <c r="J27" s="1559" t="n"/>
+      <c r="K27" s="1559" t="n"/>
+      <c r="L27" s="1559" t="n"/>
+      <c r="M27" s="1557" t="n"/>
+      <c r="N27" s="1557" t="n"/>
+      <c r="O27" s="1557" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1518" t="n">
+      <c r="P27" s="1560" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1515" t="n"/>
-      <c r="R27" s="1515" t="n"/>
-      <c r="S27" s="1515" t="n"/>
+      <c r="Q27" s="1557" t="n"/>
+      <c r="R27" s="1557" t="n"/>
+      <c r="S27" s="1557" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1514" t="n"/>
+      <c r="U27" s="1556" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -6754,47 +6880,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1525" t="inlineStr">
+      <c r="A28" s="1567" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1526" t="inlineStr">
+      <c r="B28" s="1568" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1526" t="inlineStr">
+      <c r="C28" s="1568" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1527" t="n"/>
-      <c r="E28" s="1527" t="n"/>
-      <c r="F28" s="1527" t="n"/>
-      <c r="G28" s="1527" t="n"/>
-      <c r="H28" s="1527" t="n"/>
-      <c r="I28" s="1528" t="n"/>
-      <c r="J28" s="1529" t="n"/>
-      <c r="K28" s="1529" t="n"/>
-      <c r="L28" s="1529" t="n"/>
-      <c r="M28" s="1527" t="n">
+      <c r="D28" s="1569" t="n"/>
+      <c r="E28" s="1569" t="n"/>
+      <c r="F28" s="1569" t="n"/>
+      <c r="G28" s="1569" t="n"/>
+      <c r="H28" s="1569" t="n"/>
+      <c r="I28" s="1570" t="n"/>
+      <c r="J28" s="1571" t="n"/>
+      <c r="K28" s="1571" t="n"/>
+      <c r="L28" s="1571" t="n"/>
+      <c r="M28" s="1569" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1527" t="n">
+      <c r="N28" s="1569" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1527" t="n"/>
-      <c r="P28" s="1530" t="n"/>
-      <c r="Q28" s="1527" t="n"/>
-      <c r="R28" s="1527" t="n"/>
-      <c r="S28" s="1527" t="n"/>
+      <c r="O28" s="1569" t="n"/>
+      <c r="P28" s="1572" t="n"/>
+      <c r="Q28" s="1569" t="n"/>
+      <c r="R28" s="1569" t="n"/>
+      <c r="S28" s="1569" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1526" t="n"/>
+      <c r="U28" s="1568" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -6802,53 +6928,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1501" t="inlineStr">
+      <c r="A29" s="1543" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1502" t="inlineStr">
+      <c r="B29" s="1544" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1502" t="inlineStr">
+      <c r="C29" s="1544" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1503" t="n"/>
-      <c r="E29" s="1503" t="n">
+      <c r="D29" s="1545" t="n"/>
+      <c r="E29" s="1545" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1503" t="n">
+      <c r="F29" s="1545" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1503" t="n">
+      <c r="G29" s="1545" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1503" t="n"/>
-      <c r="I29" s="1504" t="n"/>
-      <c r="J29" s="1505" t="n"/>
-      <c r="K29" s="1505" t="n"/>
-      <c r="L29" s="1505" t="n"/>
-      <c r="M29" s="1503" t="n"/>
-      <c r="N29" s="1503" t="n"/>
-      <c r="O29" s="1503" t="n">
+      <c r="H29" s="1545" t="n"/>
+      <c r="I29" s="1546" t="n"/>
+      <c r="J29" s="1547" t="n"/>
+      <c r="K29" s="1547" t="n"/>
+      <c r="L29" s="1547" t="n"/>
+      <c r="M29" s="1545" t="n"/>
+      <c r="N29" s="1545" t="n"/>
+      <c r="O29" s="1545" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1506" t="n">
+      <c r="P29" s="1548" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1503" t="n"/>
-      <c r="R29" s="1503" t="n"/>
-      <c r="S29" s="1503" t="n"/>
+      <c r="Q29" s="1545" t="n"/>
+      <c r="R29" s="1545" t="n"/>
+      <c r="S29" s="1545" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1502" t="n"/>
+      <c r="U29" s="1544" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -6856,43 +6982,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1507" t="inlineStr">
+      <c r="A30" s="1549" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1508" t="inlineStr">
+      <c r="B30" s="1550" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1508" t="inlineStr">
+      <c r="C30" s="1550" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1509" t="n"/>
-      <c r="E30" s="1509" t="n"/>
-      <c r="F30" s="1509" t="n"/>
-      <c r="G30" s="1509" t="n"/>
-      <c r="H30" s="1509" t="n"/>
-      <c r="I30" s="1510" t="n"/>
-      <c r="J30" s="1511" t="n"/>
-      <c r="K30" s="1511" t="n"/>
-      <c r="L30" s="1511" t="n"/>
-      <c r="M30" s="1509" t="n"/>
-      <c r="N30" s="1509" t="n"/>
-      <c r="O30" s="1509" t="n"/>
-      <c r="P30" s="1512" t="n"/>
-      <c r="Q30" s="1509" t="n"/>
-      <c r="R30" s="1509" t="n"/>
-      <c r="S30" s="1509" t="n"/>
+      <c r="D30" s="1551" t="n"/>
+      <c r="E30" s="1551" t="n"/>
+      <c r="F30" s="1551" t="n"/>
+      <c r="G30" s="1551" t="n"/>
+      <c r="H30" s="1551" t="n"/>
+      <c r="I30" s="1552" t="n"/>
+      <c r="J30" s="1553" t="n"/>
+      <c r="K30" s="1553" t="n"/>
+      <c r="L30" s="1553" t="n"/>
+      <c r="M30" s="1551" t="n"/>
+      <c r="N30" s="1551" t="n"/>
+      <c r="O30" s="1551" t="n"/>
+      <c r="P30" s="1554" t="n"/>
+      <c r="Q30" s="1551" t="n"/>
+      <c r="R30" s="1551" t="n"/>
+      <c r="S30" s="1551" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1508" t="n"/>
+      <c r="U30" s="1550" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -6900,53 +7026,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1513" t="inlineStr">
+      <c r="A31" s="1555" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1514" t="inlineStr">
+      <c r="B31" s="1556" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1514" t="inlineStr">
+      <c r="C31" s="1556" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1515" t="n"/>
-      <c r="E31" s="1515" t="n">
+      <c r="D31" s="1557" t="n"/>
+      <c r="E31" s="1557" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1515" t="n">
+      <c r="F31" s="1557" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1515" t="n">
+      <c r="G31" s="1557" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1515" t="n"/>
-      <c r="I31" s="1516" t="n"/>
-      <c r="J31" s="1517" t="n"/>
-      <c r="K31" s="1517" t="n"/>
-      <c r="L31" s="1517" t="n"/>
-      <c r="M31" s="1515" t="n"/>
-      <c r="N31" s="1515" t="n"/>
-      <c r="O31" s="1515" t="n">
+      <c r="H31" s="1557" t="n"/>
+      <c r="I31" s="1558" t="n"/>
+      <c r="J31" s="1559" t="n"/>
+      <c r="K31" s="1559" t="n"/>
+      <c r="L31" s="1559" t="n"/>
+      <c r="M31" s="1557" t="n"/>
+      <c r="N31" s="1557" t="n"/>
+      <c r="O31" s="1557" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1518" t="n">
+      <c r="P31" s="1560" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1515" t="n"/>
-      <c r="R31" s="1515" t="n"/>
-      <c r="S31" s="1515" t="n"/>
+      <c r="Q31" s="1557" t="n"/>
+      <c r="R31" s="1557" t="n"/>
+      <c r="S31" s="1557" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1514" t="inlineStr">
+      <c r="U31" s="1556" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -6958,49 +7084,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1525" t="inlineStr">
+      <c r="A32" s="1567" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1526" t="inlineStr">
+      <c r="B32" s="1568" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1526" t="inlineStr">
+      <c r="C32" s="1568" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1527" t="n"/>
-      <c r="E32" s="1527" t="n"/>
-      <c r="F32" s="1527" t="n"/>
-      <c r="G32" s="1527" t="n"/>
-      <c r="H32" s="1527" t="n">
+      <c r="D32" s="1569" t="n"/>
+      <c r="E32" s="1569" t="n"/>
+      <c r="F32" s="1569" t="n"/>
+      <c r="G32" s="1569" t="n"/>
+      <c r="H32" s="1569" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1528" t="n"/>
-      <c r="J32" s="1529" t="n"/>
-      <c r="K32" s="1529" t="n"/>
-      <c r="L32" s="1529" t="n"/>
-      <c r="M32" s="1527" t="n">
+      <c r="I32" s="1570" t="n"/>
+      <c r="J32" s="1571" t="n"/>
+      <c r="K32" s="1571" t="n"/>
+      <c r="L32" s="1571" t="n"/>
+      <c r="M32" s="1569" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1527" t="n">
+      <c r="N32" s="1569" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1527" t="n"/>
-      <c r="P32" s="1530" t="n"/>
-      <c r="Q32" s="1527" t="n"/>
-      <c r="R32" s="1527" t="n"/>
-      <c r="S32" s="1527" t="n"/>
+      <c r="O32" s="1569" t="n"/>
+      <c r="P32" s="1572" t="n"/>
+      <c r="Q32" s="1569" t="n"/>
+      <c r="R32" s="1569" t="n"/>
+      <c r="S32" s="1569" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1526" t="n"/>
+      <c r="U32" s="1568" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -7008,57 +7134,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1501" t="inlineStr">
+      <c r="A33" s="1543" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1502" t="inlineStr">
+      <c r="B33" s="1544" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1502" t="inlineStr">
+      <c r="C33" s="1544" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1503" t="n"/>
-      <c r="E33" s="1503" t="n">
+      <c r="D33" s="1545" t="n"/>
+      <c r="E33" s="1545" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1503" t="n">
+      <c r="F33" s="1545" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1503" t="n">
+      <c r="G33" s="1545" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1503" t="n"/>
-      <c r="I33" s="1504" t="n">
+      <c r="H33" s="1545" t="n"/>
+      <c r="I33" s="1546" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1505" t="n"/>
-      <c r="K33" s="1505" t="n"/>
-      <c r="L33" s="1505" t="n"/>
-      <c r="M33" s="1503" t="n"/>
-      <c r="N33" s="1503" t="n"/>
-      <c r="O33" s="1503" t="n">
+      <c r="J33" s="1547" t="n"/>
+      <c r="K33" s="1547" t="n"/>
+      <c r="L33" s="1547" t="n"/>
+      <c r="M33" s="1545" t="n"/>
+      <c r="N33" s="1545" t="n"/>
+      <c r="O33" s="1545" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1506" t="n">
+      <c r="P33" s="1548" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1503" t="n"/>
-      <c r="R33" s="1503" t="n">
+      <c r="Q33" s="1545" t="n"/>
+      <c r="R33" s="1545" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1503" t="n"/>
+      <c r="S33" s="1545" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1502" t="inlineStr">
+      <c r="U33" s="1544" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -7070,49 +7196,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1507" t="inlineStr">
+      <c r="A34" s="1549" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1508" t="inlineStr">
+      <c r="B34" s="1550" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1508" t="inlineStr">
+      <c r="C34" s="1550" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1509" t="n"/>
-      <c r="E34" s="1509" t="n"/>
-      <c r="F34" s="1509" t="n"/>
-      <c r="G34" s="1509" t="n"/>
-      <c r="H34" s="1509" t="n">
+      <c r="D34" s="1551" t="n"/>
+      <c r="E34" s="1551" t="n"/>
+      <c r="F34" s="1551" t="n"/>
+      <c r="G34" s="1551" t="n"/>
+      <c r="H34" s="1551" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1510" t="n"/>
-      <c r="J34" s="1511" t="n"/>
-      <c r="K34" s="1511" t="n"/>
-      <c r="L34" s="1511" t="n"/>
-      <c r="M34" s="1509" t="n">
+      <c r="I34" s="1552" t="n"/>
+      <c r="J34" s="1553" t="n"/>
+      <c r="K34" s="1553" t="n"/>
+      <c r="L34" s="1553" t="n"/>
+      <c r="M34" s="1551" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1509" t="n">
+      <c r="N34" s="1551" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1509" t="n"/>
-      <c r="P34" s="1512" t="n"/>
-      <c r="Q34" s="1509" t="n"/>
-      <c r="R34" s="1509" t="n"/>
-      <c r="S34" s="1509" t="n"/>
+      <c r="O34" s="1551" t="n"/>
+      <c r="P34" s="1554" t="n"/>
+      <c r="Q34" s="1551" t="n"/>
+      <c r="R34" s="1551" t="n"/>
+      <c r="S34" s="1551" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1508" t="n"/>
+      <c r="U34" s="1550" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -7120,57 +7246,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1513" t="inlineStr">
+      <c r="A35" s="1555" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1514" t="inlineStr">
+      <c r="B35" s="1556" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1514" t="inlineStr">
+      <c r="C35" s="1556" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1515" t="n"/>
-      <c r="E35" s="1515" t="n">
+      <c r="D35" s="1557" t="n"/>
+      <c r="E35" s="1557" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1515" t="n">
+      <c r="F35" s="1557" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1515" t="n">
+      <c r="G35" s="1557" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1515" t="n"/>
-      <c r="I35" s="1516" t="n">
+      <c r="H35" s="1557" t="n"/>
+      <c r="I35" s="1558" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1517" t="n"/>
-      <c r="K35" s="1517" t="n"/>
-      <c r="L35" s="1517" t="n"/>
-      <c r="M35" s="1515" t="n"/>
-      <c r="N35" s="1515" t="n"/>
-      <c r="O35" s="1515" t="n">
+      <c r="J35" s="1559" t="n"/>
+      <c r="K35" s="1559" t="n"/>
+      <c r="L35" s="1559" t="n"/>
+      <c r="M35" s="1557" t="n"/>
+      <c r="N35" s="1557" t="n"/>
+      <c r="O35" s="1557" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1518" t="n">
+      <c r="P35" s="1560" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1515" t="n"/>
-      <c r="R35" s="1515" t="n">
+      <c r="Q35" s="1557" t="n"/>
+      <c r="R35" s="1557" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1515" t="n"/>
+      <c r="S35" s="1557" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1514" t="inlineStr">
+      <c r="U35" s="1556" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -7182,49 +7308,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1519" t="inlineStr">
+      <c r="A36" s="1561" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1520" t="inlineStr">
+      <c r="B36" s="1562" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1520" t="inlineStr">
+      <c r="C36" s="1562" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1521" t="n"/>
-      <c r="E36" s="1521" t="n"/>
-      <c r="F36" s="1521" t="n"/>
-      <c r="G36" s="1521" t="n"/>
-      <c r="H36" s="1521" t="n">
+      <c r="D36" s="1563" t="n"/>
+      <c r="E36" s="1563" t="n"/>
+      <c r="F36" s="1563" t="n"/>
+      <c r="G36" s="1563" t="n"/>
+      <c r="H36" s="1563" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1522" t="n"/>
-      <c r="J36" s="1523" t="n"/>
-      <c r="K36" s="1523" t="n"/>
-      <c r="L36" s="1523" t="n"/>
-      <c r="M36" s="1521" t="n">
+      <c r="I36" s="1564" t="n"/>
+      <c r="J36" s="1565" t="n"/>
+      <c r="K36" s="1565" t="n"/>
+      <c r="L36" s="1565" t="n"/>
+      <c r="M36" s="1563" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1521" t="n">
+      <c r="N36" s="1563" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1521" t="n"/>
-      <c r="P36" s="1524" t="n"/>
-      <c r="Q36" s="1521" t="n"/>
-      <c r="R36" s="1521" t="n"/>
-      <c r="S36" s="1521" t="n"/>
+      <c r="O36" s="1563" t="n"/>
+      <c r="P36" s="1566" t="n"/>
+      <c r="Q36" s="1563" t="n"/>
+      <c r="R36" s="1563" t="n"/>
+      <c r="S36" s="1563" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1520" t="n"/>
+      <c r="U36" s="1562" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -7232,41 +7358,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1525" t="inlineStr">
+      <c r="A37" s="1567" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1526" t="inlineStr">
+      <c r="B37" s="1568" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1526" t="inlineStr">
+      <c r="C37" s="1568" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1527" t="n"/>
-      <c r="E37" s="1527" t="n"/>
-      <c r="F37" s="1527" t="n"/>
-      <c r="G37" s="1527" t="n"/>
-      <c r="H37" s="1527" t="n"/>
-      <c r="I37" s="1528" t="n"/>
-      <c r="J37" s="1529" t="n"/>
-      <c r="K37" s="1529" t="n"/>
-      <c r="L37" s="1529" t="n"/>
-      <c r="M37" s="1527" t="n"/>
-      <c r="N37" s="1527" t="n"/>
-      <c r="O37" s="1527" t="n"/>
-      <c r="P37" s="1530" t="n"/>
-      <c r="Q37" s="1527" t="n">
+      <c r="D37" s="1569" t="n"/>
+      <c r="E37" s="1569" t="n"/>
+      <c r="F37" s="1569" t="n"/>
+      <c r="G37" s="1569" t="n"/>
+      <c r="H37" s="1569" t="n"/>
+      <c r="I37" s="1570" t="n"/>
+      <c r="J37" s="1571" t="n"/>
+      <c r="K37" s="1571" t="n"/>
+      <c r="L37" s="1571" t="n"/>
+      <c r="M37" s="1569" t="n"/>
+      <c r="N37" s="1569" t="n"/>
+      <c r="O37" s="1569" t="n"/>
+      <c r="P37" s="1572" t="n"/>
+      <c r="Q37" s="1569" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1527" t="n"/>
-      <c r="S37" s="1527" t="n"/>
+      <c r="R37" s="1569" t="n"/>
+      <c r="S37" s="1569" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1526" t="n"/>
+      <c r="U37" s="1568" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -7274,57 +7400,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1501" t="inlineStr">
+      <c r="A38" s="1543" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1502" t="inlineStr">
+      <c r="B38" s="1544" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1502" t="inlineStr">
+      <c r="C38" s="1544" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1503" t="n"/>
-      <c r="E38" s="1503" t="n">
+      <c r="D38" s="1545" t="n"/>
+      <c r="E38" s="1545" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1503" t="n">
+      <c r="F38" s="1545" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1503" t="n">
+      <c r="G38" s="1545" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1503" t="n"/>
-      <c r="I38" s="1504" t="n">
+      <c r="H38" s="1545" t="n"/>
+      <c r="I38" s="1546" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1505" t="n"/>
-      <c r="K38" s="1505" t="n"/>
-      <c r="L38" s="1505" t="n"/>
-      <c r="M38" s="1503" t="n"/>
-      <c r="N38" s="1503" t="n"/>
-      <c r="O38" s="1503" t="n">
+      <c r="J38" s="1547" t="n"/>
+      <c r="K38" s="1547" t="n"/>
+      <c r="L38" s="1547" t="n"/>
+      <c r="M38" s="1545" t="n"/>
+      <c r="N38" s="1545" t="n"/>
+      <c r="O38" s="1545" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1506" t="n">
+      <c r="P38" s="1548" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1503" t="n"/>
-      <c r="R38" s="1503" t="n">
+      <c r="Q38" s="1545" t="n"/>
+      <c r="R38" s="1545" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1503" t="n"/>
+      <c r="S38" s="1545" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1502" t="inlineStr">
+      <c r="U38" s="1544" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -7336,49 +7462,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1531" t="inlineStr">
+      <c r="A39" s="1573" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1532" t="inlineStr">
+      <c r="B39" s="1574" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1532" t="inlineStr">
+      <c r="C39" s="1574" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1533" t="n"/>
-      <c r="E39" s="1533" t="n"/>
-      <c r="F39" s="1533" t="n"/>
-      <c r="G39" s="1533" t="n"/>
-      <c r="H39" s="1533" t="n">
+      <c r="D39" s="1575" t="n"/>
+      <c r="E39" s="1575" t="n"/>
+      <c r="F39" s="1575" t="n"/>
+      <c r="G39" s="1575" t="n"/>
+      <c r="H39" s="1575" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1534" t="n"/>
-      <c r="J39" s="1535" t="n"/>
-      <c r="K39" s="1535" t="n"/>
-      <c r="L39" s="1535" t="n"/>
-      <c r="M39" s="1533" t="n">
+      <c r="I39" s="1576" t="n"/>
+      <c r="J39" s="1577" t="n"/>
+      <c r="K39" s="1577" t="n"/>
+      <c r="L39" s="1577" t="n"/>
+      <c r="M39" s="1575" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1533" t="n">
+      <c r="N39" s="1575" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1533" t="n"/>
-      <c r="P39" s="1536" t="n"/>
-      <c r="Q39" s="1533" t="n"/>
-      <c r="R39" s="1533" t="n"/>
-      <c r="S39" s="1533" t="n"/>
+      <c r="O39" s="1575" t="n"/>
+      <c r="P39" s="1578" t="n"/>
+      <c r="Q39" s="1575" t="n"/>
+      <c r="R39" s="1575" t="n"/>
+      <c r="S39" s="1575" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1532" t="n"/>
+      <c r="U39" s="1574" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -7386,41 +7512,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1507" t="inlineStr">
+      <c r="A40" s="1549" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1508" t="inlineStr">
+      <c r="B40" s="1550" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1508" t="inlineStr">
+      <c r="C40" s="1550" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1509" t="n"/>
-      <c r="E40" s="1509" t="n"/>
-      <c r="F40" s="1509" t="n"/>
-      <c r="G40" s="1509" t="n"/>
-      <c r="H40" s="1509" t="n"/>
-      <c r="I40" s="1510" t="n"/>
-      <c r="J40" s="1511" t="n"/>
-      <c r="K40" s="1511" t="n"/>
-      <c r="L40" s="1511" t="n"/>
-      <c r="M40" s="1509" t="n"/>
-      <c r="N40" s="1509" t="n"/>
-      <c r="O40" s="1509" t="n"/>
-      <c r="P40" s="1512" t="n"/>
-      <c r="Q40" s="1509" t="n">
+      <c r="D40" s="1551" t="n"/>
+      <c r="E40" s="1551" t="n"/>
+      <c r="F40" s="1551" t="n"/>
+      <c r="G40" s="1551" t="n"/>
+      <c r="H40" s="1551" t="n"/>
+      <c r="I40" s="1552" t="n"/>
+      <c r="J40" s="1553" t="n"/>
+      <c r="K40" s="1553" t="n"/>
+      <c r="L40" s="1553" t="n"/>
+      <c r="M40" s="1551" t="n"/>
+      <c r="N40" s="1551" t="n"/>
+      <c r="O40" s="1551" t="n"/>
+      <c r="P40" s="1554" t="n"/>
+      <c r="Q40" s="1551" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1509" t="n"/>
-      <c r="S40" s="1509" t="n"/>
+      <c r="R40" s="1551" t="n"/>
+      <c r="S40" s="1551" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1508" t="n"/>
+      <c r="U40" s="1550" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -7428,57 +7554,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1513" t="inlineStr">
+      <c r="A41" s="1555" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1514" t="inlineStr">
+      <c r="B41" s="1556" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1514" t="inlineStr">
+      <c r="C41" s="1556" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1515" t="n"/>
-      <c r="E41" s="1515" t="n">
+      <c r="D41" s="1557" t="n"/>
+      <c r="E41" s="1557" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1515" t="n">
+      <c r="F41" s="1557" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1515" t="n">
+      <c r="G41" s="1557" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1515" t="n"/>
-      <c r="I41" s="1516" t="n">
+      <c r="H41" s="1557" t="n"/>
+      <c r="I41" s="1558" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1517" t="n"/>
-      <c r="K41" s="1517" t="n"/>
-      <c r="L41" s="1517" t="n"/>
-      <c r="M41" s="1515" t="n"/>
-      <c r="N41" s="1515" t="n"/>
-      <c r="O41" s="1515" t="n">
+      <c r="J41" s="1559" t="n"/>
+      <c r="K41" s="1559" t="n"/>
+      <c r="L41" s="1559" t="n"/>
+      <c r="M41" s="1557" t="n"/>
+      <c r="N41" s="1557" t="n"/>
+      <c r="O41" s="1557" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1518" t="n">
+      <c r="P41" s="1560" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1515" t="n"/>
-      <c r="R41" s="1515" t="n">
+      <c r="Q41" s="1557" t="n"/>
+      <c r="R41" s="1557" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1515" t="n"/>
+      <c r="S41" s="1557" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1514" t="inlineStr">
+      <c r="U41" s="1556" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -7490,49 +7616,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1525" t="inlineStr">
+      <c r="A42" s="1567" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1526" t="inlineStr">
+      <c r="B42" s="1568" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1526" t="inlineStr">
+      <c r="C42" s="1568" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1527" t="n"/>
-      <c r="E42" s="1527" t="n"/>
-      <c r="F42" s="1527" t="n"/>
-      <c r="G42" s="1527" t="n"/>
-      <c r="H42" s="1527" t="n">
+      <c r="D42" s="1569" t="n"/>
+      <c r="E42" s="1569" t="n"/>
+      <c r="F42" s="1569" t="n"/>
+      <c r="G42" s="1569" t="n"/>
+      <c r="H42" s="1569" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1528" t="n"/>
-      <c r="J42" s="1529" t="n"/>
-      <c r="K42" s="1529" t="n"/>
-      <c r="L42" s="1529" t="n"/>
-      <c r="M42" s="1527" t="n">
+      <c r="I42" s="1570" t="n"/>
+      <c r="J42" s="1571" t="n"/>
+      <c r="K42" s="1571" t="n"/>
+      <c r="L42" s="1571" t="n"/>
+      <c r="M42" s="1569" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1527" t="n">
+      <c r="N42" s="1569" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1527" t="n"/>
-      <c r="P42" s="1530" t="n"/>
-      <c r="Q42" s="1527" t="n"/>
-      <c r="R42" s="1527" t="n"/>
-      <c r="S42" s="1527" t="n"/>
+      <c r="O42" s="1569" t="n"/>
+      <c r="P42" s="1572" t="n"/>
+      <c r="Q42" s="1569" t="n"/>
+      <c r="R42" s="1569" t="n"/>
+      <c r="S42" s="1569" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1526" t="n"/>
+      <c r="U42" s="1568" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -7540,57 +7666,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1501" t="inlineStr">
+      <c r="A43" s="1543" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1502" t="inlineStr">
+      <c r="B43" s="1544" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1502" t="inlineStr">
+      <c r="C43" s="1544" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1503" t="n"/>
-      <c r="E43" s="1503" t="n">
+      <c r="D43" s="1545" t="n"/>
+      <c r="E43" s="1545" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1503" t="n">
+      <c r="F43" s="1545" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1503" t="n">
+      <c r="G43" s="1545" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1503" t="n"/>
-      <c r="I43" s="1504" t="n">
+      <c r="H43" s="1545" t="n"/>
+      <c r="I43" s="1546" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1505" t="n"/>
-      <c r="K43" s="1505" t="n"/>
-      <c r="L43" s="1505" t="n"/>
-      <c r="M43" s="1503" t="n"/>
-      <c r="N43" s="1503" t="n"/>
-      <c r="O43" s="1503" t="n">
+      <c r="J43" s="1547" t="n"/>
+      <c r="K43" s="1547" t="n"/>
+      <c r="L43" s="1547" t="n"/>
+      <c r="M43" s="1545" t="n"/>
+      <c r="N43" s="1545" t="n"/>
+      <c r="O43" s="1545" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1506" t="n">
+      <c r="P43" s="1548" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1503" t="n"/>
-      <c r="R43" s="1503" t="n">
+      <c r="Q43" s="1545" t="n"/>
+      <c r="R43" s="1545" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1503" t="n"/>
+      <c r="S43" s="1545" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1502" t="n"/>
+      <c r="U43" s="1544" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -7598,45 +7724,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1531" t="inlineStr">
+      <c r="A44" s="1573" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1532" t="inlineStr">
+      <c r="B44" s="1574" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1532" t="inlineStr">
+      <c r="C44" s="1574" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1533" t="n"/>
-      <c r="E44" s="1533" t="n">
+      <c r="D44" s="1575" t="n"/>
+      <c r="E44" s="1575" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1533" t="n">
+      <c r="F44" s="1575" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1533" t="n"/>
-      <c r="H44" s="1533" t="n"/>
-      <c r="I44" s="1534" t="n"/>
-      <c r="J44" s="1535" t="n"/>
-      <c r="K44" s="1535" t="n"/>
-      <c r="L44" s="1535" t="n"/>
-      <c r="M44" s="1533" t="n"/>
-      <c r="N44" s="1533" t="n"/>
-      <c r="O44" s="1533" t="n"/>
-      <c r="P44" s="1536" t="n"/>
-      <c r="Q44" s="1533" t="n"/>
-      <c r="R44" s="1533" t="n"/>
-      <c r="S44" s="1533" t="n">
+      <c r="G44" s="1575" t="n"/>
+      <c r="H44" s="1575" t="n"/>
+      <c r="I44" s="1576" t="n"/>
+      <c r="J44" s="1577" t="n"/>
+      <c r="K44" s="1577" t="n"/>
+      <c r="L44" s="1577" t="n"/>
+      <c r="M44" s="1575" t="n"/>
+      <c r="N44" s="1575" t="n"/>
+      <c r="O44" s="1575" t="n"/>
+      <c r="P44" s="1578" t="n"/>
+      <c r="Q44" s="1575" t="n"/>
+      <c r="R44" s="1575" t="n"/>
+      <c r="S44" s="1575" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1532" t="inlineStr">
+      <c r="U44" s="1574" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -7648,49 +7774,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1531" t="inlineStr">
+      <c r="A45" s="1573" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1532" t="inlineStr">
+      <c r="B45" s="1574" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1532" t="inlineStr">
+      <c r="C45" s="1574" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1533" t="n"/>
-      <c r="E45" s="1533" t="n"/>
-      <c r="F45" s="1533" t="n"/>
-      <c r="G45" s="1533" t="n"/>
-      <c r="H45" s="1533" t="n">
+      <c r="D45" s="1575" t="n"/>
+      <c r="E45" s="1575" t="n"/>
+      <c r="F45" s="1575" t="n"/>
+      <c r="G45" s="1575" t="n"/>
+      <c r="H45" s="1575" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1534" t="n"/>
-      <c r="J45" s="1535" t="n"/>
-      <c r="K45" s="1535" t="n"/>
-      <c r="L45" s="1535" t="n"/>
-      <c r="M45" s="1533" t="n">
+      <c r="I45" s="1576" t="n"/>
+      <c r="J45" s="1577" t="n"/>
+      <c r="K45" s="1577" t="n"/>
+      <c r="L45" s="1577" t="n"/>
+      <c r="M45" s="1575" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1533" t="n">
+      <c r="N45" s="1575" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1533" t="n"/>
-      <c r="P45" s="1536" t="n"/>
-      <c r="Q45" s="1533" t="n"/>
-      <c r="R45" s="1533" t="n"/>
-      <c r="S45" s="1533" t="n"/>
+      <c r="O45" s="1575" t="n"/>
+      <c r="P45" s="1578" t="n"/>
+      <c r="Q45" s="1575" t="n"/>
+      <c r="R45" s="1575" t="n"/>
+      <c r="S45" s="1575" t="n"/>
       <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1532" t="n"/>
+      <c r="U45" s="1574" t="n"/>
       <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -7698,39 +7824,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1507" t="inlineStr">
+      <c r="A46" s="1549" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B46" s="1508" t="inlineStr">
+      <c r="B46" s="1550" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="C46" s="1508" t="inlineStr">
+      <c r="C46" s="1550" t="inlineStr">
         <is>
           <t>EVENT - Clean</t>
         </is>
       </c>
-      <c r="D46" s="1509" t="n"/>
-      <c r="E46" s="1509" t="n"/>
-      <c r="F46" s="1509" t="n"/>
-      <c r="G46" s="1509" t="n"/>
-      <c r="H46" s="1509" t="n"/>
-      <c r="I46" s="1510" t="n"/>
-      <c r="J46" s="1511" t="n"/>
-      <c r="K46" s="1511" t="n"/>
-      <c r="L46" s="1511" t="n"/>
-      <c r="M46" s="1509" t="n"/>
-      <c r="N46" s="1509" t="n"/>
-      <c r="O46" s="1509" t="n"/>
-      <c r="P46" s="1512" t="n"/>
-      <c r="Q46" s="1509" t="n"/>
-      <c r="R46" s="1509" t="n"/>
-      <c r="S46" s="1509" t="n"/>
+      <c r="D46" s="1551" t="n"/>
+      <c r="E46" s="1551" t="n"/>
+      <c r="F46" s="1551" t="n"/>
+      <c r="G46" s="1551" t="n"/>
+      <c r="H46" s="1551" t="n"/>
+      <c r="I46" s="1552" t="n"/>
+      <c r="J46" s="1553" t="n"/>
+      <c r="K46" s="1553" t="n"/>
+      <c r="L46" s="1553" t="n"/>
+      <c r="M46" s="1551" t="n"/>
+      <c r="N46" s="1551" t="n"/>
+      <c r="O46" s="1551" t="n"/>
+      <c r="P46" s="1554" t="n"/>
+      <c r="Q46" s="1551" t="n"/>
+      <c r="R46" s="1551" t="n"/>
+      <c r="S46" s="1551" t="n"/>
       <c r="T46" s="631" t="n"/>
-      <c r="U46" s="1508" t="n"/>
+      <c r="U46" s="1550" t="n"/>
       <c r="V46" s="632" t="inlineStr">
         <is>
           <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
@@ -7738,51 +7864,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1513" t="inlineStr">
+      <c r="A47" s="1555" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1514" t="inlineStr">
+      <c r="B47" s="1556" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C47" s="1514" t="inlineStr">
+      <c r="C47" s="1556" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D47" s="1515" t="n"/>
-      <c r="E47" s="1515" t="n">
+      <c r="D47" s="1557" t="n"/>
+      <c r="E47" s="1557" t="n">
         <v>16.6</v>
       </c>
-      <c r="F47" s="1515" t="n">
+      <c r="F47" s="1557" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="1515" t="n">
+      <c r="G47" s="1557" t="n">
         <v>4.1</v>
       </c>
-      <c r="H47" s="1515" t="n"/>
-      <c r="I47" s="1516" t="n">
+      <c r="H47" s="1557" t="n"/>
+      <c r="I47" s="1558" t="n">
         <v>0.9</v>
       </c>
-      <c r="J47" s="1517" t="n"/>
-      <c r="K47" s="1517" t="n"/>
-      <c r="L47" s="1517" t="n"/>
-      <c r="M47" s="1515" t="n"/>
-      <c r="N47" s="1515" t="n"/>
-      <c r="O47" s="1515" t="n">
+      <c r="J47" s="1559" t="n"/>
+      <c r="K47" s="1559" t="n"/>
+      <c r="L47" s="1559" t="n"/>
+      <c r="M47" s="1557" t="n"/>
+      <c r="N47" s="1557" t="n"/>
+      <c r="O47" s="1557" t="n">
         <v>13.2</v>
       </c>
-      <c r="P47" s="1518" t="n">
+      <c r="P47" s="1560" t="n">
         <v>0</v>
       </c>
-      <c r="Q47" s="1515" t="n"/>
-      <c r="R47" s="1515" t="n">
+      <c r="Q47" s="1557" t="n"/>
+      <c r="R47" s="1557" t="n">
         <v>84.5</v>
       </c>
-      <c r="S47" s="1515" t="n">
+      <c r="S47" s="1557" t="n">
         <v>11.8</v>
       </c>
       <c r="T47" s="813" t="inlineStr">
@@ -7790,7 +7916,7 @@
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1514" t="inlineStr">
+      <c r="U47" s="1556" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
@@ -7802,49 +7928,49 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1525" t="inlineStr">
+      <c r="A48" s="1567" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B48" s="1526" t="inlineStr">
+      <c r="B48" s="1568" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C48" s="1526" t="inlineStr">
+      <c r="C48" s="1568" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D48" s="1527" t="n"/>
-      <c r="E48" s="1527" t="n"/>
-      <c r="F48" s="1527" t="n"/>
-      <c r="G48" s="1527" t="n"/>
-      <c r="H48" s="1527" t="n">
+      <c r="D48" s="1569" t="n"/>
+      <c r="E48" s="1569" t="n"/>
+      <c r="F48" s="1569" t="n"/>
+      <c r="G48" s="1569" t="n"/>
+      <c r="H48" s="1569" t="n">
         <v>15.1</v>
       </c>
-      <c r="I48" s="1528" t="n"/>
-      <c r="J48" s="1529" t="n"/>
-      <c r="K48" s="1529" t="n"/>
-      <c r="L48" s="1529" t="n"/>
-      <c r="M48" s="1527" t="n">
+      <c r="I48" s="1570" t="n"/>
+      <c r="J48" s="1571" t="n"/>
+      <c r="K48" s="1571" t="n"/>
+      <c r="L48" s="1571" t="n"/>
+      <c r="M48" s="1569" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="1527" t="n">
+      <c r="N48" s="1569" t="n">
         <v>20</v>
       </c>
-      <c r="O48" s="1527" t="n"/>
-      <c r="P48" s="1530" t="n"/>
-      <c r="Q48" s="1527" t="n"/>
-      <c r="R48" s="1527" t="n"/>
-      <c r="S48" s="1527" t="n"/>
+      <c r="O48" s="1569" t="n"/>
+      <c r="P48" s="1572" t="n"/>
+      <c r="Q48" s="1569" t="n"/>
+      <c r="R48" s="1569" t="n"/>
+      <c r="S48" s="1569" t="n"/>
       <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U48" s="1526" t="n"/>
+      <c r="U48" s="1568" t="n"/>
       <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
@@ -7852,51 +7978,51 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1501" t="inlineStr">
+      <c r="A49" s="1543" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B49" s="1502" t="inlineStr">
+      <c r="B49" s="1544" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C49" s="1502" t="inlineStr">
+      <c r="C49" s="1544" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D49" s="1503" t="n"/>
-      <c r="E49" s="1503" t="n">
+      <c r="D49" s="1545" t="n"/>
+      <c r="E49" s="1545" t="n">
         <v>16.8</v>
       </c>
-      <c r="F49" s="1503" t="n">
+      <c r="F49" s="1545" t="n">
         <v>0.2</v>
       </c>
-      <c r="G49" s="1503" t="n">
+      <c r="G49" s="1545" t="n">
         <v>3.3</v>
       </c>
-      <c r="H49" s="1503" t="n"/>
-      <c r="I49" s="1504" t="n">
+      <c r="H49" s="1545" t="n"/>
+      <c r="I49" s="1546" t="n">
         <v>1.7</v>
       </c>
-      <c r="J49" s="1505" t="n"/>
-      <c r="K49" s="1505" t="n"/>
-      <c r="L49" s="1505" t="n"/>
-      <c r="M49" s="1503" t="n"/>
-      <c r="N49" s="1503" t="n"/>
-      <c r="O49" s="1503" t="n">
+      <c r="J49" s="1547" t="n"/>
+      <c r="K49" s="1547" t="n"/>
+      <c r="L49" s="1547" t="n"/>
+      <c r="M49" s="1545" t="n"/>
+      <c r="N49" s="1545" t="n"/>
+      <c r="O49" s="1545" t="n">
         <v>13</v>
       </c>
-      <c r="P49" s="1506" t="n">
+      <c r="P49" s="1548" t="n">
         <v>0.87</v>
       </c>
-      <c r="Q49" s="1503" t="n"/>
-      <c r="R49" s="1503" t="n">
+      <c r="Q49" s="1545" t="n"/>
+      <c r="R49" s="1545" t="n">
         <v>86</v>
       </c>
-      <c r="S49" s="1503" t="n">
+      <c r="S49" s="1545" t="n">
         <v>11.65</v>
       </c>
       <c r="T49" s="624" t="inlineStr">
@@ -7904,7 +8030,7 @@
           <t>Clear now, 88F, 67% RH; sun so far 6.4h of 7h daylight (91%); today high 90F, 0.87in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U49" s="1502" t="inlineStr">
+      <c r="U49" s="1544" t="inlineStr">
         <is>
           <t>2026-07-04_1.jpeg;2026-07-04_2.jpeg;2026-07-04_3.jpeg;2026-07-04_4.jpeg</t>
         </is>
@@ -7916,49 +8042,49 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1507" t="inlineStr">
+      <c r="A50" s="1549" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B50" s="1508" t="inlineStr">
+      <c r="B50" s="1550" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C50" s="1508" t="inlineStr">
+      <c r="C50" s="1550" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D50" s="1509" t="n"/>
-      <c r="E50" s="1509" t="n"/>
-      <c r="F50" s="1509" t="n"/>
-      <c r="G50" s="1509" t="n"/>
-      <c r="H50" s="1509" t="n">
+      <c r="D50" s="1551" t="n"/>
+      <c r="E50" s="1551" t="n"/>
+      <c r="F50" s="1551" t="n"/>
+      <c r="G50" s="1551" t="n"/>
+      <c r="H50" s="1551" t="n">
         <v>14.6</v>
       </c>
-      <c r="I50" s="1510" t="n"/>
-      <c r="J50" s="1511" t="n"/>
-      <c r="K50" s="1511" t="n"/>
-      <c r="L50" s="1511" t="n"/>
-      <c r="M50" s="1509" t="n">
+      <c r="I50" s="1552" t="n"/>
+      <c r="J50" s="1553" t="n"/>
+      <c r="K50" s="1553" t="n"/>
+      <c r="L50" s="1553" t="n"/>
+      <c r="M50" s="1551" t="n">
         <v>0.5</v>
       </c>
-      <c r="N50" s="1509" t="n">
+      <c r="N50" s="1551" t="n">
         <v>20.5</v>
       </c>
-      <c r="O50" s="1509" t="n"/>
-      <c r="P50" s="1512" t="n"/>
-      <c r="Q50" s="1509" t="n"/>
-      <c r="R50" s="1509" t="n"/>
-      <c r="S50" s="1509" t="n"/>
+      <c r="O50" s="1551" t="n"/>
+      <c r="P50" s="1554" t="n"/>
+      <c r="Q50" s="1551" t="n"/>
+      <c r="R50" s="1551" t="n"/>
+      <c r="S50" s="1551" t="n"/>
       <c r="T50" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny day (high 90F, water 86F); storm forecast overnight</t>
         </is>
       </c>
-      <c r="U50" s="1508" t="n"/>
+      <c r="U50" s="1550" t="n"/>
       <c r="V50" s="632" t="inlineStr">
         <is>
           <t>0.5 gal added 7:40 PM. PARTY PRE-LOAD (Sun 7/5 1PM picnic): deliberately HALF the usual dose -- FC already high at 16.8, and John didn't want to overshoot into the high teens for guests. Sized on the retuned model (l24_hot_sunny now 4.0). Model projects ~14.6 next noon, BUT this is a known weather-mismatch case: model keys L24 off today's hot/sunny weather, while the actual loss window is a storm overnight (no UV) + cooler/cloudy Sun morning -&gt; real loss will be LOWER, so FC likely lands ~15-16 at the party (comfortable top-of-band, cushion for bather load, not overboard). =&gt; If tomorrow's noon comes in ABOVE 14.6, that's the weather mismatch, NOT the freshly-retuned constant; don't chase it. Plan: dose back up Sun evening after the crowd's out (expect a bather-load FC drop). Season total 20.5 gal. PHOTOS(4): water clear/healthy blue, bottom fully visible, no cloudiness/algae; yesterday's surface debris now gone (tracks with CC clearing to 0.2); liner step close-up normal speckled blue, no rust/stain progression. Ruler photo documents the ~11.65 cm level.</t>
@@ -7966,47 +8092,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1513" t="inlineStr">
+      <c r="A51" s="1555" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B51" s="1514" t="inlineStr">
+      <c r="B51" s="1556" t="inlineStr">
         <is>
           <t>07:45</t>
         </is>
       </c>
-      <c r="C51" s="1514" t="inlineStr">
+      <c r="C51" s="1556" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D51" s="1515" t="n"/>
-      <c r="E51" s="1515" t="n">
+      <c r="D51" s="1557" t="n"/>
+      <c r="E51" s="1557" t="n">
         <v>16</v>
       </c>
-      <c r="F51" s="1515" t="n">
+      <c r="F51" s="1557" t="n">
         <v>0.5</v>
       </c>
-      <c r="G51" s="1515" t="n"/>
-      <c r="H51" s="1515" t="n"/>
-      <c r="I51" s="1516" t="n">
+      <c r="G51" s="1557" t="n"/>
+      <c r="H51" s="1557" t="n"/>
+      <c r="I51" s="1558" t="n">
         <v>1.4</v>
       </c>
-      <c r="J51" s="1517" t="n"/>
-      <c r="K51" s="1517" t="n"/>
-      <c r="L51" s="1517" t="n"/>
-      <c r="M51" s="1515" t="n"/>
-      <c r="N51" s="1515" t="n"/>
-      <c r="O51" s="1515" t="n"/>
-      <c r="P51" s="1518" t="n">
+      <c r="J51" s="1559" t="n"/>
+      <c r="K51" s="1559" t="n"/>
+      <c r="L51" s="1559" t="n"/>
+      <c r="M51" s="1557" t="n"/>
+      <c r="N51" s="1557" t="n"/>
+      <c r="O51" s="1557" t="n"/>
+      <c r="P51" s="1560" t="n">
         <v>0.04</v>
       </c>
-      <c r="Q51" s="1515" t="n"/>
-      <c r="R51" s="1515" t="n">
+      <c r="Q51" s="1557" t="n"/>
+      <c r="R51" s="1557" t="n">
         <v>84</v>
       </c>
-      <c r="S51" s="1515" t="n">
+      <c r="S51" s="1557" t="n">
         <v>13.9</v>
       </c>
       <c r="T51" s="813" t="inlineStr">
@@ -8014,7 +8140,7 @@
           <t>Overcast now, 75F, 90% RH; sun so far 0.0h of 3h daylight (0%); today high 75F, 0.04in precip, UV max 6.5</t>
         </is>
       </c>
-      <c r="U51" s="1514" t="inlineStr">
+      <c r="U51" s="1556" t="inlineStr">
         <is>
           <t>2026-07-05_2.jpeg</t>
         </is>
@@ -8026,41 +8152,41 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1519" t="inlineStr">
+      <c r="A52" s="1561" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B52" s="1520" t="inlineStr">
+      <c r="B52" s="1562" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C52" s="1520" t="inlineStr">
+      <c r="C52" s="1562" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D52" s="1521" t="n"/>
-      <c r="E52" s="1521" t="n">
+      <c r="D52" s="1563" t="n"/>
+      <c r="E52" s="1563" t="n">
         <v>14.8</v>
       </c>
-      <c r="F52" s="1521" t="n">
+      <c r="F52" s="1563" t="n">
         <v>0.3</v>
       </c>
-      <c r="G52" s="1521" t="n"/>
-      <c r="H52" s="1521" t="n"/>
-      <c r="I52" s="1522" t="n"/>
-      <c r="J52" s="1523" t="n"/>
-      <c r="K52" s="1523" t="n"/>
-      <c r="L52" s="1523" t="n"/>
-      <c r="M52" s="1521" t="n"/>
-      <c r="N52" s="1521" t="n"/>
-      <c r="O52" s="1521" t="n"/>
-      <c r="P52" s="1524" t="n"/>
-      <c r="Q52" s="1521" t="n"/>
-      <c r="R52" s="1521" t="n"/>
-      <c r="S52" s="1521" t="n">
+      <c r="G52" s="1563" t="n"/>
+      <c r="H52" s="1563" t="n"/>
+      <c r="I52" s="1564" t="n"/>
+      <c r="J52" s="1565" t="n"/>
+      <c r="K52" s="1565" t="n"/>
+      <c r="L52" s="1565" t="n"/>
+      <c r="M52" s="1563" t="n"/>
+      <c r="N52" s="1563" t="n"/>
+      <c r="O52" s="1563" t="n"/>
+      <c r="P52" s="1566" t="n"/>
+      <c r="Q52" s="1563" t="n"/>
+      <c r="R52" s="1563" t="n"/>
+      <c r="S52" s="1563" t="n">
         <v>13.6</v>
       </c>
       <c r="T52" s="820" t="inlineStr">
@@ -8068,7 +8194,7 @@
           <t>Overcast now, 72F, 76% RH; sun so far 8.4h of 13h daylight (65%); today high 80F, 0.00in precip, UV max 6.0</t>
         </is>
       </c>
-      <c r="U52" s="1520" t="inlineStr">
+      <c r="U52" s="1562" t="inlineStr">
         <is>
           <t>2026-07-05_1.jpeg;2026-07-05_3.jpeg</t>
         </is>
@@ -8080,49 +8206,49 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1525" t="inlineStr">
+      <c r="A53" s="1567" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B53" s="1526" t="inlineStr">
+      <c r="B53" s="1568" t="inlineStr">
         <is>
           <t>19:25</t>
         </is>
       </c>
-      <c r="C53" s="1526" t="inlineStr">
+      <c r="C53" s="1568" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D53" s="1527" t="n"/>
-      <c r="E53" s="1527" t="n"/>
-      <c r="F53" s="1527" t="n"/>
-      <c r="G53" s="1527" t="n"/>
-      <c r="H53" s="1527" t="n">
+      <c r="D53" s="1569" t="n"/>
+      <c r="E53" s="1569" t="n"/>
+      <c r="F53" s="1569" t="n"/>
+      <c r="G53" s="1569" t="n"/>
+      <c r="H53" s="1569" t="n">
         <v>15.1</v>
       </c>
-      <c r="I53" s="1528" t="n"/>
-      <c r="J53" s="1529" t="n"/>
-      <c r="K53" s="1529" t="n"/>
-      <c r="L53" s="1529" t="n"/>
-      <c r="M53" s="1527" t="n">
+      <c r="I53" s="1570" t="n"/>
+      <c r="J53" s="1571" t="n"/>
+      <c r="K53" s="1571" t="n"/>
+      <c r="L53" s="1571" t="n"/>
+      <c r="M53" s="1569" t="n">
         <v>0.5</v>
       </c>
-      <c r="N53" s="1527" t="n">
+      <c r="N53" s="1569" t="n">
         <v>21</v>
       </c>
-      <c r="O53" s="1527" t="n"/>
-      <c r="P53" s="1530" t="n"/>
-      <c r="Q53" s="1527" t="n"/>
-      <c r="R53" s="1527" t="n"/>
-      <c r="S53" s="1527" t="n"/>
+      <c r="O53" s="1569" t="n"/>
+      <c r="P53" s="1572" t="n"/>
+      <c r="Q53" s="1569" t="n"/>
+      <c r="R53" s="1569" t="n"/>
+      <c r="S53" s="1569" t="n"/>
       <c r="T53" s="827" t="inlineStr">
         <is>
           <t>Cleared to partly sunny (8.4 sun hrs, high 80F, water 84F); all-day rain forecast Mon 7/6</t>
         </is>
       </c>
-      <c r="U53" s="1526" t="n"/>
+      <c r="U53" s="1568" t="n"/>
       <c r="V53" s="828" t="inlineStr">
         <is>
           <t>0.5 gal added 7:25 PM (post-party recovery dose). Sized on TOMORROW's rainy forecast (the real loss window: overcast/wet 7/6, ~0.9in rain, low UV) not today's sun -&gt; projects ~15.1 at Mon noon. Party went great (FC held 16.0-&gt;14.8, CC dropped 0.5-&gt;0.3). Season total 21.0 gal. This is the first prediction that deliberately used the next-day forecast for L24 instead of the model's default (today's weather as proxy) -- if it lands near 15.1 tomorrow, that validates feeding the forecast on weather-change days.</t>
@@ -8130,49 +8256,49 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1537" t="inlineStr">
+      <c r="A54" s="1579" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B54" s="1538" t="inlineStr">
+      <c r="B54" s="1580" t="inlineStr">
         <is>
           <t>11:40</t>
         </is>
       </c>
-      <c r="C54" s="1538" t="inlineStr">
+      <c r="C54" s="1580" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D54" s="1539" t="n"/>
-      <c r="E54" s="1539" t="n">
+      <c r="D54" s="1581" t="n"/>
+      <c r="E54" s="1581" t="n">
         <v>13.8</v>
       </c>
-      <c r="F54" s="1539" t="n">
+      <c r="F54" s="1581" t="n">
         <v>0.2</v>
       </c>
-      <c r="G54" s="1539" t="n"/>
-      <c r="H54" s="1539" t="n"/>
-      <c r="I54" s="1540" t="n">
+      <c r="G54" s="1581" t="n"/>
+      <c r="H54" s="1581" t="n"/>
+      <c r="I54" s="1582" t="n">
         <v>-1.3</v>
       </c>
-      <c r="J54" s="1541" t="n"/>
-      <c r="K54" s="1541" t="n"/>
-      <c r="L54" s="1541" t="n"/>
-      <c r="M54" s="1539" t="n"/>
-      <c r="N54" s="1539" t="n"/>
-      <c r="O54" s="1539" t="n">
+      <c r="J54" s="1583" t="n"/>
+      <c r="K54" s="1583" t="n"/>
+      <c r="L54" s="1583" t="n"/>
+      <c r="M54" s="1581" t="n"/>
+      <c r="N54" s="1581" t="n"/>
+      <c r="O54" s="1581" t="n">
         <v>0</v>
       </c>
-      <c r="P54" s="1542" t="n">
+      <c r="P54" s="1584" t="n">
         <v>2</v>
       </c>
-      <c r="Q54" s="1539" t="n"/>
-      <c r="R54" s="1539" t="n">
+      <c r="Q54" s="1581" t="n"/>
+      <c r="R54" s="1581" t="n">
         <v>81</v>
       </c>
-      <c r="S54" s="1539" t="n">
+      <c r="S54" s="1581" t="n">
         <v>15.1</v>
       </c>
       <c r="T54" s="1047" t="inlineStr">
@@ -8180,14 +8306,14 @@
           <t>Light rain now, 65F, 93% RH; sun so far 0.0h of 6h daylight (0%); today high 68F, 2.00in precip, UV max 0.5</t>
         </is>
       </c>
-      <c r="U54" s="1538" t="inlineStr">
+      <c r="U54" s="1580" t="inlineStr">
         <is>
           <t>2026-07-06_1.jpeg</t>
         </is>
       </c>
       <c r="V54" s="1048" t="inlineStr">
         <is>
-          <t>25mL x0.2. FC 13.8, CC 0.2 -- in band, all healthy. FIRST NEGATIVE prediction error (-1.3): actual 13.8 vs the 7/5 dose's 15.1 (which used the rain bucket L24=1.5). i.e. the model UNDER-estimated loss on this heavy-rain day. WHY: 2.0in of rain fell but the level only rose 0.6in (13.6-&gt;15.1 cm) -&gt; the pool is OVERFLOWING, carrying FC (and CYA) over the edge, plus rain dilution -- neither of which the UV-only rain bucket models. So heavy-rain/overflow days lose MORE than the rain bucket predicts. This is the FIRST forward rainy-day point AND it's confounded by overflow -&gt; do NOT retune the rain bucket off it (it may still be fine for light/no-overflow drizzle); just note heavy-rain != low-loss. SILVER LINING: the overflow + dilution is passively lowering CYA (currently ~150) -- exactly what we want -&gt; good trigger for a CYA recheck once it clears. fc_loss left BLANK: overflow+dilution make today's drop not a clean chemical-loss measurement. Level 15.1 (near the top, overflowing). Water temp 81 (cooling). DOSE REC TONIGHT: HOLD (no dose) -- dosing into an overflowing pool just sends chlorine over the edge, FC 13.8 is comfortably in-band, nobody's swimming in the rain, and John's low on chlorine (refill 1-2 days out). Let it ride; dose Wed when the rain clears and the refill's here. If FC dips toward floor 11 faster than expected, reassess.</t>
+          <t>25mL x0.2. FC 13.8, CC 0.2 -- in band, healthy. [CORRECTED same day: earlier note wrongly said OVERFLOWING -- it is NOT. Pool has 6+ in of freeboard. The weather feed 2.00in is the DAY forecast total, not fallen-yet; only ~0.6in has actually fallen this AM, which matches the 0.6in / 1.5cm level rise 13.6-&gt;15.1. No water over the edge.] FIRST NEGATIVE prediction error (-1.3): actual 13.8 vs the 7/5 dose 15.1 (rain bucket L24=1.5) -&gt; model UNDER-estimated loss. Likely cause: STORM since last night (not calm rain) washes organic load in (debris/runoff/nitrogen) that consumes FC -- real loss ~2.75 from the post-dose ~16.5 vs the calm-rain 1.5 estimate. Dilution only a minor part (~0.15 ppm from 0.6in add). The rain bucket is tuned for drizzle, not a storm; FIRST storm forward point -&gt; note storms lose more, but do NOT retune off one point. CYA: modest rain dilution (~0.9%) nudges it down ~1-2 ppm (NOT the big overflow-driven drop I wrongly claimed). fc_loss BLANK: off-cadence prior test (7/5 had AM+PM) + dilution -&gt; not a clean noon-to-noon value. Level 15.1 (well below overflow). Water temp 81. DOSE REC revised: a modest 0.5 gal tonight is reasonable -- the storm is actively eating FC and there is no overflow to waste it, so hold the buffer above floor; keep it small (John low on chlorine, refill 1-2 days out).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log 2026-07-06 pump-to-waste event + evening dose (1 gal, season 22.0)
Rain pushed the level above the ruler; pumped to waste back to 15.1 cm
(~2000 gal removed, rough estimate from photos). Dosed 1 gal after
emptying -- full gallon since the "low on chlorine" was actually low on
test reagents (arrived today), now corrected in the log. Adds 2 water-
level photos.
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1585">
+  <cellXfs count="1621">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -5282,6 +5282,114 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5543,7 +5651,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V54"/>
+  <dimension ref="A1:V56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -5720,35 +5828,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1543" t="inlineStr">
+      <c r="A3" s="1585" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1544" t="n"/>
-      <c r="C3" s="1544" t="inlineStr">
+      <c r="B3" s="1586" t="n"/>
+      <c r="C3" s="1586" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1545" t="n"/>
-      <c r="E3" s="1545" t="n"/>
-      <c r="F3" s="1545" t="n"/>
-      <c r="G3" s="1545" t="n"/>
-      <c r="H3" s="1545" t="n"/>
-      <c r="I3" s="1546" t="n"/>
-      <c r="J3" s="1547" t="n"/>
-      <c r="K3" s="1547" t="n"/>
-      <c r="L3" s="1547" t="n"/>
-      <c r="M3" s="1545" t="n"/>
-      <c r="N3" s="1545" t="n"/>
-      <c r="O3" s="1545" t="n"/>
-      <c r="P3" s="1548" t="n"/>
-      <c r="Q3" s="1545" t="n"/>
-      <c r="R3" s="1545" t="n"/>
-      <c r="S3" s="1545" t="n"/>
+      <c r="D3" s="1587" t="n"/>
+      <c r="E3" s="1587" t="n"/>
+      <c r="F3" s="1587" t="n"/>
+      <c r="G3" s="1587" t="n"/>
+      <c r="H3" s="1587" t="n"/>
+      <c r="I3" s="1588" t="n"/>
+      <c r="J3" s="1589" t="n"/>
+      <c r="K3" s="1589" t="n"/>
+      <c r="L3" s="1589" t="n"/>
+      <c r="M3" s="1587" t="n"/>
+      <c r="N3" s="1587" t="n"/>
+      <c r="O3" s="1587" t="n"/>
+      <c r="P3" s="1590" t="n"/>
+      <c r="Q3" s="1587" t="n"/>
+      <c r="R3" s="1587" t="n"/>
+      <c r="S3" s="1587" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1544" t="n"/>
+      <c r="U3" s="1586" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -5756,43 +5864,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1549" t="inlineStr">
+      <c r="A4" s="1591" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1550" t="inlineStr">
+      <c r="B4" s="1592" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1550" t="inlineStr">
+      <c r="C4" s="1592" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1551" t="n"/>
-      <c r="E4" s="1551" t="n"/>
-      <c r="F4" s="1551" t="n"/>
-      <c r="G4" s="1551" t="n"/>
-      <c r="H4" s="1551" t="n"/>
-      <c r="I4" s="1552" t="n"/>
-      <c r="J4" s="1553" t="n"/>
-      <c r="K4" s="1553" t="n"/>
-      <c r="L4" s="1553" t="n"/>
-      <c r="M4" s="1551" t="n">
+      <c r="D4" s="1593" t="n"/>
+      <c r="E4" s="1593" t="n"/>
+      <c r="F4" s="1593" t="n"/>
+      <c r="G4" s="1593" t="n"/>
+      <c r="H4" s="1593" t="n"/>
+      <c r="I4" s="1594" t="n"/>
+      <c r="J4" s="1595" t="n"/>
+      <c r="K4" s="1595" t="n"/>
+      <c r="L4" s="1595" t="n"/>
+      <c r="M4" s="1593" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1551" t="n">
+      <c r="N4" s="1593" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1551" t="n"/>
-      <c r="P4" s="1554" t="n"/>
-      <c r="Q4" s="1551" t="n"/>
-      <c r="R4" s="1551" t="n"/>
-      <c r="S4" s="1551" t="n"/>
+      <c r="O4" s="1593" t="n"/>
+      <c r="P4" s="1596" t="n"/>
+      <c r="Q4" s="1593" t="n"/>
+      <c r="R4" s="1593" t="n"/>
+      <c r="S4" s="1593" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1550" t="n"/>
+      <c r="U4" s="1592" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -5800,57 +5908,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1555" t="inlineStr">
+      <c r="A5" s="1597" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1556" t="inlineStr">
+      <c r="B5" s="1598" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1556" t="inlineStr">
+      <c r="C5" s="1598" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1557" t="n">
+      <c r="D5" s="1599" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1557" t="n">
+      <c r="E5" s="1599" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1557" t="n">
+      <c r="F5" s="1599" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1557" t="n"/>
-      <c r="H5" s="1557" t="n"/>
-      <c r="I5" s="1558" t="n"/>
-      <c r="J5" s="1559" t="n">
+      <c r="G5" s="1599" t="n"/>
+      <c r="H5" s="1599" t="n"/>
+      <c r="I5" s="1600" t="n"/>
+      <c r="J5" s="1601" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1559" t="n">
+      <c r="K5" s="1601" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1559" t="inlineStr">
+      <c r="L5" s="1601" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1557" t="n"/>
-      <c r="N5" s="1557" t="n"/>
-      <c r="O5" s="1557" t="n">
+      <c r="M5" s="1599" t="n"/>
+      <c r="N5" s="1599" t="n"/>
+      <c r="O5" s="1599" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1560" t="n">
+      <c r="P5" s="1602" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1557" t="n"/>
-      <c r="R5" s="1557" t="n"/>
-      <c r="S5" s="1557" t="n"/>
+      <c r="Q5" s="1599" t="n"/>
+      <c r="R5" s="1599" t="n"/>
+      <c r="S5" s="1599" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1556" t="n"/>
+      <c r="U5" s="1598" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -5858,43 +5966,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1561" t="inlineStr">
+      <c r="A6" s="1603" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1562" t="inlineStr">
+      <c r="B6" s="1604" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1562" t="inlineStr">
+      <c r="C6" s="1604" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1563" t="n"/>
-      <c r="E6" s="1563" t="n"/>
-      <c r="F6" s="1563" t="n"/>
-      <c r="G6" s="1563" t="n"/>
-      <c r="H6" s="1563" t="n"/>
-      <c r="I6" s="1564" t="n"/>
-      <c r="J6" s="1565" t="n"/>
-      <c r="K6" s="1565" t="n"/>
-      <c r="L6" s="1565" t="n"/>
-      <c r="M6" s="1563" t="n">
+      <c r="D6" s="1605" t="n"/>
+      <c r="E6" s="1605" t="n"/>
+      <c r="F6" s="1605" t="n"/>
+      <c r="G6" s="1605" t="n"/>
+      <c r="H6" s="1605" t="n"/>
+      <c r="I6" s="1606" t="n"/>
+      <c r="J6" s="1607" t="n"/>
+      <c r="K6" s="1607" t="n"/>
+      <c r="L6" s="1607" t="n"/>
+      <c r="M6" s="1605" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1563" t="n">
+      <c r="N6" s="1605" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1563" t="n"/>
-      <c r="P6" s="1566" t="n"/>
-      <c r="Q6" s="1563" t="n"/>
-      <c r="R6" s="1563" t="n"/>
-      <c r="S6" s="1563" t="n"/>
+      <c r="O6" s="1605" t="n"/>
+      <c r="P6" s="1608" t="n"/>
+      <c r="Q6" s="1605" t="n"/>
+      <c r="R6" s="1605" t="n"/>
+      <c r="S6" s="1605" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1562" t="n"/>
+      <c r="U6" s="1604" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -5902,39 +6010,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1567" t="inlineStr">
+      <c r="A7" s="1609" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1568" t="inlineStr">
+      <c r="B7" s="1610" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1568" t="inlineStr">
+      <c r="C7" s="1610" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1569" t="n"/>
-      <c r="E7" s="1569" t="n"/>
-      <c r="F7" s="1569" t="n"/>
-      <c r="G7" s="1569" t="n"/>
-      <c r="H7" s="1569" t="n"/>
-      <c r="I7" s="1570" t="n"/>
-      <c r="J7" s="1571" t="n"/>
-      <c r="K7" s="1571" t="n"/>
-      <c r="L7" s="1571" t="n"/>
-      <c r="M7" s="1569" t="n"/>
-      <c r="N7" s="1569" t="n"/>
-      <c r="O7" s="1569" t="n"/>
-      <c r="P7" s="1572" t="n"/>
-      <c r="Q7" s="1569" t="n"/>
-      <c r="R7" s="1569" t="n"/>
-      <c r="S7" s="1569" t="n"/>
+      <c r="D7" s="1611" t="n"/>
+      <c r="E7" s="1611" t="n"/>
+      <c r="F7" s="1611" t="n"/>
+      <c r="G7" s="1611" t="n"/>
+      <c r="H7" s="1611" t="n"/>
+      <c r="I7" s="1612" t="n"/>
+      <c r="J7" s="1613" t="n"/>
+      <c r="K7" s="1613" t="n"/>
+      <c r="L7" s="1613" t="n"/>
+      <c r="M7" s="1611" t="n"/>
+      <c r="N7" s="1611" t="n"/>
+      <c r="O7" s="1611" t="n"/>
+      <c r="P7" s="1614" t="n"/>
+      <c r="Q7" s="1611" t="n"/>
+      <c r="R7" s="1611" t="n"/>
+      <c r="S7" s="1611" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1568" t="n"/>
+      <c r="U7" s="1610" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -5942,39 +6050,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1543" t="inlineStr">
+      <c r="A8" s="1585" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1544" t="inlineStr">
+      <c r="B8" s="1586" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1544" t="inlineStr">
+      <c r="C8" s="1586" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1545" t="n"/>
-      <c r="E8" s="1545" t="n"/>
-      <c r="F8" s="1545" t="n"/>
-      <c r="G8" s="1545" t="n"/>
-      <c r="H8" s="1545" t="n"/>
-      <c r="I8" s="1546" t="n"/>
-      <c r="J8" s="1547" t="n"/>
-      <c r="K8" s="1547" t="n"/>
-      <c r="L8" s="1547" t="n"/>
-      <c r="M8" s="1545" t="n"/>
-      <c r="N8" s="1545" t="n"/>
-      <c r="O8" s="1545" t="n"/>
-      <c r="P8" s="1548" t="n"/>
-      <c r="Q8" s="1545" t="n"/>
-      <c r="R8" s="1545" t="n"/>
-      <c r="S8" s="1545" t="n"/>
+      <c r="D8" s="1587" t="n"/>
+      <c r="E8" s="1587" t="n"/>
+      <c r="F8" s="1587" t="n"/>
+      <c r="G8" s="1587" t="n"/>
+      <c r="H8" s="1587" t="n"/>
+      <c r="I8" s="1588" t="n"/>
+      <c r="J8" s="1589" t="n"/>
+      <c r="K8" s="1589" t="n"/>
+      <c r="L8" s="1589" t="n"/>
+      <c r="M8" s="1587" t="n"/>
+      <c r="N8" s="1587" t="n"/>
+      <c r="O8" s="1587" t="n"/>
+      <c r="P8" s="1590" t="n"/>
+      <c r="Q8" s="1587" t="n"/>
+      <c r="R8" s="1587" t="n"/>
+      <c r="S8" s="1587" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1544" t="n"/>
+      <c r="U8" s="1586" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -5982,63 +6090,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1573" t="inlineStr">
+      <c r="A9" s="1615" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1574" t="inlineStr">
+      <c r="B9" s="1616" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1574" t="inlineStr">
+      <c r="C9" s="1616" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1575" t="n">
+      <c r="D9" s="1617" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1575" t="n">
+      <c r="E9" s="1617" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1575" t="n">
+      <c r="F9" s="1617" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1575" t="n">
+      <c r="G9" s="1617" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1575" t="n"/>
-      <c r="I9" s="1576" t="n"/>
-      <c r="J9" s="1577" t="n">
+      <c r="H9" s="1617" t="n"/>
+      <c r="I9" s="1618" t="n"/>
+      <c r="J9" s="1619" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1577" t="n">
+      <c r="K9" s="1619" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1577" t="inlineStr">
+      <c r="L9" s="1619" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1575" t="n"/>
-      <c r="N9" s="1575" t="n"/>
-      <c r="O9" s="1575" t="n">
+      <c r="M9" s="1617" t="n"/>
+      <c r="N9" s="1617" t="n"/>
+      <c r="O9" s="1617" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1578" t="n">
+      <c r="P9" s="1620" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1575" t="n"/>
-      <c r="R9" s="1575" t="n"/>
-      <c r="S9" s="1575" t="n"/>
+      <c r="Q9" s="1617" t="n"/>
+      <c r="R9" s="1617" t="n"/>
+      <c r="S9" s="1617" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1574" t="n"/>
+      <c r="U9" s="1616" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -6046,43 +6154,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1573" t="inlineStr">
+      <c r="A10" s="1615" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1574" t="inlineStr">
+      <c r="B10" s="1616" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1574" t="inlineStr">
+      <c r="C10" s="1616" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1575" t="n"/>
-      <c r="E10" s="1575" t="n"/>
-      <c r="F10" s="1575" t="n"/>
-      <c r="G10" s="1575" t="n"/>
-      <c r="H10" s="1575" t="n"/>
-      <c r="I10" s="1576" t="n"/>
-      <c r="J10" s="1577" t="n"/>
-      <c r="K10" s="1577" t="n"/>
-      <c r="L10" s="1577" t="inlineStr">
+      <c r="D10" s="1617" t="n"/>
+      <c r="E10" s="1617" t="n"/>
+      <c r="F10" s="1617" t="n"/>
+      <c r="G10" s="1617" t="n"/>
+      <c r="H10" s="1617" t="n"/>
+      <c r="I10" s="1618" t="n"/>
+      <c r="J10" s="1619" t="n"/>
+      <c r="K10" s="1619" t="n"/>
+      <c r="L10" s="1619" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1575" t="n"/>
-      <c r="N10" s="1575" t="n"/>
-      <c r="O10" s="1575" t="n"/>
-      <c r="P10" s="1578" t="n"/>
-      <c r="Q10" s="1575" t="n"/>
-      <c r="R10" s="1575" t="n"/>
-      <c r="S10" s="1575" t="n"/>
+      <c r="M10" s="1617" t="n"/>
+      <c r="N10" s="1617" t="n"/>
+      <c r="O10" s="1617" t="n"/>
+      <c r="P10" s="1620" t="n"/>
+      <c r="Q10" s="1617" t="n"/>
+      <c r="R10" s="1617" t="n"/>
+      <c r="S10" s="1617" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1574" t="n"/>
+      <c r="U10" s="1616" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -6090,43 +6198,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1573" t="inlineStr">
+      <c r="A11" s="1615" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1574" t="inlineStr">
+      <c r="B11" s="1616" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1574" t="inlineStr">
+      <c r="C11" s="1616" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1575" t="n"/>
-      <c r="E11" s="1575" t="n"/>
-      <c r="F11" s="1575" t="n"/>
-      <c r="G11" s="1575" t="n"/>
-      <c r="H11" s="1575" t="n"/>
-      <c r="I11" s="1576" t="n"/>
-      <c r="J11" s="1577" t="n"/>
-      <c r="K11" s="1577" t="n"/>
-      <c r="L11" s="1577" t="n"/>
-      <c r="M11" s="1575" t="n">
+      <c r="D11" s="1617" t="n"/>
+      <c r="E11" s="1617" t="n"/>
+      <c r="F11" s="1617" t="n"/>
+      <c r="G11" s="1617" t="n"/>
+      <c r="H11" s="1617" t="n"/>
+      <c r="I11" s="1618" t="n"/>
+      <c r="J11" s="1619" t="n"/>
+      <c r="K11" s="1619" t="n"/>
+      <c r="L11" s="1619" t="n"/>
+      <c r="M11" s="1617" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1575" t="n">
+      <c r="N11" s="1617" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1575" t="n"/>
-      <c r="P11" s="1578" t="n"/>
-      <c r="Q11" s="1575" t="n"/>
-      <c r="R11" s="1575" t="n"/>
-      <c r="S11" s="1575" t="n"/>
+      <c r="O11" s="1617" t="n"/>
+      <c r="P11" s="1620" t="n"/>
+      <c r="Q11" s="1617" t="n"/>
+      <c r="R11" s="1617" t="n"/>
+      <c r="S11" s="1617" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1574" t="n"/>
+      <c r="U11" s="1616" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -6134,39 +6242,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1549" t="inlineStr">
+      <c r="A12" s="1591" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1550" t="inlineStr">
+      <c r="B12" s="1592" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1550" t="inlineStr">
+      <c r="C12" s="1592" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1551" t="n"/>
-      <c r="E12" s="1551" t="n"/>
-      <c r="F12" s="1551" t="n"/>
-      <c r="G12" s="1551" t="n"/>
-      <c r="H12" s="1551" t="n"/>
-      <c r="I12" s="1552" t="n"/>
-      <c r="J12" s="1553" t="n"/>
-      <c r="K12" s="1553" t="n"/>
-      <c r="L12" s="1553" t="n"/>
-      <c r="M12" s="1551" t="n"/>
-      <c r="N12" s="1551" t="n"/>
-      <c r="O12" s="1551" t="n"/>
-      <c r="P12" s="1554" t="n"/>
-      <c r="Q12" s="1551" t="n"/>
-      <c r="R12" s="1551" t="n"/>
-      <c r="S12" s="1551" t="n"/>
+      <c r="D12" s="1593" t="n"/>
+      <c r="E12" s="1593" t="n"/>
+      <c r="F12" s="1593" t="n"/>
+      <c r="G12" s="1593" t="n"/>
+      <c r="H12" s="1593" t="n"/>
+      <c r="I12" s="1594" t="n"/>
+      <c r="J12" s="1595" t="n"/>
+      <c r="K12" s="1595" t="n"/>
+      <c r="L12" s="1595" t="n"/>
+      <c r="M12" s="1593" t="n"/>
+      <c r="N12" s="1593" t="n"/>
+      <c r="O12" s="1593" t="n"/>
+      <c r="P12" s="1596" t="n"/>
+      <c r="Q12" s="1593" t="n"/>
+      <c r="R12" s="1593" t="n"/>
+      <c r="S12" s="1593" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1550" t="n"/>
+      <c r="U12" s="1592" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -6174,35 +6282,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1555" t="inlineStr">
+      <c r="A13" s="1597" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1556" t="n"/>
-      <c r="C13" s="1556" t="inlineStr">
+      <c r="B13" s="1598" t="n"/>
+      <c r="C13" s="1598" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1557" t="n"/>
-      <c r="E13" s="1557" t="n"/>
-      <c r="F13" s="1557" t="n"/>
-      <c r="G13" s="1557" t="n"/>
-      <c r="H13" s="1557" t="n"/>
-      <c r="I13" s="1558" t="n"/>
-      <c r="J13" s="1559" t="n"/>
-      <c r="K13" s="1559" t="n"/>
-      <c r="L13" s="1559" t="n"/>
-      <c r="M13" s="1557" t="n"/>
-      <c r="N13" s="1557" t="n"/>
-      <c r="O13" s="1557" t="n"/>
-      <c r="P13" s="1560" t="n"/>
-      <c r="Q13" s="1557" t="n"/>
-      <c r="R13" s="1557" t="n"/>
-      <c r="S13" s="1557" t="n"/>
+      <c r="D13" s="1599" t="n"/>
+      <c r="E13" s="1599" t="n"/>
+      <c r="F13" s="1599" t="n"/>
+      <c r="G13" s="1599" t="n"/>
+      <c r="H13" s="1599" t="n"/>
+      <c r="I13" s="1600" t="n"/>
+      <c r="J13" s="1601" t="n"/>
+      <c r="K13" s="1601" t="n"/>
+      <c r="L13" s="1601" t="n"/>
+      <c r="M13" s="1599" t="n"/>
+      <c r="N13" s="1599" t="n"/>
+      <c r="O13" s="1599" t="n"/>
+      <c r="P13" s="1602" t="n"/>
+      <c r="Q13" s="1599" t="n"/>
+      <c r="R13" s="1599" t="n"/>
+      <c r="S13" s="1599" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1556" t="n"/>
+      <c r="U13" s="1598" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -6210,53 +6318,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1561" t="inlineStr">
+      <c r="A14" s="1603" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1562" t="inlineStr">
+      <c r="B14" s="1604" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1562" t="inlineStr">
+      <c r="C14" s="1604" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1563" t="n"/>
-      <c r="E14" s="1563" t="n">
+      <c r="D14" s="1605" t="n"/>
+      <c r="E14" s="1605" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1563" t="n">
+      <c r="F14" s="1605" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1563" t="n">
+      <c r="G14" s="1605" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1563" t="n"/>
-      <c r="I14" s="1564" t="n"/>
-      <c r="J14" s="1565" t="n"/>
-      <c r="K14" s="1565" t="n"/>
-      <c r="L14" s="1565" t="n"/>
-      <c r="M14" s="1563" t="n"/>
-      <c r="N14" s="1563" t="n"/>
-      <c r="O14" s="1563" t="n">
+      <c r="H14" s="1605" t="n"/>
+      <c r="I14" s="1606" t="n"/>
+      <c r="J14" s="1607" t="n"/>
+      <c r="K14" s="1607" t="n"/>
+      <c r="L14" s="1607" t="n"/>
+      <c r="M14" s="1605" t="n"/>
+      <c r="N14" s="1605" t="n"/>
+      <c r="O14" s="1605" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1566" t="n">
+      <c r="P14" s="1608" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1563" t="n"/>
-      <c r="R14" s="1563" t="n"/>
-      <c r="S14" s="1563" t="n"/>
+      <c r="Q14" s="1605" t="n"/>
+      <c r="R14" s="1605" t="n"/>
+      <c r="S14" s="1605" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1562" t="n"/>
+      <c r="U14" s="1604" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -6264,43 +6372,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1561" t="inlineStr">
+      <c r="A15" s="1603" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1562" t="inlineStr">
+      <c r="B15" s="1604" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1562" t="inlineStr">
+      <c r="C15" s="1604" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1563" t="n"/>
-      <c r="E15" s="1563" t="n"/>
-      <c r="F15" s="1563" t="n"/>
-      <c r="G15" s="1563" t="n"/>
-      <c r="H15" s="1563" t="n"/>
-      <c r="I15" s="1564" t="n"/>
-      <c r="J15" s="1565" t="n"/>
-      <c r="K15" s="1565" t="n"/>
-      <c r="L15" s="1565" t="n"/>
-      <c r="M15" s="1563" t="n">
+      <c r="D15" s="1605" t="n"/>
+      <c r="E15" s="1605" t="n"/>
+      <c r="F15" s="1605" t="n"/>
+      <c r="G15" s="1605" t="n"/>
+      <c r="H15" s="1605" t="n"/>
+      <c r="I15" s="1606" t="n"/>
+      <c r="J15" s="1607" t="n"/>
+      <c r="K15" s="1607" t="n"/>
+      <c r="L15" s="1607" t="n"/>
+      <c r="M15" s="1605" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1563" t="n">
+      <c r="N15" s="1605" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1563" t="n"/>
-      <c r="P15" s="1566" t="n"/>
-      <c r="Q15" s="1563" t="n"/>
-      <c r="R15" s="1563" t="n"/>
-      <c r="S15" s="1563" t="n"/>
+      <c r="O15" s="1605" t="n"/>
+      <c r="P15" s="1608" t="n"/>
+      <c r="Q15" s="1605" t="n"/>
+      <c r="R15" s="1605" t="n"/>
+      <c r="S15" s="1605" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1562" t="n"/>
+      <c r="U15" s="1604" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -6308,39 +6416,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1567" t="inlineStr">
+      <c r="A16" s="1609" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1568" t="inlineStr">
+      <c r="B16" s="1610" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1568" t="inlineStr">
+      <c r="C16" s="1610" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1569" t="n"/>
-      <c r="E16" s="1569" t="n"/>
-      <c r="F16" s="1569" t="n"/>
-      <c r="G16" s="1569" t="n"/>
-      <c r="H16" s="1569" t="n"/>
-      <c r="I16" s="1570" t="n"/>
-      <c r="J16" s="1571" t="n"/>
-      <c r="K16" s="1571" t="n"/>
-      <c r="L16" s="1571" t="n"/>
-      <c r="M16" s="1569" t="n"/>
-      <c r="N16" s="1569" t="n"/>
-      <c r="O16" s="1569" t="n"/>
-      <c r="P16" s="1572" t="n"/>
-      <c r="Q16" s="1569" t="n"/>
-      <c r="R16" s="1569" t="n"/>
-      <c r="S16" s="1569" t="n"/>
+      <c r="D16" s="1611" t="n"/>
+      <c r="E16" s="1611" t="n"/>
+      <c r="F16" s="1611" t="n"/>
+      <c r="G16" s="1611" t="n"/>
+      <c r="H16" s="1611" t="n"/>
+      <c r="I16" s="1612" t="n"/>
+      <c r="J16" s="1613" t="n"/>
+      <c r="K16" s="1613" t="n"/>
+      <c r="L16" s="1613" t="n"/>
+      <c r="M16" s="1611" t="n"/>
+      <c r="N16" s="1611" t="n"/>
+      <c r="O16" s="1611" t="n"/>
+      <c r="P16" s="1614" t="n"/>
+      <c r="Q16" s="1611" t="n"/>
+      <c r="R16" s="1611" t="n"/>
+      <c r="S16" s="1611" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1568" t="n"/>
+      <c r="U16" s="1610" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -6348,39 +6456,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1543" t="inlineStr">
+      <c r="A17" s="1585" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1544" t="inlineStr">
+      <c r="B17" s="1586" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1544" t="inlineStr">
+      <c r="C17" s="1586" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1545" t="n"/>
-      <c r="E17" s="1545" t="n"/>
-      <c r="F17" s="1545" t="n"/>
-      <c r="G17" s="1545" t="n"/>
-      <c r="H17" s="1545" t="n"/>
-      <c r="I17" s="1546" t="n"/>
-      <c r="J17" s="1547" t="n"/>
-      <c r="K17" s="1547" t="n"/>
-      <c r="L17" s="1547" t="n"/>
-      <c r="M17" s="1545" t="n"/>
-      <c r="N17" s="1545" t="n"/>
-      <c r="O17" s="1545" t="n"/>
-      <c r="P17" s="1548" t="n"/>
-      <c r="Q17" s="1545" t="n"/>
-      <c r="R17" s="1545" t="n"/>
-      <c r="S17" s="1545" t="n"/>
+      <c r="D17" s="1587" t="n"/>
+      <c r="E17" s="1587" t="n"/>
+      <c r="F17" s="1587" t="n"/>
+      <c r="G17" s="1587" t="n"/>
+      <c r="H17" s="1587" t="n"/>
+      <c r="I17" s="1588" t="n"/>
+      <c r="J17" s="1589" t="n"/>
+      <c r="K17" s="1589" t="n"/>
+      <c r="L17" s="1589" t="n"/>
+      <c r="M17" s="1587" t="n"/>
+      <c r="N17" s="1587" t="n"/>
+      <c r="O17" s="1587" t="n"/>
+      <c r="P17" s="1590" t="n"/>
+      <c r="Q17" s="1587" t="n"/>
+      <c r="R17" s="1587" t="n"/>
+      <c r="S17" s="1587" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1544" t="n"/>
+      <c r="U17" s="1586" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -6388,53 +6496,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1573" t="inlineStr">
+      <c r="A18" s="1615" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1574" t="inlineStr">
+      <c r="B18" s="1616" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1574" t="inlineStr">
+      <c r="C18" s="1616" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1575" t="n"/>
-      <c r="E18" s="1575" t="n">
+      <c r="D18" s="1617" t="n"/>
+      <c r="E18" s="1617" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1575" t="n">
+      <c r="F18" s="1617" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1575" t="n">
+      <c r="G18" s="1617" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1575" t="n"/>
-      <c r="I18" s="1576" t="n"/>
-      <c r="J18" s="1577" t="n"/>
-      <c r="K18" s="1577" t="n"/>
-      <c r="L18" s="1577" t="n"/>
-      <c r="M18" s="1575" t="n"/>
-      <c r="N18" s="1575" t="n"/>
-      <c r="O18" s="1575" t="n">
+      <c r="H18" s="1617" t="n"/>
+      <c r="I18" s="1618" t="n"/>
+      <c r="J18" s="1619" t="n"/>
+      <c r="K18" s="1619" t="n"/>
+      <c r="L18" s="1619" t="n"/>
+      <c r="M18" s="1617" t="n"/>
+      <c r="N18" s="1617" t="n"/>
+      <c r="O18" s="1617" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1578" t="n">
+      <c r="P18" s="1620" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1575" t="n"/>
-      <c r="R18" s="1575" t="n"/>
-      <c r="S18" s="1575" t="n"/>
+      <c r="Q18" s="1617" t="n"/>
+      <c r="R18" s="1617" t="n"/>
+      <c r="S18" s="1617" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1574" t="n"/>
+      <c r="U18" s="1616" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -6442,47 +6550,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1573" t="inlineStr">
+      <c r="A19" s="1615" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1574" t="inlineStr">
+      <c r="B19" s="1616" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1574" t="inlineStr">
+      <c r="C19" s="1616" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1575" t="n"/>
-      <c r="E19" s="1575" t="n"/>
-      <c r="F19" s="1575" t="n"/>
-      <c r="G19" s="1575" t="n"/>
-      <c r="H19" s="1575" t="n"/>
-      <c r="I19" s="1576" t="n"/>
-      <c r="J19" s="1577" t="n"/>
-      <c r="K19" s="1577" t="n"/>
-      <c r="L19" s="1577" t="n"/>
-      <c r="M19" s="1575" t="n">
+      <c r="D19" s="1617" t="n"/>
+      <c r="E19" s="1617" t="n"/>
+      <c r="F19" s="1617" t="n"/>
+      <c r="G19" s="1617" t="n"/>
+      <c r="H19" s="1617" t="n"/>
+      <c r="I19" s="1618" t="n"/>
+      <c r="J19" s="1619" t="n"/>
+      <c r="K19" s="1619" t="n"/>
+      <c r="L19" s="1619" t="n"/>
+      <c r="M19" s="1617" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1575" t="n">
+      <c r="N19" s="1617" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1575" t="n"/>
-      <c r="P19" s="1578" t="n"/>
-      <c r="Q19" s="1575" t="n"/>
-      <c r="R19" s="1575" t="n"/>
-      <c r="S19" s="1575" t="n"/>
+      <c r="O19" s="1617" t="n"/>
+      <c r="P19" s="1620" t="n"/>
+      <c r="Q19" s="1617" t="n"/>
+      <c r="R19" s="1617" t="n"/>
+      <c r="S19" s="1617" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1574" t="n"/>
+      <c r="U19" s="1616" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -6490,43 +6598,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1573" t="inlineStr">
+      <c r="A20" s="1615" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1574" t="inlineStr">
+      <c r="B20" s="1616" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1574" t="inlineStr">
+      <c r="C20" s="1616" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1575" t="n"/>
-      <c r="E20" s="1575" t="n"/>
-      <c r="F20" s="1575" t="n"/>
-      <c r="G20" s="1575" t="n"/>
-      <c r="H20" s="1575" t="n"/>
-      <c r="I20" s="1576" t="n"/>
-      <c r="J20" s="1577" t="n"/>
-      <c r="K20" s="1577" t="n"/>
-      <c r="L20" s="1577" t="n"/>
-      <c r="M20" s="1575" t="n"/>
-      <c r="N20" s="1575" t="n"/>
-      <c r="O20" s="1575" t="n"/>
-      <c r="P20" s="1578" t="n"/>
-      <c r="Q20" s="1575" t="n"/>
-      <c r="R20" s="1575" t="n"/>
-      <c r="S20" s="1575" t="n"/>
+      <c r="D20" s="1617" t="n"/>
+      <c r="E20" s="1617" t="n"/>
+      <c r="F20" s="1617" t="n"/>
+      <c r="G20" s="1617" t="n"/>
+      <c r="H20" s="1617" t="n"/>
+      <c r="I20" s="1618" t="n"/>
+      <c r="J20" s="1619" t="n"/>
+      <c r="K20" s="1619" t="n"/>
+      <c r="L20" s="1619" t="n"/>
+      <c r="M20" s="1617" t="n"/>
+      <c r="N20" s="1617" t="n"/>
+      <c r="O20" s="1617" t="n"/>
+      <c r="P20" s="1620" t="n"/>
+      <c r="Q20" s="1617" t="n"/>
+      <c r="R20" s="1617" t="n"/>
+      <c r="S20" s="1617" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1574" t="n"/>
+      <c r="U20" s="1616" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -6534,39 +6642,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1549" t="inlineStr">
+      <c r="A21" s="1591" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1550" t="inlineStr">
+      <c r="B21" s="1592" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1550" t="inlineStr">
+      <c r="C21" s="1592" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1551" t="n"/>
-      <c r="E21" s="1551" t="n"/>
-      <c r="F21" s="1551" t="n"/>
-      <c r="G21" s="1551" t="n"/>
-      <c r="H21" s="1551" t="n"/>
-      <c r="I21" s="1552" t="n"/>
-      <c r="J21" s="1553" t="n"/>
-      <c r="K21" s="1553" t="n"/>
-      <c r="L21" s="1553" t="n"/>
-      <c r="M21" s="1551" t="n"/>
-      <c r="N21" s="1551" t="n"/>
-      <c r="O21" s="1551" t="n"/>
-      <c r="P21" s="1554" t="n"/>
-      <c r="Q21" s="1551" t="n"/>
-      <c r="R21" s="1551" t="n"/>
-      <c r="S21" s="1551" t="n"/>
+      <c r="D21" s="1593" t="n"/>
+      <c r="E21" s="1593" t="n"/>
+      <c r="F21" s="1593" t="n"/>
+      <c r="G21" s="1593" t="n"/>
+      <c r="H21" s="1593" t="n"/>
+      <c r="I21" s="1594" t="n"/>
+      <c r="J21" s="1595" t="n"/>
+      <c r="K21" s="1595" t="n"/>
+      <c r="L21" s="1595" t="n"/>
+      <c r="M21" s="1593" t="n"/>
+      <c r="N21" s="1593" t="n"/>
+      <c r="O21" s="1593" t="n"/>
+      <c r="P21" s="1596" t="n"/>
+      <c r="Q21" s="1593" t="n"/>
+      <c r="R21" s="1593" t="n"/>
+      <c r="S21" s="1593" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1550" t="n"/>
+      <c r="U21" s="1592" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -6574,39 +6682,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1555" t="inlineStr">
+      <c r="A22" s="1597" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1556" t="inlineStr">
+      <c r="B22" s="1598" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1556" t="inlineStr">
+      <c r="C22" s="1598" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1557" t="n"/>
-      <c r="E22" s="1557" t="n"/>
-      <c r="F22" s="1557" t="n"/>
-      <c r="G22" s="1557" t="n"/>
-      <c r="H22" s="1557" t="n"/>
-      <c r="I22" s="1558" t="n"/>
-      <c r="J22" s="1559" t="n"/>
-      <c r="K22" s="1559" t="n"/>
-      <c r="L22" s="1559" t="n"/>
-      <c r="M22" s="1557" t="n"/>
-      <c r="N22" s="1557" t="n"/>
-      <c r="O22" s="1557" t="n"/>
-      <c r="P22" s="1560" t="n"/>
-      <c r="Q22" s="1557" t="n"/>
-      <c r="R22" s="1557" t="n"/>
-      <c r="S22" s="1557" t="n"/>
+      <c r="D22" s="1599" t="n"/>
+      <c r="E22" s="1599" t="n"/>
+      <c r="F22" s="1599" t="n"/>
+      <c r="G22" s="1599" t="n"/>
+      <c r="H22" s="1599" t="n"/>
+      <c r="I22" s="1600" t="n"/>
+      <c r="J22" s="1601" t="n"/>
+      <c r="K22" s="1601" t="n"/>
+      <c r="L22" s="1601" t="n"/>
+      <c r="M22" s="1599" t="n"/>
+      <c r="N22" s="1599" t="n"/>
+      <c r="O22" s="1599" t="n"/>
+      <c r="P22" s="1602" t="n"/>
+      <c r="Q22" s="1599" t="n"/>
+      <c r="R22" s="1599" t="n"/>
+      <c r="S22" s="1599" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1556" t="n"/>
+      <c r="U22" s="1598" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -6614,53 +6722,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1561" t="inlineStr">
+      <c r="A23" s="1603" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1562" t="inlineStr">
+      <c r="B23" s="1604" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1562" t="inlineStr">
+      <c r="C23" s="1604" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1563" t="n"/>
-      <c r="E23" s="1563" t="n">
+      <c r="D23" s="1605" t="n"/>
+      <c r="E23" s="1605" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1563" t="n">
+      <c r="F23" s="1605" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1563" t="n">
+      <c r="G23" s="1605" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1563" t="n"/>
-      <c r="I23" s="1564" t="n"/>
-      <c r="J23" s="1565" t="n"/>
-      <c r="K23" s="1565" t="n"/>
-      <c r="L23" s="1565" t="n"/>
-      <c r="M23" s="1563" t="n"/>
-      <c r="N23" s="1563" t="n"/>
-      <c r="O23" s="1563" t="n">
+      <c r="H23" s="1605" t="n"/>
+      <c r="I23" s="1606" t="n"/>
+      <c r="J23" s="1607" t="n"/>
+      <c r="K23" s="1607" t="n"/>
+      <c r="L23" s="1607" t="n"/>
+      <c r="M23" s="1605" t="n"/>
+      <c r="N23" s="1605" t="n"/>
+      <c r="O23" s="1605" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1566" t="n">
+      <c r="P23" s="1608" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1563" t="n"/>
-      <c r="R23" s="1563" t="n"/>
-      <c r="S23" s="1563" t="n"/>
+      <c r="Q23" s="1605" t="n"/>
+      <c r="R23" s="1605" t="n"/>
+      <c r="S23" s="1605" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1562" t="n"/>
+      <c r="U23" s="1604" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -6668,47 +6776,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1567" t="inlineStr">
+      <c r="A24" s="1609" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1568" t="inlineStr">
+      <c r="B24" s="1610" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1568" t="inlineStr">
+      <c r="C24" s="1610" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1569" t="n"/>
-      <c r="E24" s="1569" t="n"/>
-      <c r="F24" s="1569" t="n"/>
-      <c r="G24" s="1569" t="n"/>
-      <c r="H24" s="1569" t="n"/>
-      <c r="I24" s="1570" t="n"/>
-      <c r="J24" s="1571" t="n"/>
-      <c r="K24" s="1571" t="n"/>
-      <c r="L24" s="1571" t="n"/>
-      <c r="M24" s="1569" t="n">
+      <c r="D24" s="1611" t="n"/>
+      <c r="E24" s="1611" t="n"/>
+      <c r="F24" s="1611" t="n"/>
+      <c r="G24" s="1611" t="n"/>
+      <c r="H24" s="1611" t="n"/>
+      <c r="I24" s="1612" t="n"/>
+      <c r="J24" s="1613" t="n"/>
+      <c r="K24" s="1613" t="n"/>
+      <c r="L24" s="1613" t="n"/>
+      <c r="M24" s="1611" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1569" t="n">
+      <c r="N24" s="1611" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1569" t="n"/>
-      <c r="P24" s="1572" t="n"/>
-      <c r="Q24" s="1569" t="n"/>
-      <c r="R24" s="1569" t="n"/>
-      <c r="S24" s="1569" t="n"/>
+      <c r="O24" s="1611" t="n"/>
+      <c r="P24" s="1614" t="n"/>
+      <c r="Q24" s="1611" t="n"/>
+      <c r="R24" s="1611" t="n"/>
+      <c r="S24" s="1611" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1568" t="n"/>
+      <c r="U24" s="1610" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -6716,61 +6824,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1543" t="inlineStr">
+      <c r="A25" s="1585" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1544" t="inlineStr">
+      <c r="B25" s="1586" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1544" t="inlineStr">
+      <c r="C25" s="1586" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1545" t="n">
+      <c r="D25" s="1587" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1545" t="n">
+      <c r="E25" s="1587" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1545" t="n">
+      <c r="F25" s="1587" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1545" t="n">
+      <c r="G25" s="1587" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1545" t="n"/>
-      <c r="I25" s="1546" t="n"/>
-      <c r="J25" s="1547" t="n">
+      <c r="H25" s="1587" t="n"/>
+      <c r="I25" s="1588" t="n"/>
+      <c r="J25" s="1589" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1547" t="n">
+      <c r="K25" s="1589" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1547" t="n">
+      <c r="L25" s="1589" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1545" t="n"/>
-      <c r="N25" s="1545" t="n"/>
-      <c r="O25" s="1545" t="n">
+      <c r="M25" s="1587" t="n"/>
+      <c r="N25" s="1587" t="n"/>
+      <c r="O25" s="1587" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1548" t="n">
+      <c r="P25" s="1590" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1545" t="n"/>
-      <c r="R25" s="1545" t="n"/>
-      <c r="S25" s="1545" t="n"/>
+      <c r="Q25" s="1587" t="n"/>
+      <c r="R25" s="1587" t="n"/>
+      <c r="S25" s="1587" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1544" t="n"/>
+      <c r="U25" s="1586" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -6778,47 +6886,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1549" t="inlineStr">
+      <c r="A26" s="1591" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1550" t="inlineStr">
+      <c r="B26" s="1592" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1550" t="inlineStr">
+      <c r="C26" s="1592" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1551" t="n"/>
-      <c r="E26" s="1551" t="n"/>
-      <c r="F26" s="1551" t="n"/>
-      <c r="G26" s="1551" t="n"/>
-      <c r="H26" s="1551" t="n"/>
-      <c r="I26" s="1552" t="n"/>
-      <c r="J26" s="1553" t="n"/>
-      <c r="K26" s="1553" t="n"/>
-      <c r="L26" s="1553" t="n"/>
-      <c r="M26" s="1551" t="n">
+      <c r="D26" s="1593" t="n"/>
+      <c r="E26" s="1593" t="n"/>
+      <c r="F26" s="1593" t="n"/>
+      <c r="G26" s="1593" t="n"/>
+      <c r="H26" s="1593" t="n"/>
+      <c r="I26" s="1594" t="n"/>
+      <c r="J26" s="1595" t="n"/>
+      <c r="K26" s="1595" t="n"/>
+      <c r="L26" s="1595" t="n"/>
+      <c r="M26" s="1593" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1551" t="n">
+      <c r="N26" s="1593" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1551" t="n"/>
-      <c r="P26" s="1554" t="n"/>
-      <c r="Q26" s="1551" t="n"/>
-      <c r="R26" s="1551" t="n"/>
-      <c r="S26" s="1551" t="n"/>
+      <c r="O26" s="1593" t="n"/>
+      <c r="P26" s="1596" t="n"/>
+      <c r="Q26" s="1593" t="n"/>
+      <c r="R26" s="1593" t="n"/>
+      <c r="S26" s="1593" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1550" t="n"/>
+      <c r="U26" s="1592" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -6826,53 +6934,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1555" t="inlineStr">
+      <c r="A27" s="1597" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1556" t="inlineStr">
+      <c r="B27" s="1598" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1556" t="inlineStr">
+      <c r="C27" s="1598" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1557" t="n"/>
-      <c r="E27" s="1557" t="n">
+      <c r="D27" s="1599" t="n"/>
+      <c r="E27" s="1599" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1557" t="n">
+      <c r="F27" s="1599" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1557" t="n">
+      <c r="G27" s="1599" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1557" t="n"/>
-      <c r="I27" s="1558" t="n"/>
-      <c r="J27" s="1559" t="n"/>
-      <c r="K27" s="1559" t="n"/>
-      <c r="L27" s="1559" t="n"/>
-      <c r="M27" s="1557" t="n"/>
-      <c r="N27" s="1557" t="n"/>
-      <c r="O27" s="1557" t="n">
+      <c r="H27" s="1599" t="n"/>
+      <c r="I27" s="1600" t="n"/>
+      <c r="J27" s="1601" t="n"/>
+      <c r="K27" s="1601" t="n"/>
+      <c r="L27" s="1601" t="n"/>
+      <c r="M27" s="1599" t="n"/>
+      <c r="N27" s="1599" t="n"/>
+      <c r="O27" s="1599" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1560" t="n">
+      <c r="P27" s="1602" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1557" t="n"/>
-      <c r="R27" s="1557" t="n"/>
-      <c r="S27" s="1557" t="n"/>
+      <c r="Q27" s="1599" t="n"/>
+      <c r="R27" s="1599" t="n"/>
+      <c r="S27" s="1599" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1556" t="n"/>
+      <c r="U27" s="1598" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -6880,47 +6988,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1567" t="inlineStr">
+      <c r="A28" s="1609" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1568" t="inlineStr">
+      <c r="B28" s="1610" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1568" t="inlineStr">
+      <c r="C28" s="1610" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1569" t="n"/>
-      <c r="E28" s="1569" t="n"/>
-      <c r="F28" s="1569" t="n"/>
-      <c r="G28" s="1569" t="n"/>
-      <c r="H28" s="1569" t="n"/>
-      <c r="I28" s="1570" t="n"/>
-      <c r="J28" s="1571" t="n"/>
-      <c r="K28" s="1571" t="n"/>
-      <c r="L28" s="1571" t="n"/>
-      <c r="M28" s="1569" t="n">
+      <c r="D28" s="1611" t="n"/>
+      <c r="E28" s="1611" t="n"/>
+      <c r="F28" s="1611" t="n"/>
+      <c r="G28" s="1611" t="n"/>
+      <c r="H28" s="1611" t="n"/>
+      <c r="I28" s="1612" t="n"/>
+      <c r="J28" s="1613" t="n"/>
+      <c r="K28" s="1613" t="n"/>
+      <c r="L28" s="1613" t="n"/>
+      <c r="M28" s="1611" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1569" t="n">
+      <c r="N28" s="1611" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1569" t="n"/>
-      <c r="P28" s="1572" t="n"/>
-      <c r="Q28" s="1569" t="n"/>
-      <c r="R28" s="1569" t="n"/>
-      <c r="S28" s="1569" t="n"/>
+      <c r="O28" s="1611" t="n"/>
+      <c r="P28" s="1614" t="n"/>
+      <c r="Q28" s="1611" t="n"/>
+      <c r="R28" s="1611" t="n"/>
+      <c r="S28" s="1611" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1568" t="n"/>
+      <c r="U28" s="1610" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -6928,53 +7036,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1543" t="inlineStr">
+      <c r="A29" s="1585" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1544" t="inlineStr">
+      <c r="B29" s="1586" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1544" t="inlineStr">
+      <c r="C29" s="1586" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1545" t="n"/>
-      <c r="E29" s="1545" t="n">
+      <c r="D29" s="1587" t="n"/>
+      <c r="E29" s="1587" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1545" t="n">
+      <c r="F29" s="1587" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1545" t="n">
+      <c r="G29" s="1587" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1545" t="n"/>
-      <c r="I29" s="1546" t="n"/>
-      <c r="J29" s="1547" t="n"/>
-      <c r="K29" s="1547" t="n"/>
-      <c r="L29" s="1547" t="n"/>
-      <c r="M29" s="1545" t="n"/>
-      <c r="N29" s="1545" t="n"/>
-      <c r="O29" s="1545" t="n">
+      <c r="H29" s="1587" t="n"/>
+      <c r="I29" s="1588" t="n"/>
+      <c r="J29" s="1589" t="n"/>
+      <c r="K29" s="1589" t="n"/>
+      <c r="L29" s="1589" t="n"/>
+      <c r="M29" s="1587" t="n"/>
+      <c r="N29" s="1587" t="n"/>
+      <c r="O29" s="1587" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1548" t="n">
+      <c r="P29" s="1590" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1545" t="n"/>
-      <c r="R29" s="1545" t="n"/>
-      <c r="S29" s="1545" t="n"/>
+      <c r="Q29" s="1587" t="n"/>
+      <c r="R29" s="1587" t="n"/>
+      <c r="S29" s="1587" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1544" t="n"/>
+      <c r="U29" s="1586" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -6982,43 +7090,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1549" t="inlineStr">
+      <c r="A30" s="1591" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1550" t="inlineStr">
+      <c r="B30" s="1592" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1550" t="inlineStr">
+      <c r="C30" s="1592" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1551" t="n"/>
-      <c r="E30" s="1551" t="n"/>
-      <c r="F30" s="1551" t="n"/>
-      <c r="G30" s="1551" t="n"/>
-      <c r="H30" s="1551" t="n"/>
-      <c r="I30" s="1552" t="n"/>
-      <c r="J30" s="1553" t="n"/>
-      <c r="K30" s="1553" t="n"/>
-      <c r="L30" s="1553" t="n"/>
-      <c r="M30" s="1551" t="n"/>
-      <c r="N30" s="1551" t="n"/>
-      <c r="O30" s="1551" t="n"/>
-      <c r="P30" s="1554" t="n"/>
-      <c r="Q30" s="1551" t="n"/>
-      <c r="R30" s="1551" t="n"/>
-      <c r="S30" s="1551" t="n"/>
+      <c r="D30" s="1593" t="n"/>
+      <c r="E30" s="1593" t="n"/>
+      <c r="F30" s="1593" t="n"/>
+      <c r="G30" s="1593" t="n"/>
+      <c r="H30" s="1593" t="n"/>
+      <c r="I30" s="1594" t="n"/>
+      <c r="J30" s="1595" t="n"/>
+      <c r="K30" s="1595" t="n"/>
+      <c r="L30" s="1595" t="n"/>
+      <c r="M30" s="1593" t="n"/>
+      <c r="N30" s="1593" t="n"/>
+      <c r="O30" s="1593" t="n"/>
+      <c r="P30" s="1596" t="n"/>
+      <c r="Q30" s="1593" t="n"/>
+      <c r="R30" s="1593" t="n"/>
+      <c r="S30" s="1593" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1550" t="n"/>
+      <c r="U30" s="1592" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -7026,53 +7134,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1555" t="inlineStr">
+      <c r="A31" s="1597" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1556" t="inlineStr">
+      <c r="B31" s="1598" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1556" t="inlineStr">
+      <c r="C31" s="1598" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1557" t="n"/>
-      <c r="E31" s="1557" t="n">
+      <c r="D31" s="1599" t="n"/>
+      <c r="E31" s="1599" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1557" t="n">
+      <c r="F31" s="1599" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1557" t="n">
+      <c r="G31" s="1599" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1557" t="n"/>
-      <c r="I31" s="1558" t="n"/>
-      <c r="J31" s="1559" t="n"/>
-      <c r="K31" s="1559" t="n"/>
-      <c r="L31" s="1559" t="n"/>
-      <c r="M31" s="1557" t="n"/>
-      <c r="N31" s="1557" t="n"/>
-      <c r="O31" s="1557" t="n">
+      <c r="H31" s="1599" t="n"/>
+      <c r="I31" s="1600" t="n"/>
+      <c r="J31" s="1601" t="n"/>
+      <c r="K31" s="1601" t="n"/>
+      <c r="L31" s="1601" t="n"/>
+      <c r="M31" s="1599" t="n"/>
+      <c r="N31" s="1599" t="n"/>
+      <c r="O31" s="1599" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1560" t="n">
+      <c r="P31" s="1602" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1557" t="n"/>
-      <c r="R31" s="1557" t="n"/>
-      <c r="S31" s="1557" t="n"/>
+      <c r="Q31" s="1599" t="n"/>
+      <c r="R31" s="1599" t="n"/>
+      <c r="S31" s="1599" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1556" t="inlineStr">
+      <c r="U31" s="1598" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -7084,49 +7192,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1567" t="inlineStr">
+      <c r="A32" s="1609" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1568" t="inlineStr">
+      <c r="B32" s="1610" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1568" t="inlineStr">
+      <c r="C32" s="1610" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1569" t="n"/>
-      <c r="E32" s="1569" t="n"/>
-      <c r="F32" s="1569" t="n"/>
-      <c r="G32" s="1569" t="n"/>
-      <c r="H32" s="1569" t="n">
+      <c r="D32" s="1611" t="n"/>
+      <c r="E32" s="1611" t="n"/>
+      <c r="F32" s="1611" t="n"/>
+      <c r="G32" s="1611" t="n"/>
+      <c r="H32" s="1611" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1570" t="n"/>
-      <c r="J32" s="1571" t="n"/>
-      <c r="K32" s="1571" t="n"/>
-      <c r="L32" s="1571" t="n"/>
-      <c r="M32" s="1569" t="n">
+      <c r="I32" s="1612" t="n"/>
+      <c r="J32" s="1613" t="n"/>
+      <c r="K32" s="1613" t="n"/>
+      <c r="L32" s="1613" t="n"/>
+      <c r="M32" s="1611" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1569" t="n">
+      <c r="N32" s="1611" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1569" t="n"/>
-      <c r="P32" s="1572" t="n"/>
-      <c r="Q32" s="1569" t="n"/>
-      <c r="R32" s="1569" t="n"/>
-      <c r="S32" s="1569" t="n"/>
+      <c r="O32" s="1611" t="n"/>
+      <c r="P32" s="1614" t="n"/>
+      <c r="Q32" s="1611" t="n"/>
+      <c r="R32" s="1611" t="n"/>
+      <c r="S32" s="1611" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1568" t="n"/>
+      <c r="U32" s="1610" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -7134,57 +7242,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1543" t="inlineStr">
+      <c r="A33" s="1585" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1544" t="inlineStr">
+      <c r="B33" s="1586" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1544" t="inlineStr">
+      <c r="C33" s="1586" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1545" t="n"/>
-      <c r="E33" s="1545" t="n">
+      <c r="D33" s="1587" t="n"/>
+      <c r="E33" s="1587" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1545" t="n">
+      <c r="F33" s="1587" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1545" t="n">
+      <c r="G33" s="1587" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1545" t="n"/>
-      <c r="I33" s="1546" t="n">
+      <c r="H33" s="1587" t="n"/>
+      <c r="I33" s="1588" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1547" t="n"/>
-      <c r="K33" s="1547" t="n"/>
-      <c r="L33" s="1547" t="n"/>
-      <c r="M33" s="1545" t="n"/>
-      <c r="N33" s="1545" t="n"/>
-      <c r="O33" s="1545" t="n">
+      <c r="J33" s="1589" t="n"/>
+      <c r="K33" s="1589" t="n"/>
+      <c r="L33" s="1589" t="n"/>
+      <c r="M33" s="1587" t="n"/>
+      <c r="N33" s="1587" t="n"/>
+      <c r="O33" s="1587" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1548" t="n">
+      <c r="P33" s="1590" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1545" t="n"/>
-      <c r="R33" s="1545" t="n">
+      <c r="Q33" s="1587" t="n"/>
+      <c r="R33" s="1587" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1545" t="n"/>
+      <c r="S33" s="1587" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1544" t="inlineStr">
+      <c r="U33" s="1586" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -7196,49 +7304,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1549" t="inlineStr">
+      <c r="A34" s="1591" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1550" t="inlineStr">
+      <c r="B34" s="1592" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1550" t="inlineStr">
+      <c r="C34" s="1592" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1551" t="n"/>
-      <c r="E34" s="1551" t="n"/>
-      <c r="F34" s="1551" t="n"/>
-      <c r="G34" s="1551" t="n"/>
-      <c r="H34" s="1551" t="n">
+      <c r="D34" s="1593" t="n"/>
+      <c r="E34" s="1593" t="n"/>
+      <c r="F34" s="1593" t="n"/>
+      <c r="G34" s="1593" t="n"/>
+      <c r="H34" s="1593" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1552" t="n"/>
-      <c r="J34" s="1553" t="n"/>
-      <c r="K34" s="1553" t="n"/>
-      <c r="L34" s="1553" t="n"/>
-      <c r="M34" s="1551" t="n">
+      <c r="I34" s="1594" t="n"/>
+      <c r="J34" s="1595" t="n"/>
+      <c r="K34" s="1595" t="n"/>
+      <c r="L34" s="1595" t="n"/>
+      <c r="M34" s="1593" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1551" t="n">
+      <c r="N34" s="1593" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1551" t="n"/>
-      <c r="P34" s="1554" t="n"/>
-      <c r="Q34" s="1551" t="n"/>
-      <c r="R34" s="1551" t="n"/>
-      <c r="S34" s="1551" t="n"/>
+      <c r="O34" s="1593" t="n"/>
+      <c r="P34" s="1596" t="n"/>
+      <c r="Q34" s="1593" t="n"/>
+      <c r="R34" s="1593" t="n"/>
+      <c r="S34" s="1593" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1550" t="n"/>
+      <c r="U34" s="1592" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -7246,57 +7354,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1555" t="inlineStr">
+      <c r="A35" s="1597" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1556" t="inlineStr">
+      <c r="B35" s="1598" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1556" t="inlineStr">
+      <c r="C35" s="1598" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1557" t="n"/>
-      <c r="E35" s="1557" t="n">
+      <c r="D35" s="1599" t="n"/>
+      <c r="E35" s="1599" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1557" t="n">
+      <c r="F35" s="1599" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1557" t="n">
+      <c r="G35" s="1599" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1557" t="n"/>
-      <c r="I35" s="1558" t="n">
+      <c r="H35" s="1599" t="n"/>
+      <c r="I35" s="1600" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1559" t="n"/>
-      <c r="K35" s="1559" t="n"/>
-      <c r="L35" s="1559" t="n"/>
-      <c r="M35" s="1557" t="n"/>
-      <c r="N35" s="1557" t="n"/>
-      <c r="O35" s="1557" t="n">
+      <c r="J35" s="1601" t="n"/>
+      <c r="K35" s="1601" t="n"/>
+      <c r="L35" s="1601" t="n"/>
+      <c r="M35" s="1599" t="n"/>
+      <c r="N35" s="1599" t="n"/>
+      <c r="O35" s="1599" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1560" t="n">
+      <c r="P35" s="1602" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1557" t="n"/>
-      <c r="R35" s="1557" t="n">
+      <c r="Q35" s="1599" t="n"/>
+      <c r="R35" s="1599" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1557" t="n"/>
+      <c r="S35" s="1599" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1556" t="inlineStr">
+      <c r="U35" s="1598" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -7308,49 +7416,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1561" t="inlineStr">
+      <c r="A36" s="1603" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1562" t="inlineStr">
+      <c r="B36" s="1604" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1562" t="inlineStr">
+      <c r="C36" s="1604" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1563" t="n"/>
-      <c r="E36" s="1563" t="n"/>
-      <c r="F36" s="1563" t="n"/>
-      <c r="G36" s="1563" t="n"/>
-      <c r="H36" s="1563" t="n">
+      <c r="D36" s="1605" t="n"/>
+      <c r="E36" s="1605" t="n"/>
+      <c r="F36" s="1605" t="n"/>
+      <c r="G36" s="1605" t="n"/>
+      <c r="H36" s="1605" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1564" t="n"/>
-      <c r="J36" s="1565" t="n"/>
-      <c r="K36" s="1565" t="n"/>
-      <c r="L36" s="1565" t="n"/>
-      <c r="M36" s="1563" t="n">
+      <c r="I36" s="1606" t="n"/>
+      <c r="J36" s="1607" t="n"/>
+      <c r="K36" s="1607" t="n"/>
+      <c r="L36" s="1607" t="n"/>
+      <c r="M36" s="1605" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1563" t="n">
+      <c r="N36" s="1605" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1563" t="n"/>
-      <c r="P36" s="1566" t="n"/>
-      <c r="Q36" s="1563" t="n"/>
-      <c r="R36" s="1563" t="n"/>
-      <c r="S36" s="1563" t="n"/>
+      <c r="O36" s="1605" t="n"/>
+      <c r="P36" s="1608" t="n"/>
+      <c r="Q36" s="1605" t="n"/>
+      <c r="R36" s="1605" t="n"/>
+      <c r="S36" s="1605" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1562" t="n"/>
+      <c r="U36" s="1604" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -7358,41 +7466,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1567" t="inlineStr">
+      <c r="A37" s="1609" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1568" t="inlineStr">
+      <c r="B37" s="1610" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1568" t="inlineStr">
+      <c r="C37" s="1610" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1569" t="n"/>
-      <c r="E37" s="1569" t="n"/>
-      <c r="F37" s="1569" t="n"/>
-      <c r="G37" s="1569" t="n"/>
-      <c r="H37" s="1569" t="n"/>
-      <c r="I37" s="1570" t="n"/>
-      <c r="J37" s="1571" t="n"/>
-      <c r="K37" s="1571" t="n"/>
-      <c r="L37" s="1571" t="n"/>
-      <c r="M37" s="1569" t="n"/>
-      <c r="N37" s="1569" t="n"/>
-      <c r="O37" s="1569" t="n"/>
-      <c r="P37" s="1572" t="n"/>
-      <c r="Q37" s="1569" t="n">
+      <c r="D37" s="1611" t="n"/>
+      <c r="E37" s="1611" t="n"/>
+      <c r="F37" s="1611" t="n"/>
+      <c r="G37" s="1611" t="n"/>
+      <c r="H37" s="1611" t="n"/>
+      <c r="I37" s="1612" t="n"/>
+      <c r="J37" s="1613" t="n"/>
+      <c r="K37" s="1613" t="n"/>
+      <c r="L37" s="1613" t="n"/>
+      <c r="M37" s="1611" t="n"/>
+      <c r="N37" s="1611" t="n"/>
+      <c r="O37" s="1611" t="n"/>
+      <c r="P37" s="1614" t="n"/>
+      <c r="Q37" s="1611" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1569" t="n"/>
-      <c r="S37" s="1569" t="n"/>
+      <c r="R37" s="1611" t="n"/>
+      <c r="S37" s="1611" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1568" t="n"/>
+      <c r="U37" s="1610" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -7400,57 +7508,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1543" t="inlineStr">
+      <c r="A38" s="1585" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1544" t="inlineStr">
+      <c r="B38" s="1586" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1544" t="inlineStr">
+      <c r="C38" s="1586" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1545" t="n"/>
-      <c r="E38" s="1545" t="n">
+      <c r="D38" s="1587" t="n"/>
+      <c r="E38" s="1587" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1545" t="n">
+      <c r="F38" s="1587" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1545" t="n">
+      <c r="G38" s="1587" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1545" t="n"/>
-      <c r="I38" s="1546" t="n">
+      <c r="H38" s="1587" t="n"/>
+      <c r="I38" s="1588" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1547" t="n"/>
-      <c r="K38" s="1547" t="n"/>
-      <c r="L38" s="1547" t="n"/>
-      <c r="M38" s="1545" t="n"/>
-      <c r="N38" s="1545" t="n"/>
-      <c r="O38" s="1545" t="n">
+      <c r="J38" s="1589" t="n"/>
+      <c r="K38" s="1589" t="n"/>
+      <c r="L38" s="1589" t="n"/>
+      <c r="M38" s="1587" t="n"/>
+      <c r="N38" s="1587" t="n"/>
+      <c r="O38" s="1587" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1548" t="n">
+      <c r="P38" s="1590" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1545" t="n"/>
-      <c r="R38" s="1545" t="n">
+      <c r="Q38" s="1587" t="n"/>
+      <c r="R38" s="1587" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1545" t="n"/>
+      <c r="S38" s="1587" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1544" t="inlineStr">
+      <c r="U38" s="1586" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -7462,49 +7570,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1573" t="inlineStr">
+      <c r="A39" s="1615" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1574" t="inlineStr">
+      <c r="B39" s="1616" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1574" t="inlineStr">
+      <c r="C39" s="1616" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1575" t="n"/>
-      <c r="E39" s="1575" t="n"/>
-      <c r="F39" s="1575" t="n"/>
-      <c r="G39" s="1575" t="n"/>
-      <c r="H39" s="1575" t="n">
+      <c r="D39" s="1617" t="n"/>
+      <c r="E39" s="1617" t="n"/>
+      <c r="F39" s="1617" t="n"/>
+      <c r="G39" s="1617" t="n"/>
+      <c r="H39" s="1617" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1576" t="n"/>
-      <c r="J39" s="1577" t="n"/>
-      <c r="K39" s="1577" t="n"/>
-      <c r="L39" s="1577" t="n"/>
-      <c r="M39" s="1575" t="n">
+      <c r="I39" s="1618" t="n"/>
+      <c r="J39" s="1619" t="n"/>
+      <c r="K39" s="1619" t="n"/>
+      <c r="L39" s="1619" t="n"/>
+      <c r="M39" s="1617" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1575" t="n">
+      <c r="N39" s="1617" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1575" t="n"/>
-      <c r="P39" s="1578" t="n"/>
-      <c r="Q39" s="1575" t="n"/>
-      <c r="R39" s="1575" t="n"/>
-      <c r="S39" s="1575" t="n"/>
+      <c r="O39" s="1617" t="n"/>
+      <c r="P39" s="1620" t="n"/>
+      <c r="Q39" s="1617" t="n"/>
+      <c r="R39" s="1617" t="n"/>
+      <c r="S39" s="1617" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1574" t="n"/>
+      <c r="U39" s="1616" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -7512,41 +7620,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1549" t="inlineStr">
+      <c r="A40" s="1591" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1550" t="inlineStr">
+      <c r="B40" s="1592" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1550" t="inlineStr">
+      <c r="C40" s="1592" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1551" t="n"/>
-      <c r="E40" s="1551" t="n"/>
-      <c r="F40" s="1551" t="n"/>
-      <c r="G40" s="1551" t="n"/>
-      <c r="H40" s="1551" t="n"/>
-      <c r="I40" s="1552" t="n"/>
-      <c r="J40" s="1553" t="n"/>
-      <c r="K40" s="1553" t="n"/>
-      <c r="L40" s="1553" t="n"/>
-      <c r="M40" s="1551" t="n"/>
-      <c r="N40" s="1551" t="n"/>
-      <c r="O40" s="1551" t="n"/>
-      <c r="P40" s="1554" t="n"/>
-      <c r="Q40" s="1551" t="n">
+      <c r="D40" s="1593" t="n"/>
+      <c r="E40" s="1593" t="n"/>
+      <c r="F40" s="1593" t="n"/>
+      <c r="G40" s="1593" t="n"/>
+      <c r="H40" s="1593" t="n"/>
+      <c r="I40" s="1594" t="n"/>
+      <c r="J40" s="1595" t="n"/>
+      <c r="K40" s="1595" t="n"/>
+      <c r="L40" s="1595" t="n"/>
+      <c r="M40" s="1593" t="n"/>
+      <c r="N40" s="1593" t="n"/>
+      <c r="O40" s="1593" t="n"/>
+      <c r="P40" s="1596" t="n"/>
+      <c r="Q40" s="1593" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1551" t="n"/>
-      <c r="S40" s="1551" t="n"/>
+      <c r="R40" s="1593" t="n"/>
+      <c r="S40" s="1593" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1550" t="n"/>
+      <c r="U40" s="1592" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -7554,57 +7662,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1555" t="inlineStr">
+      <c r="A41" s="1597" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1556" t="inlineStr">
+      <c r="B41" s="1598" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1556" t="inlineStr">
+      <c r="C41" s="1598" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1557" t="n"/>
-      <c r="E41" s="1557" t="n">
+      <c r="D41" s="1599" t="n"/>
+      <c r="E41" s="1599" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1557" t="n">
+      <c r="F41" s="1599" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1557" t="n">
+      <c r="G41" s="1599" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1557" t="n"/>
-      <c r="I41" s="1558" t="n">
+      <c r="H41" s="1599" t="n"/>
+      <c r="I41" s="1600" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1559" t="n"/>
-      <c r="K41" s="1559" t="n"/>
-      <c r="L41" s="1559" t="n"/>
-      <c r="M41" s="1557" t="n"/>
-      <c r="N41" s="1557" t="n"/>
-      <c r="O41" s="1557" t="n">
+      <c r="J41" s="1601" t="n"/>
+      <c r="K41" s="1601" t="n"/>
+      <c r="L41" s="1601" t="n"/>
+      <c r="M41" s="1599" t="n"/>
+      <c r="N41" s="1599" t="n"/>
+      <c r="O41" s="1599" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1560" t="n">
+      <c r="P41" s="1602" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1557" t="n"/>
-      <c r="R41" s="1557" t="n">
+      <c r="Q41" s="1599" t="n"/>
+      <c r="R41" s="1599" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1557" t="n"/>
+      <c r="S41" s="1599" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1556" t="inlineStr">
+      <c r="U41" s="1598" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -7616,49 +7724,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1567" t="inlineStr">
+      <c r="A42" s="1609" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1568" t="inlineStr">
+      <c r="B42" s="1610" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1568" t="inlineStr">
+      <c r="C42" s="1610" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1569" t="n"/>
-      <c r="E42" s="1569" t="n"/>
-      <c r="F42" s="1569" t="n"/>
-      <c r="G42" s="1569" t="n"/>
-      <c r="H42" s="1569" t="n">
+      <c r="D42" s="1611" t="n"/>
+      <c r="E42" s="1611" t="n"/>
+      <c r="F42" s="1611" t="n"/>
+      <c r="G42" s="1611" t="n"/>
+      <c r="H42" s="1611" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1570" t="n"/>
-      <c r="J42" s="1571" t="n"/>
-      <c r="K42" s="1571" t="n"/>
-      <c r="L42" s="1571" t="n"/>
-      <c r="M42" s="1569" t="n">
+      <c r="I42" s="1612" t="n"/>
+      <c r="J42" s="1613" t="n"/>
+      <c r="K42" s="1613" t="n"/>
+      <c r="L42" s="1613" t="n"/>
+      <c r="M42" s="1611" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1569" t="n">
+      <c r="N42" s="1611" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1569" t="n"/>
-      <c r="P42" s="1572" t="n"/>
-      <c r="Q42" s="1569" t="n"/>
-      <c r="R42" s="1569" t="n"/>
-      <c r="S42" s="1569" t="n"/>
+      <c r="O42" s="1611" t="n"/>
+      <c r="P42" s="1614" t="n"/>
+      <c r="Q42" s="1611" t="n"/>
+      <c r="R42" s="1611" t="n"/>
+      <c r="S42" s="1611" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1568" t="n"/>
+      <c r="U42" s="1610" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -7666,57 +7774,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1543" t="inlineStr">
+      <c r="A43" s="1585" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1544" t="inlineStr">
+      <c r="B43" s="1586" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1544" t="inlineStr">
+      <c r="C43" s="1586" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1545" t="n"/>
-      <c r="E43" s="1545" t="n">
+      <c r="D43" s="1587" t="n"/>
+      <c r="E43" s="1587" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1545" t="n">
+      <c r="F43" s="1587" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1545" t="n">
+      <c r="G43" s="1587" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1545" t="n"/>
-      <c r="I43" s="1546" t="n">
+      <c r="H43" s="1587" t="n"/>
+      <c r="I43" s="1588" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1547" t="n"/>
-      <c r="K43" s="1547" t="n"/>
-      <c r="L43" s="1547" t="n"/>
-      <c r="M43" s="1545" t="n"/>
-      <c r="N43" s="1545" t="n"/>
-      <c r="O43" s="1545" t="n">
+      <c r="J43" s="1589" t="n"/>
+      <c r="K43" s="1589" t="n"/>
+      <c r="L43" s="1589" t="n"/>
+      <c r="M43" s="1587" t="n"/>
+      <c r="N43" s="1587" t="n"/>
+      <c r="O43" s="1587" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1548" t="n">
+      <c r="P43" s="1590" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1545" t="n"/>
-      <c r="R43" s="1545" t="n">
+      <c r="Q43" s="1587" t="n"/>
+      <c r="R43" s="1587" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1545" t="n"/>
+      <c r="S43" s="1587" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1544" t="n"/>
+      <c r="U43" s="1586" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -7724,45 +7832,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1573" t="inlineStr">
+      <c r="A44" s="1615" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1574" t="inlineStr">
+      <c r="B44" s="1616" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1574" t="inlineStr">
+      <c r="C44" s="1616" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1575" t="n"/>
-      <c r="E44" s="1575" t="n">
+      <c r="D44" s="1617" t="n"/>
+      <c r="E44" s="1617" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1575" t="n">
+      <c r="F44" s="1617" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1575" t="n"/>
-      <c r="H44" s="1575" t="n"/>
-      <c r="I44" s="1576" t="n"/>
-      <c r="J44" s="1577" t="n"/>
-      <c r="K44" s="1577" t="n"/>
-      <c r="L44" s="1577" t="n"/>
-      <c r="M44" s="1575" t="n"/>
-      <c r="N44" s="1575" t="n"/>
-      <c r="O44" s="1575" t="n"/>
-      <c r="P44" s="1578" t="n"/>
-      <c r="Q44" s="1575" t="n"/>
-      <c r="R44" s="1575" t="n"/>
-      <c r="S44" s="1575" t="n">
+      <c r="G44" s="1617" t="n"/>
+      <c r="H44" s="1617" t="n"/>
+      <c r="I44" s="1618" t="n"/>
+      <c r="J44" s="1619" t="n"/>
+      <c r="K44" s="1619" t="n"/>
+      <c r="L44" s="1619" t="n"/>
+      <c r="M44" s="1617" t="n"/>
+      <c r="N44" s="1617" t="n"/>
+      <c r="O44" s="1617" t="n"/>
+      <c r="P44" s="1620" t="n"/>
+      <c r="Q44" s="1617" t="n"/>
+      <c r="R44" s="1617" t="n"/>
+      <c r="S44" s="1617" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1574" t="inlineStr">
+      <c r="U44" s="1616" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -7774,49 +7882,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1573" t="inlineStr">
+      <c r="A45" s="1615" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1574" t="inlineStr">
+      <c r="B45" s="1616" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1574" t="inlineStr">
+      <c r="C45" s="1616" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1575" t="n"/>
-      <c r="E45" s="1575" t="n"/>
-      <c r="F45" s="1575" t="n"/>
-      <c r="G45" s="1575" t="n"/>
-      <c r="H45" s="1575" t="n">
+      <c r="D45" s="1617" t="n"/>
+      <c r="E45" s="1617" t="n"/>
+      <c r="F45" s="1617" t="n"/>
+      <c r="G45" s="1617" t="n"/>
+      <c r="H45" s="1617" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1576" t="n"/>
-      <c r="J45" s="1577" t="n"/>
-      <c r="K45" s="1577" t="n"/>
-      <c r="L45" s="1577" t="n"/>
-      <c r="M45" s="1575" t="n">
+      <c r="I45" s="1618" t="n"/>
+      <c r="J45" s="1619" t="n"/>
+      <c r="K45" s="1619" t="n"/>
+      <c r="L45" s="1619" t="n"/>
+      <c r="M45" s="1617" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1575" t="n">
+      <c r="N45" s="1617" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1575" t="n"/>
-      <c r="P45" s="1578" t="n"/>
-      <c r="Q45" s="1575" t="n"/>
-      <c r="R45" s="1575" t="n"/>
-      <c r="S45" s="1575" t="n"/>
+      <c r="O45" s="1617" t="n"/>
+      <c r="P45" s="1620" t="n"/>
+      <c r="Q45" s="1617" t="n"/>
+      <c r="R45" s="1617" t="n"/>
+      <c r="S45" s="1617" t="n"/>
       <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1574" t="n"/>
+      <c r="U45" s="1616" t="n"/>
       <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -7824,39 +7932,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1549" t="inlineStr">
+      <c r="A46" s="1591" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B46" s="1550" t="inlineStr">
+      <c r="B46" s="1592" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="C46" s="1550" t="inlineStr">
+      <c r="C46" s="1592" t="inlineStr">
         <is>
           <t>EVENT - Clean</t>
         </is>
       </c>
-      <c r="D46" s="1551" t="n"/>
-      <c r="E46" s="1551" t="n"/>
-      <c r="F46" s="1551" t="n"/>
-      <c r="G46" s="1551" t="n"/>
-      <c r="H46" s="1551" t="n"/>
-      <c r="I46" s="1552" t="n"/>
-      <c r="J46" s="1553" t="n"/>
-      <c r="K46" s="1553" t="n"/>
-      <c r="L46" s="1553" t="n"/>
-      <c r="M46" s="1551" t="n"/>
-      <c r="N46" s="1551" t="n"/>
-      <c r="O46" s="1551" t="n"/>
-      <c r="P46" s="1554" t="n"/>
-      <c r="Q46" s="1551" t="n"/>
-      <c r="R46" s="1551" t="n"/>
-      <c r="S46" s="1551" t="n"/>
+      <c r="D46" s="1593" t="n"/>
+      <c r="E46" s="1593" t="n"/>
+      <c r="F46" s="1593" t="n"/>
+      <c r="G46" s="1593" t="n"/>
+      <c r="H46" s="1593" t="n"/>
+      <c r="I46" s="1594" t="n"/>
+      <c r="J46" s="1595" t="n"/>
+      <c r="K46" s="1595" t="n"/>
+      <c r="L46" s="1595" t="n"/>
+      <c r="M46" s="1593" t="n"/>
+      <c r="N46" s="1593" t="n"/>
+      <c r="O46" s="1593" t="n"/>
+      <c r="P46" s="1596" t="n"/>
+      <c r="Q46" s="1593" t="n"/>
+      <c r="R46" s="1593" t="n"/>
+      <c r="S46" s="1593" t="n"/>
       <c r="T46" s="631" t="n"/>
-      <c r="U46" s="1550" t="n"/>
+      <c r="U46" s="1592" t="n"/>
       <c r="V46" s="632" t="inlineStr">
         <is>
           <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
@@ -7864,51 +7972,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1555" t="inlineStr">
+      <c r="A47" s="1597" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1556" t="inlineStr">
+      <c r="B47" s="1598" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C47" s="1556" t="inlineStr">
+      <c r="C47" s="1598" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D47" s="1557" t="n"/>
-      <c r="E47" s="1557" t="n">
+      <c r="D47" s="1599" t="n"/>
+      <c r="E47" s="1599" t="n">
         <v>16.6</v>
       </c>
-      <c r="F47" s="1557" t="n">
+      <c r="F47" s="1599" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="1557" t="n">
+      <c r="G47" s="1599" t="n">
         <v>4.1</v>
       </c>
-      <c r="H47" s="1557" t="n"/>
-      <c r="I47" s="1558" t="n">
+      <c r="H47" s="1599" t="n"/>
+      <c r="I47" s="1600" t="n">
         <v>0.9</v>
       </c>
-      <c r="J47" s="1559" t="n"/>
-      <c r="K47" s="1559" t="n"/>
-      <c r="L47" s="1559" t="n"/>
-      <c r="M47" s="1557" t="n"/>
-      <c r="N47" s="1557" t="n"/>
-      <c r="O47" s="1557" t="n">
+      <c r="J47" s="1601" t="n"/>
+      <c r="K47" s="1601" t="n"/>
+      <c r="L47" s="1601" t="n"/>
+      <c r="M47" s="1599" t="n"/>
+      <c r="N47" s="1599" t="n"/>
+      <c r="O47" s="1599" t="n">
         <v>13.2</v>
       </c>
-      <c r="P47" s="1560" t="n">
+      <c r="P47" s="1602" t="n">
         <v>0</v>
       </c>
-      <c r="Q47" s="1557" t="n"/>
-      <c r="R47" s="1557" t="n">
+      <c r="Q47" s="1599" t="n"/>
+      <c r="R47" s="1599" t="n">
         <v>84.5</v>
       </c>
-      <c r="S47" s="1557" t="n">
+      <c r="S47" s="1599" t="n">
         <v>11.8</v>
       </c>
       <c r="T47" s="813" t="inlineStr">
@@ -7916,7 +8024,7 @@
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1556" t="inlineStr">
+      <c r="U47" s="1598" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
@@ -7928,49 +8036,49 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1567" t="inlineStr">
+      <c r="A48" s="1609" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B48" s="1568" t="inlineStr">
+      <c r="B48" s="1610" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C48" s="1568" t="inlineStr">
+      <c r="C48" s="1610" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D48" s="1569" t="n"/>
-      <c r="E48" s="1569" t="n"/>
-      <c r="F48" s="1569" t="n"/>
-      <c r="G48" s="1569" t="n"/>
-      <c r="H48" s="1569" t="n">
+      <c r="D48" s="1611" t="n"/>
+      <c r="E48" s="1611" t="n"/>
+      <c r="F48" s="1611" t="n"/>
+      <c r="G48" s="1611" t="n"/>
+      <c r="H48" s="1611" t="n">
         <v>15.1</v>
       </c>
-      <c r="I48" s="1570" t="n"/>
-      <c r="J48" s="1571" t="n"/>
-      <c r="K48" s="1571" t="n"/>
-      <c r="L48" s="1571" t="n"/>
-      <c r="M48" s="1569" t="n">
+      <c r="I48" s="1612" t="n"/>
+      <c r="J48" s="1613" t="n"/>
+      <c r="K48" s="1613" t="n"/>
+      <c r="L48" s="1613" t="n"/>
+      <c r="M48" s="1611" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="1569" t="n">
+      <c r="N48" s="1611" t="n">
         <v>20</v>
       </c>
-      <c r="O48" s="1569" t="n"/>
-      <c r="P48" s="1572" t="n"/>
-      <c r="Q48" s="1569" t="n"/>
-      <c r="R48" s="1569" t="n"/>
-      <c r="S48" s="1569" t="n"/>
+      <c r="O48" s="1611" t="n"/>
+      <c r="P48" s="1614" t="n"/>
+      <c r="Q48" s="1611" t="n"/>
+      <c r="R48" s="1611" t="n"/>
+      <c r="S48" s="1611" t="n"/>
       <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U48" s="1568" t="n"/>
+      <c r="U48" s="1610" t="n"/>
       <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
@@ -7978,51 +8086,51 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1543" t="inlineStr">
+      <c r="A49" s="1585" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B49" s="1544" t="inlineStr">
+      <c r="B49" s="1586" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C49" s="1544" t="inlineStr">
+      <c r="C49" s="1586" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D49" s="1545" t="n"/>
-      <c r="E49" s="1545" t="n">
+      <c r="D49" s="1587" t="n"/>
+      <c r="E49" s="1587" t="n">
         <v>16.8</v>
       </c>
-      <c r="F49" s="1545" t="n">
+      <c r="F49" s="1587" t="n">
         <v>0.2</v>
       </c>
-      <c r="G49" s="1545" t="n">
+      <c r="G49" s="1587" t="n">
         <v>3.3</v>
       </c>
-      <c r="H49" s="1545" t="n"/>
-      <c r="I49" s="1546" t="n">
+      <c r="H49" s="1587" t="n"/>
+      <c r="I49" s="1588" t="n">
         <v>1.7</v>
       </c>
-      <c r="J49" s="1547" t="n"/>
-      <c r="K49" s="1547" t="n"/>
-      <c r="L49" s="1547" t="n"/>
-      <c r="M49" s="1545" t="n"/>
-      <c r="N49" s="1545" t="n"/>
-      <c r="O49" s="1545" t="n">
+      <c r="J49" s="1589" t="n"/>
+      <c r="K49" s="1589" t="n"/>
+      <c r="L49" s="1589" t="n"/>
+      <c r="M49" s="1587" t="n"/>
+      <c r="N49" s="1587" t="n"/>
+      <c r="O49" s="1587" t="n">
         <v>13</v>
       </c>
-      <c r="P49" s="1548" t="n">
+      <c r="P49" s="1590" t="n">
         <v>0.87</v>
       </c>
-      <c r="Q49" s="1545" t="n"/>
-      <c r="R49" s="1545" t="n">
+      <c r="Q49" s="1587" t="n"/>
+      <c r="R49" s="1587" t="n">
         <v>86</v>
       </c>
-      <c r="S49" s="1545" t="n">
+      <c r="S49" s="1587" t="n">
         <v>11.65</v>
       </c>
       <c r="T49" s="624" t="inlineStr">
@@ -8030,7 +8138,7 @@
           <t>Clear now, 88F, 67% RH; sun so far 6.4h of 7h daylight (91%); today high 90F, 0.87in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U49" s="1544" t="inlineStr">
+      <c r="U49" s="1586" t="inlineStr">
         <is>
           <t>2026-07-04_1.jpeg;2026-07-04_2.jpeg;2026-07-04_3.jpeg;2026-07-04_4.jpeg</t>
         </is>
@@ -8042,49 +8150,49 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1549" t="inlineStr">
+      <c r="A50" s="1591" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B50" s="1550" t="inlineStr">
+      <c r="B50" s="1592" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C50" s="1550" t="inlineStr">
+      <c r="C50" s="1592" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D50" s="1551" t="n"/>
-      <c r="E50" s="1551" t="n"/>
-      <c r="F50" s="1551" t="n"/>
-      <c r="G50" s="1551" t="n"/>
-      <c r="H50" s="1551" t="n">
+      <c r="D50" s="1593" t="n"/>
+      <c r="E50" s="1593" t="n"/>
+      <c r="F50" s="1593" t="n"/>
+      <c r="G50" s="1593" t="n"/>
+      <c r="H50" s="1593" t="n">
         <v>14.6</v>
       </c>
-      <c r="I50" s="1552" t="n"/>
-      <c r="J50" s="1553" t="n"/>
-      <c r="K50" s="1553" t="n"/>
-      <c r="L50" s="1553" t="n"/>
-      <c r="M50" s="1551" t="n">
+      <c r="I50" s="1594" t="n"/>
+      <c r="J50" s="1595" t="n"/>
+      <c r="K50" s="1595" t="n"/>
+      <c r="L50" s="1595" t="n"/>
+      <c r="M50" s="1593" t="n">
         <v>0.5</v>
       </c>
-      <c r="N50" s="1551" t="n">
+      <c r="N50" s="1593" t="n">
         <v>20.5</v>
       </c>
-      <c r="O50" s="1551" t="n"/>
-      <c r="P50" s="1554" t="n"/>
-      <c r="Q50" s="1551" t="n"/>
-      <c r="R50" s="1551" t="n"/>
-      <c r="S50" s="1551" t="n"/>
+      <c r="O50" s="1593" t="n"/>
+      <c r="P50" s="1596" t="n"/>
+      <c r="Q50" s="1593" t="n"/>
+      <c r="R50" s="1593" t="n"/>
+      <c r="S50" s="1593" t="n"/>
       <c r="T50" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny day (high 90F, water 86F); storm forecast overnight</t>
         </is>
       </c>
-      <c r="U50" s="1550" t="n"/>
+      <c r="U50" s="1592" t="n"/>
       <c r="V50" s="632" t="inlineStr">
         <is>
           <t>0.5 gal added 7:40 PM. PARTY PRE-LOAD (Sun 7/5 1PM picnic): deliberately HALF the usual dose -- FC already high at 16.8, and John didn't want to overshoot into the high teens for guests. Sized on the retuned model (l24_hot_sunny now 4.0). Model projects ~14.6 next noon, BUT this is a known weather-mismatch case: model keys L24 off today's hot/sunny weather, while the actual loss window is a storm overnight (no UV) + cooler/cloudy Sun morning -&gt; real loss will be LOWER, so FC likely lands ~15-16 at the party (comfortable top-of-band, cushion for bather load, not overboard). =&gt; If tomorrow's noon comes in ABOVE 14.6, that's the weather mismatch, NOT the freshly-retuned constant; don't chase it. Plan: dose back up Sun evening after the crowd's out (expect a bather-load FC drop). Season total 20.5 gal. PHOTOS(4): water clear/healthy blue, bottom fully visible, no cloudiness/algae; yesterday's surface debris now gone (tracks with CC clearing to 0.2); liner step close-up normal speckled blue, no rust/stain progression. Ruler photo documents the ~11.65 cm level.</t>
@@ -8092,47 +8200,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1555" t="inlineStr">
+      <c r="A51" s="1597" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B51" s="1556" t="inlineStr">
+      <c r="B51" s="1598" t="inlineStr">
         <is>
           <t>07:45</t>
         </is>
       </c>
-      <c r="C51" s="1556" t="inlineStr">
+      <c r="C51" s="1598" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D51" s="1557" t="n"/>
-      <c r="E51" s="1557" t="n">
+      <c r="D51" s="1599" t="n"/>
+      <c r="E51" s="1599" t="n">
         <v>16</v>
       </c>
-      <c r="F51" s="1557" t="n">
+      <c r="F51" s="1599" t="n">
         <v>0.5</v>
       </c>
-      <c r="G51" s="1557" t="n"/>
-      <c r="H51" s="1557" t="n"/>
-      <c r="I51" s="1558" t="n">
+      <c r="G51" s="1599" t="n"/>
+      <c r="H51" s="1599" t="n"/>
+      <c r="I51" s="1600" t="n">
         <v>1.4</v>
       </c>
-      <c r="J51" s="1559" t="n"/>
-      <c r="K51" s="1559" t="n"/>
-      <c r="L51" s="1559" t="n"/>
-      <c r="M51" s="1557" t="n"/>
-      <c r="N51" s="1557" t="n"/>
-      <c r="O51" s="1557" t="n"/>
-      <c r="P51" s="1560" t="n">
+      <c r="J51" s="1601" t="n"/>
+      <c r="K51" s="1601" t="n"/>
+      <c r="L51" s="1601" t="n"/>
+      <c r="M51" s="1599" t="n"/>
+      <c r="N51" s="1599" t="n"/>
+      <c r="O51" s="1599" t="n"/>
+      <c r="P51" s="1602" t="n">
         <v>0.04</v>
       </c>
-      <c r="Q51" s="1557" t="n"/>
-      <c r="R51" s="1557" t="n">
+      <c r="Q51" s="1599" t="n"/>
+      <c r="R51" s="1599" t="n">
         <v>84</v>
       </c>
-      <c r="S51" s="1557" t="n">
+      <c r="S51" s="1599" t="n">
         <v>13.9</v>
       </c>
       <c r="T51" s="813" t="inlineStr">
@@ -8140,7 +8248,7 @@
           <t>Overcast now, 75F, 90% RH; sun so far 0.0h of 3h daylight (0%); today high 75F, 0.04in precip, UV max 6.5</t>
         </is>
       </c>
-      <c r="U51" s="1556" t="inlineStr">
+      <c r="U51" s="1598" t="inlineStr">
         <is>
           <t>2026-07-05_2.jpeg</t>
         </is>
@@ -8152,41 +8260,41 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1561" t="inlineStr">
+      <c r="A52" s="1603" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B52" s="1562" t="inlineStr">
+      <c r="B52" s="1604" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C52" s="1562" t="inlineStr">
+      <c r="C52" s="1604" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D52" s="1563" t="n"/>
-      <c r="E52" s="1563" t="n">
+      <c r="D52" s="1605" t="n"/>
+      <c r="E52" s="1605" t="n">
         <v>14.8</v>
       </c>
-      <c r="F52" s="1563" t="n">
+      <c r="F52" s="1605" t="n">
         <v>0.3</v>
       </c>
-      <c r="G52" s="1563" t="n"/>
-      <c r="H52" s="1563" t="n"/>
-      <c r="I52" s="1564" t="n"/>
-      <c r="J52" s="1565" t="n"/>
-      <c r="K52" s="1565" t="n"/>
-      <c r="L52" s="1565" t="n"/>
-      <c r="M52" s="1563" t="n"/>
-      <c r="N52" s="1563" t="n"/>
-      <c r="O52" s="1563" t="n"/>
-      <c r="P52" s="1566" t="n"/>
-      <c r="Q52" s="1563" t="n"/>
-      <c r="R52" s="1563" t="n"/>
-      <c r="S52" s="1563" t="n">
+      <c r="G52" s="1605" t="n"/>
+      <c r="H52" s="1605" t="n"/>
+      <c r="I52" s="1606" t="n"/>
+      <c r="J52" s="1607" t="n"/>
+      <c r="K52" s="1607" t="n"/>
+      <c r="L52" s="1607" t="n"/>
+      <c r="M52" s="1605" t="n"/>
+      <c r="N52" s="1605" t="n"/>
+      <c r="O52" s="1605" t="n"/>
+      <c r="P52" s="1608" t="n"/>
+      <c r="Q52" s="1605" t="n"/>
+      <c r="R52" s="1605" t="n"/>
+      <c r="S52" s="1605" t="n">
         <v>13.6</v>
       </c>
       <c r="T52" s="820" t="inlineStr">
@@ -8194,7 +8302,7 @@
           <t>Overcast now, 72F, 76% RH; sun so far 8.4h of 13h daylight (65%); today high 80F, 0.00in precip, UV max 6.0</t>
         </is>
       </c>
-      <c r="U52" s="1562" t="inlineStr">
+      <c r="U52" s="1604" t="inlineStr">
         <is>
           <t>2026-07-05_1.jpeg;2026-07-05_3.jpeg</t>
         </is>
@@ -8206,49 +8314,49 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1567" t="inlineStr">
+      <c r="A53" s="1609" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B53" s="1568" t="inlineStr">
+      <c r="B53" s="1610" t="inlineStr">
         <is>
           <t>19:25</t>
         </is>
       </c>
-      <c r="C53" s="1568" t="inlineStr">
+      <c r="C53" s="1610" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D53" s="1569" t="n"/>
-      <c r="E53" s="1569" t="n"/>
-      <c r="F53" s="1569" t="n"/>
-      <c r="G53" s="1569" t="n"/>
-      <c r="H53" s="1569" t="n">
+      <c r="D53" s="1611" t="n"/>
+      <c r="E53" s="1611" t="n"/>
+      <c r="F53" s="1611" t="n"/>
+      <c r="G53" s="1611" t="n"/>
+      <c r="H53" s="1611" t="n">
         <v>15.1</v>
       </c>
-      <c r="I53" s="1570" t="n"/>
-      <c r="J53" s="1571" t="n"/>
-      <c r="K53" s="1571" t="n"/>
-      <c r="L53" s="1571" t="n"/>
-      <c r="M53" s="1569" t="n">
+      <c r="I53" s="1612" t="n"/>
+      <c r="J53" s="1613" t="n"/>
+      <c r="K53" s="1613" t="n"/>
+      <c r="L53" s="1613" t="n"/>
+      <c r="M53" s="1611" t="n">
         <v>0.5</v>
       </c>
-      <c r="N53" s="1569" t="n">
+      <c r="N53" s="1611" t="n">
         <v>21</v>
       </c>
-      <c r="O53" s="1569" t="n"/>
-      <c r="P53" s="1572" t="n"/>
-      <c r="Q53" s="1569" t="n"/>
-      <c r="R53" s="1569" t="n"/>
-      <c r="S53" s="1569" t="n"/>
+      <c r="O53" s="1611" t="n"/>
+      <c r="P53" s="1614" t="n"/>
+      <c r="Q53" s="1611" t="n"/>
+      <c r="R53" s="1611" t="n"/>
+      <c r="S53" s="1611" t="n"/>
       <c r="T53" s="827" t="inlineStr">
         <is>
           <t>Cleared to partly sunny (8.4 sun hrs, high 80F, water 84F); all-day rain forecast Mon 7/6</t>
         </is>
       </c>
-      <c r="U53" s="1568" t="n"/>
+      <c r="U53" s="1610" t="n"/>
       <c r="V53" s="828" t="inlineStr">
         <is>
           <t>0.5 gal added 7:25 PM (post-party recovery dose). Sized on TOMORROW's rainy forecast (the real loss window: overcast/wet 7/6, ~0.9in rain, low UV) not today's sun -&gt; projects ~15.1 at Mon noon. Party went great (FC held 16.0-&gt;14.8, CC dropped 0.5-&gt;0.3). Season total 21.0 gal. This is the first prediction that deliberately used the next-day forecast for L24 instead of the model's default (today's weather as proxy) -- if it lands near 15.1 tomorrow, that validates feeding the forecast on weather-change days.</t>
@@ -8256,64 +8364,158 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1579" t="inlineStr">
+      <c r="A54" s="1585" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B54" s="1580" t="inlineStr">
+      <c r="B54" s="1586" t="inlineStr">
         <is>
           <t>11:40</t>
         </is>
       </c>
-      <c r="C54" s="1580" t="inlineStr">
+      <c r="C54" s="1586" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D54" s="1581" t="n"/>
-      <c r="E54" s="1581" t="n">
+      <c r="D54" s="1587" t="n"/>
+      <c r="E54" s="1587" t="n">
         <v>13.8</v>
       </c>
-      <c r="F54" s="1581" t="n">
+      <c r="F54" s="1587" t="n">
         <v>0.2</v>
       </c>
-      <c r="G54" s="1581" t="n"/>
-      <c r="H54" s="1581" t="n"/>
-      <c r="I54" s="1582" t="n">
+      <c r="G54" s="1587" t="n"/>
+      <c r="H54" s="1587" t="n"/>
+      <c r="I54" s="1588" t="n">
         <v>-1.3</v>
       </c>
-      <c r="J54" s="1583" t="n"/>
-      <c r="K54" s="1583" t="n"/>
-      <c r="L54" s="1583" t="n"/>
-      <c r="M54" s="1581" t="n"/>
-      <c r="N54" s="1581" t="n"/>
-      <c r="O54" s="1581" t="n">
+      <c r="J54" s="1589" t="n"/>
+      <c r="K54" s="1589" t="n"/>
+      <c r="L54" s="1589" t="n"/>
+      <c r="M54" s="1587" t="n"/>
+      <c r="N54" s="1587" t="n"/>
+      <c r="O54" s="1587" t="n">
         <v>0</v>
       </c>
-      <c r="P54" s="1584" t="n">
+      <c r="P54" s="1590" t="n">
         <v>2</v>
       </c>
-      <c r="Q54" s="1581" t="n"/>
-      <c r="R54" s="1581" t="n">
+      <c r="Q54" s="1587" t="n"/>
+      <c r="R54" s="1587" t="n">
         <v>81</v>
       </c>
-      <c r="S54" s="1581" t="n">
+      <c r="S54" s="1587" t="n">
         <v>15.1</v>
       </c>
-      <c r="T54" s="1047" t="inlineStr">
+      <c r="T54" s="624" t="inlineStr">
         <is>
           <t>Light rain now, 65F, 93% RH; sun so far 0.0h of 6h daylight (0%); today high 68F, 2.00in precip, UV max 0.5</t>
         </is>
       </c>
-      <c r="U54" s="1580" t="inlineStr">
+      <c r="U54" s="1586" t="inlineStr">
         <is>
           <t>2026-07-06_1.jpeg</t>
         </is>
       </c>
-      <c r="V54" s="1048" t="inlineStr">
-        <is>
-          <t>25mL x0.2. FC 13.8, CC 0.2 -- in band, healthy. [CORRECTED same day: earlier note wrongly said OVERFLOWING -- it is NOT. Pool has 6+ in of freeboard. The weather feed 2.00in is the DAY forecast total, not fallen-yet; only ~0.6in has actually fallen this AM, which matches the 0.6in / 1.5cm level rise 13.6-&gt;15.1. No water over the edge.] FIRST NEGATIVE prediction error (-1.3): actual 13.8 vs the 7/5 dose 15.1 (rain bucket L24=1.5) -&gt; model UNDER-estimated loss. Likely cause: STORM since last night (not calm rain) washes organic load in (debris/runoff/nitrogen) that consumes FC -- real loss ~2.75 from the post-dose ~16.5 vs the calm-rain 1.5 estimate. Dilution only a minor part (~0.15 ppm from 0.6in add). The rain bucket is tuned for drizzle, not a storm; FIRST storm forward point -&gt; note storms lose more, but do NOT retune off one point. CYA: modest rain dilution (~0.9%) nudges it down ~1-2 ppm (NOT the big overflow-driven drop I wrongly claimed). fc_loss BLANK: off-cadence prior test (7/5 had AM+PM) + dilution -&gt; not a clean noon-to-noon value. Level 15.1 (well below overflow). Water temp 81. DOSE REC revised: a modest 0.5 gal tonight is reasonable -- the storm is actively eating FC and there is no overflow to waste it, so hold the buffer above floor; keep it small (John low on chlorine, refill 1-2 days out).</t>
+      <c r="V54" s="625" t="inlineStr">
+        <is>
+          <t>25mL x0.2. FC 13.8, CC 0.2 -- in band, healthy. [CORRECTED same day: earlier note wrongly said OVERFLOWING -- it is NOT. Pool has 6+ in of freeboard. The weather feed 2.00in is the DAY forecast total, not fallen-yet; only ~0.6in has actually fallen this AM, which matches the 0.6in / 1.5cm level rise 13.6-&gt;15.1. No water over the edge.] FIRST NEGATIVE prediction error (-1.3): actual 13.8 vs the 7/5 dose 15.1 (rain bucket L24=1.5) -&gt; model UNDER-estimated loss. Likely cause: STORM since last night (not calm rain) washes organic load in (debris/runoff/nitrogen) that consumes FC -- real loss ~2.75 from the post-dose ~16.5 vs the calm-rain 1.5 estimate. Dilution only a minor part (~0.15 ppm from 0.6in add). The rain bucket is tuned for drizzle, not a storm; FIRST storm forward point -&gt; note storms lose more, but do NOT retune off one point. CYA: modest rain dilution (~0.9%) nudges it down ~1-2 ppm (NOT the big overflow-driven drop I wrongly claimed). fc_loss BLANK: off-cadence prior test (7/5 had AM+PM) + dilution -&gt; not a clean noon-to-noon value. Level 15.1 (well below overflow). Water temp 81. DOSE REC revised: a modest 0.5 gal tonight is reasonable -- the storm is actively eating FC and there is no overflow to waste it, so hold the buffer above floor; keep it small (John was low on TEST REAGENTS (arrived 7/6), NOT chlorine -- corrected).</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="1615" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B55" s="1616" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C55" s="1616" t="inlineStr">
+        <is>
+          <t>EVENT - Waste</t>
+        </is>
+      </c>
+      <c r="D55" s="1617" t="n"/>
+      <c r="E55" s="1617" t="n"/>
+      <c r="F55" s="1617" t="n"/>
+      <c r="G55" s="1617" t="n"/>
+      <c r="H55" s="1617" t="n"/>
+      <c r="I55" s="1618" t="n"/>
+      <c r="J55" s="1619" t="n"/>
+      <c r="K55" s="1619" t="n"/>
+      <c r="L55" s="1619" t="n"/>
+      <c r="M55" s="1617" t="n"/>
+      <c r="N55" s="1617" t="n"/>
+      <c r="O55" s="1617" t="n"/>
+      <c r="P55" s="1620" t="n"/>
+      <c r="Q55" s="1617" t="n"/>
+      <c r="R55" s="1617" t="n"/>
+      <c r="S55" s="1617" t="n"/>
+      <c r="T55" s="659" t="n"/>
+      <c r="U55" s="1616" t="inlineStr">
+        <is>
+          <t>2026-07-06_2.jpeg;2026-07-06_3.jpeg</t>
+        </is>
+      </c>
+      <c r="V55" s="660" t="inlineStr">
+        <is>
+          <t>Pumped to WASTE (multiport waste port, bypassing the D.E. filter) to lower the storm-raised level. The all-day rain had pushed the water ABOVE the ruler top (~16-17 cm, off-scale); pumped it back down to a readable 15.1 cm. Ran the pump while it was still raining -- pump-out (~50 GPM = ~3000 gal/hr) hugely outpaces rain-in (~100-300 gal/hr), so the level dropped steadily despite the rain. ESTIMATED WATER REMOVED ~2,000 gal (VERY ROUGH -- from oblique ruler/liner photos 2026-07-06_2/_3; drop from ~top-of-blue-liner high point down to 15.1 looks like ~4 in, x ~500 gal/in; could easily be 1,500-3,000. Pump-runtime x ~50 GPM would pin it better -- John didn't report the minutes). Consistent with the passive CYA-lowering plan: removes some high-CYA pool water, and rain is refilling it (no well stress). More rain forecast Tue 7/7 -&gt; may need to repeat; drew it toward the low end to leave headroom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="1591" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B56" s="1592" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C56" s="1592" t="inlineStr">
+        <is>
+          <t>DOSE</t>
+        </is>
+      </c>
+      <c r="D56" s="1593" t="n"/>
+      <c r="E56" s="1593" t="n"/>
+      <c r="F56" s="1593" t="n"/>
+      <c r="G56" s="1593" t="n"/>
+      <c r="H56" s="1593" t="n">
+        <v>14</v>
+      </c>
+      <c r="I56" s="1594" t="n"/>
+      <c r="J56" s="1595" t="n"/>
+      <c r="K56" s="1595" t="n"/>
+      <c r="L56" s="1595" t="n"/>
+      <c r="M56" s="1593" t="n">
+        <v>1</v>
+      </c>
+      <c r="N56" s="1593" t="n">
+        <v>22</v>
+      </c>
+      <c r="O56" s="1593" t="n"/>
+      <c r="P56" s="1596" t="n"/>
+      <c r="Q56" s="1593" t="n"/>
+      <c r="R56" s="1593" t="n"/>
+      <c r="S56" s="1593" t="n"/>
+      <c r="T56" s="631" t="inlineStr">
+        <is>
+          <t>Rain all day (2.00in total), overcast, 65-68F; more rain Tue</t>
+        </is>
+      </c>
+      <c r="U56" s="1592" t="n"/>
+      <c r="V56" s="632" t="inlineStr">
+        <is>
+          <t>1.0 gal added 7:30 PM, AFTER the pump-to-waste (correct order -- don't chlorinate water you're about to pump out). FIRST dose on the recalibrated buckets (rain L24 now 2.5 vs old 1.5). CORRECTION carried in: John is NOT low on chlorine -- he was low on TEST REAGENTS, which arrived today -- so this is the full 1 gal (not the 0.5 I'd wrongly trimmed for 'conservation'). Base FC ~13 est (noon 13.8 minus the bit of FC removed by the pump-out; not re-tested), + 1gal x3.5 - 2.5 rain loss -&gt; pred ~14.0 at Tue noon. Prediction is confounded this round (pump perturbation + no post-empty FC test) -&gt; tomorrow's error will be noisy, don't read too much into it for bucket validation. Season total 22.0 gal.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refine 7/6 waste estimate with 28-min runtime; calibrate pump to ~60 GPM (~8 min/in)
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1621">
+  <cellXfs count="1657">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -5282,6 +5282,114 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -5828,35 +5936,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1585" t="inlineStr">
+      <c r="A3" s="1621" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1586" t="n"/>
-      <c r="C3" s="1586" t="inlineStr">
+      <c r="B3" s="1622" t="n"/>
+      <c r="C3" s="1622" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1587" t="n"/>
-      <c r="E3" s="1587" t="n"/>
-      <c r="F3" s="1587" t="n"/>
-      <c r="G3" s="1587" t="n"/>
-      <c r="H3" s="1587" t="n"/>
-      <c r="I3" s="1588" t="n"/>
-      <c r="J3" s="1589" t="n"/>
-      <c r="K3" s="1589" t="n"/>
-      <c r="L3" s="1589" t="n"/>
-      <c r="M3" s="1587" t="n"/>
-      <c r="N3" s="1587" t="n"/>
-      <c r="O3" s="1587" t="n"/>
-      <c r="P3" s="1590" t="n"/>
-      <c r="Q3" s="1587" t="n"/>
-      <c r="R3" s="1587" t="n"/>
-      <c r="S3" s="1587" t="n"/>
+      <c r="D3" s="1623" t="n"/>
+      <c r="E3" s="1623" t="n"/>
+      <c r="F3" s="1623" t="n"/>
+      <c r="G3" s="1623" t="n"/>
+      <c r="H3" s="1623" t="n"/>
+      <c r="I3" s="1624" t="n"/>
+      <c r="J3" s="1625" t="n"/>
+      <c r="K3" s="1625" t="n"/>
+      <c r="L3" s="1625" t="n"/>
+      <c r="M3" s="1623" t="n"/>
+      <c r="N3" s="1623" t="n"/>
+      <c r="O3" s="1623" t="n"/>
+      <c r="P3" s="1626" t="n"/>
+      <c r="Q3" s="1623" t="n"/>
+      <c r="R3" s="1623" t="n"/>
+      <c r="S3" s="1623" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1586" t="n"/>
+      <c r="U3" s="1622" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -5864,43 +5972,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1591" t="inlineStr">
+      <c r="A4" s="1627" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1592" t="inlineStr">
+      <c r="B4" s="1628" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1592" t="inlineStr">
+      <c r="C4" s="1628" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1593" t="n"/>
-      <c r="E4" s="1593" t="n"/>
-      <c r="F4" s="1593" t="n"/>
-      <c r="G4" s="1593" t="n"/>
-      <c r="H4" s="1593" t="n"/>
-      <c r="I4" s="1594" t="n"/>
-      <c r="J4" s="1595" t="n"/>
-      <c r="K4" s="1595" t="n"/>
-      <c r="L4" s="1595" t="n"/>
-      <c r="M4" s="1593" t="n">
+      <c r="D4" s="1629" t="n"/>
+      <c r="E4" s="1629" t="n"/>
+      <c r="F4" s="1629" t="n"/>
+      <c r="G4" s="1629" t="n"/>
+      <c r="H4" s="1629" t="n"/>
+      <c r="I4" s="1630" t="n"/>
+      <c r="J4" s="1631" t="n"/>
+      <c r="K4" s="1631" t="n"/>
+      <c r="L4" s="1631" t="n"/>
+      <c r="M4" s="1629" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1593" t="n">
+      <c r="N4" s="1629" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1593" t="n"/>
-      <c r="P4" s="1596" t="n"/>
-      <c r="Q4" s="1593" t="n"/>
-      <c r="R4" s="1593" t="n"/>
-      <c r="S4" s="1593" t="n"/>
+      <c r="O4" s="1629" t="n"/>
+      <c r="P4" s="1632" t="n"/>
+      <c r="Q4" s="1629" t="n"/>
+      <c r="R4" s="1629" t="n"/>
+      <c r="S4" s="1629" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1592" t="n"/>
+      <c r="U4" s="1628" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -5908,57 +6016,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1597" t="inlineStr">
+      <c r="A5" s="1633" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1598" t="inlineStr">
+      <c r="B5" s="1634" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1598" t="inlineStr">
+      <c r="C5" s="1634" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1599" t="n">
+      <c r="D5" s="1635" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1599" t="n">
+      <c r="E5" s="1635" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1599" t="n">
+      <c r="F5" s="1635" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1599" t="n"/>
-      <c r="H5" s="1599" t="n"/>
-      <c r="I5" s="1600" t="n"/>
-      <c r="J5" s="1601" t="n">
+      <c r="G5" s="1635" t="n"/>
+      <c r="H5" s="1635" t="n"/>
+      <c r="I5" s="1636" t="n"/>
+      <c r="J5" s="1637" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1601" t="n">
+      <c r="K5" s="1637" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1601" t="inlineStr">
+      <c r="L5" s="1637" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1599" t="n"/>
-      <c r="N5" s="1599" t="n"/>
-      <c r="O5" s="1599" t="n">
+      <c r="M5" s="1635" t="n"/>
+      <c r="N5" s="1635" t="n"/>
+      <c r="O5" s="1635" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1602" t="n">
+      <c r="P5" s="1638" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1599" t="n"/>
-      <c r="R5" s="1599" t="n"/>
-      <c r="S5" s="1599" t="n"/>
+      <c r="Q5" s="1635" t="n"/>
+      <c r="R5" s="1635" t="n"/>
+      <c r="S5" s="1635" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1598" t="n"/>
+      <c r="U5" s="1634" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -5966,43 +6074,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1603" t="inlineStr">
+      <c r="A6" s="1639" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1604" t="inlineStr">
+      <c r="B6" s="1640" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1604" t="inlineStr">
+      <c r="C6" s="1640" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1605" t="n"/>
-      <c r="E6" s="1605" t="n"/>
-      <c r="F6" s="1605" t="n"/>
-      <c r="G6" s="1605" t="n"/>
-      <c r="H6" s="1605" t="n"/>
-      <c r="I6" s="1606" t="n"/>
-      <c r="J6" s="1607" t="n"/>
-      <c r="K6" s="1607" t="n"/>
-      <c r="L6" s="1607" t="n"/>
-      <c r="M6" s="1605" t="n">
+      <c r="D6" s="1641" t="n"/>
+      <c r="E6" s="1641" t="n"/>
+      <c r="F6" s="1641" t="n"/>
+      <c r="G6" s="1641" t="n"/>
+      <c r="H6" s="1641" t="n"/>
+      <c r="I6" s="1642" t="n"/>
+      <c r="J6" s="1643" t="n"/>
+      <c r="K6" s="1643" t="n"/>
+      <c r="L6" s="1643" t="n"/>
+      <c r="M6" s="1641" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1605" t="n">
+      <c r="N6" s="1641" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1605" t="n"/>
-      <c r="P6" s="1608" t="n"/>
-      <c r="Q6" s="1605" t="n"/>
-      <c r="R6" s="1605" t="n"/>
-      <c r="S6" s="1605" t="n"/>
+      <c r="O6" s="1641" t="n"/>
+      <c r="P6" s="1644" t="n"/>
+      <c r="Q6" s="1641" t="n"/>
+      <c r="R6" s="1641" t="n"/>
+      <c r="S6" s="1641" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1604" t="n"/>
+      <c r="U6" s="1640" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -6010,39 +6118,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1609" t="inlineStr">
+      <c r="A7" s="1645" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1610" t="inlineStr">
+      <c r="B7" s="1646" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1610" t="inlineStr">
+      <c r="C7" s="1646" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1611" t="n"/>
-      <c r="E7" s="1611" t="n"/>
-      <c r="F7" s="1611" t="n"/>
-      <c r="G7" s="1611" t="n"/>
-      <c r="H7" s="1611" t="n"/>
-      <c r="I7" s="1612" t="n"/>
-      <c r="J7" s="1613" t="n"/>
-      <c r="K7" s="1613" t="n"/>
-      <c r="L7" s="1613" t="n"/>
-      <c r="M7" s="1611" t="n"/>
-      <c r="N7" s="1611" t="n"/>
-      <c r="O7" s="1611" t="n"/>
-      <c r="P7" s="1614" t="n"/>
-      <c r="Q7" s="1611" t="n"/>
-      <c r="R7" s="1611" t="n"/>
-      <c r="S7" s="1611" t="n"/>
+      <c r="D7" s="1647" t="n"/>
+      <c r="E7" s="1647" t="n"/>
+      <c r="F7" s="1647" t="n"/>
+      <c r="G7" s="1647" t="n"/>
+      <c r="H7" s="1647" t="n"/>
+      <c r="I7" s="1648" t="n"/>
+      <c r="J7" s="1649" t="n"/>
+      <c r="K7" s="1649" t="n"/>
+      <c r="L7" s="1649" t="n"/>
+      <c r="M7" s="1647" t="n"/>
+      <c r="N7" s="1647" t="n"/>
+      <c r="O7" s="1647" t="n"/>
+      <c r="P7" s="1650" t="n"/>
+      <c r="Q7" s="1647" t="n"/>
+      <c r="R7" s="1647" t="n"/>
+      <c r="S7" s="1647" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1610" t="n"/>
+      <c r="U7" s="1646" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -6050,39 +6158,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1585" t="inlineStr">
+      <c r="A8" s="1621" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1586" t="inlineStr">
+      <c r="B8" s="1622" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1586" t="inlineStr">
+      <c r="C8" s="1622" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1587" t="n"/>
-      <c r="E8" s="1587" t="n"/>
-      <c r="F8" s="1587" t="n"/>
-      <c r="G8" s="1587" t="n"/>
-      <c r="H8" s="1587" t="n"/>
-      <c r="I8" s="1588" t="n"/>
-      <c r="J8" s="1589" t="n"/>
-      <c r="K8" s="1589" t="n"/>
-      <c r="L8" s="1589" t="n"/>
-      <c r="M8" s="1587" t="n"/>
-      <c r="N8" s="1587" t="n"/>
-      <c r="O8" s="1587" t="n"/>
-      <c r="P8" s="1590" t="n"/>
-      <c r="Q8" s="1587" t="n"/>
-      <c r="R8" s="1587" t="n"/>
-      <c r="S8" s="1587" t="n"/>
+      <c r="D8" s="1623" t="n"/>
+      <c r="E8" s="1623" t="n"/>
+      <c r="F8" s="1623" t="n"/>
+      <c r="G8" s="1623" t="n"/>
+      <c r="H8" s="1623" t="n"/>
+      <c r="I8" s="1624" t="n"/>
+      <c r="J8" s="1625" t="n"/>
+      <c r="K8" s="1625" t="n"/>
+      <c r="L8" s="1625" t="n"/>
+      <c r="M8" s="1623" t="n"/>
+      <c r="N8" s="1623" t="n"/>
+      <c r="O8" s="1623" t="n"/>
+      <c r="P8" s="1626" t="n"/>
+      <c r="Q8" s="1623" t="n"/>
+      <c r="R8" s="1623" t="n"/>
+      <c r="S8" s="1623" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1586" t="n"/>
+      <c r="U8" s="1622" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -6090,63 +6198,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1615" t="inlineStr">
+      <c r="A9" s="1651" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1616" t="inlineStr">
+      <c r="B9" s="1652" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1616" t="inlineStr">
+      <c r="C9" s="1652" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1617" t="n">
+      <c r="D9" s="1653" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1617" t="n">
+      <c r="E9" s="1653" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1617" t="n">
+      <c r="F9" s="1653" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1617" t="n">
+      <c r="G9" s="1653" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1617" t="n"/>
-      <c r="I9" s="1618" t="n"/>
-      <c r="J9" s="1619" t="n">
+      <c r="H9" s="1653" t="n"/>
+      <c r="I9" s="1654" t="n"/>
+      <c r="J9" s="1655" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1619" t="n">
+      <c r="K9" s="1655" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1619" t="inlineStr">
+      <c r="L9" s="1655" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1617" t="n"/>
-      <c r="N9" s="1617" t="n"/>
-      <c r="O9" s="1617" t="n">
+      <c r="M9" s="1653" t="n"/>
+      <c r="N9" s="1653" t="n"/>
+      <c r="O9" s="1653" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1620" t="n">
+      <c r="P9" s="1656" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1617" t="n"/>
-      <c r="R9" s="1617" t="n"/>
-      <c r="S9" s="1617" t="n"/>
+      <c r="Q9" s="1653" t="n"/>
+      <c r="R9" s="1653" t="n"/>
+      <c r="S9" s="1653" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1616" t="n"/>
+      <c r="U9" s="1652" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -6154,43 +6262,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1615" t="inlineStr">
+      <c r="A10" s="1651" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1616" t="inlineStr">
+      <c r="B10" s="1652" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1616" t="inlineStr">
+      <c r="C10" s="1652" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1617" t="n"/>
-      <c r="E10" s="1617" t="n"/>
-      <c r="F10" s="1617" t="n"/>
-      <c r="G10" s="1617" t="n"/>
-      <c r="H10" s="1617" t="n"/>
-      <c r="I10" s="1618" t="n"/>
-      <c r="J10" s="1619" t="n"/>
-      <c r="K10" s="1619" t="n"/>
-      <c r="L10" s="1619" t="inlineStr">
+      <c r="D10" s="1653" t="n"/>
+      <c r="E10" s="1653" t="n"/>
+      <c r="F10" s="1653" t="n"/>
+      <c r="G10" s="1653" t="n"/>
+      <c r="H10" s="1653" t="n"/>
+      <c r="I10" s="1654" t="n"/>
+      <c r="J10" s="1655" t="n"/>
+      <c r="K10" s="1655" t="n"/>
+      <c r="L10" s="1655" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1617" t="n"/>
-      <c r="N10" s="1617" t="n"/>
-      <c r="O10" s="1617" t="n"/>
-      <c r="P10" s="1620" t="n"/>
-      <c r="Q10" s="1617" t="n"/>
-      <c r="R10" s="1617" t="n"/>
-      <c r="S10" s="1617" t="n"/>
+      <c r="M10" s="1653" t="n"/>
+      <c r="N10" s="1653" t="n"/>
+      <c r="O10" s="1653" t="n"/>
+      <c r="P10" s="1656" t="n"/>
+      <c r="Q10" s="1653" t="n"/>
+      <c r="R10" s="1653" t="n"/>
+      <c r="S10" s="1653" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1616" t="n"/>
+      <c r="U10" s="1652" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -6198,43 +6306,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1615" t="inlineStr">
+      <c r="A11" s="1651" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1616" t="inlineStr">
+      <c r="B11" s="1652" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1616" t="inlineStr">
+      <c r="C11" s="1652" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1617" t="n"/>
-      <c r="E11" s="1617" t="n"/>
-      <c r="F11" s="1617" t="n"/>
-      <c r="G11" s="1617" t="n"/>
-      <c r="H11" s="1617" t="n"/>
-      <c r="I11" s="1618" t="n"/>
-      <c r="J11" s="1619" t="n"/>
-      <c r="K11" s="1619" t="n"/>
-      <c r="L11" s="1619" t="n"/>
-      <c r="M11" s="1617" t="n">
+      <c r="D11" s="1653" t="n"/>
+      <c r="E11" s="1653" t="n"/>
+      <c r="F11" s="1653" t="n"/>
+      <c r="G11" s="1653" t="n"/>
+      <c r="H11" s="1653" t="n"/>
+      <c r="I11" s="1654" t="n"/>
+      <c r="J11" s="1655" t="n"/>
+      <c r="K11" s="1655" t="n"/>
+      <c r="L11" s="1655" t="n"/>
+      <c r="M11" s="1653" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1617" t="n">
+      <c r="N11" s="1653" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1617" t="n"/>
-      <c r="P11" s="1620" t="n"/>
-      <c r="Q11" s="1617" t="n"/>
-      <c r="R11" s="1617" t="n"/>
-      <c r="S11" s="1617" t="n"/>
+      <c r="O11" s="1653" t="n"/>
+      <c r="P11" s="1656" t="n"/>
+      <c r="Q11" s="1653" t="n"/>
+      <c r="R11" s="1653" t="n"/>
+      <c r="S11" s="1653" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1616" t="n"/>
+      <c r="U11" s="1652" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -6242,39 +6350,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1591" t="inlineStr">
+      <c r="A12" s="1627" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1592" t="inlineStr">
+      <c r="B12" s="1628" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1592" t="inlineStr">
+      <c r="C12" s="1628" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1593" t="n"/>
-      <c r="E12" s="1593" t="n"/>
-      <c r="F12" s="1593" t="n"/>
-      <c r="G12" s="1593" t="n"/>
-      <c r="H12" s="1593" t="n"/>
-      <c r="I12" s="1594" t="n"/>
-      <c r="J12" s="1595" t="n"/>
-      <c r="K12" s="1595" t="n"/>
-      <c r="L12" s="1595" t="n"/>
-      <c r="M12" s="1593" t="n"/>
-      <c r="N12" s="1593" t="n"/>
-      <c r="O12" s="1593" t="n"/>
-      <c r="P12" s="1596" t="n"/>
-      <c r="Q12" s="1593" t="n"/>
-      <c r="R12" s="1593" t="n"/>
-      <c r="S12" s="1593" t="n"/>
+      <c r="D12" s="1629" t="n"/>
+      <c r="E12" s="1629" t="n"/>
+      <c r="F12" s="1629" t="n"/>
+      <c r="G12" s="1629" t="n"/>
+      <c r="H12" s="1629" t="n"/>
+      <c r="I12" s="1630" t="n"/>
+      <c r="J12" s="1631" t="n"/>
+      <c r="K12" s="1631" t="n"/>
+      <c r="L12" s="1631" t="n"/>
+      <c r="M12" s="1629" t="n"/>
+      <c r="N12" s="1629" t="n"/>
+      <c r="O12" s="1629" t="n"/>
+      <c r="P12" s="1632" t="n"/>
+      <c r="Q12" s="1629" t="n"/>
+      <c r="R12" s="1629" t="n"/>
+      <c r="S12" s="1629" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1592" t="n"/>
+      <c r="U12" s="1628" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -6282,35 +6390,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1597" t="inlineStr">
+      <c r="A13" s="1633" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1598" t="n"/>
-      <c r="C13" s="1598" t="inlineStr">
+      <c r="B13" s="1634" t="n"/>
+      <c r="C13" s="1634" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1599" t="n"/>
-      <c r="E13" s="1599" t="n"/>
-      <c r="F13" s="1599" t="n"/>
-      <c r="G13" s="1599" t="n"/>
-      <c r="H13" s="1599" t="n"/>
-      <c r="I13" s="1600" t="n"/>
-      <c r="J13" s="1601" t="n"/>
-      <c r="K13" s="1601" t="n"/>
-      <c r="L13" s="1601" t="n"/>
-      <c r="M13" s="1599" t="n"/>
-      <c r="N13" s="1599" t="n"/>
-      <c r="O13" s="1599" t="n"/>
-      <c r="P13" s="1602" t="n"/>
-      <c r="Q13" s="1599" t="n"/>
-      <c r="R13" s="1599" t="n"/>
-      <c r="S13" s="1599" t="n"/>
+      <c r="D13" s="1635" t="n"/>
+      <c r="E13" s="1635" t="n"/>
+      <c r="F13" s="1635" t="n"/>
+      <c r="G13" s="1635" t="n"/>
+      <c r="H13" s="1635" t="n"/>
+      <c r="I13" s="1636" t="n"/>
+      <c r="J13" s="1637" t="n"/>
+      <c r="K13" s="1637" t="n"/>
+      <c r="L13" s="1637" t="n"/>
+      <c r="M13" s="1635" t="n"/>
+      <c r="N13" s="1635" t="n"/>
+      <c r="O13" s="1635" t="n"/>
+      <c r="P13" s="1638" t="n"/>
+      <c r="Q13" s="1635" t="n"/>
+      <c r="R13" s="1635" t="n"/>
+      <c r="S13" s="1635" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1598" t="n"/>
+      <c r="U13" s="1634" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -6318,53 +6426,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1603" t="inlineStr">
+      <c r="A14" s="1639" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1604" t="inlineStr">
+      <c r="B14" s="1640" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1604" t="inlineStr">
+      <c r="C14" s="1640" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1605" t="n"/>
-      <c r="E14" s="1605" t="n">
+      <c r="D14" s="1641" t="n"/>
+      <c r="E14" s="1641" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1605" t="n">
+      <c r="F14" s="1641" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1605" t="n">
+      <c r="G14" s="1641" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1605" t="n"/>
-      <c r="I14" s="1606" t="n"/>
-      <c r="J14" s="1607" t="n"/>
-      <c r="K14" s="1607" t="n"/>
-      <c r="L14" s="1607" t="n"/>
-      <c r="M14" s="1605" t="n"/>
-      <c r="N14" s="1605" t="n"/>
-      <c r="O14" s="1605" t="n">
+      <c r="H14" s="1641" t="n"/>
+      <c r="I14" s="1642" t="n"/>
+      <c r="J14" s="1643" t="n"/>
+      <c r="K14" s="1643" t="n"/>
+      <c r="L14" s="1643" t="n"/>
+      <c r="M14" s="1641" t="n"/>
+      <c r="N14" s="1641" t="n"/>
+      <c r="O14" s="1641" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1608" t="n">
+      <c r="P14" s="1644" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1605" t="n"/>
-      <c r="R14" s="1605" t="n"/>
-      <c r="S14" s="1605" t="n"/>
+      <c r="Q14" s="1641" t="n"/>
+      <c r="R14" s="1641" t="n"/>
+      <c r="S14" s="1641" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1604" t="n"/>
+      <c r="U14" s="1640" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -6372,43 +6480,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1603" t="inlineStr">
+      <c r="A15" s="1639" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1604" t="inlineStr">
+      <c r="B15" s="1640" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1604" t="inlineStr">
+      <c r="C15" s="1640" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1605" t="n"/>
-      <c r="E15" s="1605" t="n"/>
-      <c r="F15" s="1605" t="n"/>
-      <c r="G15" s="1605" t="n"/>
-      <c r="H15" s="1605" t="n"/>
-      <c r="I15" s="1606" t="n"/>
-      <c r="J15" s="1607" t="n"/>
-      <c r="K15" s="1607" t="n"/>
-      <c r="L15" s="1607" t="n"/>
-      <c r="M15" s="1605" t="n">
+      <c r="D15" s="1641" t="n"/>
+      <c r="E15" s="1641" t="n"/>
+      <c r="F15" s="1641" t="n"/>
+      <c r="G15" s="1641" t="n"/>
+      <c r="H15" s="1641" t="n"/>
+      <c r="I15" s="1642" t="n"/>
+      <c r="J15" s="1643" t="n"/>
+      <c r="K15" s="1643" t="n"/>
+      <c r="L15" s="1643" t="n"/>
+      <c r="M15" s="1641" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1605" t="n">
+      <c r="N15" s="1641" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1605" t="n"/>
-      <c r="P15" s="1608" t="n"/>
-      <c r="Q15" s="1605" t="n"/>
-      <c r="R15" s="1605" t="n"/>
-      <c r="S15" s="1605" t="n"/>
+      <c r="O15" s="1641" t="n"/>
+      <c r="P15" s="1644" t="n"/>
+      <c r="Q15" s="1641" t="n"/>
+      <c r="R15" s="1641" t="n"/>
+      <c r="S15" s="1641" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1604" t="n"/>
+      <c r="U15" s="1640" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -6416,39 +6524,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1609" t="inlineStr">
+      <c r="A16" s="1645" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1610" t="inlineStr">
+      <c r="B16" s="1646" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1610" t="inlineStr">
+      <c r="C16" s="1646" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1611" t="n"/>
-      <c r="E16" s="1611" t="n"/>
-      <c r="F16" s="1611" t="n"/>
-      <c r="G16" s="1611" t="n"/>
-      <c r="H16" s="1611" t="n"/>
-      <c r="I16" s="1612" t="n"/>
-      <c r="J16" s="1613" t="n"/>
-      <c r="K16" s="1613" t="n"/>
-      <c r="L16" s="1613" t="n"/>
-      <c r="M16" s="1611" t="n"/>
-      <c r="N16" s="1611" t="n"/>
-      <c r="O16" s="1611" t="n"/>
-      <c r="P16" s="1614" t="n"/>
-      <c r="Q16" s="1611" t="n"/>
-      <c r="R16" s="1611" t="n"/>
-      <c r="S16" s="1611" t="n"/>
+      <c r="D16" s="1647" t="n"/>
+      <c r="E16" s="1647" t="n"/>
+      <c r="F16" s="1647" t="n"/>
+      <c r="G16" s="1647" t="n"/>
+      <c r="H16" s="1647" t="n"/>
+      <c r="I16" s="1648" t="n"/>
+      <c r="J16" s="1649" t="n"/>
+      <c r="K16" s="1649" t="n"/>
+      <c r="L16" s="1649" t="n"/>
+      <c r="M16" s="1647" t="n"/>
+      <c r="N16" s="1647" t="n"/>
+      <c r="O16" s="1647" t="n"/>
+      <c r="P16" s="1650" t="n"/>
+      <c r="Q16" s="1647" t="n"/>
+      <c r="R16" s="1647" t="n"/>
+      <c r="S16" s="1647" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1610" t="n"/>
+      <c r="U16" s="1646" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -6456,39 +6564,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1585" t="inlineStr">
+      <c r="A17" s="1621" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1586" t="inlineStr">
+      <c r="B17" s="1622" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1586" t="inlineStr">
+      <c r="C17" s="1622" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1587" t="n"/>
-      <c r="E17" s="1587" t="n"/>
-      <c r="F17" s="1587" t="n"/>
-      <c r="G17" s="1587" t="n"/>
-      <c r="H17" s="1587" t="n"/>
-      <c r="I17" s="1588" t="n"/>
-      <c r="J17" s="1589" t="n"/>
-      <c r="K17" s="1589" t="n"/>
-      <c r="L17" s="1589" t="n"/>
-      <c r="M17" s="1587" t="n"/>
-      <c r="N17" s="1587" t="n"/>
-      <c r="O17" s="1587" t="n"/>
-      <c r="P17" s="1590" t="n"/>
-      <c r="Q17" s="1587" t="n"/>
-      <c r="R17" s="1587" t="n"/>
-      <c r="S17" s="1587" t="n"/>
+      <c r="D17" s="1623" t="n"/>
+      <c r="E17" s="1623" t="n"/>
+      <c r="F17" s="1623" t="n"/>
+      <c r="G17" s="1623" t="n"/>
+      <c r="H17" s="1623" t="n"/>
+      <c r="I17" s="1624" t="n"/>
+      <c r="J17" s="1625" t="n"/>
+      <c r="K17" s="1625" t="n"/>
+      <c r="L17" s="1625" t="n"/>
+      <c r="M17" s="1623" t="n"/>
+      <c r="N17" s="1623" t="n"/>
+      <c r="O17" s="1623" t="n"/>
+      <c r="P17" s="1626" t="n"/>
+      <c r="Q17" s="1623" t="n"/>
+      <c r="R17" s="1623" t="n"/>
+      <c r="S17" s="1623" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1586" t="n"/>
+      <c r="U17" s="1622" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -6496,53 +6604,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1615" t="inlineStr">
+      <c r="A18" s="1651" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1616" t="inlineStr">
+      <c r="B18" s="1652" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1616" t="inlineStr">
+      <c r="C18" s="1652" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1617" t="n"/>
-      <c r="E18" s="1617" t="n">
+      <c r="D18" s="1653" t="n"/>
+      <c r="E18" s="1653" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1617" t="n">
+      <c r="F18" s="1653" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1617" t="n">
+      <c r="G18" s="1653" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1617" t="n"/>
-      <c r="I18" s="1618" t="n"/>
-      <c r="J18" s="1619" t="n"/>
-      <c r="K18" s="1619" t="n"/>
-      <c r="L18" s="1619" t="n"/>
-      <c r="M18" s="1617" t="n"/>
-      <c r="N18" s="1617" t="n"/>
-      <c r="O18" s="1617" t="n">
+      <c r="H18" s="1653" t="n"/>
+      <c r="I18" s="1654" t="n"/>
+      <c r="J18" s="1655" t="n"/>
+      <c r="K18" s="1655" t="n"/>
+      <c r="L18" s="1655" t="n"/>
+      <c r="M18" s="1653" t="n"/>
+      <c r="N18" s="1653" t="n"/>
+      <c r="O18" s="1653" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1620" t="n">
+      <c r="P18" s="1656" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1617" t="n"/>
-      <c r="R18" s="1617" t="n"/>
-      <c r="S18" s="1617" t="n"/>
+      <c r="Q18" s="1653" t="n"/>
+      <c r="R18" s="1653" t="n"/>
+      <c r="S18" s="1653" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1616" t="n"/>
+      <c r="U18" s="1652" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -6550,47 +6658,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1615" t="inlineStr">
+      <c r="A19" s="1651" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1616" t="inlineStr">
+      <c r="B19" s="1652" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1616" t="inlineStr">
+      <c r="C19" s="1652" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1617" t="n"/>
-      <c r="E19" s="1617" t="n"/>
-      <c r="F19" s="1617" t="n"/>
-      <c r="G19" s="1617" t="n"/>
-      <c r="H19" s="1617" t="n"/>
-      <c r="I19" s="1618" t="n"/>
-      <c r="J19" s="1619" t="n"/>
-      <c r="K19" s="1619" t="n"/>
-      <c r="L19" s="1619" t="n"/>
-      <c r="M19" s="1617" t="n">
+      <c r="D19" s="1653" t="n"/>
+      <c r="E19" s="1653" t="n"/>
+      <c r="F19" s="1653" t="n"/>
+      <c r="G19" s="1653" t="n"/>
+      <c r="H19" s="1653" t="n"/>
+      <c r="I19" s="1654" t="n"/>
+      <c r="J19" s="1655" t="n"/>
+      <c r="K19" s="1655" t="n"/>
+      <c r="L19" s="1655" t="n"/>
+      <c r="M19" s="1653" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1617" t="n">
+      <c r="N19" s="1653" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1617" t="n"/>
-      <c r="P19" s="1620" t="n"/>
-      <c r="Q19" s="1617" t="n"/>
-      <c r="R19" s="1617" t="n"/>
-      <c r="S19" s="1617" t="n"/>
+      <c r="O19" s="1653" t="n"/>
+      <c r="P19" s="1656" t="n"/>
+      <c r="Q19" s="1653" t="n"/>
+      <c r="R19" s="1653" t="n"/>
+      <c r="S19" s="1653" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1616" t="n"/>
+      <c r="U19" s="1652" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -6598,43 +6706,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1615" t="inlineStr">
+      <c r="A20" s="1651" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1616" t="inlineStr">
+      <c r="B20" s="1652" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1616" t="inlineStr">
+      <c r="C20" s="1652" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1617" t="n"/>
-      <c r="E20" s="1617" t="n"/>
-      <c r="F20" s="1617" t="n"/>
-      <c r="G20" s="1617" t="n"/>
-      <c r="H20" s="1617" t="n"/>
-      <c r="I20" s="1618" t="n"/>
-      <c r="J20" s="1619" t="n"/>
-      <c r="K20" s="1619" t="n"/>
-      <c r="L20" s="1619" t="n"/>
-      <c r="M20" s="1617" t="n"/>
-      <c r="N20" s="1617" t="n"/>
-      <c r="O20" s="1617" t="n"/>
-      <c r="P20" s="1620" t="n"/>
-      <c r="Q20" s="1617" t="n"/>
-      <c r="R20" s="1617" t="n"/>
-      <c r="S20" s="1617" t="n"/>
+      <c r="D20" s="1653" t="n"/>
+      <c r="E20" s="1653" t="n"/>
+      <c r="F20" s="1653" t="n"/>
+      <c r="G20" s="1653" t="n"/>
+      <c r="H20" s="1653" t="n"/>
+      <c r="I20" s="1654" t="n"/>
+      <c r="J20" s="1655" t="n"/>
+      <c r="K20" s="1655" t="n"/>
+      <c r="L20" s="1655" t="n"/>
+      <c r="M20" s="1653" t="n"/>
+      <c r="N20" s="1653" t="n"/>
+      <c r="O20" s="1653" t="n"/>
+      <c r="P20" s="1656" t="n"/>
+      <c r="Q20" s="1653" t="n"/>
+      <c r="R20" s="1653" t="n"/>
+      <c r="S20" s="1653" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1616" t="n"/>
+      <c r="U20" s="1652" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -6642,39 +6750,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1591" t="inlineStr">
+      <c r="A21" s="1627" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1592" t="inlineStr">
+      <c r="B21" s="1628" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1592" t="inlineStr">
+      <c r="C21" s="1628" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1593" t="n"/>
-      <c r="E21" s="1593" t="n"/>
-      <c r="F21" s="1593" t="n"/>
-      <c r="G21" s="1593" t="n"/>
-      <c r="H21" s="1593" t="n"/>
-      <c r="I21" s="1594" t="n"/>
-      <c r="J21" s="1595" t="n"/>
-      <c r="K21" s="1595" t="n"/>
-      <c r="L21" s="1595" t="n"/>
-      <c r="M21" s="1593" t="n"/>
-      <c r="N21" s="1593" t="n"/>
-      <c r="O21" s="1593" t="n"/>
-      <c r="P21" s="1596" t="n"/>
-      <c r="Q21" s="1593" t="n"/>
-      <c r="R21" s="1593" t="n"/>
-      <c r="S21" s="1593" t="n"/>
+      <c r="D21" s="1629" t="n"/>
+      <c r="E21" s="1629" t="n"/>
+      <c r="F21" s="1629" t="n"/>
+      <c r="G21" s="1629" t="n"/>
+      <c r="H21" s="1629" t="n"/>
+      <c r="I21" s="1630" t="n"/>
+      <c r="J21" s="1631" t="n"/>
+      <c r="K21" s="1631" t="n"/>
+      <c r="L21" s="1631" t="n"/>
+      <c r="M21" s="1629" t="n"/>
+      <c r="N21" s="1629" t="n"/>
+      <c r="O21" s="1629" t="n"/>
+      <c r="P21" s="1632" t="n"/>
+      <c r="Q21" s="1629" t="n"/>
+      <c r="R21" s="1629" t="n"/>
+      <c r="S21" s="1629" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1592" t="n"/>
+      <c r="U21" s="1628" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -6682,39 +6790,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1597" t="inlineStr">
+      <c r="A22" s="1633" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1598" t="inlineStr">
+      <c r="B22" s="1634" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1598" t="inlineStr">
+      <c r="C22" s="1634" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1599" t="n"/>
-      <c r="E22" s="1599" t="n"/>
-      <c r="F22" s="1599" t="n"/>
-      <c r="G22" s="1599" t="n"/>
-      <c r="H22" s="1599" t="n"/>
-      <c r="I22" s="1600" t="n"/>
-      <c r="J22" s="1601" t="n"/>
-      <c r="K22" s="1601" t="n"/>
-      <c r="L22" s="1601" t="n"/>
-      <c r="M22" s="1599" t="n"/>
-      <c r="N22" s="1599" t="n"/>
-      <c r="O22" s="1599" t="n"/>
-      <c r="P22" s="1602" t="n"/>
-      <c r="Q22" s="1599" t="n"/>
-      <c r="R22" s="1599" t="n"/>
-      <c r="S22" s="1599" t="n"/>
+      <c r="D22" s="1635" t="n"/>
+      <c r="E22" s="1635" t="n"/>
+      <c r="F22" s="1635" t="n"/>
+      <c r="G22" s="1635" t="n"/>
+      <c r="H22" s="1635" t="n"/>
+      <c r="I22" s="1636" t="n"/>
+      <c r="J22" s="1637" t="n"/>
+      <c r="K22" s="1637" t="n"/>
+      <c r="L22" s="1637" t="n"/>
+      <c r="M22" s="1635" t="n"/>
+      <c r="N22" s="1635" t="n"/>
+      <c r="O22" s="1635" t="n"/>
+      <c r="P22" s="1638" t="n"/>
+      <c r="Q22" s="1635" t="n"/>
+      <c r="R22" s="1635" t="n"/>
+      <c r="S22" s="1635" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1598" t="n"/>
+      <c r="U22" s="1634" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -6722,53 +6830,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1603" t="inlineStr">
+      <c r="A23" s="1639" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1604" t="inlineStr">
+      <c r="B23" s="1640" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1604" t="inlineStr">
+      <c r="C23" s="1640" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1605" t="n"/>
-      <c r="E23" s="1605" t="n">
+      <c r="D23" s="1641" t="n"/>
+      <c r="E23" s="1641" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1605" t="n">
+      <c r="F23" s="1641" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1605" t="n">
+      <c r="G23" s="1641" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1605" t="n"/>
-      <c r="I23" s="1606" t="n"/>
-      <c r="J23" s="1607" t="n"/>
-      <c r="K23" s="1607" t="n"/>
-      <c r="L23" s="1607" t="n"/>
-      <c r="M23" s="1605" t="n"/>
-      <c r="N23" s="1605" t="n"/>
-      <c r="O23" s="1605" t="n">
+      <c r="H23" s="1641" t="n"/>
+      <c r="I23" s="1642" t="n"/>
+      <c r="J23" s="1643" t="n"/>
+      <c r="K23" s="1643" t="n"/>
+      <c r="L23" s="1643" t="n"/>
+      <c r="M23" s="1641" t="n"/>
+      <c r="N23" s="1641" t="n"/>
+      <c r="O23" s="1641" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1608" t="n">
+      <c r="P23" s="1644" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1605" t="n"/>
-      <c r="R23" s="1605" t="n"/>
-      <c r="S23" s="1605" t="n"/>
+      <c r="Q23" s="1641" t="n"/>
+      <c r="R23" s="1641" t="n"/>
+      <c r="S23" s="1641" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1604" t="n"/>
+      <c r="U23" s="1640" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -6776,47 +6884,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1609" t="inlineStr">
+      <c r="A24" s="1645" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1610" t="inlineStr">
+      <c r="B24" s="1646" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1610" t="inlineStr">
+      <c r="C24" s="1646" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1611" t="n"/>
-      <c r="E24" s="1611" t="n"/>
-      <c r="F24" s="1611" t="n"/>
-      <c r="G24" s="1611" t="n"/>
-      <c r="H24" s="1611" t="n"/>
-      <c r="I24" s="1612" t="n"/>
-      <c r="J24" s="1613" t="n"/>
-      <c r="K24" s="1613" t="n"/>
-      <c r="L24" s="1613" t="n"/>
-      <c r="M24" s="1611" t="n">
+      <c r="D24" s="1647" t="n"/>
+      <c r="E24" s="1647" t="n"/>
+      <c r="F24" s="1647" t="n"/>
+      <c r="G24" s="1647" t="n"/>
+      <c r="H24" s="1647" t="n"/>
+      <c r="I24" s="1648" t="n"/>
+      <c r="J24" s="1649" t="n"/>
+      <c r="K24" s="1649" t="n"/>
+      <c r="L24" s="1649" t="n"/>
+      <c r="M24" s="1647" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1611" t="n">
+      <c r="N24" s="1647" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1611" t="n"/>
-      <c r="P24" s="1614" t="n"/>
-      <c r="Q24" s="1611" t="n"/>
-      <c r="R24" s="1611" t="n"/>
-      <c r="S24" s="1611" t="n"/>
+      <c r="O24" s="1647" t="n"/>
+      <c r="P24" s="1650" t="n"/>
+      <c r="Q24" s="1647" t="n"/>
+      <c r="R24" s="1647" t="n"/>
+      <c r="S24" s="1647" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1610" t="n"/>
+      <c r="U24" s="1646" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -6824,61 +6932,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1585" t="inlineStr">
+      <c r="A25" s="1621" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1586" t="inlineStr">
+      <c r="B25" s="1622" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1586" t="inlineStr">
+      <c r="C25" s="1622" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1587" t="n">
+      <c r="D25" s="1623" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1587" t="n">
+      <c r="E25" s="1623" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1587" t="n">
+      <c r="F25" s="1623" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1587" t="n">
+      <c r="G25" s="1623" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1587" t="n"/>
-      <c r="I25" s="1588" t="n"/>
-      <c r="J25" s="1589" t="n">
+      <c r="H25" s="1623" t="n"/>
+      <c r="I25" s="1624" t="n"/>
+      <c r="J25" s="1625" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1589" t="n">
+      <c r="K25" s="1625" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1589" t="n">
+      <c r="L25" s="1625" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1587" t="n"/>
-      <c r="N25" s="1587" t="n"/>
-      <c r="O25" s="1587" t="n">
+      <c r="M25" s="1623" t="n"/>
+      <c r="N25" s="1623" t="n"/>
+      <c r="O25" s="1623" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1590" t="n">
+      <c r="P25" s="1626" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1587" t="n"/>
-      <c r="R25" s="1587" t="n"/>
-      <c r="S25" s="1587" t="n"/>
+      <c r="Q25" s="1623" t="n"/>
+      <c r="R25" s="1623" t="n"/>
+      <c r="S25" s="1623" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1586" t="n"/>
+      <c r="U25" s="1622" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -6886,47 +6994,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1591" t="inlineStr">
+      <c r="A26" s="1627" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1592" t="inlineStr">
+      <c r="B26" s="1628" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1592" t="inlineStr">
+      <c r="C26" s="1628" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1593" t="n"/>
-      <c r="E26" s="1593" t="n"/>
-      <c r="F26" s="1593" t="n"/>
-      <c r="G26" s="1593" t="n"/>
-      <c r="H26" s="1593" t="n"/>
-      <c r="I26" s="1594" t="n"/>
-      <c r="J26" s="1595" t="n"/>
-      <c r="K26" s="1595" t="n"/>
-      <c r="L26" s="1595" t="n"/>
-      <c r="M26" s="1593" t="n">
+      <c r="D26" s="1629" t="n"/>
+      <c r="E26" s="1629" t="n"/>
+      <c r="F26" s="1629" t="n"/>
+      <c r="G26" s="1629" t="n"/>
+      <c r="H26" s="1629" t="n"/>
+      <c r="I26" s="1630" t="n"/>
+      <c r="J26" s="1631" t="n"/>
+      <c r="K26" s="1631" t="n"/>
+      <c r="L26" s="1631" t="n"/>
+      <c r="M26" s="1629" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1593" t="n">
+      <c r="N26" s="1629" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1593" t="n"/>
-      <c r="P26" s="1596" t="n"/>
-      <c r="Q26" s="1593" t="n"/>
-      <c r="R26" s="1593" t="n"/>
-      <c r="S26" s="1593" t="n"/>
+      <c r="O26" s="1629" t="n"/>
+      <c r="P26" s="1632" t="n"/>
+      <c r="Q26" s="1629" t="n"/>
+      <c r="R26" s="1629" t="n"/>
+      <c r="S26" s="1629" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1592" t="n"/>
+      <c r="U26" s="1628" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -6934,53 +7042,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1597" t="inlineStr">
+      <c r="A27" s="1633" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1598" t="inlineStr">
+      <c r="B27" s="1634" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1598" t="inlineStr">
+      <c r="C27" s="1634" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1599" t="n"/>
-      <c r="E27" s="1599" t="n">
+      <c r="D27" s="1635" t="n"/>
+      <c r="E27" s="1635" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1599" t="n">
+      <c r="F27" s="1635" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1599" t="n">
+      <c r="G27" s="1635" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1599" t="n"/>
-      <c r="I27" s="1600" t="n"/>
-      <c r="J27" s="1601" t="n"/>
-      <c r="K27" s="1601" t="n"/>
-      <c r="L27" s="1601" t="n"/>
-      <c r="M27" s="1599" t="n"/>
-      <c r="N27" s="1599" t="n"/>
-      <c r="O27" s="1599" t="n">
+      <c r="H27" s="1635" t="n"/>
+      <c r="I27" s="1636" t="n"/>
+      <c r="J27" s="1637" t="n"/>
+      <c r="K27" s="1637" t="n"/>
+      <c r="L27" s="1637" t="n"/>
+      <c r="M27" s="1635" t="n"/>
+      <c r="N27" s="1635" t="n"/>
+      <c r="O27" s="1635" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1602" t="n">
+      <c r="P27" s="1638" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1599" t="n"/>
-      <c r="R27" s="1599" t="n"/>
-      <c r="S27" s="1599" t="n"/>
+      <c r="Q27" s="1635" t="n"/>
+      <c r="R27" s="1635" t="n"/>
+      <c r="S27" s="1635" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1598" t="n"/>
+      <c r="U27" s="1634" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -6988,47 +7096,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1609" t="inlineStr">
+      <c r="A28" s="1645" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1610" t="inlineStr">
+      <c r="B28" s="1646" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1610" t="inlineStr">
+      <c r="C28" s="1646" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1611" t="n"/>
-      <c r="E28" s="1611" t="n"/>
-      <c r="F28" s="1611" t="n"/>
-      <c r="G28" s="1611" t="n"/>
-      <c r="H28" s="1611" t="n"/>
-      <c r="I28" s="1612" t="n"/>
-      <c r="J28" s="1613" t="n"/>
-      <c r="K28" s="1613" t="n"/>
-      <c r="L28" s="1613" t="n"/>
-      <c r="M28" s="1611" t="n">
+      <c r="D28" s="1647" t="n"/>
+      <c r="E28" s="1647" t="n"/>
+      <c r="F28" s="1647" t="n"/>
+      <c r="G28" s="1647" t="n"/>
+      <c r="H28" s="1647" t="n"/>
+      <c r="I28" s="1648" t="n"/>
+      <c r="J28" s="1649" t="n"/>
+      <c r="K28" s="1649" t="n"/>
+      <c r="L28" s="1649" t="n"/>
+      <c r="M28" s="1647" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1611" t="n">
+      <c r="N28" s="1647" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1611" t="n"/>
-      <c r="P28" s="1614" t="n"/>
-      <c r="Q28" s="1611" t="n"/>
-      <c r="R28" s="1611" t="n"/>
-      <c r="S28" s="1611" t="n"/>
+      <c r="O28" s="1647" t="n"/>
+      <c r="P28" s="1650" t="n"/>
+      <c r="Q28" s="1647" t="n"/>
+      <c r="R28" s="1647" t="n"/>
+      <c r="S28" s="1647" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1610" t="n"/>
+      <c r="U28" s="1646" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -7036,53 +7144,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1585" t="inlineStr">
+      <c r="A29" s="1621" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1586" t="inlineStr">
+      <c r="B29" s="1622" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1586" t="inlineStr">
+      <c r="C29" s="1622" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1587" t="n"/>
-      <c r="E29" s="1587" t="n">
+      <c r="D29" s="1623" t="n"/>
+      <c r="E29" s="1623" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1587" t="n">
+      <c r="F29" s="1623" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1587" t="n">
+      <c r="G29" s="1623" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1587" t="n"/>
-      <c r="I29" s="1588" t="n"/>
-      <c r="J29" s="1589" t="n"/>
-      <c r="K29" s="1589" t="n"/>
-      <c r="L29" s="1589" t="n"/>
-      <c r="M29" s="1587" t="n"/>
-      <c r="N29" s="1587" t="n"/>
-      <c r="O29" s="1587" t="n">
+      <c r="H29" s="1623" t="n"/>
+      <c r="I29" s="1624" t="n"/>
+      <c r="J29" s="1625" t="n"/>
+      <c r="K29" s="1625" t="n"/>
+      <c r="L29" s="1625" t="n"/>
+      <c r="M29" s="1623" t="n"/>
+      <c r="N29" s="1623" t="n"/>
+      <c r="O29" s="1623" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1590" t="n">
+      <c r="P29" s="1626" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1587" t="n"/>
-      <c r="R29" s="1587" t="n"/>
-      <c r="S29" s="1587" t="n"/>
+      <c r="Q29" s="1623" t="n"/>
+      <c r="R29" s="1623" t="n"/>
+      <c r="S29" s="1623" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1586" t="n"/>
+      <c r="U29" s="1622" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -7090,43 +7198,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1591" t="inlineStr">
+      <c r="A30" s="1627" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1592" t="inlineStr">
+      <c r="B30" s="1628" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1592" t="inlineStr">
+      <c r="C30" s="1628" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1593" t="n"/>
-      <c r="E30" s="1593" t="n"/>
-      <c r="F30" s="1593" t="n"/>
-      <c r="G30" s="1593" t="n"/>
-      <c r="H30" s="1593" t="n"/>
-      <c r="I30" s="1594" t="n"/>
-      <c r="J30" s="1595" t="n"/>
-      <c r="K30" s="1595" t="n"/>
-      <c r="L30" s="1595" t="n"/>
-      <c r="M30" s="1593" t="n"/>
-      <c r="N30" s="1593" t="n"/>
-      <c r="O30" s="1593" t="n"/>
-      <c r="P30" s="1596" t="n"/>
-      <c r="Q30" s="1593" t="n"/>
-      <c r="R30" s="1593" t="n"/>
-      <c r="S30" s="1593" t="n"/>
+      <c r="D30" s="1629" t="n"/>
+      <c r="E30" s="1629" t="n"/>
+      <c r="F30" s="1629" t="n"/>
+      <c r="G30" s="1629" t="n"/>
+      <c r="H30" s="1629" t="n"/>
+      <c r="I30" s="1630" t="n"/>
+      <c r="J30" s="1631" t="n"/>
+      <c r="K30" s="1631" t="n"/>
+      <c r="L30" s="1631" t="n"/>
+      <c r="M30" s="1629" t="n"/>
+      <c r="N30" s="1629" t="n"/>
+      <c r="O30" s="1629" t="n"/>
+      <c r="P30" s="1632" t="n"/>
+      <c r="Q30" s="1629" t="n"/>
+      <c r="R30" s="1629" t="n"/>
+      <c r="S30" s="1629" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1592" t="n"/>
+      <c r="U30" s="1628" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -7134,53 +7242,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1597" t="inlineStr">
+      <c r="A31" s="1633" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1598" t="inlineStr">
+      <c r="B31" s="1634" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1598" t="inlineStr">
+      <c r="C31" s="1634" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1599" t="n"/>
-      <c r="E31" s="1599" t="n">
+      <c r="D31" s="1635" t="n"/>
+      <c r="E31" s="1635" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1599" t="n">
+      <c r="F31" s="1635" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1599" t="n">
+      <c r="G31" s="1635" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1599" t="n"/>
-      <c r="I31" s="1600" t="n"/>
-      <c r="J31" s="1601" t="n"/>
-      <c r="K31" s="1601" t="n"/>
-      <c r="L31" s="1601" t="n"/>
-      <c r="M31" s="1599" t="n"/>
-      <c r="N31" s="1599" t="n"/>
-      <c r="O31" s="1599" t="n">
+      <c r="H31" s="1635" t="n"/>
+      <c r="I31" s="1636" t="n"/>
+      <c r="J31" s="1637" t="n"/>
+      <c r="K31" s="1637" t="n"/>
+      <c r="L31" s="1637" t="n"/>
+      <c r="M31" s="1635" t="n"/>
+      <c r="N31" s="1635" t="n"/>
+      <c r="O31" s="1635" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1602" t="n">
+      <c r="P31" s="1638" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1599" t="n"/>
-      <c r="R31" s="1599" t="n"/>
-      <c r="S31" s="1599" t="n"/>
+      <c r="Q31" s="1635" t="n"/>
+      <c r="R31" s="1635" t="n"/>
+      <c r="S31" s="1635" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1598" t="inlineStr">
+      <c r="U31" s="1634" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -7192,49 +7300,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1609" t="inlineStr">
+      <c r="A32" s="1645" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1610" t="inlineStr">
+      <c r="B32" s="1646" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1610" t="inlineStr">
+      <c r="C32" s="1646" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1611" t="n"/>
-      <c r="E32" s="1611" t="n"/>
-      <c r="F32" s="1611" t="n"/>
-      <c r="G32" s="1611" t="n"/>
-      <c r="H32" s="1611" t="n">
+      <c r="D32" s="1647" t="n"/>
+      <c r="E32" s="1647" t="n"/>
+      <c r="F32" s="1647" t="n"/>
+      <c r="G32" s="1647" t="n"/>
+      <c r="H32" s="1647" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1612" t="n"/>
-      <c r="J32" s="1613" t="n"/>
-      <c r="K32" s="1613" t="n"/>
-      <c r="L32" s="1613" t="n"/>
-      <c r="M32" s="1611" t="n">
+      <c r="I32" s="1648" t="n"/>
+      <c r="J32" s="1649" t="n"/>
+      <c r="K32" s="1649" t="n"/>
+      <c r="L32" s="1649" t="n"/>
+      <c r="M32" s="1647" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1611" t="n">
+      <c r="N32" s="1647" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1611" t="n"/>
-      <c r="P32" s="1614" t="n"/>
-      <c r="Q32" s="1611" t="n"/>
-      <c r="R32" s="1611" t="n"/>
-      <c r="S32" s="1611" t="n"/>
+      <c r="O32" s="1647" t="n"/>
+      <c r="P32" s="1650" t="n"/>
+      <c r="Q32" s="1647" t="n"/>
+      <c r="R32" s="1647" t="n"/>
+      <c r="S32" s="1647" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1610" t="n"/>
+      <c r="U32" s="1646" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -7242,57 +7350,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1585" t="inlineStr">
+      <c r="A33" s="1621" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1586" t="inlineStr">
+      <c r="B33" s="1622" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1586" t="inlineStr">
+      <c r="C33" s="1622" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1587" t="n"/>
-      <c r="E33" s="1587" t="n">
+      <c r="D33" s="1623" t="n"/>
+      <c r="E33" s="1623" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1587" t="n">
+      <c r="F33" s="1623" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1587" t="n">
+      <c r="G33" s="1623" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1587" t="n"/>
-      <c r="I33" s="1588" t="n">
+      <c r="H33" s="1623" t="n"/>
+      <c r="I33" s="1624" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1589" t="n"/>
-      <c r="K33" s="1589" t="n"/>
-      <c r="L33" s="1589" t="n"/>
-      <c r="M33" s="1587" t="n"/>
-      <c r="N33" s="1587" t="n"/>
-      <c r="O33" s="1587" t="n">
+      <c r="J33" s="1625" t="n"/>
+      <c r="K33" s="1625" t="n"/>
+      <c r="L33" s="1625" t="n"/>
+      <c r="M33" s="1623" t="n"/>
+      <c r="N33" s="1623" t="n"/>
+      <c r="O33" s="1623" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1590" t="n">
+      <c r="P33" s="1626" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1587" t="n"/>
-      <c r="R33" s="1587" t="n">
+      <c r="Q33" s="1623" t="n"/>
+      <c r="R33" s="1623" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1587" t="n"/>
+      <c r="S33" s="1623" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1586" t="inlineStr">
+      <c r="U33" s="1622" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -7304,49 +7412,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1591" t="inlineStr">
+      <c r="A34" s="1627" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1592" t="inlineStr">
+      <c r="B34" s="1628" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1592" t="inlineStr">
+      <c r="C34" s="1628" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1593" t="n"/>
-      <c r="E34" s="1593" t="n"/>
-      <c r="F34" s="1593" t="n"/>
-      <c r="G34" s="1593" t="n"/>
-      <c r="H34" s="1593" t="n">
+      <c r="D34" s="1629" t="n"/>
+      <c r="E34" s="1629" t="n"/>
+      <c r="F34" s="1629" t="n"/>
+      <c r="G34" s="1629" t="n"/>
+      <c r="H34" s="1629" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1594" t="n"/>
-      <c r="J34" s="1595" t="n"/>
-      <c r="K34" s="1595" t="n"/>
-      <c r="L34" s="1595" t="n"/>
-      <c r="M34" s="1593" t="n">
+      <c r="I34" s="1630" t="n"/>
+      <c r="J34" s="1631" t="n"/>
+      <c r="K34" s="1631" t="n"/>
+      <c r="L34" s="1631" t="n"/>
+      <c r="M34" s="1629" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1593" t="n">
+      <c r="N34" s="1629" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1593" t="n"/>
-      <c r="P34" s="1596" t="n"/>
-      <c r="Q34" s="1593" t="n"/>
-      <c r="R34" s="1593" t="n"/>
-      <c r="S34" s="1593" t="n"/>
+      <c r="O34" s="1629" t="n"/>
+      <c r="P34" s="1632" t="n"/>
+      <c r="Q34" s="1629" t="n"/>
+      <c r="R34" s="1629" t="n"/>
+      <c r="S34" s="1629" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1592" t="n"/>
+      <c r="U34" s="1628" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -7354,57 +7462,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1597" t="inlineStr">
+      <c r="A35" s="1633" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1598" t="inlineStr">
+      <c r="B35" s="1634" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1598" t="inlineStr">
+      <c r="C35" s="1634" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1599" t="n"/>
-      <c r="E35" s="1599" t="n">
+      <c r="D35" s="1635" t="n"/>
+      <c r="E35" s="1635" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1599" t="n">
+      <c r="F35" s="1635" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1599" t="n">
+      <c r="G35" s="1635" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1599" t="n"/>
-      <c r="I35" s="1600" t="n">
+      <c r="H35" s="1635" t="n"/>
+      <c r="I35" s="1636" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1601" t="n"/>
-      <c r="K35" s="1601" t="n"/>
-      <c r="L35" s="1601" t="n"/>
-      <c r="M35" s="1599" t="n"/>
-      <c r="N35" s="1599" t="n"/>
-      <c r="O35" s="1599" t="n">
+      <c r="J35" s="1637" t="n"/>
+      <c r="K35" s="1637" t="n"/>
+      <c r="L35" s="1637" t="n"/>
+      <c r="M35" s="1635" t="n"/>
+      <c r="N35" s="1635" t="n"/>
+      <c r="O35" s="1635" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1602" t="n">
+      <c r="P35" s="1638" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1599" t="n"/>
-      <c r="R35" s="1599" t="n">
+      <c r="Q35" s="1635" t="n"/>
+      <c r="R35" s="1635" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1599" t="n"/>
+      <c r="S35" s="1635" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1598" t="inlineStr">
+      <c r="U35" s="1634" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -7416,49 +7524,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1603" t="inlineStr">
+      <c r="A36" s="1639" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1604" t="inlineStr">
+      <c r="B36" s="1640" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1604" t="inlineStr">
+      <c r="C36" s="1640" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1605" t="n"/>
-      <c r="E36" s="1605" t="n"/>
-      <c r="F36" s="1605" t="n"/>
-      <c r="G36" s="1605" t="n"/>
-      <c r="H36" s="1605" t="n">
+      <c r="D36" s="1641" t="n"/>
+      <c r="E36" s="1641" t="n"/>
+      <c r="F36" s="1641" t="n"/>
+      <c r="G36" s="1641" t="n"/>
+      <c r="H36" s="1641" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1606" t="n"/>
-      <c r="J36" s="1607" t="n"/>
-      <c r="K36" s="1607" t="n"/>
-      <c r="L36" s="1607" t="n"/>
-      <c r="M36" s="1605" t="n">
+      <c r="I36" s="1642" t="n"/>
+      <c r="J36" s="1643" t="n"/>
+      <c r="K36" s="1643" t="n"/>
+      <c r="L36" s="1643" t="n"/>
+      <c r="M36" s="1641" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1605" t="n">
+      <c r="N36" s="1641" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1605" t="n"/>
-      <c r="P36" s="1608" t="n"/>
-      <c r="Q36" s="1605" t="n"/>
-      <c r="R36" s="1605" t="n"/>
-      <c r="S36" s="1605" t="n"/>
+      <c r="O36" s="1641" t="n"/>
+      <c r="P36" s="1644" t="n"/>
+      <c r="Q36" s="1641" t="n"/>
+      <c r="R36" s="1641" t="n"/>
+      <c r="S36" s="1641" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1604" t="n"/>
+      <c r="U36" s="1640" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -7466,41 +7574,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1609" t="inlineStr">
+      <c r="A37" s="1645" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1610" t="inlineStr">
+      <c r="B37" s="1646" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1610" t="inlineStr">
+      <c r="C37" s="1646" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1611" t="n"/>
-      <c r="E37" s="1611" t="n"/>
-      <c r="F37" s="1611" t="n"/>
-      <c r="G37" s="1611" t="n"/>
-      <c r="H37" s="1611" t="n"/>
-      <c r="I37" s="1612" t="n"/>
-      <c r="J37" s="1613" t="n"/>
-      <c r="K37" s="1613" t="n"/>
-      <c r="L37" s="1613" t="n"/>
-      <c r="M37" s="1611" t="n"/>
-      <c r="N37" s="1611" t="n"/>
-      <c r="O37" s="1611" t="n"/>
-      <c r="P37" s="1614" t="n"/>
-      <c r="Q37" s="1611" t="n">
+      <c r="D37" s="1647" t="n"/>
+      <c r="E37" s="1647" t="n"/>
+      <c r="F37" s="1647" t="n"/>
+      <c r="G37" s="1647" t="n"/>
+      <c r="H37" s="1647" t="n"/>
+      <c r="I37" s="1648" t="n"/>
+      <c r="J37" s="1649" t="n"/>
+      <c r="K37" s="1649" t="n"/>
+      <c r="L37" s="1649" t="n"/>
+      <c r="M37" s="1647" t="n"/>
+      <c r="N37" s="1647" t="n"/>
+      <c r="O37" s="1647" t="n"/>
+      <c r="P37" s="1650" t="n"/>
+      <c r="Q37" s="1647" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1611" t="n"/>
-      <c r="S37" s="1611" t="n"/>
+      <c r="R37" s="1647" t="n"/>
+      <c r="S37" s="1647" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1610" t="n"/>
+      <c r="U37" s="1646" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -7508,57 +7616,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1585" t="inlineStr">
+      <c r="A38" s="1621" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1586" t="inlineStr">
+      <c r="B38" s="1622" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1586" t="inlineStr">
+      <c r="C38" s="1622" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1587" t="n"/>
-      <c r="E38" s="1587" t="n">
+      <c r="D38" s="1623" t="n"/>
+      <c r="E38" s="1623" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1587" t="n">
+      <c r="F38" s="1623" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1587" t="n">
+      <c r="G38" s="1623" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1587" t="n"/>
-      <c r="I38" s="1588" t="n">
+      <c r="H38" s="1623" t="n"/>
+      <c r="I38" s="1624" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1589" t="n"/>
-      <c r="K38" s="1589" t="n"/>
-      <c r="L38" s="1589" t="n"/>
-      <c r="M38" s="1587" t="n"/>
-      <c r="N38" s="1587" t="n"/>
-      <c r="O38" s="1587" t="n">
+      <c r="J38" s="1625" t="n"/>
+      <c r="K38" s="1625" t="n"/>
+      <c r="L38" s="1625" t="n"/>
+      <c r="M38" s="1623" t="n"/>
+      <c r="N38" s="1623" t="n"/>
+      <c r="O38" s="1623" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1590" t="n">
+      <c r="P38" s="1626" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1587" t="n"/>
-      <c r="R38" s="1587" t="n">
+      <c r="Q38" s="1623" t="n"/>
+      <c r="R38" s="1623" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1587" t="n"/>
+      <c r="S38" s="1623" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1586" t="inlineStr">
+      <c r="U38" s="1622" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -7570,49 +7678,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1615" t="inlineStr">
+      <c r="A39" s="1651" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1616" t="inlineStr">
+      <c r="B39" s="1652" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1616" t="inlineStr">
+      <c r="C39" s="1652" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1617" t="n"/>
-      <c r="E39" s="1617" t="n"/>
-      <c r="F39" s="1617" t="n"/>
-      <c r="G39" s="1617" t="n"/>
-      <c r="H39" s="1617" t="n">
+      <c r="D39" s="1653" t="n"/>
+      <c r="E39" s="1653" t="n"/>
+      <c r="F39" s="1653" t="n"/>
+      <c r="G39" s="1653" t="n"/>
+      <c r="H39" s="1653" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1618" t="n"/>
-      <c r="J39" s="1619" t="n"/>
-      <c r="K39" s="1619" t="n"/>
-      <c r="L39" s="1619" t="n"/>
-      <c r="M39" s="1617" t="n">
+      <c r="I39" s="1654" t="n"/>
+      <c r="J39" s="1655" t="n"/>
+      <c r="K39" s="1655" t="n"/>
+      <c r="L39" s="1655" t="n"/>
+      <c r="M39" s="1653" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1617" t="n">
+      <c r="N39" s="1653" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1617" t="n"/>
-      <c r="P39" s="1620" t="n"/>
-      <c r="Q39" s="1617" t="n"/>
-      <c r="R39" s="1617" t="n"/>
-      <c r="S39" s="1617" t="n"/>
+      <c r="O39" s="1653" t="n"/>
+      <c r="P39" s="1656" t="n"/>
+      <c r="Q39" s="1653" t="n"/>
+      <c r="R39" s="1653" t="n"/>
+      <c r="S39" s="1653" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1616" t="n"/>
+      <c r="U39" s="1652" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -7620,41 +7728,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1591" t="inlineStr">
+      <c r="A40" s="1627" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1592" t="inlineStr">
+      <c r="B40" s="1628" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1592" t="inlineStr">
+      <c r="C40" s="1628" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1593" t="n"/>
-      <c r="E40" s="1593" t="n"/>
-      <c r="F40" s="1593" t="n"/>
-      <c r="G40" s="1593" t="n"/>
-      <c r="H40" s="1593" t="n"/>
-      <c r="I40" s="1594" t="n"/>
-      <c r="J40" s="1595" t="n"/>
-      <c r="K40" s="1595" t="n"/>
-      <c r="L40" s="1595" t="n"/>
-      <c r="M40" s="1593" t="n"/>
-      <c r="N40" s="1593" t="n"/>
-      <c r="O40" s="1593" t="n"/>
-      <c r="P40" s="1596" t="n"/>
-      <c r="Q40" s="1593" t="n">
+      <c r="D40" s="1629" t="n"/>
+      <c r="E40" s="1629" t="n"/>
+      <c r="F40" s="1629" t="n"/>
+      <c r="G40" s="1629" t="n"/>
+      <c r="H40" s="1629" t="n"/>
+      <c r="I40" s="1630" t="n"/>
+      <c r="J40" s="1631" t="n"/>
+      <c r="K40" s="1631" t="n"/>
+      <c r="L40" s="1631" t="n"/>
+      <c r="M40" s="1629" t="n"/>
+      <c r="N40" s="1629" t="n"/>
+      <c r="O40" s="1629" t="n"/>
+      <c r="P40" s="1632" t="n"/>
+      <c r="Q40" s="1629" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1593" t="n"/>
-      <c r="S40" s="1593" t="n"/>
+      <c r="R40" s="1629" t="n"/>
+      <c r="S40" s="1629" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1592" t="n"/>
+      <c r="U40" s="1628" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -7662,57 +7770,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1597" t="inlineStr">
+      <c r="A41" s="1633" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1598" t="inlineStr">
+      <c r="B41" s="1634" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1598" t="inlineStr">
+      <c r="C41" s="1634" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1599" t="n"/>
-      <c r="E41" s="1599" t="n">
+      <c r="D41" s="1635" t="n"/>
+      <c r="E41" s="1635" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1599" t="n">
+      <c r="F41" s="1635" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1599" t="n">
+      <c r="G41" s="1635" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1599" t="n"/>
-      <c r="I41" s="1600" t="n">
+      <c r="H41" s="1635" t="n"/>
+      <c r="I41" s="1636" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1601" t="n"/>
-      <c r="K41" s="1601" t="n"/>
-      <c r="L41" s="1601" t="n"/>
-      <c r="M41" s="1599" t="n"/>
-      <c r="N41" s="1599" t="n"/>
-      <c r="O41" s="1599" t="n">
+      <c r="J41" s="1637" t="n"/>
+      <c r="K41" s="1637" t="n"/>
+      <c r="L41" s="1637" t="n"/>
+      <c r="M41" s="1635" t="n"/>
+      <c r="N41" s="1635" t="n"/>
+      <c r="O41" s="1635" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1602" t="n">
+      <c r="P41" s="1638" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1599" t="n"/>
-      <c r="R41" s="1599" t="n">
+      <c r="Q41" s="1635" t="n"/>
+      <c r="R41" s="1635" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1599" t="n"/>
+      <c r="S41" s="1635" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1598" t="inlineStr">
+      <c r="U41" s="1634" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -7724,49 +7832,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1609" t="inlineStr">
+      <c r="A42" s="1645" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1610" t="inlineStr">
+      <c r="B42" s="1646" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1610" t="inlineStr">
+      <c r="C42" s="1646" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1611" t="n"/>
-      <c r="E42" s="1611" t="n"/>
-      <c r="F42" s="1611" t="n"/>
-      <c r="G42" s="1611" t="n"/>
-      <c r="H42" s="1611" t="n">
+      <c r="D42" s="1647" t="n"/>
+      <c r="E42" s="1647" t="n"/>
+      <c r="F42" s="1647" t="n"/>
+      <c r="G42" s="1647" t="n"/>
+      <c r="H42" s="1647" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1612" t="n"/>
-      <c r="J42" s="1613" t="n"/>
-      <c r="K42" s="1613" t="n"/>
-      <c r="L42" s="1613" t="n"/>
-      <c r="M42" s="1611" t="n">
+      <c r="I42" s="1648" t="n"/>
+      <c r="J42" s="1649" t="n"/>
+      <c r="K42" s="1649" t="n"/>
+      <c r="L42" s="1649" t="n"/>
+      <c r="M42" s="1647" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1611" t="n">
+      <c r="N42" s="1647" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1611" t="n"/>
-      <c r="P42" s="1614" t="n"/>
-      <c r="Q42" s="1611" t="n"/>
-      <c r="R42" s="1611" t="n"/>
-      <c r="S42" s="1611" t="n"/>
+      <c r="O42" s="1647" t="n"/>
+      <c r="P42" s="1650" t="n"/>
+      <c r="Q42" s="1647" t="n"/>
+      <c r="R42" s="1647" t="n"/>
+      <c r="S42" s="1647" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1610" t="n"/>
+      <c r="U42" s="1646" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -7774,57 +7882,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1585" t="inlineStr">
+      <c r="A43" s="1621" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1586" t="inlineStr">
+      <c r="B43" s="1622" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1586" t="inlineStr">
+      <c r="C43" s="1622" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1587" t="n"/>
-      <c r="E43" s="1587" t="n">
+      <c r="D43" s="1623" t="n"/>
+      <c r="E43" s="1623" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1587" t="n">
+      <c r="F43" s="1623" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1587" t="n">
+      <c r="G43" s="1623" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1587" t="n"/>
-      <c r="I43" s="1588" t="n">
+      <c r="H43" s="1623" t="n"/>
+      <c r="I43" s="1624" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1589" t="n"/>
-      <c r="K43" s="1589" t="n"/>
-      <c r="L43" s="1589" t="n"/>
-      <c r="M43" s="1587" t="n"/>
-      <c r="N43" s="1587" t="n"/>
-      <c r="O43" s="1587" t="n">
+      <c r="J43" s="1625" t="n"/>
+      <c r="K43" s="1625" t="n"/>
+      <c r="L43" s="1625" t="n"/>
+      <c r="M43" s="1623" t="n"/>
+      <c r="N43" s="1623" t="n"/>
+      <c r="O43" s="1623" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1590" t="n">
+      <c r="P43" s="1626" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1587" t="n"/>
-      <c r="R43" s="1587" t="n">
+      <c r="Q43" s="1623" t="n"/>
+      <c r="R43" s="1623" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1587" t="n"/>
+      <c r="S43" s="1623" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1586" t="n"/>
+      <c r="U43" s="1622" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -7832,45 +7940,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1615" t="inlineStr">
+      <c r="A44" s="1651" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1616" t="inlineStr">
+      <c r="B44" s="1652" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1616" t="inlineStr">
+      <c r="C44" s="1652" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1617" t="n"/>
-      <c r="E44" s="1617" t="n">
+      <c r="D44" s="1653" t="n"/>
+      <c r="E44" s="1653" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1617" t="n">
+      <c r="F44" s="1653" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1617" t="n"/>
-      <c r="H44" s="1617" t="n"/>
-      <c r="I44" s="1618" t="n"/>
-      <c r="J44" s="1619" t="n"/>
-      <c r="K44" s="1619" t="n"/>
-      <c r="L44" s="1619" t="n"/>
-      <c r="M44" s="1617" t="n"/>
-      <c r="N44" s="1617" t="n"/>
-      <c r="O44" s="1617" t="n"/>
-      <c r="P44" s="1620" t="n"/>
-      <c r="Q44" s="1617" t="n"/>
-      <c r="R44" s="1617" t="n"/>
-      <c r="S44" s="1617" t="n">
+      <c r="G44" s="1653" t="n"/>
+      <c r="H44" s="1653" t="n"/>
+      <c r="I44" s="1654" t="n"/>
+      <c r="J44" s="1655" t="n"/>
+      <c r="K44" s="1655" t="n"/>
+      <c r="L44" s="1655" t="n"/>
+      <c r="M44" s="1653" t="n"/>
+      <c r="N44" s="1653" t="n"/>
+      <c r="O44" s="1653" t="n"/>
+      <c r="P44" s="1656" t="n"/>
+      <c r="Q44" s="1653" t="n"/>
+      <c r="R44" s="1653" t="n"/>
+      <c r="S44" s="1653" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1616" t="inlineStr">
+      <c r="U44" s="1652" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -7882,49 +7990,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1615" t="inlineStr">
+      <c r="A45" s="1651" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1616" t="inlineStr">
+      <c r="B45" s="1652" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1616" t="inlineStr">
+      <c r="C45" s="1652" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1617" t="n"/>
-      <c r="E45" s="1617" t="n"/>
-      <c r="F45" s="1617" t="n"/>
-      <c r="G45" s="1617" t="n"/>
-      <c r="H45" s="1617" t="n">
+      <c r="D45" s="1653" t="n"/>
+      <c r="E45" s="1653" t="n"/>
+      <c r="F45" s="1653" t="n"/>
+      <c r="G45" s="1653" t="n"/>
+      <c r="H45" s="1653" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1618" t="n"/>
-      <c r="J45" s="1619" t="n"/>
-      <c r="K45" s="1619" t="n"/>
-      <c r="L45" s="1619" t="n"/>
-      <c r="M45" s="1617" t="n">
+      <c r="I45" s="1654" t="n"/>
+      <c r="J45" s="1655" t="n"/>
+      <c r="K45" s="1655" t="n"/>
+      <c r="L45" s="1655" t="n"/>
+      <c r="M45" s="1653" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1617" t="n">
+      <c r="N45" s="1653" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1617" t="n"/>
-      <c r="P45" s="1620" t="n"/>
-      <c r="Q45" s="1617" t="n"/>
-      <c r="R45" s="1617" t="n"/>
-      <c r="S45" s="1617" t="n"/>
+      <c r="O45" s="1653" t="n"/>
+      <c r="P45" s="1656" t="n"/>
+      <c r="Q45" s="1653" t="n"/>
+      <c r="R45" s="1653" t="n"/>
+      <c r="S45" s="1653" t="n"/>
       <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1616" t="n"/>
+      <c r="U45" s="1652" t="n"/>
       <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -7932,39 +8040,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1591" t="inlineStr">
+      <c r="A46" s="1627" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B46" s="1592" t="inlineStr">
+      <c r="B46" s="1628" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="C46" s="1592" t="inlineStr">
+      <c r="C46" s="1628" t="inlineStr">
         <is>
           <t>EVENT - Clean</t>
         </is>
       </c>
-      <c r="D46" s="1593" t="n"/>
-      <c r="E46" s="1593" t="n"/>
-      <c r="F46" s="1593" t="n"/>
-      <c r="G46" s="1593" t="n"/>
-      <c r="H46" s="1593" t="n"/>
-      <c r="I46" s="1594" t="n"/>
-      <c r="J46" s="1595" t="n"/>
-      <c r="K46" s="1595" t="n"/>
-      <c r="L46" s="1595" t="n"/>
-      <c r="M46" s="1593" t="n"/>
-      <c r="N46" s="1593" t="n"/>
-      <c r="O46" s="1593" t="n"/>
-      <c r="P46" s="1596" t="n"/>
-      <c r="Q46" s="1593" t="n"/>
-      <c r="R46" s="1593" t="n"/>
-      <c r="S46" s="1593" t="n"/>
+      <c r="D46" s="1629" t="n"/>
+      <c r="E46" s="1629" t="n"/>
+      <c r="F46" s="1629" t="n"/>
+      <c r="G46" s="1629" t="n"/>
+      <c r="H46" s="1629" t="n"/>
+      <c r="I46" s="1630" t="n"/>
+      <c r="J46" s="1631" t="n"/>
+      <c r="K46" s="1631" t="n"/>
+      <c r="L46" s="1631" t="n"/>
+      <c r="M46" s="1629" t="n"/>
+      <c r="N46" s="1629" t="n"/>
+      <c r="O46" s="1629" t="n"/>
+      <c r="P46" s="1632" t="n"/>
+      <c r="Q46" s="1629" t="n"/>
+      <c r="R46" s="1629" t="n"/>
+      <c r="S46" s="1629" t="n"/>
       <c r="T46" s="631" t="n"/>
-      <c r="U46" s="1592" t="n"/>
+      <c r="U46" s="1628" t="n"/>
       <c r="V46" s="632" t="inlineStr">
         <is>
           <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
@@ -7972,51 +8080,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1597" t="inlineStr">
+      <c r="A47" s="1633" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1598" t="inlineStr">
+      <c r="B47" s="1634" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C47" s="1598" t="inlineStr">
+      <c r="C47" s="1634" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D47" s="1599" t="n"/>
-      <c r="E47" s="1599" t="n">
+      <c r="D47" s="1635" t="n"/>
+      <c r="E47" s="1635" t="n">
         <v>16.6</v>
       </c>
-      <c r="F47" s="1599" t="n">
+      <c r="F47" s="1635" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="1599" t="n">
+      <c r="G47" s="1635" t="n">
         <v>4.1</v>
       </c>
-      <c r="H47" s="1599" t="n"/>
-      <c r="I47" s="1600" t="n">
+      <c r="H47" s="1635" t="n"/>
+      <c r="I47" s="1636" t="n">
         <v>0.9</v>
       </c>
-      <c r="J47" s="1601" t="n"/>
-      <c r="K47" s="1601" t="n"/>
-      <c r="L47" s="1601" t="n"/>
-      <c r="M47" s="1599" t="n"/>
-      <c r="N47" s="1599" t="n"/>
-      <c r="O47" s="1599" t="n">
+      <c r="J47" s="1637" t="n"/>
+      <c r="K47" s="1637" t="n"/>
+      <c r="L47" s="1637" t="n"/>
+      <c r="M47" s="1635" t="n"/>
+      <c r="N47" s="1635" t="n"/>
+      <c r="O47" s="1635" t="n">
         <v>13.2</v>
       </c>
-      <c r="P47" s="1602" t="n">
+      <c r="P47" s="1638" t="n">
         <v>0</v>
       </c>
-      <c r="Q47" s="1599" t="n"/>
-      <c r="R47" s="1599" t="n">
+      <c r="Q47" s="1635" t="n"/>
+      <c r="R47" s="1635" t="n">
         <v>84.5</v>
       </c>
-      <c r="S47" s="1599" t="n">
+      <c r="S47" s="1635" t="n">
         <v>11.8</v>
       </c>
       <c r="T47" s="813" t="inlineStr">
@@ -8024,7 +8132,7 @@
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1598" t="inlineStr">
+      <c r="U47" s="1634" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
@@ -8036,49 +8144,49 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1609" t="inlineStr">
+      <c r="A48" s="1645" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B48" s="1610" t="inlineStr">
+      <c r="B48" s="1646" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C48" s="1610" t="inlineStr">
+      <c r="C48" s="1646" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D48" s="1611" t="n"/>
-      <c r="E48" s="1611" t="n"/>
-      <c r="F48" s="1611" t="n"/>
-      <c r="G48" s="1611" t="n"/>
-      <c r="H48" s="1611" t="n">
+      <c r="D48" s="1647" t="n"/>
+      <c r="E48" s="1647" t="n"/>
+      <c r="F48" s="1647" t="n"/>
+      <c r="G48" s="1647" t="n"/>
+      <c r="H48" s="1647" t="n">
         <v>15.1</v>
       </c>
-      <c r="I48" s="1612" t="n"/>
-      <c r="J48" s="1613" t="n"/>
-      <c r="K48" s="1613" t="n"/>
-      <c r="L48" s="1613" t="n"/>
-      <c r="M48" s="1611" t="n">
+      <c r="I48" s="1648" t="n"/>
+      <c r="J48" s="1649" t="n"/>
+      <c r="K48" s="1649" t="n"/>
+      <c r="L48" s="1649" t="n"/>
+      <c r="M48" s="1647" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="1611" t="n">
+      <c r="N48" s="1647" t="n">
         <v>20</v>
       </c>
-      <c r="O48" s="1611" t="n"/>
-      <c r="P48" s="1614" t="n"/>
-      <c r="Q48" s="1611" t="n"/>
-      <c r="R48" s="1611" t="n"/>
-      <c r="S48" s="1611" t="n"/>
+      <c r="O48" s="1647" t="n"/>
+      <c r="P48" s="1650" t="n"/>
+      <c r="Q48" s="1647" t="n"/>
+      <c r="R48" s="1647" t="n"/>
+      <c r="S48" s="1647" t="n"/>
       <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U48" s="1610" t="n"/>
+      <c r="U48" s="1646" t="n"/>
       <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
@@ -8086,51 +8194,51 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1585" t="inlineStr">
+      <c r="A49" s="1621" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B49" s="1586" t="inlineStr">
+      <c r="B49" s="1622" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C49" s="1586" t="inlineStr">
+      <c r="C49" s="1622" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D49" s="1587" t="n"/>
-      <c r="E49" s="1587" t="n">
+      <c r="D49" s="1623" t="n"/>
+      <c r="E49" s="1623" t="n">
         <v>16.8</v>
       </c>
-      <c r="F49" s="1587" t="n">
+      <c r="F49" s="1623" t="n">
         <v>0.2</v>
       </c>
-      <c r="G49" s="1587" t="n">
+      <c r="G49" s="1623" t="n">
         <v>3.3</v>
       </c>
-      <c r="H49" s="1587" t="n"/>
-      <c r="I49" s="1588" t="n">
+      <c r="H49" s="1623" t="n"/>
+      <c r="I49" s="1624" t="n">
         <v>1.7</v>
       </c>
-      <c r="J49" s="1589" t="n"/>
-      <c r="K49" s="1589" t="n"/>
-      <c r="L49" s="1589" t="n"/>
-      <c r="M49" s="1587" t="n"/>
-      <c r="N49" s="1587" t="n"/>
-      <c r="O49" s="1587" t="n">
+      <c r="J49" s="1625" t="n"/>
+      <c r="K49" s="1625" t="n"/>
+      <c r="L49" s="1625" t="n"/>
+      <c r="M49" s="1623" t="n"/>
+      <c r="N49" s="1623" t="n"/>
+      <c r="O49" s="1623" t="n">
         <v>13</v>
       </c>
-      <c r="P49" s="1590" t="n">
+      <c r="P49" s="1626" t="n">
         <v>0.87</v>
       </c>
-      <c r="Q49" s="1587" t="n"/>
-      <c r="R49" s="1587" t="n">
+      <c r="Q49" s="1623" t="n"/>
+      <c r="R49" s="1623" t="n">
         <v>86</v>
       </c>
-      <c r="S49" s="1587" t="n">
+      <c r="S49" s="1623" t="n">
         <v>11.65</v>
       </c>
       <c r="T49" s="624" t="inlineStr">
@@ -8138,7 +8246,7 @@
           <t>Clear now, 88F, 67% RH; sun so far 6.4h of 7h daylight (91%); today high 90F, 0.87in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U49" s="1586" t="inlineStr">
+      <c r="U49" s="1622" t="inlineStr">
         <is>
           <t>2026-07-04_1.jpeg;2026-07-04_2.jpeg;2026-07-04_3.jpeg;2026-07-04_4.jpeg</t>
         </is>
@@ -8150,49 +8258,49 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1591" t="inlineStr">
+      <c r="A50" s="1627" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B50" s="1592" t="inlineStr">
+      <c r="B50" s="1628" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C50" s="1592" t="inlineStr">
+      <c r="C50" s="1628" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D50" s="1593" t="n"/>
-      <c r="E50" s="1593" t="n"/>
-      <c r="F50" s="1593" t="n"/>
-      <c r="G50" s="1593" t="n"/>
-      <c r="H50" s="1593" t="n">
+      <c r="D50" s="1629" t="n"/>
+      <c r="E50" s="1629" t="n"/>
+      <c r="F50" s="1629" t="n"/>
+      <c r="G50" s="1629" t="n"/>
+      <c r="H50" s="1629" t="n">
         <v>14.6</v>
       </c>
-      <c r="I50" s="1594" t="n"/>
-      <c r="J50" s="1595" t="n"/>
-      <c r="K50" s="1595" t="n"/>
-      <c r="L50" s="1595" t="n"/>
-      <c r="M50" s="1593" t="n">
+      <c r="I50" s="1630" t="n"/>
+      <c r="J50" s="1631" t="n"/>
+      <c r="K50" s="1631" t="n"/>
+      <c r="L50" s="1631" t="n"/>
+      <c r="M50" s="1629" t="n">
         <v>0.5</v>
       </c>
-      <c r="N50" s="1593" t="n">
+      <c r="N50" s="1629" t="n">
         <v>20.5</v>
       </c>
-      <c r="O50" s="1593" t="n"/>
-      <c r="P50" s="1596" t="n"/>
-      <c r="Q50" s="1593" t="n"/>
-      <c r="R50" s="1593" t="n"/>
-      <c r="S50" s="1593" t="n"/>
+      <c r="O50" s="1629" t="n"/>
+      <c r="P50" s="1632" t="n"/>
+      <c r="Q50" s="1629" t="n"/>
+      <c r="R50" s="1629" t="n"/>
+      <c r="S50" s="1629" t="n"/>
       <c r="T50" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny day (high 90F, water 86F); storm forecast overnight</t>
         </is>
       </c>
-      <c r="U50" s="1592" t="n"/>
+      <c r="U50" s="1628" t="n"/>
       <c r="V50" s="632" t="inlineStr">
         <is>
           <t>0.5 gal added 7:40 PM. PARTY PRE-LOAD (Sun 7/5 1PM picnic): deliberately HALF the usual dose -- FC already high at 16.8, and John didn't want to overshoot into the high teens for guests. Sized on the retuned model (l24_hot_sunny now 4.0). Model projects ~14.6 next noon, BUT this is a known weather-mismatch case: model keys L24 off today's hot/sunny weather, while the actual loss window is a storm overnight (no UV) + cooler/cloudy Sun morning -&gt; real loss will be LOWER, so FC likely lands ~15-16 at the party (comfortable top-of-band, cushion for bather load, not overboard). =&gt; If tomorrow's noon comes in ABOVE 14.6, that's the weather mismatch, NOT the freshly-retuned constant; don't chase it. Plan: dose back up Sun evening after the crowd's out (expect a bather-load FC drop). Season total 20.5 gal. PHOTOS(4): water clear/healthy blue, bottom fully visible, no cloudiness/algae; yesterday's surface debris now gone (tracks with CC clearing to 0.2); liner step close-up normal speckled blue, no rust/stain progression. Ruler photo documents the ~11.65 cm level.</t>
@@ -8200,47 +8308,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1597" t="inlineStr">
+      <c r="A51" s="1633" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B51" s="1598" t="inlineStr">
+      <c r="B51" s="1634" t="inlineStr">
         <is>
           <t>07:45</t>
         </is>
       </c>
-      <c r="C51" s="1598" t="inlineStr">
+      <c r="C51" s="1634" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D51" s="1599" t="n"/>
-      <c r="E51" s="1599" t="n">
+      <c r="D51" s="1635" t="n"/>
+      <c r="E51" s="1635" t="n">
         <v>16</v>
       </c>
-      <c r="F51" s="1599" t="n">
+      <c r="F51" s="1635" t="n">
         <v>0.5</v>
       </c>
-      <c r="G51" s="1599" t="n"/>
-      <c r="H51" s="1599" t="n"/>
-      <c r="I51" s="1600" t="n">
+      <c r="G51" s="1635" t="n"/>
+      <c r="H51" s="1635" t="n"/>
+      <c r="I51" s="1636" t="n">
         <v>1.4</v>
       </c>
-      <c r="J51" s="1601" t="n"/>
-      <c r="K51" s="1601" t="n"/>
-      <c r="L51" s="1601" t="n"/>
-      <c r="M51" s="1599" t="n"/>
-      <c r="N51" s="1599" t="n"/>
-      <c r="O51" s="1599" t="n"/>
-      <c r="P51" s="1602" t="n">
+      <c r="J51" s="1637" t="n"/>
+      <c r="K51" s="1637" t="n"/>
+      <c r="L51" s="1637" t="n"/>
+      <c r="M51" s="1635" t="n"/>
+      <c r="N51" s="1635" t="n"/>
+      <c r="O51" s="1635" t="n"/>
+      <c r="P51" s="1638" t="n">
         <v>0.04</v>
       </c>
-      <c r="Q51" s="1599" t="n"/>
-      <c r="R51" s="1599" t="n">
+      <c r="Q51" s="1635" t="n"/>
+      <c r="R51" s="1635" t="n">
         <v>84</v>
       </c>
-      <c r="S51" s="1599" t="n">
+      <c r="S51" s="1635" t="n">
         <v>13.9</v>
       </c>
       <c r="T51" s="813" t="inlineStr">
@@ -8248,7 +8356,7 @@
           <t>Overcast now, 75F, 90% RH; sun so far 0.0h of 3h daylight (0%); today high 75F, 0.04in precip, UV max 6.5</t>
         </is>
       </c>
-      <c r="U51" s="1598" t="inlineStr">
+      <c r="U51" s="1634" t="inlineStr">
         <is>
           <t>2026-07-05_2.jpeg</t>
         </is>
@@ -8260,41 +8368,41 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1603" t="inlineStr">
+      <c r="A52" s="1639" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B52" s="1604" t="inlineStr">
+      <c r="B52" s="1640" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C52" s="1604" t="inlineStr">
+      <c r="C52" s="1640" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D52" s="1605" t="n"/>
-      <c r="E52" s="1605" t="n">
+      <c r="D52" s="1641" t="n"/>
+      <c r="E52" s="1641" t="n">
         <v>14.8</v>
       </c>
-      <c r="F52" s="1605" t="n">
+      <c r="F52" s="1641" t="n">
         <v>0.3</v>
       </c>
-      <c r="G52" s="1605" t="n"/>
-      <c r="H52" s="1605" t="n"/>
-      <c r="I52" s="1606" t="n"/>
-      <c r="J52" s="1607" t="n"/>
-      <c r="K52" s="1607" t="n"/>
-      <c r="L52" s="1607" t="n"/>
-      <c r="M52" s="1605" t="n"/>
-      <c r="N52" s="1605" t="n"/>
-      <c r="O52" s="1605" t="n"/>
-      <c r="P52" s="1608" t="n"/>
-      <c r="Q52" s="1605" t="n"/>
-      <c r="R52" s="1605" t="n"/>
-      <c r="S52" s="1605" t="n">
+      <c r="G52" s="1641" t="n"/>
+      <c r="H52" s="1641" t="n"/>
+      <c r="I52" s="1642" t="n"/>
+      <c r="J52" s="1643" t="n"/>
+      <c r="K52" s="1643" t="n"/>
+      <c r="L52" s="1643" t="n"/>
+      <c r="M52" s="1641" t="n"/>
+      <c r="N52" s="1641" t="n"/>
+      <c r="O52" s="1641" t="n"/>
+      <c r="P52" s="1644" t="n"/>
+      <c r="Q52" s="1641" t="n"/>
+      <c r="R52" s="1641" t="n"/>
+      <c r="S52" s="1641" t="n">
         <v>13.6</v>
       </c>
       <c r="T52" s="820" t="inlineStr">
@@ -8302,7 +8410,7 @@
           <t>Overcast now, 72F, 76% RH; sun so far 8.4h of 13h daylight (65%); today high 80F, 0.00in precip, UV max 6.0</t>
         </is>
       </c>
-      <c r="U52" s="1604" t="inlineStr">
+      <c r="U52" s="1640" t="inlineStr">
         <is>
           <t>2026-07-05_1.jpeg;2026-07-05_3.jpeg</t>
         </is>
@@ -8314,49 +8422,49 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1609" t="inlineStr">
+      <c r="A53" s="1645" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B53" s="1610" t="inlineStr">
+      <c r="B53" s="1646" t="inlineStr">
         <is>
           <t>19:25</t>
         </is>
       </c>
-      <c r="C53" s="1610" t="inlineStr">
+      <c r="C53" s="1646" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D53" s="1611" t="n"/>
-      <c r="E53" s="1611" t="n"/>
-      <c r="F53" s="1611" t="n"/>
-      <c r="G53" s="1611" t="n"/>
-      <c r="H53" s="1611" t="n">
+      <c r="D53" s="1647" t="n"/>
+      <c r="E53" s="1647" t="n"/>
+      <c r="F53" s="1647" t="n"/>
+      <c r="G53" s="1647" t="n"/>
+      <c r="H53" s="1647" t="n">
         <v>15.1</v>
       </c>
-      <c r="I53" s="1612" t="n"/>
-      <c r="J53" s="1613" t="n"/>
-      <c r="K53" s="1613" t="n"/>
-      <c r="L53" s="1613" t="n"/>
-      <c r="M53" s="1611" t="n">
+      <c r="I53" s="1648" t="n"/>
+      <c r="J53" s="1649" t="n"/>
+      <c r="K53" s="1649" t="n"/>
+      <c r="L53" s="1649" t="n"/>
+      <c r="M53" s="1647" t="n">
         <v>0.5</v>
       </c>
-      <c r="N53" s="1611" t="n">
+      <c r="N53" s="1647" t="n">
         <v>21</v>
       </c>
-      <c r="O53" s="1611" t="n"/>
-      <c r="P53" s="1614" t="n"/>
-      <c r="Q53" s="1611" t="n"/>
-      <c r="R53" s="1611" t="n"/>
-      <c r="S53" s="1611" t="n"/>
+      <c r="O53" s="1647" t="n"/>
+      <c r="P53" s="1650" t="n"/>
+      <c r="Q53" s="1647" t="n"/>
+      <c r="R53" s="1647" t="n"/>
+      <c r="S53" s="1647" t="n"/>
       <c r="T53" s="827" t="inlineStr">
         <is>
           <t>Cleared to partly sunny (8.4 sun hrs, high 80F, water 84F); all-day rain forecast Mon 7/6</t>
         </is>
       </c>
-      <c r="U53" s="1610" t="n"/>
+      <c r="U53" s="1646" t="n"/>
       <c r="V53" s="828" t="inlineStr">
         <is>
           <t>0.5 gal added 7:25 PM (post-party recovery dose). Sized on TOMORROW's rainy forecast (the real loss window: overcast/wet 7/6, ~0.9in rain, low UV) not today's sun -&gt; projects ~15.1 at Mon noon. Party went great (FC held 16.0-&gt;14.8, CC dropped 0.5-&gt;0.3). Season total 21.0 gal. This is the first prediction that deliberately used the next-day forecast for L24 instead of the model's default (today's weather as proxy) -- if it lands near 15.1 tomorrow, that validates feeding the forecast on weather-change days.</t>
@@ -8364,49 +8472,49 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1585" t="inlineStr">
+      <c r="A54" s="1621" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B54" s="1586" t="inlineStr">
+      <c r="B54" s="1622" t="inlineStr">
         <is>
           <t>11:40</t>
         </is>
       </c>
-      <c r="C54" s="1586" t="inlineStr">
+      <c r="C54" s="1622" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D54" s="1587" t="n"/>
-      <c r="E54" s="1587" t="n">
+      <c r="D54" s="1623" t="n"/>
+      <c r="E54" s="1623" t="n">
         <v>13.8</v>
       </c>
-      <c r="F54" s="1587" t="n">
+      <c r="F54" s="1623" t="n">
         <v>0.2</v>
       </c>
-      <c r="G54" s="1587" t="n"/>
-      <c r="H54" s="1587" t="n"/>
-      <c r="I54" s="1588" t="n">
+      <c r="G54" s="1623" t="n"/>
+      <c r="H54" s="1623" t="n"/>
+      <c r="I54" s="1624" t="n">
         <v>-1.3</v>
       </c>
-      <c r="J54" s="1589" t="n"/>
-      <c r="K54" s="1589" t="n"/>
-      <c r="L54" s="1589" t="n"/>
-      <c r="M54" s="1587" t="n"/>
-      <c r="N54" s="1587" t="n"/>
-      <c r="O54" s="1587" t="n">
+      <c r="J54" s="1625" t="n"/>
+      <c r="K54" s="1625" t="n"/>
+      <c r="L54" s="1625" t="n"/>
+      <c r="M54" s="1623" t="n"/>
+      <c r="N54" s="1623" t="n"/>
+      <c r="O54" s="1623" t="n">
         <v>0</v>
       </c>
-      <c r="P54" s="1590" t="n">
+      <c r="P54" s="1626" t="n">
         <v>2</v>
       </c>
-      <c r="Q54" s="1587" t="n"/>
-      <c r="R54" s="1587" t="n">
+      <c r="Q54" s="1623" t="n"/>
+      <c r="R54" s="1623" t="n">
         <v>81</v>
       </c>
-      <c r="S54" s="1587" t="n">
+      <c r="S54" s="1623" t="n">
         <v>15.1</v>
       </c>
       <c r="T54" s="624" t="inlineStr">
@@ -8414,7 +8522,7 @@
           <t>Light rain now, 65F, 93% RH; sun so far 0.0h of 6h daylight (0%); today high 68F, 2.00in precip, UV max 0.5</t>
         </is>
       </c>
-      <c r="U54" s="1586" t="inlineStr">
+      <c r="U54" s="1622" t="inlineStr">
         <is>
           <t>2026-07-06_1.jpeg</t>
         </is>
@@ -8426,39 +8534,39 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1615" t="inlineStr">
+      <c r="A55" s="1651" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B55" s="1616" t="inlineStr">
+      <c r="B55" s="1652" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="C55" s="1616" t="inlineStr">
+      <c r="C55" s="1652" t="inlineStr">
         <is>
           <t>EVENT - Waste</t>
         </is>
       </c>
-      <c r="D55" s="1617" t="n"/>
-      <c r="E55" s="1617" t="n"/>
-      <c r="F55" s="1617" t="n"/>
-      <c r="G55" s="1617" t="n"/>
-      <c r="H55" s="1617" t="n"/>
-      <c r="I55" s="1618" t="n"/>
-      <c r="J55" s="1619" t="n"/>
-      <c r="K55" s="1619" t="n"/>
-      <c r="L55" s="1619" t="n"/>
-      <c r="M55" s="1617" t="n"/>
-      <c r="N55" s="1617" t="n"/>
-      <c r="O55" s="1617" t="n"/>
-      <c r="P55" s="1620" t="n"/>
-      <c r="Q55" s="1617" t="n"/>
-      <c r="R55" s="1617" t="n"/>
-      <c r="S55" s="1617" t="n"/>
+      <c r="D55" s="1653" t="n"/>
+      <c r="E55" s="1653" t="n"/>
+      <c r="F55" s="1653" t="n"/>
+      <c r="G55" s="1653" t="n"/>
+      <c r="H55" s="1653" t="n"/>
+      <c r="I55" s="1654" t="n"/>
+      <c r="J55" s="1655" t="n"/>
+      <c r="K55" s="1655" t="n"/>
+      <c r="L55" s="1655" t="n"/>
+      <c r="M55" s="1653" t="n"/>
+      <c r="N55" s="1653" t="n"/>
+      <c r="O55" s="1653" t="n"/>
+      <c r="P55" s="1656" t="n"/>
+      <c r="Q55" s="1653" t="n"/>
+      <c r="R55" s="1653" t="n"/>
+      <c r="S55" s="1653" t="n"/>
       <c r="T55" s="659" t="n"/>
-      <c r="U55" s="1616" t="inlineStr">
+      <c r="U55" s="1652" t="inlineStr">
         <is>
           <t>2026-07-06_2.jpeg;2026-07-06_3.jpeg</t>
         </is>
@@ -8470,49 +8578,49 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1591" t="inlineStr">
+      <c r="A56" s="1627" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B56" s="1592" t="inlineStr">
+      <c r="B56" s="1628" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C56" s="1592" t="inlineStr">
+      <c r="C56" s="1628" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D56" s="1593" t="n"/>
-      <c r="E56" s="1593" t="n"/>
-      <c r="F56" s="1593" t="n"/>
-      <c r="G56" s="1593" t="n"/>
-      <c r="H56" s="1593" t="n">
+      <c r="D56" s="1629" t="n"/>
+      <c r="E56" s="1629" t="n"/>
+      <c r="F56" s="1629" t="n"/>
+      <c r="G56" s="1629" t="n"/>
+      <c r="H56" s="1629" t="n">
         <v>14</v>
       </c>
-      <c r="I56" s="1594" t="n"/>
-      <c r="J56" s="1595" t="n"/>
-      <c r="K56" s="1595" t="n"/>
-      <c r="L56" s="1595" t="n"/>
-      <c r="M56" s="1593" t="n">
+      <c r="I56" s="1630" t="n"/>
+      <c r="J56" s="1631" t="n"/>
+      <c r="K56" s="1631" t="n"/>
+      <c r="L56" s="1631" t="n"/>
+      <c r="M56" s="1629" t="n">
         <v>1</v>
       </c>
-      <c r="N56" s="1593" t="n">
+      <c r="N56" s="1629" t="n">
         <v>22</v>
       </c>
-      <c r="O56" s="1593" t="n"/>
-      <c r="P56" s="1596" t="n"/>
-      <c r="Q56" s="1593" t="n"/>
-      <c r="R56" s="1593" t="n"/>
-      <c r="S56" s="1593" t="n"/>
+      <c r="O56" s="1629" t="n"/>
+      <c r="P56" s="1632" t="n"/>
+      <c r="Q56" s="1629" t="n"/>
+      <c r="R56" s="1629" t="n"/>
+      <c r="S56" s="1629" t="n"/>
       <c r="T56" s="631" t="inlineStr">
         <is>
           <t>Rain all day (2.00in total), overcast, 65-68F; more rain Tue</t>
         </is>
       </c>
-      <c r="U56" s="1592" t="n"/>
+      <c r="U56" s="1628" t="n"/>
       <c r="V56" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added 7:30 PM, AFTER the pump-to-waste (correct order -- don't chlorinate water you're about to pump out). FIRST dose on the recalibrated buckets (rain L24 now 2.5 vs old 1.5). CORRECTION carried in: John is NOT low on chlorine -- he was low on TEST REAGENTS, which arrived today -- so this is the full 1 gal (not the 0.5 I'd wrongly trimmed for 'conservation'). Base FC ~13 est (noon 13.8 minus the bit of FC removed by the pump-out; not re-tested), + 1gal x3.5 - 2.5 rain loss -&gt; pred ~14.0 at Tue noon. Prediction is confounded this round (pump perturbation + no post-empty FC test) -&gt; tomorrow's error will be noisy, don't read too much into it for bucket validation. Season total 22.0 gal.</t>

</xml_diff>

<commit_message>
Log 2026-07-07 noon TEST: FC 14.6, CC 0.8, level 15.5; pred +0.6 (first rainy-day noon on recalibrated 2.5 bucket)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1657">
+  <cellXfs count="1699">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -5498,6 +5498,132 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5759,7 +5885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V56"/>
+  <dimension ref="A1:V57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -5936,35 +6062,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1621" t="inlineStr">
+      <c r="A3" s="1657" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1622" t="n"/>
-      <c r="C3" s="1622" t="inlineStr">
+      <c r="B3" s="1658" t="n"/>
+      <c r="C3" s="1658" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1623" t="n"/>
-      <c r="E3" s="1623" t="n"/>
-      <c r="F3" s="1623" t="n"/>
-      <c r="G3" s="1623" t="n"/>
-      <c r="H3" s="1623" t="n"/>
-      <c r="I3" s="1624" t="n"/>
-      <c r="J3" s="1625" t="n"/>
-      <c r="K3" s="1625" t="n"/>
-      <c r="L3" s="1625" t="n"/>
-      <c r="M3" s="1623" t="n"/>
-      <c r="N3" s="1623" t="n"/>
-      <c r="O3" s="1623" t="n"/>
-      <c r="P3" s="1626" t="n"/>
-      <c r="Q3" s="1623" t="n"/>
-      <c r="R3" s="1623" t="n"/>
-      <c r="S3" s="1623" t="n"/>
+      <c r="D3" s="1659" t="n"/>
+      <c r="E3" s="1659" t="n"/>
+      <c r="F3" s="1659" t="n"/>
+      <c r="G3" s="1659" t="n"/>
+      <c r="H3" s="1659" t="n"/>
+      <c r="I3" s="1660" t="n"/>
+      <c r="J3" s="1661" t="n"/>
+      <c r="K3" s="1661" t="n"/>
+      <c r="L3" s="1661" t="n"/>
+      <c r="M3" s="1659" t="n"/>
+      <c r="N3" s="1659" t="n"/>
+      <c r="O3" s="1659" t="n"/>
+      <c r="P3" s="1662" t="n"/>
+      <c r="Q3" s="1659" t="n"/>
+      <c r="R3" s="1659" t="n"/>
+      <c r="S3" s="1659" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1622" t="n"/>
+      <c r="U3" s="1658" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -5972,43 +6098,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1627" t="inlineStr">
+      <c r="A4" s="1663" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1628" t="inlineStr">
+      <c r="B4" s="1664" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1628" t="inlineStr">
+      <c r="C4" s="1664" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1629" t="n"/>
-      <c r="E4" s="1629" t="n"/>
-      <c r="F4" s="1629" t="n"/>
-      <c r="G4" s="1629" t="n"/>
-      <c r="H4" s="1629" t="n"/>
-      <c r="I4" s="1630" t="n"/>
-      <c r="J4" s="1631" t="n"/>
-      <c r="K4" s="1631" t="n"/>
-      <c r="L4" s="1631" t="n"/>
-      <c r="M4" s="1629" t="n">
+      <c r="D4" s="1665" t="n"/>
+      <c r="E4" s="1665" t="n"/>
+      <c r="F4" s="1665" t="n"/>
+      <c r="G4" s="1665" t="n"/>
+      <c r="H4" s="1665" t="n"/>
+      <c r="I4" s="1666" t="n"/>
+      <c r="J4" s="1667" t="n"/>
+      <c r="K4" s="1667" t="n"/>
+      <c r="L4" s="1667" t="n"/>
+      <c r="M4" s="1665" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1629" t="n">
+      <c r="N4" s="1665" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1629" t="n"/>
-      <c r="P4" s="1632" t="n"/>
-      <c r="Q4" s="1629" t="n"/>
-      <c r="R4" s="1629" t="n"/>
-      <c r="S4" s="1629" t="n"/>
+      <c r="O4" s="1665" t="n"/>
+      <c r="P4" s="1668" t="n"/>
+      <c r="Q4" s="1665" t="n"/>
+      <c r="R4" s="1665" t="n"/>
+      <c r="S4" s="1665" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1628" t="n"/>
+      <c r="U4" s="1664" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -6016,57 +6142,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1633" t="inlineStr">
+      <c r="A5" s="1669" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1634" t="inlineStr">
+      <c r="B5" s="1670" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1634" t="inlineStr">
+      <c r="C5" s="1670" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1635" t="n">
+      <c r="D5" s="1671" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1635" t="n">
+      <c r="E5" s="1671" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1635" t="n">
+      <c r="F5" s="1671" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1635" t="n"/>
-      <c r="H5" s="1635" t="n"/>
-      <c r="I5" s="1636" t="n"/>
-      <c r="J5" s="1637" t="n">
+      <c r="G5" s="1671" t="n"/>
+      <c r="H5" s="1671" t="n"/>
+      <c r="I5" s="1672" t="n"/>
+      <c r="J5" s="1673" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1637" t="n">
+      <c r="K5" s="1673" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1637" t="inlineStr">
+      <c r="L5" s="1673" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1635" t="n"/>
-      <c r="N5" s="1635" t="n"/>
-      <c r="O5" s="1635" t="n">
+      <c r="M5" s="1671" t="n"/>
+      <c r="N5" s="1671" t="n"/>
+      <c r="O5" s="1671" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1638" t="n">
+      <c r="P5" s="1674" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1635" t="n"/>
-      <c r="R5" s="1635" t="n"/>
-      <c r="S5" s="1635" t="n"/>
+      <c r="Q5" s="1671" t="n"/>
+      <c r="R5" s="1671" t="n"/>
+      <c r="S5" s="1671" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1634" t="n"/>
+      <c r="U5" s="1670" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -6074,43 +6200,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1639" t="inlineStr">
+      <c r="A6" s="1675" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1640" t="inlineStr">
+      <c r="B6" s="1676" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1640" t="inlineStr">
+      <c r="C6" s="1676" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1641" t="n"/>
-      <c r="E6" s="1641" t="n"/>
-      <c r="F6" s="1641" t="n"/>
-      <c r="G6" s="1641" t="n"/>
-      <c r="H6" s="1641" t="n"/>
-      <c r="I6" s="1642" t="n"/>
-      <c r="J6" s="1643" t="n"/>
-      <c r="K6" s="1643" t="n"/>
-      <c r="L6" s="1643" t="n"/>
-      <c r="M6" s="1641" t="n">
+      <c r="D6" s="1677" t="n"/>
+      <c r="E6" s="1677" t="n"/>
+      <c r="F6" s="1677" t="n"/>
+      <c r="G6" s="1677" t="n"/>
+      <c r="H6" s="1677" t="n"/>
+      <c r="I6" s="1678" t="n"/>
+      <c r="J6" s="1679" t="n"/>
+      <c r="K6" s="1679" t="n"/>
+      <c r="L6" s="1679" t="n"/>
+      <c r="M6" s="1677" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1641" t="n">
+      <c r="N6" s="1677" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1641" t="n"/>
-      <c r="P6" s="1644" t="n"/>
-      <c r="Q6" s="1641" t="n"/>
-      <c r="R6" s="1641" t="n"/>
-      <c r="S6" s="1641" t="n"/>
+      <c r="O6" s="1677" t="n"/>
+      <c r="P6" s="1680" t="n"/>
+      <c r="Q6" s="1677" t="n"/>
+      <c r="R6" s="1677" t="n"/>
+      <c r="S6" s="1677" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1640" t="n"/>
+      <c r="U6" s="1676" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -6118,39 +6244,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1645" t="inlineStr">
+      <c r="A7" s="1681" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1646" t="inlineStr">
+      <c r="B7" s="1682" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1646" t="inlineStr">
+      <c r="C7" s="1682" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1647" t="n"/>
-      <c r="E7" s="1647" t="n"/>
-      <c r="F7" s="1647" t="n"/>
-      <c r="G7" s="1647" t="n"/>
-      <c r="H7" s="1647" t="n"/>
-      <c r="I7" s="1648" t="n"/>
-      <c r="J7" s="1649" t="n"/>
-      <c r="K7" s="1649" t="n"/>
-      <c r="L7" s="1649" t="n"/>
-      <c r="M7" s="1647" t="n"/>
-      <c r="N7" s="1647" t="n"/>
-      <c r="O7" s="1647" t="n"/>
-      <c r="P7" s="1650" t="n"/>
-      <c r="Q7" s="1647" t="n"/>
-      <c r="R7" s="1647" t="n"/>
-      <c r="S7" s="1647" t="n"/>
+      <c r="D7" s="1683" t="n"/>
+      <c r="E7" s="1683" t="n"/>
+      <c r="F7" s="1683" t="n"/>
+      <c r="G7" s="1683" t="n"/>
+      <c r="H7" s="1683" t="n"/>
+      <c r="I7" s="1684" t="n"/>
+      <c r="J7" s="1685" t="n"/>
+      <c r="K7" s="1685" t="n"/>
+      <c r="L7" s="1685" t="n"/>
+      <c r="M7" s="1683" t="n"/>
+      <c r="N7" s="1683" t="n"/>
+      <c r="O7" s="1683" t="n"/>
+      <c r="P7" s="1686" t="n"/>
+      <c r="Q7" s="1683" t="n"/>
+      <c r="R7" s="1683" t="n"/>
+      <c r="S7" s="1683" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1646" t="n"/>
+      <c r="U7" s="1682" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -6158,39 +6284,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1621" t="inlineStr">
+      <c r="A8" s="1657" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1622" t="inlineStr">
+      <c r="B8" s="1658" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1622" t="inlineStr">
+      <c r="C8" s="1658" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1623" t="n"/>
-      <c r="E8" s="1623" t="n"/>
-      <c r="F8" s="1623" t="n"/>
-      <c r="G8" s="1623" t="n"/>
-      <c r="H8" s="1623" t="n"/>
-      <c r="I8" s="1624" t="n"/>
-      <c r="J8" s="1625" t="n"/>
-      <c r="K8" s="1625" t="n"/>
-      <c r="L8" s="1625" t="n"/>
-      <c r="M8" s="1623" t="n"/>
-      <c r="N8" s="1623" t="n"/>
-      <c r="O8" s="1623" t="n"/>
-      <c r="P8" s="1626" t="n"/>
-      <c r="Q8" s="1623" t="n"/>
-      <c r="R8" s="1623" t="n"/>
-      <c r="S8" s="1623" t="n"/>
+      <c r="D8" s="1659" t="n"/>
+      <c r="E8" s="1659" t="n"/>
+      <c r="F8" s="1659" t="n"/>
+      <c r="G8" s="1659" t="n"/>
+      <c r="H8" s="1659" t="n"/>
+      <c r="I8" s="1660" t="n"/>
+      <c r="J8" s="1661" t="n"/>
+      <c r="K8" s="1661" t="n"/>
+      <c r="L8" s="1661" t="n"/>
+      <c r="M8" s="1659" t="n"/>
+      <c r="N8" s="1659" t="n"/>
+      <c r="O8" s="1659" t="n"/>
+      <c r="P8" s="1662" t="n"/>
+      <c r="Q8" s="1659" t="n"/>
+      <c r="R8" s="1659" t="n"/>
+      <c r="S8" s="1659" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1622" t="n"/>
+      <c r="U8" s="1658" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -6198,63 +6324,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1651" t="inlineStr">
+      <c r="A9" s="1687" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1652" t="inlineStr">
+      <c r="B9" s="1688" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1652" t="inlineStr">
+      <c r="C9" s="1688" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1653" t="n">
+      <c r="D9" s="1689" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1653" t="n">
+      <c r="E9" s="1689" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1653" t="n">
+      <c r="F9" s="1689" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1653" t="n">
+      <c r="G9" s="1689" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1653" t="n"/>
-      <c r="I9" s="1654" t="n"/>
-      <c r="J9" s="1655" t="n">
+      <c r="H9" s="1689" t="n"/>
+      <c r="I9" s="1690" t="n"/>
+      <c r="J9" s="1691" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1655" t="n">
+      <c r="K9" s="1691" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1655" t="inlineStr">
+      <c r="L9" s="1691" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1653" t="n"/>
-      <c r="N9" s="1653" t="n"/>
-      <c r="O9" s="1653" t="n">
+      <c r="M9" s="1689" t="n"/>
+      <c r="N9" s="1689" t="n"/>
+      <c r="O9" s="1689" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1656" t="n">
+      <c r="P9" s="1692" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1653" t="n"/>
-      <c r="R9" s="1653" t="n"/>
-      <c r="S9" s="1653" t="n"/>
+      <c r="Q9" s="1689" t="n"/>
+      <c r="R9" s="1689" t="n"/>
+      <c r="S9" s="1689" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1652" t="n"/>
+      <c r="U9" s="1688" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -6262,43 +6388,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1651" t="inlineStr">
+      <c r="A10" s="1687" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1652" t="inlineStr">
+      <c r="B10" s="1688" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1652" t="inlineStr">
+      <c r="C10" s="1688" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1653" t="n"/>
-      <c r="E10" s="1653" t="n"/>
-      <c r="F10" s="1653" t="n"/>
-      <c r="G10" s="1653" t="n"/>
-      <c r="H10" s="1653" t="n"/>
-      <c r="I10" s="1654" t="n"/>
-      <c r="J10" s="1655" t="n"/>
-      <c r="K10" s="1655" t="n"/>
-      <c r="L10" s="1655" t="inlineStr">
+      <c r="D10" s="1689" t="n"/>
+      <c r="E10" s="1689" t="n"/>
+      <c r="F10" s="1689" t="n"/>
+      <c r="G10" s="1689" t="n"/>
+      <c r="H10" s="1689" t="n"/>
+      <c r="I10" s="1690" t="n"/>
+      <c r="J10" s="1691" t="n"/>
+      <c r="K10" s="1691" t="n"/>
+      <c r="L10" s="1691" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1653" t="n"/>
-      <c r="N10" s="1653" t="n"/>
-      <c r="O10" s="1653" t="n"/>
-      <c r="P10" s="1656" t="n"/>
-      <c r="Q10" s="1653" t="n"/>
-      <c r="R10" s="1653" t="n"/>
-      <c r="S10" s="1653" t="n"/>
+      <c r="M10" s="1689" t="n"/>
+      <c r="N10" s="1689" t="n"/>
+      <c r="O10" s="1689" t="n"/>
+      <c r="P10" s="1692" t="n"/>
+      <c r="Q10" s="1689" t="n"/>
+      <c r="R10" s="1689" t="n"/>
+      <c r="S10" s="1689" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1652" t="n"/>
+      <c r="U10" s="1688" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -6306,43 +6432,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1651" t="inlineStr">
+      <c r="A11" s="1687" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1652" t="inlineStr">
+      <c r="B11" s="1688" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1652" t="inlineStr">
+      <c r="C11" s="1688" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1653" t="n"/>
-      <c r="E11" s="1653" t="n"/>
-      <c r="F11" s="1653" t="n"/>
-      <c r="G11" s="1653" t="n"/>
-      <c r="H11" s="1653" t="n"/>
-      <c r="I11" s="1654" t="n"/>
-      <c r="J11" s="1655" t="n"/>
-      <c r="K11" s="1655" t="n"/>
-      <c r="L11" s="1655" t="n"/>
-      <c r="M11" s="1653" t="n">
+      <c r="D11" s="1689" t="n"/>
+      <c r="E11" s="1689" t="n"/>
+      <c r="F11" s="1689" t="n"/>
+      <c r="G11" s="1689" t="n"/>
+      <c r="H11" s="1689" t="n"/>
+      <c r="I11" s="1690" t="n"/>
+      <c r="J11" s="1691" t="n"/>
+      <c r="K11" s="1691" t="n"/>
+      <c r="L11" s="1691" t="n"/>
+      <c r="M11" s="1689" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1653" t="n">
+      <c r="N11" s="1689" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1653" t="n"/>
-      <c r="P11" s="1656" t="n"/>
-      <c r="Q11" s="1653" t="n"/>
-      <c r="R11" s="1653" t="n"/>
-      <c r="S11" s="1653" t="n"/>
+      <c r="O11" s="1689" t="n"/>
+      <c r="P11" s="1692" t="n"/>
+      <c r="Q11" s="1689" t="n"/>
+      <c r="R11" s="1689" t="n"/>
+      <c r="S11" s="1689" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1652" t="n"/>
+      <c r="U11" s="1688" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -6350,39 +6476,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1627" t="inlineStr">
+      <c r="A12" s="1663" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1628" t="inlineStr">
+      <c r="B12" s="1664" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1628" t="inlineStr">
+      <c r="C12" s="1664" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1629" t="n"/>
-      <c r="E12" s="1629" t="n"/>
-      <c r="F12" s="1629" t="n"/>
-      <c r="G12" s="1629" t="n"/>
-      <c r="H12" s="1629" t="n"/>
-      <c r="I12" s="1630" t="n"/>
-      <c r="J12" s="1631" t="n"/>
-      <c r="K12" s="1631" t="n"/>
-      <c r="L12" s="1631" t="n"/>
-      <c r="M12" s="1629" t="n"/>
-      <c r="N12" s="1629" t="n"/>
-      <c r="O12" s="1629" t="n"/>
-      <c r="P12" s="1632" t="n"/>
-      <c r="Q12" s="1629" t="n"/>
-      <c r="R12" s="1629" t="n"/>
-      <c r="S12" s="1629" t="n"/>
+      <c r="D12" s="1665" t="n"/>
+      <c r="E12" s="1665" t="n"/>
+      <c r="F12" s="1665" t="n"/>
+      <c r="G12" s="1665" t="n"/>
+      <c r="H12" s="1665" t="n"/>
+      <c r="I12" s="1666" t="n"/>
+      <c r="J12" s="1667" t="n"/>
+      <c r="K12" s="1667" t="n"/>
+      <c r="L12" s="1667" t="n"/>
+      <c r="M12" s="1665" t="n"/>
+      <c r="N12" s="1665" t="n"/>
+      <c r="O12" s="1665" t="n"/>
+      <c r="P12" s="1668" t="n"/>
+      <c r="Q12" s="1665" t="n"/>
+      <c r="R12" s="1665" t="n"/>
+      <c r="S12" s="1665" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1628" t="n"/>
+      <c r="U12" s="1664" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -6390,35 +6516,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1633" t="inlineStr">
+      <c r="A13" s="1669" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1634" t="n"/>
-      <c r="C13" s="1634" t="inlineStr">
+      <c r="B13" s="1670" t="n"/>
+      <c r="C13" s="1670" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1635" t="n"/>
-      <c r="E13" s="1635" t="n"/>
-      <c r="F13" s="1635" t="n"/>
-      <c r="G13" s="1635" t="n"/>
-      <c r="H13" s="1635" t="n"/>
-      <c r="I13" s="1636" t="n"/>
-      <c r="J13" s="1637" t="n"/>
-      <c r="K13" s="1637" t="n"/>
-      <c r="L13" s="1637" t="n"/>
-      <c r="M13" s="1635" t="n"/>
-      <c r="N13" s="1635" t="n"/>
-      <c r="O13" s="1635" t="n"/>
-      <c r="P13" s="1638" t="n"/>
-      <c r="Q13" s="1635" t="n"/>
-      <c r="R13" s="1635" t="n"/>
-      <c r="S13" s="1635" t="n"/>
+      <c r="D13" s="1671" t="n"/>
+      <c r="E13" s="1671" t="n"/>
+      <c r="F13" s="1671" t="n"/>
+      <c r="G13" s="1671" t="n"/>
+      <c r="H13" s="1671" t="n"/>
+      <c r="I13" s="1672" t="n"/>
+      <c r="J13" s="1673" t="n"/>
+      <c r="K13" s="1673" t="n"/>
+      <c r="L13" s="1673" t="n"/>
+      <c r="M13" s="1671" t="n"/>
+      <c r="N13" s="1671" t="n"/>
+      <c r="O13" s="1671" t="n"/>
+      <c r="P13" s="1674" t="n"/>
+      <c r="Q13" s="1671" t="n"/>
+      <c r="R13" s="1671" t="n"/>
+      <c r="S13" s="1671" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1634" t="n"/>
+      <c r="U13" s="1670" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -6426,53 +6552,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1639" t="inlineStr">
+      <c r="A14" s="1675" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1640" t="inlineStr">
+      <c r="B14" s="1676" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1640" t="inlineStr">
+      <c r="C14" s="1676" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1641" t="n"/>
-      <c r="E14" s="1641" t="n">
+      <c r="D14" s="1677" t="n"/>
+      <c r="E14" s="1677" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1641" t="n">
+      <c r="F14" s="1677" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1641" t="n">
+      <c r="G14" s="1677" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1641" t="n"/>
-      <c r="I14" s="1642" t="n"/>
-      <c r="J14" s="1643" t="n"/>
-      <c r="K14" s="1643" t="n"/>
-      <c r="L14" s="1643" t="n"/>
-      <c r="M14" s="1641" t="n"/>
-      <c r="N14" s="1641" t="n"/>
-      <c r="O14" s="1641" t="n">
+      <c r="H14" s="1677" t="n"/>
+      <c r="I14" s="1678" t="n"/>
+      <c r="J14" s="1679" t="n"/>
+      <c r="K14" s="1679" t="n"/>
+      <c r="L14" s="1679" t="n"/>
+      <c r="M14" s="1677" t="n"/>
+      <c r="N14" s="1677" t="n"/>
+      <c r="O14" s="1677" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1644" t="n">
+      <c r="P14" s="1680" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1641" t="n"/>
-      <c r="R14" s="1641" t="n"/>
-      <c r="S14" s="1641" t="n"/>
+      <c r="Q14" s="1677" t="n"/>
+      <c r="R14" s="1677" t="n"/>
+      <c r="S14" s="1677" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1640" t="n"/>
+      <c r="U14" s="1676" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -6480,43 +6606,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1639" t="inlineStr">
+      <c r="A15" s="1675" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1640" t="inlineStr">
+      <c r="B15" s="1676" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1640" t="inlineStr">
+      <c r="C15" s="1676" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1641" t="n"/>
-      <c r="E15" s="1641" t="n"/>
-      <c r="F15" s="1641" t="n"/>
-      <c r="G15" s="1641" t="n"/>
-      <c r="H15" s="1641" t="n"/>
-      <c r="I15" s="1642" t="n"/>
-      <c r="J15" s="1643" t="n"/>
-      <c r="K15" s="1643" t="n"/>
-      <c r="L15" s="1643" t="n"/>
-      <c r="M15" s="1641" t="n">
+      <c r="D15" s="1677" t="n"/>
+      <c r="E15" s="1677" t="n"/>
+      <c r="F15" s="1677" t="n"/>
+      <c r="G15" s="1677" t="n"/>
+      <c r="H15" s="1677" t="n"/>
+      <c r="I15" s="1678" t="n"/>
+      <c r="J15" s="1679" t="n"/>
+      <c r="K15" s="1679" t="n"/>
+      <c r="L15" s="1679" t="n"/>
+      <c r="M15" s="1677" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1641" t="n">
+      <c r="N15" s="1677" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1641" t="n"/>
-      <c r="P15" s="1644" t="n"/>
-      <c r="Q15" s="1641" t="n"/>
-      <c r="R15" s="1641" t="n"/>
-      <c r="S15" s="1641" t="n"/>
+      <c r="O15" s="1677" t="n"/>
+      <c r="P15" s="1680" t="n"/>
+      <c r="Q15" s="1677" t="n"/>
+      <c r="R15" s="1677" t="n"/>
+      <c r="S15" s="1677" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1640" t="n"/>
+      <c r="U15" s="1676" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -6524,39 +6650,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1645" t="inlineStr">
+      <c r="A16" s="1681" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1646" t="inlineStr">
+      <c r="B16" s="1682" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1646" t="inlineStr">
+      <c r="C16" s="1682" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1647" t="n"/>
-      <c r="E16" s="1647" t="n"/>
-      <c r="F16" s="1647" t="n"/>
-      <c r="G16" s="1647" t="n"/>
-      <c r="H16" s="1647" t="n"/>
-      <c r="I16" s="1648" t="n"/>
-      <c r="J16" s="1649" t="n"/>
-      <c r="K16" s="1649" t="n"/>
-      <c r="L16" s="1649" t="n"/>
-      <c r="M16" s="1647" t="n"/>
-      <c r="N16" s="1647" t="n"/>
-      <c r="O16" s="1647" t="n"/>
-      <c r="P16" s="1650" t="n"/>
-      <c r="Q16" s="1647" t="n"/>
-      <c r="R16" s="1647" t="n"/>
-      <c r="S16" s="1647" t="n"/>
+      <c r="D16" s="1683" t="n"/>
+      <c r="E16" s="1683" t="n"/>
+      <c r="F16" s="1683" t="n"/>
+      <c r="G16" s="1683" t="n"/>
+      <c r="H16" s="1683" t="n"/>
+      <c r="I16" s="1684" t="n"/>
+      <c r="J16" s="1685" t="n"/>
+      <c r="K16" s="1685" t="n"/>
+      <c r="L16" s="1685" t="n"/>
+      <c r="M16" s="1683" t="n"/>
+      <c r="N16" s="1683" t="n"/>
+      <c r="O16" s="1683" t="n"/>
+      <c r="P16" s="1686" t="n"/>
+      <c r="Q16" s="1683" t="n"/>
+      <c r="R16" s="1683" t="n"/>
+      <c r="S16" s="1683" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1646" t="n"/>
+      <c r="U16" s="1682" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -6564,39 +6690,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1621" t="inlineStr">
+      <c r="A17" s="1657" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1622" t="inlineStr">
+      <c r="B17" s="1658" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1622" t="inlineStr">
+      <c r="C17" s="1658" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1623" t="n"/>
-      <c r="E17" s="1623" t="n"/>
-      <c r="F17" s="1623" t="n"/>
-      <c r="G17" s="1623" t="n"/>
-      <c r="H17" s="1623" t="n"/>
-      <c r="I17" s="1624" t="n"/>
-      <c r="J17" s="1625" t="n"/>
-      <c r="K17" s="1625" t="n"/>
-      <c r="L17" s="1625" t="n"/>
-      <c r="M17" s="1623" t="n"/>
-      <c r="N17" s="1623" t="n"/>
-      <c r="O17" s="1623" t="n"/>
-      <c r="P17" s="1626" t="n"/>
-      <c r="Q17" s="1623" t="n"/>
-      <c r="R17" s="1623" t="n"/>
-      <c r="S17" s="1623" t="n"/>
+      <c r="D17" s="1659" t="n"/>
+      <c r="E17" s="1659" t="n"/>
+      <c r="F17" s="1659" t="n"/>
+      <c r="G17" s="1659" t="n"/>
+      <c r="H17" s="1659" t="n"/>
+      <c r="I17" s="1660" t="n"/>
+      <c r="J17" s="1661" t="n"/>
+      <c r="K17" s="1661" t="n"/>
+      <c r="L17" s="1661" t="n"/>
+      <c r="M17" s="1659" t="n"/>
+      <c r="N17" s="1659" t="n"/>
+      <c r="O17" s="1659" t="n"/>
+      <c r="P17" s="1662" t="n"/>
+      <c r="Q17" s="1659" t="n"/>
+      <c r="R17" s="1659" t="n"/>
+      <c r="S17" s="1659" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1622" t="n"/>
+      <c r="U17" s="1658" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -6604,53 +6730,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1651" t="inlineStr">
+      <c r="A18" s="1687" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1652" t="inlineStr">
+      <c r="B18" s="1688" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1652" t="inlineStr">
+      <c r="C18" s="1688" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1653" t="n"/>
-      <c r="E18" s="1653" t="n">
+      <c r="D18" s="1689" t="n"/>
+      <c r="E18" s="1689" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1653" t="n">
+      <c r="F18" s="1689" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1653" t="n">
+      <c r="G18" s="1689" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1653" t="n"/>
-      <c r="I18" s="1654" t="n"/>
-      <c r="J18" s="1655" t="n"/>
-      <c r="K18" s="1655" t="n"/>
-      <c r="L18" s="1655" t="n"/>
-      <c r="M18" s="1653" t="n"/>
-      <c r="N18" s="1653" t="n"/>
-      <c r="O18" s="1653" t="n">
+      <c r="H18" s="1689" t="n"/>
+      <c r="I18" s="1690" t="n"/>
+      <c r="J18" s="1691" t="n"/>
+      <c r="K18" s="1691" t="n"/>
+      <c r="L18" s="1691" t="n"/>
+      <c r="M18" s="1689" t="n"/>
+      <c r="N18" s="1689" t="n"/>
+      <c r="O18" s="1689" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1656" t="n">
+      <c r="P18" s="1692" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1653" t="n"/>
-      <c r="R18" s="1653" t="n"/>
-      <c r="S18" s="1653" t="n"/>
+      <c r="Q18" s="1689" t="n"/>
+      <c r="R18" s="1689" t="n"/>
+      <c r="S18" s="1689" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1652" t="n"/>
+      <c r="U18" s="1688" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -6658,47 +6784,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1651" t="inlineStr">
+      <c r="A19" s="1687" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1652" t="inlineStr">
+      <c r="B19" s="1688" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1652" t="inlineStr">
+      <c r="C19" s="1688" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1653" t="n"/>
-      <c r="E19" s="1653" t="n"/>
-      <c r="F19" s="1653" t="n"/>
-      <c r="G19" s="1653" t="n"/>
-      <c r="H19" s="1653" t="n"/>
-      <c r="I19" s="1654" t="n"/>
-      <c r="J19" s="1655" t="n"/>
-      <c r="K19" s="1655" t="n"/>
-      <c r="L19" s="1655" t="n"/>
-      <c r="M19" s="1653" t="n">
+      <c r="D19" s="1689" t="n"/>
+      <c r="E19" s="1689" t="n"/>
+      <c r="F19" s="1689" t="n"/>
+      <c r="G19" s="1689" t="n"/>
+      <c r="H19" s="1689" t="n"/>
+      <c r="I19" s="1690" t="n"/>
+      <c r="J19" s="1691" t="n"/>
+      <c r="K19" s="1691" t="n"/>
+      <c r="L19" s="1691" t="n"/>
+      <c r="M19" s="1689" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1653" t="n">
+      <c r="N19" s="1689" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1653" t="n"/>
-      <c r="P19" s="1656" t="n"/>
-      <c r="Q19" s="1653" t="n"/>
-      <c r="R19" s="1653" t="n"/>
-      <c r="S19" s="1653" t="n"/>
+      <c r="O19" s="1689" t="n"/>
+      <c r="P19" s="1692" t="n"/>
+      <c r="Q19" s="1689" t="n"/>
+      <c r="R19" s="1689" t="n"/>
+      <c r="S19" s="1689" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1652" t="n"/>
+      <c r="U19" s="1688" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -6706,43 +6832,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1651" t="inlineStr">
+      <c r="A20" s="1687" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1652" t="inlineStr">
+      <c r="B20" s="1688" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1652" t="inlineStr">
+      <c r="C20" s="1688" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1653" t="n"/>
-      <c r="E20" s="1653" t="n"/>
-      <c r="F20" s="1653" t="n"/>
-      <c r="G20" s="1653" t="n"/>
-      <c r="H20" s="1653" t="n"/>
-      <c r="I20" s="1654" t="n"/>
-      <c r="J20" s="1655" t="n"/>
-      <c r="K20" s="1655" t="n"/>
-      <c r="L20" s="1655" t="n"/>
-      <c r="M20" s="1653" t="n"/>
-      <c r="N20" s="1653" t="n"/>
-      <c r="O20" s="1653" t="n"/>
-      <c r="P20" s="1656" t="n"/>
-      <c r="Q20" s="1653" t="n"/>
-      <c r="R20" s="1653" t="n"/>
-      <c r="S20" s="1653" t="n"/>
+      <c r="D20" s="1689" t="n"/>
+      <c r="E20" s="1689" t="n"/>
+      <c r="F20" s="1689" t="n"/>
+      <c r="G20" s="1689" t="n"/>
+      <c r="H20" s="1689" t="n"/>
+      <c r="I20" s="1690" t="n"/>
+      <c r="J20" s="1691" t="n"/>
+      <c r="K20" s="1691" t="n"/>
+      <c r="L20" s="1691" t="n"/>
+      <c r="M20" s="1689" t="n"/>
+      <c r="N20" s="1689" t="n"/>
+      <c r="O20" s="1689" t="n"/>
+      <c r="P20" s="1692" t="n"/>
+      <c r="Q20" s="1689" t="n"/>
+      <c r="R20" s="1689" t="n"/>
+      <c r="S20" s="1689" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1652" t="n"/>
+      <c r="U20" s="1688" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -6750,39 +6876,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1627" t="inlineStr">
+      <c r="A21" s="1663" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1628" t="inlineStr">
+      <c r="B21" s="1664" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1628" t="inlineStr">
+      <c r="C21" s="1664" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1629" t="n"/>
-      <c r="E21" s="1629" t="n"/>
-      <c r="F21" s="1629" t="n"/>
-      <c r="G21" s="1629" t="n"/>
-      <c r="H21" s="1629" t="n"/>
-      <c r="I21" s="1630" t="n"/>
-      <c r="J21" s="1631" t="n"/>
-      <c r="K21" s="1631" t="n"/>
-      <c r="L21" s="1631" t="n"/>
-      <c r="M21" s="1629" t="n"/>
-      <c r="N21" s="1629" t="n"/>
-      <c r="O21" s="1629" t="n"/>
-      <c r="P21" s="1632" t="n"/>
-      <c r="Q21" s="1629" t="n"/>
-      <c r="R21" s="1629" t="n"/>
-      <c r="S21" s="1629" t="n"/>
+      <c r="D21" s="1665" t="n"/>
+      <c r="E21" s="1665" t="n"/>
+      <c r="F21" s="1665" t="n"/>
+      <c r="G21" s="1665" t="n"/>
+      <c r="H21" s="1665" t="n"/>
+      <c r="I21" s="1666" t="n"/>
+      <c r="J21" s="1667" t="n"/>
+      <c r="K21" s="1667" t="n"/>
+      <c r="L21" s="1667" t="n"/>
+      <c r="M21" s="1665" t="n"/>
+      <c r="N21" s="1665" t="n"/>
+      <c r="O21" s="1665" t="n"/>
+      <c r="P21" s="1668" t="n"/>
+      <c r="Q21" s="1665" t="n"/>
+      <c r="R21" s="1665" t="n"/>
+      <c r="S21" s="1665" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1628" t="n"/>
+      <c r="U21" s="1664" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -6790,39 +6916,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1633" t="inlineStr">
+      <c r="A22" s="1669" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1634" t="inlineStr">
+      <c r="B22" s="1670" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1634" t="inlineStr">
+      <c r="C22" s="1670" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1635" t="n"/>
-      <c r="E22" s="1635" t="n"/>
-      <c r="F22" s="1635" t="n"/>
-      <c r="G22" s="1635" t="n"/>
-      <c r="H22" s="1635" t="n"/>
-      <c r="I22" s="1636" t="n"/>
-      <c r="J22" s="1637" t="n"/>
-      <c r="K22" s="1637" t="n"/>
-      <c r="L22" s="1637" t="n"/>
-      <c r="M22" s="1635" t="n"/>
-      <c r="N22" s="1635" t="n"/>
-      <c r="O22" s="1635" t="n"/>
-      <c r="P22" s="1638" t="n"/>
-      <c r="Q22" s="1635" t="n"/>
-      <c r="R22" s="1635" t="n"/>
-      <c r="S22" s="1635" t="n"/>
+      <c r="D22" s="1671" t="n"/>
+      <c r="E22" s="1671" t="n"/>
+      <c r="F22" s="1671" t="n"/>
+      <c r="G22" s="1671" t="n"/>
+      <c r="H22" s="1671" t="n"/>
+      <c r="I22" s="1672" t="n"/>
+      <c r="J22" s="1673" t="n"/>
+      <c r="K22" s="1673" t="n"/>
+      <c r="L22" s="1673" t="n"/>
+      <c r="M22" s="1671" t="n"/>
+      <c r="N22" s="1671" t="n"/>
+      <c r="O22" s="1671" t="n"/>
+      <c r="P22" s="1674" t="n"/>
+      <c r="Q22" s="1671" t="n"/>
+      <c r="R22" s="1671" t="n"/>
+      <c r="S22" s="1671" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1634" t="n"/>
+      <c r="U22" s="1670" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -6830,53 +6956,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1639" t="inlineStr">
+      <c r="A23" s="1675" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1640" t="inlineStr">
+      <c r="B23" s="1676" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1640" t="inlineStr">
+      <c r="C23" s="1676" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1641" t="n"/>
-      <c r="E23" s="1641" t="n">
+      <c r="D23" s="1677" t="n"/>
+      <c r="E23" s="1677" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1641" t="n">
+      <c r="F23" s="1677" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1641" t="n">
+      <c r="G23" s="1677" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1641" t="n"/>
-      <c r="I23" s="1642" t="n"/>
-      <c r="J23" s="1643" t="n"/>
-      <c r="K23" s="1643" t="n"/>
-      <c r="L23" s="1643" t="n"/>
-      <c r="M23" s="1641" t="n"/>
-      <c r="N23" s="1641" t="n"/>
-      <c r="O23" s="1641" t="n">
+      <c r="H23" s="1677" t="n"/>
+      <c r="I23" s="1678" t="n"/>
+      <c r="J23" s="1679" t="n"/>
+      <c r="K23" s="1679" t="n"/>
+      <c r="L23" s="1679" t="n"/>
+      <c r="M23" s="1677" t="n"/>
+      <c r="N23" s="1677" t="n"/>
+      <c r="O23" s="1677" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1644" t="n">
+      <c r="P23" s="1680" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1641" t="n"/>
-      <c r="R23" s="1641" t="n"/>
-      <c r="S23" s="1641" t="n"/>
+      <c r="Q23" s="1677" t="n"/>
+      <c r="R23" s="1677" t="n"/>
+      <c r="S23" s="1677" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1640" t="n"/>
+      <c r="U23" s="1676" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -6884,47 +7010,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1645" t="inlineStr">
+      <c r="A24" s="1681" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1646" t="inlineStr">
+      <c r="B24" s="1682" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1646" t="inlineStr">
+      <c r="C24" s="1682" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1647" t="n"/>
-      <c r="E24" s="1647" t="n"/>
-      <c r="F24" s="1647" t="n"/>
-      <c r="G24" s="1647" t="n"/>
-      <c r="H24" s="1647" t="n"/>
-      <c r="I24" s="1648" t="n"/>
-      <c r="J24" s="1649" t="n"/>
-      <c r="K24" s="1649" t="n"/>
-      <c r="L24" s="1649" t="n"/>
-      <c r="M24" s="1647" t="n">
+      <c r="D24" s="1683" t="n"/>
+      <c r="E24" s="1683" t="n"/>
+      <c r="F24" s="1683" t="n"/>
+      <c r="G24" s="1683" t="n"/>
+      <c r="H24" s="1683" t="n"/>
+      <c r="I24" s="1684" t="n"/>
+      <c r="J24" s="1685" t="n"/>
+      <c r="K24" s="1685" t="n"/>
+      <c r="L24" s="1685" t="n"/>
+      <c r="M24" s="1683" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1647" t="n">
+      <c r="N24" s="1683" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1647" t="n"/>
-      <c r="P24" s="1650" t="n"/>
-      <c r="Q24" s="1647" t="n"/>
-      <c r="R24" s="1647" t="n"/>
-      <c r="S24" s="1647" t="n"/>
+      <c r="O24" s="1683" t="n"/>
+      <c r="P24" s="1686" t="n"/>
+      <c r="Q24" s="1683" t="n"/>
+      <c r="R24" s="1683" t="n"/>
+      <c r="S24" s="1683" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1646" t="n"/>
+      <c r="U24" s="1682" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -6932,61 +7058,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1621" t="inlineStr">
+      <c r="A25" s="1657" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1622" t="inlineStr">
+      <c r="B25" s="1658" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1622" t="inlineStr">
+      <c r="C25" s="1658" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1623" t="n">
+      <c r="D25" s="1659" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1623" t="n">
+      <c r="E25" s="1659" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1623" t="n">
+      <c r="F25" s="1659" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1623" t="n">
+      <c r="G25" s="1659" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1623" t="n"/>
-      <c r="I25" s="1624" t="n"/>
-      <c r="J25" s="1625" t="n">
+      <c r="H25" s="1659" t="n"/>
+      <c r="I25" s="1660" t="n"/>
+      <c r="J25" s="1661" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1625" t="n">
+      <c r="K25" s="1661" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1625" t="n">
+      <c r="L25" s="1661" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1623" t="n"/>
-      <c r="N25" s="1623" t="n"/>
-      <c r="O25" s="1623" t="n">
+      <c r="M25" s="1659" t="n"/>
+      <c r="N25" s="1659" t="n"/>
+      <c r="O25" s="1659" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1626" t="n">
+      <c r="P25" s="1662" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1623" t="n"/>
-      <c r="R25" s="1623" t="n"/>
-      <c r="S25" s="1623" t="n"/>
+      <c r="Q25" s="1659" t="n"/>
+      <c r="R25" s="1659" t="n"/>
+      <c r="S25" s="1659" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1622" t="n"/>
+      <c r="U25" s="1658" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -6994,47 +7120,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1627" t="inlineStr">
+      <c r="A26" s="1663" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1628" t="inlineStr">
+      <c r="B26" s="1664" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1628" t="inlineStr">
+      <c r="C26" s="1664" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1629" t="n"/>
-      <c r="E26" s="1629" t="n"/>
-      <c r="F26" s="1629" t="n"/>
-      <c r="G26" s="1629" t="n"/>
-      <c r="H26" s="1629" t="n"/>
-      <c r="I26" s="1630" t="n"/>
-      <c r="J26" s="1631" t="n"/>
-      <c r="K26" s="1631" t="n"/>
-      <c r="L26" s="1631" t="n"/>
-      <c r="M26" s="1629" t="n">
+      <c r="D26" s="1665" t="n"/>
+      <c r="E26" s="1665" t="n"/>
+      <c r="F26" s="1665" t="n"/>
+      <c r="G26" s="1665" t="n"/>
+      <c r="H26" s="1665" t="n"/>
+      <c r="I26" s="1666" t="n"/>
+      <c r="J26" s="1667" t="n"/>
+      <c r="K26" s="1667" t="n"/>
+      <c r="L26" s="1667" t="n"/>
+      <c r="M26" s="1665" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1629" t="n">
+      <c r="N26" s="1665" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1629" t="n"/>
-      <c r="P26" s="1632" t="n"/>
-      <c r="Q26" s="1629" t="n"/>
-      <c r="R26" s="1629" t="n"/>
-      <c r="S26" s="1629" t="n"/>
+      <c r="O26" s="1665" t="n"/>
+      <c r="P26" s="1668" t="n"/>
+      <c r="Q26" s="1665" t="n"/>
+      <c r="R26" s="1665" t="n"/>
+      <c r="S26" s="1665" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1628" t="n"/>
+      <c r="U26" s="1664" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -7042,53 +7168,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1633" t="inlineStr">
+      <c r="A27" s="1669" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1634" t="inlineStr">
+      <c r="B27" s="1670" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1634" t="inlineStr">
+      <c r="C27" s="1670" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1635" t="n"/>
-      <c r="E27" s="1635" t="n">
+      <c r="D27" s="1671" t="n"/>
+      <c r="E27" s="1671" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1635" t="n">
+      <c r="F27" s="1671" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1635" t="n">
+      <c r="G27" s="1671" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1635" t="n"/>
-      <c r="I27" s="1636" t="n"/>
-      <c r="J27" s="1637" t="n"/>
-      <c r="K27" s="1637" t="n"/>
-      <c r="L27" s="1637" t="n"/>
-      <c r="M27" s="1635" t="n"/>
-      <c r="N27" s="1635" t="n"/>
-      <c r="O27" s="1635" t="n">
+      <c r="H27" s="1671" t="n"/>
+      <c r="I27" s="1672" t="n"/>
+      <c r="J27" s="1673" t="n"/>
+      <c r="K27" s="1673" t="n"/>
+      <c r="L27" s="1673" t="n"/>
+      <c r="M27" s="1671" t="n"/>
+      <c r="N27" s="1671" t="n"/>
+      <c r="O27" s="1671" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1638" t="n">
+      <c r="P27" s="1674" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1635" t="n"/>
-      <c r="R27" s="1635" t="n"/>
-      <c r="S27" s="1635" t="n"/>
+      <c r="Q27" s="1671" t="n"/>
+      <c r="R27" s="1671" t="n"/>
+      <c r="S27" s="1671" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1634" t="n"/>
+      <c r="U27" s="1670" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -7096,47 +7222,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1645" t="inlineStr">
+      <c r="A28" s="1681" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1646" t="inlineStr">
+      <c r="B28" s="1682" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1646" t="inlineStr">
+      <c r="C28" s="1682" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1647" t="n"/>
-      <c r="E28" s="1647" t="n"/>
-      <c r="F28" s="1647" t="n"/>
-      <c r="G28" s="1647" t="n"/>
-      <c r="H28" s="1647" t="n"/>
-      <c r="I28" s="1648" t="n"/>
-      <c r="J28" s="1649" t="n"/>
-      <c r="K28" s="1649" t="n"/>
-      <c r="L28" s="1649" t="n"/>
-      <c r="M28" s="1647" t="n">
+      <c r="D28" s="1683" t="n"/>
+      <c r="E28" s="1683" t="n"/>
+      <c r="F28" s="1683" t="n"/>
+      <c r="G28" s="1683" t="n"/>
+      <c r="H28" s="1683" t="n"/>
+      <c r="I28" s="1684" t="n"/>
+      <c r="J28" s="1685" t="n"/>
+      <c r="K28" s="1685" t="n"/>
+      <c r="L28" s="1685" t="n"/>
+      <c r="M28" s="1683" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1647" t="n">
+      <c r="N28" s="1683" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1647" t="n"/>
-      <c r="P28" s="1650" t="n"/>
-      <c r="Q28" s="1647" t="n"/>
-      <c r="R28" s="1647" t="n"/>
-      <c r="S28" s="1647" t="n"/>
+      <c r="O28" s="1683" t="n"/>
+      <c r="P28" s="1686" t="n"/>
+      <c r="Q28" s="1683" t="n"/>
+      <c r="R28" s="1683" t="n"/>
+      <c r="S28" s="1683" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1646" t="n"/>
+      <c r="U28" s="1682" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -7144,53 +7270,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1621" t="inlineStr">
+      <c r="A29" s="1657" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1622" t="inlineStr">
+      <c r="B29" s="1658" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1622" t="inlineStr">
+      <c r="C29" s="1658" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1623" t="n"/>
-      <c r="E29" s="1623" t="n">
+      <c r="D29" s="1659" t="n"/>
+      <c r="E29" s="1659" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1623" t="n">
+      <c r="F29" s="1659" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1623" t="n">
+      <c r="G29" s="1659" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1623" t="n"/>
-      <c r="I29" s="1624" t="n"/>
-      <c r="J29" s="1625" t="n"/>
-      <c r="K29" s="1625" t="n"/>
-      <c r="L29" s="1625" t="n"/>
-      <c r="M29" s="1623" t="n"/>
-      <c r="N29" s="1623" t="n"/>
-      <c r="O29" s="1623" t="n">
+      <c r="H29" s="1659" t="n"/>
+      <c r="I29" s="1660" t="n"/>
+      <c r="J29" s="1661" t="n"/>
+      <c r="K29" s="1661" t="n"/>
+      <c r="L29" s="1661" t="n"/>
+      <c r="M29" s="1659" t="n"/>
+      <c r="N29" s="1659" t="n"/>
+      <c r="O29" s="1659" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1626" t="n">
+      <c r="P29" s="1662" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1623" t="n"/>
-      <c r="R29" s="1623" t="n"/>
-      <c r="S29" s="1623" t="n"/>
+      <c r="Q29" s="1659" t="n"/>
+      <c r="R29" s="1659" t="n"/>
+      <c r="S29" s="1659" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1622" t="n"/>
+      <c r="U29" s="1658" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -7198,43 +7324,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1627" t="inlineStr">
+      <c r="A30" s="1663" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1628" t="inlineStr">
+      <c r="B30" s="1664" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1628" t="inlineStr">
+      <c r="C30" s="1664" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1629" t="n"/>
-      <c r="E30" s="1629" t="n"/>
-      <c r="F30" s="1629" t="n"/>
-      <c r="G30" s="1629" t="n"/>
-      <c r="H30" s="1629" t="n"/>
-      <c r="I30" s="1630" t="n"/>
-      <c r="J30" s="1631" t="n"/>
-      <c r="K30" s="1631" t="n"/>
-      <c r="L30" s="1631" t="n"/>
-      <c r="M30" s="1629" t="n"/>
-      <c r="N30" s="1629" t="n"/>
-      <c r="O30" s="1629" t="n"/>
-      <c r="P30" s="1632" t="n"/>
-      <c r="Q30" s="1629" t="n"/>
-      <c r="R30" s="1629" t="n"/>
-      <c r="S30" s="1629" t="n"/>
+      <c r="D30" s="1665" t="n"/>
+      <c r="E30" s="1665" t="n"/>
+      <c r="F30" s="1665" t="n"/>
+      <c r="G30" s="1665" t="n"/>
+      <c r="H30" s="1665" t="n"/>
+      <c r="I30" s="1666" t="n"/>
+      <c r="J30" s="1667" t="n"/>
+      <c r="K30" s="1667" t="n"/>
+      <c r="L30" s="1667" t="n"/>
+      <c r="M30" s="1665" t="n"/>
+      <c r="N30" s="1665" t="n"/>
+      <c r="O30" s="1665" t="n"/>
+      <c r="P30" s="1668" t="n"/>
+      <c r="Q30" s="1665" t="n"/>
+      <c r="R30" s="1665" t="n"/>
+      <c r="S30" s="1665" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1628" t="n"/>
+      <c r="U30" s="1664" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -7242,53 +7368,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1633" t="inlineStr">
+      <c r="A31" s="1669" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1634" t="inlineStr">
+      <c r="B31" s="1670" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1634" t="inlineStr">
+      <c r="C31" s="1670" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1635" t="n"/>
-      <c r="E31" s="1635" t="n">
+      <c r="D31" s="1671" t="n"/>
+      <c r="E31" s="1671" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1635" t="n">
+      <c r="F31" s="1671" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1635" t="n">
+      <c r="G31" s="1671" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1635" t="n"/>
-      <c r="I31" s="1636" t="n"/>
-      <c r="J31" s="1637" t="n"/>
-      <c r="K31" s="1637" t="n"/>
-      <c r="L31" s="1637" t="n"/>
-      <c r="M31" s="1635" t="n"/>
-      <c r="N31" s="1635" t="n"/>
-      <c r="O31" s="1635" t="n">
+      <c r="H31" s="1671" t="n"/>
+      <c r="I31" s="1672" t="n"/>
+      <c r="J31" s="1673" t="n"/>
+      <c r="K31" s="1673" t="n"/>
+      <c r="L31" s="1673" t="n"/>
+      <c r="M31" s="1671" t="n"/>
+      <c r="N31" s="1671" t="n"/>
+      <c r="O31" s="1671" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1638" t="n">
+      <c r="P31" s="1674" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1635" t="n"/>
-      <c r="R31" s="1635" t="n"/>
-      <c r="S31" s="1635" t="n"/>
+      <c r="Q31" s="1671" t="n"/>
+      <c r="R31" s="1671" t="n"/>
+      <c r="S31" s="1671" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1634" t="inlineStr">
+      <c r="U31" s="1670" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -7300,49 +7426,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1645" t="inlineStr">
+      <c r="A32" s="1681" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1646" t="inlineStr">
+      <c r="B32" s="1682" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1646" t="inlineStr">
+      <c r="C32" s="1682" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1647" t="n"/>
-      <c r="E32" s="1647" t="n"/>
-      <c r="F32" s="1647" t="n"/>
-      <c r="G32" s="1647" t="n"/>
-      <c r="H32" s="1647" t="n">
+      <c r="D32" s="1683" t="n"/>
+      <c r="E32" s="1683" t="n"/>
+      <c r="F32" s="1683" t="n"/>
+      <c r="G32" s="1683" t="n"/>
+      <c r="H32" s="1683" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1648" t="n"/>
-      <c r="J32" s="1649" t="n"/>
-      <c r="K32" s="1649" t="n"/>
-      <c r="L32" s="1649" t="n"/>
-      <c r="M32" s="1647" t="n">
+      <c r="I32" s="1684" t="n"/>
+      <c r="J32" s="1685" t="n"/>
+      <c r="K32" s="1685" t="n"/>
+      <c r="L32" s="1685" t="n"/>
+      <c r="M32" s="1683" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1647" t="n">
+      <c r="N32" s="1683" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1647" t="n"/>
-      <c r="P32" s="1650" t="n"/>
-      <c r="Q32" s="1647" t="n"/>
-      <c r="R32" s="1647" t="n"/>
-      <c r="S32" s="1647" t="n"/>
+      <c r="O32" s="1683" t="n"/>
+      <c r="P32" s="1686" t="n"/>
+      <c r="Q32" s="1683" t="n"/>
+      <c r="R32" s="1683" t="n"/>
+      <c r="S32" s="1683" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1646" t="n"/>
+      <c r="U32" s="1682" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -7350,57 +7476,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1621" t="inlineStr">
+      <c r="A33" s="1657" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1622" t="inlineStr">
+      <c r="B33" s="1658" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1622" t="inlineStr">
+      <c r="C33" s="1658" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1623" t="n"/>
-      <c r="E33" s="1623" t="n">
+      <c r="D33" s="1659" t="n"/>
+      <c r="E33" s="1659" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1623" t="n">
+      <c r="F33" s="1659" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1623" t="n">
+      <c r="G33" s="1659" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1623" t="n"/>
-      <c r="I33" s="1624" t="n">
+      <c r="H33" s="1659" t="n"/>
+      <c r="I33" s="1660" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1625" t="n"/>
-      <c r="K33" s="1625" t="n"/>
-      <c r="L33" s="1625" t="n"/>
-      <c r="M33" s="1623" t="n"/>
-      <c r="N33" s="1623" t="n"/>
-      <c r="O33" s="1623" t="n">
+      <c r="J33" s="1661" t="n"/>
+      <c r="K33" s="1661" t="n"/>
+      <c r="L33" s="1661" t="n"/>
+      <c r="M33" s="1659" t="n"/>
+      <c r="N33" s="1659" t="n"/>
+      <c r="O33" s="1659" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1626" t="n">
+      <c r="P33" s="1662" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1623" t="n"/>
-      <c r="R33" s="1623" t="n">
+      <c r="Q33" s="1659" t="n"/>
+      <c r="R33" s="1659" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1623" t="n"/>
+      <c r="S33" s="1659" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1622" t="inlineStr">
+      <c r="U33" s="1658" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -7412,49 +7538,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1627" t="inlineStr">
+      <c r="A34" s="1663" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1628" t="inlineStr">
+      <c r="B34" s="1664" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1628" t="inlineStr">
+      <c r="C34" s="1664" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1629" t="n"/>
-      <c r="E34" s="1629" t="n"/>
-      <c r="F34" s="1629" t="n"/>
-      <c r="G34" s="1629" t="n"/>
-      <c r="H34" s="1629" t="n">
+      <c r="D34" s="1665" t="n"/>
+      <c r="E34" s="1665" t="n"/>
+      <c r="F34" s="1665" t="n"/>
+      <c r="G34" s="1665" t="n"/>
+      <c r="H34" s="1665" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1630" t="n"/>
-      <c r="J34" s="1631" t="n"/>
-      <c r="K34" s="1631" t="n"/>
-      <c r="L34" s="1631" t="n"/>
-      <c r="M34" s="1629" t="n">
+      <c r="I34" s="1666" t="n"/>
+      <c r="J34" s="1667" t="n"/>
+      <c r="K34" s="1667" t="n"/>
+      <c r="L34" s="1667" t="n"/>
+      <c r="M34" s="1665" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1629" t="n">
+      <c r="N34" s="1665" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1629" t="n"/>
-      <c r="P34" s="1632" t="n"/>
-      <c r="Q34" s="1629" t="n"/>
-      <c r="R34" s="1629" t="n"/>
-      <c r="S34" s="1629" t="n"/>
+      <c r="O34" s="1665" t="n"/>
+      <c r="P34" s="1668" t="n"/>
+      <c r="Q34" s="1665" t="n"/>
+      <c r="R34" s="1665" t="n"/>
+      <c r="S34" s="1665" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1628" t="n"/>
+      <c r="U34" s="1664" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -7462,57 +7588,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1633" t="inlineStr">
+      <c r="A35" s="1669" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1634" t="inlineStr">
+      <c r="B35" s="1670" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1634" t="inlineStr">
+      <c r="C35" s="1670" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1635" t="n"/>
-      <c r="E35" s="1635" t="n">
+      <c r="D35" s="1671" t="n"/>
+      <c r="E35" s="1671" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1635" t="n">
+      <c r="F35" s="1671" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1635" t="n">
+      <c r="G35" s="1671" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1635" t="n"/>
-      <c r="I35" s="1636" t="n">
+      <c r="H35" s="1671" t="n"/>
+      <c r="I35" s="1672" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1637" t="n"/>
-      <c r="K35" s="1637" t="n"/>
-      <c r="L35" s="1637" t="n"/>
-      <c r="M35" s="1635" t="n"/>
-      <c r="N35" s="1635" t="n"/>
-      <c r="O35" s="1635" t="n">
+      <c r="J35" s="1673" t="n"/>
+      <c r="K35" s="1673" t="n"/>
+      <c r="L35" s="1673" t="n"/>
+      <c r="M35" s="1671" t="n"/>
+      <c r="N35" s="1671" t="n"/>
+      <c r="O35" s="1671" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1638" t="n">
+      <c r="P35" s="1674" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1635" t="n"/>
-      <c r="R35" s="1635" t="n">
+      <c r="Q35" s="1671" t="n"/>
+      <c r="R35" s="1671" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1635" t="n"/>
+      <c r="S35" s="1671" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1634" t="inlineStr">
+      <c r="U35" s="1670" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -7524,49 +7650,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1639" t="inlineStr">
+      <c r="A36" s="1675" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1640" t="inlineStr">
+      <c r="B36" s="1676" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1640" t="inlineStr">
+      <c r="C36" s="1676" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1641" t="n"/>
-      <c r="E36" s="1641" t="n"/>
-      <c r="F36" s="1641" t="n"/>
-      <c r="G36" s="1641" t="n"/>
-      <c r="H36" s="1641" t="n">
+      <c r="D36" s="1677" t="n"/>
+      <c r="E36" s="1677" t="n"/>
+      <c r="F36" s="1677" t="n"/>
+      <c r="G36" s="1677" t="n"/>
+      <c r="H36" s="1677" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1642" t="n"/>
-      <c r="J36" s="1643" t="n"/>
-      <c r="K36" s="1643" t="n"/>
-      <c r="L36" s="1643" t="n"/>
-      <c r="M36" s="1641" t="n">
+      <c r="I36" s="1678" t="n"/>
+      <c r="J36" s="1679" t="n"/>
+      <c r="K36" s="1679" t="n"/>
+      <c r="L36" s="1679" t="n"/>
+      <c r="M36" s="1677" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1641" t="n">
+      <c r="N36" s="1677" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1641" t="n"/>
-      <c r="P36" s="1644" t="n"/>
-      <c r="Q36" s="1641" t="n"/>
-      <c r="R36" s="1641" t="n"/>
-      <c r="S36" s="1641" t="n"/>
+      <c r="O36" s="1677" t="n"/>
+      <c r="P36" s="1680" t="n"/>
+      <c r="Q36" s="1677" t="n"/>
+      <c r="R36" s="1677" t="n"/>
+      <c r="S36" s="1677" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1640" t="n"/>
+      <c r="U36" s="1676" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -7574,41 +7700,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1645" t="inlineStr">
+      <c r="A37" s="1681" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1646" t="inlineStr">
+      <c r="B37" s="1682" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1646" t="inlineStr">
+      <c r="C37" s="1682" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1647" t="n"/>
-      <c r="E37" s="1647" t="n"/>
-      <c r="F37" s="1647" t="n"/>
-      <c r="G37" s="1647" t="n"/>
-      <c r="H37" s="1647" t="n"/>
-      <c r="I37" s="1648" t="n"/>
-      <c r="J37" s="1649" t="n"/>
-      <c r="K37" s="1649" t="n"/>
-      <c r="L37" s="1649" t="n"/>
-      <c r="M37" s="1647" t="n"/>
-      <c r="N37" s="1647" t="n"/>
-      <c r="O37" s="1647" t="n"/>
-      <c r="P37" s="1650" t="n"/>
-      <c r="Q37" s="1647" t="n">
+      <c r="D37" s="1683" t="n"/>
+      <c r="E37" s="1683" t="n"/>
+      <c r="F37" s="1683" t="n"/>
+      <c r="G37" s="1683" t="n"/>
+      <c r="H37" s="1683" t="n"/>
+      <c r="I37" s="1684" t="n"/>
+      <c r="J37" s="1685" t="n"/>
+      <c r="K37" s="1685" t="n"/>
+      <c r="L37" s="1685" t="n"/>
+      <c r="M37" s="1683" t="n"/>
+      <c r="N37" s="1683" t="n"/>
+      <c r="O37" s="1683" t="n"/>
+      <c r="P37" s="1686" t="n"/>
+      <c r="Q37" s="1683" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1647" t="n"/>
-      <c r="S37" s="1647" t="n"/>
+      <c r="R37" s="1683" t="n"/>
+      <c r="S37" s="1683" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1646" t="n"/>
+      <c r="U37" s="1682" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -7616,57 +7742,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1621" t="inlineStr">
+      <c r="A38" s="1657" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1622" t="inlineStr">
+      <c r="B38" s="1658" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1622" t="inlineStr">
+      <c r="C38" s="1658" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1623" t="n"/>
-      <c r="E38" s="1623" t="n">
+      <c r="D38" s="1659" t="n"/>
+      <c r="E38" s="1659" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1623" t="n">
+      <c r="F38" s="1659" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1623" t="n">
+      <c r="G38" s="1659" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1623" t="n"/>
-      <c r="I38" s="1624" t="n">
+      <c r="H38" s="1659" t="n"/>
+      <c r="I38" s="1660" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1625" t="n"/>
-      <c r="K38" s="1625" t="n"/>
-      <c r="L38" s="1625" t="n"/>
-      <c r="M38" s="1623" t="n"/>
-      <c r="N38" s="1623" t="n"/>
-      <c r="O38" s="1623" t="n">
+      <c r="J38" s="1661" t="n"/>
+      <c r="K38" s="1661" t="n"/>
+      <c r="L38" s="1661" t="n"/>
+      <c r="M38" s="1659" t="n"/>
+      <c r="N38" s="1659" t="n"/>
+      <c r="O38" s="1659" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1626" t="n">
+      <c r="P38" s="1662" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1623" t="n"/>
-      <c r="R38" s="1623" t="n">
+      <c r="Q38" s="1659" t="n"/>
+      <c r="R38" s="1659" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1623" t="n"/>
+      <c r="S38" s="1659" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1622" t="inlineStr">
+      <c r="U38" s="1658" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -7678,49 +7804,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1651" t="inlineStr">
+      <c r="A39" s="1687" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1652" t="inlineStr">
+      <c r="B39" s="1688" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1652" t="inlineStr">
+      <c r="C39" s="1688" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1653" t="n"/>
-      <c r="E39" s="1653" t="n"/>
-      <c r="F39" s="1653" t="n"/>
-      <c r="G39" s="1653" t="n"/>
-      <c r="H39" s="1653" t="n">
+      <c r="D39" s="1689" t="n"/>
+      <c r="E39" s="1689" t="n"/>
+      <c r="F39" s="1689" t="n"/>
+      <c r="G39" s="1689" t="n"/>
+      <c r="H39" s="1689" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1654" t="n"/>
-      <c r="J39" s="1655" t="n"/>
-      <c r="K39" s="1655" t="n"/>
-      <c r="L39" s="1655" t="n"/>
-      <c r="M39" s="1653" t="n">
+      <c r="I39" s="1690" t="n"/>
+      <c r="J39" s="1691" t="n"/>
+      <c r="K39" s="1691" t="n"/>
+      <c r="L39" s="1691" t="n"/>
+      <c r="M39" s="1689" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1653" t="n">
+      <c r="N39" s="1689" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1653" t="n"/>
-      <c r="P39" s="1656" t="n"/>
-      <c r="Q39" s="1653" t="n"/>
-      <c r="R39" s="1653" t="n"/>
-      <c r="S39" s="1653" t="n"/>
+      <c r="O39" s="1689" t="n"/>
+      <c r="P39" s="1692" t="n"/>
+      <c r="Q39" s="1689" t="n"/>
+      <c r="R39" s="1689" t="n"/>
+      <c r="S39" s="1689" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1652" t="n"/>
+      <c r="U39" s="1688" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -7728,41 +7854,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1627" t="inlineStr">
+      <c r="A40" s="1663" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1628" t="inlineStr">
+      <c r="B40" s="1664" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1628" t="inlineStr">
+      <c r="C40" s="1664" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1629" t="n"/>
-      <c r="E40" s="1629" t="n"/>
-      <c r="F40" s="1629" t="n"/>
-      <c r="G40" s="1629" t="n"/>
-      <c r="H40" s="1629" t="n"/>
-      <c r="I40" s="1630" t="n"/>
-      <c r="J40" s="1631" t="n"/>
-      <c r="K40" s="1631" t="n"/>
-      <c r="L40" s="1631" t="n"/>
-      <c r="M40" s="1629" t="n"/>
-      <c r="N40" s="1629" t="n"/>
-      <c r="O40" s="1629" t="n"/>
-      <c r="P40" s="1632" t="n"/>
-      <c r="Q40" s="1629" t="n">
+      <c r="D40" s="1665" t="n"/>
+      <c r="E40" s="1665" t="n"/>
+      <c r="F40" s="1665" t="n"/>
+      <c r="G40" s="1665" t="n"/>
+      <c r="H40" s="1665" t="n"/>
+      <c r="I40" s="1666" t="n"/>
+      <c r="J40" s="1667" t="n"/>
+      <c r="K40" s="1667" t="n"/>
+      <c r="L40" s="1667" t="n"/>
+      <c r="M40" s="1665" t="n"/>
+      <c r="N40" s="1665" t="n"/>
+      <c r="O40" s="1665" t="n"/>
+      <c r="P40" s="1668" t="n"/>
+      <c r="Q40" s="1665" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1629" t="n"/>
-      <c r="S40" s="1629" t="n"/>
+      <c r="R40" s="1665" t="n"/>
+      <c r="S40" s="1665" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1628" t="n"/>
+      <c r="U40" s="1664" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -7770,57 +7896,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1633" t="inlineStr">
+      <c r="A41" s="1669" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1634" t="inlineStr">
+      <c r="B41" s="1670" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1634" t="inlineStr">
+      <c r="C41" s="1670" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1635" t="n"/>
-      <c r="E41" s="1635" t="n">
+      <c r="D41" s="1671" t="n"/>
+      <c r="E41" s="1671" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1635" t="n">
+      <c r="F41" s="1671" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1635" t="n">
+      <c r="G41" s="1671" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1635" t="n"/>
-      <c r="I41" s="1636" t="n">
+      <c r="H41" s="1671" t="n"/>
+      <c r="I41" s="1672" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1637" t="n"/>
-      <c r="K41" s="1637" t="n"/>
-      <c r="L41" s="1637" t="n"/>
-      <c r="M41" s="1635" t="n"/>
-      <c r="N41" s="1635" t="n"/>
-      <c r="O41" s="1635" t="n">
+      <c r="J41" s="1673" t="n"/>
+      <c r="K41" s="1673" t="n"/>
+      <c r="L41" s="1673" t="n"/>
+      <c r="M41" s="1671" t="n"/>
+      <c r="N41" s="1671" t="n"/>
+      <c r="O41" s="1671" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1638" t="n">
+      <c r="P41" s="1674" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1635" t="n"/>
-      <c r="R41" s="1635" t="n">
+      <c r="Q41" s="1671" t="n"/>
+      <c r="R41" s="1671" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1635" t="n"/>
+      <c r="S41" s="1671" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1634" t="inlineStr">
+      <c r="U41" s="1670" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -7832,49 +7958,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1645" t="inlineStr">
+      <c r="A42" s="1681" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1646" t="inlineStr">
+      <c r="B42" s="1682" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1646" t="inlineStr">
+      <c r="C42" s="1682" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1647" t="n"/>
-      <c r="E42" s="1647" t="n"/>
-      <c r="F42" s="1647" t="n"/>
-      <c r="G42" s="1647" t="n"/>
-      <c r="H42" s="1647" t="n">
+      <c r="D42" s="1683" t="n"/>
+      <c r="E42" s="1683" t="n"/>
+      <c r="F42" s="1683" t="n"/>
+      <c r="G42" s="1683" t="n"/>
+      <c r="H42" s="1683" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1648" t="n"/>
-      <c r="J42" s="1649" t="n"/>
-      <c r="K42" s="1649" t="n"/>
-      <c r="L42" s="1649" t="n"/>
-      <c r="M42" s="1647" t="n">
+      <c r="I42" s="1684" t="n"/>
+      <c r="J42" s="1685" t="n"/>
+      <c r="K42" s="1685" t="n"/>
+      <c r="L42" s="1685" t="n"/>
+      <c r="M42" s="1683" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1647" t="n">
+      <c r="N42" s="1683" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1647" t="n"/>
-      <c r="P42" s="1650" t="n"/>
-      <c r="Q42" s="1647" t="n"/>
-      <c r="R42" s="1647" t="n"/>
-      <c r="S42" s="1647" t="n"/>
+      <c r="O42" s="1683" t="n"/>
+      <c r="P42" s="1686" t="n"/>
+      <c r="Q42" s="1683" t="n"/>
+      <c r="R42" s="1683" t="n"/>
+      <c r="S42" s="1683" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1646" t="n"/>
+      <c r="U42" s="1682" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -7882,57 +8008,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1621" t="inlineStr">
+      <c r="A43" s="1657" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1622" t="inlineStr">
+      <c r="B43" s="1658" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1622" t="inlineStr">
+      <c r="C43" s="1658" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1623" t="n"/>
-      <c r="E43" s="1623" t="n">
+      <c r="D43" s="1659" t="n"/>
+      <c r="E43" s="1659" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1623" t="n">
+      <c r="F43" s="1659" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1623" t="n">
+      <c r="G43" s="1659" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1623" t="n"/>
-      <c r="I43" s="1624" t="n">
+      <c r="H43" s="1659" t="n"/>
+      <c r="I43" s="1660" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1625" t="n"/>
-      <c r="K43" s="1625" t="n"/>
-      <c r="L43" s="1625" t="n"/>
-      <c r="M43" s="1623" t="n"/>
-      <c r="N43" s="1623" t="n"/>
-      <c r="O43" s="1623" t="n">
+      <c r="J43" s="1661" t="n"/>
+      <c r="K43" s="1661" t="n"/>
+      <c r="L43" s="1661" t="n"/>
+      <c r="M43" s="1659" t="n"/>
+      <c r="N43" s="1659" t="n"/>
+      <c r="O43" s="1659" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1626" t="n">
+      <c r="P43" s="1662" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1623" t="n"/>
-      <c r="R43" s="1623" t="n">
+      <c r="Q43" s="1659" t="n"/>
+      <c r="R43" s="1659" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1623" t="n"/>
+      <c r="S43" s="1659" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1622" t="n"/>
+      <c r="U43" s="1658" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -7940,45 +8066,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1651" t="inlineStr">
+      <c r="A44" s="1687" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1652" t="inlineStr">
+      <c r="B44" s="1688" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1652" t="inlineStr">
+      <c r="C44" s="1688" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1653" t="n"/>
-      <c r="E44" s="1653" t="n">
+      <c r="D44" s="1689" t="n"/>
+      <c r="E44" s="1689" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1653" t="n">
+      <c r="F44" s="1689" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1653" t="n"/>
-      <c r="H44" s="1653" t="n"/>
-      <c r="I44" s="1654" t="n"/>
-      <c r="J44" s="1655" t="n"/>
-      <c r="K44" s="1655" t="n"/>
-      <c r="L44" s="1655" t="n"/>
-      <c r="M44" s="1653" t="n"/>
-      <c r="N44" s="1653" t="n"/>
-      <c r="O44" s="1653" t="n"/>
-      <c r="P44" s="1656" t="n"/>
-      <c r="Q44" s="1653" t="n"/>
-      <c r="R44" s="1653" t="n"/>
-      <c r="S44" s="1653" t="n">
+      <c r="G44" s="1689" t="n"/>
+      <c r="H44" s="1689" t="n"/>
+      <c r="I44" s="1690" t="n"/>
+      <c r="J44" s="1691" t="n"/>
+      <c r="K44" s="1691" t="n"/>
+      <c r="L44" s="1691" t="n"/>
+      <c r="M44" s="1689" t="n"/>
+      <c r="N44" s="1689" t="n"/>
+      <c r="O44" s="1689" t="n"/>
+      <c r="P44" s="1692" t="n"/>
+      <c r="Q44" s="1689" t="n"/>
+      <c r="R44" s="1689" t="n"/>
+      <c r="S44" s="1689" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1652" t="inlineStr">
+      <c r="U44" s="1688" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -7990,49 +8116,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1651" t="inlineStr">
+      <c r="A45" s="1687" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1652" t="inlineStr">
+      <c r="B45" s="1688" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1652" t="inlineStr">
+      <c r="C45" s="1688" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1653" t="n"/>
-      <c r="E45" s="1653" t="n"/>
-      <c r="F45" s="1653" t="n"/>
-      <c r="G45" s="1653" t="n"/>
-      <c r="H45" s="1653" t="n">
+      <c r="D45" s="1689" t="n"/>
+      <c r="E45" s="1689" t="n"/>
+      <c r="F45" s="1689" t="n"/>
+      <c r="G45" s="1689" t="n"/>
+      <c r="H45" s="1689" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1654" t="n"/>
-      <c r="J45" s="1655" t="n"/>
-      <c r="K45" s="1655" t="n"/>
-      <c r="L45" s="1655" t="n"/>
-      <c r="M45" s="1653" t="n">
+      <c r="I45" s="1690" t="n"/>
+      <c r="J45" s="1691" t="n"/>
+      <c r="K45" s="1691" t="n"/>
+      <c r="L45" s="1691" t="n"/>
+      <c r="M45" s="1689" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1653" t="n">
+      <c r="N45" s="1689" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1653" t="n"/>
-      <c r="P45" s="1656" t="n"/>
-      <c r="Q45" s="1653" t="n"/>
-      <c r="R45" s="1653" t="n"/>
-      <c r="S45" s="1653" t="n"/>
+      <c r="O45" s="1689" t="n"/>
+      <c r="P45" s="1692" t="n"/>
+      <c r="Q45" s="1689" t="n"/>
+      <c r="R45" s="1689" t="n"/>
+      <c r="S45" s="1689" t="n"/>
       <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1652" t="n"/>
+      <c r="U45" s="1688" t="n"/>
       <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -8040,39 +8166,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1627" t="inlineStr">
+      <c r="A46" s="1663" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B46" s="1628" t="inlineStr">
+      <c r="B46" s="1664" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="C46" s="1628" t="inlineStr">
+      <c r="C46" s="1664" t="inlineStr">
         <is>
           <t>EVENT - Clean</t>
         </is>
       </c>
-      <c r="D46" s="1629" t="n"/>
-      <c r="E46" s="1629" t="n"/>
-      <c r="F46" s="1629" t="n"/>
-      <c r="G46" s="1629" t="n"/>
-      <c r="H46" s="1629" t="n"/>
-      <c r="I46" s="1630" t="n"/>
-      <c r="J46" s="1631" t="n"/>
-      <c r="K46" s="1631" t="n"/>
-      <c r="L46" s="1631" t="n"/>
-      <c r="M46" s="1629" t="n"/>
-      <c r="N46" s="1629" t="n"/>
-      <c r="O46" s="1629" t="n"/>
-      <c r="P46" s="1632" t="n"/>
-      <c r="Q46" s="1629" t="n"/>
-      <c r="R46" s="1629" t="n"/>
-      <c r="S46" s="1629" t="n"/>
+      <c r="D46" s="1665" t="n"/>
+      <c r="E46" s="1665" t="n"/>
+      <c r="F46" s="1665" t="n"/>
+      <c r="G46" s="1665" t="n"/>
+      <c r="H46" s="1665" t="n"/>
+      <c r="I46" s="1666" t="n"/>
+      <c r="J46" s="1667" t="n"/>
+      <c r="K46" s="1667" t="n"/>
+      <c r="L46" s="1667" t="n"/>
+      <c r="M46" s="1665" t="n"/>
+      <c r="N46" s="1665" t="n"/>
+      <c r="O46" s="1665" t="n"/>
+      <c r="P46" s="1668" t="n"/>
+      <c r="Q46" s="1665" t="n"/>
+      <c r="R46" s="1665" t="n"/>
+      <c r="S46" s="1665" t="n"/>
       <c r="T46" s="631" t="n"/>
-      <c r="U46" s="1628" t="n"/>
+      <c r="U46" s="1664" t="n"/>
       <c r="V46" s="632" t="inlineStr">
         <is>
           <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
@@ -8080,51 +8206,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1633" t="inlineStr">
+      <c r="A47" s="1669" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1634" t="inlineStr">
+      <c r="B47" s="1670" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C47" s="1634" t="inlineStr">
+      <c r="C47" s="1670" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D47" s="1635" t="n"/>
-      <c r="E47" s="1635" t="n">
+      <c r="D47" s="1671" t="n"/>
+      <c r="E47" s="1671" t="n">
         <v>16.6</v>
       </c>
-      <c r="F47" s="1635" t="n">
+      <c r="F47" s="1671" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="1635" t="n">
+      <c r="G47" s="1671" t="n">
         <v>4.1</v>
       </c>
-      <c r="H47" s="1635" t="n"/>
-      <c r="I47" s="1636" t="n">
+      <c r="H47" s="1671" t="n"/>
+      <c r="I47" s="1672" t="n">
         <v>0.9</v>
       </c>
-      <c r="J47" s="1637" t="n"/>
-      <c r="K47" s="1637" t="n"/>
-      <c r="L47" s="1637" t="n"/>
-      <c r="M47" s="1635" t="n"/>
-      <c r="N47" s="1635" t="n"/>
-      <c r="O47" s="1635" t="n">
+      <c r="J47" s="1673" t="n"/>
+      <c r="K47" s="1673" t="n"/>
+      <c r="L47" s="1673" t="n"/>
+      <c r="M47" s="1671" t="n"/>
+      <c r="N47" s="1671" t="n"/>
+      <c r="O47" s="1671" t="n">
         <v>13.2</v>
       </c>
-      <c r="P47" s="1638" t="n">
+      <c r="P47" s="1674" t="n">
         <v>0</v>
       </c>
-      <c r="Q47" s="1635" t="n"/>
-      <c r="R47" s="1635" t="n">
+      <c r="Q47" s="1671" t="n"/>
+      <c r="R47" s="1671" t="n">
         <v>84.5</v>
       </c>
-      <c r="S47" s="1635" t="n">
+      <c r="S47" s="1671" t="n">
         <v>11.8</v>
       </c>
       <c r="T47" s="813" t="inlineStr">
@@ -8132,7 +8258,7 @@
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1634" t="inlineStr">
+      <c r="U47" s="1670" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
@@ -8144,49 +8270,49 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1645" t="inlineStr">
+      <c r="A48" s="1681" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B48" s="1646" t="inlineStr">
+      <c r="B48" s="1682" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C48" s="1646" t="inlineStr">
+      <c r="C48" s="1682" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D48" s="1647" t="n"/>
-      <c r="E48" s="1647" t="n"/>
-      <c r="F48" s="1647" t="n"/>
-      <c r="G48" s="1647" t="n"/>
-      <c r="H48" s="1647" t="n">
+      <c r="D48" s="1683" t="n"/>
+      <c r="E48" s="1683" t="n"/>
+      <c r="F48" s="1683" t="n"/>
+      <c r="G48" s="1683" t="n"/>
+      <c r="H48" s="1683" t="n">
         <v>15.1</v>
       </c>
-      <c r="I48" s="1648" t="n"/>
-      <c r="J48" s="1649" t="n"/>
-      <c r="K48" s="1649" t="n"/>
-      <c r="L48" s="1649" t="n"/>
-      <c r="M48" s="1647" t="n">
+      <c r="I48" s="1684" t="n"/>
+      <c r="J48" s="1685" t="n"/>
+      <c r="K48" s="1685" t="n"/>
+      <c r="L48" s="1685" t="n"/>
+      <c r="M48" s="1683" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="1647" t="n">
+      <c r="N48" s="1683" t="n">
         <v>20</v>
       </c>
-      <c r="O48" s="1647" t="n"/>
-      <c r="P48" s="1650" t="n"/>
-      <c r="Q48" s="1647" t="n"/>
-      <c r="R48" s="1647" t="n"/>
-      <c r="S48" s="1647" t="n"/>
+      <c r="O48" s="1683" t="n"/>
+      <c r="P48" s="1686" t="n"/>
+      <c r="Q48" s="1683" t="n"/>
+      <c r="R48" s="1683" t="n"/>
+      <c r="S48" s="1683" t="n"/>
       <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U48" s="1646" t="n"/>
+      <c r="U48" s="1682" t="n"/>
       <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
@@ -8194,51 +8320,51 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1621" t="inlineStr">
+      <c r="A49" s="1657" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B49" s="1622" t="inlineStr">
+      <c r="B49" s="1658" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C49" s="1622" t="inlineStr">
+      <c r="C49" s="1658" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D49" s="1623" t="n"/>
-      <c r="E49" s="1623" t="n">
+      <c r="D49" s="1659" t="n"/>
+      <c r="E49" s="1659" t="n">
         <v>16.8</v>
       </c>
-      <c r="F49" s="1623" t="n">
+      <c r="F49" s="1659" t="n">
         <v>0.2</v>
       </c>
-      <c r="G49" s="1623" t="n">
+      <c r="G49" s="1659" t="n">
         <v>3.3</v>
       </c>
-      <c r="H49" s="1623" t="n"/>
-      <c r="I49" s="1624" t="n">
+      <c r="H49" s="1659" t="n"/>
+      <c r="I49" s="1660" t="n">
         <v>1.7</v>
       </c>
-      <c r="J49" s="1625" t="n"/>
-      <c r="K49" s="1625" t="n"/>
-      <c r="L49" s="1625" t="n"/>
-      <c r="M49" s="1623" t="n"/>
-      <c r="N49" s="1623" t="n"/>
-      <c r="O49" s="1623" t="n">
+      <c r="J49" s="1661" t="n"/>
+      <c r="K49" s="1661" t="n"/>
+      <c r="L49" s="1661" t="n"/>
+      <c r="M49" s="1659" t="n"/>
+      <c r="N49" s="1659" t="n"/>
+      <c r="O49" s="1659" t="n">
         <v>13</v>
       </c>
-      <c r="P49" s="1626" t="n">
+      <c r="P49" s="1662" t="n">
         <v>0.87</v>
       </c>
-      <c r="Q49" s="1623" t="n"/>
-      <c r="R49" s="1623" t="n">
+      <c r="Q49" s="1659" t="n"/>
+      <c r="R49" s="1659" t="n">
         <v>86</v>
       </c>
-      <c r="S49" s="1623" t="n">
+      <c r="S49" s="1659" t="n">
         <v>11.65</v>
       </c>
       <c r="T49" s="624" t="inlineStr">
@@ -8246,7 +8372,7 @@
           <t>Clear now, 88F, 67% RH; sun so far 6.4h of 7h daylight (91%); today high 90F, 0.87in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U49" s="1622" t="inlineStr">
+      <c r="U49" s="1658" t="inlineStr">
         <is>
           <t>2026-07-04_1.jpeg;2026-07-04_2.jpeg;2026-07-04_3.jpeg;2026-07-04_4.jpeg</t>
         </is>
@@ -8258,49 +8384,49 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1627" t="inlineStr">
+      <c r="A50" s="1663" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B50" s="1628" t="inlineStr">
+      <c r="B50" s="1664" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C50" s="1628" t="inlineStr">
+      <c r="C50" s="1664" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D50" s="1629" t="n"/>
-      <c r="E50" s="1629" t="n"/>
-      <c r="F50" s="1629" t="n"/>
-      <c r="G50" s="1629" t="n"/>
-      <c r="H50" s="1629" t="n">
+      <c r="D50" s="1665" t="n"/>
+      <c r="E50" s="1665" t="n"/>
+      <c r="F50" s="1665" t="n"/>
+      <c r="G50" s="1665" t="n"/>
+      <c r="H50" s="1665" t="n">
         <v>14.6</v>
       </c>
-      <c r="I50" s="1630" t="n"/>
-      <c r="J50" s="1631" t="n"/>
-      <c r="K50" s="1631" t="n"/>
-      <c r="L50" s="1631" t="n"/>
-      <c r="M50" s="1629" t="n">
+      <c r="I50" s="1666" t="n"/>
+      <c r="J50" s="1667" t="n"/>
+      <c r="K50" s="1667" t="n"/>
+      <c r="L50" s="1667" t="n"/>
+      <c r="M50" s="1665" t="n">
         <v>0.5</v>
       </c>
-      <c r="N50" s="1629" t="n">
+      <c r="N50" s="1665" t="n">
         <v>20.5</v>
       </c>
-      <c r="O50" s="1629" t="n"/>
-      <c r="P50" s="1632" t="n"/>
-      <c r="Q50" s="1629" t="n"/>
-      <c r="R50" s="1629" t="n"/>
-      <c r="S50" s="1629" t="n"/>
+      <c r="O50" s="1665" t="n"/>
+      <c r="P50" s="1668" t="n"/>
+      <c r="Q50" s="1665" t="n"/>
+      <c r="R50" s="1665" t="n"/>
+      <c r="S50" s="1665" t="n"/>
       <c r="T50" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny day (high 90F, water 86F); storm forecast overnight</t>
         </is>
       </c>
-      <c r="U50" s="1628" t="n"/>
+      <c r="U50" s="1664" t="n"/>
       <c r="V50" s="632" t="inlineStr">
         <is>
           <t>0.5 gal added 7:40 PM. PARTY PRE-LOAD (Sun 7/5 1PM picnic): deliberately HALF the usual dose -- FC already high at 16.8, and John didn't want to overshoot into the high teens for guests. Sized on the retuned model (l24_hot_sunny now 4.0). Model projects ~14.6 next noon, BUT this is a known weather-mismatch case: model keys L24 off today's hot/sunny weather, while the actual loss window is a storm overnight (no UV) + cooler/cloudy Sun morning -&gt; real loss will be LOWER, so FC likely lands ~15-16 at the party (comfortable top-of-band, cushion for bather load, not overboard). =&gt; If tomorrow's noon comes in ABOVE 14.6, that's the weather mismatch, NOT the freshly-retuned constant; don't chase it. Plan: dose back up Sun evening after the crowd's out (expect a bather-load FC drop). Season total 20.5 gal. PHOTOS(4): water clear/healthy blue, bottom fully visible, no cloudiness/algae; yesterday's surface debris now gone (tracks with CC clearing to 0.2); liner step close-up normal speckled blue, no rust/stain progression. Ruler photo documents the ~11.65 cm level.</t>
@@ -8308,47 +8434,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1633" t="inlineStr">
+      <c r="A51" s="1669" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B51" s="1634" t="inlineStr">
+      <c r="B51" s="1670" t="inlineStr">
         <is>
           <t>07:45</t>
         </is>
       </c>
-      <c r="C51" s="1634" t="inlineStr">
+      <c r="C51" s="1670" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D51" s="1635" t="n"/>
-      <c r="E51" s="1635" t="n">
+      <c r="D51" s="1671" t="n"/>
+      <c r="E51" s="1671" t="n">
         <v>16</v>
       </c>
-      <c r="F51" s="1635" t="n">
+      <c r="F51" s="1671" t="n">
         <v>0.5</v>
       </c>
-      <c r="G51" s="1635" t="n"/>
-      <c r="H51" s="1635" t="n"/>
-      <c r="I51" s="1636" t="n">
+      <c r="G51" s="1671" t="n"/>
+      <c r="H51" s="1671" t="n"/>
+      <c r="I51" s="1672" t="n">
         <v>1.4</v>
       </c>
-      <c r="J51" s="1637" t="n"/>
-      <c r="K51" s="1637" t="n"/>
-      <c r="L51" s="1637" t="n"/>
-      <c r="M51" s="1635" t="n"/>
-      <c r="N51" s="1635" t="n"/>
-      <c r="O51" s="1635" t="n"/>
-      <c r="P51" s="1638" t="n">
+      <c r="J51" s="1673" t="n"/>
+      <c r="K51" s="1673" t="n"/>
+      <c r="L51" s="1673" t="n"/>
+      <c r="M51" s="1671" t="n"/>
+      <c r="N51" s="1671" t="n"/>
+      <c r="O51" s="1671" t="n"/>
+      <c r="P51" s="1674" t="n">
         <v>0.04</v>
       </c>
-      <c r="Q51" s="1635" t="n"/>
-      <c r="R51" s="1635" t="n">
+      <c r="Q51" s="1671" t="n"/>
+      <c r="R51" s="1671" t="n">
         <v>84</v>
       </c>
-      <c r="S51" s="1635" t="n">
+      <c r="S51" s="1671" t="n">
         <v>13.9</v>
       </c>
       <c r="T51" s="813" t="inlineStr">
@@ -8356,7 +8482,7 @@
           <t>Overcast now, 75F, 90% RH; sun so far 0.0h of 3h daylight (0%); today high 75F, 0.04in precip, UV max 6.5</t>
         </is>
       </c>
-      <c r="U51" s="1634" t="inlineStr">
+      <c r="U51" s="1670" t="inlineStr">
         <is>
           <t>2026-07-05_2.jpeg</t>
         </is>
@@ -8368,41 +8494,41 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1639" t="inlineStr">
+      <c r="A52" s="1675" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B52" s="1640" t="inlineStr">
+      <c r="B52" s="1676" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C52" s="1640" t="inlineStr">
+      <c r="C52" s="1676" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D52" s="1641" t="n"/>
-      <c r="E52" s="1641" t="n">
+      <c r="D52" s="1677" t="n"/>
+      <c r="E52" s="1677" t="n">
         <v>14.8</v>
       </c>
-      <c r="F52" s="1641" t="n">
+      <c r="F52" s="1677" t="n">
         <v>0.3</v>
       </c>
-      <c r="G52" s="1641" t="n"/>
-      <c r="H52" s="1641" t="n"/>
-      <c r="I52" s="1642" t="n"/>
-      <c r="J52" s="1643" t="n"/>
-      <c r="K52" s="1643" t="n"/>
-      <c r="L52" s="1643" t="n"/>
-      <c r="M52" s="1641" t="n"/>
-      <c r="N52" s="1641" t="n"/>
-      <c r="O52" s="1641" t="n"/>
-      <c r="P52" s="1644" t="n"/>
-      <c r="Q52" s="1641" t="n"/>
-      <c r="R52" s="1641" t="n"/>
-      <c r="S52" s="1641" t="n">
+      <c r="G52" s="1677" t="n"/>
+      <c r="H52" s="1677" t="n"/>
+      <c r="I52" s="1678" t="n"/>
+      <c r="J52" s="1679" t="n"/>
+      <c r="K52" s="1679" t="n"/>
+      <c r="L52" s="1679" t="n"/>
+      <c r="M52" s="1677" t="n"/>
+      <c r="N52" s="1677" t="n"/>
+      <c r="O52" s="1677" t="n"/>
+      <c r="P52" s="1680" t="n"/>
+      <c r="Q52" s="1677" t="n"/>
+      <c r="R52" s="1677" t="n"/>
+      <c r="S52" s="1677" t="n">
         <v>13.6</v>
       </c>
       <c r="T52" s="820" t="inlineStr">
@@ -8410,7 +8536,7 @@
           <t>Overcast now, 72F, 76% RH; sun so far 8.4h of 13h daylight (65%); today high 80F, 0.00in precip, UV max 6.0</t>
         </is>
       </c>
-      <c r="U52" s="1640" t="inlineStr">
+      <c r="U52" s="1676" t="inlineStr">
         <is>
           <t>2026-07-05_1.jpeg;2026-07-05_3.jpeg</t>
         </is>
@@ -8422,49 +8548,49 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1645" t="inlineStr">
+      <c r="A53" s="1681" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B53" s="1646" t="inlineStr">
+      <c r="B53" s="1682" t="inlineStr">
         <is>
           <t>19:25</t>
         </is>
       </c>
-      <c r="C53" s="1646" t="inlineStr">
+      <c r="C53" s="1682" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D53" s="1647" t="n"/>
-      <c r="E53" s="1647" t="n"/>
-      <c r="F53" s="1647" t="n"/>
-      <c r="G53" s="1647" t="n"/>
-      <c r="H53" s="1647" t="n">
+      <c r="D53" s="1683" t="n"/>
+      <c r="E53" s="1683" t="n"/>
+      <c r="F53" s="1683" t="n"/>
+      <c r="G53" s="1683" t="n"/>
+      <c r="H53" s="1683" t="n">
         <v>15.1</v>
       </c>
-      <c r="I53" s="1648" t="n"/>
-      <c r="J53" s="1649" t="n"/>
-      <c r="K53" s="1649" t="n"/>
-      <c r="L53" s="1649" t="n"/>
-      <c r="M53" s="1647" t="n">
+      <c r="I53" s="1684" t="n"/>
+      <c r="J53" s="1685" t="n"/>
+      <c r="K53" s="1685" t="n"/>
+      <c r="L53" s="1685" t="n"/>
+      <c r="M53" s="1683" t="n">
         <v>0.5</v>
       </c>
-      <c r="N53" s="1647" t="n">
+      <c r="N53" s="1683" t="n">
         <v>21</v>
       </c>
-      <c r="O53" s="1647" t="n"/>
-      <c r="P53" s="1650" t="n"/>
-      <c r="Q53" s="1647" t="n"/>
-      <c r="R53" s="1647" t="n"/>
-      <c r="S53" s="1647" t="n"/>
+      <c r="O53" s="1683" t="n"/>
+      <c r="P53" s="1686" t="n"/>
+      <c r="Q53" s="1683" t="n"/>
+      <c r="R53" s="1683" t="n"/>
+      <c r="S53" s="1683" t="n"/>
       <c r="T53" s="827" t="inlineStr">
         <is>
           <t>Cleared to partly sunny (8.4 sun hrs, high 80F, water 84F); all-day rain forecast Mon 7/6</t>
         </is>
       </c>
-      <c r="U53" s="1646" t="n"/>
+      <c r="U53" s="1682" t="n"/>
       <c r="V53" s="828" t="inlineStr">
         <is>
           <t>0.5 gal added 7:25 PM (post-party recovery dose). Sized on TOMORROW's rainy forecast (the real loss window: overcast/wet 7/6, ~0.9in rain, low UV) not today's sun -&gt; projects ~15.1 at Mon noon. Party went great (FC held 16.0-&gt;14.8, CC dropped 0.5-&gt;0.3). Season total 21.0 gal. This is the first prediction that deliberately used the next-day forecast for L24 instead of the model's default (today's weather as proxy) -- if it lands near 15.1 tomorrow, that validates feeding the forecast on weather-change days.</t>
@@ -8472,49 +8598,49 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1621" t="inlineStr">
+      <c r="A54" s="1657" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B54" s="1622" t="inlineStr">
+      <c r="B54" s="1658" t="inlineStr">
         <is>
           <t>11:40</t>
         </is>
       </c>
-      <c r="C54" s="1622" t="inlineStr">
+      <c r="C54" s="1658" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D54" s="1623" t="n"/>
-      <c r="E54" s="1623" t="n">
+      <c r="D54" s="1659" t="n"/>
+      <c r="E54" s="1659" t="n">
         <v>13.8</v>
       </c>
-      <c r="F54" s="1623" t="n">
+      <c r="F54" s="1659" t="n">
         <v>0.2</v>
       </c>
-      <c r="G54" s="1623" t="n"/>
-      <c r="H54" s="1623" t="n"/>
-      <c r="I54" s="1624" t="n">
+      <c r="G54" s="1659" t="n"/>
+      <c r="H54" s="1659" t="n"/>
+      <c r="I54" s="1660" t="n">
         <v>-1.3</v>
       </c>
-      <c r="J54" s="1625" t="n"/>
-      <c r="K54" s="1625" t="n"/>
-      <c r="L54" s="1625" t="n"/>
-      <c r="M54" s="1623" t="n"/>
-      <c r="N54" s="1623" t="n"/>
-      <c r="O54" s="1623" t="n">
+      <c r="J54" s="1661" t="n"/>
+      <c r="K54" s="1661" t="n"/>
+      <c r="L54" s="1661" t="n"/>
+      <c r="M54" s="1659" t="n"/>
+      <c r="N54" s="1659" t="n"/>
+      <c r="O54" s="1659" t="n">
         <v>0</v>
       </c>
-      <c r="P54" s="1626" t="n">
+      <c r="P54" s="1662" t="n">
         <v>2</v>
       </c>
-      <c r="Q54" s="1623" t="n"/>
-      <c r="R54" s="1623" t="n">
+      <c r="Q54" s="1659" t="n"/>
+      <c r="R54" s="1659" t="n">
         <v>81</v>
       </c>
-      <c r="S54" s="1623" t="n">
+      <c r="S54" s="1659" t="n">
         <v>15.1</v>
       </c>
       <c r="T54" s="624" t="inlineStr">
@@ -8522,7 +8648,7 @@
           <t>Light rain now, 65F, 93% RH; sun so far 0.0h of 6h daylight (0%); today high 68F, 2.00in precip, UV max 0.5</t>
         </is>
       </c>
-      <c r="U54" s="1622" t="inlineStr">
+      <c r="U54" s="1658" t="inlineStr">
         <is>
           <t>2026-07-06_1.jpeg</t>
         </is>
@@ -8534,39 +8660,39 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1651" t="inlineStr">
+      <c r="A55" s="1687" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B55" s="1652" t="inlineStr">
+      <c r="B55" s="1688" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="C55" s="1652" t="inlineStr">
+      <c r="C55" s="1688" t="inlineStr">
         <is>
           <t>EVENT - Waste</t>
         </is>
       </c>
-      <c r="D55" s="1653" t="n"/>
-      <c r="E55" s="1653" t="n"/>
-      <c r="F55" s="1653" t="n"/>
-      <c r="G55" s="1653" t="n"/>
-      <c r="H55" s="1653" t="n"/>
-      <c r="I55" s="1654" t="n"/>
-      <c r="J55" s="1655" t="n"/>
-      <c r="K55" s="1655" t="n"/>
-      <c r="L55" s="1655" t="n"/>
-      <c r="M55" s="1653" t="n"/>
-      <c r="N55" s="1653" t="n"/>
-      <c r="O55" s="1653" t="n"/>
-      <c r="P55" s="1656" t="n"/>
-      <c r="Q55" s="1653" t="n"/>
-      <c r="R55" s="1653" t="n"/>
-      <c r="S55" s="1653" t="n"/>
+      <c r="D55" s="1689" t="n"/>
+      <c r="E55" s="1689" t="n"/>
+      <c r="F55" s="1689" t="n"/>
+      <c r="G55" s="1689" t="n"/>
+      <c r="H55" s="1689" t="n"/>
+      <c r="I55" s="1690" t="n"/>
+      <c r="J55" s="1691" t="n"/>
+      <c r="K55" s="1691" t="n"/>
+      <c r="L55" s="1691" t="n"/>
+      <c r="M55" s="1689" t="n"/>
+      <c r="N55" s="1689" t="n"/>
+      <c r="O55" s="1689" t="n"/>
+      <c r="P55" s="1692" t="n"/>
+      <c r="Q55" s="1689" t="n"/>
+      <c r="R55" s="1689" t="n"/>
+      <c r="S55" s="1689" t="n"/>
       <c r="T55" s="659" t="n"/>
-      <c r="U55" s="1652" t="inlineStr">
+      <c r="U55" s="1688" t="inlineStr">
         <is>
           <t>2026-07-06_2.jpeg;2026-07-06_3.jpeg</t>
         </is>
@@ -8578,52 +8704,112 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1627" t="inlineStr">
+      <c r="A56" s="1663" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B56" s="1628" t="inlineStr">
+      <c r="B56" s="1664" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C56" s="1628" t="inlineStr">
+      <c r="C56" s="1664" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D56" s="1629" t="n"/>
-      <c r="E56" s="1629" t="n"/>
-      <c r="F56" s="1629" t="n"/>
-      <c r="G56" s="1629" t="n"/>
-      <c r="H56" s="1629" t="n">
+      <c r="D56" s="1665" t="n"/>
+      <c r="E56" s="1665" t="n"/>
+      <c r="F56" s="1665" t="n"/>
+      <c r="G56" s="1665" t="n"/>
+      <c r="H56" s="1665" t="n">
         <v>14</v>
       </c>
-      <c r="I56" s="1630" t="n"/>
-      <c r="J56" s="1631" t="n"/>
-      <c r="K56" s="1631" t="n"/>
-      <c r="L56" s="1631" t="n"/>
-      <c r="M56" s="1629" t="n">
+      <c r="I56" s="1666" t="n"/>
+      <c r="J56" s="1667" t="n"/>
+      <c r="K56" s="1667" t="n"/>
+      <c r="L56" s="1667" t="n"/>
+      <c r="M56" s="1665" t="n">
         <v>1</v>
       </c>
-      <c r="N56" s="1629" t="n">
+      <c r="N56" s="1665" t="n">
         <v>22</v>
       </c>
-      <c r="O56" s="1629" t="n"/>
-      <c r="P56" s="1632" t="n"/>
-      <c r="Q56" s="1629" t="n"/>
-      <c r="R56" s="1629" t="n"/>
-      <c r="S56" s="1629" t="n"/>
+      <c r="O56" s="1665" t="n"/>
+      <c r="P56" s="1668" t="n"/>
+      <c r="Q56" s="1665" t="n"/>
+      <c r="R56" s="1665" t="n"/>
+      <c r="S56" s="1665" t="n"/>
       <c r="T56" s="631" t="inlineStr">
         <is>
           <t>Rain all day (2.00in total), overcast, 65-68F; more rain Tue</t>
         </is>
       </c>
-      <c r="U56" s="1628" t="n"/>
+      <c r="U56" s="1664" t="n"/>
       <c r="V56" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added 7:30 PM, AFTER the pump-to-waste (correct order -- don't chlorinate water you're about to pump out). FIRST dose on the recalibrated buckets (rain L24 now 2.5 vs old 1.5). CORRECTION carried in: John is NOT low on chlorine -- he was low on TEST REAGENTS, which arrived today -- so this is the full 1 gal (not the 0.5 I'd wrongly trimmed for 'conservation'). Base FC ~13 est (noon 13.8 minus the bit of FC removed by the pump-out; not re-tested), + 1gal x3.5 - 2.5 rain loss -&gt; pred ~14.0 at Tue noon. Prediction is confounded this round (pump perturbation + no post-empty FC test) -&gt; tomorrow's error will be noisy, don't read too much into it for bucket validation. Season total 22.0 gal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="1693" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B57" s="1694" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="C57" s="1694" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="D57" s="1695" t="n"/>
+      <c r="E57" s="1695" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="F57" s="1695" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G57" s="1695" t="n"/>
+      <c r="H57" s="1695" t="n"/>
+      <c r="I57" s="1696" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J57" s="1697" t="n"/>
+      <c r="K57" s="1697" t="n"/>
+      <c r="L57" s="1697" t="n"/>
+      <c r="M57" s="1695" t="n"/>
+      <c r="N57" s="1695" t="n"/>
+      <c r="O57" s="1695" t="n">
+        <v>0</v>
+      </c>
+      <c r="P57" s="1698" t="n"/>
+      <c r="Q57" s="1695" t="n"/>
+      <c r="R57" s="1695" t="n">
+        <v>76</v>
+      </c>
+      <c r="S57" s="1695" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="T57" s="1199" t="inlineStr">
+        <is>
+          <t>Overcast now, 66F, 91% RH; sun so far 0.0h of 6h daylight (0%); today high 69F, 0.00in precip, UV max 1.4</t>
+        </is>
+      </c>
+      <c r="U57" s="1694" t="inlineStr">
+        <is>
+          <t>2026-07-07_1.jpeg</t>
+        </is>
+      </c>
+      <c r="V57" s="1200" t="inlineStr">
+        <is>
+          <t>25mL x0.2. FC 14.6, CC 0.8 -- in band, healthy (FC/CYA 9.7%, comfortably above the ~7.5% min). PREDICTION: pred error +0.6 (actual 14.6 vs 7/6 dose's 14.0) -- FIRST noon on the recalibrated rain bucket (L24 2.5, up from old 1.5). Small miss, lost slightly LESS than modeled. CONFOUNDED though: yesterday's pump-to-waste removed chlorinated water + rain dilution, and the dose base FC was ESTIMATED ~13 (not re-tested post-empty) -- so do NOT retune off this single point. Directionally encouraging vs 7/6's -1.3 on the old 1.5 bucket (narrowing moved the rainy-day error from -1.3 toward 0). CC UP 0.2 -&gt; 0.8: two days of storm runoff washing organic/N load in (same mechanism as the 7/5 0.2-&gt;0.5 tick). 0.8 is above the 0.5 flag but still a trace; FC 14.6 is plenty to oxidize it -- expect it to clear over the next day or two now the rain has stopped. WATCH: if CC climbs toward 1.0+ or FC can't knock it down, revisit. fc_loss BLANK: noon-to-noon confounded by the pump-to-waste + 1gal dose + rain dilution -- not a clean value. Water temp 76 continues the cold-front slide (86-&gt;84-&gt;81-&gt;76); will rebound when sun returns. Level 15.5 cm (+0.4 vs yesterday's post-pump 15.1 -- overnight storm tail); rain has now STOPPED (feed 0.00in today) so the level should hold / slowly evaporate down -- no pump needed. rain_in left blank: trace overnight rise but no measurable daytime rain and the day isn't over. PHOTO documents the 15.5 level (tight ruler crop; water clear where visible, no debris).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log 2026-07-07 evening DOSE: 1.5 gal pre-load for away-day (pred 17.4 Wed noon; coast to ~13.5 Thu)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1699">
+  <cellXfs count="1735">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -5624,6 +5624,114 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="3" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -5885,7 +5993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V57"/>
+  <dimension ref="A1:V58"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col width="15.14" customWidth="1" min="1" max="1"/>
@@ -6062,35 +6170,35 @@
       <c r="V2" s="839" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="1657" t="inlineStr">
+      <c r="A3" s="1699" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B3" s="1658" t="n"/>
-      <c r="C3" s="1658" t="inlineStr">
+      <c r="B3" s="1700" t="n"/>
+      <c r="C3" s="1700" t="inlineStr">
         <is>
           <t>EVENT - Open</t>
         </is>
       </c>
-      <c r="D3" s="1659" t="n"/>
-      <c r="E3" s="1659" t="n"/>
-      <c r="F3" s="1659" t="n"/>
-      <c r="G3" s="1659" t="n"/>
-      <c r="H3" s="1659" t="n"/>
-      <c r="I3" s="1660" t="n"/>
-      <c r="J3" s="1661" t="n"/>
-      <c r="K3" s="1661" t="n"/>
-      <c r="L3" s="1661" t="n"/>
-      <c r="M3" s="1659" t="n"/>
-      <c r="N3" s="1659" t="n"/>
-      <c r="O3" s="1659" t="n"/>
-      <c r="P3" s="1662" t="n"/>
-      <c r="Q3" s="1659" t="n"/>
-      <c r="R3" s="1659" t="n"/>
-      <c r="S3" s="1659" t="n"/>
+      <c r="D3" s="1701" t="n"/>
+      <c r="E3" s="1701" t="n"/>
+      <c r="F3" s="1701" t="n"/>
+      <c r="G3" s="1701" t="n"/>
+      <c r="H3" s="1701" t="n"/>
+      <c r="I3" s="1702" t="n"/>
+      <c r="J3" s="1703" t="n"/>
+      <c r="K3" s="1703" t="n"/>
+      <c r="L3" s="1703" t="n"/>
+      <c r="M3" s="1701" t="n"/>
+      <c r="N3" s="1701" t="n"/>
+      <c r="O3" s="1701" t="n"/>
+      <c r="P3" s="1704" t="n"/>
+      <c r="Q3" s="1701" t="n"/>
+      <c r="R3" s="1701" t="n"/>
+      <c r="S3" s="1701" t="n"/>
       <c r="T3" s="624" t="n"/>
-      <c r="U3" s="1658" t="n"/>
+      <c r="U3" s="1700" t="n"/>
       <c r="V3" s="625" t="inlineStr">
         <is>
           <t>Pool open for season. Switched from trichlor tabs to liquid chlorine (Pool Tech 12.5%) due to high CYA. Pulled tabs from skimmer/feeder.</t>
@@ -6098,43 +6206,43 @@
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="1663" t="inlineStr">
+      <c r="A4" s="1705" t="inlineStr">
         <is>
           <t>2026-06-18</t>
         </is>
       </c>
-      <c r="B4" s="1664" t="inlineStr">
+      <c r="B4" s="1706" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C4" s="1664" t="inlineStr">
+      <c r="C4" s="1706" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D4" s="1665" t="n"/>
-      <c r="E4" s="1665" t="n"/>
-      <c r="F4" s="1665" t="n"/>
-      <c r="G4" s="1665" t="n"/>
-      <c r="H4" s="1665" t="n"/>
-      <c r="I4" s="1666" t="n"/>
-      <c r="J4" s="1667" t="n"/>
-      <c r="K4" s="1667" t="n"/>
-      <c r="L4" s="1667" t="n"/>
-      <c r="M4" s="1665" t="n">
+      <c r="D4" s="1707" t="n"/>
+      <c r="E4" s="1707" t="n"/>
+      <c r="F4" s="1707" t="n"/>
+      <c r="G4" s="1707" t="n"/>
+      <c r="H4" s="1707" t="n"/>
+      <c r="I4" s="1708" t="n"/>
+      <c r="J4" s="1709" t="n"/>
+      <c r="K4" s="1709" t="n"/>
+      <c r="L4" s="1709" t="n"/>
+      <c r="M4" s="1707" t="n">
         <v>3</v>
       </c>
-      <c r="N4" s="1665" t="n">
+      <c r="N4" s="1707" t="n">
         <v>3</v>
       </c>
-      <c r="O4" s="1665" t="n"/>
-      <c r="P4" s="1668" t="n"/>
-      <c r="Q4" s="1665" t="n"/>
-      <c r="R4" s="1665" t="n"/>
-      <c r="S4" s="1665" t="n"/>
+      <c r="O4" s="1707" t="n"/>
+      <c r="P4" s="1710" t="n"/>
+      <c r="Q4" s="1707" t="n"/>
+      <c r="R4" s="1707" t="n"/>
+      <c r="S4" s="1707" t="n"/>
       <c r="T4" s="631" t="n"/>
-      <c r="U4" s="1664" t="n"/>
+      <c r="U4" s="1706" t="n"/>
       <c r="V4" s="632" t="inlineStr">
         <is>
           <t>Initial 3 gal added; let pump run overnight to mix. FC before ~0.4.</t>
@@ -6142,57 +6250,57 @@
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="1669" t="inlineStr">
+      <c r="A5" s="1711" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B5" s="1670" t="inlineStr">
+      <c r="B5" s="1712" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C5" s="1670" t="inlineStr">
+      <c r="C5" s="1712" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D5" s="1671" t="n">
+      <c r="D5" s="1713" t="n">
         <v>7.3</v>
       </c>
-      <c r="E5" s="1671" t="n">
+      <c r="E5" s="1713" t="n">
         <v>3.4</v>
       </c>
-      <c r="F5" s="1671" t="n">
+      <c r="F5" s="1713" t="n">
         <v>0.2</v>
       </c>
-      <c r="G5" s="1671" t="n"/>
-      <c r="H5" s="1671" t="n"/>
-      <c r="I5" s="1672" t="n"/>
-      <c r="J5" s="1673" t="n">
+      <c r="G5" s="1713" t="n"/>
+      <c r="H5" s="1713" t="n"/>
+      <c r="I5" s="1714" t="n"/>
+      <c r="J5" s="1715" t="n">
         <v>140</v>
       </c>
-      <c r="K5" s="1673" t="n">
+      <c r="K5" s="1715" t="n">
         <v>160</v>
       </c>
-      <c r="L5" s="1673" t="inlineStr">
+      <c r="L5" s="1715" t="inlineStr">
         <is>
           <t>~100</t>
         </is>
       </c>
-      <c r="M5" s="1671" t="n"/>
-      <c r="N5" s="1671" t="n"/>
-      <c r="O5" s="1671" t="n">
+      <c r="M5" s="1713" t="n"/>
+      <c r="N5" s="1713" t="n"/>
+      <c r="O5" s="1713" t="n">
         <v>13.7</v>
       </c>
-      <c r="P5" s="1674" t="n">
+      <c r="P5" s="1716" t="n">
         <v>0</v>
       </c>
-      <c r="Q5" s="1671" t="n"/>
-      <c r="R5" s="1671" t="n"/>
-      <c r="S5" s="1671" t="n"/>
+      <c r="Q5" s="1713" t="n"/>
+      <c r="R5" s="1713" t="n"/>
+      <c r="S5" s="1713" t="n"/>
       <c r="T5" s="813" t="n"/>
-      <c r="U5" s="1670" t="n"/>
+      <c r="U5" s="1712" t="n"/>
       <c r="V5" s="814" t="inlineStr">
         <is>
           <t>25 mL fill, x0.2. First clean panel. (CYA later found &gt;100 - see 6/20.)</t>
@@ -6200,43 +6308,43 @@
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="1675" t="inlineStr">
+      <c r="A6" s="1717" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B6" s="1676" t="inlineStr">
+      <c r="B6" s="1718" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="C6" s="1676" t="inlineStr">
+      <c r="C6" s="1718" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D6" s="1677" t="n"/>
-      <c r="E6" s="1677" t="n"/>
-      <c r="F6" s="1677" t="n"/>
-      <c r="G6" s="1677" t="n"/>
-      <c r="H6" s="1677" t="n"/>
-      <c r="I6" s="1678" t="n"/>
-      <c r="J6" s="1679" t="n"/>
-      <c r="K6" s="1679" t="n"/>
-      <c r="L6" s="1679" t="n"/>
-      <c r="M6" s="1677" t="n">
+      <c r="D6" s="1719" t="n"/>
+      <c r="E6" s="1719" t="n"/>
+      <c r="F6" s="1719" t="n"/>
+      <c r="G6" s="1719" t="n"/>
+      <c r="H6" s="1719" t="n"/>
+      <c r="I6" s="1720" t="n"/>
+      <c r="J6" s="1721" t="n"/>
+      <c r="K6" s="1721" t="n"/>
+      <c r="L6" s="1721" t="n"/>
+      <c r="M6" s="1719" t="n">
         <v>1.5</v>
       </c>
-      <c r="N6" s="1677" t="n">
+      <c r="N6" s="1719" t="n">
         <v>4.5</v>
       </c>
-      <c r="O6" s="1677" t="n"/>
-      <c r="P6" s="1680" t="n"/>
-      <c r="Q6" s="1677" t="n"/>
-      <c r="R6" s="1677" t="n"/>
-      <c r="S6" s="1677" t="n"/>
+      <c r="O6" s="1719" t="n"/>
+      <c r="P6" s="1722" t="n"/>
+      <c r="Q6" s="1719" t="n"/>
+      <c r="R6" s="1719" t="n"/>
+      <c r="S6" s="1719" t="n"/>
       <c r="T6" s="820" t="n"/>
-      <c r="U6" s="1676" t="n"/>
+      <c r="U6" s="1718" t="n"/>
       <c r="V6" s="821" t="inlineStr">
         <is>
           <t>Added to correct low FC (3.4 below floor). Est. +5.1 -&gt; ~8.5. Pump running.</t>
@@ -6244,39 +6352,39 @@
       </c>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="1681" t="inlineStr">
+      <c r="A7" s="1723" t="inlineStr">
         <is>
           <t>2026-06-19</t>
         </is>
       </c>
-      <c r="B7" s="1682" t="inlineStr">
+      <c r="B7" s="1724" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C7" s="1682" t="inlineStr">
+      <c r="C7" s="1724" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D7" s="1683" t="n"/>
-      <c r="E7" s="1683" t="n"/>
-      <c r="F7" s="1683" t="n"/>
-      <c r="G7" s="1683" t="n"/>
-      <c r="H7" s="1683" t="n"/>
-      <c r="I7" s="1684" t="n"/>
-      <c r="J7" s="1685" t="n"/>
-      <c r="K7" s="1685" t="n"/>
-      <c r="L7" s="1685" t="n"/>
-      <c r="M7" s="1683" t="n"/>
-      <c r="N7" s="1683" t="n"/>
-      <c r="O7" s="1683" t="n"/>
-      <c r="P7" s="1686" t="n"/>
-      <c r="Q7" s="1683" t="n"/>
-      <c r="R7" s="1683" t="n"/>
-      <c r="S7" s="1683" t="n"/>
+      <c r="D7" s="1725" t="n"/>
+      <c r="E7" s="1725" t="n"/>
+      <c r="F7" s="1725" t="n"/>
+      <c r="G7" s="1725" t="n"/>
+      <c r="H7" s="1725" t="n"/>
+      <c r="I7" s="1726" t="n"/>
+      <c r="J7" s="1727" t="n"/>
+      <c r="K7" s="1727" t="n"/>
+      <c r="L7" s="1727" t="n"/>
+      <c r="M7" s="1725" t="n"/>
+      <c r="N7" s="1725" t="n"/>
+      <c r="O7" s="1725" t="n"/>
+      <c r="P7" s="1728" t="n"/>
+      <c r="Q7" s="1725" t="n"/>
+      <c r="R7" s="1725" t="n"/>
+      <c r="S7" s="1725" t="n"/>
       <c r="T7" s="827" t="n"/>
-      <c r="U7" s="1682" t="n"/>
+      <c r="U7" s="1724" t="n"/>
       <c r="V7" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -6284,39 +6392,39 @@
       </c>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="1657" t="inlineStr">
+      <c r="A8" s="1699" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B8" s="1658" t="inlineStr">
+      <c r="B8" s="1700" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C8" s="1658" t="inlineStr">
+      <c r="C8" s="1700" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D8" s="1659" t="n"/>
-      <c r="E8" s="1659" t="n"/>
-      <c r="F8" s="1659" t="n"/>
-      <c r="G8" s="1659" t="n"/>
-      <c r="H8" s="1659" t="n"/>
-      <c r="I8" s="1660" t="n"/>
-      <c r="J8" s="1661" t="n"/>
-      <c r="K8" s="1661" t="n"/>
-      <c r="L8" s="1661" t="n"/>
-      <c r="M8" s="1659" t="n"/>
-      <c r="N8" s="1659" t="n"/>
-      <c r="O8" s="1659" t="n"/>
-      <c r="P8" s="1662" t="n"/>
-      <c r="Q8" s="1659" t="n"/>
-      <c r="R8" s="1659" t="n"/>
-      <c r="S8" s="1659" t="n"/>
+      <c r="D8" s="1701" t="n"/>
+      <c r="E8" s="1701" t="n"/>
+      <c r="F8" s="1701" t="n"/>
+      <c r="G8" s="1701" t="n"/>
+      <c r="H8" s="1701" t="n"/>
+      <c r="I8" s="1702" t="n"/>
+      <c r="J8" s="1703" t="n"/>
+      <c r="K8" s="1703" t="n"/>
+      <c r="L8" s="1703" t="n"/>
+      <c r="M8" s="1701" t="n"/>
+      <c r="N8" s="1701" t="n"/>
+      <c r="O8" s="1701" t="n"/>
+      <c r="P8" s="1704" t="n"/>
+      <c r="Q8" s="1701" t="n"/>
+      <c r="R8" s="1701" t="n"/>
+      <c r="S8" s="1701" t="n"/>
       <c r="T8" s="624" t="n"/>
-      <c r="U8" s="1658" t="n"/>
+      <c r="U8" s="1700" t="n"/>
       <c r="V8" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (~7 AM, approximate - planned schedule).</t>
@@ -6324,63 +6432,63 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1687" t="inlineStr">
+      <c r="A9" s="1729" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B9" s="1688" t="inlineStr">
+      <c r="B9" s="1730" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C9" s="1688" t="inlineStr">
+      <c r="C9" s="1730" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D9" s="1689" t="n">
+      <c r="D9" s="1731" t="n">
         <v>7.3</v>
       </c>
-      <c r="E9" s="1689" t="n">
+      <c r="E9" s="1731" t="n">
         <v>4.6</v>
       </c>
-      <c r="F9" s="1689" t="n">
+      <c r="F9" s="1731" t="n">
         <v>0.2</v>
       </c>
-      <c r="G9" s="1689" t="n">
+      <c r="G9" s="1731" t="n">
         <v>4.1</v>
       </c>
-      <c r="H9" s="1689" t="n"/>
-      <c r="I9" s="1690" t="n"/>
-      <c r="J9" s="1691" t="n">
+      <c r="H9" s="1731" t="n"/>
+      <c r="I9" s="1732" t="n"/>
+      <c r="J9" s="1733" t="n">
         <v>130</v>
       </c>
-      <c r="K9" s="1691" t="n">
+      <c r="K9" s="1733" t="n">
         <v>150</v>
       </c>
-      <c r="L9" s="1691" t="inlineStr">
+      <c r="L9" s="1733" t="inlineStr">
         <is>
           <t>&gt;100</t>
         </is>
       </c>
-      <c r="M9" s="1689" t="n"/>
-      <c r="N9" s="1689" t="n"/>
-      <c r="O9" s="1689" t="n">
+      <c r="M9" s="1731" t="n"/>
+      <c r="N9" s="1731" t="n"/>
+      <c r="O9" s="1731" t="n">
         <v>14</v>
       </c>
-      <c r="P9" s="1692" t="n">
+      <c r="P9" s="1734" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="1689" t="n"/>
-      <c r="R9" s="1689" t="n"/>
-      <c r="S9" s="1689" t="n"/>
+      <c r="Q9" s="1731" t="n"/>
+      <c r="R9" s="1731" t="n"/>
+      <c r="S9" s="1731" t="n"/>
       <c r="T9" s="659" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, 80s</t>
         </is>
       </c>
-      <c r="U9" s="1688" t="n"/>
+      <c r="U9" s="1730" t="n"/>
       <c r="V9" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC dropped ~8.5-&gt;4.6 (~3.9/22hr) = ~4 ppm/day sunny-day loss. CYA off scale (&gt;100).</t>
@@ -6388,43 +6496,43 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1687" t="inlineStr">
+      <c r="A10" s="1729" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B10" s="1688" t="inlineStr">
+      <c r="B10" s="1730" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C10" s="1688" t="inlineStr">
+      <c r="C10" s="1730" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D10" s="1689" t="n"/>
-      <c r="E10" s="1689" t="n"/>
-      <c r="F10" s="1689" t="n"/>
-      <c r="G10" s="1689" t="n"/>
-      <c r="H10" s="1689" t="n"/>
-      <c r="I10" s="1690" t="n"/>
-      <c r="J10" s="1691" t="n"/>
-      <c r="K10" s="1691" t="n"/>
-      <c r="L10" s="1691" t="inlineStr">
+      <c r="D10" s="1731" t="n"/>
+      <c r="E10" s="1731" t="n"/>
+      <c r="F10" s="1731" t="n"/>
+      <c r="G10" s="1731" t="n"/>
+      <c r="H10" s="1731" t="n"/>
+      <c r="I10" s="1732" t="n"/>
+      <c r="J10" s="1733" t="n"/>
+      <c r="K10" s="1733" t="n"/>
+      <c r="L10" s="1733" t="inlineStr">
         <is>
           <t>~160</t>
         </is>
       </c>
-      <c r="M10" s="1689" t="n"/>
-      <c r="N10" s="1689" t="n"/>
-      <c r="O10" s="1689" t="n"/>
-      <c r="P10" s="1692" t="n"/>
-      <c r="Q10" s="1689" t="n"/>
-      <c r="R10" s="1689" t="n"/>
-      <c r="S10" s="1689" t="n"/>
+      <c r="M10" s="1731" t="n"/>
+      <c r="N10" s="1731" t="n"/>
+      <c r="O10" s="1731" t="n"/>
+      <c r="P10" s="1734" t="n"/>
+      <c r="Q10" s="1731" t="n"/>
+      <c r="R10" s="1731" t="n"/>
+      <c r="S10" s="1731" t="n"/>
       <c r="T10" s="659" t="n"/>
-      <c r="U10" s="1688" t="n"/>
+      <c r="U10" s="1730" t="n"/>
       <c r="V10" s="660" t="inlineStr">
         <is>
           <t>Diluted CYA test: 50/50 pool+distilled read ~80, x2 = ~160. Old reagents, approximate (+/-15).</t>
@@ -6432,43 +6540,43 @@
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="1687" t="inlineStr">
+      <c r="A11" s="1729" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B11" s="1688" t="inlineStr">
+      <c r="B11" s="1730" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C11" s="1688" t="inlineStr">
+      <c r="C11" s="1730" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D11" s="1689" t="n"/>
-      <c r="E11" s="1689" t="n"/>
-      <c r="F11" s="1689" t="n"/>
-      <c r="G11" s="1689" t="n"/>
-      <c r="H11" s="1689" t="n"/>
-      <c r="I11" s="1690" t="n"/>
-      <c r="J11" s="1691" t="n"/>
-      <c r="K11" s="1691" t="n"/>
-      <c r="L11" s="1691" t="n"/>
-      <c r="M11" s="1689" t="n">
+      <c r="D11" s="1731" t="n"/>
+      <c r="E11" s="1731" t="n"/>
+      <c r="F11" s="1731" t="n"/>
+      <c r="G11" s="1731" t="n"/>
+      <c r="H11" s="1731" t="n"/>
+      <c r="I11" s="1732" t="n"/>
+      <c r="J11" s="1733" t="n"/>
+      <c r="K11" s="1733" t="n"/>
+      <c r="L11" s="1733" t="n"/>
+      <c r="M11" s="1731" t="n">
         <v>2</v>
       </c>
-      <c r="N11" s="1689" t="n">
+      <c r="N11" s="1731" t="n">
         <v>6.5</v>
       </c>
-      <c r="O11" s="1689" t="n"/>
-      <c r="P11" s="1692" t="n"/>
-      <c r="Q11" s="1689" t="n"/>
-      <c r="R11" s="1689" t="n"/>
-      <c r="S11" s="1689" t="n"/>
+      <c r="O11" s="1731" t="n"/>
+      <c r="P11" s="1734" t="n"/>
+      <c r="Q11" s="1731" t="n"/>
+      <c r="R11" s="1731" t="n"/>
+      <c r="S11" s="1731" t="n"/>
       <c r="T11" s="659" t="n"/>
-      <c r="U11" s="1688" t="n"/>
+      <c r="U11" s="1730" t="n"/>
       <c r="V11" s="660" t="inlineStr">
         <is>
           <t>Top-up toward target band for CYA ~160 (floor ~11).</t>
@@ -6476,39 +6584,39 @@
       </c>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="1663" t="inlineStr">
+      <c r="A12" s="1705" t="inlineStr">
         <is>
           <t>2026-06-20</t>
         </is>
       </c>
-      <c r="B12" s="1664" t="inlineStr">
+      <c r="B12" s="1706" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="C12" s="1664" t="inlineStr">
+      <c r="C12" s="1706" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D12" s="1665" t="n"/>
-      <c r="E12" s="1665" t="n"/>
-      <c r="F12" s="1665" t="n"/>
-      <c r="G12" s="1665" t="n"/>
-      <c r="H12" s="1665" t="n"/>
-      <c r="I12" s="1666" t="n"/>
-      <c r="J12" s="1667" t="n"/>
-      <c r="K12" s="1667" t="n"/>
-      <c r="L12" s="1667" t="n"/>
-      <c r="M12" s="1665" t="n"/>
-      <c r="N12" s="1665" t="n"/>
-      <c r="O12" s="1665" t="n"/>
-      <c r="P12" s="1668" t="n"/>
-      <c r="Q12" s="1665" t="n"/>
-      <c r="R12" s="1665" t="n"/>
-      <c r="S12" s="1665" t="n"/>
+      <c r="D12" s="1707" t="n"/>
+      <c r="E12" s="1707" t="n"/>
+      <c r="F12" s="1707" t="n"/>
+      <c r="G12" s="1707" t="n"/>
+      <c r="H12" s="1707" t="n"/>
+      <c r="I12" s="1708" t="n"/>
+      <c r="J12" s="1709" t="n"/>
+      <c r="K12" s="1709" t="n"/>
+      <c r="L12" s="1709" t="n"/>
+      <c r="M12" s="1707" t="n"/>
+      <c r="N12" s="1707" t="n"/>
+      <c r="O12" s="1707" t="n"/>
+      <c r="P12" s="1710" t="n"/>
+      <c r="Q12" s="1707" t="n"/>
+      <c r="R12" s="1707" t="n"/>
+      <c r="S12" s="1707" t="n"/>
       <c r="T12" s="631" t="n"/>
-      <c r="U12" s="1664" t="n"/>
+      <c r="U12" s="1706" t="n"/>
       <c r="V12" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10 PM, approximate - planned schedule).</t>
@@ -6516,35 +6624,35 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="1669" t="inlineStr">
+      <c r="A13" s="1711" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B13" s="1670" t="n"/>
-      <c r="C13" s="1670" t="inlineStr">
+      <c r="B13" s="1712" t="n"/>
+      <c r="C13" s="1712" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D13" s="1671" t="n"/>
-      <c r="E13" s="1671" t="n"/>
-      <c r="F13" s="1671" t="n"/>
-      <c r="G13" s="1671" t="n"/>
-      <c r="H13" s="1671" t="n"/>
-      <c r="I13" s="1672" t="n"/>
-      <c r="J13" s="1673" t="n"/>
-      <c r="K13" s="1673" t="n"/>
-      <c r="L13" s="1673" t="n"/>
-      <c r="M13" s="1671" t="n"/>
-      <c r="N13" s="1671" t="n"/>
-      <c r="O13" s="1671" t="n"/>
-      <c r="P13" s="1674" t="n"/>
-      <c r="Q13" s="1671" t="n"/>
-      <c r="R13" s="1671" t="n"/>
-      <c r="S13" s="1671" t="n"/>
+      <c r="D13" s="1713" t="n"/>
+      <c r="E13" s="1713" t="n"/>
+      <c r="F13" s="1713" t="n"/>
+      <c r="G13" s="1713" t="n"/>
+      <c r="H13" s="1713" t="n"/>
+      <c r="I13" s="1714" t="n"/>
+      <c r="J13" s="1715" t="n"/>
+      <c r="K13" s="1715" t="n"/>
+      <c r="L13" s="1715" t="n"/>
+      <c r="M13" s="1713" t="n"/>
+      <c r="N13" s="1713" t="n"/>
+      <c r="O13" s="1713" t="n"/>
+      <c r="P13" s="1716" t="n"/>
+      <c r="Q13" s="1713" t="n"/>
+      <c r="R13" s="1713" t="n"/>
+      <c r="S13" s="1713" t="n"/>
       <c r="T13" s="813" t="n"/>
-      <c r="U13" s="1670" t="n"/>
+      <c r="U13" s="1712" t="n"/>
       <c r="V13" s="814" t="inlineStr">
         <is>
           <t>No water added today. Dog swam ~1 min (negligible load). Rain expected 6/22 afternoon.</t>
@@ -6552,53 +6660,53 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="1675" t="inlineStr">
+      <c r="A14" s="1717" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B14" s="1676" t="inlineStr">
+      <c r="B14" s="1718" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="C14" s="1676" t="inlineStr">
+      <c r="C14" s="1718" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D14" s="1677" t="n"/>
-      <c r="E14" s="1677" t="n">
+      <c r="D14" s="1719" t="n"/>
+      <c r="E14" s="1719" t="n">
         <v>10.2</v>
       </c>
-      <c r="F14" s="1677" t="n">
+      <c r="F14" s="1719" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="1677" t="n">
+      <c r="G14" s="1719" t="n">
         <v>1.4</v>
       </c>
-      <c r="H14" s="1677" t="n"/>
-      <c r="I14" s="1678" t="n"/>
-      <c r="J14" s="1679" t="n"/>
-      <c r="K14" s="1679" t="n"/>
-      <c r="L14" s="1679" t="n"/>
-      <c r="M14" s="1677" t="n"/>
-      <c r="N14" s="1677" t="n"/>
-      <c r="O14" s="1677" t="n">
+      <c r="H14" s="1719" t="n"/>
+      <c r="I14" s="1720" t="n"/>
+      <c r="J14" s="1721" t="n"/>
+      <c r="K14" s="1721" t="n"/>
+      <c r="L14" s="1721" t="n"/>
+      <c r="M14" s="1719" t="n"/>
+      <c r="N14" s="1719" t="n"/>
+      <c r="O14" s="1719" t="n">
         <v>13.6</v>
       </c>
-      <c r="P14" s="1680" t="n">
+      <c r="P14" s="1722" t="n">
         <v>0</v>
       </c>
-      <c r="Q14" s="1677" t="n"/>
-      <c r="R14" s="1677" t="n"/>
-      <c r="S14" s="1677" t="n"/>
+      <c r="Q14" s="1719" t="n"/>
+      <c r="R14" s="1719" t="n"/>
+      <c r="S14" s="1719" t="n"/>
       <c r="T14" s="820" t="inlineStr">
         <is>
           <t>Super sunny, dry, low humidity, low-mid 80s</t>
         </is>
       </c>
-      <c r="U14" s="1676" t="n"/>
+      <c r="U14" s="1718" t="n"/>
       <c r="V14" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 10.2 (just below floor 11), CC 0.</t>
@@ -6606,43 +6714,43 @@
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="1675" t="inlineStr">
+      <c r="A15" s="1717" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B15" s="1676" t="inlineStr">
+      <c r="B15" s="1718" t="inlineStr">
         <is>
           <t>~11:30</t>
         </is>
       </c>
-      <c r="C15" s="1676" t="inlineStr">
+      <c r="C15" s="1718" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D15" s="1677" t="n"/>
-      <c r="E15" s="1677" t="n"/>
-      <c r="F15" s="1677" t="n"/>
-      <c r="G15" s="1677" t="n"/>
-      <c r="H15" s="1677" t="n"/>
-      <c r="I15" s="1678" t="n"/>
-      <c r="J15" s="1679" t="n"/>
-      <c r="K15" s="1679" t="n"/>
-      <c r="L15" s="1679" t="n"/>
-      <c r="M15" s="1677" t="n">
+      <c r="D15" s="1719" t="n"/>
+      <c r="E15" s="1719" t="n"/>
+      <c r="F15" s="1719" t="n"/>
+      <c r="G15" s="1719" t="n"/>
+      <c r="H15" s="1719" t="n"/>
+      <c r="I15" s="1720" t="n"/>
+      <c r="J15" s="1721" t="n"/>
+      <c r="K15" s="1721" t="n"/>
+      <c r="L15" s="1721" t="n"/>
+      <c r="M15" s="1719" t="n">
         <v>1.5</v>
       </c>
-      <c r="N15" s="1677" t="n">
+      <c r="N15" s="1719" t="n">
         <v>8</v>
       </c>
-      <c r="O15" s="1677" t="n"/>
-      <c r="P15" s="1680" t="n"/>
-      <c r="Q15" s="1677" t="n"/>
-      <c r="R15" s="1677" t="n"/>
-      <c r="S15" s="1677" t="n"/>
+      <c r="O15" s="1719" t="n"/>
+      <c r="P15" s="1722" t="n"/>
+      <c r="Q15" s="1719" t="n"/>
+      <c r="R15" s="1719" t="n"/>
+      <c r="S15" s="1719" t="n"/>
       <c r="T15" s="820" t="n"/>
-      <c r="U15" s="1676" t="n"/>
+      <c r="U15" s="1718" t="n"/>
       <c r="V15" s="821" t="inlineStr">
         <is>
           <t>Target top of band ~16. 1.5 gal ~ +5.3 -&gt; ~15.5. Pump running.</t>
@@ -6650,39 +6758,39 @@
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="1681" t="inlineStr">
+      <c r="A16" s="1723" t="inlineStr">
         <is>
           <t>2026-06-21</t>
         </is>
       </c>
-      <c r="B16" s="1682" t="inlineStr">
+      <c r="B16" s="1724" t="inlineStr">
         <is>
           <t>22:40</t>
         </is>
       </c>
-      <c r="C16" s="1682" t="inlineStr">
+      <c r="C16" s="1724" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D16" s="1683" t="n"/>
-      <c r="E16" s="1683" t="n"/>
-      <c r="F16" s="1683" t="n"/>
-      <c r="G16" s="1683" t="n"/>
-      <c r="H16" s="1683" t="n"/>
-      <c r="I16" s="1684" t="n"/>
-      <c r="J16" s="1685" t="n"/>
-      <c r="K16" s="1685" t="n"/>
-      <c r="L16" s="1685" t="n"/>
-      <c r="M16" s="1683" t="n"/>
-      <c r="N16" s="1683" t="n"/>
-      <c r="O16" s="1683" t="n"/>
-      <c r="P16" s="1686" t="n"/>
-      <c r="Q16" s="1683" t="n"/>
-      <c r="R16" s="1683" t="n"/>
-      <c r="S16" s="1683" t="n"/>
+      <c r="D16" s="1725" t="n"/>
+      <c r="E16" s="1725" t="n"/>
+      <c r="F16" s="1725" t="n"/>
+      <c r="G16" s="1725" t="n"/>
+      <c r="H16" s="1725" t="n"/>
+      <c r="I16" s="1726" t="n"/>
+      <c r="J16" s="1727" t="n"/>
+      <c r="K16" s="1727" t="n"/>
+      <c r="L16" s="1727" t="n"/>
+      <c r="M16" s="1725" t="n"/>
+      <c r="N16" s="1725" t="n"/>
+      <c r="O16" s="1725" t="n"/>
+      <c r="P16" s="1728" t="n"/>
+      <c r="Q16" s="1725" t="n"/>
+      <c r="R16" s="1725" t="n"/>
+      <c r="S16" s="1725" t="n"/>
       <c r="T16" s="827" t="n"/>
-      <c r="U16" s="1682" t="n"/>
+      <c r="U16" s="1724" t="n"/>
       <c r="V16" s="828" t="inlineStr">
         <is>
           <t>Pump OFF for night (~10:40 PM).</t>
@@ -6690,39 +6798,39 @@
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="1657" t="inlineStr">
+      <c r="A17" s="1699" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B17" s="1658" t="inlineStr">
+      <c r="B17" s="1700" t="inlineStr">
         <is>
           <t>07:00</t>
         </is>
       </c>
-      <c r="C17" s="1658" t="inlineStr">
+      <c r="C17" s="1700" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D17" s="1659" t="n"/>
-      <c r="E17" s="1659" t="n"/>
-      <c r="F17" s="1659" t="n"/>
-      <c r="G17" s="1659" t="n"/>
-      <c r="H17" s="1659" t="n"/>
-      <c r="I17" s="1660" t="n"/>
-      <c r="J17" s="1661" t="n"/>
-      <c r="K17" s="1661" t="n"/>
-      <c r="L17" s="1661" t="n"/>
-      <c r="M17" s="1659" t="n"/>
-      <c r="N17" s="1659" t="n"/>
-      <c r="O17" s="1659" t="n"/>
-      <c r="P17" s="1662" t="n"/>
-      <c r="Q17" s="1659" t="n"/>
-      <c r="R17" s="1659" t="n"/>
-      <c r="S17" s="1659" t="n"/>
+      <c r="D17" s="1701" t="n"/>
+      <c r="E17" s="1701" t="n"/>
+      <c r="F17" s="1701" t="n"/>
+      <c r="G17" s="1701" t="n"/>
+      <c r="H17" s="1701" t="n"/>
+      <c r="I17" s="1702" t="n"/>
+      <c r="J17" s="1703" t="n"/>
+      <c r="K17" s="1703" t="n"/>
+      <c r="L17" s="1703" t="n"/>
+      <c r="M17" s="1701" t="n"/>
+      <c r="N17" s="1701" t="n"/>
+      <c r="O17" s="1701" t="n"/>
+      <c r="P17" s="1704" t="n"/>
+      <c r="Q17" s="1701" t="n"/>
+      <c r="R17" s="1701" t="n"/>
+      <c r="S17" s="1701" t="n"/>
       <c r="T17" s="624" t="n"/>
-      <c r="U17" s="1658" t="n"/>
+      <c r="U17" s="1700" t="n"/>
       <c r="V17" s="625" t="inlineStr">
         <is>
           <t>Pump ON for the day (7 AM).</t>
@@ -6730,53 +6838,53 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="1687" t="inlineStr">
+      <c r="A18" s="1729" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B18" s="1688" t="inlineStr">
+      <c r="B18" s="1730" t="inlineStr">
         <is>
           <t>11:55</t>
         </is>
       </c>
-      <c r="C18" s="1688" t="inlineStr">
+      <c r="C18" s="1730" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D18" s="1689" t="n"/>
-      <c r="E18" s="1689" t="n">
+      <c r="D18" s="1731" t="n"/>
+      <c r="E18" s="1731" t="n">
         <v>12</v>
       </c>
-      <c r="F18" s="1689" t="n">
+      <c r="F18" s="1731" t="n">
         <v>0.4</v>
       </c>
-      <c r="G18" s="1689" t="n">
+      <c r="G18" s="1731" t="n">
         <v>3.4</v>
       </c>
-      <c r="H18" s="1689" t="n"/>
-      <c r="I18" s="1690" t="n"/>
-      <c r="J18" s="1691" t="n"/>
-      <c r="K18" s="1691" t="n"/>
-      <c r="L18" s="1691" t="n"/>
-      <c r="M18" s="1689" t="n"/>
-      <c r="N18" s="1689" t="n"/>
-      <c r="O18" s="1689" t="n">
+      <c r="H18" s="1731" t="n"/>
+      <c r="I18" s="1732" t="n"/>
+      <c r="J18" s="1733" t="n"/>
+      <c r="K18" s="1733" t="n"/>
+      <c r="L18" s="1733" t="n"/>
+      <c r="M18" s="1731" t="n"/>
+      <c r="N18" s="1731" t="n"/>
+      <c r="O18" s="1731" t="n">
         <v>0.3</v>
       </c>
-      <c r="P18" s="1692" t="n">
+      <c r="P18" s="1734" t="n">
         <v>0.33</v>
       </c>
-      <c r="Q18" s="1689" t="n"/>
-      <c r="R18" s="1689" t="n"/>
-      <c r="S18" s="1689" t="n"/>
+      <c r="Q18" s="1731" t="n"/>
+      <c r="R18" s="1731" t="n"/>
+      <c r="S18" s="1731" t="n"/>
       <c r="T18" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F, 74% humidity, 0 in precip</t>
         </is>
       </c>
-      <c r="U18" s="1688" t="n"/>
+      <c r="U18" s="1730" t="n"/>
       <c r="V18" s="660" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 12.0 (above floor 11, below target band 13-16), CC 0.4 (slightly above ~0 goal). Cool/cloudy = low UV loss day.</t>
@@ -6784,47 +6892,47 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="1687" t="inlineStr">
+      <c r="A19" s="1729" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B19" s="1688" t="inlineStr">
+      <c r="B19" s="1730" t="inlineStr">
         <is>
           <t>12:00</t>
         </is>
       </c>
-      <c r="C19" s="1688" t="inlineStr">
+      <c r="C19" s="1730" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D19" s="1689" t="n"/>
-      <c r="E19" s="1689" t="n"/>
-      <c r="F19" s="1689" t="n"/>
-      <c r="G19" s="1689" t="n"/>
-      <c r="H19" s="1689" t="n"/>
-      <c r="I19" s="1690" t="n"/>
-      <c r="J19" s="1691" t="n"/>
-      <c r="K19" s="1691" t="n"/>
-      <c r="L19" s="1691" t="n"/>
-      <c r="M19" s="1689" t="n">
+      <c r="D19" s="1731" t="n"/>
+      <c r="E19" s="1731" t="n"/>
+      <c r="F19" s="1731" t="n"/>
+      <c r="G19" s="1731" t="n"/>
+      <c r="H19" s="1731" t="n"/>
+      <c r="I19" s="1732" t="n"/>
+      <c r="J19" s="1733" t="n"/>
+      <c r="K19" s="1733" t="n"/>
+      <c r="L19" s="1733" t="n"/>
+      <c r="M19" s="1731" t="n">
         <v>1</v>
       </c>
-      <c r="N19" s="1689" t="n">
+      <c r="N19" s="1731" t="n">
         <v>9</v>
       </c>
-      <c r="O19" s="1689" t="n"/>
-      <c r="P19" s="1692" t="n"/>
-      <c r="Q19" s="1689" t="n"/>
-      <c r="R19" s="1689" t="n"/>
-      <c r="S19" s="1689" t="n"/>
+      <c r="O19" s="1731" t="n"/>
+      <c r="P19" s="1734" t="n"/>
+      <c r="Q19" s="1731" t="n"/>
+      <c r="R19" s="1731" t="n"/>
+      <c r="S19" s="1731" t="n"/>
       <c r="T19" s="659" t="inlineStr">
         <is>
           <t>Mostly cloudy, 69F</t>
         </is>
       </c>
-      <c r="U19" s="1688" t="n"/>
+      <c r="U19" s="1730" t="n"/>
       <c r="V19" s="660" t="inlineStr">
         <is>
           <t>Dose to ~16 top of band. 1.0 gal ~ +3.5 -&gt; ~15.5. Conservative on a low-loss cloudy day. Higher FC should clear CC 0.4 by tomorrow. Pump running.</t>
@@ -6832,43 +6940,43 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="1687" t="inlineStr">
+      <c r="A20" s="1729" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B20" s="1688" t="inlineStr">
+      <c r="B20" s="1730" t="inlineStr">
         <is>
           <t>afternoon</t>
         </is>
       </c>
-      <c r="C20" s="1688" t="inlineStr">
+      <c r="C20" s="1730" t="inlineStr">
         <is>
           <t>EVENT - Storm</t>
         </is>
       </c>
-      <c r="D20" s="1689" t="n"/>
-      <c r="E20" s="1689" t="n"/>
-      <c r="F20" s="1689" t="n"/>
-      <c r="G20" s="1689" t="n"/>
-      <c r="H20" s="1689" t="n"/>
-      <c r="I20" s="1690" t="n"/>
-      <c r="J20" s="1691" t="n"/>
-      <c r="K20" s="1691" t="n"/>
-      <c r="L20" s="1691" t="n"/>
-      <c r="M20" s="1689" t="n"/>
-      <c r="N20" s="1689" t="n"/>
-      <c r="O20" s="1689" t="n"/>
-      <c r="P20" s="1692" t="n"/>
-      <c r="Q20" s="1689" t="n"/>
-      <c r="R20" s="1689" t="n"/>
-      <c r="S20" s="1689" t="n"/>
+      <c r="D20" s="1731" t="n"/>
+      <c r="E20" s="1731" t="n"/>
+      <c r="F20" s="1731" t="n"/>
+      <c r="G20" s="1731" t="n"/>
+      <c r="H20" s="1731" t="n"/>
+      <c r="I20" s="1732" t="n"/>
+      <c r="J20" s="1733" t="n"/>
+      <c r="K20" s="1733" t="n"/>
+      <c r="L20" s="1733" t="n"/>
+      <c r="M20" s="1731" t="n"/>
+      <c r="N20" s="1731" t="n"/>
+      <c r="O20" s="1731" t="n"/>
+      <c r="P20" s="1734" t="n"/>
+      <c r="Q20" s="1731" t="n"/>
+      <c r="R20" s="1731" t="n"/>
+      <c r="S20" s="1731" t="n"/>
       <c r="T20" s="659" t="inlineStr">
         <is>
           <t>Rain/thunderstorms 1 PM through overnight</t>
         </is>
       </c>
-      <c r="U20" s="1688" t="n"/>
+      <c r="U20" s="1730" t="n"/>
       <c r="V20" s="660" t="inlineStr">
         <is>
           <t>Forecast: showers building ~1 PM, peak ~6 PM (96%, 0.12 in), rain/TS all evening + overnight. Est. ~0.3-0.4 in today, ~1+ in through Tue AM. ~1,000+ gal rainwater into 34,400 gal pool = passive CYA dilution (~2-3%). Plenty of freeboard, no overfill concern. Negligible FC loss (no UV).</t>
@@ -6876,39 +6984,39 @@
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="1663" t="inlineStr">
+      <c r="A21" s="1705" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="B21" s="1664" t="inlineStr">
+      <c r="B21" s="1706" t="inlineStr">
         <is>
           <t>22:10</t>
         </is>
       </c>
-      <c r="C21" s="1664" t="inlineStr">
+      <c r="C21" s="1706" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D21" s="1665" t="n"/>
-      <c r="E21" s="1665" t="n"/>
-      <c r="F21" s="1665" t="n"/>
-      <c r="G21" s="1665" t="n"/>
-      <c r="H21" s="1665" t="n"/>
-      <c r="I21" s="1666" t="n"/>
-      <c r="J21" s="1667" t="n"/>
-      <c r="K21" s="1667" t="n"/>
-      <c r="L21" s="1667" t="n"/>
-      <c r="M21" s="1665" t="n"/>
-      <c r="N21" s="1665" t="n"/>
-      <c r="O21" s="1665" t="n"/>
-      <c r="P21" s="1668" t="n"/>
-      <c r="Q21" s="1665" t="n"/>
-      <c r="R21" s="1665" t="n"/>
-      <c r="S21" s="1665" t="n"/>
+      <c r="D21" s="1707" t="n"/>
+      <c r="E21" s="1707" t="n"/>
+      <c r="F21" s="1707" t="n"/>
+      <c r="G21" s="1707" t="n"/>
+      <c r="H21" s="1707" t="n"/>
+      <c r="I21" s="1708" t="n"/>
+      <c r="J21" s="1709" t="n"/>
+      <c r="K21" s="1709" t="n"/>
+      <c r="L21" s="1709" t="n"/>
+      <c r="M21" s="1707" t="n"/>
+      <c r="N21" s="1707" t="n"/>
+      <c r="O21" s="1707" t="n"/>
+      <c r="P21" s="1710" t="n"/>
+      <c r="Q21" s="1707" t="n"/>
+      <c r="R21" s="1707" t="n"/>
+      <c r="S21" s="1707" t="n"/>
       <c r="T21" s="631" t="n"/>
-      <c r="U21" s="1664" t="n"/>
+      <c r="U21" s="1706" t="n"/>
       <c r="V21" s="632" t="inlineStr">
         <is>
           <t>Pump OFF for night (10:10 PM).</t>
@@ -6916,39 +7024,39 @@
       </c>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="1669" t="inlineStr">
+      <c r="A22" s="1711" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B22" s="1670" t="inlineStr">
+      <c r="B22" s="1712" t="inlineStr">
         <is>
           <t>07:10</t>
         </is>
       </c>
-      <c r="C22" s="1670" t="inlineStr">
+      <c r="C22" s="1712" t="inlineStr">
         <is>
           <t>PUMP</t>
         </is>
       </c>
-      <c r="D22" s="1671" t="n"/>
-      <c r="E22" s="1671" t="n"/>
-      <c r="F22" s="1671" t="n"/>
-      <c r="G22" s="1671" t="n"/>
-      <c r="H22" s="1671" t="n"/>
-      <c r="I22" s="1672" t="n"/>
-      <c r="J22" s="1673" t="n"/>
-      <c r="K22" s="1673" t="n"/>
-      <c r="L22" s="1673" t="n"/>
-      <c r="M22" s="1671" t="n"/>
-      <c r="N22" s="1671" t="n"/>
-      <c r="O22" s="1671" t="n"/>
-      <c r="P22" s="1674" t="n"/>
-      <c r="Q22" s="1671" t="n"/>
-      <c r="R22" s="1671" t="n"/>
-      <c r="S22" s="1671" t="n"/>
+      <c r="D22" s="1713" t="n"/>
+      <c r="E22" s="1713" t="n"/>
+      <c r="F22" s="1713" t="n"/>
+      <c r="G22" s="1713" t="n"/>
+      <c r="H22" s="1713" t="n"/>
+      <c r="I22" s="1714" t="n"/>
+      <c r="J22" s="1715" t="n"/>
+      <c r="K22" s="1715" t="n"/>
+      <c r="L22" s="1715" t="n"/>
+      <c r="M22" s="1713" t="n"/>
+      <c r="N22" s="1713" t="n"/>
+      <c r="O22" s="1713" t="n"/>
+      <c r="P22" s="1716" t="n"/>
+      <c r="Q22" s="1713" t="n"/>
+      <c r="R22" s="1713" t="n"/>
+      <c r="S22" s="1713" t="n"/>
       <c r="T22" s="813" t="n"/>
-      <c r="U22" s="1670" t="n"/>
+      <c r="U22" s="1712" t="n"/>
       <c r="V22" s="814" t="inlineStr">
         <is>
           <t>Pump ON for the day (7:10 AM).</t>
@@ -6956,53 +7064,53 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="1675" t="inlineStr">
+      <c r="A23" s="1717" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B23" s="1676" t="inlineStr">
+      <c r="B23" s="1718" t="inlineStr">
         <is>
           <t>12:01</t>
         </is>
       </c>
-      <c r="C23" s="1676" t="inlineStr">
+      <c r="C23" s="1718" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D23" s="1677" t="n"/>
-      <c r="E23" s="1677" t="n">
+      <c r="D23" s="1719" t="n"/>
+      <c r="E23" s="1719" t="n">
         <v>14</v>
       </c>
-      <c r="F23" s="1677" t="n">
+      <c r="F23" s="1719" t="n">
         <v>0.4</v>
       </c>
-      <c r="G23" s="1677" t="n">
+      <c r="G23" s="1719" t="n">
         <v>1.5</v>
       </c>
-      <c r="H23" s="1677" t="n"/>
-      <c r="I23" s="1678" t="n"/>
-      <c r="J23" s="1679" t="n"/>
-      <c r="K23" s="1679" t="n"/>
-      <c r="L23" s="1679" t="n"/>
-      <c r="M23" s="1677" t="n"/>
-      <c r="N23" s="1677" t="n"/>
-      <c r="O23" s="1677" t="n">
+      <c r="H23" s="1719" t="n"/>
+      <c r="I23" s="1720" t="n"/>
+      <c r="J23" s="1721" t="n"/>
+      <c r="K23" s="1721" t="n"/>
+      <c r="L23" s="1721" t="n"/>
+      <c r="M23" s="1719" t="n"/>
+      <c r="N23" s="1719" t="n"/>
+      <c r="O23" s="1719" t="n">
         <v>0</v>
       </c>
-      <c r="P23" s="1680" t="n">
+      <c r="P23" s="1722" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q23" s="1677" t="n"/>
-      <c r="R23" s="1677" t="n"/>
-      <c r="S23" s="1677" t="n"/>
+      <c r="Q23" s="1719" t="n"/>
+      <c r="R23" s="1719" t="n"/>
+      <c r="S23" s="1719" t="n"/>
       <c r="T23" s="820" t="inlineStr">
         <is>
           <t>Overcast, 70F, 87% RH; today high 72F, 0.09in precip, UV max 1.1</t>
         </is>
       </c>
-      <c r="U23" s="1676" t="n"/>
+      <c r="U23" s="1718" t="n"/>
       <c r="V23" s="821" t="inlineStr">
         <is>
           <t>25 mL x0.2. FC 14.0 (in band 13-16, above floor 11), CC 0.4. CC holding at 0.4 (same as 6/22) - below 0.5 flag but 2nd day, watching.</t>
@@ -7010,47 +7118,47 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="1681" t="inlineStr">
+      <c r="A24" s="1723" t="inlineStr">
         <is>
           <t>2026-06-23</t>
         </is>
       </c>
-      <c r="B24" s="1682" t="inlineStr">
+      <c r="B24" s="1724" t="inlineStr">
         <is>
           <t>~12:30</t>
         </is>
       </c>
-      <c r="C24" s="1682" t="inlineStr">
+      <c r="C24" s="1724" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D24" s="1683" t="n"/>
-      <c r="E24" s="1683" t="n"/>
-      <c r="F24" s="1683" t="n"/>
-      <c r="G24" s="1683" t="n"/>
-      <c r="H24" s="1683" t="n"/>
-      <c r="I24" s="1684" t="n"/>
-      <c r="J24" s="1685" t="n"/>
-      <c r="K24" s="1685" t="n"/>
-      <c r="L24" s="1685" t="n"/>
-      <c r="M24" s="1683" t="n">
+      <c r="D24" s="1725" t="n"/>
+      <c r="E24" s="1725" t="n"/>
+      <c r="F24" s="1725" t="n"/>
+      <c r="G24" s="1725" t="n"/>
+      <c r="H24" s="1725" t="n"/>
+      <c r="I24" s="1726" t="n"/>
+      <c r="J24" s="1727" t="n"/>
+      <c r="K24" s="1727" t="n"/>
+      <c r="L24" s="1727" t="n"/>
+      <c r="M24" s="1725" t="n">
         <v>0.5</v>
       </c>
-      <c r="N24" s="1683" t="n">
+      <c r="N24" s="1725" t="n">
         <v>9.5</v>
       </c>
-      <c r="O24" s="1683" t="n"/>
-      <c r="P24" s="1686" t="n"/>
-      <c r="Q24" s="1683" t="n"/>
-      <c r="R24" s="1683" t="n"/>
-      <c r="S24" s="1683" t="n"/>
+      <c r="O24" s="1725" t="n"/>
+      <c r="P24" s="1728" t="n"/>
+      <c r="Q24" s="1725" t="n"/>
+      <c r="R24" s="1725" t="n"/>
+      <c r="S24" s="1725" t="n"/>
       <c r="T24" s="827" t="inlineStr">
         <is>
           <t>Overcast, 70F, low UV</t>
         </is>
       </c>
-      <c r="U24" s="1682" t="n"/>
+      <c r="U24" s="1724" t="n"/>
       <c r="V24" s="828" t="inlineStr">
         <is>
           <t>0.5 gal ~ +1.75 -&gt; ~15.8 (top of band ~16). Cloudy/low-UV day, est ~1.75 ppm loss -&gt; ~14 next noon, still in band. Higher FC should help clear CC 0.4. Added ~12:30 PM, pump running.</t>
@@ -7058,61 +7166,61 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="1657" t="inlineStr">
+      <c r="A25" s="1699" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B25" s="1658" t="inlineStr">
+      <c r="B25" s="1700" t="inlineStr">
         <is>
           <t>13:30</t>
         </is>
       </c>
-      <c r="C25" s="1658" t="inlineStr">
+      <c r="C25" s="1700" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D25" s="1659" t="n">
+      <c r="D25" s="1701" t="n">
         <v>7.6</v>
       </c>
-      <c r="E25" s="1659" t="n">
+      <c r="E25" s="1701" t="n">
         <v>11.2</v>
       </c>
-      <c r="F25" s="1659" t="n">
+      <c r="F25" s="1701" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="1659" t="n">
+      <c r="G25" s="1701" t="n">
         <v>4.6</v>
       </c>
-      <c r="H25" s="1659" t="n"/>
-      <c r="I25" s="1660" t="n"/>
-      <c r="J25" s="1661" t="n">
+      <c r="H25" s="1701" t="n"/>
+      <c r="I25" s="1702" t="n"/>
+      <c r="J25" s="1703" t="n">
         <v>170</v>
       </c>
-      <c r="K25" s="1661" t="n">
+      <c r="K25" s="1703" t="n">
         <v>150</v>
       </c>
-      <c r="L25" s="1661" t="n">
+      <c r="L25" s="1703" t="n">
         <v>150</v>
       </c>
-      <c r="M25" s="1659" t="n"/>
-      <c r="N25" s="1659" t="n"/>
-      <c r="O25" s="1659" t="n">
+      <c r="M25" s="1701" t="n"/>
+      <c r="N25" s="1701" t="n"/>
+      <c r="O25" s="1701" t="n">
         <v>13.6</v>
       </c>
-      <c r="P25" s="1662" t="n">
+      <c r="P25" s="1704" t="n">
         <v>0</v>
       </c>
-      <c r="Q25" s="1659" t="n"/>
-      <c r="R25" s="1659" t="n"/>
-      <c r="S25" s="1659" t="n"/>
+      <c r="Q25" s="1701" t="n"/>
+      <c r="R25" s="1701" t="n"/>
+      <c r="S25" s="1701" t="n"/>
       <c r="T25" s="624" t="inlineStr">
         <is>
           <t>Clear, 79F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U25" s="1658" t="n"/>
+      <c r="U25" s="1700" t="n"/>
       <c r="V25" s="625" t="inlineStr">
         <is>
           <t>FULL BATTERY on FRESH FAS-DPD reagents (25mL x0.2). FC 11.2 (at floor 11), CC 0.0 (confirms 6/22-23 0.4 was old-reagent noise). CYA ~150 via dilution (was ~160 old) -&gt; new anchor, cya_current=150. TA 170 &amp; pH 7.6 (both up from old ~130/~7.3) - leaving alone per rules, watch pH if &gt;7.8. CH 150 (irrelevant on vinyl). NOTE: fc_loss 4.6 crosses old-&gt;fresh reagent change, partly reagent bias.</t>
@@ -7120,47 +7228,47 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="1663" t="inlineStr">
+      <c r="A26" s="1705" t="inlineStr">
         <is>
           <t>2026-06-24</t>
         </is>
       </c>
-      <c r="B26" s="1664" t="inlineStr">
+      <c r="B26" s="1706" t="inlineStr">
         <is>
           <t>~13:45</t>
         </is>
       </c>
-      <c r="C26" s="1664" t="inlineStr">
+      <c r="C26" s="1706" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D26" s="1665" t="n"/>
-      <c r="E26" s="1665" t="n"/>
-      <c r="F26" s="1665" t="n"/>
-      <c r="G26" s="1665" t="n"/>
-      <c r="H26" s="1665" t="n"/>
-      <c r="I26" s="1666" t="n"/>
-      <c r="J26" s="1667" t="n"/>
-      <c r="K26" s="1667" t="n"/>
-      <c r="L26" s="1667" t="n"/>
-      <c r="M26" s="1665" t="n">
+      <c r="D26" s="1707" t="n"/>
+      <c r="E26" s="1707" t="n"/>
+      <c r="F26" s="1707" t="n"/>
+      <c r="G26" s="1707" t="n"/>
+      <c r="H26" s="1707" t="n"/>
+      <c r="I26" s="1708" t="n"/>
+      <c r="J26" s="1709" t="n"/>
+      <c r="K26" s="1709" t="n"/>
+      <c r="L26" s="1709" t="n"/>
+      <c r="M26" s="1707" t="n">
         <v>1.25</v>
       </c>
-      <c r="N26" s="1665" t="n">
+      <c r="N26" s="1707" t="n">
         <v>10.75</v>
       </c>
-      <c r="O26" s="1665" t="n"/>
-      <c r="P26" s="1668" t="n"/>
-      <c r="Q26" s="1665" t="n"/>
-      <c r="R26" s="1665" t="n"/>
-      <c r="S26" s="1665" t="n"/>
+      <c r="O26" s="1707" t="n"/>
+      <c r="P26" s="1710" t="n"/>
+      <c r="Q26" s="1707" t="n"/>
+      <c r="R26" s="1707" t="n"/>
+      <c r="S26" s="1707" t="n"/>
       <c r="T26" s="631" t="inlineStr">
         <is>
           <t>Clear, 79F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U26" s="1664" t="n"/>
+      <c r="U26" s="1706" t="n"/>
       <c r="V26" s="632" t="inlineStr">
         <is>
           <t>Recommended 1.25 gal (rounded up from 1.0 nominal for high-UV day). ~ +4.4 -&gt; FC ~15.6 (aim ~15). Sunny ~4 ppm loss -&gt; ~11.6 next noon, just above floor 11. First big-sun day after rainy stretch. Confirmed added ~1:45 PM. Pump on (auto 7-22).</t>
@@ -7168,53 +7276,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1669" t="inlineStr">
+      <c r="A27" s="1711" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B27" s="1670" t="inlineStr">
+      <c r="B27" s="1712" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C27" s="1670" t="inlineStr">
+      <c r="C27" s="1712" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D27" s="1671" t="n"/>
-      <c r="E27" s="1671" t="n">
+      <c r="D27" s="1713" t="n"/>
+      <c r="E27" s="1713" t="n">
         <v>14.4</v>
       </c>
-      <c r="F27" s="1671" t="n">
+      <c r="F27" s="1713" t="n">
         <v>0</v>
       </c>
-      <c r="G27" s="1671" t="n">
+      <c r="G27" s="1713" t="n">
         <v>1.2</v>
       </c>
-      <c r="H27" s="1671" t="n"/>
-      <c r="I27" s="1672" t="n"/>
-      <c r="J27" s="1673" t="n"/>
-      <c r="K27" s="1673" t="n"/>
-      <c r="L27" s="1673" t="n"/>
-      <c r="M27" s="1671" t="n"/>
-      <c r="N27" s="1671" t="n"/>
-      <c r="O27" s="1671" t="n">
+      <c r="H27" s="1713" t="n"/>
+      <c r="I27" s="1714" t="n"/>
+      <c r="J27" s="1715" t="n"/>
+      <c r="K27" s="1715" t="n"/>
+      <c r="L27" s="1715" t="n"/>
+      <c r="M27" s="1713" t="n"/>
+      <c r="N27" s="1713" t="n"/>
+      <c r="O27" s="1713" t="n">
         <v>11.6</v>
       </c>
-      <c r="P27" s="1674" t="n">
+      <c r="P27" s="1716" t="n">
         <v>0</v>
       </c>
-      <c r="Q27" s="1671" t="n"/>
-      <c r="R27" s="1671" t="n"/>
-      <c r="S27" s="1671" t="n"/>
+      <c r="Q27" s="1713" t="n"/>
+      <c r="R27" s="1713" t="n"/>
+      <c r="S27" s="1713" t="n"/>
       <c r="T27" s="813" t="inlineStr">
         <is>
           <t>Clear, 75F, 40% RH; today high 80F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U27" s="1670" t="n"/>
+      <c r="U27" s="1712" t="n"/>
       <c r="V27" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.4 (in band 13-15, at aim 15), CC 0.0. Yesterday's ~15.6 -&gt; 14.4 = only ~1.2 ppm loss over ~23h vs ~4 projected. Dose-timing artifact (dosed 1:45PM, missed peak UV) + high-CYA protection. Watching whether sunny=4.0 in dose.py is too high.</t>
@@ -7222,47 +7330,47 @@
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1681" t="inlineStr">
+      <c r="A28" s="1723" t="inlineStr">
         <is>
           <t>2026-06-25</t>
         </is>
       </c>
-      <c r="B28" s="1682" t="inlineStr">
+      <c r="B28" s="1724" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C28" s="1682" t="inlineStr">
+      <c r="C28" s="1724" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D28" s="1683" t="n"/>
-      <c r="E28" s="1683" t="n"/>
-      <c r="F28" s="1683" t="n"/>
-      <c r="G28" s="1683" t="n"/>
-      <c r="H28" s="1683" t="n"/>
-      <c r="I28" s="1684" t="n"/>
-      <c r="J28" s="1685" t="n"/>
-      <c r="K28" s="1685" t="n"/>
-      <c r="L28" s="1685" t="n"/>
-      <c r="M28" s="1683" t="n">
+      <c r="D28" s="1725" t="n"/>
+      <c r="E28" s="1725" t="n"/>
+      <c r="F28" s="1725" t="n"/>
+      <c r="G28" s="1725" t="n"/>
+      <c r="H28" s="1725" t="n"/>
+      <c r="I28" s="1726" t="n"/>
+      <c r="J28" s="1727" t="n"/>
+      <c r="K28" s="1727" t="n"/>
+      <c r="L28" s="1727" t="n"/>
+      <c r="M28" s="1725" t="n">
         <v>0.25</v>
       </c>
-      <c r="N28" s="1683" t="n">
+      <c r="N28" s="1725" t="n">
         <v>11</v>
       </c>
-      <c r="O28" s="1683" t="n"/>
-      <c r="P28" s="1686" t="n"/>
-      <c r="Q28" s="1683" t="n"/>
-      <c r="R28" s="1683" t="n"/>
-      <c r="S28" s="1683" t="n"/>
+      <c r="O28" s="1725" t="n"/>
+      <c r="P28" s="1728" t="n"/>
+      <c r="Q28" s="1725" t="n"/>
+      <c r="R28" s="1725" t="n"/>
+      <c r="S28" s="1725" t="n"/>
       <c r="T28" s="827" t="inlineStr">
         <is>
           <t>Clear, 75F, sunny, UV 7.8</t>
         </is>
       </c>
-      <c r="U28" s="1682" t="n"/>
+      <c r="U28" s="1724" t="n"/>
       <c r="V28" s="828" t="inlineStr">
         <is>
           <t>0.25 gal top-up. First evening dose under new routine. Added 6:30 PM - pool already out of direct sun by then (shaded earlier than ~8:25 sunset). FC 14.4 at aim -&gt; ~15.3, minimal overnight loss. Pump on (auto off 10 PM).</t>
@@ -7270,53 +7378,53 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="1657" t="inlineStr">
+      <c r="A29" s="1699" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B29" s="1658" t="inlineStr">
+      <c r="B29" s="1700" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C29" s="1658" t="inlineStr">
+      <c r="C29" s="1700" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D29" s="1659" t="n"/>
-      <c r="E29" s="1659" t="n">
+      <c r="D29" s="1701" t="n"/>
+      <c r="E29" s="1701" t="n">
         <v>14.2</v>
       </c>
-      <c r="F29" s="1659" t="n">
+      <c r="F29" s="1701" t="n">
         <v>0</v>
       </c>
-      <c r="G29" s="1659" t="n">
+      <c r="G29" s="1701" t="n">
         <v>1.1</v>
       </c>
-      <c r="H29" s="1659" t="n"/>
-      <c r="I29" s="1660" t="n"/>
-      <c r="J29" s="1661" t="n"/>
-      <c r="K29" s="1661" t="n"/>
-      <c r="L29" s="1661" t="n"/>
-      <c r="M29" s="1659" t="n"/>
-      <c r="N29" s="1659" t="n"/>
-      <c r="O29" s="1659" t="n">
+      <c r="H29" s="1701" t="n"/>
+      <c r="I29" s="1702" t="n"/>
+      <c r="J29" s="1703" t="n"/>
+      <c r="K29" s="1703" t="n"/>
+      <c r="L29" s="1703" t="n"/>
+      <c r="M29" s="1701" t="n"/>
+      <c r="N29" s="1701" t="n"/>
+      <c r="O29" s="1701" t="n">
         <v>5.8</v>
       </c>
-      <c r="P29" s="1662" t="n">
+      <c r="P29" s="1704" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q29" s="1659" t="n"/>
-      <c r="R29" s="1659" t="n"/>
-      <c r="S29" s="1659" t="n"/>
+      <c r="Q29" s="1701" t="n"/>
+      <c r="R29" s="1701" t="n"/>
+      <c r="S29" s="1701" t="n"/>
       <c r="T29" s="624" t="inlineStr">
         <is>
           <t>Overcast, 69F, 94% RH; today high 75F, 0.15in precip, UV max 5.8</t>
         </is>
       </c>
-      <c r="U29" s="1658" t="n"/>
+      <c r="U29" s="1700" t="n"/>
       <c r="V29" s="625" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.2 (in band 13-15), CC 0.0. Evening-dose validation: 15.3 (6:30PM dose 6/25) -&gt; 14.2 = ~1.1 ppm loss over ~18h (rain/overcast, evening dose skipped all UV). Some rain overnight.</t>
@@ -7324,43 +7432,43 @@
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="1663" t="inlineStr">
+      <c r="A30" s="1705" t="inlineStr">
         <is>
           <t>2026-06-26</t>
         </is>
       </c>
-      <c r="B30" s="1664" t="inlineStr">
+      <c r="B30" s="1706" t="inlineStr">
         <is>
           <t>12:25</t>
         </is>
       </c>
-      <c r="C30" s="1664" t="inlineStr">
+      <c r="C30" s="1706" t="inlineStr">
         <is>
           <t>NOTE</t>
         </is>
       </c>
-      <c r="D30" s="1665" t="n"/>
-      <c r="E30" s="1665" t="n"/>
-      <c r="F30" s="1665" t="n"/>
-      <c r="G30" s="1665" t="n"/>
-      <c r="H30" s="1665" t="n"/>
-      <c r="I30" s="1666" t="n"/>
-      <c r="J30" s="1667" t="n"/>
-      <c r="K30" s="1667" t="n"/>
-      <c r="L30" s="1667" t="n"/>
-      <c r="M30" s="1665" t="n"/>
-      <c r="N30" s="1665" t="n"/>
-      <c r="O30" s="1665" t="n"/>
-      <c r="P30" s="1668" t="n"/>
-      <c r="Q30" s="1665" t="n"/>
-      <c r="R30" s="1665" t="n"/>
-      <c r="S30" s="1665" t="n"/>
+      <c r="D30" s="1707" t="n"/>
+      <c r="E30" s="1707" t="n"/>
+      <c r="F30" s="1707" t="n"/>
+      <c r="G30" s="1707" t="n"/>
+      <c r="H30" s="1707" t="n"/>
+      <c r="I30" s="1708" t="n"/>
+      <c r="J30" s="1709" t="n"/>
+      <c r="K30" s="1709" t="n"/>
+      <c r="L30" s="1709" t="n"/>
+      <c r="M30" s="1707" t="n"/>
+      <c r="N30" s="1707" t="n"/>
+      <c r="O30" s="1707" t="n"/>
+      <c r="P30" s="1710" t="n"/>
+      <c r="Q30" s="1707" t="n"/>
+      <c r="R30" s="1707" t="n"/>
+      <c r="S30" s="1707" t="n"/>
       <c r="T30" s="631" t="inlineStr">
         <is>
           <t>Overcast/rain, low UV</t>
         </is>
       </c>
-      <c r="U30" s="1664" t="n"/>
+      <c r="U30" s="1706" t="n"/>
       <c r="V30" s="632" t="inlineStr">
         <is>
           <t>NO DOSE today. FC 14.2 well in band on a low-loss rainy day; projected ~13 by next noon, above floor 11. Held chlorine for efficiency (dose.py nominal was 0.25 to top of band).</t>
@@ -7368,53 +7476,53 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="1669" t="inlineStr">
+      <c r="A31" s="1711" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B31" s="1670" t="inlineStr">
+      <c r="B31" s="1712" t="inlineStr">
         <is>
           <t>12:35</t>
         </is>
       </c>
-      <c r="C31" s="1670" t="inlineStr">
+      <c r="C31" s="1712" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D31" s="1671" t="n"/>
-      <c r="E31" s="1671" t="n">
+      <c r="D31" s="1713" t="n"/>
+      <c r="E31" s="1713" t="n">
         <v>10.6</v>
       </c>
-      <c r="F31" s="1671" t="n">
+      <c r="F31" s="1713" t="n">
         <v>0</v>
       </c>
-      <c r="G31" s="1671" t="n">
+      <c r="G31" s="1713" t="n">
         <v>3.6</v>
       </c>
-      <c r="H31" s="1671" t="n"/>
-      <c r="I31" s="1672" t="n"/>
-      <c r="J31" s="1673" t="n"/>
-      <c r="K31" s="1673" t="n"/>
-      <c r="L31" s="1673" t="n"/>
-      <c r="M31" s="1671" t="n"/>
-      <c r="N31" s="1671" t="n"/>
-      <c r="O31" s="1671" t="n">
+      <c r="H31" s="1713" t="n"/>
+      <c r="I31" s="1714" t="n"/>
+      <c r="J31" s="1715" t="n"/>
+      <c r="K31" s="1715" t="n"/>
+      <c r="L31" s="1715" t="n"/>
+      <c r="M31" s="1713" t="n"/>
+      <c r="N31" s="1713" t="n"/>
+      <c r="O31" s="1713" t="n">
         <v>5.2</v>
       </c>
-      <c r="P31" s="1674" t="n">
+      <c r="P31" s="1716" t="n">
         <v>0</v>
       </c>
-      <c r="Q31" s="1671" t="n"/>
-      <c r="R31" s="1671" t="n"/>
-      <c r="S31" s="1671" t="n"/>
+      <c r="Q31" s="1713" t="n"/>
+      <c r="R31" s="1713" t="n"/>
+      <c r="S31" s="1713" t="n"/>
       <c r="T31" s="813" t="inlineStr">
         <is>
           <t>Sunny AM (~5 sunshine hrs), clouded over ~12:25; 77-79F</t>
         </is>
       </c>
-      <c r="U31" s="1670" t="inlineStr">
+      <c r="U31" s="1712" t="inlineStr">
         <is>
           <t>2026-06-27_1-3.jpg</t>
         </is>
@@ -7426,49 +7534,49 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="1681" t="inlineStr">
+      <c r="A32" s="1723" t="inlineStr">
         <is>
           <t>2026-06-27</t>
         </is>
       </c>
-      <c r="B32" s="1682" t="inlineStr">
+      <c r="B32" s="1724" t="inlineStr">
         <is>
           <t>17:35</t>
         </is>
       </c>
-      <c r="C32" s="1682" t="inlineStr">
+      <c r="C32" s="1724" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D32" s="1683" t="n"/>
-      <c r="E32" s="1683" t="n"/>
-      <c r="F32" s="1683" t="n"/>
-      <c r="G32" s="1683" t="n"/>
-      <c r="H32" s="1683" t="n">
+      <c r="D32" s="1725" t="n"/>
+      <c r="E32" s="1725" t="n"/>
+      <c r="F32" s="1725" t="n"/>
+      <c r="G32" s="1725" t="n"/>
+      <c r="H32" s="1725" t="n">
         <v>12.8</v>
       </c>
-      <c r="I32" s="1684" t="n"/>
-      <c r="J32" s="1685" t="n"/>
-      <c r="K32" s="1685" t="n"/>
-      <c r="L32" s="1685" t="n"/>
-      <c r="M32" s="1683" t="n">
+      <c r="I32" s="1726" t="n"/>
+      <c r="J32" s="1727" t="n"/>
+      <c r="K32" s="1727" t="n"/>
+      <c r="L32" s="1727" t="n"/>
+      <c r="M32" s="1725" t="n">
         <v>1.5</v>
       </c>
-      <c r="N32" s="1683" t="n">
+      <c r="N32" s="1725" t="n">
         <v>12.5</v>
       </c>
-      <c r="O32" s="1683" t="n"/>
-      <c r="P32" s="1686" t="n"/>
-      <c r="Q32" s="1683" t="n"/>
-      <c r="R32" s="1683" t="n"/>
-      <c r="S32" s="1683" t="n"/>
+      <c r="O32" s="1725" t="n"/>
+      <c r="P32" s="1728" t="n"/>
+      <c r="Q32" s="1725" t="n"/>
+      <c r="R32" s="1725" t="n"/>
+      <c r="S32" s="1725" t="n"/>
       <c r="T32" s="827" t="inlineStr">
         <is>
           <t>Overcast, 79F</t>
         </is>
       </c>
-      <c r="U32" s="1682" t="n"/>
+      <c r="U32" s="1724" t="n"/>
       <c r="V32" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 5:35 PM (pool shaded, pump running). Rebuild after FC dipped just below floor; 1.5 gal ~ +5.25 -&gt; ~15.8. Season total 12.5 gal.</t>
@@ -7476,57 +7584,57 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="1657" t="inlineStr">
+      <c r="A33" s="1699" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B33" s="1658" t="inlineStr">
+      <c r="B33" s="1700" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C33" s="1658" t="inlineStr">
+      <c r="C33" s="1700" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D33" s="1659" t="n"/>
-      <c r="E33" s="1659" t="n">
+      <c r="D33" s="1701" t="n"/>
+      <c r="E33" s="1701" t="n">
         <v>12.8</v>
       </c>
-      <c r="F33" s="1659" t="n">
+      <c r="F33" s="1701" t="n">
         <v>0.2</v>
       </c>
-      <c r="G33" s="1659" t="n">
+      <c r="G33" s="1701" t="n">
         <v>3</v>
       </c>
-      <c r="H33" s="1659" t="n"/>
-      <c r="I33" s="1660" t="n">
+      <c r="H33" s="1701" t="n"/>
+      <c r="I33" s="1702" t="n">
         <v>0</v>
       </c>
-      <c r="J33" s="1661" t="n"/>
-      <c r="K33" s="1661" t="n"/>
-      <c r="L33" s="1661" t="n"/>
-      <c r="M33" s="1659" t="n"/>
-      <c r="N33" s="1659" t="n"/>
-      <c r="O33" s="1659" t="n">
+      <c r="J33" s="1703" t="n"/>
+      <c r="K33" s="1703" t="n"/>
+      <c r="L33" s="1703" t="n"/>
+      <c r="M33" s="1701" t="n"/>
+      <c r="N33" s="1701" t="n"/>
+      <c r="O33" s="1701" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="P33" s="1662" t="n">
+      <c r="P33" s="1704" t="n">
         <v>0</v>
       </c>
-      <c r="Q33" s="1659" t="n"/>
-      <c r="R33" s="1659" t="n">
+      <c r="Q33" s="1701" t="n"/>
+      <c r="R33" s="1701" t="n">
         <v>79</v>
       </c>
-      <c r="S33" s="1659" t="n"/>
+      <c r="S33" s="1701" t="n"/>
       <c r="T33" s="624" t="inlineStr">
         <is>
           <t>Sunny day (~9 sun hrs), 75-79F, clouded at midday; UV max 7.5</t>
         </is>
       </c>
-      <c r="U33" s="1658" t="inlineStr">
+      <c r="U33" s="1700" t="inlineStr">
         <is>
           <t>2026-06-28_1-4.jpg</t>
         </is>
@@ -7538,49 +7646,49 @@
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="1663" t="inlineStr">
+      <c r="A34" s="1705" t="inlineStr">
         <is>
           <t>2026-06-28</t>
         </is>
       </c>
-      <c r="B34" s="1664" t="inlineStr">
+      <c r="B34" s="1706" t="inlineStr">
         <is>
           <t>~17:55</t>
         </is>
       </c>
-      <c r="C34" s="1664" t="inlineStr">
+      <c r="C34" s="1706" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D34" s="1665" t="n"/>
-      <c r="E34" s="1665" t="n"/>
-      <c r="F34" s="1665" t="n"/>
-      <c r="G34" s="1665" t="n"/>
-      <c r="H34" s="1665" t="n">
+      <c r="D34" s="1707" t="n"/>
+      <c r="E34" s="1707" t="n"/>
+      <c r="F34" s="1707" t="n"/>
+      <c r="G34" s="1707" t="n"/>
+      <c r="H34" s="1707" t="n">
         <v>12.3</v>
       </c>
-      <c r="I34" s="1666" t="n"/>
-      <c r="J34" s="1667" t="n"/>
-      <c r="K34" s="1667" t="n"/>
-      <c r="L34" s="1667" t="n"/>
-      <c r="M34" s="1665" t="n">
+      <c r="I34" s="1708" t="n"/>
+      <c r="J34" s="1709" t="n"/>
+      <c r="K34" s="1709" t="n"/>
+      <c r="L34" s="1709" t="n"/>
+      <c r="M34" s="1707" t="n">
         <v>1</v>
       </c>
-      <c r="N34" s="1665" t="n">
+      <c r="N34" s="1707" t="n">
         <v>13.5</v>
       </c>
-      <c r="O34" s="1665" t="n"/>
-      <c r="P34" s="1668" t="n"/>
-      <c r="Q34" s="1665" t="n"/>
-      <c r="R34" s="1665" t="n"/>
-      <c r="S34" s="1665" t="n"/>
+      <c r="O34" s="1707" t="n"/>
+      <c r="P34" s="1710" t="n"/>
+      <c r="Q34" s="1707" t="n"/>
+      <c r="R34" s="1707" t="n"/>
+      <c r="S34" s="1707" t="n"/>
       <c r="T34" s="631" t="inlineStr">
         <is>
           <t>Sunny, 75-79F, UV 7.5</t>
         </is>
       </c>
-      <c r="U34" s="1664" t="n"/>
+      <c r="U34" s="1706" t="n"/>
       <c r="V34" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added ~5:55 PM (photos timestamped 5:59; pool shaded, pump running). Targets ~15. Season total 13.5 gal.</t>
@@ -7588,57 +7696,57 @@
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="1669" t="inlineStr">
+      <c r="A35" s="1711" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B35" s="1670" t="inlineStr">
+      <c r="B35" s="1712" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C35" s="1670" t="inlineStr">
+      <c r="C35" s="1712" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D35" s="1671" t="n"/>
-      <c r="E35" s="1671" t="n">
+      <c r="D35" s="1713" t="n"/>
+      <c r="E35" s="1713" t="n">
         <v>14</v>
       </c>
-      <c r="F35" s="1671" t="n">
+      <c r="F35" s="1713" t="n">
         <v>0.2</v>
       </c>
-      <c r="G35" s="1671" t="n">
+      <c r="G35" s="1713" t="n">
         <v>2.3</v>
       </c>
-      <c r="H35" s="1671" t="n"/>
-      <c r="I35" s="1672" t="n">
+      <c r="H35" s="1713" t="n"/>
+      <c r="I35" s="1714" t="n">
         <v>1.7</v>
       </c>
-      <c r="J35" s="1673" t="n"/>
-      <c r="K35" s="1673" t="n"/>
-      <c r="L35" s="1673" t="n"/>
-      <c r="M35" s="1671" t="n"/>
-      <c r="N35" s="1671" t="n"/>
-      <c r="O35" s="1671" t="n">
+      <c r="J35" s="1715" t="n"/>
+      <c r="K35" s="1715" t="n"/>
+      <c r="L35" s="1715" t="n"/>
+      <c r="M35" s="1713" t="n"/>
+      <c r="N35" s="1713" t="n"/>
+      <c r="O35" s="1713" t="n">
         <v>12.2</v>
       </c>
-      <c r="P35" s="1674" t="n">
+      <c r="P35" s="1716" t="n">
         <v>0</v>
       </c>
-      <c r="Q35" s="1671" t="n"/>
-      <c r="R35" s="1671" t="n">
+      <c r="Q35" s="1713" t="n"/>
+      <c r="R35" s="1713" t="n">
         <v>80</v>
       </c>
-      <c r="S35" s="1671" t="n"/>
+      <c r="S35" s="1713" t="n"/>
       <c r="T35" s="813" t="inlineStr">
         <is>
           <t>Very sunny + hot (~12 sun hrs), high 82F, UV 7.8; hot all week</t>
         </is>
       </c>
-      <c r="U35" s="1670" t="inlineStr">
+      <c r="U35" s="1712" t="inlineStr">
         <is>
           <t>2026-06-29_1-4.jpg</t>
         </is>
@@ -7650,49 +7758,49 @@
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="1675" t="inlineStr">
+      <c r="A36" s="1717" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B36" s="1676" t="inlineStr">
+      <c r="B36" s="1718" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C36" s="1676" t="inlineStr">
+      <c r="C36" s="1718" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D36" s="1677" t="n"/>
-      <c r="E36" s="1677" t="n"/>
-      <c r="F36" s="1677" t="n"/>
-      <c r="G36" s="1677" t="n"/>
-      <c r="H36" s="1677" t="n">
+      <c r="D36" s="1719" t="n"/>
+      <c r="E36" s="1719" t="n"/>
+      <c r="F36" s="1719" t="n"/>
+      <c r="G36" s="1719" t="n"/>
+      <c r="H36" s="1719" t="n">
         <v>14.2</v>
       </c>
-      <c r="I36" s="1678" t="n"/>
-      <c r="J36" s="1679" t="n"/>
-      <c r="K36" s="1679" t="n"/>
-      <c r="L36" s="1679" t="n"/>
-      <c r="M36" s="1677" t="n">
+      <c r="I36" s="1720" t="n"/>
+      <c r="J36" s="1721" t="n"/>
+      <c r="K36" s="1721" t="n"/>
+      <c r="L36" s="1721" t="n"/>
+      <c r="M36" s="1719" t="n">
         <v>1.5</v>
       </c>
-      <c r="N36" s="1677" t="n">
+      <c r="N36" s="1719" t="n">
         <v>15</v>
       </c>
-      <c r="O36" s="1677" t="n"/>
-      <c r="P36" s="1680" t="n"/>
-      <c r="Q36" s="1677" t="n"/>
-      <c r="R36" s="1677" t="n"/>
-      <c r="S36" s="1677" t="n"/>
+      <c r="O36" s="1719" t="n"/>
+      <c r="P36" s="1722" t="n"/>
+      <c r="Q36" s="1719" t="n"/>
+      <c r="R36" s="1719" t="n"/>
+      <c r="S36" s="1719" t="n"/>
       <c r="T36" s="820" t="inlineStr">
         <is>
           <t>Very sunny, high 82F, UV 7.8</t>
         </is>
       </c>
-      <c r="U36" s="1676" t="n"/>
+      <c r="U36" s="1718" t="n"/>
       <c r="V36" s="821" t="inlineStr">
         <is>
           <t>1.5 gal added 6:30 PM (leftover 0.5 + full 1.0 - easier than measuring 0.25). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot very-sunny day. Projects ~14 next noon. Season total 15.0 gal.</t>
@@ -7700,41 +7808,41 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="1681" t="inlineStr">
+      <c r="A37" s="1723" t="inlineStr">
         <is>
           <t>2026-06-29</t>
         </is>
       </c>
-      <c r="B37" s="1682" t="inlineStr">
+      <c r="B37" s="1724" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C37" s="1682" t="inlineStr">
+      <c r="C37" s="1724" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D37" s="1683" t="n"/>
-      <c r="E37" s="1683" t="n"/>
-      <c r="F37" s="1683" t="n"/>
-      <c r="G37" s="1683" t="n"/>
-      <c r="H37" s="1683" t="n"/>
-      <c r="I37" s="1684" t="n"/>
-      <c r="J37" s="1685" t="n"/>
-      <c r="K37" s="1685" t="n"/>
-      <c r="L37" s="1685" t="n"/>
-      <c r="M37" s="1683" t="n"/>
-      <c r="N37" s="1683" t="n"/>
-      <c r="O37" s="1683" t="n"/>
-      <c r="P37" s="1686" t="n"/>
-      <c r="Q37" s="1683" t="n">
+      <c r="D37" s="1725" t="n"/>
+      <c r="E37" s="1725" t="n"/>
+      <c r="F37" s="1725" t="n"/>
+      <c r="G37" s="1725" t="n"/>
+      <c r="H37" s="1725" t="n"/>
+      <c r="I37" s="1726" t="n"/>
+      <c r="J37" s="1727" t="n"/>
+      <c r="K37" s="1727" t="n"/>
+      <c r="L37" s="1727" t="n"/>
+      <c r="M37" s="1725" t="n"/>
+      <c r="N37" s="1725" t="n"/>
+      <c r="O37" s="1725" t="n"/>
+      <c r="P37" s="1728" t="n"/>
+      <c r="Q37" s="1725" t="n">
         <v>93</v>
       </c>
-      <c r="R37" s="1683" t="n"/>
-      <c r="S37" s="1683" t="n"/>
+      <c r="R37" s="1725" t="n"/>
+      <c r="S37" s="1725" t="n"/>
       <c r="T37" s="827" t="n"/>
-      <c r="U37" s="1682" t="n"/>
+      <c r="U37" s="1724" t="n"/>
       <c r="V37" s="828" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 30 min @ ~3.1 GPM = ~93 gal into 34,400. CYA dilution ~0.3% (~0.4 ppm) - negligible/day, nudges passive CYA lowering. Brings well metals (Fe/Mn) -&gt; sequestrant pending (John checking for metal-out). Week well-water cumulative: ~93 gal.</t>
@@ -7742,57 +7850,57 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="1657" t="inlineStr">
+      <c r="A38" s="1699" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B38" s="1658" t="inlineStr">
+      <c r="B38" s="1700" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C38" s="1658" t="inlineStr">
+      <c r="C38" s="1700" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D38" s="1659" t="n"/>
-      <c r="E38" s="1659" t="n">
+      <c r="D38" s="1701" t="n"/>
+      <c r="E38" s="1701" t="n">
         <v>14.6</v>
       </c>
-      <c r="F38" s="1659" t="n">
+      <c r="F38" s="1701" t="n">
         <v>0</v>
       </c>
-      <c r="G38" s="1659" t="n">
+      <c r="G38" s="1701" t="n">
         <v>4.7</v>
       </c>
-      <c r="H38" s="1659" t="n"/>
-      <c r="I38" s="1660" t="n">
+      <c r="H38" s="1701" t="n"/>
+      <c r="I38" s="1702" t="n">
         <v>0.4</v>
       </c>
-      <c r="J38" s="1661" t="n"/>
-      <c r="K38" s="1661" t="n"/>
-      <c r="L38" s="1661" t="n"/>
-      <c r="M38" s="1659" t="n"/>
-      <c r="N38" s="1659" t="n"/>
-      <c r="O38" s="1659" t="n">
+      <c r="J38" s="1703" t="n"/>
+      <c r="K38" s="1703" t="n"/>
+      <c r="L38" s="1703" t="n"/>
+      <c r="M38" s="1701" t="n"/>
+      <c r="N38" s="1701" t="n"/>
+      <c r="O38" s="1701" t="n">
         <v>10.2</v>
       </c>
-      <c r="P38" s="1662" t="n">
+      <c r="P38" s="1704" t="n">
         <v>0</v>
       </c>
-      <c r="Q38" s="1659" t="n"/>
-      <c r="R38" s="1659" t="n">
+      <c r="Q38" s="1701" t="n"/>
+      <c r="R38" s="1701" t="n">
         <v>80.5</v>
       </c>
-      <c r="S38" s="1659" t="n"/>
+      <c r="S38" s="1701" t="n"/>
       <c r="T38" s="624" t="inlineStr">
         <is>
           <t>Super sunny + hot, high 84F (~10 sun hrs), UV 7.9</t>
         </is>
       </c>
-      <c r="U38" s="1658" t="inlineStr">
+      <c r="U38" s="1700" t="inlineStr">
         <is>
           <t>2026-06-30_1-4.jpg</t>
         </is>
@@ -7804,49 +7912,49 @@
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="1687" t="inlineStr">
+      <c r="A39" s="1729" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B39" s="1688" t="inlineStr">
+      <c r="B39" s="1730" t="inlineStr">
         <is>
           <t>18:50</t>
         </is>
       </c>
-      <c r="C39" s="1688" t="inlineStr">
+      <c r="C39" s="1730" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D39" s="1689" t="n"/>
-      <c r="E39" s="1689" t="n"/>
-      <c r="F39" s="1689" t="n"/>
-      <c r="G39" s="1689" t="n"/>
-      <c r="H39" s="1689" t="n">
+      <c r="D39" s="1731" t="n"/>
+      <c r="E39" s="1731" t="n"/>
+      <c r="F39" s="1731" t="n"/>
+      <c r="G39" s="1731" t="n"/>
+      <c r="H39" s="1731" t="n">
         <v>14.8</v>
       </c>
-      <c r="I39" s="1690" t="n"/>
-      <c r="J39" s="1691" t="n"/>
-      <c r="K39" s="1691" t="n"/>
-      <c r="L39" s="1691" t="n"/>
-      <c r="M39" s="1689" t="n">
+      <c r="I39" s="1732" t="n"/>
+      <c r="J39" s="1733" t="n"/>
+      <c r="K39" s="1733" t="n"/>
+      <c r="L39" s="1733" t="n"/>
+      <c r="M39" s="1731" t="n">
         <v>1.5</v>
       </c>
-      <c r="N39" s="1689" t="n">
+      <c r="N39" s="1731" t="n">
         <v>16.5</v>
       </c>
-      <c r="O39" s="1689" t="n"/>
-      <c r="P39" s="1692" t="n"/>
-      <c r="Q39" s="1689" t="n"/>
-      <c r="R39" s="1689" t="n"/>
-      <c r="S39" s="1689" t="n"/>
+      <c r="O39" s="1731" t="n"/>
+      <c r="P39" s="1734" t="n"/>
+      <c r="Q39" s="1731" t="n"/>
+      <c r="R39" s="1731" t="n"/>
+      <c r="S39" s="1731" t="n"/>
       <c r="T39" s="659" t="inlineStr">
         <is>
           <t>Super sunny, high 84F, UV 7.9</t>
         </is>
       </c>
-      <c r="U39" s="1688" t="n"/>
+      <c r="U39" s="1730" t="n"/>
       <c r="V39" s="660" t="inlineStr">
         <is>
           <t>1.5 gal added 6:50 PM (pump running). ~ +5.25 -&gt; ~16.5-17 evening; buffer for hot sunny stretch. Projects ~12-13 next noon. Season total 16.5 gal.</t>
@@ -7854,41 +7962,41 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="1663" t="inlineStr">
+      <c r="A40" s="1705" t="inlineStr">
         <is>
           <t>2026-06-30</t>
         </is>
       </c>
-      <c r="B40" s="1664" t="inlineStr">
+      <c r="B40" s="1706" t="inlineStr">
         <is>
           <t>evening</t>
         </is>
       </c>
-      <c r="C40" s="1664" t="inlineStr">
+      <c r="C40" s="1706" t="inlineStr">
         <is>
           <t>EVENT - Fill</t>
         </is>
       </c>
-      <c r="D40" s="1665" t="n"/>
-      <c r="E40" s="1665" t="n"/>
-      <c r="F40" s="1665" t="n"/>
-      <c r="G40" s="1665" t="n"/>
-      <c r="H40" s="1665" t="n"/>
-      <c r="I40" s="1666" t="n"/>
-      <c r="J40" s="1667" t="n"/>
-      <c r="K40" s="1667" t="n"/>
-      <c r="L40" s="1667" t="n"/>
-      <c r="M40" s="1665" t="n"/>
-      <c r="N40" s="1665" t="n"/>
-      <c r="O40" s="1665" t="n"/>
-      <c r="P40" s="1668" t="n"/>
-      <c r="Q40" s="1665" t="n">
+      <c r="D40" s="1707" t="n"/>
+      <c r="E40" s="1707" t="n"/>
+      <c r="F40" s="1707" t="n"/>
+      <c r="G40" s="1707" t="n"/>
+      <c r="H40" s="1707" t="n"/>
+      <c r="I40" s="1708" t="n"/>
+      <c r="J40" s="1709" t="n"/>
+      <c r="K40" s="1709" t="n"/>
+      <c r="L40" s="1709" t="n"/>
+      <c r="M40" s="1707" t="n"/>
+      <c r="N40" s="1707" t="n"/>
+      <c r="O40" s="1707" t="n"/>
+      <c r="P40" s="1710" t="n"/>
+      <c r="Q40" s="1707" t="n">
         <v>158</v>
       </c>
-      <c r="R40" s="1665" t="n"/>
-      <c r="S40" s="1665" t="n"/>
+      <c r="R40" s="1707" t="n"/>
+      <c r="S40" s="1707" t="n"/>
       <c r="T40" s="631" t="n"/>
-      <c r="U40" s="1664" t="n"/>
+      <c r="U40" s="1706" t="n"/>
       <c r="V40" s="632" t="inlineStr">
         <is>
           <t>Well-water top-off: hose 51 min @ ~3.1 GPM = ~158 gal into 34,400 (level +~0.32 in / 5/16). CYA dilution ~0.5% (~0.7 ppm). Brings well metals -&gt; sequestrant (Pool Mate Metal Out) to be dosed later. WEEK well-water cumulative: ~251 gal (6/29 93 + 6/30 158).</t>
@@ -7896,57 +8004,57 @@
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="1669" t="inlineStr">
+      <c r="A41" s="1711" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B41" s="1670" t="inlineStr">
+      <c r="B41" s="1712" t="inlineStr">
         <is>
           <t>12:10</t>
         </is>
       </c>
-      <c r="C41" s="1670" t="inlineStr">
+      <c r="C41" s="1712" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D41" s="1671" t="n"/>
-      <c r="E41" s="1671" t="n">
+      <c r="D41" s="1713" t="n"/>
+      <c r="E41" s="1713" t="n">
         <v>14.8</v>
       </c>
-      <c r="F41" s="1671" t="n">
+      <c r="F41" s="1713" t="n">
         <v>0.2</v>
       </c>
-      <c r="G41" s="1671" t="n">
+      <c r="G41" s="1713" t="n">
         <v>5.1</v>
       </c>
-      <c r="H41" s="1671" t="n"/>
-      <c r="I41" s="1672" t="n">
+      <c r="H41" s="1713" t="n"/>
+      <c r="I41" s="1714" t="n">
         <v>0</v>
       </c>
-      <c r="J41" s="1673" t="n"/>
-      <c r="K41" s="1673" t="n"/>
-      <c r="L41" s="1673" t="n"/>
-      <c r="M41" s="1671" t="n"/>
-      <c r="N41" s="1671" t="n"/>
-      <c r="O41" s="1671" t="n">
+      <c r="J41" s="1715" t="n"/>
+      <c r="K41" s="1715" t="n"/>
+      <c r="L41" s="1715" t="n"/>
+      <c r="M41" s="1713" t="n"/>
+      <c r="N41" s="1713" t="n"/>
+      <c r="O41" s="1713" t="n">
         <v>12</v>
       </c>
-      <c r="P41" s="1674" t="n">
+      <c r="P41" s="1716" t="n">
         <v>0.47</v>
       </c>
-      <c r="Q41" s="1671" t="n"/>
-      <c r="R41" s="1671" t="n">
+      <c r="Q41" s="1713" t="n"/>
+      <c r="R41" s="1713" t="n">
         <v>81</v>
       </c>
-      <c r="S41" s="1671" t="n"/>
+      <c r="S41" s="1713" t="n"/>
       <c r="T41" s="813" t="inlineStr">
         <is>
           <t>Clear, 81F, 77% RH; today high 86F, 0.47in precip (early/later, not midday), UV max 7.9</t>
         </is>
       </c>
-      <c r="U41" s="1670" t="inlineStr">
+      <c r="U41" s="1712" t="inlineStr">
         <is>
           <t>2026-07-01_1-3.jpg</t>
         </is>
@@ -7958,49 +8066,49 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="1681" t="inlineStr">
+      <c r="A42" s="1723" t="inlineStr">
         <is>
           <t>2026-07-01</t>
         </is>
       </c>
-      <c r="B42" s="1682" t="inlineStr">
+      <c r="B42" s="1724" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C42" s="1682" t="inlineStr">
+      <c r="C42" s="1724" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D42" s="1683" t="n"/>
-      <c r="E42" s="1683" t="n"/>
-      <c r="F42" s="1683" t="n"/>
-      <c r="G42" s="1683" t="n"/>
-      <c r="H42" s="1683" t="n">
+      <c r="D42" s="1725" t="n"/>
+      <c r="E42" s="1725" t="n"/>
+      <c r="F42" s="1725" t="n"/>
+      <c r="G42" s="1725" t="n"/>
+      <c r="H42" s="1725" t="n">
         <v>15.1</v>
       </c>
-      <c r="I42" s="1684" t="n"/>
-      <c r="J42" s="1685" t="n"/>
-      <c r="K42" s="1685" t="n"/>
-      <c r="L42" s="1685" t="n"/>
-      <c r="M42" s="1683" t="n">
+      <c r="I42" s="1726" t="n"/>
+      <c r="J42" s="1727" t="n"/>
+      <c r="K42" s="1727" t="n"/>
+      <c r="L42" s="1727" t="n"/>
+      <c r="M42" s="1725" t="n">
         <v>1.5</v>
       </c>
-      <c r="N42" s="1683" t="n">
+      <c r="N42" s="1725" t="n">
         <v>18</v>
       </c>
-      <c r="O42" s="1683" t="n"/>
-      <c r="P42" s="1686" t="n"/>
-      <c r="Q42" s="1683" t="n"/>
-      <c r="R42" s="1683" t="n"/>
-      <c r="S42" s="1683" t="n"/>
+      <c r="O42" s="1725" t="n"/>
+      <c r="P42" s="1728" t="n"/>
+      <c r="Q42" s="1725" t="n"/>
+      <c r="R42" s="1725" t="n"/>
+      <c r="S42" s="1725" t="n"/>
       <c r="T42" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 86F, UV 7.9</t>
         </is>
       </c>
-      <c r="U42" s="1682" t="n"/>
+      <c r="U42" s="1724" t="n"/>
       <c r="V42" s="828" t="inlineStr">
         <is>
           <t>1.5 gal added 7:30 PM (pump running; within the 6:30-9:15 window). Calibrated evening-model rec (L24=5.0, hot &amp; sunny: sun 12h, water 81F); ~ +5.25. Held buffer on the hottest/sunniest day yet per no-skip lesson (daytime calc alone said 0). Season total 18.0 gal.</t>
@@ -8008,57 +8116,57 @@
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="1657" t="inlineStr">
+      <c r="A43" s="1699" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B43" s="1658" t="inlineStr">
+      <c r="B43" s="1700" t="inlineStr">
         <is>
           <t>12:30</t>
         </is>
       </c>
-      <c r="C43" s="1658" t="inlineStr">
+      <c r="C43" s="1700" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D43" s="1659" t="n"/>
-      <c r="E43" s="1659" t="n">
+      <c r="D43" s="1701" t="n"/>
+      <c r="E43" s="1701" t="n">
         <v>17.2</v>
       </c>
-      <c r="F43" s="1659" t="n">
+      <c r="F43" s="1701" t="n">
         <v>0</v>
       </c>
-      <c r="G43" s="1659" t="n">
+      <c r="G43" s="1701" t="n">
         <v>2.9</v>
       </c>
-      <c r="H43" s="1659" t="n"/>
-      <c r="I43" s="1660" t="n">
+      <c r="H43" s="1701" t="n"/>
+      <c r="I43" s="1702" t="n">
         <v>2.1</v>
       </c>
-      <c r="J43" s="1661" t="n"/>
-      <c r="K43" s="1661" t="n"/>
-      <c r="L43" s="1661" t="n"/>
-      <c r="M43" s="1659" t="n"/>
-      <c r="N43" s="1659" t="n"/>
-      <c r="O43" s="1659" t="n">
+      <c r="J43" s="1703" t="n"/>
+      <c r="K43" s="1703" t="n"/>
+      <c r="L43" s="1703" t="n"/>
+      <c r="M43" s="1701" t="n"/>
+      <c r="N43" s="1701" t="n"/>
+      <c r="O43" s="1701" t="n">
         <v>13.2</v>
       </c>
-      <c r="P43" s="1662" t="n">
+      <c r="P43" s="1704" t="n">
         <v>0</v>
       </c>
-      <c r="Q43" s="1659" t="n"/>
-      <c r="R43" s="1659" t="n">
+      <c r="Q43" s="1701" t="n"/>
+      <c r="R43" s="1701" t="n">
         <v>83</v>
       </c>
-      <c r="S43" s="1659" t="n"/>
+      <c r="S43" s="1701" t="n"/>
       <c r="T43" s="624" t="inlineStr">
         <is>
           <t>Clear now, 85F, 83% RH; sun so far 5.4h of 7h daylight (76%); today high 92F, 0.00in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U43" s="1658" t="n"/>
+      <c r="U43" s="1700" t="n"/>
       <c r="V43" s="625" t="inlineStr">
         <is>
           <t>Pred error unusually large (+2.1) vs last night's 15.1 projection, despite a hot/sunny day where loss should run faster, not slower. John also flagged uncertainty about R-0870 powder dosing (dipper is small, gets crusty) -- but powder amount isn't part of the FAS-DPD titration math, so that's an unlikely source. Worth watching next test to see if this was a one-off read or a real trend.</t>
@@ -8066,45 +8174,45 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="1687" t="inlineStr">
+      <c r="A44" s="1729" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B44" s="1688" t="inlineStr">
+      <c r="B44" s="1730" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C44" s="1688" t="inlineStr">
+      <c r="C44" s="1730" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D44" s="1689" t="n"/>
-      <c r="E44" s="1689" t="n">
+      <c r="D44" s="1731" t="n"/>
+      <c r="E44" s="1731" t="n">
         <v>15.4</v>
       </c>
-      <c r="F44" s="1689" t="n">
+      <c r="F44" s="1731" t="n">
         <v>0.4</v>
       </c>
-      <c r="G44" s="1689" t="n"/>
-      <c r="H44" s="1689" t="n"/>
-      <c r="I44" s="1690" t="n"/>
-      <c r="J44" s="1691" t="n"/>
-      <c r="K44" s="1691" t="n"/>
-      <c r="L44" s="1691" t="n"/>
-      <c r="M44" s="1689" t="n"/>
-      <c r="N44" s="1689" t="n"/>
-      <c r="O44" s="1689" t="n"/>
-      <c r="P44" s="1692" t="n"/>
-      <c r="Q44" s="1689" t="n"/>
-      <c r="R44" s="1689" t="n"/>
-      <c r="S44" s="1689" t="n">
+      <c r="G44" s="1731" t="n"/>
+      <c r="H44" s="1731" t="n"/>
+      <c r="I44" s="1732" t="n"/>
+      <c r="J44" s="1733" t="n"/>
+      <c r="K44" s="1733" t="n"/>
+      <c r="L44" s="1733" t="n"/>
+      <c r="M44" s="1731" t="n"/>
+      <c r="N44" s="1731" t="n"/>
+      <c r="O44" s="1731" t="n"/>
+      <c r="P44" s="1734" t="n"/>
+      <c r="Q44" s="1731" t="n"/>
+      <c r="R44" s="1731" t="n"/>
+      <c r="S44" s="1731" t="n">
         <v>11.9</v>
       </c>
       <c r="T44" s="659" t="n"/>
-      <c r="U44" s="1688" t="inlineStr">
+      <c r="U44" s="1730" t="inlineStr">
         <is>
           <t>2026-07-02_1.jpeg;2026-07-02_2.jpeg;2026-07-02_3.jpeg;2026-07-02_4.jpeg</t>
         </is>
@@ -8116,49 +8224,49 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="1687" t="inlineStr">
+      <c r="A45" s="1729" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B45" s="1688" t="inlineStr">
+      <c r="B45" s="1730" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C45" s="1688" t="inlineStr">
+      <c r="C45" s="1730" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D45" s="1689" t="n"/>
-      <c r="E45" s="1689" t="n"/>
-      <c r="F45" s="1689" t="n"/>
-      <c r="G45" s="1689" t="n"/>
-      <c r="H45" s="1689" t="n">
+      <c r="D45" s="1731" t="n"/>
+      <c r="E45" s="1731" t="n"/>
+      <c r="F45" s="1731" t="n"/>
+      <c r="G45" s="1731" t="n"/>
+      <c r="H45" s="1731" t="n">
         <v>15.7</v>
       </c>
-      <c r="I45" s="1690" t="n"/>
-      <c r="J45" s="1691" t="n"/>
-      <c r="K45" s="1691" t="n"/>
-      <c r="L45" s="1691" t="n"/>
-      <c r="M45" s="1689" t="n">
+      <c r="I45" s="1732" t="n"/>
+      <c r="J45" s="1733" t="n"/>
+      <c r="K45" s="1733" t="n"/>
+      <c r="L45" s="1733" t="n"/>
+      <c r="M45" s="1731" t="n">
         <v>1</v>
       </c>
-      <c r="N45" s="1689" t="n">
+      <c r="N45" s="1731" t="n">
         <v>19</v>
       </c>
-      <c r="O45" s="1689" t="n"/>
-      <c r="P45" s="1692" t="n"/>
-      <c r="Q45" s="1689" t="n"/>
-      <c r="R45" s="1689" t="n"/>
-      <c r="S45" s="1689" t="n"/>
+      <c r="O45" s="1731" t="n"/>
+      <c r="P45" s="1734" t="n"/>
+      <c r="Q45" s="1731" t="n"/>
+      <c r="R45" s="1731" t="n"/>
+      <c r="S45" s="1731" t="n"/>
       <c r="T45" s="659" t="inlineStr">
         <is>
           <t>Hot/sunny, high 92F, water 83F, UV 7.9</t>
         </is>
       </c>
-      <c r="U45" s="1688" t="n"/>
+      <c r="U45" s="1730" t="n"/>
       <c r="V45" s="660" t="inlineStr">
         <is>
           <t>1.0 gal added 8:30 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's NOON FC 17.2 (the model's intended anchor), L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 83F). Raw 0.80 -&gt; rounded 1.0 gal. Evening recheck (15.4 at 7:45 PM) confirmed the noon 17.2 was a real reading, not a fluke -- NOT used as the dose anchor (would double-count the ~1.8 ppm afternoon loss already reflected in it). Season total 19.0 gal. NOTE: this morning's forward prediction missed high (pred 15.1, actual 17.2, +2.1) -&gt; model may be over-estimating loss on hot/sunny days; if tomorrow also lands above the 15.7 projection, consider trimming CONFIG['evening_l24']['l24_hot_sunny'].</t>
@@ -8166,39 +8274,39 @@
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="1663" t="inlineStr">
+      <c r="A46" s="1705" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B46" s="1664" t="inlineStr">
+      <c r="B46" s="1706" t="inlineStr">
         <is>
           <t>night</t>
         </is>
       </c>
-      <c r="C46" s="1664" t="inlineStr">
+      <c r="C46" s="1706" t="inlineStr">
         <is>
           <t>EVENT - Clean</t>
         </is>
       </c>
-      <c r="D46" s="1665" t="n"/>
-      <c r="E46" s="1665" t="n"/>
-      <c r="F46" s="1665" t="n"/>
-      <c r="G46" s="1665" t="n"/>
-      <c r="H46" s="1665" t="n"/>
-      <c r="I46" s="1666" t="n"/>
-      <c r="J46" s="1667" t="n"/>
-      <c r="K46" s="1667" t="n"/>
-      <c r="L46" s="1667" t="n"/>
-      <c r="M46" s="1665" t="n"/>
-      <c r="N46" s="1665" t="n"/>
-      <c r="O46" s="1665" t="n"/>
-      <c r="P46" s="1668" t="n"/>
-      <c r="Q46" s="1665" t="n"/>
-      <c r="R46" s="1665" t="n"/>
-      <c r="S46" s="1665" t="n"/>
+      <c r="D46" s="1707" t="n"/>
+      <c r="E46" s="1707" t="n"/>
+      <c r="F46" s="1707" t="n"/>
+      <c r="G46" s="1707" t="n"/>
+      <c r="H46" s="1707" t="n"/>
+      <c r="I46" s="1708" t="n"/>
+      <c r="J46" s="1709" t="n"/>
+      <c r="K46" s="1709" t="n"/>
+      <c r="L46" s="1709" t="n"/>
+      <c r="M46" s="1707" t="n"/>
+      <c r="N46" s="1707" t="n"/>
+      <c r="O46" s="1707" t="n"/>
+      <c r="P46" s="1710" t="n"/>
+      <c r="Q46" s="1707" t="n"/>
+      <c r="R46" s="1707" t="n"/>
+      <c r="S46" s="1707" t="n"/>
       <c r="T46" s="631" t="n"/>
-      <c r="U46" s="1664" t="n"/>
+      <c r="U46" s="1706" t="n"/>
       <c r="V46" s="632" t="inlineStr">
         <is>
           <t>Magic Eraser (melamine foam) cleaning of the vinyl liner ALL THE WAY AROUND, above the waterline. Reported 2026-07-03 as a likely contributor to the CC creep (0.0 -&gt; 0.4 -&gt; 0.6). Chemistry: melamine is very nitrogen-rich (a triazine triamine, ~66% N), so shed foam micro-particles PLUS the scrubbed-off waterline scum/oils are both nitrogen/organic load that free chlorine converts to chloramines (= combined chlorine). One-time event -&gt; expect CC to fall over the next day or two as FC oxidizes it and the filter clears the bits. Watch: if CC keeps RISING past ~1.0 despite high FC and no more cleaning, look further (this + the floating surface debris are the two benign explanations).</t>
@@ -8206,51 +8314,51 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="1669" t="inlineStr">
+      <c r="A47" s="1711" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B47" s="1670" t="inlineStr">
+      <c r="B47" s="1712" t="inlineStr">
         <is>
           <t>12:15</t>
         </is>
       </c>
-      <c r="C47" s="1670" t="inlineStr">
+      <c r="C47" s="1712" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D47" s="1671" t="n"/>
-      <c r="E47" s="1671" t="n">
+      <c r="D47" s="1713" t="n"/>
+      <c r="E47" s="1713" t="n">
         <v>16.6</v>
       </c>
-      <c r="F47" s="1671" t="n">
+      <c r="F47" s="1713" t="n">
         <v>0.6</v>
       </c>
-      <c r="G47" s="1671" t="n">
+      <c r="G47" s="1713" t="n">
         <v>4.1</v>
       </c>
-      <c r="H47" s="1671" t="n"/>
-      <c r="I47" s="1672" t="n">
+      <c r="H47" s="1713" t="n"/>
+      <c r="I47" s="1714" t="n">
         <v>0.9</v>
       </c>
-      <c r="J47" s="1673" t="n"/>
-      <c r="K47" s="1673" t="n"/>
-      <c r="L47" s="1673" t="n"/>
-      <c r="M47" s="1671" t="n"/>
-      <c r="N47" s="1671" t="n"/>
-      <c r="O47" s="1671" t="n">
+      <c r="J47" s="1715" t="n"/>
+      <c r="K47" s="1715" t="n"/>
+      <c r="L47" s="1715" t="n"/>
+      <c r="M47" s="1713" t="n"/>
+      <c r="N47" s="1713" t="n"/>
+      <c r="O47" s="1713" t="n">
         <v>13.2</v>
       </c>
-      <c r="P47" s="1674" t="n">
+      <c r="P47" s="1716" t="n">
         <v>0</v>
       </c>
-      <c r="Q47" s="1671" t="n"/>
-      <c r="R47" s="1671" t="n">
+      <c r="Q47" s="1713" t="n"/>
+      <c r="R47" s="1713" t="n">
         <v>84.5</v>
       </c>
-      <c r="S47" s="1671" t="n">
+      <c r="S47" s="1713" t="n">
         <v>11.8</v>
       </c>
       <c r="T47" s="813" t="inlineStr">
@@ -8258,7 +8366,7 @@
           <t>Clear now, 89F, 64% RH; sun so far 6.4h of 7h daylight (92%); today high 94F, 0.00in precip, UV max 7.8</t>
         </is>
       </c>
-      <c r="U47" s="1670" t="inlineStr">
+      <c r="U47" s="1712" t="inlineStr">
         <is>
           <t>2026-07-03_1.jpeg;2026-07-03_2.jpeg;2026-07-03_3.jpeg;2026-07-03_4.jpeg;2026-07-03_5.jpeg</t>
         </is>
@@ -8270,49 +8378,49 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="1681" t="inlineStr">
+      <c r="A48" s="1723" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B48" s="1682" t="inlineStr">
+      <c r="B48" s="1724" t="inlineStr">
         <is>
           <t>19:45</t>
         </is>
       </c>
-      <c r="C48" s="1682" t="inlineStr">
+      <c r="C48" s="1724" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D48" s="1683" t="n"/>
-      <c r="E48" s="1683" t="n"/>
-      <c r="F48" s="1683" t="n"/>
-      <c r="G48" s="1683" t="n"/>
-      <c r="H48" s="1683" t="n">
+      <c r="D48" s="1725" t="n"/>
+      <c r="E48" s="1725" t="n"/>
+      <c r="F48" s="1725" t="n"/>
+      <c r="G48" s="1725" t="n"/>
+      <c r="H48" s="1725" t="n">
         <v>15.1</v>
       </c>
-      <c r="I48" s="1684" t="n"/>
-      <c r="J48" s="1685" t="n"/>
-      <c r="K48" s="1685" t="n"/>
-      <c r="L48" s="1685" t="n"/>
-      <c r="M48" s="1683" t="n">
+      <c r="I48" s="1726" t="n"/>
+      <c r="J48" s="1727" t="n"/>
+      <c r="K48" s="1727" t="n"/>
+      <c r="L48" s="1727" t="n"/>
+      <c r="M48" s="1725" t="n">
         <v>1</v>
       </c>
-      <c r="N48" s="1683" t="n">
+      <c r="N48" s="1725" t="n">
         <v>20</v>
       </c>
-      <c r="O48" s="1683" t="n"/>
-      <c r="P48" s="1686" t="n"/>
-      <c r="Q48" s="1683" t="n"/>
-      <c r="R48" s="1683" t="n"/>
-      <c r="S48" s="1683" t="n"/>
+      <c r="O48" s="1725" t="n"/>
+      <c r="P48" s="1728" t="n"/>
+      <c r="Q48" s="1725" t="n"/>
+      <c r="R48" s="1725" t="n"/>
+      <c r="S48" s="1725" t="n"/>
       <c r="T48" s="827" t="inlineStr">
         <is>
           <t>Hot/sunny, high 94F, water 84.5F, UV 7.8</t>
         </is>
       </c>
-      <c r="U48" s="1682" t="n"/>
+      <c r="U48" s="1724" t="n"/>
       <c r="V48" s="828" t="inlineStr">
         <is>
           <t>1.0 gal added 7:45 PM (pump running; within the 6:30-9:15 window, before 10 PM off). Calibrated evening model off today's noon FC 16.6, L24=5.0 (hot &amp; sunny: 13.2 sun hrs, water 84.5F). Kept the full gallon despite FC already at 16.6 -- the CC creep (0.0-&gt;0.4-&gt;0.6) wants FC held up to oxidize it. Season total 20.0 gal. PHOTOS(5): water clear/healthy blue in all wide shots, bottom fully visible, no cloudiness or algae; liner step close-up shows normal speckled blue, NO rust/stain progression. NOTABLE: one surface shot shows scattered floating debris (small leaves/organic bits) -- likely the source of the CC creep (organic load -&gt; chloramines as FC oxidizes it). Recommend skimming/netting it out; higher FC should clear the CC. Ruler photo documents the 11.8 cm level. Model note: this dose's prediction (15.1) is the forward-validation target for 7/4 noon; if it lands high again (&gt;15.1) that's a 3rd hot-day over-prediction -&gt; nudge l24_hot_sunny toward ~4.5.</t>
@@ -8320,51 +8428,51 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="1657" t="inlineStr">
+      <c r="A49" s="1699" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B49" s="1658" t="inlineStr">
+      <c r="B49" s="1700" t="inlineStr">
         <is>
           <t>12:40</t>
         </is>
       </c>
-      <c r="C49" s="1658" t="inlineStr">
+      <c r="C49" s="1700" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D49" s="1659" t="n"/>
-      <c r="E49" s="1659" t="n">
+      <c r="D49" s="1701" t="n"/>
+      <c r="E49" s="1701" t="n">
         <v>16.8</v>
       </c>
-      <c r="F49" s="1659" t="n">
+      <c r="F49" s="1701" t="n">
         <v>0.2</v>
       </c>
-      <c r="G49" s="1659" t="n">
+      <c r="G49" s="1701" t="n">
         <v>3.3</v>
       </c>
-      <c r="H49" s="1659" t="n"/>
-      <c r="I49" s="1660" t="n">
+      <c r="H49" s="1701" t="n"/>
+      <c r="I49" s="1702" t="n">
         <v>1.7</v>
       </c>
-      <c r="J49" s="1661" t="n"/>
-      <c r="K49" s="1661" t="n"/>
-      <c r="L49" s="1661" t="n"/>
-      <c r="M49" s="1659" t="n"/>
-      <c r="N49" s="1659" t="n"/>
-      <c r="O49" s="1659" t="n">
+      <c r="J49" s="1703" t="n"/>
+      <c r="K49" s="1703" t="n"/>
+      <c r="L49" s="1703" t="n"/>
+      <c r="M49" s="1701" t="n"/>
+      <c r="N49" s="1701" t="n"/>
+      <c r="O49" s="1701" t="n">
         <v>13</v>
       </c>
-      <c r="P49" s="1662" t="n">
+      <c r="P49" s="1704" t="n">
         <v>0.87</v>
       </c>
-      <c r="Q49" s="1659" t="n"/>
-      <c r="R49" s="1659" t="n">
+      <c r="Q49" s="1701" t="n"/>
+      <c r="R49" s="1701" t="n">
         <v>86</v>
       </c>
-      <c r="S49" s="1659" t="n">
+      <c r="S49" s="1701" t="n">
         <v>11.65</v>
       </c>
       <c r="T49" s="624" t="inlineStr">
@@ -8372,7 +8480,7 @@
           <t>Clear now, 88F, 67% RH; sun so far 6.4h of 7h daylight (91%); today high 90F, 0.87in precip, UV max 7.9</t>
         </is>
       </c>
-      <c r="U49" s="1658" t="inlineStr">
+      <c r="U49" s="1700" t="inlineStr">
         <is>
           <t>2026-07-04_1.jpeg;2026-07-04_2.jpeg;2026-07-04_3.jpeg;2026-07-04_4.jpeg</t>
         </is>
@@ -8384,49 +8492,49 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="1663" t="inlineStr">
+      <c r="A50" s="1705" t="inlineStr">
         <is>
           <t>2026-07-04</t>
         </is>
       </c>
-      <c r="B50" s="1664" t="inlineStr">
+      <c r="B50" s="1706" t="inlineStr">
         <is>
           <t>19:40</t>
         </is>
       </c>
-      <c r="C50" s="1664" t="inlineStr">
+      <c r="C50" s="1706" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D50" s="1665" t="n"/>
-      <c r="E50" s="1665" t="n"/>
-      <c r="F50" s="1665" t="n"/>
-      <c r="G50" s="1665" t="n"/>
-      <c r="H50" s="1665" t="n">
+      <c r="D50" s="1707" t="n"/>
+      <c r="E50" s="1707" t="n"/>
+      <c r="F50" s="1707" t="n"/>
+      <c r="G50" s="1707" t="n"/>
+      <c r="H50" s="1707" t="n">
         <v>14.6</v>
       </c>
-      <c r="I50" s="1666" t="n"/>
-      <c r="J50" s="1667" t="n"/>
-      <c r="K50" s="1667" t="n"/>
-      <c r="L50" s="1667" t="n"/>
-      <c r="M50" s="1665" t="n">
+      <c r="I50" s="1708" t="n"/>
+      <c r="J50" s="1709" t="n"/>
+      <c r="K50" s="1709" t="n"/>
+      <c r="L50" s="1709" t="n"/>
+      <c r="M50" s="1707" t="n">
         <v>0.5</v>
       </c>
-      <c r="N50" s="1665" t="n">
+      <c r="N50" s="1707" t="n">
         <v>20.5</v>
       </c>
-      <c r="O50" s="1665" t="n"/>
-      <c r="P50" s="1668" t="n"/>
-      <c r="Q50" s="1665" t="n"/>
-      <c r="R50" s="1665" t="n"/>
-      <c r="S50" s="1665" t="n"/>
+      <c r="O50" s="1707" t="n"/>
+      <c r="P50" s="1710" t="n"/>
+      <c r="Q50" s="1707" t="n"/>
+      <c r="R50" s="1707" t="n"/>
+      <c r="S50" s="1707" t="n"/>
       <c r="T50" s="631" t="inlineStr">
         <is>
           <t>Hot/sunny day (high 90F, water 86F); storm forecast overnight</t>
         </is>
       </c>
-      <c r="U50" s="1664" t="n"/>
+      <c r="U50" s="1706" t="n"/>
       <c r="V50" s="632" t="inlineStr">
         <is>
           <t>0.5 gal added 7:40 PM. PARTY PRE-LOAD (Sun 7/5 1PM picnic): deliberately HALF the usual dose -- FC already high at 16.8, and John didn't want to overshoot into the high teens for guests. Sized on the retuned model (l24_hot_sunny now 4.0). Model projects ~14.6 next noon, BUT this is a known weather-mismatch case: model keys L24 off today's hot/sunny weather, while the actual loss window is a storm overnight (no UV) + cooler/cloudy Sun morning -&gt; real loss will be LOWER, so FC likely lands ~15-16 at the party (comfortable top-of-band, cushion for bather load, not overboard). =&gt; If tomorrow's noon comes in ABOVE 14.6, that's the weather mismatch, NOT the freshly-retuned constant; don't chase it. Plan: dose back up Sun evening after the crowd's out (expect a bather-load FC drop). Season total 20.5 gal. PHOTOS(4): water clear/healthy blue, bottom fully visible, no cloudiness/algae; yesterday's surface debris now gone (tracks with CC clearing to 0.2); liner step close-up normal speckled blue, no rust/stain progression. Ruler photo documents the ~11.65 cm level.</t>
@@ -8434,47 +8542,47 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="1669" t="inlineStr">
+      <c r="A51" s="1711" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B51" s="1670" t="inlineStr">
+      <c r="B51" s="1712" t="inlineStr">
         <is>
           <t>07:45</t>
         </is>
       </c>
-      <c r="C51" s="1670" t="inlineStr">
+      <c r="C51" s="1712" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D51" s="1671" t="n"/>
-      <c r="E51" s="1671" t="n">
+      <c r="D51" s="1713" t="n"/>
+      <c r="E51" s="1713" t="n">
         <v>16</v>
       </c>
-      <c r="F51" s="1671" t="n">
+      <c r="F51" s="1713" t="n">
         <v>0.5</v>
       </c>
-      <c r="G51" s="1671" t="n"/>
-      <c r="H51" s="1671" t="n"/>
-      <c r="I51" s="1672" t="n">
+      <c r="G51" s="1713" t="n"/>
+      <c r="H51" s="1713" t="n"/>
+      <c r="I51" s="1714" t="n">
         <v>1.4</v>
       </c>
-      <c r="J51" s="1673" t="n"/>
-      <c r="K51" s="1673" t="n"/>
-      <c r="L51" s="1673" t="n"/>
-      <c r="M51" s="1671" t="n"/>
-      <c r="N51" s="1671" t="n"/>
-      <c r="O51" s="1671" t="n"/>
-      <c r="P51" s="1674" t="n">
+      <c r="J51" s="1715" t="n"/>
+      <c r="K51" s="1715" t="n"/>
+      <c r="L51" s="1715" t="n"/>
+      <c r="M51" s="1713" t="n"/>
+      <c r="N51" s="1713" t="n"/>
+      <c r="O51" s="1713" t="n"/>
+      <c r="P51" s="1716" t="n">
         <v>0.04</v>
       </c>
-      <c r="Q51" s="1671" t="n"/>
-      <c r="R51" s="1671" t="n">
+      <c r="Q51" s="1713" t="n"/>
+      <c r="R51" s="1713" t="n">
         <v>84</v>
       </c>
-      <c r="S51" s="1671" t="n">
+      <c r="S51" s="1713" t="n">
         <v>13.9</v>
       </c>
       <c r="T51" s="813" t="inlineStr">
@@ -8482,7 +8590,7 @@
           <t>Overcast now, 75F, 90% RH; sun so far 0.0h of 3h daylight (0%); today high 75F, 0.04in precip, UV max 6.5</t>
         </is>
       </c>
-      <c r="U51" s="1670" t="inlineStr">
+      <c r="U51" s="1712" t="inlineStr">
         <is>
           <t>2026-07-05_2.jpeg</t>
         </is>
@@ -8494,41 +8602,41 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="1675" t="inlineStr">
+      <c r="A52" s="1717" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B52" s="1676" t="inlineStr">
+      <c r="B52" s="1718" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C52" s="1676" t="inlineStr">
+      <c r="C52" s="1718" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D52" s="1677" t="n"/>
-      <c r="E52" s="1677" t="n">
+      <c r="D52" s="1719" t="n"/>
+      <c r="E52" s="1719" t="n">
         <v>14.8</v>
       </c>
-      <c r="F52" s="1677" t="n">
+      <c r="F52" s="1719" t="n">
         <v>0.3</v>
       </c>
-      <c r="G52" s="1677" t="n"/>
-      <c r="H52" s="1677" t="n"/>
-      <c r="I52" s="1678" t="n"/>
-      <c r="J52" s="1679" t="n"/>
-      <c r="K52" s="1679" t="n"/>
-      <c r="L52" s="1679" t="n"/>
-      <c r="M52" s="1677" t="n"/>
-      <c r="N52" s="1677" t="n"/>
-      <c r="O52" s="1677" t="n"/>
-      <c r="P52" s="1680" t="n"/>
-      <c r="Q52" s="1677" t="n"/>
-      <c r="R52" s="1677" t="n"/>
-      <c r="S52" s="1677" t="n">
+      <c r="G52" s="1719" t="n"/>
+      <c r="H52" s="1719" t="n"/>
+      <c r="I52" s="1720" t="n"/>
+      <c r="J52" s="1721" t="n"/>
+      <c r="K52" s="1721" t="n"/>
+      <c r="L52" s="1721" t="n"/>
+      <c r="M52" s="1719" t="n"/>
+      <c r="N52" s="1719" t="n"/>
+      <c r="O52" s="1719" t="n"/>
+      <c r="P52" s="1722" t="n"/>
+      <c r="Q52" s="1719" t="n"/>
+      <c r="R52" s="1719" t="n"/>
+      <c r="S52" s="1719" t="n">
         <v>13.6</v>
       </c>
       <c r="T52" s="820" t="inlineStr">
@@ -8536,7 +8644,7 @@
           <t>Overcast now, 72F, 76% RH; sun so far 8.4h of 13h daylight (65%); today high 80F, 0.00in precip, UV max 6.0</t>
         </is>
       </c>
-      <c r="U52" s="1676" t="inlineStr">
+      <c r="U52" s="1718" t="inlineStr">
         <is>
           <t>2026-07-05_1.jpeg;2026-07-05_3.jpeg</t>
         </is>
@@ -8548,49 +8656,49 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="1681" t="inlineStr">
+      <c r="A53" s="1723" t="inlineStr">
         <is>
           <t>2026-07-05</t>
         </is>
       </c>
-      <c r="B53" s="1682" t="inlineStr">
+      <c r="B53" s="1724" t="inlineStr">
         <is>
           <t>19:25</t>
         </is>
       </c>
-      <c r="C53" s="1682" t="inlineStr">
+      <c r="C53" s="1724" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D53" s="1683" t="n"/>
-      <c r="E53" s="1683" t="n"/>
-      <c r="F53" s="1683" t="n"/>
-      <c r="G53" s="1683" t="n"/>
-      <c r="H53" s="1683" t="n">
+      <c r="D53" s="1725" t="n"/>
+      <c r="E53" s="1725" t="n"/>
+      <c r="F53" s="1725" t="n"/>
+      <c r="G53" s="1725" t="n"/>
+      <c r="H53" s="1725" t="n">
         <v>15.1</v>
       </c>
-      <c r="I53" s="1684" t="n"/>
-      <c r="J53" s="1685" t="n"/>
-      <c r="K53" s="1685" t="n"/>
-      <c r="L53" s="1685" t="n"/>
-      <c r="M53" s="1683" t="n">
+      <c r="I53" s="1726" t="n"/>
+      <c r="J53" s="1727" t="n"/>
+      <c r="K53" s="1727" t="n"/>
+      <c r="L53" s="1727" t="n"/>
+      <c r="M53" s="1725" t="n">
         <v>0.5</v>
       </c>
-      <c r="N53" s="1683" t="n">
+      <c r="N53" s="1725" t="n">
         <v>21</v>
       </c>
-      <c r="O53" s="1683" t="n"/>
-      <c r="P53" s="1686" t="n"/>
-      <c r="Q53" s="1683" t="n"/>
-      <c r="R53" s="1683" t="n"/>
-      <c r="S53" s="1683" t="n"/>
+      <c r="O53" s="1725" t="n"/>
+      <c r="P53" s="1728" t="n"/>
+      <c r="Q53" s="1725" t="n"/>
+      <c r="R53" s="1725" t="n"/>
+      <c r="S53" s="1725" t="n"/>
       <c r="T53" s="827" t="inlineStr">
         <is>
           <t>Cleared to partly sunny (8.4 sun hrs, high 80F, water 84F); all-day rain forecast Mon 7/6</t>
         </is>
       </c>
-      <c r="U53" s="1682" t="n"/>
+      <c r="U53" s="1724" t="n"/>
       <c r="V53" s="828" t="inlineStr">
         <is>
           <t>0.5 gal added 7:25 PM (post-party recovery dose). Sized on TOMORROW's rainy forecast (the real loss window: overcast/wet 7/6, ~0.9in rain, low UV) not today's sun -&gt; projects ~15.1 at Mon noon. Party went great (FC held 16.0-&gt;14.8, CC dropped 0.5-&gt;0.3). Season total 21.0 gal. This is the first prediction that deliberately used the next-day forecast for L24 instead of the model's default (today's weather as proxy) -- if it lands near 15.1 tomorrow, that validates feeding the forecast on weather-change days.</t>
@@ -8598,49 +8706,49 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="1657" t="inlineStr">
+      <c r="A54" s="1699" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B54" s="1658" t="inlineStr">
+      <c r="B54" s="1700" t="inlineStr">
         <is>
           <t>11:40</t>
         </is>
       </c>
-      <c r="C54" s="1658" t="inlineStr">
+      <c r="C54" s="1700" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D54" s="1659" t="n"/>
-      <c r="E54" s="1659" t="n">
+      <c r="D54" s="1701" t="n"/>
+      <c r="E54" s="1701" t="n">
         <v>13.8</v>
       </c>
-      <c r="F54" s="1659" t="n">
+      <c r="F54" s="1701" t="n">
         <v>0.2</v>
       </c>
-      <c r="G54" s="1659" t="n"/>
-      <c r="H54" s="1659" t="n"/>
-      <c r="I54" s="1660" t="n">
+      <c r="G54" s="1701" t="n"/>
+      <c r="H54" s="1701" t="n"/>
+      <c r="I54" s="1702" t="n">
         <v>-1.3</v>
       </c>
-      <c r="J54" s="1661" t="n"/>
-      <c r="K54" s="1661" t="n"/>
-      <c r="L54" s="1661" t="n"/>
-      <c r="M54" s="1659" t="n"/>
-      <c r="N54" s="1659" t="n"/>
-      <c r="O54" s="1659" t="n">
+      <c r="J54" s="1703" t="n"/>
+      <c r="K54" s="1703" t="n"/>
+      <c r="L54" s="1703" t="n"/>
+      <c r="M54" s="1701" t="n"/>
+      <c r="N54" s="1701" t="n"/>
+      <c r="O54" s="1701" t="n">
         <v>0</v>
       </c>
-      <c r="P54" s="1662" t="n">
+      <c r="P54" s="1704" t="n">
         <v>2</v>
       </c>
-      <c r="Q54" s="1659" t="n"/>
-      <c r="R54" s="1659" t="n">
+      <c r="Q54" s="1701" t="n"/>
+      <c r="R54" s="1701" t="n">
         <v>81</v>
       </c>
-      <c r="S54" s="1659" t="n">
+      <c r="S54" s="1701" t="n">
         <v>15.1</v>
       </c>
       <c r="T54" s="624" t="inlineStr">
@@ -8648,7 +8756,7 @@
           <t>Light rain now, 65F, 93% RH; sun so far 0.0h of 6h daylight (0%); today high 68F, 2.00in precip, UV max 0.5</t>
         </is>
       </c>
-      <c r="U54" s="1658" t="inlineStr">
+      <c r="U54" s="1700" t="inlineStr">
         <is>
           <t>2026-07-06_1.jpeg</t>
         </is>
@@ -8660,39 +8768,39 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="1687" t="inlineStr">
+      <c r="A55" s="1729" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B55" s="1688" t="inlineStr">
+      <c r="B55" s="1730" t="inlineStr">
         <is>
           <t>19:15</t>
         </is>
       </c>
-      <c r="C55" s="1688" t="inlineStr">
+      <c r="C55" s="1730" t="inlineStr">
         <is>
           <t>EVENT - Waste</t>
         </is>
       </c>
-      <c r="D55" s="1689" t="n"/>
-      <c r="E55" s="1689" t="n"/>
-      <c r="F55" s="1689" t="n"/>
-      <c r="G55" s="1689" t="n"/>
-      <c r="H55" s="1689" t="n"/>
-      <c r="I55" s="1690" t="n"/>
-      <c r="J55" s="1691" t="n"/>
-      <c r="K55" s="1691" t="n"/>
-      <c r="L55" s="1691" t="n"/>
-      <c r="M55" s="1689" t="n"/>
-      <c r="N55" s="1689" t="n"/>
-      <c r="O55" s="1689" t="n"/>
-      <c r="P55" s="1692" t="n"/>
-      <c r="Q55" s="1689" t="n"/>
-      <c r="R55" s="1689" t="n"/>
-      <c r="S55" s="1689" t="n"/>
+      <c r="D55" s="1731" t="n"/>
+      <c r="E55" s="1731" t="n"/>
+      <c r="F55" s="1731" t="n"/>
+      <c r="G55" s="1731" t="n"/>
+      <c r="H55" s="1731" t="n"/>
+      <c r="I55" s="1732" t="n"/>
+      <c r="J55" s="1733" t="n"/>
+      <c r="K55" s="1733" t="n"/>
+      <c r="L55" s="1733" t="n"/>
+      <c r="M55" s="1731" t="n"/>
+      <c r="N55" s="1731" t="n"/>
+      <c r="O55" s="1731" t="n"/>
+      <c r="P55" s="1734" t="n"/>
+      <c r="Q55" s="1731" t="n"/>
+      <c r="R55" s="1731" t="n"/>
+      <c r="S55" s="1731" t="n"/>
       <c r="T55" s="659" t="n"/>
-      <c r="U55" s="1688" t="inlineStr">
+      <c r="U55" s="1730" t="inlineStr">
         <is>
           <t>2026-07-06_2.jpeg;2026-07-06_3.jpeg</t>
         </is>
@@ -8704,49 +8812,49 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="1663" t="inlineStr">
+      <c r="A56" s="1705" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B56" s="1664" t="inlineStr">
+      <c r="B56" s="1706" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C56" s="1664" t="inlineStr">
+      <c r="C56" s="1706" t="inlineStr">
         <is>
           <t>DOSE</t>
         </is>
       </c>
-      <c r="D56" s="1665" t="n"/>
-      <c r="E56" s="1665" t="n"/>
-      <c r="F56" s="1665" t="n"/>
-      <c r="G56" s="1665" t="n"/>
-      <c r="H56" s="1665" t="n">
+      <c r="D56" s="1707" t="n"/>
+      <c r="E56" s="1707" t="n"/>
+      <c r="F56" s="1707" t="n"/>
+      <c r="G56" s="1707" t="n"/>
+      <c r="H56" s="1707" t="n">
         <v>14</v>
       </c>
-      <c r="I56" s="1666" t="n"/>
-      <c r="J56" s="1667" t="n"/>
-      <c r="K56" s="1667" t="n"/>
-      <c r="L56" s="1667" t="n"/>
-      <c r="M56" s="1665" t="n">
+      <c r="I56" s="1708" t="n"/>
+      <c r="J56" s="1709" t="n"/>
+      <c r="K56" s="1709" t="n"/>
+      <c r="L56" s="1709" t="n"/>
+      <c r="M56" s="1707" t="n">
         <v>1</v>
       </c>
-      <c r="N56" s="1665" t="n">
+      <c r="N56" s="1707" t="n">
         <v>22</v>
       </c>
-      <c r="O56" s="1665" t="n"/>
-      <c r="P56" s="1668" t="n"/>
-      <c r="Q56" s="1665" t="n"/>
-      <c r="R56" s="1665" t="n"/>
-      <c r="S56" s="1665" t="n"/>
+      <c r="O56" s="1707" t="n"/>
+      <c r="P56" s="1710" t="n"/>
+      <c r="Q56" s="1707" t="n"/>
+      <c r="R56" s="1707" t="n"/>
+      <c r="S56" s="1707" t="n"/>
       <c r="T56" s="631" t="inlineStr">
         <is>
           <t>Rain all day (2.00in total), overcast, 65-68F; more rain Tue</t>
         </is>
       </c>
-      <c r="U56" s="1664" t="n"/>
+      <c r="U56" s="1706" t="n"/>
       <c r="V56" s="632" t="inlineStr">
         <is>
           <t>1.0 gal added 7:30 PM, AFTER the pump-to-waste (correct order -- don't chlorinate water you're about to pump out). FIRST dose on the recalibrated buckets (rain L24 now 2.5 vs old 1.5). CORRECTION carried in: John is NOT low on chlorine -- he was low on TEST REAGENTS, which arrived today -- so this is the full 1 gal (not the 0.5 I'd wrongly trimmed for 'conservation'). Base FC ~13 est (noon 13.8 minus the bit of FC removed by the pump-out; not re-tested), + 1gal x3.5 - 2.5 rain loss -&gt; pred ~14.0 at Tue noon. Prediction is confounded this round (pump perturbation + no post-empty FC test) -&gt; tomorrow's error will be noisy, don't read too much into it for bucket validation. Season total 22.0 gal.</t>
@@ -8754,62 +8862,112 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="1693" t="inlineStr">
+      <c r="A57" s="1711" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B57" s="1694" t="inlineStr">
+      <c r="B57" s="1712" t="inlineStr">
         <is>
           <t>11:50</t>
         </is>
       </c>
-      <c r="C57" s="1694" t="inlineStr">
+      <c r="C57" s="1712" t="inlineStr">
         <is>
           <t>TEST</t>
         </is>
       </c>
-      <c r="D57" s="1695" t="n"/>
-      <c r="E57" s="1695" t="n">
+      <c r="D57" s="1713" t="n"/>
+      <c r="E57" s="1713" t="n">
         <v>14.6</v>
       </c>
-      <c r="F57" s="1695" t="n">
+      <c r="F57" s="1713" t="n">
         <v>0.8</v>
       </c>
-      <c r="G57" s="1695" t="n"/>
-      <c r="H57" s="1695" t="n"/>
-      <c r="I57" s="1696" t="n">
+      <c r="G57" s="1713" t="n"/>
+      <c r="H57" s="1713" t="n"/>
+      <c r="I57" s="1714" t="n">
         <v>0.6</v>
       </c>
-      <c r="J57" s="1697" t="n"/>
-      <c r="K57" s="1697" t="n"/>
-      <c r="L57" s="1697" t="n"/>
-      <c r="M57" s="1695" t="n"/>
-      <c r="N57" s="1695" t="n"/>
-      <c r="O57" s="1695" t="n">
+      <c r="J57" s="1715" t="n"/>
+      <c r="K57" s="1715" t="n"/>
+      <c r="L57" s="1715" t="n"/>
+      <c r="M57" s="1713" t="n"/>
+      <c r="N57" s="1713" t="n"/>
+      <c r="O57" s="1713" t="n">
         <v>0</v>
       </c>
-      <c r="P57" s="1698" t="n"/>
-      <c r="Q57" s="1695" t="n"/>
-      <c r="R57" s="1695" t="n">
+      <c r="P57" s="1716" t="n"/>
+      <c r="Q57" s="1713" t="n"/>
+      <c r="R57" s="1713" t="n">
         <v>76</v>
       </c>
-      <c r="S57" s="1695" t="n">
+      <c r="S57" s="1713" t="n">
         <v>15.5</v>
       </c>
-      <c r="T57" s="1199" t="inlineStr">
+      <c r="T57" s="813" t="inlineStr">
         <is>
           <t>Overcast now, 66F, 91% RH; sun so far 0.0h of 6h daylight (0%); today high 69F, 0.00in precip, UV max 1.4</t>
         </is>
       </c>
-      <c r="U57" s="1694" t="inlineStr">
+      <c r="U57" s="1712" t="inlineStr">
         <is>
           <t>2026-07-07_1.jpeg</t>
         </is>
       </c>
-      <c r="V57" s="1200" t="inlineStr">
+      <c r="V57" s="814" t="inlineStr">
         <is>
           <t>25mL x0.2. FC 14.6, CC 0.8 -- in band, healthy (FC/CYA 9.7%, comfortably above the ~7.5% min). PREDICTION: pred error +0.6 (actual 14.6 vs 7/6 dose's 14.0) -- FIRST noon on the recalibrated rain bucket (L24 2.5, up from old 1.5). Small miss, lost slightly LESS than modeled. CONFOUNDED though: yesterday's pump-to-waste removed chlorinated water + rain dilution, and the dose base FC was ESTIMATED ~13 (not re-tested post-empty) -- so do NOT retune off this single point. Directionally encouraging vs 7/6's -1.3 on the old 1.5 bucket (narrowing moved the rainy-day error from -1.3 toward 0). CC UP 0.2 -&gt; 0.8: two days of storm runoff washing organic/N load in (same mechanism as the 7/5 0.2-&gt;0.5 tick). 0.8 is above the 0.5 flag but still a trace; FC 14.6 is plenty to oxidize it -- expect it to clear over the next day or two now the rain has stopped. WATCH: if CC climbs toward 1.0+ or FC can't knock it down, revisit. fc_loss BLANK: noon-to-noon confounded by the pump-to-waste + 1gal dose + rain dilution -- not a clean value. Water temp 76 continues the cold-front slide (86-&gt;84-&gt;81-&gt;76); will rebound when sun returns. Level 15.5 cm (+0.4 vs yesterday's post-pump 15.1 -- overnight storm tail); rain has now STOPPED (feed 0.00in today) so the level should hold / slowly evaporate down -- no pump needed. rain_in left blank: trace overnight rise but no measurable daytime rain and the day isn't over. PHOTO documents the 15.5 level (tight ruler crop; water clear where visible, no debris).</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="1723" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B58" s="1724" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C58" s="1724" t="inlineStr">
+        <is>
+          <t>DOSE</t>
+        </is>
+      </c>
+      <c r="D58" s="1725" t="n"/>
+      <c r="E58" s="1725" t="n"/>
+      <c r="F58" s="1725" t="n"/>
+      <c r="G58" s="1725" t="n"/>
+      <c r="H58" s="1725" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="I58" s="1726" t="n"/>
+      <c r="J58" s="1727" t="n"/>
+      <c r="K58" s="1727" t="n"/>
+      <c r="L58" s="1727" t="n"/>
+      <c r="M58" s="1725" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N58" s="1725" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="O58" s="1725" t="n"/>
+      <c r="P58" s="1728" t="n"/>
+      <c r="Q58" s="1725" t="n"/>
+      <c r="R58" s="1725" t="n"/>
+      <c r="S58" s="1725" t="n"/>
+      <c r="T58" s="827" t="inlineStr">
+        <is>
+          <t>Overcast/cool at dose (66-70F, 0 sun today); forecast flips to full sun Wed 7/8 (13.5 sun-hrs, 78F, UV 7.8) then sunny Thu 7/9 (82F)</t>
+        </is>
+      </c>
+      <c r="U58" s="1724" t="n"/>
+      <c r="V58" s="828" t="inlineStr">
+        <is>
+          <t>1.5 gal added 6:30 PM. DELIBERATE PRE-LOAD for John's away-day: he can't dose Wed 7/8 evening (away until very late), and the forecast flips to FULL SUN Wed (13.5 sun-hrs, 78F, UV 7.8) + sunny Thu -- a 2-day high-loss coast with no evening top-up. Sized 1.5 (vs the ~1.0 a normal day would call for) to keep FC safely above the 10.5 floor across both sunny days. PROJECTION: ~17.3 at Wed noon (this leg is mostly overnight + a sunny Wed morning, L24~2.5), then the full sunny Wed day pulls it to ~13.5-14 at Thu 7/9 noon when John rechecks + resumes dosing -- comfortable margin above floor throughout. Peak tonight ~19 (harmless at CYA 150; shock is 40+, and nobody swims Wed). CC ANGLE: high FC + Wed's strong UV should finish oxidizing the 0.8 CC -- watch Wed noon test for it dropping. PREDICTION NOTE: John CAN still test Wed noon, so this dose gets scored cleanly one-noon-out (~17.3 target) despite the skipped evening dose; the further 2-day coast to Thu is tracked separately (noisier). Level high (15.5) but Wed's sun evaporates it down; no rain till a light 0.2in Thu -&gt; nothing to pump while away. Season total 23.5 gal.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Log 2026-07-08 noon TEST: FC 18.0, CC 0.3, level 15.0; pred +0.6 (away-day pre-load validated, CC cleared)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Pool_Log.xlsx
+++ b/Pool_Log.xlsx
@@ -538,7 +538,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1735">
+  <cellXfs count="1777">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -5732,6 +5732,132 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="7" fillId="0" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="3" bo